<commit_message>
Update amplitude website 2026-07-07
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rf338f7d700884015"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="2" r:id="R88a8ff336d564331"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="3" r:id="Ra48c71ae96864fb2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="4" r:id="Rddd81dd5e51f40d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="5" r:id="Ra18ff62a19b04dca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="6" r:id="Rb4033f7664484331"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="7" r:id="R3f02d051ef2245dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="8" r:id="R162c4cee1ed645b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R2cf5cebb27ab4e28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="2" r:id="R60d95cb8c52149ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="3" r:id="Rb881b96f2fd14a82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="4" r:id="R8ed9804b104845d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="5" r:id="Ra40c569daa604403"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="6" r:id="Ref60e8e650624f60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="7" r:id="R4c577a5cc44a471e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="8" r:id="Rc5f11a3f1d1247b8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -448,25 +448,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-07-03</x:v>
+        <x:v>2026-07-07</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>8740.668</x:v>
+        <x:v>8489.476</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>8559.285</x:v>
+        <x:v>8261.398</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>181.4</x:v>
+        <x:v>228.1</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>586</x:v>
+        <x:v>1076</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>195.3</x:v>
+        <x:v>215.2</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -477,25 +477,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-07-03</x:v>
+        <x:v>2026-07-07</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>8860.416</x:v>
+        <x:v>8663.665</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>8636.15</x:v>
+        <x:v>8457.576</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>224.3</x:v>
+        <x:v>206.1</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>680.9</x:v>
+        <x:v>1139.2</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>227</x:v>
+        <x:v>227.8</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -506,25 +506,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-07-03</x:v>
+        <x:v>2026-07-07</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>4073.88</x:v>
+        <x:v>4028.514</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>4027.255</x:v>
+        <x:v>3971.713</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>46.6</x:v>
+        <x:v>56.8</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>176.9</x:v>
+        <x:v>288.4</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>59</x:v>
+        <x:v>57.7</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -535,25 +535,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-07-03</x:v>
+        <x:v>2026-07-07</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>8475</x:v>
+        <x:v>8274.2</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>8337.8</x:v>
+        <x:v>8068.8</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>137.2</x:v>
+        <x:v>205.4</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>498.2</x:v>
+        <x:v>910.4</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>166.1</x:v>
+        <x:v>182.1</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -564,25 +564,25 @@
         <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>2026-07-03</x:v>
+        <x:v>2026-07-07</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:v>8650</x:v>
+        <x:v>8478.8</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>8442</x:v>
+        <x:v>8281</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>208</x:v>
+        <x:v>197.8</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>646.8</x:v>
+        <x:v>1052.8</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
-        <x:v>215.6</x:v>
+        <x:v>210.6</x:v>
       </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
@@ -593,25 +593,25 @@
         <x:v>IF主力</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>2026-07-03</x:v>
+        <x:v>2026-07-07</x:v>
       </x:c>
       <x:c r="C9" s="10" t="n">
-        <x:v>4810.4</x:v>
+        <x:v>4752.6</x:v>
       </x:c>
       <x:c r="D9" s="10" t="n">
-        <x:v>4728</x:v>
+        <x:v>4671.4</x:v>
       </x:c>
       <x:c r="E9" s="12" t="n">
-        <x:v>82.4</x:v>
+        <x:v>81.2</x:v>
       </x:c>
       <x:c r="F9" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G9" s="10" t="n">
-        <x:v>275</x:v>
+        <x:v>436.4</x:v>
       </x:c>
       <x:c r="H9" s="10" t="n">
-        <x:v>91.7</x:v>
+        <x:v>87.3</x:v>
       </x:c>
       <x:c r="I9" s="10" t="n">
         <x:v>90</x:v>
@@ -622,25 +622,25 @@
         <x:v>IH主力</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>2026-07-03</x:v>
+        <x:v>2026-07-07</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:v>2912</x:v>
+        <x:v>2908.4</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
-        <x:v>2873.6</x:v>
+        <x:v>2862.4</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
-        <x:v>38.4</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="F10" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G10" s="10" t="n">
-        <x:v>159.2</x:v>
+        <x:v>242.8</x:v>
       </x:c>
       <x:c r="H10" s="10" t="n">
-        <x:v>53.1</x:v>
+        <x:v>48.6</x:v>
       </x:c>
       <x:c r="I10" s="10" t="n">
         <x:v>60</x:v>
@@ -654,7 +654,7 @@
         <x:v>2026-07-01</x:v>
       </x:c>
       <x:c r="C13" s="14" t="str">
-        <x:v>2026-07-04</x:v>
+        <x:v>2026-07-07</x:v>
       </x:c>
       <x:c r="D13" s="14" t="str">
         <x:v>数据源</x:v>
@@ -879,35 +879,83 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="27" t="str">
+    <x:row r="7">
+      <x:c r="A7" s="21" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="21" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C7" s="21" t="str">
+        <x:v>7月6日</x:v>
+      </x:c>
+      <x:c r="D7" s="22" t="n">
+        <x:v>8694.805</x:v>
+      </x:c>
+      <x:c r="E7" s="22" t="n">
+        <x:v>8432.897</x:v>
+      </x:c>
+      <x:c r="F7" s="24" t="n">
+        <x:f>ROUND(D7-E7,1)</x:f>
+        <x:v>261.9</x:v>
+      </x:c>
+      <x:c r="G7" s="21" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="21" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="21" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C8" s="21" t="str">
+        <x:v>7月7日</x:v>
+      </x:c>
+      <x:c r="D8" s="22" t="n">
+        <x:v>8489.476</x:v>
+      </x:c>
+      <x:c r="E8" s="22" t="n">
+        <x:v>8261.398</x:v>
+      </x:c>
+      <x:c r="F8" s="24" t="n">
+        <x:f>ROUND(D8-E8,1)</x:f>
+        <x:v>228.1</x:v>
+      </x:c>
+      <x:c r="G8" s="21" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="27" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B9" s="28" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C9" s="28"/>
-      <x:c r="D9" s="28"/>
-      <x:c r="E9" s="28"/>
-      <x:c r="F9" s="29" t="n">
-        <x:f>SUM(F4:F6)</x:f>
-        <x:v>586</x:v>
-      </x:c>
-      <x:c r="G9" s="28"/>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="27" t="str">
+      <x:c r="B11" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C11" s="28"/>
+      <x:c r="D11" s="28"/>
+      <x:c r="E11" s="28"/>
+      <x:c r="F11" s="29" t="n">
+        <x:f>SUM(F4:F8)</x:f>
+        <x:v>1076</x:v>
+      </x:c>
+      <x:c r="G11" s="28"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="27" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B10" s="28"/>
-      <x:c r="C10" s="28"/>
-      <x:c r="D10" s="28"/>
-      <x:c r="E10" s="28"/>
-      <x:c r="F10" s="31" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(F4:F6),0),1)</x:f>
-        <x:v>195.3</x:v>
-      </x:c>
-      <x:c r="G10" s="28"/>
+      <x:c r="B12" s="28"/>
+      <x:c r="C12" s="28"/>
+      <x:c r="D12" s="28"/>
+      <x:c r="E12" s="28"/>
+      <x:c r="F12" s="31" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(F4:F8),0),1)</x:f>
+        <x:v>215.2</x:v>
+      </x:c>
+      <x:c r="G12" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1030,35 +1078,83 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="27" t="str">
+    <x:row r="7">
+      <x:c r="A7" s="21" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="21" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C7" s="21" t="str">
+        <x:v>7月6日</x:v>
+      </x:c>
+      <x:c r="D7" s="22" t="n">
+        <x:v>8823.05</x:v>
+      </x:c>
+      <x:c r="E7" s="22" t="n">
+        <x:v>8570.892</x:v>
+      </x:c>
+      <x:c r="F7" s="24" t="n">
+        <x:f>ROUND(D7-E7,1)</x:f>
+        <x:v>252.2</x:v>
+      </x:c>
+      <x:c r="G7" s="21" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="21" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="21" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C8" s="21" t="str">
+        <x:v>7月7日</x:v>
+      </x:c>
+      <x:c r="D8" s="22" t="n">
+        <x:v>8663.665</x:v>
+      </x:c>
+      <x:c r="E8" s="22" t="n">
+        <x:v>8457.576</x:v>
+      </x:c>
+      <x:c r="F8" s="24" t="n">
+        <x:f>ROUND(D8-E8,1)</x:f>
+        <x:v>206.1</x:v>
+      </x:c>
+      <x:c r="G8" s="21" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="27" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B9" s="28" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C9" s="28"/>
-      <x:c r="D9" s="28"/>
-      <x:c r="E9" s="28"/>
-      <x:c r="F9" s="29" t="n">
-        <x:f>SUM(F4:F6)</x:f>
-        <x:v>680.9000000000001</x:v>
-      </x:c>
-      <x:c r="G9" s="28"/>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="27" t="str">
+      <x:c r="B11" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C11" s="28"/>
+      <x:c r="D11" s="28"/>
+      <x:c r="E11" s="28"/>
+      <x:c r="F11" s="29" t="n">
+        <x:f>SUM(F4:F8)</x:f>
+        <x:v>1139.2</x:v>
+      </x:c>
+      <x:c r="G11" s="28"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="27" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B10" s="28"/>
-      <x:c r="C10" s="28"/>
-      <x:c r="D10" s="28"/>
-      <x:c r="E10" s="28"/>
-      <x:c r="F10" s="31" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(F4:F6),0),1)</x:f>
-        <x:v>227</x:v>
-      </x:c>
-      <x:c r="G10" s="28"/>
+      <x:c r="B12" s="28"/>
+      <x:c r="C12" s="28"/>
+      <x:c r="D12" s="28"/>
+      <x:c r="E12" s="28"/>
+      <x:c r="F12" s="31" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(F4:F8),0),1)</x:f>
+        <x:v>227.8</x:v>
+      </x:c>
+      <x:c r="G12" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1181,35 +1277,83 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="27" t="str">
+    <x:row r="7">
+      <x:c r="A7" s="21" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="21" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C7" s="21" t="str">
+        <x:v>7月6日</x:v>
+      </x:c>
+      <x:c r="D7" s="22" t="n">
+        <x:v>4060.069</x:v>
+      </x:c>
+      <x:c r="E7" s="22" t="n">
+        <x:v>4005.414</x:v>
+      </x:c>
+      <x:c r="F7" s="24" t="n">
+        <x:f>ROUND(D7-E7,1)</x:f>
+        <x:v>54.7</x:v>
+      </x:c>
+      <x:c r="G7" s="21" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="21" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="21" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C8" s="21" t="str">
+        <x:v>7月7日</x:v>
+      </x:c>
+      <x:c r="D8" s="22" t="n">
+        <x:v>4028.514</x:v>
+      </x:c>
+      <x:c r="E8" s="22" t="n">
+        <x:v>3971.713</x:v>
+      </x:c>
+      <x:c r="F8" s="24" t="n">
+        <x:f>ROUND(D8-E8,1)</x:f>
+        <x:v>56.8</x:v>
+      </x:c>
+      <x:c r="G8" s="21" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="27" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B9" s="28" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C9" s="28"/>
-      <x:c r="D9" s="28"/>
-      <x:c r="E9" s="28"/>
-      <x:c r="F9" s="29" t="n">
-        <x:f>SUM(F4:F6)</x:f>
-        <x:v>176.9</x:v>
-      </x:c>
-      <x:c r="G9" s="28"/>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="27" t="str">
+      <x:c r="B11" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C11" s="28"/>
+      <x:c r="D11" s="28"/>
+      <x:c r="E11" s="28"/>
+      <x:c r="F11" s="29" t="n">
+        <x:f>SUM(F4:F8)</x:f>
+        <x:v>288.40000000000003</x:v>
+      </x:c>
+      <x:c r="G11" s="28"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="27" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B10" s="28"/>
-      <x:c r="C10" s="28"/>
-      <x:c r="D10" s="28"/>
-      <x:c r="E10" s="28"/>
-      <x:c r="F10" s="31" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(F4:F6),0),1)</x:f>
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="G10" s="28"/>
+      <x:c r="B12" s="28"/>
+      <x:c r="C12" s="28"/>
+      <x:c r="D12" s="28"/>
+      <x:c r="E12" s="28"/>
+      <x:c r="F12" s="31" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(F4:F8),0),1)</x:f>
+        <x:v>57.7</x:v>
+      </x:c>
+      <x:c r="G12" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1332,35 +1476,83 @@
         <x:v>IM2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="27" t="str">
+    <x:row r="7">
+      <x:c r="A7" s="21" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="21" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C7" s="21" t="str">
+        <x:v>7月6日</x:v>
+      </x:c>
+      <x:c r="D7" s="22" t="n">
+        <x:v>8419.8</x:v>
+      </x:c>
+      <x:c r="E7" s="22" t="n">
+        <x:v>8213</x:v>
+      </x:c>
+      <x:c r="F7" s="24" t="n">
+        <x:f>ROUND(D7-E7,1)</x:f>
+        <x:v>206.8</x:v>
+      </x:c>
+      <x:c r="G7" s="21" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="21" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="21" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C8" s="21" t="str">
+        <x:v>7月7日</x:v>
+      </x:c>
+      <x:c r="D8" s="22" t="n">
+        <x:v>8274.2</x:v>
+      </x:c>
+      <x:c r="E8" s="22" t="n">
+        <x:v>8068.8</x:v>
+      </x:c>
+      <x:c r="F8" s="24" t="n">
+        <x:f>ROUND(D8-E8,1)</x:f>
+        <x:v>205.4</x:v>
+      </x:c>
+      <x:c r="G8" s="21" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="27" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B9" s="28" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C9" s="28"/>
-      <x:c r="D9" s="28"/>
-      <x:c r="E9" s="28"/>
-      <x:c r="F9" s="29" t="n">
-        <x:f>SUM(F4:F6)</x:f>
-        <x:v>498.2</x:v>
-      </x:c>
-      <x:c r="G9" s="28"/>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="27" t="str">
+      <x:c r="B11" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C11" s="28"/>
+      <x:c r="D11" s="28"/>
+      <x:c r="E11" s="28"/>
+      <x:c r="F11" s="29" t="n">
+        <x:f>SUM(F4:F8)</x:f>
+        <x:v>910.4</x:v>
+      </x:c>
+      <x:c r="G11" s="28"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="27" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B10" s="28"/>
-      <x:c r="C10" s="28"/>
-      <x:c r="D10" s="28"/>
-      <x:c r="E10" s="28"/>
-      <x:c r="F10" s="31" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(F4:F6),0),1)</x:f>
-        <x:v>166.1</x:v>
-      </x:c>
-      <x:c r="G10" s="28"/>
+      <x:c r="B12" s="28"/>
+      <x:c r="C12" s="28"/>
+      <x:c r="D12" s="28"/>
+      <x:c r="E12" s="28"/>
+      <x:c r="F12" s="31" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(F4:F8),0),1)</x:f>
+        <x:v>182.1</x:v>
+      </x:c>
+      <x:c r="G12" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1483,35 +1675,83 @@
         <x:v>IC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="27" t="str">
+    <x:row r="7">
+      <x:c r="A7" s="21" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="21" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C7" s="21" t="str">
+        <x:v>7月6日</x:v>
+      </x:c>
+      <x:c r="D7" s="22" t="n">
+        <x:v>8584.2</x:v>
+      </x:c>
+      <x:c r="E7" s="22" t="n">
+        <x:v>8376</x:v>
+      </x:c>
+      <x:c r="F7" s="24" t="n">
+        <x:f>ROUND(D7-E7,1)</x:f>
+        <x:v>208.2</x:v>
+      </x:c>
+      <x:c r="G7" s="21" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="21" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="21" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C8" s="21" t="str">
+        <x:v>7月7日</x:v>
+      </x:c>
+      <x:c r="D8" s="22" t="n">
+        <x:v>8478.8</x:v>
+      </x:c>
+      <x:c r="E8" s="22" t="n">
+        <x:v>8281</x:v>
+      </x:c>
+      <x:c r="F8" s="24" t="n">
+        <x:f>ROUND(D8-E8,1)</x:f>
+        <x:v>197.8</x:v>
+      </x:c>
+      <x:c r="G8" s="21" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="27" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B9" s="28" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C9" s="28"/>
-      <x:c r="D9" s="28"/>
-      <x:c r="E9" s="28"/>
-      <x:c r="F9" s="29" t="n">
-        <x:f>SUM(F4:F6)</x:f>
-        <x:v>646.8</x:v>
-      </x:c>
-      <x:c r="G9" s="28"/>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="27" t="str">
+      <x:c r="B11" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C11" s="28"/>
+      <x:c r="D11" s="28"/>
+      <x:c r="E11" s="28"/>
+      <x:c r="F11" s="29" t="n">
+        <x:f>SUM(F4:F8)</x:f>
+        <x:v>1052.8</x:v>
+      </x:c>
+      <x:c r="G11" s="28"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="27" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B10" s="28"/>
-      <x:c r="C10" s="28"/>
-      <x:c r="D10" s="28"/>
-      <x:c r="E10" s="28"/>
-      <x:c r="F10" s="31" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(F4:F6),0),1)</x:f>
-        <x:v>215.6</x:v>
-      </x:c>
-      <x:c r="G10" s="28"/>
+      <x:c r="B12" s="28"/>
+      <x:c r="C12" s="28"/>
+      <x:c r="D12" s="28"/>
+      <x:c r="E12" s="28"/>
+      <x:c r="F12" s="31" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(F4:F8),0),1)</x:f>
+        <x:v>210.6</x:v>
+      </x:c>
+      <x:c r="G12" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1634,35 +1874,83 @@
         <x:v>IF2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="27" t="str">
+    <x:row r="7">
+      <x:c r="A7" s="21" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="21" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C7" s="21" t="str">
+        <x:v>7月6日</x:v>
+      </x:c>
+      <x:c r="D7" s="22" t="n">
+        <x:v>4781.2</x:v>
+      </x:c>
+      <x:c r="E7" s="22" t="n">
+        <x:v>4701</x:v>
+      </x:c>
+      <x:c r="F7" s="22" t="n">
+        <x:f>ROUND(D7-E7,1)</x:f>
+        <x:v>80.2</x:v>
+      </x:c>
+      <x:c r="G7" s="21" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="21" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="21" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C8" s="21" t="str">
+        <x:v>7月7日</x:v>
+      </x:c>
+      <x:c r="D8" s="22" t="n">
+        <x:v>4752.6</x:v>
+      </x:c>
+      <x:c r="E8" s="22" t="n">
+        <x:v>4671.4</x:v>
+      </x:c>
+      <x:c r="F8" s="22" t="n">
+        <x:f>ROUND(D8-E8,1)</x:f>
+        <x:v>81.2</x:v>
+      </x:c>
+      <x:c r="G8" s="21" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="27" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B9" s="28" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C9" s="28"/>
-      <x:c r="D9" s="28"/>
-      <x:c r="E9" s="28"/>
-      <x:c r="F9" s="29" t="n">
-        <x:f>SUM(F4:F6)</x:f>
-        <x:v>275</x:v>
-      </x:c>
-      <x:c r="G9" s="28"/>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="27" t="str">
+      <x:c r="B11" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C11" s="28"/>
+      <x:c r="D11" s="28"/>
+      <x:c r="E11" s="28"/>
+      <x:c r="F11" s="29" t="n">
+        <x:f>SUM(F4:F8)</x:f>
+        <x:v>436.4</x:v>
+      </x:c>
+      <x:c r="G11" s="28"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="27" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B10" s="28"/>
-      <x:c r="C10" s="28"/>
-      <x:c r="D10" s="28"/>
-      <x:c r="E10" s="28"/>
-      <x:c r="F10" s="31" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(F4:F6),0),1)</x:f>
-        <x:v>91.7</x:v>
-      </x:c>
-      <x:c r="G10" s="28"/>
+      <x:c r="B12" s="28"/>
+      <x:c r="C12" s="28"/>
+      <x:c r="D12" s="28"/>
+      <x:c r="E12" s="28"/>
+      <x:c r="F12" s="31" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(F4:F8),0),1)</x:f>
+        <x:v>87.3</x:v>
+      </x:c>
+      <x:c r="G12" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1785,35 +2073,83 @@
         <x:v>IH2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="27" t="str">
+    <x:row r="7">
+      <x:c r="A7" s="21" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="21" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C7" s="21" t="str">
+        <x:v>7月6日</x:v>
+      </x:c>
+      <x:c r="D7" s="22" t="n">
+        <x:v>2915</x:v>
+      </x:c>
+      <x:c r="E7" s="22" t="n">
+        <x:v>2877.4</x:v>
+      </x:c>
+      <x:c r="F7" s="22" t="n">
+        <x:f>ROUND(D7-E7,1)</x:f>
+        <x:v>37.6</x:v>
+      </x:c>
+      <x:c r="G7" s="21" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="21" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="21" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C8" s="21" t="str">
+        <x:v>7月7日</x:v>
+      </x:c>
+      <x:c r="D8" s="22" t="n">
+        <x:v>2908.4</x:v>
+      </x:c>
+      <x:c r="E8" s="22" t="n">
+        <x:v>2862.4</x:v>
+      </x:c>
+      <x:c r="F8" s="22" t="n">
+        <x:f>ROUND(D8-E8,1)</x:f>
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="G8" s="21" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="27" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B9" s="28" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C9" s="28"/>
-      <x:c r="D9" s="28"/>
-      <x:c r="E9" s="28"/>
-      <x:c r="F9" s="29" t="n">
-        <x:f>SUM(F4:F6)</x:f>
-        <x:v>159.2</x:v>
-      </x:c>
-      <x:c r="G9" s="28"/>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="27" t="str">
+      <x:c r="B11" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C11" s="28"/>
+      <x:c r="D11" s="28"/>
+      <x:c r="E11" s="28"/>
+      <x:c r="F11" s="29" t="n">
+        <x:f>SUM(F4:F8)</x:f>
+        <x:v>242.79999999999998</x:v>
+      </x:c>
+      <x:c r="G11" s="28"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="27" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B10" s="28"/>
-      <x:c r="C10" s="28"/>
-      <x:c r="D10" s="28"/>
-      <x:c r="E10" s="28"/>
-      <x:c r="F10" s="31" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(F4:F6),0),1)</x:f>
-        <x:v>53.1</x:v>
-      </x:c>
-      <x:c r="G10" s="28"/>
+      <x:c r="B12" s="28"/>
+      <x:c r="C12" s="28"/>
+      <x:c r="D12" s="28"/>
+      <x:c r="E12" s="28"/>
+      <x:c r="F12" s="31" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(F4:F8),0),1)</x:f>
+        <x:v>48.6</x:v>
+      </x:c>
+      <x:c r="G12" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Add open close and daily pct columns
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R2cf5cebb27ab4e28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="2" r:id="R60d95cb8c52149ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="3" r:id="Rb881b96f2fd14a82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="4" r:id="R8ed9804b104845d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="5" r:id="Ra40c569daa604403"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="6" r:id="Ref60e8e650624f60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="7" r:id="R4c577a5cc44a471e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="8" r:id="Rc5f11a3f1d1247b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rb14655d492dd4e41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="2" r:id="R63665d8505b54c0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="3" r:id="R2a3b94c57eb44308"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="4" r:id="Rc28ddba8238045d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="5" r:id="Rb1f571463aa24452"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="6" r:id="R05d5c033756346d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="7" r:id="Rdabfcbebac744bfe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="8" r:id="R103bacfe40af47be"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20,8 +20,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="2">
     <x:numFmt numFmtId="200" formatCode="General"/>
+    <x:numFmt numFmtId="201" formatCode="0.0%"/>
   </x:numFmts>
   <x:fonts count="7">
     <x:font>
@@ -125,7 +126,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="32">
+  <x:cellXfs count="33">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -171,6 +172,9 @@
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="5" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -776,7 +780,10 @@
     <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
@@ -795,15 +802,24 @@
         <x:v>日期</x:v>
       </x:c>
       <x:c r="D3" s="18" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="E3" s="18" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E3" s="18" t="str">
+      <x:c r="F3" s="18" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F3" s="18" t="str">
+      <x:c r="G3" s="18" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="H3" s="18" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I3" s="18" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="G3" s="18" t="str">
+      <x:c r="J3" s="18" t="str">
         <x:v>标的</x:v>
       </x:c>
     </x:row>
@@ -818,16 +834,25 @@
         <x:v>7月1日</x:v>
       </x:c>
       <x:c r="D4" s="22" t="n">
+        <x:v>8827.47</x:v>
+      </x:c>
+      <x:c r="E4" s="22" t="n">
         <x:v>8944.195</x:v>
       </x:c>
-      <x:c r="E4" s="22" t="n">
+      <x:c r="F4" s="22" t="n">
         <x:v>8806.646</x:v>
       </x:c>
-      <x:c r="F4" s="22" t="n">
-        <x:f>ROUND(D4-E4,1)</x:f>
+      <x:c r="G4" s="22" t="n">
+        <x:v>8876.63</x:v>
+      </x:c>
+      <x:c r="H4" s="23" t="n">
+        <x:v>0.007587471477740637</x:v>
+      </x:c>
+      <x:c r="I4" s="22" t="n">
+        <x:f>ROUND(E4-F4,1)</x:f>
         <x:v>137.5</x:v>
       </x:c>
-      <x:c r="G4" s="21" t="str">
+      <x:c r="J4" s="21" t="str">
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
@@ -842,16 +867,25 @@
         <x:v>7月2日</x:v>
       </x:c>
       <x:c r="D5" s="22" t="n">
+        <x:v>8688.291</x:v>
+      </x:c>
+      <x:c r="E5" s="22" t="n">
         <x:v>8865.966</x:v>
       </x:c>
-      <x:c r="E5" s="22" t="n">
+      <x:c r="F5" s="22" t="n">
         <x:v>8598.869</x:v>
       </x:c>
-      <x:c r="F5" s="24" t="n">
-        <x:f>ROUND(D5-E5,1)</x:f>
+      <x:c r="G5" s="22" t="n">
+        <x:v>8625.334</x:v>
+      </x:c>
+      <x:c r="H5" s="23" t="n">
+        <x:v>-0.02830984281196791</x:v>
+      </x:c>
+      <x:c r="I5" s="25" t="n">
+        <x:f>ROUND(E5-F5,1)</x:f>
         <x:v>267.1</x:v>
       </x:c>
-      <x:c r="G5" s="21" t="str">
+      <x:c r="J5" s="21" t="str">
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
@@ -866,16 +900,25 @@
         <x:v>7月3日</x:v>
       </x:c>
       <x:c r="D6" s="22" t="n">
+        <x:v>8627.382</x:v>
+      </x:c>
+      <x:c r="E6" s="22" t="n">
         <x:v>8740.668</x:v>
       </x:c>
-      <x:c r="E6" s="22" t="n">
+      <x:c r="F6" s="22" t="n">
         <x:v>8559.285</x:v>
       </x:c>
-      <x:c r="F6" s="24" t="n">
-        <x:f>ROUND(D6-E6,1)</x:f>
+      <x:c r="G6" s="22" t="n">
+        <x:v>8620.789</x:v>
+      </x:c>
+      <x:c r="H6" s="23" t="n">
+        <x:v>-0.0005269361163289243</x:v>
+      </x:c>
+      <x:c r="I6" s="25" t="n">
+        <x:f>ROUND(E6-F6,1)</x:f>
         <x:v>181.4</x:v>
       </x:c>
-      <x:c r="G6" s="21" t="str">
+      <x:c r="J6" s="21" t="str">
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
@@ -890,16 +933,25 @@
         <x:v>7月6日</x:v>
       </x:c>
       <x:c r="D7" s="22" t="n">
+        <x:v>8669.123</x:v>
+      </x:c>
+      <x:c r="E7" s="22" t="n">
         <x:v>8694.805</x:v>
       </x:c>
-      <x:c r="E7" s="22" t="n">
+      <x:c r="F7" s="22" t="n">
         <x:v>8432.897</x:v>
       </x:c>
-      <x:c r="F7" s="24" t="n">
-        <x:f>ROUND(D7-E7,1)</x:f>
+      <x:c r="G7" s="22" t="n">
+        <x:v>8472.603</x:v>
+      </x:c>
+      <x:c r="H7" s="23" t="n">
+        <x:v>-0.01718937790960917</x:v>
+      </x:c>
+      <x:c r="I7" s="25" t="n">
+        <x:f>ROUND(E7-F7,1)</x:f>
         <x:v>261.9</x:v>
       </x:c>
-      <x:c r="G7" s="21" t="str">
+      <x:c r="J7" s="21" t="str">
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
@@ -914,52 +966,67 @@
         <x:v>7月7日</x:v>
       </x:c>
       <x:c r="D8" s="22" t="n">
+        <x:v>8436.389</x:v>
+      </x:c>
+      <x:c r="E8" s="22" t="n">
         <x:v>8489.476</x:v>
       </x:c>
-      <x:c r="E8" s="22" t="n">
+      <x:c r="F8" s="22" t="n">
         <x:v>8261.398</x:v>
       </x:c>
-      <x:c r="F8" s="24" t="n">
-        <x:f>ROUND(D8-E8,1)</x:f>
+      <x:c r="G8" s="22" t="n">
+        <x:v>8301.804</x:v>
+      </x:c>
+      <x:c r="H8" s="23" t="n">
+        <x:v>-0.02015897593691085</x:v>
+      </x:c>
+      <x:c r="I8" s="25" t="n">
+        <x:f>ROUND(E8-F8,1)</x:f>
         <x:v>228.1</x:v>
       </x:c>
-      <x:c r="G8" s="21" t="str">
+      <x:c r="J8" s="21" t="str">
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="27" t="str">
+      <x:c r="A11" s="28" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B11" s="28" t="n">
+      <x:c r="B11" s="29" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C11" s="28"/>
-      <x:c r="D11" s="28"/>
-      <x:c r="E11" s="28"/>
-      <x:c r="F11" s="29" t="n">
-        <x:f>SUM(F4:F8)</x:f>
+      <x:c r="C11" s="29"/>
+      <x:c r="D11" s="29"/>
+      <x:c r="E11" s="29"/>
+      <x:c r="F11" s="29"/>
+      <x:c r="G11" s="29"/>
+      <x:c r="H11" s="29"/>
+      <x:c r="I11" s="30" t="n">
+        <x:f>SUM(I4:I8)</x:f>
         <x:v>1076</x:v>
       </x:c>
-      <x:c r="G11" s="28"/>
+      <x:c r="J11" s="29"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="27" t="str">
+      <x:c r="A12" s="28" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B12" s="28"/>
-      <x:c r="C12" s="28"/>
-      <x:c r="D12" s="28"/>
-      <x:c r="E12" s="28"/>
-      <x:c r="F12" s="31" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(F4:F8),0),1)</x:f>
+      <x:c r="B12" s="29"/>
+      <x:c r="C12" s="29"/>
+      <x:c r="D12" s="29"/>
+      <x:c r="E12" s="29"/>
+      <x:c r="F12" s="29"/>
+      <x:c r="G12" s="29"/>
+      <x:c r="H12" s="29"/>
+      <x:c r="I12" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I4:I8),0),1)</x:f>
         <x:v>215.2</x:v>
       </x:c>
-      <x:c r="G12" s="28"/>
+      <x:c r="J12" s="29"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:G1"/>
+    <x:mergeCell ref="A1:J1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -975,7 +1042,10 @@
     <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
@@ -994,15 +1064,24 @@
         <x:v>日期</x:v>
       </x:c>
       <x:c r="D3" s="18" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="E3" s="18" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E3" s="18" t="str">
+      <x:c r="F3" s="18" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F3" s="18" t="str">
+      <x:c r="G3" s="18" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="H3" s="18" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I3" s="18" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="G3" s="18" t="str">
+      <x:c r="J3" s="18" t="str">
         <x:v>标的</x:v>
       </x:c>
     </x:row>
@@ -1017,16 +1096,25 @@
         <x:v>7月1日</x:v>
       </x:c>
       <x:c r="D4" s="22" t="n">
+        <x:v>9052.043</x:v>
+      </x:c>
+      <x:c r="E4" s="22" t="n">
         <x:v>9147.559</x:v>
       </x:c>
-      <x:c r="E4" s="22" t="n">
+      <x:c r="F4" s="22" t="n">
         <x:v>8956.185</x:v>
       </x:c>
-      <x:c r="F4" s="24" t="n">
-        <x:f>ROUND(D4-E4,1)</x:f>
+      <x:c r="G4" s="22" t="n">
+        <x:v>9028.933</x:v>
+      </x:c>
+      <x:c r="H4" s="23" t="n">
+        <x:v>-0.0002708335017277408</x:v>
+      </x:c>
+      <x:c r="I4" s="25" t="n">
+        <x:f>ROUND(E4-F4,1)</x:f>
         <x:v>191.4</x:v>
       </x:c>
-      <x:c r="G4" s="21" t="str">
+      <x:c r="J4" s="21" t="str">
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
@@ -1041,16 +1129,25 @@
         <x:v>7月2日</x:v>
       </x:c>
       <x:c r="D5" s="22" t="n">
+        <x:v>8829.621</x:v>
+      </x:c>
+      <x:c r="E5" s="22" t="n">
         <x:v>8932.647</x:v>
       </x:c>
-      <x:c r="E5" s="22" t="n">
+      <x:c r="F5" s="22" t="n">
         <x:v>8667.419</x:v>
       </x:c>
-      <x:c r="F5" s="24" t="n">
-        <x:f>ROUND(D5-E5,1)</x:f>
+      <x:c r="G5" s="22" t="n">
+        <x:v>8694.176</x:v>
+      </x:c>
+      <x:c r="H5" s="23" t="n">
+        <x:v>-0.03707603102160595</x:v>
+      </x:c>
+      <x:c r="I5" s="25" t="n">
+        <x:f>ROUND(E5-F5,1)</x:f>
         <x:v>265.2</x:v>
       </x:c>
-      <x:c r="G5" s="21" t="str">
+      <x:c r="J5" s="21" t="str">
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
@@ -1065,16 +1162,25 @@
         <x:v>7月3日</x:v>
       </x:c>
       <x:c r="D6" s="22" t="n">
+        <x:v>8702.327</x:v>
+      </x:c>
+      <x:c r="E6" s="22" t="n">
         <x:v>8860.416</x:v>
       </x:c>
-      <x:c r="E6" s="22" t="n">
+      <x:c r="F6" s="22" t="n">
         <x:v>8636.15</x:v>
       </x:c>
-      <x:c r="F6" s="24" t="n">
-        <x:f>ROUND(D6-E6,1)</x:f>
+      <x:c r="G6" s="22" t="n">
+        <x:v>8745.261</x:v>
+      </x:c>
+      <x:c r="H6" s="23" t="n">
+        <x:v>0.00587577247113491</x:v>
+      </x:c>
+      <x:c r="I6" s="25" t="n">
+        <x:f>ROUND(E6-F6,1)</x:f>
         <x:v>224.3</x:v>
       </x:c>
-      <x:c r="G6" s="21" t="str">
+      <x:c r="J6" s="21" t="str">
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
@@ -1089,16 +1195,25 @@
         <x:v>7月6日</x:v>
       </x:c>
       <x:c r="D7" s="22" t="n">
+        <x:v>8790.967</x:v>
+      </x:c>
+      <x:c r="E7" s="22" t="n">
         <x:v>8823.05</x:v>
       </x:c>
-      <x:c r="E7" s="22" t="n">
+      <x:c r="F7" s="22" t="n">
         <x:v>8570.892</x:v>
       </x:c>
-      <x:c r="F7" s="24" t="n">
-        <x:f>ROUND(D7-E7,1)</x:f>
+      <x:c r="G7" s="22" t="n">
+        <x:v>8651.134</x:v>
+      </x:c>
+      <x:c r="H7" s="23" t="n">
+        <x:v>-0.01076320077811288</x:v>
+      </x:c>
+      <x:c r="I7" s="25" t="n">
+        <x:f>ROUND(E7-F7,1)</x:f>
         <x:v>252.2</x:v>
       </x:c>
-      <x:c r="G7" s="21" t="str">
+      <x:c r="J7" s="21" t="str">
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
@@ -1113,52 +1228,67 @@
         <x:v>7月7日</x:v>
       </x:c>
       <x:c r="D8" s="22" t="n">
+        <x:v>8604.076</x:v>
+      </x:c>
+      <x:c r="E8" s="22" t="n">
         <x:v>8663.665</x:v>
       </x:c>
-      <x:c r="E8" s="22" t="n">
+      <x:c r="F8" s="22" t="n">
         <x:v>8457.576</x:v>
       </x:c>
-      <x:c r="F8" s="24" t="n">
-        <x:f>ROUND(D8-E8,1)</x:f>
+      <x:c r="G8" s="22" t="n">
+        <x:v>8508.789</x:v>
+      </x:c>
+      <x:c r="H8" s="23" t="n">
+        <x:v>-0.01645391228479398</x:v>
+      </x:c>
+      <x:c r="I8" s="25" t="n">
+        <x:f>ROUND(E8-F8,1)</x:f>
         <x:v>206.1</x:v>
       </x:c>
-      <x:c r="G8" s="21" t="str">
+      <x:c r="J8" s="21" t="str">
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="27" t="str">
+      <x:c r="A11" s="28" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B11" s="28" t="n">
+      <x:c r="B11" s="29" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C11" s="28"/>
-      <x:c r="D11" s="28"/>
-      <x:c r="E11" s="28"/>
-      <x:c r="F11" s="29" t="n">
-        <x:f>SUM(F4:F8)</x:f>
+      <x:c r="C11" s="29"/>
+      <x:c r="D11" s="29"/>
+      <x:c r="E11" s="29"/>
+      <x:c r="F11" s="29"/>
+      <x:c r="G11" s="29"/>
+      <x:c r="H11" s="29"/>
+      <x:c r="I11" s="30" t="n">
+        <x:f>SUM(I4:I8)</x:f>
         <x:v>1139.2</x:v>
       </x:c>
-      <x:c r="G11" s="28"/>
+      <x:c r="J11" s="29"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="27" t="str">
+      <x:c r="A12" s="28" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B12" s="28"/>
-      <x:c r="C12" s="28"/>
-      <x:c r="D12" s="28"/>
-      <x:c r="E12" s="28"/>
-      <x:c r="F12" s="31" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(F4:F8),0),1)</x:f>
+      <x:c r="B12" s="29"/>
+      <x:c r="C12" s="29"/>
+      <x:c r="D12" s="29"/>
+      <x:c r="E12" s="29"/>
+      <x:c r="F12" s="29"/>
+      <x:c r="G12" s="29"/>
+      <x:c r="H12" s="29"/>
+      <x:c r="I12" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I4:I8),0),1)</x:f>
         <x:v>227.8</x:v>
       </x:c>
-      <x:c r="G12" s="28"/>
+      <x:c r="J12" s="29"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:G1"/>
+    <x:mergeCell ref="A1:J1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1174,7 +1304,10 @@
     <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
@@ -1193,15 +1326,24 @@
         <x:v>日期</x:v>
       </x:c>
       <x:c r="D3" s="18" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="E3" s="18" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E3" s="18" t="str">
+      <x:c r="F3" s="18" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F3" s="18" t="str">
+      <x:c r="G3" s="18" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="H3" s="18" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I3" s="18" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="G3" s="18" t="str">
+      <x:c r="J3" s="18" t="str">
         <x:v>标的</x:v>
       </x:c>
     </x:row>
@@ -1216,16 +1358,25 @@
         <x:v>7月1日</x:v>
       </x:c>
       <x:c r="D4" s="22" t="n">
+        <x:v>4090.76</x:v>
+      </x:c>
+      <x:c r="E4" s="22" t="n">
         <x:v>4143.314</x:v>
       </x:c>
-      <x:c r="E4" s="22" t="n">
+      <x:c r="F4" s="22" t="n">
         <x:v>4087.535</x:v>
       </x:c>
-      <x:c r="F4" s="24" t="n">
-        <x:f>ROUND(D4-E4,1)</x:f>
+      <x:c r="G4" s="22" t="n">
+        <x:v>4112.445</x:v>
+      </x:c>
+      <x:c r="H4" s="23" t="n">
+        <x:v>0.004407975093768224</x:v>
+      </x:c>
+      <x:c r="I4" s="25" t="n">
+        <x:f>ROUND(E4-F4,1)</x:f>
         <x:v>55.8</x:v>
       </x:c>
-      <x:c r="G4" s="21" t="str">
+      <x:c r="J4" s="21" t="str">
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
@@ -1240,16 +1391,25 @@
         <x:v>7月2日</x:v>
       </x:c>
       <x:c r="D5" s="22" t="n">
+        <x:v>4054.086</x:v>
+      </x:c>
+      <x:c r="E5" s="22" t="n">
         <x:v>4093.678</x:v>
       </x:c>
-      <x:c r="E5" s="22" t="n">
+      <x:c r="F5" s="22" t="n">
         <x:v>4019.215</x:v>
       </x:c>
-      <x:c r="F5" s="24" t="n">
-        <x:f>ROUND(D5-E5,1)</x:f>
+      <x:c r="G5" s="22" t="n">
+        <x:v>4028.904</x:v>
+      </x:c>
+      <x:c r="H5" s="23" t="n">
+        <x:v>-0.020314192651816554</x:v>
+      </x:c>
+      <x:c r="I5" s="25" t="n">
+        <x:f>ROUND(E5-F5,1)</x:f>
         <x:v>74.5</x:v>
       </x:c>
-      <x:c r="G5" s="21" t="str">
+      <x:c r="J5" s="21" t="str">
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
@@ -1264,16 +1424,25 @@
         <x:v>7月3日</x:v>
       </x:c>
       <x:c r="D6" s="22" t="n">
+        <x:v>4031.335</x:v>
+      </x:c>
+      <x:c r="E6" s="22" t="n">
         <x:v>4073.88</x:v>
       </x:c>
-      <x:c r="E6" s="22" t="n">
+      <x:c r="F6" s="22" t="n">
         <x:v>4027.255</x:v>
       </x:c>
-      <x:c r="F6" s="22" t="n">
-        <x:f>ROUND(D6-E6,1)</x:f>
+      <x:c r="G6" s="22" t="n">
+        <x:v>4043.643</x:v>
+      </x:c>
+      <x:c r="H6" s="23" t="n">
+        <x:v>0.0036583150156965782</x:v>
+      </x:c>
+      <x:c r="I6" s="22" t="n">
+        <x:f>ROUND(E6-F6,1)</x:f>
         <x:v>46.6</x:v>
       </x:c>
-      <x:c r="G6" s="21" t="str">
+      <x:c r="J6" s="21" t="str">
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
@@ -1288,16 +1457,25 @@
         <x:v>7月6日</x:v>
       </x:c>
       <x:c r="D7" s="22" t="n">
+        <x:v>4059.194</x:v>
+      </x:c>
+      <x:c r="E7" s="22" t="n">
         <x:v>4060.069</x:v>
       </x:c>
-      <x:c r="E7" s="22" t="n">
+      <x:c r="F7" s="22" t="n">
         <x:v>4005.414</x:v>
       </x:c>
-      <x:c r="F7" s="24" t="n">
-        <x:f>ROUND(D7-E7,1)</x:f>
+      <x:c r="G7" s="22" t="n">
+        <x:v>4041.238</x:v>
+      </x:c>
+      <x:c r="H7" s="23" t="n">
+        <x:v>-0.000594760714533904</x:v>
+      </x:c>
+      <x:c r="I7" s="25" t="n">
+        <x:f>ROUND(E7-F7,1)</x:f>
         <x:v>54.7</x:v>
       </x:c>
-      <x:c r="G7" s="21" t="str">
+      <x:c r="J7" s="21" t="str">
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
@@ -1312,52 +1490,67 @@
         <x:v>7月7日</x:v>
       </x:c>
       <x:c r="D8" s="22" t="n">
+        <x:v>4019.494</x:v>
+      </x:c>
+      <x:c r="E8" s="22" t="n">
         <x:v>4028.514</x:v>
       </x:c>
-      <x:c r="E8" s="22" t="n">
+      <x:c r="F8" s="22" t="n">
         <x:v>3971.713</x:v>
       </x:c>
-      <x:c r="F8" s="24" t="n">
-        <x:f>ROUND(D8-E8,1)</x:f>
+      <x:c r="G8" s="22" t="n">
+        <x:v>3990.235</x:v>
+      </x:c>
+      <x:c r="H8" s="23" t="n">
+        <x:v>-0.01262063753730902</x:v>
+      </x:c>
+      <x:c r="I8" s="25" t="n">
+        <x:f>ROUND(E8-F8,1)</x:f>
         <x:v>56.8</x:v>
       </x:c>
-      <x:c r="G8" s="21" t="str">
+      <x:c r="J8" s="21" t="str">
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="27" t="str">
+      <x:c r="A11" s="28" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B11" s="28" t="n">
+      <x:c r="B11" s="29" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C11" s="28"/>
-      <x:c r="D11" s="28"/>
-      <x:c r="E11" s="28"/>
-      <x:c r="F11" s="29" t="n">
-        <x:f>SUM(F4:F8)</x:f>
+      <x:c r="C11" s="29"/>
+      <x:c r="D11" s="29"/>
+      <x:c r="E11" s="29"/>
+      <x:c r="F11" s="29"/>
+      <x:c r="G11" s="29"/>
+      <x:c r="H11" s="29"/>
+      <x:c r="I11" s="30" t="n">
+        <x:f>SUM(I4:I8)</x:f>
         <x:v>288.40000000000003</x:v>
       </x:c>
-      <x:c r="G11" s="28"/>
+      <x:c r="J11" s="29"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="27" t="str">
+      <x:c r="A12" s="28" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B12" s="28"/>
-      <x:c r="C12" s="28"/>
-      <x:c r="D12" s="28"/>
-      <x:c r="E12" s="28"/>
-      <x:c r="F12" s="31" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(F4:F8),0),1)</x:f>
+      <x:c r="B12" s="29"/>
+      <x:c r="C12" s="29"/>
+      <x:c r="D12" s="29"/>
+      <x:c r="E12" s="29"/>
+      <x:c r="F12" s="29"/>
+      <x:c r="G12" s="29"/>
+      <x:c r="H12" s="29"/>
+      <x:c r="I12" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I4:I8),0),1)</x:f>
         <x:v>57.7</x:v>
       </x:c>
-      <x:c r="G12" s="28"/>
+      <x:c r="J12" s="29"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:G1"/>
+    <x:mergeCell ref="A1:J1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1373,7 +1566,10 @@
     <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
@@ -1392,15 +1588,24 @@
         <x:v>日期</x:v>
       </x:c>
       <x:c r="D3" s="18" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="E3" s="18" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E3" s="18" t="str">
+      <x:c r="F3" s="18" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F3" s="18" t="str">
+      <x:c r="G3" s="18" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="H3" s="18" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I3" s="18" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="G3" s="18" t="str">
+      <x:c r="J3" s="18" t="str">
         <x:v>标的</x:v>
       </x:c>
     </x:row>
@@ -1415,16 +1620,25 @@
         <x:v>7月1日</x:v>
       </x:c>
       <x:c r="D4" s="22" t="n">
+        <x:v>8500</x:v>
+      </x:c>
+      <x:c r="E4" s="22" t="n">
         <x:v>8629</x:v>
       </x:c>
-      <x:c r="E4" s="22" t="n">
+      <x:c r="F4" s="22" t="n">
         <x:v>8480</x:v>
       </x:c>
-      <x:c r="F4" s="22" t="n">
-        <x:f>ROUND(D4-E4,1)</x:f>
+      <x:c r="G4" s="22" t="n">
+        <x:v>8517.6</x:v>
+      </x:c>
+      <x:c r="H4" s="23" t="n">
+        <x:v>0.00157569201100638</x:v>
+      </x:c>
+      <x:c r="I4" s="22" t="n">
+        <x:f>ROUND(E4-F4,1)</x:f>
         <x:v>149</x:v>
       </x:c>
-      <x:c r="G4" s="21" t="str">
+      <x:c r="J4" s="21" t="str">
         <x:v>IM2609</x:v>
       </x:c>
     </x:row>
@@ -1439,16 +1653,25 @@
         <x:v>7月2日</x:v>
       </x:c>
       <x:c r="D5" s="22" t="n">
+        <x:v>8475.4</x:v>
+      </x:c>
+      <x:c r="E5" s="22" t="n">
         <x:v>8556</x:v>
       </x:c>
-      <x:c r="E5" s="22" t="n">
+      <x:c r="F5" s="22" t="n">
         <x:v>8344</x:v>
       </x:c>
-      <x:c r="F5" s="24" t="n">
-        <x:f>ROUND(D5-E5,1)</x:f>
+      <x:c r="G5" s="22" t="n">
+        <x:v>8370.2</x:v>
+      </x:c>
+      <x:c r="H5" s="23" t="n">
+        <x:v>-0.017305344228421116</x:v>
+      </x:c>
+      <x:c r="I5" s="25" t="n">
+        <x:f>ROUND(E5-F5,1)</x:f>
         <x:v>212</x:v>
       </x:c>
-      <x:c r="G5" s="21" t="str">
+      <x:c r="J5" s="21" t="str">
         <x:v>IM2609</x:v>
       </x:c>
     </x:row>
@@ -1463,16 +1686,25 @@
         <x:v>7月3日</x:v>
       </x:c>
       <x:c r="D6" s="22" t="n">
+        <x:v>8401</x:v>
+      </x:c>
+      <x:c r="E6" s="22" t="n">
         <x:v>8475</x:v>
       </x:c>
-      <x:c r="E6" s="22" t="n">
+      <x:c r="F6" s="22" t="n">
         <x:v>8337.8</x:v>
       </x:c>
-      <x:c r="F6" s="22" t="n">
-        <x:f>ROUND(D6-E6,1)</x:f>
+      <x:c r="G6" s="22" t="n">
+        <x:v>8373</x:v>
+      </x:c>
+      <x:c r="H6" s="23" t="n">
+        <x:v>0.00033452008315215664</x:v>
+      </x:c>
+      <x:c r="I6" s="22" t="n">
+        <x:f>ROUND(E6-F6,1)</x:f>
         <x:v>137.2</x:v>
       </x:c>
-      <x:c r="G6" s="21" t="str">
+      <x:c r="J6" s="21" t="str">
         <x:v>IM2609</x:v>
       </x:c>
     </x:row>
@@ -1487,16 +1719,25 @@
         <x:v>7月6日</x:v>
       </x:c>
       <x:c r="D7" s="22" t="n">
+        <x:v>8403</x:v>
+      </x:c>
+      <x:c r="E7" s="22" t="n">
         <x:v>8419.8</x:v>
       </x:c>
-      <x:c r="E7" s="22" t="n">
+      <x:c r="F7" s="22" t="n">
         <x:v>8213</x:v>
       </x:c>
-      <x:c r="F7" s="24" t="n">
-        <x:f>ROUND(D7-E7,1)</x:f>
+      <x:c r="G7" s="22" t="n">
+        <x:v>8265</x:v>
+      </x:c>
+      <x:c r="H7" s="23" t="n">
+        <x:v>-0.012898602651379432</x:v>
+      </x:c>
+      <x:c r="I7" s="25" t="n">
+        <x:f>ROUND(E7-F7,1)</x:f>
         <x:v>206.8</x:v>
       </x:c>
-      <x:c r="G7" s="21" t="str">
+      <x:c r="J7" s="21" t="str">
         <x:v>IM2609</x:v>
       </x:c>
     </x:row>
@@ -1511,52 +1752,67 @@
         <x:v>7月7日</x:v>
       </x:c>
       <x:c r="D8" s="22" t="n">
+        <x:v>8235</x:v>
+      </x:c>
+      <x:c r="E8" s="22" t="n">
         <x:v>8274.2</x:v>
       </x:c>
-      <x:c r="E8" s="22" t="n">
+      <x:c r="F8" s="22" t="n">
         <x:v>8068.8</x:v>
       </x:c>
-      <x:c r="F8" s="24" t="n">
-        <x:f>ROUND(D8-E8,1)</x:f>
+      <x:c r="G8" s="22" t="n">
+        <x:v>8115.2</x:v>
+      </x:c>
+      <x:c r="H8" s="23" t="n">
+        <x:v>-0.018124621899576532</x:v>
+      </x:c>
+      <x:c r="I8" s="25" t="n">
+        <x:f>ROUND(E8-F8,1)</x:f>
         <x:v>205.4</x:v>
       </x:c>
-      <x:c r="G8" s="21" t="str">
+      <x:c r="J8" s="21" t="str">
         <x:v>IM2609</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="27" t="str">
+      <x:c r="A11" s="28" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B11" s="28" t="n">
+      <x:c r="B11" s="29" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C11" s="28"/>
-      <x:c r="D11" s="28"/>
-      <x:c r="E11" s="28"/>
-      <x:c r="F11" s="29" t="n">
-        <x:f>SUM(F4:F8)</x:f>
+      <x:c r="C11" s="29"/>
+      <x:c r="D11" s="29"/>
+      <x:c r="E11" s="29"/>
+      <x:c r="F11" s="29"/>
+      <x:c r="G11" s="29"/>
+      <x:c r="H11" s="29"/>
+      <x:c r="I11" s="30" t="n">
+        <x:f>SUM(I4:I8)</x:f>
         <x:v>910.4</x:v>
       </x:c>
-      <x:c r="G11" s="28"/>
+      <x:c r="J11" s="29"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="27" t="str">
+      <x:c r="A12" s="28" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B12" s="28"/>
-      <x:c r="C12" s="28"/>
-      <x:c r="D12" s="28"/>
-      <x:c r="E12" s="28"/>
-      <x:c r="F12" s="31" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(F4:F8),0),1)</x:f>
+      <x:c r="B12" s="29"/>
+      <x:c r="C12" s="29"/>
+      <x:c r="D12" s="29"/>
+      <x:c r="E12" s="29"/>
+      <x:c r="F12" s="29"/>
+      <x:c r="G12" s="29"/>
+      <x:c r="H12" s="29"/>
+      <x:c r="I12" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I4:I8),0),1)</x:f>
         <x:v>182.1</x:v>
       </x:c>
-      <x:c r="G12" s="28"/>
+      <x:c r="J12" s="29"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:G1"/>
+    <x:mergeCell ref="A1:J1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1572,7 +1828,10 @@
     <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
@@ -1591,15 +1850,24 @@
         <x:v>日期</x:v>
       </x:c>
       <x:c r="D3" s="18" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="E3" s="18" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E3" s="18" t="str">
+      <x:c r="F3" s="18" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F3" s="18" t="str">
+      <x:c r="G3" s="18" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="H3" s="18" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I3" s="18" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="G3" s="18" t="str">
+      <x:c r="J3" s="18" t="str">
         <x:v>标的</x:v>
       </x:c>
     </x:row>
@@ -1614,16 +1882,25 @@
         <x:v>7月1日</x:v>
       </x:c>
       <x:c r="D4" s="22" t="n">
+        <x:v>8763</x:v>
+      </x:c>
+      <x:c r="E4" s="22" t="n">
         <x:v>8873.8</x:v>
       </x:c>
-      <x:c r="E4" s="22" t="n">
+      <x:c r="F4" s="22" t="n">
         <x:v>8656.8</x:v>
       </x:c>
-      <x:c r="F4" s="24" t="n">
-        <x:f>ROUND(D4-E4,1)</x:f>
+      <x:c r="G4" s="22" t="n">
+        <x:v>8713</x:v>
+      </x:c>
+      <x:c r="H4" s="23" t="n">
+        <x:v>-0.007969941933280156</x:v>
+      </x:c>
+      <x:c r="I4" s="25" t="n">
+        <x:f>ROUND(E4-F4,1)</x:f>
         <x:v>217</x:v>
       </x:c>
-      <x:c r="G4" s="21" t="str">
+      <x:c r="J4" s="21" t="str">
         <x:v>IC2609</x:v>
       </x:c>
     </x:row>
@@ -1638,16 +1915,25 @@
         <x:v>7月2日</x:v>
       </x:c>
       <x:c r="D5" s="22" t="n">
+        <x:v>8616</x:v>
+      </x:c>
+      <x:c r="E5" s="22" t="n">
         <x:v>8678.6</x:v>
       </x:c>
-      <x:c r="E5" s="22" t="n">
+      <x:c r="F5" s="22" t="n">
         <x:v>8456.8</x:v>
       </x:c>
-      <x:c r="F5" s="24" t="n">
-        <x:f>ROUND(D5-E5,1)</x:f>
+      <x:c r="G5" s="22" t="n">
+        <x:v>8488</x:v>
+      </x:c>
+      <x:c r="H5" s="23" t="n">
+        <x:v>-0.025823482153104593</x:v>
+      </x:c>
+      <x:c r="I5" s="25" t="n">
+        <x:f>ROUND(E5-F5,1)</x:f>
         <x:v>221.8</x:v>
       </x:c>
-      <x:c r="G5" s="21" t="str">
+      <x:c r="J5" s="21" t="str">
         <x:v>IC2609</x:v>
       </x:c>
     </x:row>
@@ -1662,16 +1948,25 @@
         <x:v>7月3日</x:v>
       </x:c>
       <x:c r="D6" s="22" t="n">
+        <x:v>8519</x:v>
+      </x:c>
+      <x:c r="E6" s="22" t="n">
         <x:v>8650</x:v>
       </x:c>
-      <x:c r="E6" s="22" t="n">
+      <x:c r="F6" s="22" t="n">
         <x:v>8442</x:v>
       </x:c>
-      <x:c r="F6" s="24" t="n">
-        <x:f>ROUND(D6-E6,1)</x:f>
+      <x:c r="G6" s="22" t="n">
+        <x:v>8538</x:v>
+      </x:c>
+      <x:c r="H6" s="23" t="n">
+        <x:v>0.005890669180018904</x:v>
+      </x:c>
+      <x:c r="I6" s="25" t="n">
+        <x:f>ROUND(E6-F6,1)</x:f>
         <x:v>208</x:v>
       </x:c>
-      <x:c r="G6" s="21" t="str">
+      <x:c r="J6" s="21" t="str">
         <x:v>IC2609</x:v>
       </x:c>
     </x:row>
@@ -1686,16 +1981,25 @@
         <x:v>7月6日</x:v>
       </x:c>
       <x:c r="D7" s="22" t="n">
+        <x:v>8574.4</x:v>
+      </x:c>
+      <x:c r="E7" s="22" t="n">
         <x:v>8584.2</x:v>
       </x:c>
-      <x:c r="E7" s="22" t="n">
+      <x:c r="F7" s="22" t="n">
         <x:v>8376</x:v>
       </x:c>
-      <x:c r="F7" s="24" t="n">
-        <x:f>ROUND(D7-E7,1)</x:f>
+      <x:c r="G7" s="22" t="n">
+        <x:v>8467</x:v>
+      </x:c>
+      <x:c r="H7" s="23" t="n">
+        <x:v>-0.008315764816116178</x:v>
+      </x:c>
+      <x:c r="I7" s="25" t="n">
+        <x:f>ROUND(E7-F7,1)</x:f>
         <x:v>208.2</x:v>
       </x:c>
-      <x:c r="G7" s="21" t="str">
+      <x:c r="J7" s="21" t="str">
         <x:v>IC2609</x:v>
       </x:c>
     </x:row>
@@ -1710,52 +2014,67 @@
         <x:v>7月7日</x:v>
       </x:c>
       <x:c r="D8" s="22" t="n">
+        <x:v>8420</x:v>
+      </x:c>
+      <x:c r="E8" s="22" t="n">
         <x:v>8478.8</x:v>
       </x:c>
-      <x:c r="E8" s="22" t="n">
+      <x:c r="F8" s="22" t="n">
         <x:v>8281</x:v>
       </x:c>
-      <x:c r="F8" s="24" t="n">
-        <x:f>ROUND(D8-E8,1)</x:f>
+      <x:c r="G8" s="22" t="n">
+        <x:v>8322.6</x:v>
+      </x:c>
+      <x:c r="H8" s="23" t="n">
+        <x:v>-0.01705444667532774</x:v>
+      </x:c>
+      <x:c r="I8" s="25" t="n">
+        <x:f>ROUND(E8-F8,1)</x:f>
         <x:v>197.8</x:v>
       </x:c>
-      <x:c r="G8" s="21" t="str">
+      <x:c r="J8" s="21" t="str">
         <x:v>IC2609</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="27" t="str">
+      <x:c r="A11" s="28" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B11" s="28" t="n">
+      <x:c r="B11" s="29" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C11" s="28"/>
-      <x:c r="D11" s="28"/>
-      <x:c r="E11" s="28"/>
-      <x:c r="F11" s="29" t="n">
-        <x:f>SUM(F4:F8)</x:f>
+      <x:c r="C11" s="29"/>
+      <x:c r="D11" s="29"/>
+      <x:c r="E11" s="29"/>
+      <x:c r="F11" s="29"/>
+      <x:c r="G11" s="29"/>
+      <x:c r="H11" s="29"/>
+      <x:c r="I11" s="30" t="n">
+        <x:f>SUM(I4:I8)</x:f>
         <x:v>1052.8</x:v>
       </x:c>
-      <x:c r="G11" s="28"/>
+      <x:c r="J11" s="29"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="27" t="str">
+      <x:c r="A12" s="28" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B12" s="28"/>
-      <x:c r="C12" s="28"/>
-      <x:c r="D12" s="28"/>
-      <x:c r="E12" s="28"/>
-      <x:c r="F12" s="31" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(F4:F8),0),1)</x:f>
+      <x:c r="B12" s="29"/>
+      <x:c r="C12" s="29"/>
+      <x:c r="D12" s="29"/>
+      <x:c r="E12" s="29"/>
+      <x:c r="F12" s="29"/>
+      <x:c r="G12" s="29"/>
+      <x:c r="H12" s="29"/>
+      <x:c r="I12" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I4:I8),0),1)</x:f>
         <x:v>210.6</x:v>
       </x:c>
-      <x:c r="G12" s="28"/>
+      <x:c r="J12" s="29"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:G1"/>
+    <x:mergeCell ref="A1:J1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1771,7 +2090,10 @@
     <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
@@ -1790,15 +2112,24 @@
         <x:v>日期</x:v>
       </x:c>
       <x:c r="D3" s="18" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="E3" s="18" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E3" s="18" t="str">
+      <x:c r="F3" s="18" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F3" s="18" t="str">
+      <x:c r="G3" s="18" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="H3" s="18" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I3" s="18" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="G3" s="18" t="str">
+      <x:c r="J3" s="18" t="str">
         <x:v>标的</x:v>
       </x:c>
     </x:row>
@@ -1813,16 +2144,25 @@
         <x:v>7月1日</x:v>
       </x:c>
       <x:c r="D4" s="22" t="n">
+        <x:v>4855.8</x:v>
+      </x:c>
+      <x:c r="E4" s="22" t="n">
         <x:v>4899.6</x:v>
       </x:c>
-      <x:c r="E4" s="22" t="n">
+      <x:c r="F4" s="22" t="n">
         <x:v>4802.2</x:v>
       </x:c>
-      <x:c r="F4" s="24" t="n">
-        <x:f>ROUND(D4-E4,1)</x:f>
+      <x:c r="G4" s="22" t="n">
+        <x:v>4831.2</x:v>
+      </x:c>
+      <x:c r="H4" s="23" t="n">
+        <x:v>-0.0050661065118003945</x:v>
+      </x:c>
+      <x:c r="I4" s="25" t="n">
+        <x:f>ROUND(E4-F4,1)</x:f>
         <x:v>97.4</x:v>
       </x:c>
-      <x:c r="G4" s="21" t="str">
+      <x:c r="J4" s="21" t="str">
         <x:v>IF2609</x:v>
       </x:c>
     </x:row>
@@ -1837,16 +2177,25 @@
         <x:v>7月2日</x:v>
       </x:c>
       <x:c r="D5" s="22" t="n">
+        <x:v>4769</x:v>
+      </x:c>
+      <x:c r="E5" s="22" t="n">
         <x:v>4800.2</x:v>
       </x:c>
-      <x:c r="E5" s="22" t="n">
+      <x:c r="F5" s="22" t="n">
         <x:v>4705</x:v>
       </x:c>
-      <x:c r="F5" s="24" t="n">
-        <x:f>ROUND(D5-E5,1)</x:f>
+      <x:c r="G5" s="22" t="n">
+        <x:v>4719.4</x:v>
+      </x:c>
+      <x:c r="H5" s="23" t="n">
+        <x:v>-0.02314124855108468</x:v>
+      </x:c>
+      <x:c r="I5" s="25" t="n">
+        <x:f>ROUND(E5-F5,1)</x:f>
         <x:v>95.2</x:v>
       </x:c>
-      <x:c r="G5" s="21" t="str">
+      <x:c r="J5" s="21" t="str">
         <x:v>IF2609</x:v>
       </x:c>
     </x:row>
@@ -1861,16 +2210,25 @@
         <x:v>7月3日</x:v>
       </x:c>
       <x:c r="D6" s="22" t="n">
+        <x:v>4733.8</x:v>
+      </x:c>
+      <x:c r="E6" s="22" t="n">
         <x:v>4810.4</x:v>
       </x:c>
-      <x:c r="E6" s="22" t="n">
+      <x:c r="F6" s="22" t="n">
         <x:v>4728</x:v>
       </x:c>
-      <x:c r="F6" s="22" t="n">
-        <x:f>ROUND(D6-E6,1)</x:f>
+      <x:c r="G6" s="22" t="n">
+        <x:v>4752.2</x:v>
+      </x:c>
+      <x:c r="H6" s="23" t="n">
+        <x:v>0.006950036021528216</x:v>
+      </x:c>
+      <x:c r="I6" s="22" t="n">
+        <x:f>ROUND(E6-F6,1)</x:f>
         <x:v>82.4</x:v>
       </x:c>
-      <x:c r="G6" s="21" t="str">
+      <x:c r="J6" s="21" t="str">
         <x:v>IF2609</x:v>
       </x:c>
     </x:row>
@@ -1885,16 +2243,25 @@
         <x:v>7月6日</x:v>
       </x:c>
       <x:c r="D7" s="22" t="n">
+        <x:v>4781</x:v>
+      </x:c>
+      <x:c r="E7" s="22" t="n">
         <x:v>4781.2</x:v>
       </x:c>
-      <x:c r="E7" s="22" t="n">
+      <x:c r="F7" s="22" t="n">
         <x:v>4701</x:v>
       </x:c>
-      <x:c r="F7" s="22" t="n">
-        <x:f>ROUND(D7-E7,1)</x:f>
+      <x:c r="G7" s="22" t="n">
+        <x:v>4753.2</x:v>
+      </x:c>
+      <x:c r="H7" s="23" t="n">
+        <x:v>0.00021042885400435196</x:v>
+      </x:c>
+      <x:c r="I7" s="22" t="n">
+        <x:f>ROUND(E7-F7,1)</x:f>
         <x:v>80.2</x:v>
       </x:c>
-      <x:c r="G7" s="21" t="str">
+      <x:c r="J7" s="21" t="str">
         <x:v>IF2609</x:v>
       </x:c>
     </x:row>
@@ -1909,52 +2276,67 @@
         <x:v>7月7日</x:v>
       </x:c>
       <x:c r="D8" s="22" t="n">
+        <x:v>4725.6</x:v>
+      </x:c>
+      <x:c r="E8" s="22" t="n">
         <x:v>4752.6</x:v>
       </x:c>
-      <x:c r="E8" s="22" t="n">
+      <x:c r="F8" s="22" t="n">
         <x:v>4671.4</x:v>
       </x:c>
-      <x:c r="F8" s="22" t="n">
-        <x:f>ROUND(D8-E8,1)</x:f>
+      <x:c r="G8" s="22" t="n">
+        <x:v>4703.4</x:v>
+      </x:c>
+      <x:c r="H8" s="23" t="n">
+        <x:v>-0.01047715223428436</x:v>
+      </x:c>
+      <x:c r="I8" s="22" t="n">
+        <x:f>ROUND(E8-F8,1)</x:f>
         <x:v>81.2</x:v>
       </x:c>
-      <x:c r="G8" s="21" t="str">
+      <x:c r="J8" s="21" t="str">
         <x:v>IF2609</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="27" t="str">
+      <x:c r="A11" s="28" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B11" s="28" t="n">
+      <x:c r="B11" s="29" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C11" s="28"/>
-      <x:c r="D11" s="28"/>
-      <x:c r="E11" s="28"/>
-      <x:c r="F11" s="29" t="n">
-        <x:f>SUM(F4:F8)</x:f>
+      <x:c r="C11" s="29"/>
+      <x:c r="D11" s="29"/>
+      <x:c r="E11" s="29"/>
+      <x:c r="F11" s="29"/>
+      <x:c r="G11" s="29"/>
+      <x:c r="H11" s="29"/>
+      <x:c r="I11" s="30" t="n">
+        <x:f>SUM(I4:I8)</x:f>
         <x:v>436.4</x:v>
       </x:c>
-      <x:c r="G11" s="28"/>
+      <x:c r="J11" s="29"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="27" t="str">
+      <x:c r="A12" s="28" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B12" s="28"/>
-      <x:c r="C12" s="28"/>
-      <x:c r="D12" s="28"/>
-      <x:c r="E12" s="28"/>
-      <x:c r="F12" s="31" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(F4:F8),0),1)</x:f>
+      <x:c r="B12" s="29"/>
+      <x:c r="C12" s="29"/>
+      <x:c r="D12" s="29"/>
+      <x:c r="E12" s="29"/>
+      <x:c r="F12" s="29"/>
+      <x:c r="G12" s="29"/>
+      <x:c r="H12" s="29"/>
+      <x:c r="I12" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I4:I8),0),1)</x:f>
         <x:v>87.3</x:v>
       </x:c>
-      <x:c r="G12" s="28"/>
+      <x:c r="J12" s="29"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:G1"/>
+    <x:mergeCell ref="A1:J1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1970,7 +2352,10 @@
     <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
@@ -1989,15 +2374,24 @@
         <x:v>日期</x:v>
       </x:c>
       <x:c r="D3" s="18" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="E3" s="18" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E3" s="18" t="str">
+      <x:c r="F3" s="18" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F3" s="18" t="str">
+      <x:c r="G3" s="18" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="H3" s="18" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I3" s="18" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="G3" s="18" t="str">
+      <x:c r="J3" s="18" t="str">
         <x:v>标的</x:v>
       </x:c>
     </x:row>
@@ -2012,16 +2406,25 @@
         <x:v>7月1日</x:v>
       </x:c>
       <x:c r="D4" s="22" t="n">
+        <x:v>2932</x:v>
+      </x:c>
+      <x:c r="E4" s="22" t="n">
         <x:v>2976</x:v>
       </x:c>
-      <x:c r="E4" s="22" t="n">
+      <x:c r="F4" s="22" t="n">
         <x:v>2918.2</x:v>
       </x:c>
-      <x:c r="F4" s="22" t="n">
-        <x:f>ROUND(D4-E4,1)</x:f>
+      <x:c r="G4" s="22" t="n">
+        <x:v>2934.6</x:v>
+      </x:c>
+      <x:c r="H4" s="23" t="n">
+        <x:v>-0.0011572498298162426</x:v>
+      </x:c>
+      <x:c r="I4" s="22" t="n">
+        <x:f>ROUND(E4-F4,1)</x:f>
         <x:v>57.8</x:v>
       </x:c>
-      <x:c r="G4" s="21" t="str">
+      <x:c r="J4" s="21" t="str">
         <x:v>IH2609</x:v>
       </x:c>
     </x:row>
@@ -2036,16 +2439,25 @@
         <x:v>7月2日</x:v>
       </x:c>
       <x:c r="D5" s="22" t="n">
+        <x:v>2923</x:v>
+      </x:c>
+      <x:c r="E5" s="22" t="n">
         <x:v>2924.8</x:v>
       </x:c>
-      <x:c r="E5" s="22" t="n">
+      <x:c r="F5" s="22" t="n">
         <x:v>2861.8</x:v>
       </x:c>
-      <x:c r="F5" s="24" t="n">
-        <x:f>ROUND(D5-E5,1)</x:f>
+      <x:c r="G5" s="22" t="n">
+        <x:v>2871</x:v>
+      </x:c>
+      <x:c r="H5" s="23" t="n">
+        <x:v>-0.02167245961970965</x:v>
+      </x:c>
+      <x:c r="I5" s="25" t="n">
+        <x:f>ROUND(E5-F5,1)</x:f>
         <x:v>63</x:v>
       </x:c>
-      <x:c r="G5" s="21" t="str">
+      <x:c r="J5" s="21" t="str">
         <x:v>IH2609</x:v>
       </x:c>
     </x:row>
@@ -2060,16 +2472,25 @@
         <x:v>7月3日</x:v>
       </x:c>
       <x:c r="D6" s="22" t="n">
+        <x:v>2876.6</x:v>
+      </x:c>
+      <x:c r="E6" s="22" t="n">
         <x:v>2912</x:v>
       </x:c>
-      <x:c r="E6" s="22" t="n">
+      <x:c r="F6" s="22" t="n">
         <x:v>2873.6</x:v>
       </x:c>
-      <x:c r="F6" s="22" t="n">
-        <x:f>ROUND(D6-E6,1)</x:f>
+      <x:c r="G6" s="22" t="n">
+        <x:v>2886.6</x:v>
+      </x:c>
+      <x:c r="H6" s="23" t="n">
+        <x:v>0.005433646812957216</x:v>
+      </x:c>
+      <x:c r="I6" s="22" t="n">
+        <x:f>ROUND(E6-F6,1)</x:f>
         <x:v>38.4</x:v>
       </x:c>
-      <x:c r="G6" s="21" t="str">
+      <x:c r="J6" s="21" t="str">
         <x:v>IH2609</x:v>
       </x:c>
     </x:row>
@@ -2084,16 +2505,25 @@
         <x:v>7月6日</x:v>
       </x:c>
       <x:c r="D7" s="22" t="n">
+        <x:v>2899</x:v>
+      </x:c>
+      <x:c r="E7" s="22" t="n">
         <x:v>2915</x:v>
       </x:c>
-      <x:c r="E7" s="22" t="n">
+      <x:c r="F7" s="22" t="n">
         <x:v>2877.4</x:v>
       </x:c>
-      <x:c r="F7" s="22" t="n">
-        <x:f>ROUND(D7-E7,1)</x:f>
+      <x:c r="G7" s="22" t="n">
+        <x:v>2905.2</x:v>
+      </x:c>
+      <x:c r="H7" s="23" t="n">
+        <x:v>0.00644356682602365</x:v>
+      </x:c>
+      <x:c r="I7" s="22" t="n">
+        <x:f>ROUND(E7-F7,1)</x:f>
         <x:v>37.6</x:v>
       </x:c>
-      <x:c r="G7" s="21" t="str">
+      <x:c r="J7" s="21" t="str">
         <x:v>IH2609</x:v>
       </x:c>
     </x:row>
@@ -2108,52 +2538,67 @@
         <x:v>7月7日</x:v>
       </x:c>
       <x:c r="D8" s="22" t="n">
+        <x:v>2888</x:v>
+      </x:c>
+      <x:c r="E8" s="22" t="n">
         <x:v>2908.4</x:v>
       </x:c>
-      <x:c r="E8" s="22" t="n">
+      <x:c r="F8" s="22" t="n">
         <x:v>2862.4</x:v>
       </x:c>
-      <x:c r="F8" s="22" t="n">
-        <x:f>ROUND(D8-E8,1)</x:f>
+      <x:c r="G8" s="22" t="n">
+        <x:v>2870.6</x:v>
+      </x:c>
+      <x:c r="H8" s="23" t="n">
+        <x:v>-0.01190967919592456</x:v>
+      </x:c>
+      <x:c r="I8" s="22" t="n">
+        <x:f>ROUND(E8-F8,1)</x:f>
         <x:v>46</x:v>
       </x:c>
-      <x:c r="G8" s="21" t="str">
+      <x:c r="J8" s="21" t="str">
         <x:v>IH2609</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="27" t="str">
+      <x:c r="A11" s="28" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B11" s="28" t="n">
+      <x:c r="B11" s="29" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C11" s="28"/>
-      <x:c r="D11" s="28"/>
-      <x:c r="E11" s="28"/>
-      <x:c r="F11" s="29" t="n">
-        <x:f>SUM(F4:F8)</x:f>
+      <x:c r="C11" s="29"/>
+      <x:c r="D11" s="29"/>
+      <x:c r="E11" s="29"/>
+      <x:c r="F11" s="29"/>
+      <x:c r="G11" s="29"/>
+      <x:c r="H11" s="29"/>
+      <x:c r="I11" s="30" t="n">
+        <x:f>SUM(I4:I8)</x:f>
         <x:v>242.79999999999998</x:v>
       </x:c>
-      <x:c r="G11" s="28"/>
+      <x:c r="J11" s="29"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="27" t="str">
+      <x:c r="A12" s="28" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B12" s="28"/>
-      <x:c r="C12" s="28"/>
-      <x:c r="D12" s="28"/>
-      <x:c r="E12" s="28"/>
-      <x:c r="F12" s="31" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(F4:F8),0),1)</x:f>
+      <x:c r="B12" s="29"/>
+      <x:c r="C12" s="29"/>
+      <x:c r="D12" s="29"/>
+      <x:c r="E12" s="29"/>
+      <x:c r="F12" s="29"/>
+      <x:c r="G12" s="29"/>
+      <x:c r="H12" s="29"/>
+      <x:c r="I12" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I4:I8),0),1)</x:f>
         <x:v>48.6</x:v>
       </x:c>
-      <x:c r="G12" s="28"/>
+      <x:c r="J12" s="29"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:G1"/>
+    <x:mergeCell ref="A1:J1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Update amplitude website 2026-07-08
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rb14655d492dd4e41"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="2" r:id="R63665d8505b54c0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="3" r:id="R2a3b94c57eb44308"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="4" r:id="Rc28ddba8238045d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="5" r:id="Rb1f571463aa24452"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="6" r:id="R05d5c033756346d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="7" r:id="Rdabfcbebac744bfe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="8" r:id="R103bacfe40af47be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R0463bc26e7a34cbc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="2" r:id="R8ceccae98c994111"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="3" r:id="R10e0d03ffffd4b8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="4" r:id="R7e8ea77416f540ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="5" r:id="Rcd586f0d23254ea6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="6" r:id="R0d4dea95cd1244ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="7" r:id="R21d8d30ed58f450e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="8" r:id="R90dbed18b43d45da"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -452,25 +452,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-07-07</x:v>
+        <x:v>2026-07-08</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>8489.476</x:v>
+        <x:v>8328.965</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>8261.398</x:v>
+        <x:v>8117.861</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>228.1</x:v>
+        <x:v>211.1</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>1076</x:v>
+        <x:v>1287.1</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>215.2</x:v>
+        <x:v>214.5</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -481,22 +481,22 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-07-07</x:v>
+        <x:v>2026-07-08</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>8663.665</x:v>
+        <x:v>8571.525</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>8457.576</x:v>
+        <x:v>8343.923</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>206.1</x:v>
+        <x:v>227.6</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>1139.2</x:v>
+        <x:v>1366.8</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
         <x:v>227.8</x:v>
@@ -510,25 +510,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-07-07</x:v>
+        <x:v>2026-07-08</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>4028.514</x:v>
+        <x:v>4016.026</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3971.713</x:v>
+        <x:v>3967.913</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>56.8</x:v>
+        <x:v>48.1</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>288.4</x:v>
+        <x:v>336.5</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>57.7</x:v>
+        <x:v>56.1</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -539,25 +539,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-07-07</x:v>
+        <x:v>2026-07-08</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>8274.2</x:v>
+        <x:v>8149.8</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>8068.8</x:v>
+        <x:v>7965</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>205.4</x:v>
+        <x:v>184.8</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>910.4</x:v>
+        <x:v>1095.2</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>182.1</x:v>
+        <x:v>182.5</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -568,25 +568,25 @@
         <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>2026-07-07</x:v>
+        <x:v>2026-07-08</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:v>8478.8</x:v>
+        <x:v>8376</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>8281</x:v>
+        <x:v>8203.6</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>197.8</x:v>
+        <x:v>172.4</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>1052.8</x:v>
+        <x:v>1225.2</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
-        <x:v>210.6</x:v>
+        <x:v>204.2</x:v>
       </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
@@ -597,25 +597,25 @@
         <x:v>IF主力</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>2026-07-07</x:v>
+        <x:v>2026-07-08</x:v>
       </x:c>
       <x:c r="C9" s="10" t="n">
-        <x:v>4752.6</x:v>
+        <x:v>4747.6</x:v>
       </x:c>
       <x:c r="D9" s="10" t="n">
-        <x:v>4671.4</x:v>
+        <x:v>4666</x:v>
       </x:c>
       <x:c r="E9" s="12" t="n">
-        <x:v>81.2</x:v>
+        <x:v>81.6</x:v>
       </x:c>
       <x:c r="F9" s="9" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G9" s="10" t="n">
-        <x:v>436.4</x:v>
+        <x:v>518</x:v>
       </x:c>
       <x:c r="H9" s="10" t="n">
-        <x:v>87.3</x:v>
+        <x:v>86.3</x:v>
       </x:c>
       <x:c r="I9" s="10" t="n">
         <x:v>90</x:v>
@@ -626,25 +626,25 @@
         <x:v>IH主力</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>2026-07-07</x:v>
+        <x:v>2026-07-08</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:v>2908.4</x:v>
+        <x:v>2911</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
-        <x:v>2862.4</x:v>
+        <x:v>2866.2</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
-        <x:v>46</x:v>
+        <x:v>44.8</x:v>
       </x:c>
       <x:c r="F10" s="9" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G10" s="10" t="n">
-        <x:v>242.8</x:v>
+        <x:v>287.6</x:v>
       </x:c>
       <x:c r="H10" s="10" t="n">
-        <x:v>48.6</x:v>
+        <x:v>47.9</x:v>
       </x:c>
       <x:c r="I10" s="10" t="n">
         <x:v>60</x:v>
@@ -658,7 +658,7 @@
         <x:v>2026-07-01</x:v>
       </x:c>
       <x:c r="C13" s="14" t="str">
-        <x:v>2026-07-07</x:v>
+        <x:v>2026-07-08</x:v>
       </x:c>
       <x:c r="D13" s="14" t="str">
         <x:v>数据源</x:v>
@@ -988,41 +988,74 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="28" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B11" s="29" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C11" s="29"/>
-      <x:c r="D11" s="29"/>
-      <x:c r="E11" s="29"/>
-      <x:c r="F11" s="29"/>
-      <x:c r="G11" s="29"/>
-      <x:c r="H11" s="29"/>
-      <x:c r="I11" s="30" t="n">
-        <x:f>SUM(I4:I8)</x:f>
-        <x:v>1076</x:v>
-      </x:c>
-      <x:c r="J11" s="29"/>
+    <x:row r="9">
+      <x:c r="A9" s="21" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B9" s="21" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C9" s="21" t="str">
+        <x:v>7月8日</x:v>
+      </x:c>
+      <x:c r="D9" s="22" t="n">
+        <x:v>8315.962</x:v>
+      </x:c>
+      <x:c r="E9" s="22" t="n">
+        <x:v>8328.965</x:v>
+      </x:c>
+      <x:c r="F9" s="22" t="n">
+        <x:v>8117.861</x:v>
+      </x:c>
+      <x:c r="G9" s="22" t="n">
+        <x:v>8117.861</x:v>
+      </x:c>
+      <x:c r="H9" s="23" t="n">
+        <x:v>-0.02215699142017813</x:v>
+      </x:c>
+      <x:c r="I9" s="25" t="n">
+        <x:f>ROUND(E9-F9,1)</x:f>
+        <x:v>211.1</x:v>
+      </x:c>
+      <x:c r="J9" s="21" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="28" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B12" s="29"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B12" s="29" t="n">
+        <x:v>6</x:v>
+      </x:c>
       <x:c r="C12" s="29"/>
       <x:c r="D12" s="29"/>
       <x:c r="E12" s="29"/>
       <x:c r="F12" s="29"/>
       <x:c r="G12" s="29"/>
       <x:c r="H12" s="29"/>
-      <x:c r="I12" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I4:I8),0),1)</x:f>
-        <x:v>215.2</x:v>
+      <x:c r="I12" s="30" t="n">
+        <x:f>SUM(I4:I9)</x:f>
+        <x:v>1287.1</x:v>
       </x:c>
       <x:c r="J12" s="29"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="28" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B13" s="29"/>
+      <x:c r="C13" s="29"/>
+      <x:c r="D13" s="29"/>
+      <x:c r="E13" s="29"/>
+      <x:c r="F13" s="29"/>
+      <x:c r="G13" s="29"/>
+      <x:c r="H13" s="29"/>
+      <x:c r="I13" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I4:I9),0),1)</x:f>
+        <x:v>214.5</x:v>
+      </x:c>
+      <x:c r="J13" s="29"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1250,41 +1283,74 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="28" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B11" s="29" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C11" s="29"/>
-      <x:c r="D11" s="29"/>
-      <x:c r="E11" s="29"/>
-      <x:c r="F11" s="29"/>
-      <x:c r="G11" s="29"/>
-      <x:c r="H11" s="29"/>
-      <x:c r="I11" s="30" t="n">
-        <x:f>SUM(I4:I8)</x:f>
-        <x:v>1139.2</x:v>
-      </x:c>
-      <x:c r="J11" s="29"/>
+    <x:row r="9">
+      <x:c r="A9" s="21" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B9" s="21" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C9" s="21" t="str">
+        <x:v>7月8日</x:v>
+      </x:c>
+      <x:c r="D9" s="22" t="n">
+        <x:v>8539.016</x:v>
+      </x:c>
+      <x:c r="E9" s="22" t="n">
+        <x:v>8571.525</x:v>
+      </x:c>
+      <x:c r="F9" s="22" t="n">
+        <x:v>8343.923</x:v>
+      </x:c>
+      <x:c r="G9" s="22" t="n">
+        <x:v>8390.019</x:v>
+      </x:c>
+      <x:c r="H9" s="23" t="n">
+        <x:v>-0.013958508079116805</x:v>
+      </x:c>
+      <x:c r="I9" s="25" t="n">
+        <x:f>ROUND(E9-F9,1)</x:f>
+        <x:v>227.6</x:v>
+      </x:c>
+      <x:c r="J9" s="21" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="28" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B12" s="29"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B12" s="29" t="n">
+        <x:v>6</x:v>
+      </x:c>
       <x:c r="C12" s="29"/>
       <x:c r="D12" s="29"/>
       <x:c r="E12" s="29"/>
       <x:c r="F12" s="29"/>
       <x:c r="G12" s="29"/>
       <x:c r="H12" s="29"/>
-      <x:c r="I12" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I4:I8),0),1)</x:f>
+      <x:c r="I12" s="30" t="n">
+        <x:f>SUM(I4:I9)</x:f>
+        <x:v>1366.8</x:v>
+      </x:c>
+      <x:c r="J12" s="29"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="28" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B13" s="29"/>
+      <x:c r="C13" s="29"/>
+      <x:c r="D13" s="29"/>
+      <x:c r="E13" s="29"/>
+      <x:c r="F13" s="29"/>
+      <x:c r="G13" s="29"/>
+      <x:c r="H13" s="29"/>
+      <x:c r="I13" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I4:I9),0),1)</x:f>
         <x:v>227.8</x:v>
       </x:c>
-      <x:c r="J12" s="29"/>
+      <x:c r="J13" s="29"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1512,41 +1578,74 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="28" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B11" s="29" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C11" s="29"/>
-      <x:c r="D11" s="29"/>
-      <x:c r="E11" s="29"/>
-      <x:c r="F11" s="29"/>
-      <x:c r="G11" s="29"/>
-      <x:c r="H11" s="29"/>
-      <x:c r="I11" s="30" t="n">
-        <x:f>SUM(I4:I8)</x:f>
-        <x:v>288.40000000000003</x:v>
-      </x:c>
-      <x:c r="J11" s="29"/>
+    <x:row r="9">
+      <x:c r="A9" s="21" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B9" s="21" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C9" s="21" t="str">
+        <x:v>7月8日</x:v>
+      </x:c>
+      <x:c r="D9" s="22" t="n">
+        <x:v>3996.807</x:v>
+      </x:c>
+      <x:c r="E9" s="22" t="n">
+        <x:v>4016.026</x:v>
+      </x:c>
+      <x:c r="F9" s="22" t="n">
+        <x:v>3967.913</x:v>
+      </x:c>
+      <x:c r="G9" s="22" t="n">
+        <x:v>3970.88</x:v>
+      </x:c>
+      <x:c r="H9" s="23" t="n">
+        <x:v>-0.004850591506515234</x:v>
+      </x:c>
+      <x:c r="I9" s="22" t="n">
+        <x:f>ROUND(E9-F9,1)</x:f>
+        <x:v>48.1</x:v>
+      </x:c>
+      <x:c r="J9" s="21" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="28" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B12" s="29"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B12" s="29" t="n">
+        <x:v>6</x:v>
+      </x:c>
       <x:c r="C12" s="29"/>
       <x:c r="D12" s="29"/>
       <x:c r="E12" s="29"/>
       <x:c r="F12" s="29"/>
       <x:c r="G12" s="29"/>
       <x:c r="H12" s="29"/>
-      <x:c r="I12" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I4:I8),0),1)</x:f>
-        <x:v>57.7</x:v>
+      <x:c r="I12" s="30" t="n">
+        <x:f>SUM(I4:I9)</x:f>
+        <x:v>336.50000000000006</x:v>
       </x:c>
       <x:c r="J12" s="29"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="28" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B13" s="29"/>
+      <x:c r="C13" s="29"/>
+      <x:c r="D13" s="29"/>
+      <x:c r="E13" s="29"/>
+      <x:c r="F13" s="29"/>
+      <x:c r="G13" s="29"/>
+      <x:c r="H13" s="29"/>
+      <x:c r="I13" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I4:I9),0),1)</x:f>
+        <x:v>56.1</x:v>
+      </x:c>
+      <x:c r="J13" s="29"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1774,41 +1873,74 @@
         <x:v>IM2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="28" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B11" s="29" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C11" s="29"/>
-      <x:c r="D11" s="29"/>
-      <x:c r="E11" s="29"/>
-      <x:c r="F11" s="29"/>
-      <x:c r="G11" s="29"/>
-      <x:c r="H11" s="29"/>
-      <x:c r="I11" s="30" t="n">
-        <x:f>SUM(I4:I8)</x:f>
-        <x:v>910.4</x:v>
-      </x:c>
-      <x:c r="J11" s="29"/>
+    <x:row r="9">
+      <x:c r="A9" s="21" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B9" s="21" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C9" s="21" t="str">
+        <x:v>7月8日</x:v>
+      </x:c>
+      <x:c r="D9" s="22" t="n">
+        <x:v>8140.2</x:v>
+      </x:c>
+      <x:c r="E9" s="22" t="n">
+        <x:v>8149.8</x:v>
+      </x:c>
+      <x:c r="F9" s="22" t="n">
+        <x:v>7965</x:v>
+      </x:c>
+      <x:c r="G9" s="22" t="n">
+        <x:v>7974</x:v>
+      </x:c>
+      <x:c r="H9" s="23" t="n">
+        <x:v>-0.017399447949526747</x:v>
+      </x:c>
+      <x:c r="I9" s="22" t="n">
+        <x:f>ROUND(E9-F9,1)</x:f>
+        <x:v>184.8</x:v>
+      </x:c>
+      <x:c r="J9" s="21" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="28" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B12" s="29"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B12" s="29" t="n">
+        <x:v>6</x:v>
+      </x:c>
       <x:c r="C12" s="29"/>
       <x:c r="D12" s="29"/>
       <x:c r="E12" s="29"/>
       <x:c r="F12" s="29"/>
       <x:c r="G12" s="29"/>
       <x:c r="H12" s="29"/>
-      <x:c r="I12" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I4:I8),0),1)</x:f>
-        <x:v>182.1</x:v>
+      <x:c r="I12" s="30" t="n">
+        <x:f>SUM(I4:I9)</x:f>
+        <x:v>1095.2</x:v>
       </x:c>
       <x:c r="J12" s="29"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="28" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B13" s="29"/>
+      <x:c r="C13" s="29"/>
+      <x:c r="D13" s="29"/>
+      <x:c r="E13" s="29"/>
+      <x:c r="F13" s="29"/>
+      <x:c r="G13" s="29"/>
+      <x:c r="H13" s="29"/>
+      <x:c r="I13" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I4:I9),0),1)</x:f>
+        <x:v>182.5</x:v>
+      </x:c>
+      <x:c r="J13" s="29"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2036,41 +2168,74 @@
         <x:v>IC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="28" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B11" s="29" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C11" s="29"/>
-      <x:c r="D11" s="29"/>
-      <x:c r="E11" s="29"/>
-      <x:c r="F11" s="29"/>
-      <x:c r="G11" s="29"/>
-      <x:c r="H11" s="29"/>
-      <x:c r="I11" s="30" t="n">
-        <x:f>SUM(I4:I8)</x:f>
-        <x:v>1052.8</x:v>
-      </x:c>
-      <x:c r="J11" s="29"/>
+    <x:row r="9">
+      <x:c r="A9" s="21" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B9" s="21" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C9" s="21" t="str">
+        <x:v>7月8日</x:v>
+      </x:c>
+      <x:c r="D9" s="22" t="n">
+        <x:v>8376</x:v>
+      </x:c>
+      <x:c r="E9" s="22" t="n">
+        <x:v>8376</x:v>
+      </x:c>
+      <x:c r="F9" s="22" t="n">
+        <x:v>8203.6</x:v>
+      </x:c>
+      <x:c r="G9" s="22" t="n">
+        <x:v>8255.2</x:v>
+      </x:c>
+      <x:c r="H9" s="23" t="n">
+        <x:v>-0.008098430778843091</x:v>
+      </x:c>
+      <x:c r="I9" s="25" t="n">
+        <x:f>ROUND(E9-F9,1)</x:f>
+        <x:v>172.4</x:v>
+      </x:c>
+      <x:c r="J9" s="21" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="28" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B12" s="29"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B12" s="29" t="n">
+        <x:v>6</x:v>
+      </x:c>
       <x:c r="C12" s="29"/>
       <x:c r="D12" s="29"/>
       <x:c r="E12" s="29"/>
       <x:c r="F12" s="29"/>
       <x:c r="G12" s="29"/>
       <x:c r="H12" s="29"/>
-      <x:c r="I12" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I4:I8),0),1)</x:f>
-        <x:v>210.6</x:v>
+      <x:c r="I12" s="30" t="n">
+        <x:f>SUM(I4:I9)</x:f>
+        <x:v>1225.2</x:v>
       </x:c>
       <x:c r="J12" s="29"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="28" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B13" s="29"/>
+      <x:c r="C13" s="29"/>
+      <x:c r="D13" s="29"/>
+      <x:c r="E13" s="29"/>
+      <x:c r="F13" s="29"/>
+      <x:c r="G13" s="29"/>
+      <x:c r="H13" s="29"/>
+      <x:c r="I13" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I4:I9),0),1)</x:f>
+        <x:v>204.2</x:v>
+      </x:c>
+      <x:c r="J13" s="29"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2298,41 +2463,74 @@
         <x:v>IF2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="28" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B11" s="29" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C11" s="29"/>
-      <x:c r="D11" s="29"/>
-      <x:c r="E11" s="29"/>
-      <x:c r="F11" s="29"/>
-      <x:c r="G11" s="29"/>
-      <x:c r="H11" s="29"/>
-      <x:c r="I11" s="30" t="n">
-        <x:f>SUM(I4:I8)</x:f>
-        <x:v>436.4</x:v>
-      </x:c>
-      <x:c r="J11" s="29"/>
+    <x:row r="9">
+      <x:c r="A9" s="21" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B9" s="21" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C9" s="21" t="str">
+        <x:v>7月8日</x:v>
+      </x:c>
+      <x:c r="D9" s="22" t="n">
+        <x:v>4728</x:v>
+      </x:c>
+      <x:c r="E9" s="22" t="n">
+        <x:v>4747.6</x:v>
+      </x:c>
+      <x:c r="F9" s="22" t="n">
+        <x:v>4666</x:v>
+      </x:c>
+      <x:c r="G9" s="22" t="n">
+        <x:v>4668</x:v>
+      </x:c>
+      <x:c r="H9" s="23" t="n">
+        <x:v>-0.007526470213037317</x:v>
+      </x:c>
+      <x:c r="I9" s="22" t="n">
+        <x:f>ROUND(E9-F9,1)</x:f>
+        <x:v>81.6</x:v>
+      </x:c>
+      <x:c r="J9" s="21" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="28" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B12" s="29"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B12" s="29" t="n">
+        <x:v>6</x:v>
+      </x:c>
       <x:c r="C12" s="29"/>
       <x:c r="D12" s="29"/>
       <x:c r="E12" s="29"/>
       <x:c r="F12" s="29"/>
       <x:c r="G12" s="29"/>
       <x:c r="H12" s="29"/>
-      <x:c r="I12" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I4:I8),0),1)</x:f>
-        <x:v>87.3</x:v>
+      <x:c r="I12" s="30" t="n">
+        <x:f>SUM(I4:I9)</x:f>
+        <x:v>518</x:v>
       </x:c>
       <x:c r="J12" s="29"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="28" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B13" s="29"/>
+      <x:c r="C13" s="29"/>
+      <x:c r="D13" s="29"/>
+      <x:c r="E13" s="29"/>
+      <x:c r="F13" s="29"/>
+      <x:c r="G13" s="29"/>
+      <x:c r="H13" s="29"/>
+      <x:c r="I13" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I4:I9),0),1)</x:f>
+        <x:v>86.3</x:v>
+      </x:c>
+      <x:c r="J13" s="29"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2560,41 +2758,74 @@
         <x:v>IH2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="28" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B11" s="29" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C11" s="29"/>
-      <x:c r="D11" s="29"/>
-      <x:c r="E11" s="29"/>
-      <x:c r="F11" s="29"/>
-      <x:c r="G11" s="29"/>
-      <x:c r="H11" s="29"/>
-      <x:c r="I11" s="30" t="n">
-        <x:f>SUM(I4:I8)</x:f>
-        <x:v>242.79999999999998</x:v>
-      </x:c>
-      <x:c r="J11" s="29"/>
+    <x:row r="9">
+      <x:c r="A9" s="21" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B9" s="21" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C9" s="21" t="str">
+        <x:v>7月8日</x:v>
+      </x:c>
+      <x:c r="D9" s="22" t="n">
+        <x:v>2877.4</x:v>
+      </x:c>
+      <x:c r="E9" s="22" t="n">
+        <x:v>2911</x:v>
+      </x:c>
+      <x:c r="F9" s="22" t="n">
+        <x:v>2866.2</x:v>
+      </x:c>
+      <x:c r="G9" s="22" t="n">
+        <x:v>2868</x:v>
+      </x:c>
+      <x:c r="H9" s="23" t="n">
+        <x:v>-0.0009057339928933983</x:v>
+      </x:c>
+      <x:c r="I9" s="22" t="n">
+        <x:f>ROUND(E9-F9,1)</x:f>
+        <x:v>44.8</x:v>
+      </x:c>
+      <x:c r="J9" s="21" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="28" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B12" s="29"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B12" s="29" t="n">
+        <x:v>6</x:v>
+      </x:c>
       <x:c r="C12" s="29"/>
       <x:c r="D12" s="29"/>
       <x:c r="E12" s="29"/>
       <x:c r="F12" s="29"/>
       <x:c r="G12" s="29"/>
       <x:c r="H12" s="29"/>
-      <x:c r="I12" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I4:I8),0),1)</x:f>
-        <x:v>48.6</x:v>
+      <x:c r="I12" s="30" t="n">
+        <x:f>SUM(I4:I9)</x:f>
+        <x:v>287.59999999999997</x:v>
       </x:c>
       <x:c r="J12" s="29"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="28" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B13" s="29"/>
+      <x:c r="C13" s="29"/>
+      <x:c r="D13" s="29"/>
+      <x:c r="E13" s="29"/>
+      <x:c r="F13" s="29"/>
+      <x:c r="G13" s="29"/>
+      <x:c r="H13" s="29"/>
+      <x:c r="I13" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I4:I9),0),1)</x:f>
+        <x:v>47.9</x:v>
+      </x:c>
+      <x:c r="J13" s="29"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-07-09
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R0463bc26e7a34cbc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="2" r:id="R8ceccae98c994111"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="3" r:id="R10e0d03ffffd4b8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="4" r:id="R7e8ea77416f540ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="5" r:id="Rcd586f0d23254ea6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="6" r:id="R0d4dea95cd1244ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="7" r:id="R21d8d30ed58f450e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="8" r:id="R90dbed18b43d45da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R648f0ab299b14737"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="2" r:id="R31a642352a0245b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="3" r:id="R018bea44329b4a8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="4" r:id="R29035ee1361b49a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="5" r:id="Rd3d5e86e9b544b7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="6" r:id="R15d2c516d6d240df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="7" r:id="Rf8b3134efe4c4718"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="8" r:id="R15dc4b47d4ee41b5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -658,7 +658,7 @@
         <x:v>2026-07-01</x:v>
       </x:c>
       <x:c r="C13" s="14" t="str">
-        <x:v>2026-07-08</x:v>
+        <x:v>2026-07-09</x:v>
       </x:c>
       <x:c r="D13" s="14" t="str">
         <x:v>数据源</x:v>

</xml_diff>

<commit_message>
Update amplitude website 2026-07-10
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R1a071e1a86b84c16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="2" r:id="R495647af42844e36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="3" r:id="R80d9b179477d4f6e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="4" r:id="R0af3dd2ca92a4c4b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="5" r:id="R4ad30927804245e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="6" r:id="R8888543b2f554386"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="7" r:id="R6a32c53f3d394117"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="8" r:id="R6b86a9283bad4b09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R2b9264bc3d524f00"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="2" r:id="Ra0d1703e15c2454b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="3" r:id="R9c4c00a23d814e12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="4" r:id="R0592a88082344fff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="5" r:id="R953a07066a034f30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="6" r:id="R60c15dce550b40be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="7" r:id="R937022fb83b1413a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="8" r:id="R9839bde03dbd4c72"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -469,25 +469,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-07-09</x:v>
+        <x:v>2026-07-10</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>8312.621</x:v>
+        <x:v>8438.194</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7978.806</x:v>
+        <x:v>8198.308</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>333.8</x:v>
+        <x:v>239.9</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>1620.9</x:v>
+        <x:v>1860.8</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>231.6</x:v>
+        <x:v>232.6</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -498,25 +498,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-07-09</x:v>
+        <x:v>2026-07-10</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>8659.65</x:v>
+        <x:v>8783.249</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>8281.953</x:v>
+        <x:v>8503.245</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>377.7</x:v>
+        <x:v>280</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>1744.5</x:v>
+        <x:v>2024.5</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>249.2</x:v>
+        <x:v>253.1</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -527,25 +527,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-07-09</x:v>
+        <x:v>2026-07-10</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>4040.539</x:v>
+        <x:v>4074.828</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3938.878</x:v>
+        <x:v>3995.807</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>101.7</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>438.2</x:v>
+        <x:v>517.2</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>62.6</x:v>
+        <x:v>64.7</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -556,25 +556,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-07-08</x:v>
+        <x:v>2026-07-10</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>8149.8</x:v>
+        <x:v>8244.8</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>7965</x:v>
+        <x:v>8016</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>184.8</x:v>
+        <x:v>228.8</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>6</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>1095.2</x:v>
+        <x:v>1596</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>182.5</x:v>
+        <x:v>199.5</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -585,25 +585,25 @@
         <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>2026-07-09</x:v>
+        <x:v>2026-07-10</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:v>8509.2</x:v>
+        <x:v>8618</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>8173</x:v>
+        <x:v>8330</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>336.2</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>1561.4</x:v>
+        <x:v>1849.4</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
-        <x:v>223.1</x:v>
+        <x:v>231.2</x:v>
       </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
@@ -614,25 +614,25 @@
         <x:v>IF主力</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>2026-07-08</x:v>
+        <x:v>2026-07-10</x:v>
       </x:c>
       <x:c r="C9" s="10" t="n">
-        <x:v>4747.6</x:v>
+        <x:v>4822.2</x:v>
       </x:c>
       <x:c r="D9" s="10" t="n">
-        <x:v>4666</x:v>
+        <x:v>4703.6</x:v>
       </x:c>
       <x:c r="E9" s="12" t="n">
-        <x:v>81.6</x:v>
+        <x:v>118.6</x:v>
       </x:c>
       <x:c r="F9" s="9" t="n">
-        <x:v>6</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G9" s="10" t="n">
-        <x:v>518</x:v>
+        <x:v>775.4</x:v>
       </x:c>
       <x:c r="H9" s="10" t="n">
-        <x:v>86.3</x:v>
+        <x:v>96.9</x:v>
       </x:c>
       <x:c r="I9" s="10" t="n">
         <x:v>90</x:v>
@@ -643,25 +643,25 @@
         <x:v>IH主力</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>2026-07-09</x:v>
+        <x:v>2026-07-10</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:v>2956.2</x:v>
+        <x:v>2983.8</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
-        <x:v>2875</x:v>
+        <x:v>2908.2</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
-        <x:v>81.2</x:v>
+        <x:v>75.6</x:v>
       </x:c>
       <x:c r="F10" s="9" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G10" s="10" t="n">
-        <x:v>368.8</x:v>
+        <x:v>444.4</x:v>
       </x:c>
       <x:c r="H10" s="10" t="n">
-        <x:v>52.7</x:v>
+        <x:v>55.6</x:v>
       </x:c>
       <x:c r="I10" s="10" t="n">
         <x:v>60</x:v>
@@ -675,7 +675,7 @@
         <x:v>2026-07-01</x:v>
       </x:c>
       <x:c r="C13" s="14" t="str">
-        <x:v>2026-07-09</x:v>
+        <x:v>2026-07-10</x:v>
       </x:c>
       <x:c r="D13" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1096,31 +1096,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="30" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B13" s="31" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C13" s="31"/>
-      <x:c r="D13" s="31"/>
-      <x:c r="E13" s="31"/>
-      <x:c r="F13" s="31"/>
-      <x:c r="G13" s="31"/>
-      <x:c r="H13" s="31"/>
-      <x:c r="I13" s="31"/>
-      <x:c r="J13" s="32" t="n">
-        <x:f>SUM(J4:J10)</x:f>
-        <x:v>1620.8999999999999</x:v>
-      </x:c>
-      <x:c r="K13" s="31"/>
+    <x:row r="11">
+      <x:c r="A11" s="21" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B11" s="21" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C11" s="21" t="str">
+        <x:v>7月10日</x:v>
+      </x:c>
+      <x:c r="D11" s="22" t="n">
+        <x:v>8312.492</x:v>
+      </x:c>
+      <x:c r="E11" s="22" t="n">
+        <x:v>8438.194</x:v>
+      </x:c>
+      <x:c r="F11" s="22" t="n">
+        <x:v>8198.308</x:v>
+      </x:c>
+      <x:c r="G11" s="22" t="n">
+        <x:v>8198.308</x:v>
+      </x:c>
+      <x:c r="H11" s="22" t="n">
+        <x:v>-101.8</x:v>
+      </x:c>
+      <x:c r="I11" s="23" t="n">
+        <x:v>-0.012261211552615503</x:v>
+      </x:c>
+      <x:c r="J11" s="27" t="n">
+        <x:f>ROUND(E11-F11,1)</x:f>
+        <x:v>239.9</x:v>
+      </x:c>
+      <x:c r="K11" s="21" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="30" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B14" s="31"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B14" s="31" t="n">
+        <x:v>8</x:v>
+      </x:c>
       <x:c r="C14" s="31"/>
       <x:c r="D14" s="31"/>
       <x:c r="E14" s="31"/>
@@ -1128,11 +1146,29 @@
       <x:c r="G14" s="31"/>
       <x:c r="H14" s="31"/>
       <x:c r="I14" s="31"/>
-      <x:c r="J14" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J10),0),1)</x:f>
-        <x:v>231.6</x:v>
+      <x:c r="J14" s="32" t="n">
+        <x:f>SUM(J4:J11)</x:f>
+        <x:v>1860.8</x:v>
       </x:c>
       <x:c r="K14" s="31"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="30" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B15" s="31"/>
+      <x:c r="C15" s="31"/>
+      <x:c r="D15" s="31"/>
+      <x:c r="E15" s="31"/>
+      <x:c r="F15" s="31"/>
+      <x:c r="G15" s="31"/>
+      <x:c r="H15" s="31"/>
+      <x:c r="I15" s="31"/>
+      <x:c r="J15" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
+        <x:v>232.6</x:v>
+      </x:c>
+      <x:c r="K15" s="31"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1451,31 +1487,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="30" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B13" s="31" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C13" s="31"/>
-      <x:c r="D13" s="31"/>
-      <x:c r="E13" s="31"/>
-      <x:c r="F13" s="31"/>
-      <x:c r="G13" s="31"/>
-      <x:c r="H13" s="31"/>
-      <x:c r="I13" s="31"/>
-      <x:c r="J13" s="32" t="n">
-        <x:f>SUM(J4:J10)</x:f>
-        <x:v>1744.5</x:v>
-      </x:c>
-      <x:c r="K13" s="31"/>
+    <x:row r="11">
+      <x:c r="A11" s="21" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B11" s="21" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C11" s="21" t="str">
+        <x:v>7月10日</x:v>
+      </x:c>
+      <x:c r="D11" s="22" t="n">
+        <x:v>8672.363</x:v>
+      </x:c>
+      <x:c r="E11" s="22" t="n">
+        <x:v>8783.249</x:v>
+      </x:c>
+      <x:c r="F11" s="22" t="n">
+        <x:v>8503.245</x:v>
+      </x:c>
+      <x:c r="G11" s="22" t="n">
+        <x:v>8503.971</x:v>
+      </x:c>
+      <x:c r="H11" s="22" t="n">
+        <x:v>-148.8</x:v>
+      </x:c>
+      <x:c r="I11" s="23" t="n">
+        <x:v>-0.01719862051382992</x:v>
+      </x:c>
+      <x:c r="J11" s="27" t="n">
+        <x:f>ROUND(E11-F11,1)</x:f>
+        <x:v>280</x:v>
+      </x:c>
+      <x:c r="K11" s="21" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="30" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B14" s="31"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B14" s="31" t="n">
+        <x:v>8</x:v>
+      </x:c>
       <x:c r="C14" s="31"/>
       <x:c r="D14" s="31"/>
       <x:c r="E14" s="31"/>
@@ -1483,11 +1537,29 @@
       <x:c r="G14" s="31"/>
       <x:c r="H14" s="31"/>
       <x:c r="I14" s="31"/>
-      <x:c r="J14" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J10),0),1)</x:f>
-        <x:v>249.2</x:v>
+      <x:c r="J14" s="32" t="n">
+        <x:f>SUM(J4:J11)</x:f>
+        <x:v>2024.5</x:v>
       </x:c>
       <x:c r="K14" s="31"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="30" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B15" s="31"/>
+      <x:c r="C15" s="31"/>
+      <x:c r="D15" s="31"/>
+      <x:c r="E15" s="31"/>
+      <x:c r="F15" s="31"/>
+      <x:c r="G15" s="31"/>
+      <x:c r="H15" s="31"/>
+      <x:c r="I15" s="31"/>
+      <x:c r="J15" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
+        <x:v>253.1</x:v>
+      </x:c>
+      <x:c r="K15" s="31"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1806,31 +1878,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="30" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B13" s="31" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C13" s="31"/>
-      <x:c r="D13" s="31"/>
-      <x:c r="E13" s="31"/>
-      <x:c r="F13" s="31"/>
-      <x:c r="G13" s="31"/>
-      <x:c r="H13" s="31"/>
-      <x:c r="I13" s="31"/>
-      <x:c r="J13" s="32" t="n">
-        <x:f>SUM(J4:J10)</x:f>
-        <x:v>438.20000000000005</x:v>
-      </x:c>
-      <x:c r="K13" s="31"/>
+    <x:row r="11">
+      <x:c r="A11" s="21" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B11" s="21" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C11" s="21" t="str">
+        <x:v>7月10日</x:v>
+      </x:c>
+      <x:c r="D11" s="22" t="n">
+        <x:v>4031.537</x:v>
+      </x:c>
+      <x:c r="E11" s="22" t="n">
+        <x:v>4074.828</x:v>
+      </x:c>
+      <x:c r="F11" s="22" t="n">
+        <x:v>3995.807</x:v>
+      </x:c>
+      <x:c r="G11" s="22" t="n">
+        <x:v>3996.162</x:v>
+      </x:c>
+      <x:c r="H11" s="22" t="n">
+        <x:v>-40.4</x:v>
+      </x:c>
+      <x:c r="I11" s="23" t="n">
+        <x:v>-0.010014893766715938</x:v>
+      </x:c>
+      <x:c r="J11" s="27" t="n">
+        <x:f>ROUND(E11-F11,1)</x:f>
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="K11" s="21" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="30" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B14" s="31"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B14" s="31" t="n">
+        <x:v>8</x:v>
+      </x:c>
       <x:c r="C14" s="31"/>
       <x:c r="D14" s="31"/>
       <x:c r="E14" s="31"/>
@@ -1838,11 +1928,29 @@
       <x:c r="G14" s="31"/>
       <x:c r="H14" s="31"/>
       <x:c r="I14" s="31"/>
-      <x:c r="J14" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J10),0),1)</x:f>
-        <x:v>62.6</x:v>
+      <x:c r="J14" s="32" t="n">
+        <x:f>SUM(J4:J11)</x:f>
+        <x:v>517.2</x:v>
       </x:c>
       <x:c r="K14" s="31"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="30" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B15" s="31"/>
+      <x:c r="C15" s="31"/>
+      <x:c r="D15" s="31"/>
+      <x:c r="E15" s="31"/>
+      <x:c r="F15" s="31"/>
+      <x:c r="G15" s="31"/>
+      <x:c r="H15" s="31"/>
+      <x:c r="I15" s="31"/>
+      <x:c r="J15" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
+        <x:v>64.7</x:v>
+      </x:c>
+      <x:c r="K15" s="31"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2113,43 +2221,111 @@
         <x:v>IM2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="30" t="str">
+    <x:row r="10">
+      <x:c r="A10" s="21" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B10" s="21" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C10" s="21" t="str">
+        <x:v>7月9日</x:v>
+      </x:c>
+      <x:c r="D10" s="22" t="n">
+        <x:v>8034.8</x:v>
+      </x:c>
+      <x:c r="E10" s="22" t="n">
+        <x:v>8140.2</x:v>
+      </x:c>
+      <x:c r="F10" s="22" t="n">
+        <x:v>7868.2</x:v>
+      </x:c>
+      <x:c r="G10" s="22" t="n">
+        <x:v>8127.4</x:v>
+      </x:c>
+      <x:c r="H10" s="22"/>
+      <x:c r="I10" s="23" t="n">
+        <x:v>0.019237521946325442</x:v>
+      </x:c>
+      <x:c r="J10" s="27" t="n">
+        <x:f>ROUND(E10-F10,1)</x:f>
+        <x:v>272</x:v>
+      </x:c>
+      <x:c r="K10" s="21" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="21" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B11" s="21" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C11" s="21" t="str">
+        <x:v>7月10日</x:v>
+      </x:c>
+      <x:c r="D11" s="22" t="n">
+        <x:v>8140.2</x:v>
+      </x:c>
+      <x:c r="E11" s="22" t="n">
+        <x:v>8244.8</x:v>
+      </x:c>
+      <x:c r="F11" s="22" t="n">
+        <x:v>8016</x:v>
+      </x:c>
+      <x:c r="G11" s="22" t="n">
+        <x:v>8019.4</x:v>
+      </x:c>
+      <x:c r="H11" s="22"/>
+      <x:c r="I11" s="23" t="n">
+        <x:v>-0.013288382508551355</x:v>
+      </x:c>
+      <x:c r="J11" s="27" t="n">
+        <x:f>ROUND(E11-F11,1)</x:f>
+        <x:v>228.8</x:v>
+      </x:c>
+      <x:c r="K11" s="21" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="30" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B12" s="31" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="C12" s="31"/>
-      <x:c r="D12" s="31"/>
-      <x:c r="E12" s="31"/>
-      <x:c r="F12" s="31"/>
-      <x:c r="G12" s="31"/>
-      <x:c r="H12" s="31"/>
-      <x:c r="I12" s="31"/>
-      <x:c r="J12" s="32" t="n">
-        <x:f>SUM(J4:J9)</x:f>
-        <x:v>1095.2</x:v>
-      </x:c>
-      <x:c r="K12" s="31"/>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="30" t="str">
+      <x:c r="B14" s="31" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C14" s="31"/>
+      <x:c r="D14" s="31"/>
+      <x:c r="E14" s="31"/>
+      <x:c r="F14" s="31"/>
+      <x:c r="G14" s="31"/>
+      <x:c r="H14" s="31"/>
+      <x:c r="I14" s="31"/>
+      <x:c r="J14" s="32" t="n">
+        <x:f>SUM(J4:J11)</x:f>
+        <x:v>1596</x:v>
+      </x:c>
+      <x:c r="K14" s="31"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="30" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B13" s="31"/>
-      <x:c r="C13" s="31"/>
-      <x:c r="D13" s="31"/>
-      <x:c r="E13" s="31"/>
-      <x:c r="F13" s="31"/>
-      <x:c r="G13" s="31"/>
-      <x:c r="H13" s="31"/>
-      <x:c r="I13" s="31"/>
-      <x:c r="J13" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J9),0),1)</x:f>
-        <x:v>182.5</x:v>
-      </x:c>
-      <x:c r="K13" s="31"/>
+      <x:c r="B15" s="31"/>
+      <x:c r="C15" s="31"/>
+      <x:c r="D15" s="31"/>
+      <x:c r="E15" s="31"/>
+      <x:c r="F15" s="31"/>
+      <x:c r="G15" s="31"/>
+      <x:c r="H15" s="31"/>
+      <x:c r="I15" s="31"/>
+      <x:c r="J15" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
+        <x:v>199.5</x:v>
+      </x:c>
+      <x:c r="K15" s="31"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2442,9 +2618,7 @@
       <x:c r="G10" s="22" t="n">
         <x:v>8502.4</x:v>
       </x:c>
-      <x:c r="H10" s="25" t="n">
-        <x:v>247.2</x:v>
-      </x:c>
+      <x:c r="H10" s="22"/>
       <x:c r="I10" s="23" t="n">
         <x:v>0.029944762089349597</x:v>
       </x:c>
@@ -2456,31 +2630,47 @@
         <x:v>IC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="30" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B13" s="31" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C13" s="31"/>
-      <x:c r="D13" s="31"/>
-      <x:c r="E13" s="31"/>
-      <x:c r="F13" s="31"/>
-      <x:c r="G13" s="31"/>
-      <x:c r="H13" s="31"/>
-      <x:c r="I13" s="31"/>
-      <x:c r="J13" s="32" t="n">
-        <x:f>SUM(J4:J10)</x:f>
-        <x:v>1561.4</x:v>
-      </x:c>
-      <x:c r="K13" s="31"/>
+    <x:row r="11">
+      <x:c r="A11" s="21" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B11" s="21" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C11" s="21" t="str">
+        <x:v>7月10日</x:v>
+      </x:c>
+      <x:c r="D11" s="22" t="n">
+        <x:v>8522</x:v>
+      </x:c>
+      <x:c r="E11" s="22" t="n">
+        <x:v>8618</x:v>
+      </x:c>
+      <x:c r="F11" s="22" t="n">
+        <x:v>8330</x:v>
+      </x:c>
+      <x:c r="G11" s="22" t="n">
+        <x:v>8333</x:v>
+      </x:c>
+      <x:c r="H11" s="22"/>
+      <x:c r="I11" s="23" t="n">
+        <x:v>-0.019923786225065854</x:v>
+      </x:c>
+      <x:c r="J11" s="27" t="n">
+        <x:f>ROUND(E11-F11,1)</x:f>
+        <x:v>288</x:v>
+      </x:c>
+      <x:c r="K11" s="21" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="30" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B14" s="31"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B14" s="31" t="n">
+        <x:v>8</x:v>
+      </x:c>
       <x:c r="C14" s="31"/>
       <x:c r="D14" s="31"/>
       <x:c r="E14" s="31"/>
@@ -2488,11 +2678,29 @@
       <x:c r="G14" s="31"/>
       <x:c r="H14" s="31"/>
       <x:c r="I14" s="31"/>
-      <x:c r="J14" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J10),0),1)</x:f>
-        <x:v>223.1</x:v>
+      <x:c r="J14" s="32" t="n">
+        <x:f>SUM(J4:J11)</x:f>
+        <x:v>1849.4</x:v>
       </x:c>
       <x:c r="K14" s="31"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="30" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B15" s="31"/>
+      <x:c r="C15" s="31"/>
+      <x:c r="D15" s="31"/>
+      <x:c r="E15" s="31"/>
+      <x:c r="F15" s="31"/>
+      <x:c r="G15" s="31"/>
+      <x:c r="H15" s="31"/>
+      <x:c r="I15" s="31"/>
+      <x:c r="J15" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
+        <x:v>231.2</x:v>
+      </x:c>
+      <x:c r="K15" s="31"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2763,43 +2971,111 @@
         <x:v>IF2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="30" t="str">
+    <x:row r="10">
+      <x:c r="A10" s="21" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B10" s="21" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C10" s="21" t="str">
+        <x:v>7月9日</x:v>
+      </x:c>
+      <x:c r="D10" s="22" t="n">
+        <x:v>4690</x:v>
+      </x:c>
+      <x:c r="E10" s="22" t="n">
+        <x:v>4804</x:v>
+      </x:c>
+      <x:c r="F10" s="22" t="n">
+        <x:v>4665.2</x:v>
+      </x:c>
+      <x:c r="G10" s="22" t="n">
+        <x:v>4780.8</x:v>
+      </x:c>
+      <x:c r="H10" s="22"/>
+      <x:c r="I10" s="23" t="n">
+        <x:v>0.02416452442159378</x:v>
+      </x:c>
+      <x:c r="J10" s="27" t="n">
+        <x:f>ROUND(E10-F10,1)</x:f>
+        <x:v>138.8</x:v>
+      </x:c>
+      <x:c r="K10" s="21" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="21" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B11" s="21" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C11" s="21" t="str">
+        <x:v>7月10日</x:v>
+      </x:c>
+      <x:c r="D11" s="22" t="n">
+        <x:v>4790.2</x:v>
+      </x:c>
+      <x:c r="E11" s="22" t="n">
+        <x:v>4822.2</x:v>
+      </x:c>
+      <x:c r="F11" s="22" t="n">
+        <x:v>4703.6</x:v>
+      </x:c>
+      <x:c r="G11" s="22" t="n">
+        <x:v>4704.6</x:v>
+      </x:c>
+      <x:c r="H11" s="22"/>
+      <x:c r="I11" s="23" t="n">
+        <x:v>-0.015938755020080242</x:v>
+      </x:c>
+      <x:c r="J11" s="27" t="n">
+        <x:f>ROUND(E11-F11,1)</x:f>
+        <x:v>118.6</x:v>
+      </x:c>
+      <x:c r="K11" s="21" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="30" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B12" s="31" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="C12" s="31"/>
-      <x:c r="D12" s="31"/>
-      <x:c r="E12" s="31"/>
-      <x:c r="F12" s="31"/>
-      <x:c r="G12" s="31"/>
-      <x:c r="H12" s="31"/>
-      <x:c r="I12" s="31"/>
-      <x:c r="J12" s="32" t="n">
-        <x:f>SUM(J4:J9)</x:f>
-        <x:v>518</x:v>
-      </x:c>
-      <x:c r="K12" s="31"/>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="30" t="str">
+      <x:c r="B14" s="31" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C14" s="31"/>
+      <x:c r="D14" s="31"/>
+      <x:c r="E14" s="31"/>
+      <x:c r="F14" s="31"/>
+      <x:c r="G14" s="31"/>
+      <x:c r="H14" s="31"/>
+      <x:c r="I14" s="31"/>
+      <x:c r="J14" s="32" t="n">
+        <x:f>SUM(J4:J11)</x:f>
+        <x:v>775.4</x:v>
+      </x:c>
+      <x:c r="K14" s="31"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="30" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B13" s="31"/>
-      <x:c r="C13" s="31"/>
-      <x:c r="D13" s="31"/>
-      <x:c r="E13" s="31"/>
-      <x:c r="F13" s="31"/>
-      <x:c r="G13" s="31"/>
-      <x:c r="H13" s="31"/>
-      <x:c r="I13" s="31"/>
-      <x:c r="J13" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J9),0),1)</x:f>
-        <x:v>86.3</x:v>
-      </x:c>
-      <x:c r="K13" s="31"/>
+      <x:c r="B15" s="31"/>
+      <x:c r="C15" s="31"/>
+      <x:c r="D15" s="31"/>
+      <x:c r="E15" s="31"/>
+      <x:c r="F15" s="31"/>
+      <x:c r="G15" s="31"/>
+      <x:c r="H15" s="31"/>
+      <x:c r="I15" s="31"/>
+      <x:c r="J15" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
+        <x:v>96.9</x:v>
+      </x:c>
+      <x:c r="K15" s="31"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3092,9 +3368,7 @@
       <x:c r="G10" s="22" t="n">
         <x:v>2939.8</x:v>
       </x:c>
-      <x:c r="H10" s="22" t="n">
-        <x:v>71.8</x:v>
-      </x:c>
+      <x:c r="H10" s="22"/>
       <x:c r="I10" s="23" t="n">
         <x:v>0.025034867503486824</x:v>
       </x:c>
@@ -3106,31 +3380,47 @@
         <x:v>IH2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="30" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B13" s="31" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C13" s="31"/>
-      <x:c r="D13" s="31"/>
-      <x:c r="E13" s="31"/>
-      <x:c r="F13" s="31"/>
-      <x:c r="G13" s="31"/>
-      <x:c r="H13" s="31"/>
-      <x:c r="I13" s="31"/>
-      <x:c r="J13" s="32" t="n">
-        <x:f>SUM(J4:J10)</x:f>
-        <x:v>368.79999999999995</x:v>
-      </x:c>
-      <x:c r="K13" s="31"/>
+    <x:row r="11">
+      <x:c r="A11" s="21" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B11" s="21" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C11" s="21" t="str">
+        <x:v>7月10日</x:v>
+      </x:c>
+      <x:c r="D11" s="22" t="n">
+        <x:v>2945.2</x:v>
+      </x:c>
+      <x:c r="E11" s="22" t="n">
+        <x:v>2983.8</x:v>
+      </x:c>
+      <x:c r="F11" s="22" t="n">
+        <x:v>2908.2</x:v>
+      </x:c>
+      <x:c r="G11" s="22" t="n">
+        <x:v>2910.2</x:v>
+      </x:c>
+      <x:c r="H11" s="22"/>
+      <x:c r="I11" s="23" t="n">
+        <x:v>-0.010068712157289772</x:v>
+      </x:c>
+      <x:c r="J11" s="27" t="n">
+        <x:f>ROUND(E11-F11,1)</x:f>
+        <x:v>75.6</x:v>
+      </x:c>
+      <x:c r="K11" s="21" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="30" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B14" s="31"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B14" s="31" t="n">
+        <x:v>8</x:v>
+      </x:c>
       <x:c r="C14" s="31"/>
       <x:c r="D14" s="31"/>
       <x:c r="E14" s="31"/>
@@ -3138,11 +3428,29 @@
       <x:c r="G14" s="31"/>
       <x:c r="H14" s="31"/>
       <x:c r="I14" s="31"/>
-      <x:c r="J14" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J10),0),1)</x:f>
-        <x:v>52.7</x:v>
+      <x:c r="J14" s="32" t="n">
+        <x:f>SUM(J4:J11)</x:f>
+        <x:v>444.4</x:v>
       </x:c>
       <x:c r="K14" s="31"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="30" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B15" s="31"/>
+      <x:c r="C15" s="31"/>
+      <x:c r="D15" s="31"/>
+      <x:c r="E15" s="31"/>
+      <x:c r="F15" s="31"/>
+      <x:c r="G15" s="31"/>
+      <x:c r="H15" s="31"/>
+      <x:c r="I15" s="31"/>
+      <x:c r="J15" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
+        <x:v>55.6</x:v>
+      </x:c>
+      <x:c r="K15" s="31"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-07-16
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R2b9264bc3d524f00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="2" r:id="Ra0d1703e15c2454b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="3" r:id="R9c4c00a23d814e12"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="4" r:id="R0592a88082344fff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="5" r:id="R953a07066a034f30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="6" r:id="R60c15dce550b40be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="7" r:id="R937022fb83b1413a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="8" r:id="R9839bde03dbd4c72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R60c9281a5acb47d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="2" r:id="R32a9d8b7ac134401"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="3" r:id="Rb5fe1f3718c34605"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="4" r:id="Rc1112e54eaf04081"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="5" r:id="Re119cce047e34857"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="6" r:id="R964a75b7476743d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="7" r:id="Ra2fb89318cab416b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="8" r:id="R8e6663f6f95b44d2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -469,25 +469,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-07-10</x:v>
+        <x:v>2026-07-16</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>8438.194</x:v>
+        <x:v>7836.39</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>8198.308</x:v>
+        <x:v>7591.421</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>239.9</x:v>
+        <x:v>245</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>1860.8</x:v>
+        <x:v>2980.3</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>232.6</x:v>
+        <x:v>248.4</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -498,25 +498,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-07-10</x:v>
+        <x:v>2026-07-16</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>8783.249</x:v>
+        <x:v>8148.042</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>8503.245</x:v>
+        <x:v>7907.097</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>280</x:v>
+        <x:v>240.9</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>2024.5</x:v>
+        <x:v>3125.3</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>253.1</x:v>
+        <x:v>260.4</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -527,25 +527,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-07-10</x:v>
+        <x:v>2026-07-16</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>4074.828</x:v>
+        <x:v>3940.451</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3995.807</x:v>
+        <x:v>3867.601</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>79</x:v>
+        <x:v>72.8</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>517.2</x:v>
+        <x:v>808.2</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>64.7</x:v>
+        <x:v>67.4</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -556,25 +556,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-07-10</x:v>
+        <x:v>2026-07-16</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>8244.8</x:v>
+        <x:v>7750.2</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>8016</x:v>
+        <x:v>7511</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>228.8</x:v>
+        <x:v>239.2</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>1596</x:v>
+        <x:v>2629.2</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>199.5</x:v>
+        <x:v>219.1</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -585,25 +585,25 @@
         <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>2026-07-10</x:v>
+        <x:v>2026-07-16</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:v>8618</x:v>
+        <x:v>8054.4</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>8330</x:v>
+        <x:v>7823</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>288</x:v>
+        <x:v>231.4</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>1849.4</x:v>
+        <x:v>2906.4</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
-        <x:v>231.2</x:v>
+        <x:v>242.2</x:v>
       </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
@@ -614,25 +614,25 @@
         <x:v>IF主力</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>2026-07-10</x:v>
+        <x:v>2026-07-16</x:v>
       </x:c>
       <x:c r="C9" s="10" t="n">
-        <x:v>4822.2</x:v>
+        <x:v>4712.6</x:v>
       </x:c>
       <x:c r="D9" s="10" t="n">
-        <x:v>4703.6</x:v>
+        <x:v>4618</x:v>
       </x:c>
       <x:c r="E9" s="12" t="n">
-        <x:v>118.6</x:v>
+        <x:v>94.6</x:v>
       </x:c>
       <x:c r="F9" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G9" s="10" t="n">
-        <x:v>775.4</x:v>
+        <x:v>1133.8</x:v>
       </x:c>
       <x:c r="H9" s="10" t="n">
-        <x:v>96.9</x:v>
+        <x:v>94.5</x:v>
       </x:c>
       <x:c r="I9" s="10" t="n">
         <x:v>90</x:v>
@@ -643,25 +643,25 @@
         <x:v>IH主力</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>2026-07-10</x:v>
+        <x:v>2026-07-16</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:v>2983.8</x:v>
+        <x:v>2911.8</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
-        <x:v>2908.2</x:v>
+        <x:v>2853.4</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
-        <x:v>75.6</x:v>
+        <x:v>58.4</x:v>
       </x:c>
       <x:c r="F10" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G10" s="10" t="n">
-        <x:v>444.4</x:v>
+        <x:v>649</x:v>
       </x:c>
       <x:c r="H10" s="10" t="n">
-        <x:v>55.6</x:v>
+        <x:v>54.1</x:v>
       </x:c>
       <x:c r="I10" s="10" t="n">
         <x:v>60</x:v>
@@ -675,7 +675,7 @@
         <x:v>2026-07-01</x:v>
       </x:c>
       <x:c r="C13" s="14" t="str">
-        <x:v>2026-07-10</x:v>
+        <x:v>2026-07-16</x:v>
       </x:c>
       <x:c r="D13" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1132,43 +1132,187 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="21" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B12" s="21" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C12" s="21" t="str">
+        <x:v>7月13日</x:v>
+      </x:c>
+      <x:c r="D12" s="22" t="n">
+        <x:v>8124.363</x:v>
+      </x:c>
+      <x:c r="E12" s="22" t="n">
+        <x:v>8171.504</x:v>
+      </x:c>
+      <x:c r="F12" s="22" t="n">
+        <x:v>7769.292</x:v>
+      </x:c>
+      <x:c r="G12" s="22" t="n">
+        <x:v>7787.853</x:v>
+      </x:c>
+      <x:c r="H12" s="25" t="n">
+        <x:v>-410.5</x:v>
+      </x:c>
+      <x:c r="I12" s="23" t="n">
+        <x:v>-0.050065818459126055</x:v>
+      </x:c>
+      <x:c r="J12" s="27" t="n">
+        <x:f>ROUND(E12-F12,1)</x:f>
+        <x:v>402.2</x:v>
+      </x:c>
+      <x:c r="K12" s="21" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="21" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B13" s="21" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C13" s="21" t="str">
+        <x:v>7月14日</x:v>
+      </x:c>
+      <x:c r="D13" s="22" t="n">
+        <x:v>7799.813</x:v>
+      </x:c>
+      <x:c r="E13" s="22" t="n">
+        <x:v>7934.103</x:v>
+      </x:c>
+      <x:c r="F13" s="22" t="n">
+        <x:v>7657.671</x:v>
+      </x:c>
+      <x:c r="G13" s="22" t="n">
+        <x:v>7925.123</x:v>
+      </x:c>
+      <x:c r="H13" s="22" t="n">
+        <x:v>137.3</x:v>
+      </x:c>
+      <x:c r="I13" s="23" t="n">
+        <x:v>0.017626167314662933</x:v>
+      </x:c>
+      <x:c r="J13" s="27" t="n">
+        <x:f>ROUND(E13-F13,1)</x:f>
+        <x:v>276.4</x:v>
+      </x:c>
+      <x:c r="K13" s="21" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
+    </x:row>
     <x:row r="14">
-      <x:c r="A14" s="30" t="str">
+      <x:c r="A14" s="21" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B14" s="21" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C14" s="21" t="str">
+        <x:v>7月15日</x:v>
+      </x:c>
+      <x:c r="D14" s="22" t="n">
+        <x:v>7959.374</x:v>
+      </x:c>
+      <x:c r="E14" s="22" t="n">
+        <x:v>7979.077</x:v>
+      </x:c>
+      <x:c r="F14" s="22" t="n">
+        <x:v>7783.219</x:v>
+      </x:c>
+      <x:c r="G14" s="22" t="n">
+        <x:v>7817.831</x:v>
+      </x:c>
+      <x:c r="H14" s="22" t="n">
+        <x:v>-107.3</x:v>
+      </x:c>
+      <x:c r="I14" s="23" t="n">
+        <x:v>-0.01353821259304111</x:v>
+      </x:c>
+      <x:c r="J14" s="27" t="n">
+        <x:f>ROUND(E14-F14,1)</x:f>
+        <x:v>195.9</x:v>
+      </x:c>
+      <x:c r="K14" s="21" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="21" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B15" s="21" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C15" s="21" t="str">
+        <x:v>7月16日</x:v>
+      </x:c>
+      <x:c r="D15" s="22" t="n">
+        <x:v>7713.135</x:v>
+      </x:c>
+      <x:c r="E15" s="22" t="n">
+        <x:v>7836.39</x:v>
+      </x:c>
+      <x:c r="F15" s="22" t="n">
+        <x:v>7591.421</x:v>
+      </x:c>
+      <x:c r="G15" s="22" t="n">
+        <x:v>7631.762</x:v>
+      </x:c>
+      <x:c r="H15" s="25" t="n">
+        <x:v>-186.1</x:v>
+      </x:c>
+      <x:c r="I15" s="23" t="n">
+        <x:v>-0.02380059123815803</x:v>
+      </x:c>
+      <x:c r="J15" s="27" t="n">
+        <x:f>ROUND(E15-F15,1)</x:f>
+        <x:v>245</x:v>
+      </x:c>
+      <x:c r="K15" s="21" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="30" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B14" s="31" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C14" s="31"/>
-      <x:c r="D14" s="31"/>
-      <x:c r="E14" s="31"/>
-      <x:c r="F14" s="31"/>
-      <x:c r="G14" s="31"/>
-      <x:c r="H14" s="31"/>
-      <x:c r="I14" s="31"/>
-      <x:c r="J14" s="32" t="n">
-        <x:f>SUM(J4:J11)</x:f>
-        <x:v>1860.8</x:v>
-      </x:c>
-      <x:c r="K14" s="31"/>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="30" t="str">
+      <x:c r="B18" s="31" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C18" s="31"/>
+      <x:c r="D18" s="31"/>
+      <x:c r="E18" s="31"/>
+      <x:c r="F18" s="31"/>
+      <x:c r="G18" s="31"/>
+      <x:c r="H18" s="31"/>
+      <x:c r="I18" s="31"/>
+      <x:c r="J18" s="32" t="n">
+        <x:f>SUM(J4:J15)</x:f>
+        <x:v>2980.3</x:v>
+      </x:c>
+      <x:c r="K18" s="31"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="30" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B15" s="31"/>
-      <x:c r="C15" s="31"/>
-      <x:c r="D15" s="31"/>
-      <x:c r="E15" s="31"/>
-      <x:c r="F15" s="31"/>
-      <x:c r="G15" s="31"/>
-      <x:c r="H15" s="31"/>
-      <x:c r="I15" s="31"/>
-      <x:c r="J15" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
-        <x:v>232.6</x:v>
-      </x:c>
-      <x:c r="K15" s="31"/>
+      <x:c r="B19" s="31"/>
+      <x:c r="C19" s="31"/>
+      <x:c r="D19" s="31"/>
+      <x:c r="E19" s="31"/>
+      <x:c r="F19" s="31"/>
+      <x:c r="G19" s="31"/>
+      <x:c r="H19" s="31"/>
+      <x:c r="I19" s="31"/>
+      <x:c r="J19" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
+        <x:v>248.4</x:v>
+      </x:c>
+      <x:c r="K19" s="31"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1523,43 +1667,187 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="21" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B12" s="21" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C12" s="21" t="str">
+        <x:v>7月13日</x:v>
+      </x:c>
+      <x:c r="D12" s="22" t="n">
+        <x:v>8409.143</x:v>
+      </x:c>
+      <x:c r="E12" s="22" t="n">
+        <x:v>8457.692</x:v>
+      </x:c>
+      <x:c r="F12" s="22" t="n">
+        <x:v>8106.269</x:v>
+      </x:c>
+      <x:c r="G12" s="22" t="n">
+        <x:v>8138.144</x:v>
+      </x:c>
+      <x:c r="H12" s="25" t="n">
+        <x:v>-365.8</x:v>
+      </x:c>
+      <x:c r="I12" s="23" t="n">
+        <x:v>-0.04301837341637216</x:v>
+      </x:c>
+      <x:c r="J12" s="27" t="n">
+        <x:f>ROUND(E12-F12,1)</x:f>
+        <x:v>351.4</x:v>
+      </x:c>
+      <x:c r="K12" s="21" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="21" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B13" s="21" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C13" s="21" t="str">
+        <x:v>7月14日</x:v>
+      </x:c>
+      <x:c r="D13" s="22" t="n">
+        <x:v>8135.046</x:v>
+      </x:c>
+      <x:c r="E13" s="22" t="n">
+        <x:v>8275.96</x:v>
+      </x:c>
+      <x:c r="F13" s="22" t="n">
+        <x:v>7955.308</x:v>
+      </x:c>
+      <x:c r="G13" s="22" t="n">
+        <x:v>8275.939</x:v>
+      </x:c>
+      <x:c r="H13" s="22" t="n">
+        <x:v>137.8</x:v>
+      </x:c>
+      <x:c r="I13" s="23" t="n">
+        <x:v>0.016931993339021734</x:v>
+      </x:c>
+      <x:c r="J13" s="27" t="n">
+        <x:f>ROUND(E13-F13,1)</x:f>
+        <x:v>320.7</x:v>
+      </x:c>
+      <x:c r="K13" s="21" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+    </x:row>
     <x:row r="14">
-      <x:c r="A14" s="30" t="str">
+      <x:c r="A14" s="21" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B14" s="21" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C14" s="21" t="str">
+        <x:v>7月15日</x:v>
+      </x:c>
+      <x:c r="D14" s="22" t="n">
+        <x:v>8294.142</x:v>
+      </x:c>
+      <x:c r="E14" s="22" t="n">
+        <x:v>8305.272</x:v>
+      </x:c>
+      <x:c r="F14" s="22" t="n">
+        <x:v>8117.459</x:v>
+      </x:c>
+      <x:c r="G14" s="22" t="n">
+        <x:v>8147.579</x:v>
+      </x:c>
+      <x:c r="H14" s="22" t="n">
+        <x:v>-128.4</x:v>
+      </x:c>
+      <x:c r="I14" s="23" t="n">
+        <x:v>-0.015510022488082642</x:v>
+      </x:c>
+      <x:c r="J14" s="27" t="n">
+        <x:f>ROUND(E14-F14,1)</x:f>
+        <x:v>187.8</x:v>
+      </x:c>
+      <x:c r="K14" s="21" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="21" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B15" s="21" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C15" s="21" t="str">
+        <x:v>7月16日</x:v>
+      </x:c>
+      <x:c r="D15" s="22" t="n">
+        <x:v>8006.449</x:v>
+      </x:c>
+      <x:c r="E15" s="22" t="n">
+        <x:v>8148.042</x:v>
+      </x:c>
+      <x:c r="F15" s="22" t="n">
+        <x:v>7907.097</x:v>
+      </x:c>
+      <x:c r="G15" s="22" t="n">
+        <x:v>7955.664</x:v>
+      </x:c>
+      <x:c r="H15" s="25" t="n">
+        <x:v>-191.9</x:v>
+      </x:c>
+      <x:c r="I15" s="23" t="n">
+        <x:v>-0.02355484985171663</x:v>
+      </x:c>
+      <x:c r="J15" s="27" t="n">
+        <x:f>ROUND(E15-F15,1)</x:f>
+        <x:v>240.9</x:v>
+      </x:c>
+      <x:c r="K15" s="21" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="30" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B14" s="31" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C14" s="31"/>
-      <x:c r="D14" s="31"/>
-      <x:c r="E14" s="31"/>
-      <x:c r="F14" s="31"/>
-      <x:c r="G14" s="31"/>
-      <x:c r="H14" s="31"/>
-      <x:c r="I14" s="31"/>
-      <x:c r="J14" s="32" t="n">
-        <x:f>SUM(J4:J11)</x:f>
-        <x:v>2024.5</x:v>
-      </x:c>
-      <x:c r="K14" s="31"/>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="30" t="str">
+      <x:c r="B18" s="31" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C18" s="31"/>
+      <x:c r="D18" s="31"/>
+      <x:c r="E18" s="31"/>
+      <x:c r="F18" s="31"/>
+      <x:c r="G18" s="31"/>
+      <x:c r="H18" s="31"/>
+      <x:c r="I18" s="31"/>
+      <x:c r="J18" s="32" t="n">
+        <x:f>SUM(J4:J15)</x:f>
+        <x:v>3125.3</x:v>
+      </x:c>
+      <x:c r="K18" s="31"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="30" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B15" s="31"/>
-      <x:c r="C15" s="31"/>
-      <x:c r="D15" s="31"/>
-      <x:c r="E15" s="31"/>
-      <x:c r="F15" s="31"/>
-      <x:c r="G15" s="31"/>
-      <x:c r="H15" s="31"/>
-      <x:c r="I15" s="31"/>
-      <x:c r="J15" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
-        <x:v>253.1</x:v>
-      </x:c>
-      <x:c r="K15" s="31"/>
+      <x:c r="B19" s="31"/>
+      <x:c r="C19" s="31"/>
+      <x:c r="D19" s="31"/>
+      <x:c r="E19" s="31"/>
+      <x:c r="F19" s="31"/>
+      <x:c r="G19" s="31"/>
+      <x:c r="H19" s="31"/>
+      <x:c r="I19" s="31"/>
+      <x:c r="J19" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
+        <x:v>260.4</x:v>
+      </x:c>
+      <x:c r="K19" s="31"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1914,43 +2202,187 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="21" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B12" s="21" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C12" s="21" t="str">
+        <x:v>7月13日</x:v>
+      </x:c>
+      <x:c r="D12" s="22" t="n">
+        <x:v>3966.023</x:v>
+      </x:c>
+      <x:c r="E12" s="22" t="n">
+        <x:v>3983.054</x:v>
+      </x:c>
+      <x:c r="F12" s="22" t="n">
+        <x:v>3900.668</x:v>
+      </x:c>
+      <x:c r="G12" s="22" t="n">
+        <x:v>3913.794</x:v>
+      </x:c>
+      <x:c r="H12" s="22" t="n">
+        <x:v>-82.4</x:v>
+      </x:c>
+      <x:c r="I12" s="23" t="n">
+        <x:v>-0.020611777000031473</x:v>
+      </x:c>
+      <x:c r="J12" s="27" t="n">
+        <x:f>ROUND(E12-F12,1)</x:f>
+        <x:v>82.4</x:v>
+      </x:c>
+      <x:c r="K12" s="21" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="21" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B13" s="21" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C13" s="21" t="str">
+        <x:v>7月14日</x:v>
+      </x:c>
+      <x:c r="D13" s="22" t="n">
+        <x:v>3909.274</x:v>
+      </x:c>
+      <x:c r="E13" s="22" t="n">
+        <x:v>3967.126</x:v>
+      </x:c>
+      <x:c r="F13" s="22" t="n">
+        <x:v>3869.304</x:v>
+      </x:c>
+      <x:c r="G13" s="22" t="n">
+        <x:v>3967.126</x:v>
+      </x:c>
+      <x:c r="H13" s="22" t="n">
+        <x:v>53.3</x:v>
+      </x:c>
+      <x:c r="I13" s="23" t="n">
+        <x:v>0.01362667529256778</x:v>
+      </x:c>
+      <x:c r="J13" s="27" t="n">
+        <x:f>ROUND(E13-F13,1)</x:f>
+        <x:v>97.8</x:v>
+      </x:c>
+      <x:c r="K13" s="21" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+    </x:row>
     <x:row r="14">
-      <x:c r="A14" s="30" t="str">
+      <x:c r="A14" s="21" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B14" s="21" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C14" s="21" t="str">
+        <x:v>7月15日</x:v>
+      </x:c>
+      <x:c r="D14" s="22" t="n">
+        <x:v>3963.727</x:v>
+      </x:c>
+      <x:c r="E14" s="22" t="n">
+        <x:v>3981.672</x:v>
+      </x:c>
+      <x:c r="F14" s="22" t="n">
+        <x:v>3943.695</x:v>
+      </x:c>
+      <x:c r="G14" s="22" t="n">
+        <x:v>3955.578</x:v>
+      </x:c>
+      <x:c r="H14" s="22" t="n">
+        <x:v>-11.5</x:v>
+      </x:c>
+      <x:c r="I14" s="23" t="n">
+        <x:v>-0.002910923424161549</x:v>
+      </x:c>
+      <x:c r="J14" s="22" t="n">
+        <x:f>ROUND(E14-F14,1)</x:f>
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="K14" s="21" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="21" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B15" s="21" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C15" s="21" t="str">
+        <x:v>7月16日</x:v>
+      </x:c>
+      <x:c r="D15" s="22" t="n">
+        <x:v>3912.381</x:v>
+      </x:c>
+      <x:c r="E15" s="22" t="n">
+        <x:v>3940.451</x:v>
+      </x:c>
+      <x:c r="F15" s="22" t="n">
+        <x:v>3867.601</x:v>
+      </x:c>
+      <x:c r="G15" s="22" t="n">
+        <x:v>3882.413</x:v>
+      </x:c>
+      <x:c r="H15" s="22" t="n">
+        <x:v>-73.2</x:v>
+      </x:c>
+      <x:c r="I15" s="23" t="n">
+        <x:v>-0.01849666470993616</x:v>
+      </x:c>
+      <x:c r="J15" s="27" t="n">
+        <x:f>ROUND(E15-F15,1)</x:f>
+        <x:v>72.8</x:v>
+      </x:c>
+      <x:c r="K15" s="21" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="30" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B14" s="31" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C14" s="31"/>
-      <x:c r="D14" s="31"/>
-      <x:c r="E14" s="31"/>
-      <x:c r="F14" s="31"/>
-      <x:c r="G14" s="31"/>
-      <x:c r="H14" s="31"/>
-      <x:c r="I14" s="31"/>
-      <x:c r="J14" s="32" t="n">
-        <x:f>SUM(J4:J11)</x:f>
-        <x:v>517.2</x:v>
-      </x:c>
-      <x:c r="K14" s="31"/>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="30" t="str">
+      <x:c r="B18" s="31" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C18" s="31"/>
+      <x:c r="D18" s="31"/>
+      <x:c r="E18" s="31"/>
+      <x:c r="F18" s="31"/>
+      <x:c r="G18" s="31"/>
+      <x:c r="H18" s="31"/>
+      <x:c r="I18" s="31"/>
+      <x:c r="J18" s="32" t="n">
+        <x:f>SUM(J4:J15)</x:f>
+        <x:v>808.1999999999999</x:v>
+      </x:c>
+      <x:c r="K18" s="31"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="30" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B15" s="31"/>
-      <x:c r="C15" s="31"/>
-      <x:c r="D15" s="31"/>
-      <x:c r="E15" s="31"/>
-      <x:c r="F15" s="31"/>
-      <x:c r="G15" s="31"/>
-      <x:c r="H15" s="31"/>
-      <x:c r="I15" s="31"/>
-      <x:c r="J15" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
-        <x:v>64.7</x:v>
-      </x:c>
-      <x:c r="K15" s="31"/>
+      <x:c r="B19" s="31"/>
+      <x:c r="C19" s="31"/>
+      <x:c r="D19" s="31"/>
+      <x:c r="E19" s="31"/>
+      <x:c r="F19" s="31"/>
+      <x:c r="G19" s="31"/>
+      <x:c r="H19" s="31"/>
+      <x:c r="I19" s="31"/>
+      <x:c r="J19" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
+        <x:v>67.4</x:v>
+      </x:c>
+      <x:c r="K19" s="31"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2289,43 +2721,179 @@
         <x:v>IM2609</x:v>
       </x:c>
     </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="21" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B12" s="21" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C12" s="21" t="str">
+        <x:v>7月13日</x:v>
+      </x:c>
+      <x:c r="D12" s="22" t="n">
+        <x:v>7995</x:v>
+      </x:c>
+      <x:c r="E12" s="22" t="n">
+        <x:v>8029.8</x:v>
+      </x:c>
+      <x:c r="F12" s="22" t="n">
+        <x:v>7651</x:v>
+      </x:c>
+      <x:c r="G12" s="22" t="n">
+        <x:v>7684.4</x:v>
+      </x:c>
+      <x:c r="H12" s="22"/>
+      <x:c r="I12" s="23" t="n">
+        <x:v>-0.04177369878045745</x:v>
+      </x:c>
+      <x:c r="J12" s="27" t="n">
+        <x:f>ROUND(E12-F12,1)</x:f>
+        <x:v>378.8</x:v>
+      </x:c>
+      <x:c r="K12" s="21" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="21" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B13" s="21" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C13" s="21" t="str">
+        <x:v>7月14日</x:v>
+      </x:c>
+      <x:c r="D13" s="22" t="n">
+        <x:v>7720</x:v>
+      </x:c>
+      <x:c r="E13" s="22" t="n">
+        <x:v>7810.6</x:v>
+      </x:c>
+      <x:c r="F13" s="22" t="n">
+        <x:v>7580</x:v>
+      </x:c>
+      <x:c r="G13" s="22" t="n">
+        <x:v>7788</x:v>
+      </x:c>
+      <x:c r="H13" s="22"/>
+      <x:c r="I13" s="23" t="n">
+        <x:v>0.013481859351413217</x:v>
+      </x:c>
+      <x:c r="J13" s="27" t="n">
+        <x:f>ROUND(E13-F13,1)</x:f>
+        <x:v>230.6</x:v>
+      </x:c>
+      <x:c r="K13" s="21" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+    </x:row>
     <x:row r="14">
-      <x:c r="A14" s="30" t="str">
+      <x:c r="A14" s="21" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B14" s="21" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C14" s="21" t="str">
+        <x:v>7月15日</x:v>
+      </x:c>
+      <x:c r="D14" s="22" t="n">
+        <x:v>7838</x:v>
+      </x:c>
+      <x:c r="E14" s="22" t="n">
+        <x:v>7846</x:v>
+      </x:c>
+      <x:c r="F14" s="22" t="n">
+        <x:v>7661.4</x:v>
+      </x:c>
+      <x:c r="G14" s="22" t="n">
+        <x:v>7723.2</x:v>
+      </x:c>
+      <x:c r="H14" s="22"/>
+      <x:c r="I14" s="23" t="n">
+        <x:v>-0.008320493066255819</x:v>
+      </x:c>
+      <x:c r="J14" s="22" t="n">
+        <x:f>ROUND(E14-F14,1)</x:f>
+        <x:v>184.6</x:v>
+      </x:c>
+      <x:c r="K14" s="21" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="21" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B15" s="21" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C15" s="21" t="str">
+        <x:v>7月16日</x:v>
+      </x:c>
+      <x:c r="D15" s="22" t="n">
+        <x:v>7648.6</x:v>
+      </x:c>
+      <x:c r="E15" s="22" t="n">
+        <x:v>7750.2</x:v>
+      </x:c>
+      <x:c r="F15" s="22" t="n">
+        <x:v>7511</x:v>
+      </x:c>
+      <x:c r="G15" s="22" t="n">
+        <x:v>7552.6</x:v>
+      </x:c>
+      <x:c r="H15" s="22"/>
+      <x:c r="I15" s="23" t="n">
+        <x:v>-0.022089289413714464</x:v>
+      </x:c>
+      <x:c r="J15" s="27" t="n">
+        <x:f>ROUND(E15-F15,1)</x:f>
+        <x:v>239.2</x:v>
+      </x:c>
+      <x:c r="K15" s="21" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="30" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B14" s="31" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C14" s="31"/>
-      <x:c r="D14" s="31"/>
-      <x:c r="E14" s="31"/>
-      <x:c r="F14" s="31"/>
-      <x:c r="G14" s="31"/>
-      <x:c r="H14" s="31"/>
-      <x:c r="I14" s="31"/>
-      <x:c r="J14" s="32" t="n">
-        <x:f>SUM(J4:J11)</x:f>
-        <x:v>1596</x:v>
-      </x:c>
-      <x:c r="K14" s="31"/>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="30" t="str">
+      <x:c r="B18" s="31" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C18" s="31"/>
+      <x:c r="D18" s="31"/>
+      <x:c r="E18" s="31"/>
+      <x:c r="F18" s="31"/>
+      <x:c r="G18" s="31"/>
+      <x:c r="H18" s="31"/>
+      <x:c r="I18" s="31"/>
+      <x:c r="J18" s="32" t="n">
+        <x:f>SUM(J4:J15)</x:f>
+        <x:v>2629.2</x:v>
+      </x:c>
+      <x:c r="K18" s="31"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="30" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B15" s="31"/>
-      <x:c r="C15" s="31"/>
-      <x:c r="D15" s="31"/>
-      <x:c r="E15" s="31"/>
-      <x:c r="F15" s="31"/>
-      <x:c r="G15" s="31"/>
-      <x:c r="H15" s="31"/>
-      <x:c r="I15" s="31"/>
-      <x:c r="J15" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
-        <x:v>199.5</x:v>
-      </x:c>
-      <x:c r="K15" s="31"/>
+      <x:c r="B19" s="31"/>
+      <x:c r="C19" s="31"/>
+      <x:c r="D19" s="31"/>
+      <x:c r="E19" s="31"/>
+      <x:c r="F19" s="31"/>
+      <x:c r="G19" s="31"/>
+      <x:c r="H19" s="31"/>
+      <x:c r="I19" s="31"/>
+      <x:c r="J19" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
+        <x:v>219.1</x:v>
+      </x:c>
+      <x:c r="K19" s="31"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2664,43 +3232,179 @@
         <x:v>IC2609</x:v>
       </x:c>
     </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="21" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B12" s="21" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C12" s="21" t="str">
+        <x:v>7月13日</x:v>
+      </x:c>
+      <x:c r="D12" s="22" t="n">
+        <x:v>8303</x:v>
+      </x:c>
+      <x:c r="E12" s="22" t="n">
+        <x:v>8328</x:v>
+      </x:c>
+      <x:c r="F12" s="22" t="n">
+        <x:v>7995.8</x:v>
+      </x:c>
+      <x:c r="G12" s="22" t="n">
+        <x:v>8021.6</x:v>
+      </x:c>
+      <x:c r="H12" s="22"/>
+      <x:c r="I12" s="23" t="n">
+        <x:v>-0.037369494779791124</x:v>
+      </x:c>
+      <x:c r="J12" s="27" t="n">
+        <x:f>ROUND(E12-F12,1)</x:f>
+        <x:v>332.2</x:v>
+      </x:c>
+      <x:c r="K12" s="21" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="21" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B13" s="21" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C13" s="21" t="str">
+        <x:v>7月14日</x:v>
+      </x:c>
+      <x:c r="D13" s="22" t="n">
+        <x:v>8043.2</x:v>
+      </x:c>
+      <x:c r="E13" s="22" t="n">
+        <x:v>8166</x:v>
+      </x:c>
+      <x:c r="F13" s="22" t="n">
+        <x:v>7881</x:v>
+      </x:c>
+      <x:c r="G13" s="22" t="n">
+        <x:v>8117</x:v>
+      </x:c>
+      <x:c r="H13" s="22"/>
+      <x:c r="I13" s="23" t="n">
+        <x:v>0.011892889199162315</x:v>
+      </x:c>
+      <x:c r="J13" s="27" t="n">
+        <x:f>ROUND(E13-F13,1)</x:f>
+        <x:v>285</x:v>
+      </x:c>
+      <x:c r="K13" s="21" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+    </x:row>
     <x:row r="14">
-      <x:c r="A14" s="30" t="str">
+      <x:c r="A14" s="21" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B14" s="21" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C14" s="21" t="str">
+        <x:v>7月15日</x:v>
+      </x:c>
+      <x:c r="D14" s="22" t="n">
+        <x:v>8160</x:v>
+      </x:c>
+      <x:c r="E14" s="22" t="n">
+        <x:v>8192.2</x:v>
+      </x:c>
+      <x:c r="F14" s="22" t="n">
+        <x:v>7983.8</x:v>
+      </x:c>
+      <x:c r="G14" s="22" t="n">
+        <x:v>8046.4</x:v>
+      </x:c>
+      <x:c r="H14" s="22"/>
+      <x:c r="I14" s="23" t="n">
+        <x:v>-0.008697794751755583</x:v>
+      </x:c>
+      <x:c r="J14" s="27" t="n">
+        <x:f>ROUND(E14-F14,1)</x:f>
+        <x:v>208.4</x:v>
+      </x:c>
+      <x:c r="K14" s="21" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="21" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B15" s="21" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C15" s="21" t="str">
+        <x:v>7月16日</x:v>
+      </x:c>
+      <x:c r="D15" s="22" t="n">
+        <x:v>7955.4</x:v>
+      </x:c>
+      <x:c r="E15" s="22" t="n">
+        <x:v>8054.4</x:v>
+      </x:c>
+      <x:c r="F15" s="22" t="n">
+        <x:v>7823</x:v>
+      </x:c>
+      <x:c r="G15" s="22" t="n">
+        <x:v>7869.6</x:v>
+      </x:c>
+      <x:c r="H15" s="22"/>
+      <x:c r="I15" s="23" t="n">
+        <x:v>-0.021972559156890004</x:v>
+      </x:c>
+      <x:c r="J15" s="27" t="n">
+        <x:f>ROUND(E15-F15,1)</x:f>
+        <x:v>231.4</x:v>
+      </x:c>
+      <x:c r="K15" s="21" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="30" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B14" s="31" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C14" s="31"/>
-      <x:c r="D14" s="31"/>
-      <x:c r="E14" s="31"/>
-      <x:c r="F14" s="31"/>
-      <x:c r="G14" s="31"/>
-      <x:c r="H14" s="31"/>
-      <x:c r="I14" s="31"/>
-      <x:c r="J14" s="32" t="n">
-        <x:f>SUM(J4:J11)</x:f>
-        <x:v>1849.4</x:v>
-      </x:c>
-      <x:c r="K14" s="31"/>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="30" t="str">
+      <x:c r="B18" s="31" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C18" s="31"/>
+      <x:c r="D18" s="31"/>
+      <x:c r="E18" s="31"/>
+      <x:c r="F18" s="31"/>
+      <x:c r="G18" s="31"/>
+      <x:c r="H18" s="31"/>
+      <x:c r="I18" s="31"/>
+      <x:c r="J18" s="32" t="n">
+        <x:f>SUM(J4:J15)</x:f>
+        <x:v>2906.4</x:v>
+      </x:c>
+      <x:c r="K18" s="31"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="30" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B15" s="31"/>
-      <x:c r="C15" s="31"/>
-      <x:c r="D15" s="31"/>
-      <x:c r="E15" s="31"/>
-      <x:c r="F15" s="31"/>
-      <x:c r="G15" s="31"/>
-      <x:c r="H15" s="31"/>
-      <x:c r="I15" s="31"/>
-      <x:c r="J15" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
-        <x:v>231.2</x:v>
-      </x:c>
-      <x:c r="K15" s="31"/>
+      <x:c r="B19" s="31"/>
+      <x:c r="C19" s="31"/>
+      <x:c r="D19" s="31"/>
+      <x:c r="E19" s="31"/>
+      <x:c r="F19" s="31"/>
+      <x:c r="G19" s="31"/>
+      <x:c r="H19" s="31"/>
+      <x:c r="I19" s="31"/>
+      <x:c r="J19" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
+        <x:v>242.2</x:v>
+      </x:c>
+      <x:c r="K19" s="31"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3039,43 +3743,179 @@
         <x:v>IF2609</x:v>
       </x:c>
     </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="21" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B12" s="21" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C12" s="21" t="str">
+        <x:v>7月13日</x:v>
+      </x:c>
+      <x:c r="D12" s="22" t="n">
+        <x:v>4691</x:v>
+      </x:c>
+      <x:c r="E12" s="22" t="n">
+        <x:v>4705</x:v>
+      </x:c>
+      <x:c r="F12" s="22" t="n">
+        <x:v>4610.2</x:v>
+      </x:c>
+      <x:c r="G12" s="22" t="n">
+        <x:v>4634.6</x:v>
+      </x:c>
+      <x:c r="H12" s="22"/>
+      <x:c r="I12" s="23" t="n">
+        <x:v>-0.014879054542362824</x:v>
+      </x:c>
+      <x:c r="J12" s="27" t="n">
+        <x:f>ROUND(E12-F12,1)</x:f>
+        <x:v>94.8</x:v>
+      </x:c>
+      <x:c r="K12" s="21" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="21" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B13" s="21" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C13" s="21" t="str">
+        <x:v>7月14日</x:v>
+      </x:c>
+      <x:c r="D13" s="22" t="n">
+        <x:v>4640</x:v>
+      </x:c>
+      <x:c r="E13" s="22" t="n">
+        <x:v>4713.2</x:v>
+      </x:c>
+      <x:c r="F13" s="22" t="n">
+        <x:v>4593</x:v>
+      </x:c>
+      <x:c r="G13" s="22" t="n">
+        <x:v>4690</x:v>
+      </x:c>
+      <x:c r="H13" s="22"/>
+      <x:c r="I13" s="23" t="n">
+        <x:v>0.011953566650843683</x:v>
+      </x:c>
+      <x:c r="J13" s="27" t="n">
+        <x:f>ROUND(E13-F13,1)</x:f>
+        <x:v>120.2</x:v>
+      </x:c>
+      <x:c r="K13" s="21" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+    </x:row>
     <x:row r="14">
-      <x:c r="A14" s="30" t="str">
+      <x:c r="A14" s="21" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B14" s="21" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C14" s="21" t="str">
+        <x:v>7月15日</x:v>
+      </x:c>
+      <x:c r="D14" s="22" t="n">
+        <x:v>4706</x:v>
+      </x:c>
+      <x:c r="E14" s="22" t="n">
+        <x:v>4739.4</x:v>
+      </x:c>
+      <x:c r="F14" s="22" t="n">
+        <x:v>4690.6</x:v>
+      </x:c>
+      <x:c r="G14" s="22" t="n">
+        <x:v>4717.4</x:v>
+      </x:c>
+      <x:c r="H14" s="22"/>
+      <x:c r="I14" s="23" t="n">
+        <x:v>0.005842217484008483</x:v>
+      </x:c>
+      <x:c r="J14" s="22" t="n">
+        <x:f>ROUND(E14-F14,1)</x:f>
+        <x:v>48.8</x:v>
+      </x:c>
+      <x:c r="K14" s="21" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="21" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B15" s="21" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C15" s="21" t="str">
+        <x:v>7月16日</x:v>
+      </x:c>
+      <x:c r="D15" s="22" t="n">
+        <x:v>4677</x:v>
+      </x:c>
+      <x:c r="E15" s="22" t="n">
+        <x:v>4712.6</x:v>
+      </x:c>
+      <x:c r="F15" s="22" t="n">
+        <x:v>4618</x:v>
+      </x:c>
+      <x:c r="G15" s="22" t="n">
+        <x:v>4645.6</x:v>
+      </x:c>
+      <x:c r="H15" s="22"/>
+      <x:c r="I15" s="23" t="n">
+        <x:v>-0.015220248441938256</x:v>
+      </x:c>
+      <x:c r="J15" s="27" t="n">
+        <x:f>ROUND(E15-F15,1)</x:f>
+        <x:v>94.6</x:v>
+      </x:c>
+      <x:c r="K15" s="21" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="30" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B14" s="31" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C14" s="31"/>
-      <x:c r="D14" s="31"/>
-      <x:c r="E14" s="31"/>
-      <x:c r="F14" s="31"/>
-      <x:c r="G14" s="31"/>
-      <x:c r="H14" s="31"/>
-      <x:c r="I14" s="31"/>
-      <x:c r="J14" s="32" t="n">
-        <x:f>SUM(J4:J11)</x:f>
-        <x:v>775.4</x:v>
-      </x:c>
-      <x:c r="K14" s="31"/>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="30" t="str">
+      <x:c r="B18" s="31" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C18" s="31"/>
+      <x:c r="D18" s="31"/>
+      <x:c r="E18" s="31"/>
+      <x:c r="F18" s="31"/>
+      <x:c r="G18" s="31"/>
+      <x:c r="H18" s="31"/>
+      <x:c r="I18" s="31"/>
+      <x:c r="J18" s="32" t="n">
+        <x:f>SUM(J4:J15)</x:f>
+        <x:v>1133.8</x:v>
+      </x:c>
+      <x:c r="K18" s="31"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="30" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B15" s="31"/>
-      <x:c r="C15" s="31"/>
-      <x:c r="D15" s="31"/>
-      <x:c r="E15" s="31"/>
-      <x:c r="F15" s="31"/>
-      <x:c r="G15" s="31"/>
-      <x:c r="H15" s="31"/>
-      <x:c r="I15" s="31"/>
-      <x:c r="J15" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
-        <x:v>96.9</x:v>
-      </x:c>
-      <x:c r="K15" s="31"/>
+      <x:c r="B19" s="31"/>
+      <x:c r="C19" s="31"/>
+      <x:c r="D19" s="31"/>
+      <x:c r="E19" s="31"/>
+      <x:c r="F19" s="31"/>
+      <x:c r="G19" s="31"/>
+      <x:c r="H19" s="31"/>
+      <x:c r="I19" s="31"/>
+      <x:c r="J19" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
+        <x:v>94.5</x:v>
+      </x:c>
+      <x:c r="K19" s="31"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3414,43 +4254,179 @@
         <x:v>IH2609</x:v>
       </x:c>
     </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="21" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B12" s="21" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C12" s="21" t="str">
+        <x:v>7月13日</x:v>
+      </x:c>
+      <x:c r="D12" s="22" t="n">
+        <x:v>2895.8</x:v>
+      </x:c>
+      <x:c r="E12" s="22" t="n">
+        <x:v>2908.6</x:v>
+      </x:c>
+      <x:c r="F12" s="22" t="n">
+        <x:v>2858</x:v>
+      </x:c>
+      <x:c r="G12" s="22" t="n">
+        <x:v>2872.6</x:v>
+      </x:c>
+      <x:c r="H12" s="22"/>
+      <x:c r="I12" s="23" t="n">
+        <x:v>-0.012920074221702937</x:v>
+      </x:c>
+      <x:c r="J12" s="22" t="n">
+        <x:f>ROUND(E12-F12,1)</x:f>
+        <x:v>50.6</x:v>
+      </x:c>
+      <x:c r="K12" s="21" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="21" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B13" s="21" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C13" s="21" t="str">
+        <x:v>7月14日</x:v>
+      </x:c>
+      <x:c r="D13" s="22" t="n">
+        <x:v>2872</x:v>
+      </x:c>
+      <x:c r="E13" s="22" t="n">
+        <x:v>2894</x:v>
+      </x:c>
+      <x:c r="F13" s="22" t="n">
+        <x:v>2831.4</x:v>
+      </x:c>
+      <x:c r="G13" s="22" t="n">
+        <x:v>2891.2</x:v>
+      </x:c>
+      <x:c r="H13" s="22"/>
+      <x:c r="I13" s="23" t="n">
+        <x:v>0.006474970410081493</x:v>
+      </x:c>
+      <x:c r="J13" s="27" t="n">
+        <x:f>ROUND(E13-F13,1)</x:f>
+        <x:v>62.6</x:v>
+      </x:c>
+      <x:c r="K13" s="21" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+    </x:row>
     <x:row r="14">
-      <x:c r="A14" s="30" t="str">
+      <x:c r="A14" s="21" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B14" s="21" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C14" s="21" t="str">
+        <x:v>7月15日</x:v>
+      </x:c>
+      <x:c r="D14" s="22" t="n">
+        <x:v>2900</x:v>
+      </x:c>
+      <x:c r="E14" s="22" t="n">
+        <x:v>2924</x:v>
+      </x:c>
+      <x:c r="F14" s="22" t="n">
+        <x:v>2891</x:v>
+      </x:c>
+      <x:c r="G14" s="22" t="n">
+        <x:v>2914</x:v>
+      </x:c>
+      <x:c r="H14" s="22"/>
+      <x:c r="I14" s="23" t="n">
+        <x:v>0.007885998893193191</x:v>
+      </x:c>
+      <x:c r="J14" s="22" t="n">
+        <x:f>ROUND(E14-F14,1)</x:f>
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="K14" s="21" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="21" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B15" s="21" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C15" s="21" t="str">
+        <x:v>7月16日</x:v>
+      </x:c>
+      <x:c r="D15" s="22" t="n">
+        <x:v>2889</x:v>
+      </x:c>
+      <x:c r="E15" s="22" t="n">
+        <x:v>2911.8</x:v>
+      </x:c>
+      <x:c r="F15" s="22" t="n">
+        <x:v>2853.4</x:v>
+      </x:c>
+      <x:c r="G15" s="22" t="n">
+        <x:v>2867.8</x:v>
+      </x:c>
+      <x:c r="H15" s="22"/>
+      <x:c r="I15" s="23" t="n">
+        <x:v>-0.015854495538778268</x:v>
+      </x:c>
+      <x:c r="J15" s="22" t="n">
+        <x:f>ROUND(E15-F15,1)</x:f>
+        <x:v>58.4</x:v>
+      </x:c>
+      <x:c r="K15" s="21" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="30" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B14" s="31" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C14" s="31"/>
-      <x:c r="D14" s="31"/>
-      <x:c r="E14" s="31"/>
-      <x:c r="F14" s="31"/>
-      <x:c r="G14" s="31"/>
-      <x:c r="H14" s="31"/>
-      <x:c r="I14" s="31"/>
-      <x:c r="J14" s="32" t="n">
-        <x:f>SUM(J4:J11)</x:f>
-        <x:v>444.4</x:v>
-      </x:c>
-      <x:c r="K14" s="31"/>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="30" t="str">
+      <x:c r="B18" s="31" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C18" s="31"/>
+      <x:c r="D18" s="31"/>
+      <x:c r="E18" s="31"/>
+      <x:c r="F18" s="31"/>
+      <x:c r="G18" s="31"/>
+      <x:c r="H18" s="31"/>
+      <x:c r="I18" s="31"/>
+      <x:c r="J18" s="32" t="n">
+        <x:f>SUM(J4:J15)</x:f>
+        <x:v>649</x:v>
+      </x:c>
+      <x:c r="K18" s="31"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="30" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B15" s="31"/>
-      <x:c r="C15" s="31"/>
-      <x:c r="D15" s="31"/>
-      <x:c r="E15" s="31"/>
-      <x:c r="F15" s="31"/>
-      <x:c r="G15" s="31"/>
-      <x:c r="H15" s="31"/>
-      <x:c r="I15" s="31"/>
-      <x:c r="J15" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
-        <x:v>55.6</x:v>
-      </x:c>
-      <x:c r="K15" s="31"/>
+      <x:c r="B19" s="31"/>
+      <x:c r="C19" s="31"/>
+      <x:c r="D19" s="31"/>
+      <x:c r="E19" s="31"/>
+      <x:c r="F19" s="31"/>
+      <x:c r="G19" s="31"/>
+      <x:c r="H19" s="31"/>
+      <x:c r="I19" s="31"/>
+      <x:c r="J19" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
+        <x:v>54.1</x:v>
+      </x:c>
+      <x:c r="K19" s="31"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-07-17
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R3cb54c95a8e34ecb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="2" r:id="R902f800c2dfd454e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="3" r:id="Rea22f0e9cc3f4dd1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="4" r:id="R796a8bfd45a34f2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="5" r:id="Rfedbca72fab94f39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="6" r:id="R111e62eb666a477f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="7" r:id="R325ea8c2e8b345a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="8" r:id="R02dd5a33abee4a50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R2965192986d54293"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="2" r:id="Rd1e8ae8771a7410d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="3" r:id="R133a6d1eb2384b30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="4" r:id="Rcd72ef20500c4cfe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="5" r:id="Rad1b9aec6b0340a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="6" r:id="R9e92c78a80a64724"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="7" r:id="R46ae41261300410c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="8" r:id="R7b3b722d5a1f459c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -24,7 +24,7 @@
     <x:numFmt numFmtId="200" formatCode="General"/>
     <x:numFmt numFmtId="201" formatCode="0.0%"/>
   </x:numFmts>
-  <x:fonts count="8">
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -69,8 +69,14 @@
       <x:color rgb="FFE11D48"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF1E3A8A"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -100,6 +106,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFFF00"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDBEAFE"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -137,7 +148,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="35">
+  <x:cellXfs count="43">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -198,6 +209,30 @@
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="7" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="5" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="5" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="8" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="8" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="8" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="8" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -469,25 +504,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-07-16</x:v>
+        <x:v>2026-07-17</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7836.39</x:v>
+        <x:v>7605.613</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7591.421</x:v>
+        <x:v>7163.309</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>245</x:v>
+        <x:v>442.3</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>2980.3</x:v>
+        <x:v>3422.6</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>248.4</x:v>
+        <x:v>263.3</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -498,25 +533,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-07-16</x:v>
+        <x:v>2026-07-17</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>8148.042</x:v>
+        <x:v>7908.739</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7907.097</x:v>
+        <x:v>7474.151</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>240.9</x:v>
+        <x:v>434.6</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>3125.3</x:v>
+        <x:v>3559.9</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>260.4</x:v>
+        <x:v>273.8</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -527,25 +562,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-07-16</x:v>
+        <x:v>2026-07-17</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3940.451</x:v>
+        <x:v>3869.215</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3867.601</x:v>
+        <x:v>3745.174</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>72.8</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>808.2</x:v>
+        <x:v>932.2</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>67.4</x:v>
+        <x:v>71.7</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -556,25 +591,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-07-16</x:v>
+        <x:v>2026-07-17</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>7750.2</x:v>
+        <x:v>7534.6</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>7511</x:v>
+        <x:v>7018.8</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>239.2</x:v>
+        <x:v>515.8</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>2629.2</x:v>
+        <x:v>3145</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>219.1</x:v>
+        <x:v>241.9</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -675,7 +710,7 @@
         <x:v>2026-07-01</x:v>
       </x:c>
       <x:c r="C13" s="14" t="str">
-        <x:v>2026-07-16</x:v>
+        <x:v>2026-07-17</x:v>
       </x:c>
       <x:c r="D13" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1276,43 +1311,79 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="30" t="str">
+    <x:row r="16">
+      <x:c r="A16" s="31" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B16" s="31" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C16" s="31" t="str">
+        <x:v>7月17日</x:v>
+      </x:c>
+      <x:c r="D16" s="32" t="n">
+        <x:v>7599.388</x:v>
+      </x:c>
+      <x:c r="E16" s="32" t="n">
+        <x:v>7605.613</x:v>
+      </x:c>
+      <x:c r="F16" s="32" t="n">
+        <x:v>7163.309</x:v>
+      </x:c>
+      <x:c r="G16" s="32" t="n">
+        <x:v>7167.996</x:v>
+      </x:c>
+      <x:c r="H16" s="25" t="n">
+        <x:v>-463.8</x:v>
+      </x:c>
+      <x:c r="I16" s="33" t="n">
+        <x:v>-0.06076788034008396</x:v>
+      </x:c>
+      <x:c r="J16" s="27" t="n">
+        <x:f>ROUND(E16-F16,1)</x:f>
+        <x:v>442.3</x:v>
+      </x:c>
+      <x:c r="K16" s="31" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="38" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B18" s="31" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="C18" s="31"/>
-      <x:c r="D18" s="31"/>
-      <x:c r="E18" s="31"/>
-      <x:c r="F18" s="31"/>
-      <x:c r="G18" s="31"/>
-      <x:c r="H18" s="31"/>
-      <x:c r="I18" s="31"/>
-      <x:c r="J18" s="32" t="n">
-        <x:f>SUM(J4:J15)</x:f>
-        <x:v>2980.3</x:v>
-      </x:c>
-      <x:c r="K18" s="31"/>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="30" t="str">
+      <x:c r="B19" s="39" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="C19" s="39"/>
+      <x:c r="D19" s="39"/>
+      <x:c r="E19" s="39"/>
+      <x:c r="F19" s="39"/>
+      <x:c r="G19" s="39"/>
+      <x:c r="H19" s="39"/>
+      <x:c r="I19" s="39"/>
+      <x:c r="J19" s="40" t="n">
+        <x:f>SUM(J4:J16)</x:f>
+        <x:v>3422.6000000000004</x:v>
+      </x:c>
+      <x:c r="K19" s="39"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="38" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B19" s="31"/>
-      <x:c r="C19" s="31"/>
-      <x:c r="D19" s="31"/>
-      <x:c r="E19" s="31"/>
-      <x:c r="F19" s="31"/>
-      <x:c r="G19" s="31"/>
-      <x:c r="H19" s="31"/>
-      <x:c r="I19" s="31"/>
-      <x:c r="J19" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
-        <x:v>248.4</x:v>
-      </x:c>
-      <x:c r="K19" s="31"/>
+      <x:c r="B20" s="39"/>
+      <x:c r="C20" s="39"/>
+      <x:c r="D20" s="39"/>
+      <x:c r="E20" s="39"/>
+      <x:c r="F20" s="39"/>
+      <x:c r="G20" s="39"/>
+      <x:c r="H20" s="39"/>
+      <x:c r="I20" s="39"/>
+      <x:c r="J20" s="42" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
+        <x:v>263.3</x:v>
+      </x:c>
+      <x:c r="K20" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1811,43 +1882,79 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="30" t="str">
+    <x:row r="16">
+      <x:c r="A16" s="31" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B16" s="31" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C16" s="31" t="str">
+        <x:v>7月17日</x:v>
+      </x:c>
+      <x:c r="D16" s="32" t="n">
+        <x:v>7900.097</x:v>
+      </x:c>
+      <x:c r="E16" s="32" t="n">
+        <x:v>7908.739</x:v>
+      </x:c>
+      <x:c r="F16" s="32" t="n">
+        <x:v>7474.151</x:v>
+      </x:c>
+      <x:c r="G16" s="32" t="n">
+        <x:v>7513.763</x:v>
+      </x:c>
+      <x:c r="H16" s="25" t="n">
+        <x:v>-441.9</x:v>
+      </x:c>
+      <x:c r="I16" s="33" t="n">
+        <x:v>-0.05554545792783605</x:v>
+      </x:c>
+      <x:c r="J16" s="27" t="n">
+        <x:f>ROUND(E16-F16,1)</x:f>
+        <x:v>434.6</x:v>
+      </x:c>
+      <x:c r="K16" s="31" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="38" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B18" s="31" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="C18" s="31"/>
-      <x:c r="D18" s="31"/>
-      <x:c r="E18" s="31"/>
-      <x:c r="F18" s="31"/>
-      <x:c r="G18" s="31"/>
-      <x:c r="H18" s="31"/>
-      <x:c r="I18" s="31"/>
-      <x:c r="J18" s="32" t="n">
-        <x:f>SUM(J4:J15)</x:f>
-        <x:v>3125.3</x:v>
-      </x:c>
-      <x:c r="K18" s="31"/>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="30" t="str">
+      <x:c r="B19" s="39" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="C19" s="39"/>
+      <x:c r="D19" s="39"/>
+      <x:c r="E19" s="39"/>
+      <x:c r="F19" s="39"/>
+      <x:c r="G19" s="39"/>
+      <x:c r="H19" s="39"/>
+      <x:c r="I19" s="39"/>
+      <x:c r="J19" s="40" t="n">
+        <x:f>SUM(J4:J16)</x:f>
+        <x:v>3559.9</x:v>
+      </x:c>
+      <x:c r="K19" s="39"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="38" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B19" s="31"/>
-      <x:c r="C19" s="31"/>
-      <x:c r="D19" s="31"/>
-      <x:c r="E19" s="31"/>
-      <x:c r="F19" s="31"/>
-      <x:c r="G19" s="31"/>
-      <x:c r="H19" s="31"/>
-      <x:c r="I19" s="31"/>
-      <x:c r="J19" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
-        <x:v>260.4</x:v>
-      </x:c>
-      <x:c r="K19" s="31"/>
+      <x:c r="B20" s="39"/>
+      <x:c r="C20" s="39"/>
+      <x:c r="D20" s="39"/>
+      <x:c r="E20" s="39"/>
+      <x:c r="F20" s="39"/>
+      <x:c r="G20" s="39"/>
+      <x:c r="H20" s="39"/>
+      <x:c r="I20" s="39"/>
+      <x:c r="J20" s="42" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
+        <x:v>273.8</x:v>
+      </x:c>
+      <x:c r="K20" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2346,43 +2453,79 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="30" t="str">
+    <x:row r="16">
+      <x:c r="A16" s="31" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B16" s="31" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C16" s="31" t="str">
+        <x:v>7月17日</x:v>
+      </x:c>
+      <x:c r="D16" s="32" t="n">
+        <x:v>3865.317</x:v>
+      </x:c>
+      <x:c r="E16" s="32" t="n">
+        <x:v>3869.215</x:v>
+      </x:c>
+      <x:c r="F16" s="32" t="n">
+        <x:v>3745.174</x:v>
+      </x:c>
+      <x:c r="G16" s="32" t="n">
+        <x:v>3764.155</x:v>
+      </x:c>
+      <x:c r="H16" s="32" t="n">
+        <x:v>-118.3</x:v>
+      </x:c>
+      <x:c r="I16" s="33" t="n">
+        <x:v>-0.030459922733619527</x:v>
+      </x:c>
+      <x:c r="J16" s="27" t="n">
+        <x:f>ROUND(E16-F16,1)</x:f>
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="K16" s="31" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="38" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B18" s="31" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="C18" s="31"/>
-      <x:c r="D18" s="31"/>
-      <x:c r="E18" s="31"/>
-      <x:c r="F18" s="31"/>
-      <x:c r="G18" s="31"/>
-      <x:c r="H18" s="31"/>
-      <x:c r="I18" s="31"/>
-      <x:c r="J18" s="32" t="n">
-        <x:f>SUM(J4:J15)</x:f>
-        <x:v>808.1999999999999</x:v>
-      </x:c>
-      <x:c r="K18" s="31"/>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="30" t="str">
+      <x:c r="B19" s="39" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="C19" s="39"/>
+      <x:c r="D19" s="39"/>
+      <x:c r="E19" s="39"/>
+      <x:c r="F19" s="39"/>
+      <x:c r="G19" s="39"/>
+      <x:c r="H19" s="39"/>
+      <x:c r="I19" s="39"/>
+      <x:c r="J19" s="40" t="n">
+        <x:f>SUM(J4:J16)</x:f>
+        <x:v>932.1999999999999</x:v>
+      </x:c>
+      <x:c r="K19" s="39"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="38" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B19" s="31"/>
-      <x:c r="C19" s="31"/>
-      <x:c r="D19" s="31"/>
-      <x:c r="E19" s="31"/>
-      <x:c r="F19" s="31"/>
-      <x:c r="G19" s="31"/>
-      <x:c r="H19" s="31"/>
-      <x:c r="I19" s="31"/>
-      <x:c r="J19" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
-        <x:v>67.4</x:v>
-      </x:c>
-      <x:c r="K19" s="31"/>
+      <x:c r="B20" s="39"/>
+      <x:c r="C20" s="39"/>
+      <x:c r="D20" s="39"/>
+      <x:c r="E20" s="39"/>
+      <x:c r="F20" s="39"/>
+      <x:c r="G20" s="39"/>
+      <x:c r="H20" s="39"/>
+      <x:c r="I20" s="39"/>
+      <x:c r="J20" s="42" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
+        <x:v>71.7</x:v>
+      </x:c>
+      <x:c r="K20" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2881,43 +3024,79 @@
         <x:v>IM2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="30" t="str">
+    <x:row r="16">
+      <x:c r="A16" s="31" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B16" s="31" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C16" s="31" t="str">
+        <x:v>7月17日</x:v>
+      </x:c>
+      <x:c r="D16" s="32" t="n">
+        <x:v>7520</x:v>
+      </x:c>
+      <x:c r="E16" s="32" t="n">
+        <x:v>7534.6</x:v>
+      </x:c>
+      <x:c r="F16" s="32" t="n">
+        <x:v>7018.8</x:v>
+      </x:c>
+      <x:c r="G16" s="32" t="n">
+        <x:v>7065.2</x:v>
+      </x:c>
+      <x:c r="H16" s="25" t="n">
+        <x:v>-487.4</x:v>
+      </x:c>
+      <x:c r="I16" s="33" t="n">
+        <x:v>-0.06453406773826242</x:v>
+      </x:c>
+      <x:c r="J16" s="27" t="n">
+        <x:f>ROUND(E16-F16,1)</x:f>
+        <x:v>515.8</x:v>
+      </x:c>
+      <x:c r="K16" s="31" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="38" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B18" s="31" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="C18" s="31"/>
-      <x:c r="D18" s="31"/>
-      <x:c r="E18" s="31"/>
-      <x:c r="F18" s="31"/>
-      <x:c r="G18" s="31"/>
-      <x:c r="H18" s="31"/>
-      <x:c r="I18" s="31"/>
-      <x:c r="J18" s="32" t="n">
-        <x:f>SUM(J4:J15)</x:f>
-        <x:v>2629.2</x:v>
-      </x:c>
-      <x:c r="K18" s="31"/>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="30" t="str">
+      <x:c r="B19" s="39" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="C19" s="39"/>
+      <x:c r="D19" s="39"/>
+      <x:c r="E19" s="39"/>
+      <x:c r="F19" s="39"/>
+      <x:c r="G19" s="39"/>
+      <x:c r="H19" s="39"/>
+      <x:c r="I19" s="39"/>
+      <x:c r="J19" s="40" t="n">
+        <x:f>SUM(J4:J16)</x:f>
+        <x:v>3145</x:v>
+      </x:c>
+      <x:c r="K19" s="39"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="38" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B19" s="31"/>
-      <x:c r="C19" s="31"/>
-      <x:c r="D19" s="31"/>
-      <x:c r="E19" s="31"/>
-      <x:c r="F19" s="31"/>
-      <x:c r="G19" s="31"/>
-      <x:c r="H19" s="31"/>
-      <x:c r="I19" s="31"/>
-      <x:c r="J19" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
-        <x:v>219.1</x:v>
-      </x:c>
-      <x:c r="K19" s="31"/>
+      <x:c r="B20" s="39"/>
+      <x:c r="C20" s="39"/>
+      <x:c r="D20" s="39"/>
+      <x:c r="E20" s="39"/>
+      <x:c r="F20" s="39"/>
+      <x:c r="G20" s="39"/>
+      <x:c r="H20" s="39"/>
+      <x:c r="I20" s="39"/>
+      <x:c r="J20" s="42" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
+        <x:v>241.9</x:v>
+      </x:c>
+      <x:c r="K20" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3417,42 +3596,42 @@
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="30" t="str">
+      <x:c r="A18" s="38" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B18" s="31" t="n">
+      <x:c r="B18" s="39" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="C18" s="31"/>
-      <x:c r="D18" s="31"/>
-      <x:c r="E18" s="31"/>
-      <x:c r="F18" s="31"/>
-      <x:c r="G18" s="31"/>
-      <x:c r="H18" s="31"/>
-      <x:c r="I18" s="31"/>
-      <x:c r="J18" s="32" t="n">
+      <x:c r="C18" s="39"/>
+      <x:c r="D18" s="39"/>
+      <x:c r="E18" s="39"/>
+      <x:c r="F18" s="39"/>
+      <x:c r="G18" s="39"/>
+      <x:c r="H18" s="39"/>
+      <x:c r="I18" s="39"/>
+      <x:c r="J18" s="40" t="n">
         <x:f>SUM(J4:J15)</x:f>
         <x:v>2906.4</x:v>
       </x:c>
-      <x:c r="K18" s="31"/>
+      <x:c r="K18" s="39"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="30" t="str">
+      <x:c r="A19" s="38" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B19" s="31"/>
-      <x:c r="C19" s="31"/>
-      <x:c r="D19" s="31"/>
-      <x:c r="E19" s="31"/>
-      <x:c r="F19" s="31"/>
-      <x:c r="G19" s="31"/>
-      <x:c r="H19" s="31"/>
-      <x:c r="I19" s="31"/>
-      <x:c r="J19" s="34" t="n">
+      <x:c r="B19" s="39"/>
+      <x:c r="C19" s="39"/>
+      <x:c r="D19" s="39"/>
+      <x:c r="E19" s="39"/>
+      <x:c r="F19" s="39"/>
+      <x:c r="G19" s="39"/>
+      <x:c r="H19" s="39"/>
+      <x:c r="I19" s="39"/>
+      <x:c r="J19" s="42" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
         <x:v>242.2</x:v>
       </x:c>
-      <x:c r="K19" s="31"/>
+      <x:c r="K19" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3952,42 +4131,42 @@
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="30" t="str">
+      <x:c r="A18" s="38" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B18" s="31" t="n">
+      <x:c r="B18" s="39" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="C18" s="31"/>
-      <x:c r="D18" s="31"/>
-      <x:c r="E18" s="31"/>
-      <x:c r="F18" s="31"/>
-      <x:c r="G18" s="31"/>
-      <x:c r="H18" s="31"/>
-      <x:c r="I18" s="31"/>
-      <x:c r="J18" s="32" t="n">
+      <x:c r="C18" s="39"/>
+      <x:c r="D18" s="39"/>
+      <x:c r="E18" s="39"/>
+      <x:c r="F18" s="39"/>
+      <x:c r="G18" s="39"/>
+      <x:c r="H18" s="39"/>
+      <x:c r="I18" s="39"/>
+      <x:c r="J18" s="40" t="n">
         <x:f>SUM(J4:J15)</x:f>
         <x:v>1133.8</x:v>
       </x:c>
-      <x:c r="K18" s="31"/>
+      <x:c r="K18" s="39"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="30" t="str">
+      <x:c r="A19" s="38" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B19" s="31"/>
-      <x:c r="C19" s="31"/>
-      <x:c r="D19" s="31"/>
-      <x:c r="E19" s="31"/>
-      <x:c r="F19" s="31"/>
-      <x:c r="G19" s="31"/>
-      <x:c r="H19" s="31"/>
-      <x:c r="I19" s="31"/>
-      <x:c r="J19" s="34" t="n">
+      <x:c r="B19" s="39"/>
+      <x:c r="C19" s="39"/>
+      <x:c r="D19" s="39"/>
+      <x:c r="E19" s="39"/>
+      <x:c r="F19" s="39"/>
+      <x:c r="G19" s="39"/>
+      <x:c r="H19" s="39"/>
+      <x:c r="I19" s="39"/>
+      <x:c r="J19" s="42" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
         <x:v>94.5</x:v>
       </x:c>
-      <x:c r="K19" s="31"/>
+      <x:c r="K19" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4487,42 +4666,42 @@
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="30" t="str">
+      <x:c r="A18" s="38" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B18" s="31" t="n">
+      <x:c r="B18" s="39" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="C18" s="31"/>
-      <x:c r="D18" s="31"/>
-      <x:c r="E18" s="31"/>
-      <x:c r="F18" s="31"/>
-      <x:c r="G18" s="31"/>
-      <x:c r="H18" s="31"/>
-      <x:c r="I18" s="31"/>
-      <x:c r="J18" s="32" t="n">
+      <x:c r="C18" s="39"/>
+      <x:c r="D18" s="39"/>
+      <x:c r="E18" s="39"/>
+      <x:c r="F18" s="39"/>
+      <x:c r="G18" s="39"/>
+      <x:c r="H18" s="39"/>
+      <x:c r="I18" s="39"/>
+      <x:c r="J18" s="40" t="n">
         <x:f>SUM(J4:J15)</x:f>
         <x:v>649</x:v>
       </x:c>
-      <x:c r="K18" s="31"/>
+      <x:c r="K18" s="39"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="30" t="str">
+      <x:c r="A19" s="38" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B19" s="31"/>
-      <x:c r="C19" s="31"/>
-      <x:c r="D19" s="31"/>
-      <x:c r="E19" s="31"/>
-      <x:c r="F19" s="31"/>
-      <x:c r="G19" s="31"/>
-      <x:c r="H19" s="31"/>
-      <x:c r="I19" s="31"/>
-      <x:c r="J19" s="34" t="n">
+      <x:c r="B19" s="39"/>
+      <x:c r="C19" s="39"/>
+      <x:c r="D19" s="39"/>
+      <x:c r="E19" s="39"/>
+      <x:c r="F19" s="39"/>
+      <x:c r="G19" s="39"/>
+      <x:c r="H19" s="39"/>
+      <x:c r="I19" s="39"/>
+      <x:c r="J19" s="42" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
         <x:v>54.1</x:v>
       </x:c>
-      <x:c r="K19" s="31"/>
+      <x:c r="K19" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-07-20
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R8c4e9776523949c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="2" r:id="R2c0730a634c14fef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="3" r:id="R3340b55858fe41a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="4" r:id="R43da96350098451b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="5" r:id="Ra3aa133931c74544"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="6" r:id="R84e64d00df614aa1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="7" r:id="R5b5c081fbec44644"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="8" r:id="R82cb90fd3bd2434c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rd4b672d6d19b4aba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="2" r:id="Ree2542267407402b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="3" r:id="R79a67a0e439f4402"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="4" r:id="R8b3ba79b137748fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="5" r:id="R3f46f99a32ca4e35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="6" r:id="Rd56b5d34edf04bc7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="7" r:id="R799a76ece4674774"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="8" r:id="R7a1ad1f77d3d410f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -504,25 +504,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-07-17</x:v>
+        <x:v>2026-07-20</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7605.613</x:v>
+        <x:v>7298.122</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7163.309</x:v>
+        <x:v>6824.145</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>442.3</x:v>
+        <x:v>474</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>3422.6</x:v>
+        <x:v>3896.6</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>263.3</x:v>
+        <x:v>278.3</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -533,25 +533,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-07-17</x:v>
+        <x:v>2026-07-20</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7908.739</x:v>
+        <x:v>7626.489</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7474.151</x:v>
+        <x:v>7253.518</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>434.6</x:v>
+        <x:v>373</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>3559.9</x:v>
+        <x:v>3932.9</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>273.8</x:v>
+        <x:v>280.9</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -562,25 +562,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-07-17</x:v>
+        <x:v>2026-07-20</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3869.215</x:v>
+        <x:v>3831.659</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3745.174</x:v>
+        <x:v>3741.11</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>124</x:v>
+        <x:v>90.5</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>932.2</x:v>
+        <x:v>1022.7</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>71.7</x:v>
+        <x:v>73.1</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -591,25 +591,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-07-17</x:v>
+        <x:v>2026-07-20</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>7534.6</x:v>
+        <x:v>7237</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>7018.8</x:v>
+        <x:v>6652.2</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>515.8</x:v>
+        <x:v>584.8</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>3145</x:v>
+        <x:v>3729.8</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>241.9</x:v>
+        <x:v>266.4</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -620,25 +620,25 @@
         <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>2026-07-17</x:v>
+        <x:v>2026-07-20</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:v>7848.2</x:v>
+        <x:v>7561.8</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>7362.8</x:v>
+        <x:v>7092</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>485.4</x:v>
+        <x:v>469.8</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>3391.8</x:v>
+        <x:v>3861.6</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
-        <x:v>260.9</x:v>
+        <x:v>275.8</x:v>
       </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
@@ -649,25 +649,25 @@
         <x:v>IF主力</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>2026-07-17</x:v>
+        <x:v>2026-07-20</x:v>
       </x:c>
       <x:c r="C9" s="10" t="n">
-        <x:v>4633.8</x:v>
+        <x:v>4590</x:v>
       </x:c>
       <x:c r="D9" s="10" t="n">
-        <x:v>4441.4</x:v>
+        <x:v>4465</x:v>
       </x:c>
       <x:c r="E9" s="12" t="n">
-        <x:v>192.4</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="F9" s="9" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G9" s="10" t="n">
-        <x:v>1326.2</x:v>
+        <x:v>1451.2</x:v>
       </x:c>
       <x:c r="H9" s="10" t="n">
-        <x:v>102</x:v>
+        <x:v>103.7</x:v>
       </x:c>
       <x:c r="I9" s="10" t="n">
         <x:v>90</x:v>
@@ -678,25 +678,25 @@
         <x:v>IH主力</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>2026-07-17</x:v>
+        <x:v>2026-07-20</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:v>2864.8</x:v>
+        <x:v>2884.6</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
-        <x:v>2782.6</x:v>
+        <x:v>2820</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
-        <x:v>82.2</x:v>
+        <x:v>64.6</x:v>
       </x:c>
       <x:c r="F10" s="9" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G10" s="10" t="n">
-        <x:v>731.2</x:v>
+        <x:v>795.8</x:v>
       </x:c>
       <x:c r="H10" s="10" t="n">
-        <x:v>56.2</x:v>
+        <x:v>56.8</x:v>
       </x:c>
       <x:c r="I10" s="10" t="n">
         <x:v>60</x:v>
@@ -710,7 +710,7 @@
         <x:v>2026-07-01</x:v>
       </x:c>
       <x:c r="C13" s="14" t="str">
-        <x:v>2026-07-17</x:v>
+        <x:v>2026-07-20</x:v>
       </x:c>
       <x:c r="D13" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1347,31 +1347,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="38" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B19" s="39" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C19" s="39"/>
-      <x:c r="D19" s="39"/>
-      <x:c r="E19" s="39"/>
-      <x:c r="F19" s="39"/>
-      <x:c r="G19" s="39"/>
-      <x:c r="H19" s="39"/>
-      <x:c r="I19" s="39"/>
-      <x:c r="J19" s="40" t="n">
-        <x:f>SUM(J4:J16)</x:f>
-        <x:v>3422.6000000000004</x:v>
-      </x:c>
-      <x:c r="K19" s="39"/>
+    <x:row r="17">
+      <x:c r="A17" s="21" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B17" s="21" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C17" s="21" t="str">
+        <x:v>7月20日</x:v>
+      </x:c>
+      <x:c r="D17" s="22" t="n">
+        <x:v>7256.267</x:v>
+      </x:c>
+      <x:c r="E17" s="22" t="n">
+        <x:v>7298.122</x:v>
+      </x:c>
+      <x:c r="F17" s="22" t="n">
+        <x:v>6824.145</x:v>
+      </x:c>
+      <x:c r="G17" s="22" t="n">
+        <x:v>6965.376</x:v>
+      </x:c>
+      <x:c r="H17" s="25" t="n">
+        <x:v>-202.6</x:v>
+      </x:c>
+      <x:c r="I17" s="23" t="n">
+        <x:v>-0.028267314881314065</x:v>
+      </x:c>
+      <x:c r="J17" s="27" t="n">
+        <x:f>ROUND(E17-F17,1)</x:f>
+        <x:v>474</x:v>
+      </x:c>
+      <x:c r="K17" s="21" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="38" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B20" s="39"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B20" s="39" t="n">
+        <x:v>14</x:v>
+      </x:c>
       <x:c r="C20" s="39"/>
       <x:c r="D20" s="39"/>
       <x:c r="E20" s="39"/>
@@ -1379,11 +1397,29 @@
       <x:c r="G20" s="39"/>
       <x:c r="H20" s="39"/>
       <x:c r="I20" s="39"/>
-      <x:c r="J20" s="42" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
-        <x:v>263.3</x:v>
+      <x:c r="J20" s="40" t="n">
+        <x:f>SUM(J4:J17)</x:f>
+        <x:v>3896.6000000000004</x:v>
       </x:c>
       <x:c r="K20" s="39"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="38" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B21" s="39"/>
+      <x:c r="C21" s="39"/>
+      <x:c r="D21" s="39"/>
+      <x:c r="E21" s="39"/>
+      <x:c r="F21" s="39"/>
+      <x:c r="G21" s="39"/>
+      <x:c r="H21" s="39"/>
+      <x:c r="I21" s="39"/>
+      <x:c r="J21" s="42" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
+        <x:v>278.3</x:v>
+      </x:c>
+      <x:c r="K21" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1918,31 +1954,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="38" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B19" s="39" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C19" s="39"/>
-      <x:c r="D19" s="39"/>
-      <x:c r="E19" s="39"/>
-      <x:c r="F19" s="39"/>
-      <x:c r="G19" s="39"/>
-      <x:c r="H19" s="39"/>
-      <x:c r="I19" s="39"/>
-      <x:c r="J19" s="40" t="n">
-        <x:f>SUM(J4:J16)</x:f>
-        <x:v>3559.9</x:v>
-      </x:c>
-      <x:c r="K19" s="39"/>
+    <x:row r="17">
+      <x:c r="A17" s="21" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B17" s="21" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C17" s="21" t="str">
+        <x:v>7月20日</x:v>
+      </x:c>
+      <x:c r="D17" s="22" t="n">
+        <x:v>7597.769</x:v>
+      </x:c>
+      <x:c r="E17" s="22" t="n">
+        <x:v>7626.489</x:v>
+      </x:c>
+      <x:c r="F17" s="22" t="n">
+        <x:v>7253.518</x:v>
+      </x:c>
+      <x:c r="G17" s="22" t="n">
+        <x:v>7411.313</x:v>
+      </x:c>
+      <x:c r="H17" s="22" t="n">
+        <x:v>-102.4</x:v>
+      </x:c>
+      <x:c r="I17" s="23" t="n">
+        <x:v>-0.013634978904711215</x:v>
+      </x:c>
+      <x:c r="J17" s="27" t="n">
+        <x:f>ROUND(E17-F17,1)</x:f>
+        <x:v>373</x:v>
+      </x:c>
+      <x:c r="K17" s="21" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="38" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B20" s="39"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B20" s="39" t="n">
+        <x:v>14</x:v>
+      </x:c>
       <x:c r="C20" s="39"/>
       <x:c r="D20" s="39"/>
       <x:c r="E20" s="39"/>
@@ -1950,11 +2004,29 @@
       <x:c r="G20" s="39"/>
       <x:c r="H20" s="39"/>
       <x:c r="I20" s="39"/>
-      <x:c r="J20" s="42" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
-        <x:v>273.8</x:v>
+      <x:c r="J20" s="40" t="n">
+        <x:f>SUM(J4:J17)</x:f>
+        <x:v>3932.9</x:v>
       </x:c>
       <x:c r="K20" s="39"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="38" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B21" s="39"/>
+      <x:c r="C21" s="39"/>
+      <x:c r="D21" s="39"/>
+      <x:c r="E21" s="39"/>
+      <x:c r="F21" s="39"/>
+      <x:c r="G21" s="39"/>
+      <x:c r="H21" s="39"/>
+      <x:c r="I21" s="39"/>
+      <x:c r="J21" s="42" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
+        <x:v>280.9</x:v>
+      </x:c>
+      <x:c r="K21" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2489,31 +2561,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="38" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B19" s="39" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C19" s="39"/>
-      <x:c r="D19" s="39"/>
-      <x:c r="E19" s="39"/>
-      <x:c r="F19" s="39"/>
-      <x:c r="G19" s="39"/>
-      <x:c r="H19" s="39"/>
-      <x:c r="I19" s="39"/>
-      <x:c r="J19" s="40" t="n">
-        <x:f>SUM(J4:J16)</x:f>
-        <x:v>932.1999999999999</x:v>
-      </x:c>
-      <x:c r="K19" s="39"/>
+    <x:row r="17">
+      <x:c r="A17" s="21" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B17" s="21" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C17" s="21" t="str">
+        <x:v>7月20日</x:v>
+      </x:c>
+      <x:c r="D17" s="22" t="n">
+        <x:v>3791.662</x:v>
+      </x:c>
+      <x:c r="E17" s="22" t="n">
+        <x:v>3831.659</x:v>
+      </x:c>
+      <x:c r="F17" s="22" t="n">
+        <x:v>3741.11</x:v>
+      </x:c>
+      <x:c r="G17" s="22" t="n">
+        <x:v>3796.281</x:v>
+      </x:c>
+      <x:c r="H17" s="22" t="n">
+        <x:v>32.1</x:v>
+      </x:c>
+      <x:c r="I17" s="23" t="n">
+        <x:v>0.008534717619226528</x:v>
+      </x:c>
+      <x:c r="J17" s="27" t="n">
+        <x:f>ROUND(E17-F17,1)</x:f>
+        <x:v>90.5</x:v>
+      </x:c>
+      <x:c r="K17" s="21" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="38" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B20" s="39"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B20" s="39" t="n">
+        <x:v>14</x:v>
+      </x:c>
       <x:c r="C20" s="39"/>
       <x:c r="D20" s="39"/>
       <x:c r="E20" s="39"/>
@@ -2521,11 +2611,29 @@
       <x:c r="G20" s="39"/>
       <x:c r="H20" s="39"/>
       <x:c r="I20" s="39"/>
-      <x:c r="J20" s="42" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
-        <x:v>71.7</x:v>
+      <x:c r="J20" s="40" t="n">
+        <x:f>SUM(J4:J17)</x:f>
+        <x:v>1022.6999999999999</x:v>
       </x:c>
       <x:c r="K20" s="39"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="38" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B21" s="39"/>
+      <x:c r="C21" s="39"/>
+      <x:c r="D21" s="39"/>
+      <x:c r="E21" s="39"/>
+      <x:c r="F21" s="39"/>
+      <x:c r="G21" s="39"/>
+      <x:c r="H21" s="39"/>
+      <x:c r="I21" s="39"/>
+      <x:c r="J21" s="42" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
+        <x:v>73.1</x:v>
+      </x:c>
+      <x:c r="K21" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3060,31 +3168,49 @@
         <x:v>IM2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="38" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B19" s="39" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C19" s="39"/>
-      <x:c r="D19" s="39"/>
-      <x:c r="E19" s="39"/>
-      <x:c r="F19" s="39"/>
-      <x:c r="G19" s="39"/>
-      <x:c r="H19" s="39"/>
-      <x:c r="I19" s="39"/>
-      <x:c r="J19" s="40" t="n">
-        <x:f>SUM(J4:J16)</x:f>
-        <x:v>3145</x:v>
-      </x:c>
-      <x:c r="K19" s="39"/>
+    <x:row r="17">
+      <x:c r="A17" s="21" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B17" s="21" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C17" s="21" t="str">
+        <x:v>7月20日</x:v>
+      </x:c>
+      <x:c r="D17" s="22" t="n">
+        <x:v>7165.2</x:v>
+      </x:c>
+      <x:c r="E17" s="22" t="n">
+        <x:v>7237</x:v>
+      </x:c>
+      <x:c r="F17" s="22" t="n">
+        <x:v>6652.2</x:v>
+      </x:c>
+      <x:c r="G17" s="22" t="n">
+        <x:v>6849.8</x:v>
+      </x:c>
+      <x:c r="H17" s="25" t="n">
+        <x:v>-215.4</x:v>
+      </x:c>
+      <x:c r="I17" s="23" t="n">
+        <x:v>-0.030487459661439065</x:v>
+      </x:c>
+      <x:c r="J17" s="27" t="n">
+        <x:f>ROUND(E17-F17,1)</x:f>
+        <x:v>584.8</x:v>
+      </x:c>
+      <x:c r="K17" s="21" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="38" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B20" s="39"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B20" s="39" t="n">
+        <x:v>14</x:v>
+      </x:c>
       <x:c r="C20" s="39"/>
       <x:c r="D20" s="39"/>
       <x:c r="E20" s="39"/>
@@ -3092,11 +3218,29 @@
       <x:c r="G20" s="39"/>
       <x:c r="H20" s="39"/>
       <x:c r="I20" s="39"/>
-      <x:c r="J20" s="42" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
-        <x:v>241.9</x:v>
+      <x:c r="J20" s="40" t="n">
+        <x:f>SUM(J4:J17)</x:f>
+        <x:v>3729.8</x:v>
       </x:c>
       <x:c r="K20" s="39"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="38" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B21" s="39"/>
+      <x:c r="C21" s="39"/>
+      <x:c r="D21" s="39"/>
+      <x:c r="E21" s="39"/>
+      <x:c r="F21" s="39"/>
+      <x:c r="G21" s="39"/>
+      <x:c r="H21" s="39"/>
+      <x:c r="I21" s="39"/>
+      <x:c r="J21" s="42" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
+        <x:v>266.4</x:v>
+      </x:c>
+      <x:c r="K21" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3631,31 +3775,49 @@
         <x:v>IC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="38" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B19" s="39" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C19" s="39"/>
-      <x:c r="D19" s="39"/>
-      <x:c r="E19" s="39"/>
-      <x:c r="F19" s="39"/>
-      <x:c r="G19" s="39"/>
-      <x:c r="H19" s="39"/>
-      <x:c r="I19" s="39"/>
-      <x:c r="J19" s="40" t="n">
-        <x:f>SUM(J4:J16)</x:f>
-        <x:v>3391.8</x:v>
-      </x:c>
-      <x:c r="K19" s="39"/>
+    <x:row r="17">
+      <x:c r="A17" s="21" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B17" s="21" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C17" s="21" t="str">
+        <x:v>7月20日</x:v>
+      </x:c>
+      <x:c r="D17" s="22" t="n">
+        <x:v>7490</x:v>
+      </x:c>
+      <x:c r="E17" s="22" t="n">
+        <x:v>7561.8</x:v>
+      </x:c>
+      <x:c r="F17" s="22" t="n">
+        <x:v>7092</x:v>
+      </x:c>
+      <x:c r="G17" s="22" t="n">
+        <x:v>7302.2</x:v>
+      </x:c>
+      <x:c r="H17" s="22" t="n">
+        <x:v>-86.8</x:v>
+      </x:c>
+      <x:c r="I17" s="23" t="n">
+        <x:v>-0.011747191771552368</x:v>
+      </x:c>
+      <x:c r="J17" s="27" t="n">
+        <x:f>ROUND(E17-F17,1)</x:f>
+        <x:v>469.8</x:v>
+      </x:c>
+      <x:c r="K17" s="21" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="38" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B20" s="39"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B20" s="39" t="n">
+        <x:v>14</x:v>
+      </x:c>
       <x:c r="C20" s="39"/>
       <x:c r="D20" s="39"/>
       <x:c r="E20" s="39"/>
@@ -3663,11 +3825,29 @@
       <x:c r="G20" s="39"/>
       <x:c r="H20" s="39"/>
       <x:c r="I20" s="39"/>
-      <x:c r="J20" s="42" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
-        <x:v>260.9</x:v>
+      <x:c r="J20" s="40" t="n">
+        <x:f>SUM(J4:J17)</x:f>
+        <x:v>3861.6000000000004</x:v>
       </x:c>
       <x:c r="K20" s="39"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="38" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B21" s="39"/>
+      <x:c r="C21" s="39"/>
+      <x:c r="D21" s="39"/>
+      <x:c r="E21" s="39"/>
+      <x:c r="F21" s="39"/>
+      <x:c r="G21" s="39"/>
+      <x:c r="H21" s="39"/>
+      <x:c r="I21" s="39"/>
+      <x:c r="J21" s="42" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
+        <x:v>275.8</x:v>
+      </x:c>
+      <x:c r="K21" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4202,31 +4382,49 @@
         <x:v>IF2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="38" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B19" s="39" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C19" s="39"/>
-      <x:c r="D19" s="39"/>
-      <x:c r="E19" s="39"/>
-      <x:c r="F19" s="39"/>
-      <x:c r="G19" s="39"/>
-      <x:c r="H19" s="39"/>
-      <x:c r="I19" s="39"/>
-      <x:c r="J19" s="40" t="n">
-        <x:f>SUM(J4:J16)</x:f>
-        <x:v>1326.2</x:v>
-      </x:c>
-      <x:c r="K19" s="39"/>
+    <x:row r="17">
+      <x:c r="A17" s="21" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B17" s="21" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C17" s="21" t="str">
+        <x:v>7月20日</x:v>
+      </x:c>
+      <x:c r="D17" s="22" t="n">
+        <x:v>4530</x:v>
+      </x:c>
+      <x:c r="E17" s="22" t="n">
+        <x:v>4590</x:v>
+      </x:c>
+      <x:c r="F17" s="22" t="n">
+        <x:v>4465</x:v>
+      </x:c>
+      <x:c r="G17" s="22" t="n">
+        <x:v>4545.8</x:v>
+      </x:c>
+      <x:c r="H17" s="22" t="n">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="I17" s="23" t="n">
+        <x:v>0.016093701104206604</x:v>
+      </x:c>
+      <x:c r="J17" s="27" t="n">
+        <x:f>ROUND(E17-F17,1)</x:f>
+        <x:v>125</x:v>
+      </x:c>
+      <x:c r="K17" s="21" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="38" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B20" s="39"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B20" s="39" t="n">
+        <x:v>14</x:v>
+      </x:c>
       <x:c r="C20" s="39"/>
       <x:c r="D20" s="39"/>
       <x:c r="E20" s="39"/>
@@ -4234,11 +4432,29 @@
       <x:c r="G20" s="39"/>
       <x:c r="H20" s="39"/>
       <x:c r="I20" s="39"/>
-      <x:c r="J20" s="42" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
-        <x:v>102</x:v>
+      <x:c r="J20" s="40" t="n">
+        <x:f>SUM(J4:J17)</x:f>
+        <x:v>1451.2</x:v>
       </x:c>
       <x:c r="K20" s="39"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="38" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B21" s="39"/>
+      <x:c r="C21" s="39"/>
+      <x:c r="D21" s="39"/>
+      <x:c r="E21" s="39"/>
+      <x:c r="F21" s="39"/>
+      <x:c r="G21" s="39"/>
+      <x:c r="H21" s="39"/>
+      <x:c r="I21" s="39"/>
+      <x:c r="J21" s="42" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
+        <x:v>103.7</x:v>
+      </x:c>
+      <x:c r="K21" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4773,31 +4989,49 @@
         <x:v>IH2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="38" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B19" s="39" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C19" s="39"/>
-      <x:c r="D19" s="39"/>
-      <x:c r="E19" s="39"/>
-      <x:c r="F19" s="39"/>
-      <x:c r="G19" s="39"/>
-      <x:c r="H19" s="39"/>
-      <x:c r="I19" s="39"/>
-      <x:c r="J19" s="40" t="n">
-        <x:f>SUM(J4:J16)</x:f>
-        <x:v>731.2</x:v>
-      </x:c>
-      <x:c r="K19" s="39"/>
+    <x:row r="17">
+      <x:c r="A17" s="21" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B17" s="21" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C17" s="21" t="str">
+        <x:v>7月20日</x:v>
+      </x:c>
+      <x:c r="D17" s="22" t="n">
+        <x:v>2820</x:v>
+      </x:c>
+      <x:c r="E17" s="22" t="n">
+        <x:v>2884.6</x:v>
+      </x:c>
+      <x:c r="F17" s="22" t="n">
+        <x:v>2820</x:v>
+      </x:c>
+      <x:c r="G17" s="22" t="n">
+        <x:v>2874</x:v>
+      </x:c>
+      <x:c r="H17" s="22" t="n">
+        <x:v>77.6</x:v>
+      </x:c>
+      <x:c r="I17" s="23" t="n">
+        <x:v>0.027749964239736746</x:v>
+      </x:c>
+      <x:c r="J17" s="27" t="n">
+        <x:f>ROUND(E17-F17,1)</x:f>
+        <x:v>64.6</x:v>
+      </x:c>
+      <x:c r="K17" s="21" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="38" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B20" s="39"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B20" s="39" t="n">
+        <x:v>14</x:v>
+      </x:c>
       <x:c r="C20" s="39"/>
       <x:c r="D20" s="39"/>
       <x:c r="E20" s="39"/>
@@ -4805,11 +5039,29 @@
       <x:c r="G20" s="39"/>
       <x:c r="H20" s="39"/>
       <x:c r="I20" s="39"/>
-      <x:c r="J20" s="42" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
-        <x:v>56.2</x:v>
+      <x:c r="J20" s="40" t="n">
+        <x:f>SUM(J4:J17)</x:f>
+        <x:v>795.8000000000001</x:v>
       </x:c>
       <x:c r="K20" s="39"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="38" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B21" s="39"/>
+      <x:c r="C21" s="39"/>
+      <x:c r="D21" s="39"/>
+      <x:c r="E21" s="39"/>
+      <x:c r="F21" s="39"/>
+      <x:c r="G21" s="39"/>
+      <x:c r="H21" s="39"/>
+      <x:c r="I21" s="39"/>
+      <x:c r="J21" s="42" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
+        <x:v>56.8</x:v>
+      </x:c>
+      <x:c r="K21" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-07-21
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R99bdd3e5cb794024"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="2" r:id="R3e60d3916414416e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="3" r:id="R658ef4cbc5994f41"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="4" r:id="Rba894c1ec1c64c92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="5" r:id="R39a72d6c91904221"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="6" r:id="Rd358df731760489a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="7" r:id="R96f9a9d047c04617"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="8" r:id="R08ddc178ad2b4b90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Ra45153128f964a56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="2" r:id="R3be160698fb94f07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="3" r:id="R45458a7ede114146"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="4" r:id="R513f769d3f2b4fff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="5" r:id="R219e4e49eb054f15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="6" r:id="Refc394b5f785468a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="7" r:id="R15bb1f17c503427c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="8" r:id="Rc6268522859d4261"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -504,25 +504,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-07-20</x:v>
+        <x:v>2026-07-21</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7298.122</x:v>
+        <x:v>7264.338</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>6824.145</x:v>
+        <x:v>6714.187</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>474</x:v>
+        <x:v>550.2</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>3896.6</x:v>
+        <x:v>4446.8</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>278.3</x:v>
+        <x:v>296.5</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -533,25 +533,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-07-20</x:v>
+        <x:v>2026-07-21</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7626.489</x:v>
+        <x:v>7802.755</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7253.518</x:v>
+        <x:v>7270.954</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>373</x:v>
+        <x:v>531.8</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>3932.9</x:v>
+        <x:v>4464.7</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>280.9</x:v>
+        <x:v>297.6</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -562,25 +562,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-07-20</x:v>
+        <x:v>2026-07-21</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3831.659</x:v>
+        <x:v>3864.6</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3741.11</x:v>
+        <x:v>3743.36</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>90.5</x:v>
+        <x:v>121.2</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>1022.7</x:v>
+        <x:v>1143.9</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>73.1</x:v>
+        <x:v>76.3</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -591,25 +591,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-07-20</x:v>
+        <x:v>2026-07-21</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>7237</x:v>
+        <x:v>7175.8</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>6652.2</x:v>
+        <x:v>6641.8</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>584.8</x:v>
+        <x:v>534</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>3729.8</x:v>
+        <x:v>4263.8</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>266.4</x:v>
+        <x:v>284.3</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -620,25 +620,25 @@
         <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>2026-07-20</x:v>
+        <x:v>2026-07-21</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:v>7561.8</x:v>
+        <x:v>7700.6</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>7092</x:v>
+        <x:v>7201.2</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>469.8</x:v>
+        <x:v>499.4</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>3861.6</x:v>
+        <x:v>4361</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
-        <x:v>275.8</x:v>
+        <x:v>290.7</x:v>
       </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
@@ -649,25 +649,25 @@
         <x:v>IF主力</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>2026-07-20</x:v>
+        <x:v>2026-07-21</x:v>
       </x:c>
       <x:c r="C9" s="10" t="n">
-        <x:v>4590</x:v>
+        <x:v>4673.8</x:v>
       </x:c>
       <x:c r="D9" s="10" t="n">
-        <x:v>4465</x:v>
+        <x:v>4524.4</x:v>
       </x:c>
       <x:c r="E9" s="12" t="n">
-        <x:v>125</x:v>
+        <x:v>149.4</x:v>
       </x:c>
       <x:c r="F9" s="9" t="n">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G9" s="10" t="n">
-        <x:v>1451.2</x:v>
+        <x:v>1600.6</x:v>
       </x:c>
       <x:c r="H9" s="10" t="n">
-        <x:v>103.7</x:v>
+        <x:v>106.7</x:v>
       </x:c>
       <x:c r="I9" s="10" t="n">
         <x:v>90</x:v>
@@ -678,25 +678,25 @@
         <x:v>IH主力</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>2026-07-20</x:v>
+        <x:v>2026-07-21</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:v>2884.6</x:v>
+        <x:v>2933</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
-        <x:v>2820</x:v>
+        <x:v>2875.2</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
-        <x:v>64.6</x:v>
+        <x:v>57.8</x:v>
       </x:c>
       <x:c r="F10" s="9" t="n">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G10" s="10" t="n">
-        <x:v>795.8</x:v>
+        <x:v>853.6</x:v>
       </x:c>
       <x:c r="H10" s="10" t="n">
-        <x:v>56.8</x:v>
+        <x:v>56.9</x:v>
       </x:c>
       <x:c r="I10" s="10" t="n">
         <x:v>60</x:v>
@@ -710,7 +710,7 @@
         <x:v>2026-07-01</x:v>
       </x:c>
       <x:c r="C13" s="14" t="str">
-        <x:v>2026-07-20</x:v>
+        <x:v>2026-07-21</x:v>
       </x:c>
       <x:c r="D13" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1383,31 +1383,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="38" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B20" s="39" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C20" s="39"/>
-      <x:c r="D20" s="39"/>
-      <x:c r="E20" s="39"/>
-      <x:c r="F20" s="39"/>
-      <x:c r="G20" s="39"/>
-      <x:c r="H20" s="39"/>
-      <x:c r="I20" s="39"/>
-      <x:c r="J20" s="40" t="n">
-        <x:f>SUM(J4:J17)</x:f>
-        <x:v>3896.6000000000004</x:v>
-      </x:c>
-      <x:c r="K20" s="39"/>
+    <x:row r="18">
+      <x:c r="A18" s="21" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B18" s="21" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C18" s="21" t="str">
+        <x:v>7月21日</x:v>
+      </x:c>
+      <x:c r="D18" s="22" t="n">
+        <x:v>6975.893</x:v>
+      </x:c>
+      <x:c r="E18" s="22" t="n">
+        <x:v>7264.338</x:v>
+      </x:c>
+      <x:c r="F18" s="22" t="n">
+        <x:v>6714.187</x:v>
+      </x:c>
+      <x:c r="G18" s="22" t="n">
+        <x:v>7259.863</x:v>
+      </x:c>
+      <x:c r="H18" s="25" t="n">
+        <x:v>294.5</x:v>
+      </x:c>
+      <x:c r="I18" s="23" t="n">
+        <x:v>0.042278693928367916</x:v>
+      </x:c>
+      <x:c r="J18" s="27" t="n">
+        <x:f>ROUND(E18-F18,1)</x:f>
+        <x:v>550.2</x:v>
+      </x:c>
+      <x:c r="K18" s="21" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="38" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B21" s="39"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B21" s="39" t="n">
+        <x:v>15</x:v>
+      </x:c>
       <x:c r="C21" s="39"/>
       <x:c r="D21" s="39"/>
       <x:c r="E21" s="39"/>
@@ -1415,11 +1433,29 @@
       <x:c r="G21" s="39"/>
       <x:c r="H21" s="39"/>
       <x:c r="I21" s="39"/>
-      <x:c r="J21" s="42" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
-        <x:v>278.3</x:v>
+      <x:c r="J21" s="40" t="n">
+        <x:f>SUM(J4:J18)</x:f>
+        <x:v>4446.8</x:v>
       </x:c>
       <x:c r="K21" s="39"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="38" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B22" s="39"/>
+      <x:c r="C22" s="39"/>
+      <x:c r="D22" s="39"/>
+      <x:c r="E22" s="39"/>
+      <x:c r="F22" s="39"/>
+      <x:c r="G22" s="39"/>
+      <x:c r="H22" s="39"/>
+      <x:c r="I22" s="39"/>
+      <x:c r="J22" s="42" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
+        <x:v>296.5</x:v>
+      </x:c>
+      <x:c r="K22" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1990,31 +2026,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="38" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B20" s="39" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C20" s="39"/>
-      <x:c r="D20" s="39"/>
-      <x:c r="E20" s="39"/>
-      <x:c r="F20" s="39"/>
-      <x:c r="G20" s="39"/>
-      <x:c r="H20" s="39"/>
-      <x:c r="I20" s="39"/>
-      <x:c r="J20" s="40" t="n">
-        <x:f>SUM(J4:J17)</x:f>
-        <x:v>3932.9</x:v>
-      </x:c>
-      <x:c r="K20" s="39"/>
+    <x:row r="18">
+      <x:c r="A18" s="21" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B18" s="21" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C18" s="21" t="str">
+        <x:v>7月21日</x:v>
+      </x:c>
+      <x:c r="D18" s="22" t="n">
+        <x:v>7437.452</x:v>
+      </x:c>
+      <x:c r="E18" s="22" t="n">
+        <x:v>7802.755</x:v>
+      </x:c>
+      <x:c r="F18" s="22" t="n">
+        <x:v>7270.954</x:v>
+      </x:c>
+      <x:c r="G18" s="22" t="n">
+        <x:v>7800.609</x:v>
+      </x:c>
+      <x:c r="H18" s="25" t="n">
+        <x:v>389.3</x:v>
+      </x:c>
+      <x:c r="I18" s="23" t="n">
+        <x:v>0.052527264737031176</x:v>
+      </x:c>
+      <x:c r="J18" s="27" t="n">
+        <x:f>ROUND(E18-F18,1)</x:f>
+        <x:v>531.8</x:v>
+      </x:c>
+      <x:c r="K18" s="21" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="38" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B21" s="39"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B21" s="39" t="n">
+        <x:v>15</x:v>
+      </x:c>
       <x:c r="C21" s="39"/>
       <x:c r="D21" s="39"/>
       <x:c r="E21" s="39"/>
@@ -2022,11 +2076,29 @@
       <x:c r="G21" s="39"/>
       <x:c r="H21" s="39"/>
       <x:c r="I21" s="39"/>
-      <x:c r="J21" s="42" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
-        <x:v>280.9</x:v>
+      <x:c r="J21" s="40" t="n">
+        <x:f>SUM(J4:J18)</x:f>
+        <x:v>4464.7</x:v>
       </x:c>
       <x:c r="K21" s="39"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="38" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B22" s="39"/>
+      <x:c r="C22" s="39"/>
+      <x:c r="D22" s="39"/>
+      <x:c r="E22" s="39"/>
+      <x:c r="F22" s="39"/>
+      <x:c r="G22" s="39"/>
+      <x:c r="H22" s="39"/>
+      <x:c r="I22" s="39"/>
+      <x:c r="J22" s="42" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
+        <x:v>297.6</x:v>
+      </x:c>
+      <x:c r="K22" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2597,31 +2669,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="38" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B20" s="39" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C20" s="39"/>
-      <x:c r="D20" s="39"/>
-      <x:c r="E20" s="39"/>
-      <x:c r="F20" s="39"/>
-      <x:c r="G20" s="39"/>
-      <x:c r="H20" s="39"/>
-      <x:c r="I20" s="39"/>
-      <x:c r="J20" s="40" t="n">
-        <x:f>SUM(J4:J17)</x:f>
-        <x:v>1022.6999999999999</x:v>
-      </x:c>
-      <x:c r="K20" s="39"/>
+    <x:row r="18">
+      <x:c r="A18" s="21" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B18" s="21" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C18" s="21" t="str">
+        <x:v>7月21日</x:v>
+      </x:c>
+      <x:c r="D18" s="22" t="n">
+        <x:v>3812.162</x:v>
+      </x:c>
+      <x:c r="E18" s="22" t="n">
+        <x:v>3864.6</x:v>
+      </x:c>
+      <x:c r="F18" s="22" t="n">
+        <x:v>3743.36</x:v>
+      </x:c>
+      <x:c r="G18" s="22" t="n">
+        <x:v>3864.367</x:v>
+      </x:c>
+      <x:c r="H18" s="22" t="n">
+        <x:v>68.1</x:v>
+      </x:c>
+      <x:c r="I18" s="23" t="n">
+        <x:v>0.01793492104509653</x:v>
+      </x:c>
+      <x:c r="J18" s="27" t="n">
+        <x:f>ROUND(E18-F18,1)</x:f>
+        <x:v>121.2</x:v>
+      </x:c>
+      <x:c r="K18" s="21" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="38" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B21" s="39"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B21" s="39" t="n">
+        <x:v>15</x:v>
+      </x:c>
       <x:c r="C21" s="39"/>
       <x:c r="D21" s="39"/>
       <x:c r="E21" s="39"/>
@@ -2629,11 +2719,29 @@
       <x:c r="G21" s="39"/>
       <x:c r="H21" s="39"/>
       <x:c r="I21" s="39"/>
-      <x:c r="J21" s="42" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
-        <x:v>73.1</x:v>
+      <x:c r="J21" s="40" t="n">
+        <x:f>SUM(J4:J18)</x:f>
+        <x:v>1143.8999999999999</x:v>
       </x:c>
       <x:c r="K21" s="39"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="38" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B22" s="39"/>
+      <x:c r="C22" s="39"/>
+      <x:c r="D22" s="39"/>
+      <x:c r="E22" s="39"/>
+      <x:c r="F22" s="39"/>
+      <x:c r="G22" s="39"/>
+      <x:c r="H22" s="39"/>
+      <x:c r="I22" s="39"/>
+      <x:c r="J22" s="42" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
+        <x:v>76.3</x:v>
+      </x:c>
+      <x:c r="K22" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3204,31 +3312,49 @@
         <x:v>IM2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="38" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B20" s="39" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C20" s="39"/>
-      <x:c r="D20" s="39"/>
-      <x:c r="E20" s="39"/>
-      <x:c r="F20" s="39"/>
-      <x:c r="G20" s="39"/>
-      <x:c r="H20" s="39"/>
-      <x:c r="I20" s="39"/>
-      <x:c r="J20" s="40" t="n">
-        <x:f>SUM(J4:J17)</x:f>
-        <x:v>3729.8</x:v>
-      </x:c>
-      <x:c r="K20" s="39"/>
+    <x:row r="18">
+      <x:c r="A18" s="21" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B18" s="21" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C18" s="21" t="str">
+        <x:v>7月21日</x:v>
+      </x:c>
+      <x:c r="D18" s="22" t="n">
+        <x:v>6920</x:v>
+      </x:c>
+      <x:c r="E18" s="22" t="n">
+        <x:v>7175.8</x:v>
+      </x:c>
+      <x:c r="F18" s="22" t="n">
+        <x:v>6641.8</x:v>
+      </x:c>
+      <x:c r="G18" s="22" t="n">
+        <x:v>7164.4</x:v>
+      </x:c>
+      <x:c r="H18" s="25" t="n">
+        <x:v>314.6</x:v>
+      </x:c>
+      <x:c r="I18" s="23" t="n">
+        <x:v>0.04592834827294223</x:v>
+      </x:c>
+      <x:c r="J18" s="27" t="n">
+        <x:f>ROUND(E18-F18,1)</x:f>
+        <x:v>534</x:v>
+      </x:c>
+      <x:c r="K18" s="21" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="38" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B21" s="39"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B21" s="39" t="n">
+        <x:v>15</x:v>
+      </x:c>
       <x:c r="C21" s="39"/>
       <x:c r="D21" s="39"/>
       <x:c r="E21" s="39"/>
@@ -3236,11 +3362,29 @@
       <x:c r="G21" s="39"/>
       <x:c r="H21" s="39"/>
       <x:c r="I21" s="39"/>
-      <x:c r="J21" s="42" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
-        <x:v>266.4</x:v>
+      <x:c r="J21" s="40" t="n">
+        <x:f>SUM(J4:J18)</x:f>
+        <x:v>4263.8</x:v>
       </x:c>
       <x:c r="K21" s="39"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="38" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B22" s="39"/>
+      <x:c r="C22" s="39"/>
+      <x:c r="D22" s="39"/>
+      <x:c r="E22" s="39"/>
+      <x:c r="F22" s="39"/>
+      <x:c r="G22" s="39"/>
+      <x:c r="H22" s="39"/>
+      <x:c r="I22" s="39"/>
+      <x:c r="J22" s="42" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
+        <x:v>284.3</x:v>
+      </x:c>
+      <x:c r="K22" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3811,31 +3955,49 @@
         <x:v>IC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="38" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B20" s="39" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C20" s="39"/>
-      <x:c r="D20" s="39"/>
-      <x:c r="E20" s="39"/>
-      <x:c r="F20" s="39"/>
-      <x:c r="G20" s="39"/>
-      <x:c r="H20" s="39"/>
-      <x:c r="I20" s="39"/>
-      <x:c r="J20" s="40" t="n">
-        <x:f>SUM(J4:J17)</x:f>
-        <x:v>3861.6000000000004</x:v>
-      </x:c>
-      <x:c r="K20" s="39"/>
+    <x:row r="18">
+      <x:c r="A18" s="21" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B18" s="21" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C18" s="21" t="str">
+        <x:v>7月21日</x:v>
+      </x:c>
+      <x:c r="D18" s="22" t="n">
+        <x:v>7385</x:v>
+      </x:c>
+      <x:c r="E18" s="22" t="n">
+        <x:v>7700.6</x:v>
+      </x:c>
+      <x:c r="F18" s="22" t="n">
+        <x:v>7201.2</x:v>
+      </x:c>
+      <x:c r="G18" s="22" t="n">
+        <x:v>7685.8</x:v>
+      </x:c>
+      <x:c r="H18" s="25" t="n">
+        <x:v>383.6</x:v>
+      </x:c>
+      <x:c r="I18" s="23" t="n">
+        <x:v>0.052532113609597086</x:v>
+      </x:c>
+      <x:c r="J18" s="27" t="n">
+        <x:f>ROUND(E18-F18,1)</x:f>
+        <x:v>499.4</x:v>
+      </x:c>
+      <x:c r="K18" s="21" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="38" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B21" s="39"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B21" s="39" t="n">
+        <x:v>15</x:v>
+      </x:c>
       <x:c r="C21" s="39"/>
       <x:c r="D21" s="39"/>
       <x:c r="E21" s="39"/>
@@ -3843,11 +4005,29 @@
       <x:c r="G21" s="39"/>
       <x:c r="H21" s="39"/>
       <x:c r="I21" s="39"/>
-      <x:c r="J21" s="42" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
-        <x:v>275.8</x:v>
+      <x:c r="J21" s="40" t="n">
+        <x:f>SUM(J4:J18)</x:f>
+        <x:v>4361</x:v>
       </x:c>
       <x:c r="K21" s="39"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="38" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B22" s="39"/>
+      <x:c r="C22" s="39"/>
+      <x:c r="D22" s="39"/>
+      <x:c r="E22" s="39"/>
+      <x:c r="F22" s="39"/>
+      <x:c r="G22" s="39"/>
+      <x:c r="H22" s="39"/>
+      <x:c r="I22" s="39"/>
+      <x:c r="J22" s="42" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
+        <x:v>290.7</x:v>
+      </x:c>
+      <x:c r="K22" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4418,31 +4598,49 @@
         <x:v>IF2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="38" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B20" s="39" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C20" s="39"/>
-      <x:c r="D20" s="39"/>
-      <x:c r="E20" s="39"/>
-      <x:c r="F20" s="39"/>
-      <x:c r="G20" s="39"/>
-      <x:c r="H20" s="39"/>
-      <x:c r="I20" s="39"/>
-      <x:c r="J20" s="40" t="n">
-        <x:f>SUM(J4:J17)</x:f>
-        <x:v>1451.2</x:v>
-      </x:c>
-      <x:c r="K20" s="39"/>
+    <x:row r="18">
+      <x:c r="A18" s="21" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B18" s="21" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C18" s="21" t="str">
+        <x:v>7月21日</x:v>
+      </x:c>
+      <x:c r="D18" s="22" t="n">
+        <x:v>4563.8</x:v>
+      </x:c>
+      <x:c r="E18" s="22" t="n">
+        <x:v>4673.8</x:v>
+      </x:c>
+      <x:c r="F18" s="22" t="n">
+        <x:v>4524.4</x:v>
+      </x:c>
+      <x:c r="G18" s="22" t="n">
+        <x:v>4662.4</x:v>
+      </x:c>
+      <x:c r="H18" s="22" t="n">
+        <x:v>116.6</x:v>
+      </x:c>
+      <x:c r="I18" s="23" t="n">
+        <x:v>0.02565005059615455</x:v>
+      </x:c>
+      <x:c r="J18" s="27" t="n">
+        <x:f>ROUND(E18-F18,1)</x:f>
+        <x:v>149.4</x:v>
+      </x:c>
+      <x:c r="K18" s="21" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="38" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B21" s="39"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B21" s="39" t="n">
+        <x:v>15</x:v>
+      </x:c>
       <x:c r="C21" s="39"/>
       <x:c r="D21" s="39"/>
       <x:c r="E21" s="39"/>
@@ -4450,11 +4648,29 @@
       <x:c r="G21" s="39"/>
       <x:c r="H21" s="39"/>
       <x:c r="I21" s="39"/>
-      <x:c r="J21" s="42" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
-        <x:v>103.7</x:v>
+      <x:c r="J21" s="40" t="n">
+        <x:f>SUM(J4:J18)</x:f>
+        <x:v>1600.6000000000001</x:v>
       </x:c>
       <x:c r="K21" s="39"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="38" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B22" s="39"/>
+      <x:c r="C22" s="39"/>
+      <x:c r="D22" s="39"/>
+      <x:c r="E22" s="39"/>
+      <x:c r="F22" s="39"/>
+      <x:c r="G22" s="39"/>
+      <x:c r="H22" s="39"/>
+      <x:c r="I22" s="39"/>
+      <x:c r="J22" s="42" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
+        <x:v>106.7</x:v>
+      </x:c>
+      <x:c r="K22" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5025,31 +5241,49 @@
         <x:v>IH2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="38" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B20" s="39" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C20" s="39"/>
-      <x:c r="D20" s="39"/>
-      <x:c r="E20" s="39"/>
-      <x:c r="F20" s="39"/>
-      <x:c r="G20" s="39"/>
-      <x:c r="H20" s="39"/>
-      <x:c r="I20" s="39"/>
-      <x:c r="J20" s="40" t="n">
-        <x:f>SUM(J4:J17)</x:f>
-        <x:v>795.8000000000001</x:v>
-      </x:c>
-      <x:c r="K20" s="39"/>
+    <x:row r="18">
+      <x:c r="A18" s="21" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B18" s="21" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C18" s="21" t="str">
+        <x:v>7月21日</x:v>
+      </x:c>
+      <x:c r="D18" s="22" t="n">
+        <x:v>2896</x:v>
+      </x:c>
+      <x:c r="E18" s="22" t="n">
+        <x:v>2933</x:v>
+      </x:c>
+      <x:c r="F18" s="22" t="n">
+        <x:v>2875.2</x:v>
+      </x:c>
+      <x:c r="G18" s="22" t="n">
+        <x:v>2923.6</x:v>
+      </x:c>
+      <x:c r="H18" s="22" t="n">
+        <x:v>49.6</x:v>
+      </x:c>
+      <x:c r="I18" s="23" t="n">
+        <x:v>0.017258176757132926</x:v>
+      </x:c>
+      <x:c r="J18" s="22" t="n">
+        <x:f>ROUND(E18-F18,1)</x:f>
+        <x:v>57.8</x:v>
+      </x:c>
+      <x:c r="K18" s="21" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="38" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B21" s="39"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B21" s="39" t="n">
+        <x:v>15</x:v>
+      </x:c>
       <x:c r="C21" s="39"/>
       <x:c r="D21" s="39"/>
       <x:c r="E21" s="39"/>
@@ -5057,11 +5291,29 @@
       <x:c r="G21" s="39"/>
       <x:c r="H21" s="39"/>
       <x:c r="I21" s="39"/>
-      <x:c r="J21" s="42" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
-        <x:v>56.8</x:v>
+      <x:c r="J21" s="40" t="n">
+        <x:f>SUM(J4:J18)</x:f>
+        <x:v>853.6</x:v>
       </x:c>
       <x:c r="K21" s="39"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="38" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B22" s="39"/>
+      <x:c r="C22" s="39"/>
+      <x:c r="D22" s="39"/>
+      <x:c r="E22" s="39"/>
+      <x:c r="F22" s="39"/>
+      <x:c r="G22" s="39"/>
+      <x:c r="H22" s="39"/>
+      <x:c r="I22" s="39"/>
+      <x:c r="J22" s="42" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
+        <x:v>56.9</x:v>
+      </x:c>
+      <x:c r="K22" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-07-22
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Ra8e8a498c4814f8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="2" r:id="R0ed5dd17dd7640c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="3" r:id="Rfc3f07345f2940e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="4" r:id="Rbbc8fc1d26594eae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="5" r:id="R0d490363f08d44f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="6" r:id="Ra73225998cf1411f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="7" r:id="R88cb62827fa144b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="8" r:id="Re99638923f2f43ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R605b1f3b46e74e21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="2" r:id="R7980cb43aaf0460e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="3" r:id="Rdcbb999361d54eca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="4" r:id="R790f1c59bfa8430e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="5" r:id="Re839fa9c001b4ab5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="6" r:id="R79e3903ed2e44388"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="7" r:id="Rfe938295c48a450d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="8" r:id="R591e6633a1c9476f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -504,25 +504,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-07-21</x:v>
+        <x:v>2026-07-22</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7264.338</x:v>
+        <x:v>7302.454</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>6714.187</x:v>
+        <x:v>7118.66</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>550.2</x:v>
+        <x:v>183.8</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>4446.8</x:v>
+        <x:v>4630.6</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>296.5</x:v>
+        <x:v>289.4</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -533,25 +533,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-07-21</x:v>
+        <x:v>2026-07-22</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7802.755</x:v>
+        <x:v>7889.446</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7270.954</x:v>
+        <x:v>7701.221</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>531.8</x:v>
+        <x:v>188.2</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>4464.7</x:v>
+        <x:v>4652.9</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>297.6</x:v>
+        <x:v>290.8</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -562,25 +562,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-07-21</x:v>
+        <x:v>2026-07-22</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3864.6</x:v>
+        <x:v>3884.435</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3743.36</x:v>
+        <x:v>3839.665</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>121.2</x:v>
+        <x:v>44.8</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>1143.9</x:v>
+        <x:v>1188.7</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>76.3</x:v>
+        <x:v>74.3</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -591,25 +591,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-07-21</x:v>
+        <x:v>2026-07-22</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>7175.8</x:v>
+        <x:v>7194.6</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>6641.8</x:v>
+        <x:v>6985.8</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>534</x:v>
+        <x:v>208.8</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>4263.8</x:v>
+        <x:v>4472.6</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>284.3</x:v>
+        <x:v>279.5</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -620,25 +620,25 @@
         <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>2026-07-21</x:v>
+        <x:v>2026-07-22</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:v>7700.6</x:v>
+        <x:v>7765.6</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>7201.2</x:v>
+        <x:v>7583.8</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>499.4</x:v>
+        <x:v>181.8</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>4361</x:v>
+        <x:v>4542.8</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
-        <x:v>290.7</x:v>
+        <x:v>283.9</x:v>
       </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
@@ -710,7 +710,7 @@
         <x:v>2026-07-01</x:v>
       </x:c>
       <x:c r="C13" s="14" t="str">
-        <x:v>2026-07-21</x:v>
+        <x:v>2026-07-22</x:v>
       </x:c>
       <x:c r="D13" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1419,31 +1419,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="38" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B21" s="39" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C21" s="39"/>
-      <x:c r="D21" s="39"/>
-      <x:c r="E21" s="39"/>
-      <x:c r="F21" s="39"/>
-      <x:c r="G21" s="39"/>
-      <x:c r="H21" s="39"/>
-      <x:c r="I21" s="39"/>
-      <x:c r="J21" s="40" t="n">
-        <x:f>SUM(J4:J18)</x:f>
-        <x:v>4446.8</x:v>
-      </x:c>
-      <x:c r="K21" s="39"/>
+    <x:row r="19">
+      <x:c r="A19" s="21" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B19" s="21" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C19" s="21" t="str">
+        <x:v>7月22日</x:v>
+      </x:c>
+      <x:c r="D19" s="22" t="n">
+        <x:v>7196.863</x:v>
+      </x:c>
+      <x:c r="E19" s="22" t="n">
+        <x:v>7302.454</x:v>
+      </x:c>
+      <x:c r="F19" s="22" t="n">
+        <x:v>7118.66</x:v>
+      </x:c>
+      <x:c r="G19" s="22" t="n">
+        <x:v>7158.762</x:v>
+      </x:c>
+      <x:c r="H19" s="22" t="n">
+        <x:v>-101.1</x:v>
+      </x:c>
+      <x:c r="I19" s="23" t="n">
+        <x:v>-0.01392602036705104</x:v>
+      </x:c>
+      <x:c r="J19" s="27" t="n">
+        <x:f>ROUND(E19-F19,1)</x:f>
+        <x:v>183.8</x:v>
+      </x:c>
+      <x:c r="K19" s="21" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="38" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B22" s="39"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B22" s="39" t="n">
+        <x:v>16</x:v>
+      </x:c>
       <x:c r="C22" s="39"/>
       <x:c r="D22" s="39"/>
       <x:c r="E22" s="39"/>
@@ -1451,11 +1469,29 @@
       <x:c r="G22" s="39"/>
       <x:c r="H22" s="39"/>
       <x:c r="I22" s="39"/>
-      <x:c r="J22" s="42" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
-        <x:v>296.5</x:v>
+      <x:c r="J22" s="40" t="n">
+        <x:f>SUM(J4:J19)</x:f>
+        <x:v>4630.6</x:v>
       </x:c>
       <x:c r="K22" s="39"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="38" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B23" s="39"/>
+      <x:c r="C23" s="39"/>
+      <x:c r="D23" s="39"/>
+      <x:c r="E23" s="39"/>
+      <x:c r="F23" s="39"/>
+      <x:c r="G23" s="39"/>
+      <x:c r="H23" s="39"/>
+      <x:c r="I23" s="39"/>
+      <x:c r="J23" s="42" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
+        <x:v>289.4</x:v>
+      </x:c>
+      <x:c r="K23" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2062,31 +2098,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="38" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B21" s="39" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C21" s="39"/>
-      <x:c r="D21" s="39"/>
-      <x:c r="E21" s="39"/>
-      <x:c r="F21" s="39"/>
-      <x:c r="G21" s="39"/>
-      <x:c r="H21" s="39"/>
-      <x:c r="I21" s="39"/>
-      <x:c r="J21" s="40" t="n">
-        <x:f>SUM(J4:J18)</x:f>
-        <x:v>4464.7</x:v>
-      </x:c>
-      <x:c r="K21" s="39"/>
+    <x:row r="19">
+      <x:c r="A19" s="21" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B19" s="21" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C19" s="21" t="str">
+        <x:v>7月22日</x:v>
+      </x:c>
+      <x:c r="D19" s="22" t="n">
+        <x:v>7741.906</x:v>
+      </x:c>
+      <x:c r="E19" s="22" t="n">
+        <x:v>7889.446</x:v>
+      </x:c>
+      <x:c r="F19" s="22" t="n">
+        <x:v>7701.221</x:v>
+      </x:c>
+      <x:c r="G19" s="22" t="n">
+        <x:v>7751.662</x:v>
+      </x:c>
+      <x:c r="H19" s="22" t="n">
+        <x:v>-48.9</x:v>
+      </x:c>
+      <x:c r="I19" s="23" t="n">
+        <x:v>-0.006274766495795392</x:v>
+      </x:c>
+      <x:c r="J19" s="27" t="n">
+        <x:f>ROUND(E19-F19,1)</x:f>
+        <x:v>188.2</x:v>
+      </x:c>
+      <x:c r="K19" s="21" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="38" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B22" s="39"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B22" s="39" t="n">
+        <x:v>16</x:v>
+      </x:c>
       <x:c r="C22" s="39"/>
       <x:c r="D22" s="39"/>
       <x:c r="E22" s="39"/>
@@ -2094,11 +2148,29 @@
       <x:c r="G22" s="39"/>
       <x:c r="H22" s="39"/>
       <x:c r="I22" s="39"/>
-      <x:c r="J22" s="42" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
-        <x:v>297.6</x:v>
+      <x:c r="J22" s="40" t="n">
+        <x:f>SUM(J4:J19)</x:f>
+        <x:v>4652.9</x:v>
       </x:c>
       <x:c r="K22" s="39"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="38" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B23" s="39"/>
+      <x:c r="C23" s="39"/>
+      <x:c r="D23" s="39"/>
+      <x:c r="E23" s="39"/>
+      <x:c r="F23" s="39"/>
+      <x:c r="G23" s="39"/>
+      <x:c r="H23" s="39"/>
+      <x:c r="I23" s="39"/>
+      <x:c r="J23" s="42" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
+        <x:v>290.8</x:v>
+      </x:c>
+      <x:c r="K23" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2705,31 +2777,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="38" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B21" s="39" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C21" s="39"/>
-      <x:c r="D21" s="39"/>
-      <x:c r="E21" s="39"/>
-      <x:c r="F21" s="39"/>
-      <x:c r="G21" s="39"/>
-      <x:c r="H21" s="39"/>
-      <x:c r="I21" s="39"/>
-      <x:c r="J21" s="40" t="n">
-        <x:f>SUM(J4:J18)</x:f>
-        <x:v>1143.8999999999999</x:v>
-      </x:c>
-      <x:c r="K21" s="39"/>
+    <x:row r="19">
+      <x:c r="A19" s="21" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B19" s="21" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C19" s="21" t="str">
+        <x:v>7月22日</x:v>
+      </x:c>
+      <x:c r="D19" s="22" t="n">
+        <x:v>3839.665</x:v>
+      </x:c>
+      <x:c r="E19" s="22" t="n">
+        <x:v>3884.435</x:v>
+      </x:c>
+      <x:c r="F19" s="22" t="n">
+        <x:v>3839.665</x:v>
+      </x:c>
+      <x:c r="G19" s="22" t="n">
+        <x:v>3867.034</x:v>
+      </x:c>
+      <x:c r="H19" s="22" t="n">
+        <x:v>2.7</x:v>
+      </x:c>
+      <x:c r="I19" s="23" t="n">
+        <x:v>0.0006901518411681629</x:v>
+      </x:c>
+      <x:c r="J19" s="22" t="n">
+        <x:f>ROUND(E19-F19,1)</x:f>
+        <x:v>44.8</x:v>
+      </x:c>
+      <x:c r="K19" s="21" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="38" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B22" s="39"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B22" s="39" t="n">
+        <x:v>16</x:v>
+      </x:c>
       <x:c r="C22" s="39"/>
       <x:c r="D22" s="39"/>
       <x:c r="E22" s="39"/>
@@ -2737,11 +2827,29 @@
       <x:c r="G22" s="39"/>
       <x:c r="H22" s="39"/>
       <x:c r="I22" s="39"/>
-      <x:c r="J22" s="42" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
-        <x:v>76.3</x:v>
+      <x:c r="J22" s="40" t="n">
+        <x:f>SUM(J4:J19)</x:f>
+        <x:v>1188.6999999999998</x:v>
       </x:c>
       <x:c r="K22" s="39"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="38" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B23" s="39"/>
+      <x:c r="C23" s="39"/>
+      <x:c r="D23" s="39"/>
+      <x:c r="E23" s="39"/>
+      <x:c r="F23" s="39"/>
+      <x:c r="G23" s="39"/>
+      <x:c r="H23" s="39"/>
+      <x:c r="I23" s="39"/>
+      <x:c r="J23" s="42" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
+        <x:v>74.3</x:v>
+      </x:c>
+      <x:c r="K23" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3348,31 +3456,49 @@
         <x:v>IM2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="38" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B21" s="39" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C21" s="39"/>
-      <x:c r="D21" s="39"/>
-      <x:c r="E21" s="39"/>
-      <x:c r="F21" s="39"/>
-      <x:c r="G21" s="39"/>
-      <x:c r="H21" s="39"/>
-      <x:c r="I21" s="39"/>
-      <x:c r="J21" s="40" t="n">
-        <x:f>SUM(J4:J18)</x:f>
-        <x:v>4263.8</x:v>
-      </x:c>
-      <x:c r="K21" s="39"/>
+    <x:row r="19">
+      <x:c r="A19" s="21" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B19" s="21" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C19" s="21" t="str">
+        <x:v>7月22日</x:v>
+      </x:c>
+      <x:c r="D19" s="22" t="n">
+        <x:v>7148</x:v>
+      </x:c>
+      <x:c r="E19" s="22" t="n">
+        <x:v>7194.6</x:v>
+      </x:c>
+      <x:c r="F19" s="22" t="n">
+        <x:v>6985.8</x:v>
+      </x:c>
+      <x:c r="G19" s="22" t="n">
+        <x:v>7028.8</x:v>
+      </x:c>
+      <x:c r="H19" s="22" t="n">
+        <x:v>-135.6</x:v>
+      </x:c>
+      <x:c r="I19" s="23" t="n">
+        <x:v>-0.018926916420076934</x:v>
+      </x:c>
+      <x:c r="J19" s="27" t="n">
+        <x:f>ROUND(E19-F19,1)</x:f>
+        <x:v>208.8</x:v>
+      </x:c>
+      <x:c r="K19" s="21" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="38" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B22" s="39"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B22" s="39" t="n">
+        <x:v>16</x:v>
+      </x:c>
       <x:c r="C22" s="39"/>
       <x:c r="D22" s="39"/>
       <x:c r="E22" s="39"/>
@@ -3380,11 +3506,29 @@
       <x:c r="G22" s="39"/>
       <x:c r="H22" s="39"/>
       <x:c r="I22" s="39"/>
-      <x:c r="J22" s="42" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
-        <x:v>284.3</x:v>
+      <x:c r="J22" s="40" t="n">
+        <x:f>SUM(J4:J19)</x:f>
+        <x:v>4472.6</x:v>
       </x:c>
       <x:c r="K22" s="39"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="38" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B23" s="39"/>
+      <x:c r="C23" s="39"/>
+      <x:c r="D23" s="39"/>
+      <x:c r="E23" s="39"/>
+      <x:c r="F23" s="39"/>
+      <x:c r="G23" s="39"/>
+      <x:c r="H23" s="39"/>
+      <x:c r="I23" s="39"/>
+      <x:c r="J23" s="42" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
+        <x:v>279.5</x:v>
+      </x:c>
+      <x:c r="K23" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3991,31 +4135,49 @@
         <x:v>IC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="38" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B21" s="39" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C21" s="39"/>
-      <x:c r="D21" s="39"/>
-      <x:c r="E21" s="39"/>
-      <x:c r="F21" s="39"/>
-      <x:c r="G21" s="39"/>
-      <x:c r="H21" s="39"/>
-      <x:c r="I21" s="39"/>
-      <x:c r="J21" s="40" t="n">
-        <x:f>SUM(J4:J18)</x:f>
-        <x:v>4361</x:v>
-      </x:c>
-      <x:c r="K21" s="39"/>
+    <x:row r="19">
+      <x:c r="A19" s="21" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B19" s="21" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C19" s="21" t="str">
+        <x:v>7月22日</x:v>
+      </x:c>
+      <x:c r="D19" s="22" t="n">
+        <x:v>7674.8</x:v>
+      </x:c>
+      <x:c r="E19" s="22" t="n">
+        <x:v>7765.6</x:v>
+      </x:c>
+      <x:c r="F19" s="22" t="n">
+        <x:v>7583.8</x:v>
+      </x:c>
+      <x:c r="G19" s="22" t="n">
+        <x:v>7611</x:v>
+      </x:c>
+      <x:c r="H19" s="22" t="n">
+        <x:v>-74.8</x:v>
+      </x:c>
+      <x:c r="I19" s="23" t="n">
+        <x:v>-0.009732233469515239</x:v>
+      </x:c>
+      <x:c r="J19" s="27" t="n">
+        <x:f>ROUND(E19-F19,1)</x:f>
+        <x:v>181.8</x:v>
+      </x:c>
+      <x:c r="K19" s="21" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="38" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B22" s="39"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B22" s="39" t="n">
+        <x:v>16</x:v>
+      </x:c>
       <x:c r="C22" s="39"/>
       <x:c r="D22" s="39"/>
       <x:c r="E22" s="39"/>
@@ -4023,11 +4185,29 @@
       <x:c r="G22" s="39"/>
       <x:c r="H22" s="39"/>
       <x:c r="I22" s="39"/>
-      <x:c r="J22" s="42" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
-        <x:v>290.7</x:v>
+      <x:c r="J22" s="40" t="n">
+        <x:f>SUM(J4:J19)</x:f>
+        <x:v>4542.8</x:v>
       </x:c>
       <x:c r="K22" s="39"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="38" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B23" s="39"/>
+      <x:c r="C23" s="39"/>
+      <x:c r="D23" s="39"/>
+      <x:c r="E23" s="39"/>
+      <x:c r="F23" s="39"/>
+      <x:c r="G23" s="39"/>
+      <x:c r="H23" s="39"/>
+      <x:c r="I23" s="39"/>
+      <x:c r="J23" s="42" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
+        <x:v>283.9</x:v>
+      </x:c>
+      <x:c r="K23" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-07-23
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Ra5a8ccd4c8b24085"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="2" r:id="R247cd7bd2997429a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="3" r:id="Rcff06f0c30f4472e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="4" r:id="R54b6e10631014f57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="5" r:id="R2f14a8389e734c6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="6" r:id="R502456081abd4190"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="7" r:id="R50521e01858e45f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="8" r:id="Rd635f3ae6f4b4dc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R195fddeadd404999"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="2" r:id="Re0b55415a2f849d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="3" r:id="Rbbbc0d8167664efc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="4" r:id="R91c32729d2df4353"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="5" r:id="R7298744e8cd3401e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="6" r:id="Rfc6a73ef47c4453f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="7" r:id="Rccef4ad20afb4a23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="8" r:id="Rd929ab10a4414784"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -504,25 +504,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-23</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7302.454</x:v>
+        <x:v>7247.141</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7118.66</x:v>
+        <x:v>7113.498</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>183.8</x:v>
+        <x:v>133.6</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>4630.6</x:v>
+        <x:v>4764.2</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>289.4</x:v>
+        <x:v>280.2</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -533,25 +533,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-23</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7889.446</x:v>
+        <x:v>7795.35</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7701.221</x:v>
+        <x:v>7658.999</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>188.2</x:v>
+        <x:v>136.4</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>4652.9</x:v>
+        <x:v>4789.3</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>290.8</x:v>
+        <x:v>281.7</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -562,25 +562,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-23</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3884.435</x:v>
+        <x:v>3878.832</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3839.665</x:v>
+        <x:v>3851.706</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>44.8</x:v>
+        <x:v>27.1</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>1188.7</x:v>
+        <x:v>1215.8</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>74.3</x:v>
+        <x:v>71.5</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -710,7 +710,7 @@
         <x:v>2026-07-01</x:v>
       </x:c>
       <x:c r="C13" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-23</x:v>
       </x:c>
       <x:c r="D13" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1455,31 +1455,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="38" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B22" s="39" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="C22" s="39"/>
-      <x:c r="D22" s="39"/>
-      <x:c r="E22" s="39"/>
-      <x:c r="F22" s="39"/>
-      <x:c r="G22" s="39"/>
-      <x:c r="H22" s="39"/>
-      <x:c r="I22" s="39"/>
-      <x:c r="J22" s="40" t="n">
-        <x:f>SUM(J4:J19)</x:f>
-        <x:v>4630.6</x:v>
-      </x:c>
-      <x:c r="K22" s="39"/>
+    <x:row r="20">
+      <x:c r="A20" s="21" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B20" s="21" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C20" s="21" t="str">
+        <x:v>7月23日</x:v>
+      </x:c>
+      <x:c r="D20" s="22" t="n">
+        <x:v>7169.543</x:v>
+      </x:c>
+      <x:c r="E20" s="22" t="n">
+        <x:v>7247.141</x:v>
+      </x:c>
+      <x:c r="F20" s="22" t="n">
+        <x:v>7113.498</x:v>
+      </x:c>
+      <x:c r="G20" s="22" t="n">
+        <x:v>7195.5</x:v>
+      </x:c>
+      <x:c r="H20" s="22" t="n">
+        <x:v>36.7</x:v>
+      </x:c>
+      <x:c r="I20" s="23" t="n">
+        <x:v>0.0051318929166803695</x:v>
+      </x:c>
+      <x:c r="J20" s="22" t="n">
+        <x:f>ROUND(E20-F20,1)</x:f>
+        <x:v>133.6</x:v>
+      </x:c>
+      <x:c r="K20" s="21" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="38" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B23" s="39"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B23" s="39" t="n">
+        <x:v>17</x:v>
+      </x:c>
       <x:c r="C23" s="39"/>
       <x:c r="D23" s="39"/>
       <x:c r="E23" s="39"/>
@@ -1487,11 +1505,29 @@
       <x:c r="G23" s="39"/>
       <x:c r="H23" s="39"/>
       <x:c r="I23" s="39"/>
-      <x:c r="J23" s="42" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
-        <x:v>289.4</x:v>
+      <x:c r="J23" s="40" t="n">
+        <x:f>SUM(J4:J20)</x:f>
+        <x:v>4764.200000000001</x:v>
       </x:c>
       <x:c r="K23" s="39"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="38" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B24" s="39"/>
+      <x:c r="C24" s="39"/>
+      <x:c r="D24" s="39"/>
+      <x:c r="E24" s="39"/>
+      <x:c r="F24" s="39"/>
+      <x:c r="G24" s="39"/>
+      <x:c r="H24" s="39"/>
+      <x:c r="I24" s="39"/>
+      <x:c r="J24" s="42" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
+        <x:v>280.2</x:v>
+      </x:c>
+      <x:c r="K24" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2134,31 +2170,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="38" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B22" s="39" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="C22" s="39"/>
-      <x:c r="D22" s="39"/>
-      <x:c r="E22" s="39"/>
-      <x:c r="F22" s="39"/>
-      <x:c r="G22" s="39"/>
-      <x:c r="H22" s="39"/>
-      <x:c r="I22" s="39"/>
-      <x:c r="J22" s="40" t="n">
-        <x:f>SUM(J4:J19)</x:f>
-        <x:v>4652.9</x:v>
-      </x:c>
-      <x:c r="K22" s="39"/>
+    <x:row r="20">
+      <x:c r="A20" s="21" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B20" s="21" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C20" s="21" t="str">
+        <x:v>7月23日</x:v>
+      </x:c>
+      <x:c r="D20" s="22" t="n">
+        <x:v>7750.852</x:v>
+      </x:c>
+      <x:c r="E20" s="22" t="n">
+        <x:v>7795.35</x:v>
+      </x:c>
+      <x:c r="F20" s="22" t="n">
+        <x:v>7658.999</x:v>
+      </x:c>
+      <x:c r="G20" s="22" t="n">
+        <x:v>7734.31</x:v>
+      </x:c>
+      <x:c r="H20" s="22" t="n">
+        <x:v>-17.4</x:v>
+      </x:c>
+      <x:c r="I20" s="23" t="n">
+        <x:v>-0.0022384876946388577</x:v>
+      </x:c>
+      <x:c r="J20" s="22" t="n">
+        <x:f>ROUND(E20-F20,1)</x:f>
+        <x:v>136.4</x:v>
+      </x:c>
+      <x:c r="K20" s="21" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="38" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B23" s="39"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B23" s="39" t="n">
+        <x:v>17</x:v>
+      </x:c>
       <x:c r="C23" s="39"/>
       <x:c r="D23" s="39"/>
       <x:c r="E23" s="39"/>
@@ -2166,11 +2220,29 @@
       <x:c r="G23" s="39"/>
       <x:c r="H23" s="39"/>
       <x:c r="I23" s="39"/>
-      <x:c r="J23" s="42" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
-        <x:v>290.8</x:v>
+      <x:c r="J23" s="40" t="n">
+        <x:f>SUM(J4:J20)</x:f>
+        <x:v>4789.299999999999</x:v>
       </x:c>
       <x:c r="K23" s="39"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="38" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B24" s="39"/>
+      <x:c r="C24" s="39"/>
+      <x:c r="D24" s="39"/>
+      <x:c r="E24" s="39"/>
+      <x:c r="F24" s="39"/>
+      <x:c r="G24" s="39"/>
+      <x:c r="H24" s="39"/>
+      <x:c r="I24" s="39"/>
+      <x:c r="J24" s="42" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
+        <x:v>281.7</x:v>
+      </x:c>
+      <x:c r="K24" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2813,31 +2885,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="38" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B22" s="39" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="C22" s="39"/>
-      <x:c r="D22" s="39"/>
-      <x:c r="E22" s="39"/>
-      <x:c r="F22" s="39"/>
-      <x:c r="G22" s="39"/>
-      <x:c r="H22" s="39"/>
-      <x:c r="I22" s="39"/>
-      <x:c r="J22" s="40" t="n">
-        <x:f>SUM(J4:J19)</x:f>
-        <x:v>1188.6999999999998</x:v>
-      </x:c>
-      <x:c r="K22" s="39"/>
+    <x:row r="20">
+      <x:c r="A20" s="21" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B20" s="21" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C20" s="21" t="str">
+        <x:v>7月23日</x:v>
+      </x:c>
+      <x:c r="D20" s="22" t="n">
+        <x:v>3868.087</x:v>
+      </x:c>
+      <x:c r="E20" s="22" t="n">
+        <x:v>3878.832</x:v>
+      </x:c>
+      <x:c r="F20" s="22" t="n">
+        <x:v>3851.706</x:v>
+      </x:c>
+      <x:c r="G20" s="22" t="n">
+        <x:v>3876.777</x:v>
+      </x:c>
+      <x:c r="H20" s="22" t="n">
+        <x:v>9.7</x:v>
+      </x:c>
+      <x:c r="I20" s="23" t="n">
+        <x:v>0.0025195020266177703</x:v>
+      </x:c>
+      <x:c r="J20" s="22" t="n">
+        <x:f>ROUND(E20-F20,1)</x:f>
+        <x:v>27.1</x:v>
+      </x:c>
+      <x:c r="K20" s="21" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="38" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B23" s="39"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B23" s="39" t="n">
+        <x:v>17</x:v>
+      </x:c>
       <x:c r="C23" s="39"/>
       <x:c r="D23" s="39"/>
       <x:c r="E23" s="39"/>
@@ -2845,11 +2935,29 @@
       <x:c r="G23" s="39"/>
       <x:c r="H23" s="39"/>
       <x:c r="I23" s="39"/>
-      <x:c r="J23" s="42" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
-        <x:v>74.3</x:v>
+      <x:c r="J23" s="40" t="n">
+        <x:f>SUM(J4:J20)</x:f>
+        <x:v>1215.7999999999997</x:v>
       </x:c>
       <x:c r="K23" s="39"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="38" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B24" s="39"/>
+      <x:c r="C24" s="39"/>
+      <x:c r="D24" s="39"/>
+      <x:c r="E24" s="39"/>
+      <x:c r="F24" s="39"/>
+      <x:c r="G24" s="39"/>
+      <x:c r="H24" s="39"/>
+      <x:c r="I24" s="39"/>
+      <x:c r="J24" s="42" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
+        <x:v>71.5</x:v>
+      </x:c>
+      <x:c r="K24" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-07-31
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R5c093119470d493b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="2" r:id="Rb16e6c46bad04a80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="3" r:id="R26aabe8e4a414d51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="4" r:id="R6637b9b171c545ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="5" r:id="R03bfe7d97db24c22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="6" r:id="R5dfa1056d0704c62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="7" r:id="R2ad8a6580f2248c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="8" r:id="R8dab89f43d014194"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Ree9f6a9b28664b4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="2" r:id="R26a7372c1ad84e9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="3" r:id="R8f858f11acd840bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="4" r:id="Rb7c6fc3be46d4163"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="5" r:id="Ra1a20f2a81204b27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="6" r:id="R835842e16a674103"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="7" r:id="R1a15533f58974ac8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="8" r:id="R17817fe79a0e48da"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -504,25 +504,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-07-23</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7247.141</x:v>
+        <x:v>7218.06</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7113.498</x:v>
+        <x:v>7071.05</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>133.6</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>17</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>4764.2</x:v>
+        <x:v>6057.6</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>280.2</x:v>
+        <x:v>263.4</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -533,25 +533,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-07-23</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7795.35</x:v>
+        <x:v>7638.78</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7658.999</x:v>
+        <x:v>7487.43</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>136.4</x:v>
+        <x:v>151.3</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>17</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>4789.3</x:v>
+        <x:v>6161.7</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>281.7</x:v>
+        <x:v>267.9</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -562,25 +562,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-07-23</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3878.832</x:v>
+        <x:v>3847.09</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3851.706</x:v>
+        <x:v>3822.37</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>27.1</x:v>
+        <x:v>24.7</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>17</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>1215.8</x:v>
+        <x:v>1539.5</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>71.5</x:v>
+        <x:v>66.9</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -591,25 +591,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-07-23</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>7159.6</x:v>
+        <x:v>7205</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>7000.6</x:v>
+        <x:v>6986</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>159</x:v>
+        <x:v>219</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>17</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>4631.6</x:v>
+        <x:v>6087.2</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>272.4</x:v>
+        <x:v>264.7</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -620,25 +620,25 @@
         <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>2026-07-23</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:v>7693</x:v>
+        <x:v>7611.8</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>7538</x:v>
+        <x:v>7389.6</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>155</x:v>
+        <x:v>222.2</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>17</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>4697.8</x:v>
+        <x:v>6264.2</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
-        <x:v>276.3</x:v>
+        <x:v>272.4</x:v>
       </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
@@ -649,25 +649,25 @@
         <x:v>IF主力</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>2026-07-23</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
       <x:c r="C9" s="10" t="n">
-        <x:v>4682.6</x:v>
+        <x:v>4619.4</x:v>
       </x:c>
       <x:c r="D9" s="10" t="n">
-        <x:v>4644</x:v>
+        <x:v>4532.2</x:v>
       </x:c>
       <x:c r="E9" s="12" t="n">
-        <x:v>38.6</x:v>
+        <x:v>87.2</x:v>
       </x:c>
       <x:c r="F9" s="9" t="n">
-        <x:v>17</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="G9" s="10" t="n">
-        <x:v>1713</x:v>
+        <x:v>2304.4</x:v>
       </x:c>
       <x:c r="H9" s="10" t="n">
-        <x:v>100.8</x:v>
+        <x:v>100.2</x:v>
       </x:c>
       <x:c r="I9" s="10" t="n">
         <x:v>90</x:v>
@@ -678,25 +678,25 @@
         <x:v>IH主力</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>2026-07-23</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:v>2969.6</x:v>
+        <x:v>2927</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
-        <x:v>2938.8</x:v>
+        <x:v>2886.4</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
-        <x:v>30.8</x:v>
+        <x:v>40.6</x:v>
       </x:c>
       <x:c r="F10" s="9" t="n">
-        <x:v>17</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="G10" s="10" t="n">
-        <x:v>956.4</x:v>
+        <x:v>1221.6</x:v>
       </x:c>
       <x:c r="H10" s="10" t="n">
-        <x:v>56.3</x:v>
+        <x:v>53.1</x:v>
       </x:c>
       <x:c r="I10" s="10" t="n">
         <x:v>60</x:v>
@@ -710,7 +710,7 @@
         <x:v>2026-07-01</x:v>
       </x:c>
       <x:c r="C13" s="14" t="str">
-        <x:v>2026-07-23</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
       <x:c r="D13" s="14" t="str">
         <x:v>数据源</x:v>
@@ -727,7 +727,7 @@
         <x:v>指数日线</x:v>
       </x:c>
       <x:c r="D14" s="7" t="str">
-        <x:v>https://money.finance.sina.com.cn/quotes_service/api/json_v2.php/CN_MarketData.getKLineData?symbol=sh000852&amp;scale=240&amp;ma=no&amp;datalen=80</x:v>
+        <x:v>https://web.ifzq.gtimg.cn/appstock/app/fqkline/get?param=sh000852,day,,,80,qfq</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -741,7 +741,7 @@
         <x:v>指数日线</x:v>
       </x:c>
       <x:c r="D15" s="7" t="str">
-        <x:v>https://money.finance.sina.com.cn/quotes_service/api/json_v2.php/CN_MarketData.getKLineData?symbol=sh000905&amp;scale=240&amp;ma=no&amp;datalen=80</x:v>
+        <x:v>https://web.ifzq.gtimg.cn/appstock/app/fqkline/get?param=sh000905,day,,,80,qfq</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -755,7 +755,7 @@
         <x:v>指数日线</x:v>
       </x:c>
       <x:c r="D16" s="7" t="str">
-        <x:v>https://money.finance.sina.com.cn/quotes_service/api/json_v2.php/CN_MarketData.getKLineData?symbol=sh000001&amp;scale=240&amp;ma=no&amp;datalen=80</x:v>
+        <x:v>https://web.ifzq.gtimg.cn/appstock/app/fqkline/get?param=sh000001,day,,,80,qfq</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -893,10 +893,10 @@
         <x:v>8827.47</x:v>
       </x:c>
       <x:c r="E4" s="22" t="n">
-        <x:v>8944.195</x:v>
+        <x:v>8944.19</x:v>
       </x:c>
       <x:c r="F4" s="22" t="n">
-        <x:v>8806.646</x:v>
+        <x:v>8806.65</x:v>
       </x:c>
       <x:c r="G4" s="22" t="n">
         <x:v>8876.63</x:v>
@@ -905,7 +905,7 @@
         <x:v>66.8</x:v>
       </x:c>
       <x:c r="I4" s="23" t="n">
-        <x:v>0.007587471477740637</x:v>
+        <x:v>0.007587013992387925</x:v>
       </x:c>
       <x:c r="J4" s="22" t="n">
         <x:f>ROUND(E4-F4,1)</x:f>
@@ -926,22 +926,22 @@
         <x:v>7月2日</x:v>
       </x:c>
       <x:c r="D5" s="22" t="n">
-        <x:v>8688.291</x:v>
+        <x:v>8688.29</x:v>
       </x:c>
       <x:c r="E5" s="22" t="n">
-        <x:v>8865.966</x:v>
+        <x:v>8865.97</x:v>
       </x:c>
       <x:c r="F5" s="22" t="n">
-        <x:v>8598.869</x:v>
+        <x:v>8598.87</x:v>
       </x:c>
       <x:c r="G5" s="22" t="n">
-        <x:v>8625.334</x:v>
+        <x:v>8625.33</x:v>
       </x:c>
       <x:c r="H5" s="25" t="n">
         <x:v>-251.3</x:v>
       </x:c>
       <x:c r="I5" s="23" t="n">
-        <x:v>-0.02830984281196791</x:v>
+        <x:v>-0.028310293433431277</x:v>
       </x:c>
       <x:c r="J5" s="27" t="n">
         <x:f>ROUND(E5-F5,1)</x:f>
@@ -962,22 +962,22 @@
         <x:v>7月3日</x:v>
       </x:c>
       <x:c r="D6" s="22" t="n">
-        <x:v>8627.382</x:v>
+        <x:v>8627.38</x:v>
       </x:c>
       <x:c r="E6" s="22" t="n">
-        <x:v>8740.668</x:v>
+        <x:v>8740.67</x:v>
       </x:c>
       <x:c r="F6" s="22" t="n">
-        <x:v>8559.285</x:v>
+        <x:v>8559.28</x:v>
       </x:c>
       <x:c r="G6" s="22" t="n">
-        <x:v>8620.789</x:v>
+        <x:v>8620.79</x:v>
       </x:c>
       <x:c r="H6" s="22" t="n">
         <x:v>-4.5</x:v>
       </x:c>
       <x:c r="I6" s="23" t="n">
-        <x:v>-0.0005269361163289243</x:v>
+        <x:v>-0.0005263566727300439</x:v>
       </x:c>
       <x:c r="J6" s="27" t="n">
         <x:f>ROUND(E6-F6,1)</x:f>
@@ -998,22 +998,22 @@
         <x:v>7月6日</x:v>
       </x:c>
       <x:c r="D7" s="22" t="n">
-        <x:v>8669.123</x:v>
+        <x:v>8669.12</x:v>
       </x:c>
       <x:c r="E7" s="22" t="n">
-        <x:v>8694.805</x:v>
+        <x:v>8694.8</x:v>
       </x:c>
       <x:c r="F7" s="22" t="n">
-        <x:v>8432.897</x:v>
+        <x:v>8432.9</x:v>
       </x:c>
       <x:c r="G7" s="22" t="n">
-        <x:v>8472.603</x:v>
+        <x:v>8472.6</x:v>
       </x:c>
       <x:c r="H7" s="22" t="n">
         <x:v>-148.2</x:v>
       </x:c>
       <x:c r="I7" s="23" t="n">
-        <x:v>-0.01718937790960917</x:v>
+        <x:v>-0.01718983991026346</x:v>
       </x:c>
       <x:c r="J7" s="27" t="n">
         <x:f>ROUND(E7-F7,1)</x:f>
@@ -1034,22 +1034,22 @@
         <x:v>7月7日</x:v>
       </x:c>
       <x:c r="D8" s="22" t="n">
-        <x:v>8436.389</x:v>
+        <x:v>8436.39</x:v>
       </x:c>
       <x:c r="E8" s="22" t="n">
-        <x:v>8489.476</x:v>
+        <x:v>8489.48</x:v>
       </x:c>
       <x:c r="F8" s="22" t="n">
-        <x:v>8261.398</x:v>
+        <x:v>8261.4</x:v>
       </x:c>
       <x:c r="G8" s="22" t="n">
-        <x:v>8301.804</x:v>
+        <x:v>8301.8</x:v>
       </x:c>
       <x:c r="H8" s="25" t="n">
         <x:v>-170.8</x:v>
       </x:c>
       <x:c r="I8" s="23" t="n">
-        <x:v>-0.02015897593691085</x:v>
+        <x:v>-0.020159101102377175</x:v>
       </x:c>
       <x:c r="J8" s="27" t="n">
         <x:f>ROUND(E8-F8,1)</x:f>
@@ -1070,22 +1070,22 @@
         <x:v>7月8日</x:v>
       </x:c>
       <x:c r="D9" s="22" t="n">
-        <x:v>8315.962</x:v>
+        <x:v>8315.96</x:v>
       </x:c>
       <x:c r="E9" s="22" t="n">
-        <x:v>8328.965</x:v>
+        <x:v>8328.96</x:v>
       </x:c>
       <x:c r="F9" s="22" t="n">
-        <x:v>8117.861</x:v>
+        <x:v>8117.86</x:v>
       </x:c>
       <x:c r="G9" s="22" t="n">
-        <x:v>8117.861</x:v>
+        <x:v>8117.86</x:v>
       </x:c>
       <x:c r="H9" s="25" t="n">
         <x:v>-183.9</x:v>
       </x:c>
       <x:c r="I9" s="23" t="n">
-        <x:v>-0.02215699142017813</x:v>
+        <x:v>-0.02215664072851664</x:v>
       </x:c>
       <x:c r="J9" s="27" t="n">
         <x:f>ROUND(E9-F9,1)</x:f>
@@ -1106,22 +1106,22 @@
         <x:v>7月9日</x:v>
       </x:c>
       <x:c r="D10" s="22" t="n">
-        <x:v>8161.859</x:v>
+        <x:v>8161.86</x:v>
       </x:c>
       <x:c r="E10" s="22" t="n">
-        <x:v>8312.621</x:v>
+        <x:v>8312.62</x:v>
       </x:c>
       <x:c r="F10" s="22" t="n">
-        <x:v>7978.806</x:v>
+        <x:v>7978.81</x:v>
       </x:c>
       <x:c r="G10" s="22" t="n">
-        <x:v>8300.077</x:v>
+        <x:v>8300.08</x:v>
       </x:c>
       <x:c r="H10" s="25" t="n">
         <x:v>182.2</x:v>
       </x:c>
       <x:c r="I10" s="23" t="n">
-        <x:v>0.0224463069766776</x:v>
+        <x:v>0.022446802482427586</x:v>
       </x:c>
       <x:c r="J10" s="27" t="n">
         <x:f>ROUND(E10-F10,1)</x:f>
@@ -1142,22 +1142,22 @@
         <x:v>7月10日</x:v>
       </x:c>
       <x:c r="D11" s="22" t="n">
-        <x:v>8312.492</x:v>
+        <x:v>8312.49</x:v>
       </x:c>
       <x:c r="E11" s="22" t="n">
-        <x:v>8438.194</x:v>
+        <x:v>8438.19</x:v>
       </x:c>
       <x:c r="F11" s="22" t="n">
-        <x:v>8198.308</x:v>
+        <x:v>8198.31</x:v>
       </x:c>
       <x:c r="G11" s="22" t="n">
-        <x:v>8198.308</x:v>
+        <x:v>8198.31</x:v>
       </x:c>
       <x:c r="H11" s="22" t="n">
         <x:v>-101.8</x:v>
       </x:c>
       <x:c r="I11" s="23" t="n">
-        <x:v>-0.012261211552615503</x:v>
+        <x:v>-0.012261327601661764</x:v>
       </x:c>
       <x:c r="J11" s="27" t="n">
         <x:f>ROUND(E11-F11,1)</x:f>
@@ -1178,22 +1178,22 @@
         <x:v>7月13日</x:v>
       </x:c>
       <x:c r="D12" s="22" t="n">
-        <x:v>8124.363</x:v>
+        <x:v>8124.36</x:v>
       </x:c>
       <x:c r="E12" s="22" t="n">
-        <x:v>8171.504</x:v>
+        <x:v>8171.5</x:v>
       </x:c>
       <x:c r="F12" s="22" t="n">
-        <x:v>7769.292</x:v>
+        <x:v>7769.29</x:v>
       </x:c>
       <x:c r="G12" s="22" t="n">
-        <x:v>7787.853</x:v>
+        <x:v>7787.85</x:v>
       </x:c>
       <x:c r="H12" s="25" t="n">
         <x:v>-410.5</x:v>
       </x:c>
       <x:c r="I12" s="23" t="n">
-        <x:v>-0.050065818459126055</x:v>
+        <x:v>-0.050066416127226065</x:v>
       </x:c>
       <x:c r="J12" s="27" t="n">
         <x:f>ROUND(E12-F12,1)</x:f>
@@ -1214,22 +1214,22 @@
         <x:v>7月14日</x:v>
       </x:c>
       <x:c r="D13" s="22" t="n">
-        <x:v>7799.813</x:v>
+        <x:v>7799.81</x:v>
       </x:c>
       <x:c r="E13" s="22" t="n">
-        <x:v>7934.103</x:v>
+        <x:v>7934.1</x:v>
       </x:c>
       <x:c r="F13" s="22" t="n">
-        <x:v>7657.671</x:v>
+        <x:v>7657.67</x:v>
       </x:c>
       <x:c r="G13" s="22" t="n">
-        <x:v>7925.123</x:v>
+        <x:v>7925.12</x:v>
       </x:c>
       <x:c r="H13" s="22" t="n">
         <x:v>137.3</x:v>
       </x:c>
       <x:c r="I13" s="23" t="n">
-        <x:v>0.017626167314662933</x:v>
+        <x:v>0.017626174104534487</x:v>
       </x:c>
       <x:c r="J13" s="27" t="n">
         <x:f>ROUND(E13-F13,1)</x:f>
@@ -1250,22 +1250,22 @@
         <x:v>7月15日</x:v>
       </x:c>
       <x:c r="D14" s="22" t="n">
-        <x:v>7959.374</x:v>
+        <x:v>7959.37</x:v>
       </x:c>
       <x:c r="E14" s="22" t="n">
-        <x:v>7979.077</x:v>
+        <x:v>7979.08</x:v>
       </x:c>
       <x:c r="F14" s="22" t="n">
-        <x:v>7783.219</x:v>
+        <x:v>7783.22</x:v>
       </x:c>
       <x:c r="G14" s="22" t="n">
-        <x:v>7817.831</x:v>
+        <x:v>7817.83</x:v>
       </x:c>
       <x:c r="H14" s="22" t="n">
         <x:v>-107.3</x:v>
       </x:c>
       <x:c r="I14" s="23" t="n">
-        <x:v>-0.01353821259304111</x:v>
+        <x:v>-0.013537965355729598</x:v>
       </x:c>
       <x:c r="J14" s="27" t="n">
         <x:f>ROUND(E14-F14,1)</x:f>
@@ -1286,22 +1286,22 @@
         <x:v>7月16日</x:v>
       </x:c>
       <x:c r="D15" s="22" t="n">
-        <x:v>7713.135</x:v>
+        <x:v>7713.14</x:v>
       </x:c>
       <x:c r="E15" s="22" t="n">
         <x:v>7836.39</x:v>
       </x:c>
       <x:c r="F15" s="22" t="n">
-        <x:v>7591.421</x:v>
+        <x:v>7591.42</x:v>
       </x:c>
       <x:c r="G15" s="22" t="n">
-        <x:v>7631.762</x:v>
+        <x:v>7631.76</x:v>
       </x:c>
       <x:c r="H15" s="25" t="n">
         <x:v>-186.1</x:v>
       </x:c>
       <x:c r="I15" s="23" t="n">
-        <x:v>-0.02380059123815803</x:v>
+        <x:v>-0.023800722195289503</x:v>
       </x:c>
       <x:c r="J15" s="27" t="n">
         <x:f>ROUND(E15-F15,1)</x:f>
@@ -1322,22 +1322,22 @@
         <x:v>7月17日</x:v>
       </x:c>
       <x:c r="D16" s="32" t="n">
-        <x:v>7599.388</x:v>
+        <x:v>7599.39</x:v>
       </x:c>
       <x:c r="E16" s="32" t="n">
-        <x:v>7605.613</x:v>
+        <x:v>7605.61</x:v>
       </x:c>
       <x:c r="F16" s="32" t="n">
-        <x:v>7163.309</x:v>
+        <x:v>7163.31</x:v>
       </x:c>
       <x:c r="G16" s="32" t="n">
-        <x:v>7167.996</x:v>
+        <x:v>7168</x:v>
       </x:c>
       <x:c r="H16" s="25" t="n">
         <x:v>-463.8</x:v>
       </x:c>
       <x:c r="I16" s="33" t="n">
-        <x:v>-0.06076788034008396</x:v>
+        <x:v>-0.06076711007683677</x:v>
       </x:c>
       <x:c r="J16" s="27" t="n">
         <x:f>ROUND(E16-F16,1)</x:f>
@@ -1358,22 +1358,22 @@
         <x:v>7月20日</x:v>
       </x:c>
       <x:c r="D17" s="22" t="n">
-        <x:v>7256.267</x:v>
+        <x:v>7256.27</x:v>
       </x:c>
       <x:c r="E17" s="22" t="n">
-        <x:v>7298.122</x:v>
+        <x:v>7298.12</x:v>
       </x:c>
       <x:c r="F17" s="22" t="n">
-        <x:v>6824.145</x:v>
+        <x:v>6824.14</x:v>
       </x:c>
       <x:c r="G17" s="22" t="n">
-        <x:v>6965.376</x:v>
+        <x:v>6965.38</x:v>
       </x:c>
       <x:c r="H17" s="25" t="n">
         <x:v>-202.6</x:v>
       </x:c>
       <x:c r="I17" s="23" t="n">
-        <x:v>-0.028267314881314065</x:v>
+        <x:v>-0.028267299107142874</x:v>
       </x:c>
       <x:c r="J17" s="27" t="n">
         <x:f>ROUND(E17-F17,1)</x:f>
@@ -1394,22 +1394,22 @@
         <x:v>7月21日</x:v>
       </x:c>
       <x:c r="D18" s="22" t="n">
-        <x:v>6975.893</x:v>
+        <x:v>6975.89</x:v>
       </x:c>
       <x:c r="E18" s="22" t="n">
-        <x:v>7264.338</x:v>
+        <x:v>7264.34</x:v>
       </x:c>
       <x:c r="F18" s="22" t="n">
-        <x:v>6714.187</x:v>
+        <x:v>6714.19</x:v>
       </x:c>
       <x:c r="G18" s="22" t="n">
-        <x:v>7259.863</x:v>
+        <x:v>7259.86</x:v>
       </x:c>
       <x:c r="H18" s="25" t="n">
         <x:v>294.5</x:v>
       </x:c>
       <x:c r="I18" s="23" t="n">
-        <x:v>0.042278693928367916</x:v>
+        <x:v>0.042277664678739724</x:v>
       </x:c>
       <x:c r="J18" s="27" t="n">
         <x:f>ROUND(E18-F18,1)</x:f>
@@ -1430,22 +1430,22 @@
         <x:v>7月22日</x:v>
       </x:c>
       <x:c r="D19" s="22" t="n">
-        <x:v>7196.863</x:v>
+        <x:v>7196.86</x:v>
       </x:c>
       <x:c r="E19" s="22" t="n">
-        <x:v>7302.454</x:v>
+        <x:v>7302.45</x:v>
       </x:c>
       <x:c r="F19" s="22" t="n">
         <x:v>7118.66</x:v>
       </x:c>
       <x:c r="G19" s="22" t="n">
-        <x:v>7158.762</x:v>
+        <x:v>7158.76</x:v>
       </x:c>
       <x:c r="H19" s="22" t="n">
         <x:v>-101.1</x:v>
       </x:c>
       <x:c r="I19" s="23" t="n">
-        <x:v>-0.01392602036705104</x:v>
+        <x:v>-0.013925888378012674</x:v>
       </x:c>
       <x:c r="J19" s="27" t="n">
         <x:f>ROUND(E19-F19,1)</x:f>
@@ -1466,13 +1466,13 @@
         <x:v>7月23日</x:v>
       </x:c>
       <x:c r="D20" s="22" t="n">
-        <x:v>7169.543</x:v>
+        <x:v>7169.54</x:v>
       </x:c>
       <x:c r="E20" s="22" t="n">
-        <x:v>7247.141</x:v>
+        <x:v>7247.14</x:v>
       </x:c>
       <x:c r="F20" s="22" t="n">
-        <x:v>7113.498</x:v>
+        <x:v>7113.5</x:v>
       </x:c>
       <x:c r="G20" s="22" t="n">
         <x:v>7195.5</x:v>
@@ -1481,7 +1481,7 @@
         <x:v>36.7</x:v>
       </x:c>
       <x:c r="I20" s="23" t="n">
-        <x:v>0.0051318929166803695</x:v>
+        <x:v>0.005132173728411127</x:v>
       </x:c>
       <x:c r="J20" s="22" t="n">
         <x:f>ROUND(E20-F20,1)</x:f>
@@ -1491,43 +1491,259 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="21" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B21" s="21" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C21" s="21" t="str">
+        <x:v>7月24日</x:v>
+      </x:c>
+      <x:c r="D21" s="22" t="n">
+        <x:v>7109.25</x:v>
+      </x:c>
+      <x:c r="E21" s="22" t="n">
+        <x:v>7174.55</x:v>
+      </x:c>
+      <x:c r="F21" s="22" t="n">
+        <x:v>6995.69</x:v>
+      </x:c>
+      <x:c r="G21" s="22" t="n">
+        <x:v>6995.69</x:v>
+      </x:c>
+      <x:c r="H21" s="25" t="n">
+        <x:v>-199.8</x:v>
+      </x:c>
+      <x:c r="I21" s="23" t="n">
+        <x:v>-0.027768744354110253</x:v>
+      </x:c>
+      <x:c r="J21" s="22" t="n">
+        <x:f>ROUND(E21-F21,1)</x:f>
+        <x:v>178.9</x:v>
+      </x:c>
+      <x:c r="K21" s="21" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="21" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B22" s="21" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C22" s="21" t="str">
+        <x:v>7月27日</x:v>
+      </x:c>
+      <x:c r="D22" s="22" t="n">
+        <x:v>6981.16</x:v>
+      </x:c>
+      <x:c r="E22" s="22" t="n">
+        <x:v>7228.78</x:v>
+      </x:c>
+      <x:c r="F22" s="22" t="n">
+        <x:v>6972.28</x:v>
+      </x:c>
+      <x:c r="G22" s="22" t="n">
+        <x:v>7228.78</x:v>
+      </x:c>
+      <x:c r="H22" s="25" t="n">
+        <x:v>233.1</x:v>
+      </x:c>
+      <x:c r="I22" s="23" t="n">
+        <x:v>0.03331908646609549</x:v>
+      </x:c>
+      <x:c r="J22" s="27" t="n">
+        <x:f>ROUND(E22-F22,1)</x:f>
+        <x:v>256.5</x:v>
+      </x:c>
+      <x:c r="K22" s="21" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
+    </x:row>
     <x:row r="23">
-      <x:c r="A23" s="38" t="str">
+      <x:c r="A23" s="21" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B23" s="21" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C23" s="21" t="str">
+        <x:v>7月28日</x:v>
+      </x:c>
+      <x:c r="D23" s="22" t="n">
+        <x:v>7135.73</x:v>
+      </x:c>
+      <x:c r="E23" s="22" t="n">
+        <x:v>7189.18</x:v>
+      </x:c>
+      <x:c r="F23" s="22" t="n">
+        <x:v>6992.94</x:v>
+      </x:c>
+      <x:c r="G23" s="22" t="n">
+        <x:v>7026.28</x:v>
+      </x:c>
+      <x:c r="H23" s="25" t="n">
+        <x:v>-202.5</x:v>
+      </x:c>
+      <x:c r="I23" s="23" t="n">
+        <x:v>-0.028013025711115858</x:v>
+      </x:c>
+      <x:c r="J23" s="27" t="n">
+        <x:f>ROUND(E23-F23,1)</x:f>
+        <x:v>196.2</x:v>
+      </x:c>
+      <x:c r="K23" s="21" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="21" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B24" s="21" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C24" s="21" t="str">
+        <x:v>7月29日</x:v>
+      </x:c>
+      <x:c r="D24" s="22" t="n">
+        <x:v>7020.22</x:v>
+      </x:c>
+      <x:c r="E24" s="22" t="n">
+        <x:v>7132.35</x:v>
+      </x:c>
+      <x:c r="F24" s="22" t="n">
+        <x:v>6897.39</x:v>
+      </x:c>
+      <x:c r="G24" s="22" t="n">
+        <x:v>7095.19</x:v>
+      </x:c>
+      <x:c r="H24" s="22" t="n">
+        <x:v>68.9</x:v>
+      </x:c>
+      <x:c r="I24" s="23" t="n">
+        <x:v>0.009807465685967465</x:v>
+      </x:c>
+      <x:c r="J24" s="27" t="n">
+        <x:f>ROUND(E24-F24,1)</x:f>
+        <x:v>235</x:v>
+      </x:c>
+      <x:c r="K24" s="21" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="21" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B25" s="21" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C25" s="21" t="str">
+        <x:v>7月30日</x:v>
+      </x:c>
+      <x:c r="D25" s="22" t="n">
+        <x:v>7053.09</x:v>
+      </x:c>
+      <x:c r="E25" s="22" t="n">
+        <x:v>7121.52</x:v>
+      </x:c>
+      <x:c r="F25" s="22" t="n">
+        <x:v>6841.75</x:v>
+      </x:c>
+      <x:c r="G25" s="22" t="n">
+        <x:v>6900.66</x:v>
+      </x:c>
+      <x:c r="H25" s="25" t="n">
+        <x:v>-194.5</x:v>
+      </x:c>
+      <x:c r="I25" s="23" t="n">
+        <x:v>-0.027417165713673586</x:v>
+      </x:c>
+      <x:c r="J25" s="27" t="n">
+        <x:f>ROUND(E25-F25,1)</x:f>
+        <x:v>279.8</x:v>
+      </x:c>
+      <x:c r="K25" s="21" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="21" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B26" s="21" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C26" s="21" t="str">
+        <x:v>7月31日</x:v>
+      </x:c>
+      <x:c r="D26" s="22" t="n">
+        <x:v>7082.75</x:v>
+      </x:c>
+      <x:c r="E26" s="22" t="n">
+        <x:v>7218.06</x:v>
+      </x:c>
+      <x:c r="F26" s="22" t="n">
+        <x:v>7071.05</x:v>
+      </x:c>
+      <x:c r="G26" s="22" t="n">
+        <x:v>7075.51</x:v>
+      </x:c>
+      <x:c r="H26" s="25" t="n">
+        <x:v>174.9</x:v>
+      </x:c>
+      <x:c r="I26" s="23" t="n">
+        <x:v>0.02533815606043488</x:v>
+      </x:c>
+      <x:c r="J26" s="22" t="n">
+        <x:f>ROUND(E26-F26,1)</x:f>
+        <x:v>147</x:v>
+      </x:c>
+      <x:c r="K26" s="21" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="38" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B23" s="39" t="n">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="C23" s="39"/>
-      <x:c r="D23" s="39"/>
-      <x:c r="E23" s="39"/>
-      <x:c r="F23" s="39"/>
-      <x:c r="G23" s="39"/>
-      <x:c r="H23" s="39"/>
-      <x:c r="I23" s="39"/>
-      <x:c r="J23" s="40" t="n">
-        <x:f>SUM(J4:J20)</x:f>
-        <x:v>4764.200000000001</x:v>
-      </x:c>
-      <x:c r="K23" s="39"/>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="38" t="str">
+      <x:c r="B29" s="39" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="C29" s="39"/>
+      <x:c r="D29" s="39"/>
+      <x:c r="E29" s="39"/>
+      <x:c r="F29" s="39"/>
+      <x:c r="G29" s="39"/>
+      <x:c r="H29" s="39"/>
+      <x:c r="I29" s="39"/>
+      <x:c r="J29" s="40" t="n">
+        <x:f>SUM(J4:J26)</x:f>
+        <x:v>6057.6</x:v>
+      </x:c>
+      <x:c r="K29" s="39"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="38" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B24" s="39"/>
-      <x:c r="C24" s="39"/>
-      <x:c r="D24" s="39"/>
-      <x:c r="E24" s="39"/>
-      <x:c r="F24" s="39"/>
-      <x:c r="G24" s="39"/>
-      <x:c r="H24" s="39"/>
-      <x:c r="I24" s="39"/>
-      <x:c r="J24" s="42" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
-        <x:v>280.2</x:v>
-      </x:c>
-      <x:c r="K24" s="39"/>
+      <x:c r="B30" s="39"/>
+      <x:c r="C30" s="39"/>
+      <x:c r="D30" s="39"/>
+      <x:c r="E30" s="39"/>
+      <x:c r="F30" s="39"/>
+      <x:c r="G30" s="39"/>
+      <x:c r="H30" s="39"/>
+      <x:c r="I30" s="39"/>
+      <x:c r="J30" s="42" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J26),0),1)</x:f>
+        <x:v>263.4</x:v>
+      </x:c>
+      <x:c r="K30" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1605,22 +1821,22 @@
         <x:v>7月1日</x:v>
       </x:c>
       <x:c r="D4" s="22" t="n">
-        <x:v>9052.043</x:v>
+        <x:v>9052.04</x:v>
       </x:c>
       <x:c r="E4" s="22" t="n">
-        <x:v>9147.559</x:v>
+        <x:v>9147.56</x:v>
       </x:c>
       <x:c r="F4" s="22" t="n">
-        <x:v>8956.185</x:v>
+        <x:v>8956.18</x:v>
       </x:c>
       <x:c r="G4" s="22" t="n">
-        <x:v>9028.933</x:v>
+        <x:v>9028.93</x:v>
       </x:c>
       <x:c r="H4" s="22" t="n">
         <x:v>-2.4</x:v>
       </x:c>
       <x:c r="I4" s="23" t="n">
-        <x:v>-0.0002708335017277408</x:v>
+        <x:v>-0.000271276371938578</x:v>
       </x:c>
       <x:c r="J4" s="27" t="n">
         <x:f>ROUND(E4-F4,1)</x:f>
@@ -1641,22 +1857,22 @@
         <x:v>7月2日</x:v>
       </x:c>
       <x:c r="D5" s="22" t="n">
-        <x:v>8829.621</x:v>
+        <x:v>8829.62</x:v>
       </x:c>
       <x:c r="E5" s="22" t="n">
-        <x:v>8932.647</x:v>
+        <x:v>8932.65</x:v>
       </x:c>
       <x:c r="F5" s="22" t="n">
-        <x:v>8667.419</x:v>
+        <x:v>8667.42</x:v>
       </x:c>
       <x:c r="G5" s="22" t="n">
-        <x:v>8694.176</x:v>
+        <x:v>8694.18</x:v>
       </x:c>
       <x:c r="H5" s="25" t="n">
-        <x:v>-334.8</x:v>
+        <x:v>-334.7</x:v>
       </x:c>
       <x:c r="I5" s="23" t="n">
-        <x:v>-0.03707603102160595</x:v>
+        <x:v>-0.037075268055018706</x:v>
       </x:c>
       <x:c r="J5" s="27" t="n">
         <x:f>ROUND(E5-F5,1)</x:f>
@@ -1677,22 +1893,22 @@
         <x:v>7月3日</x:v>
       </x:c>
       <x:c r="D6" s="22" t="n">
-        <x:v>8702.327</x:v>
+        <x:v>8702.33</x:v>
       </x:c>
       <x:c r="E6" s="22" t="n">
-        <x:v>8860.416</x:v>
+        <x:v>8860.42</x:v>
       </x:c>
       <x:c r="F6" s="22" t="n">
         <x:v>8636.15</x:v>
       </x:c>
       <x:c r="G6" s="22" t="n">
-        <x:v>8745.261</x:v>
+        <x:v>8745.26</x:v>
       </x:c>
       <x:c r="H6" s="22" t="n">
         <x:v>51.1</x:v>
       </x:c>
       <x:c r="I6" s="23" t="n">
-        <x:v>0.00587577247113491</x:v>
+        <x:v>0.005875194670457606</x:v>
       </x:c>
       <x:c r="J6" s="27" t="n">
         <x:f>ROUND(E6-F6,1)</x:f>
@@ -1713,22 +1929,22 @@
         <x:v>7月6日</x:v>
       </x:c>
       <x:c r="D7" s="22" t="n">
-        <x:v>8790.967</x:v>
+        <x:v>8790.97</x:v>
       </x:c>
       <x:c r="E7" s="22" t="n">
         <x:v>8823.05</x:v>
       </x:c>
       <x:c r="F7" s="22" t="n">
-        <x:v>8570.892</x:v>
+        <x:v>8570.89</x:v>
       </x:c>
       <x:c r="G7" s="22" t="n">
-        <x:v>8651.134</x:v>
+        <x:v>8651.13</x:v>
       </x:c>
       <x:c r="H7" s="22" t="n">
         <x:v>-94.1</x:v>
       </x:c>
       <x:c r="I7" s="23" t="n">
-        <x:v>-0.01076320077811288</x:v>
+        <x:v>-0.010763545051833856</x:v>
       </x:c>
       <x:c r="J7" s="27" t="n">
         <x:f>ROUND(E7-F7,1)</x:f>
@@ -1749,22 +1965,22 @@
         <x:v>7月7日</x:v>
       </x:c>
       <x:c r="D8" s="22" t="n">
-        <x:v>8604.076</x:v>
+        <x:v>8604.08</x:v>
       </x:c>
       <x:c r="E8" s="22" t="n">
-        <x:v>8663.665</x:v>
+        <x:v>8663.67</x:v>
       </x:c>
       <x:c r="F8" s="22" t="n">
-        <x:v>8457.576</x:v>
+        <x:v>8457.58</x:v>
       </x:c>
       <x:c r="G8" s="22" t="n">
-        <x:v>8508.789</x:v>
+        <x:v>8508.79</x:v>
       </x:c>
       <x:c r="H8" s="22" t="n">
         <x:v>-142.3</x:v>
       </x:c>
       <x:c r="I8" s="23" t="n">
-        <x:v>-0.01645391228479398</x:v>
+        <x:v>-0.016453341933365784</x:v>
       </x:c>
       <x:c r="J8" s="27" t="n">
         <x:f>ROUND(E8-F8,1)</x:f>
@@ -1785,22 +2001,22 @@
         <x:v>7月8日</x:v>
       </x:c>
       <x:c r="D9" s="22" t="n">
-        <x:v>8539.016</x:v>
+        <x:v>8539.02</x:v>
       </x:c>
       <x:c r="E9" s="22" t="n">
-        <x:v>8571.525</x:v>
+        <x:v>8571.52</x:v>
       </x:c>
       <x:c r="F9" s="22" t="n">
-        <x:v>8343.923</x:v>
+        <x:v>8343.92</x:v>
       </x:c>
       <x:c r="G9" s="22" t="n">
-        <x:v>8390.019</x:v>
+        <x:v>8390.02</x:v>
       </x:c>
       <x:c r="H9" s="22" t="n">
         <x:v>-118.8</x:v>
       </x:c>
       <x:c r="I9" s="23" t="n">
-        <x:v>-0.013958508079116805</x:v>
+        <x:v>-0.013958506438635832</x:v>
       </x:c>
       <x:c r="J9" s="27" t="n">
         <x:f>ROUND(E9-F9,1)</x:f>
@@ -1821,22 +2037,22 @@
         <x:v>7月9日</x:v>
       </x:c>
       <x:c r="D10" s="22" t="n">
-        <x:v>8437.147</x:v>
+        <x:v>8437.15</x:v>
       </x:c>
       <x:c r="E10" s="22" t="n">
         <x:v>8659.65</x:v>
       </x:c>
       <x:c r="F10" s="22" t="n">
-        <x:v>8281.953</x:v>
+        <x:v>8281.95</x:v>
       </x:c>
       <x:c r="G10" s="22" t="n">
-        <x:v>8652.787</x:v>
+        <x:v>8652.79</x:v>
       </x:c>
       <x:c r="H10" s="25" t="n">
         <x:v>262.8</x:v>
       </x:c>
       <x:c r="I10" s="23" t="n">
-        <x:v>0.03131911858602465</x:v>
+        <x:v>0.03131935323157764</x:v>
       </x:c>
       <x:c r="J10" s="27" t="n">
         <x:f>ROUND(E10-F10,1)</x:f>
@@ -1857,22 +2073,22 @@
         <x:v>7月10日</x:v>
       </x:c>
       <x:c r="D11" s="22" t="n">
-        <x:v>8672.363</x:v>
+        <x:v>8672.36</x:v>
       </x:c>
       <x:c r="E11" s="22" t="n">
-        <x:v>8783.249</x:v>
+        <x:v>8783.25</x:v>
       </x:c>
       <x:c r="F11" s="22" t="n">
-        <x:v>8503.245</x:v>
+        <x:v>8503.24</x:v>
       </x:c>
       <x:c r="G11" s="22" t="n">
-        <x:v>8503.971</x:v>
+        <x:v>8503.97</x:v>
       </x:c>
       <x:c r="H11" s="22" t="n">
         <x:v>-148.8</x:v>
       </x:c>
       <x:c r="I11" s="23" t="n">
-        <x:v>-0.01719862051382992</x:v>
+        <x:v>-0.01719907682955457</x:v>
       </x:c>
       <x:c r="J11" s="27" t="n">
         <x:f>ROUND(E11-F11,1)</x:f>
@@ -1893,22 +2109,22 @@
         <x:v>7月13日</x:v>
       </x:c>
       <x:c r="D12" s="22" t="n">
-        <x:v>8409.143</x:v>
+        <x:v>8409.14</x:v>
       </x:c>
       <x:c r="E12" s="22" t="n">
-        <x:v>8457.692</x:v>
+        <x:v>8457.69</x:v>
       </x:c>
       <x:c r="F12" s="22" t="n">
-        <x:v>8106.269</x:v>
+        <x:v>8106.27</x:v>
       </x:c>
       <x:c r="G12" s="22" t="n">
-        <x:v>8138.144</x:v>
+        <x:v>8138.14</x:v>
       </x:c>
       <x:c r="H12" s="25" t="n">
         <x:v>-365.8</x:v>
       </x:c>
       <x:c r="I12" s="23" t="n">
-        <x:v>-0.04301837341637216</x:v>
+        <x:v>-0.04301873125140365</x:v>
       </x:c>
       <x:c r="J12" s="27" t="n">
         <x:f>ROUND(E12-F12,1)</x:f>
@@ -1929,26 +2145,26 @@
         <x:v>7月14日</x:v>
       </x:c>
       <x:c r="D13" s="22" t="n">
-        <x:v>8135.046</x:v>
+        <x:v>8135.05</x:v>
       </x:c>
       <x:c r="E13" s="22" t="n">
         <x:v>8275.96</x:v>
       </x:c>
       <x:c r="F13" s="22" t="n">
-        <x:v>7955.308</x:v>
+        <x:v>7955.31</x:v>
       </x:c>
       <x:c r="G13" s="22" t="n">
-        <x:v>8275.939</x:v>
+        <x:v>8275.94</x:v>
       </x:c>
       <x:c r="H13" s="22" t="n">
         <x:v>137.8</x:v>
       </x:c>
       <x:c r="I13" s="23" t="n">
-        <x:v>0.016931993339021734</x:v>
+        <x:v>0.016932616052316662</x:v>
       </x:c>
       <x:c r="J13" s="27" t="n">
         <x:f>ROUND(E13-F13,1)</x:f>
-        <x:v>320.7</x:v>
+        <x:v>320.6</x:v>
       </x:c>
       <x:c r="K13" s="21" t="str">
         <x:v>中证500</x:v>
@@ -1965,22 +2181,22 @@
         <x:v>7月15日</x:v>
       </x:c>
       <x:c r="D14" s="22" t="n">
-        <x:v>8294.142</x:v>
+        <x:v>8294.14</x:v>
       </x:c>
       <x:c r="E14" s="22" t="n">
-        <x:v>8305.272</x:v>
+        <x:v>8305.27</x:v>
       </x:c>
       <x:c r="F14" s="22" t="n">
-        <x:v>8117.459</x:v>
+        <x:v>8117.46</x:v>
       </x:c>
       <x:c r="G14" s="22" t="n">
-        <x:v>8147.579</x:v>
+        <x:v>8147.58</x:v>
       </x:c>
       <x:c r="H14" s="22" t="n">
         <x:v>-128.4</x:v>
       </x:c>
       <x:c r="I14" s="23" t="n">
-        <x:v>-0.015510022488082642</x:v>
+        <x:v>-0.015510020613972664</x:v>
       </x:c>
       <x:c r="J14" s="27" t="n">
         <x:f>ROUND(E14-F14,1)</x:f>
@@ -2001,22 +2217,22 @@
         <x:v>7月16日</x:v>
       </x:c>
       <x:c r="D15" s="22" t="n">
-        <x:v>8006.449</x:v>
+        <x:v>8006.45</x:v>
       </x:c>
       <x:c r="E15" s="22" t="n">
-        <x:v>8148.042</x:v>
+        <x:v>8148.04</x:v>
       </x:c>
       <x:c r="F15" s="22" t="n">
-        <x:v>7907.097</x:v>
+        <x:v>7907.1</x:v>
       </x:c>
       <x:c r="G15" s="22" t="n">
-        <x:v>7955.664</x:v>
+        <x:v>7955.66</x:v>
       </x:c>
       <x:c r="H15" s="25" t="n">
         <x:v>-191.9</x:v>
       </x:c>
       <x:c r="I15" s="23" t="n">
-        <x:v>-0.02355484985171663</x:v>
+        <x:v>-0.02355546063984648</x:v>
       </x:c>
       <x:c r="J15" s="27" t="n">
         <x:f>ROUND(E15-F15,1)</x:f>
@@ -2037,22 +2253,22 @@
         <x:v>7月17日</x:v>
       </x:c>
       <x:c r="D16" s="32" t="n">
-        <x:v>7900.097</x:v>
+        <x:v>7900.1</x:v>
       </x:c>
       <x:c r="E16" s="32" t="n">
-        <x:v>7908.739</x:v>
+        <x:v>7908.74</x:v>
       </x:c>
       <x:c r="F16" s="32" t="n">
-        <x:v>7474.151</x:v>
+        <x:v>7474.15</x:v>
       </x:c>
       <x:c r="G16" s="32" t="n">
-        <x:v>7513.763</x:v>
+        <x:v>7513.76</x:v>
       </x:c>
       <x:c r="H16" s="25" t="n">
         <x:v>-441.9</x:v>
       </x:c>
       <x:c r="I16" s="33" t="n">
-        <x:v>-0.05554545792783605</x:v>
+        <x:v>-0.05554536015867939</x:v>
       </x:c>
       <x:c r="J16" s="27" t="n">
         <x:f>ROUND(E16-F16,1)</x:f>
@@ -2073,22 +2289,22 @@
         <x:v>7月20日</x:v>
       </x:c>
       <x:c r="D17" s="22" t="n">
-        <x:v>7597.769</x:v>
+        <x:v>7597.77</x:v>
       </x:c>
       <x:c r="E17" s="22" t="n">
-        <x:v>7626.489</x:v>
+        <x:v>7626.49</x:v>
       </x:c>
       <x:c r="F17" s="22" t="n">
-        <x:v>7253.518</x:v>
+        <x:v>7253.52</x:v>
       </x:c>
       <x:c r="G17" s="22" t="n">
-        <x:v>7411.313</x:v>
+        <x:v>7411.31</x:v>
       </x:c>
       <x:c r="H17" s="22" t="n">
         <x:v>-102.4</x:v>
       </x:c>
       <x:c r="I17" s="23" t="n">
-        <x:v>-0.013634978904711215</x:v>
+        <x:v>-0.013634984348714907</x:v>
       </x:c>
       <x:c r="J17" s="27" t="n">
         <x:f>ROUND(E17-F17,1)</x:f>
@@ -2109,22 +2325,22 @@
         <x:v>7月21日</x:v>
       </x:c>
       <x:c r="D18" s="22" t="n">
-        <x:v>7437.452</x:v>
+        <x:v>7437.45</x:v>
       </x:c>
       <x:c r="E18" s="22" t="n">
-        <x:v>7802.755</x:v>
+        <x:v>7802.75</x:v>
       </x:c>
       <x:c r="F18" s="22" t="n">
-        <x:v>7270.954</x:v>
+        <x:v>7270.95</x:v>
       </x:c>
       <x:c r="G18" s="22" t="n">
-        <x:v>7800.609</x:v>
+        <x:v>7800.61</x:v>
       </x:c>
       <x:c r="H18" s="25" t="n">
         <x:v>389.3</x:v>
       </x:c>
       <x:c r="I18" s="23" t="n">
-        <x:v>0.052527264737031176</x:v>
+        <x:v>0.0525278257150219</x:v>
       </x:c>
       <x:c r="J18" s="27" t="n">
         <x:f>ROUND(E18-F18,1)</x:f>
@@ -2145,22 +2361,22 @@
         <x:v>7月22日</x:v>
       </x:c>
       <x:c r="D19" s="22" t="n">
-        <x:v>7741.906</x:v>
+        <x:v>7741.91</x:v>
       </x:c>
       <x:c r="E19" s="22" t="n">
-        <x:v>7889.446</x:v>
+        <x:v>7889.45</x:v>
       </x:c>
       <x:c r="F19" s="22" t="n">
-        <x:v>7701.221</x:v>
+        <x:v>7701.22</x:v>
       </x:c>
       <x:c r="G19" s="22" t="n">
-        <x:v>7751.662</x:v>
+        <x:v>7751.66</x:v>
       </x:c>
       <x:c r="H19" s="22" t="n">
         <x:v>-48.9</x:v>
       </x:c>
       <x:c r="I19" s="23" t="n">
-        <x:v>-0.006274766495795392</x:v>
+        <x:v>-0.006275150276709107</x:v>
       </x:c>
       <x:c r="J19" s="27" t="n">
         <x:f>ROUND(E19-F19,1)</x:f>
@@ -2181,22 +2397,22 @@
         <x:v>7月23日</x:v>
       </x:c>
       <x:c r="D20" s="22" t="n">
-        <x:v>7750.852</x:v>
+        <x:v>7750.85</x:v>
       </x:c>
       <x:c r="E20" s="22" t="n">
         <x:v>7795.35</x:v>
       </x:c>
       <x:c r="F20" s="22" t="n">
-        <x:v>7658.999</x:v>
+        <x:v>7659</x:v>
       </x:c>
       <x:c r="G20" s="22" t="n">
         <x:v>7734.31</x:v>
       </x:c>
       <x:c r="H20" s="22" t="n">
-        <x:v>-17.4</x:v>
+        <x:v>-17.3</x:v>
       </x:c>
       <x:c r="I20" s="23" t="n">
-        <x:v>-0.0022384876946388577</x:v>
+        <x:v>-0.0022382302629371242</x:v>
       </x:c>
       <x:c r="J20" s="22" t="n">
         <x:f>ROUND(E20-F20,1)</x:f>
@@ -2206,43 +2422,259 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="21" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B21" s="21" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C21" s="21" t="str">
+        <x:v>7月24日</x:v>
+      </x:c>
+      <x:c r="D21" s="22" t="n">
+        <x:v>7625.2</x:v>
+      </x:c>
+      <x:c r="E21" s="22" t="n">
+        <x:v>7703.6</x:v>
+      </x:c>
+      <x:c r="F21" s="22" t="n">
+        <x:v>7532.67</x:v>
+      </x:c>
+      <x:c r="G21" s="22" t="n">
+        <x:v>7532.7</x:v>
+      </x:c>
+      <x:c r="H21" s="25" t="n">
+        <x:v>-201.6</x:v>
+      </x:c>
+      <x:c r="I21" s="23" t="n">
+        <x:v>-0.026066966542587555</x:v>
+      </x:c>
+      <x:c r="J21" s="27" t="n">
+        <x:f>ROUND(E21-F21,1)</x:f>
+        <x:v>170.9</x:v>
+      </x:c>
+      <x:c r="K21" s="21" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="21" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B22" s="21" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C22" s="21" t="str">
+        <x:v>7月27日</x:v>
+      </x:c>
+      <x:c r="D22" s="22" t="n">
+        <x:v>7512.4</x:v>
+      </x:c>
+      <x:c r="E22" s="22" t="n">
+        <x:v>7721.4</x:v>
+      </x:c>
+      <x:c r="F22" s="22" t="n">
+        <x:v>7466.54</x:v>
+      </x:c>
+      <x:c r="G22" s="22" t="n">
+        <x:v>7720.6</x:v>
+      </x:c>
+      <x:c r="H22" s="25" t="n">
+        <x:v>187.9</x:v>
+      </x:c>
+      <x:c r="I22" s="23" t="n">
+        <x:v>0.024944574986392798</x:v>
+      </x:c>
+      <x:c r="J22" s="27" t="n">
+        <x:f>ROUND(E22-F22,1)</x:f>
+        <x:v>254.9</x:v>
+      </x:c>
+      <x:c r="K22" s="21" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+    </x:row>
     <x:row r="23">
-      <x:c r="A23" s="38" t="str">
+      <x:c r="A23" s="21" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B23" s="21" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C23" s="21" t="str">
+        <x:v>7月28日</x:v>
+      </x:c>
+      <x:c r="D23" s="22" t="n">
+        <x:v>7589.76</x:v>
+      </x:c>
+      <x:c r="E23" s="22" t="n">
+        <x:v>7646.02</x:v>
+      </x:c>
+      <x:c r="F23" s="22" t="n">
+        <x:v>7412.63</x:v>
+      </x:c>
+      <x:c r="G23" s="22" t="n">
+        <x:v>7443.43</x:v>
+      </x:c>
+      <x:c r="H23" s="25" t="n">
+        <x:v>-277.2</x:v>
+      </x:c>
+      <x:c r="I23" s="23" t="n">
+        <x:v>-0.03590005958086162</x:v>
+      </x:c>
+      <x:c r="J23" s="27" t="n">
+        <x:f>ROUND(E23-F23,1)</x:f>
+        <x:v>233.4</x:v>
+      </x:c>
+      <x:c r="K23" s="21" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="21" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B24" s="21" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C24" s="21" t="str">
+        <x:v>7月29日</x:v>
+      </x:c>
+      <x:c r="D24" s="22" t="n">
+        <x:v>7444.8</x:v>
+      </x:c>
+      <x:c r="E24" s="22" t="n">
+        <x:v>7572.81</x:v>
+      </x:c>
+      <x:c r="F24" s="22" t="n">
+        <x:v>7325.36</x:v>
+      </x:c>
+      <x:c r="G24" s="22" t="n">
+        <x:v>7524.51</x:v>
+      </x:c>
+      <x:c r="H24" s="22" t="n">
+        <x:v>81.1</x:v>
+      </x:c>
+      <x:c r="I24" s="23" t="n">
+        <x:v>0.010892827634571667</x:v>
+      </x:c>
+      <x:c r="J24" s="27" t="n">
+        <x:f>ROUND(E24-F24,1)</x:f>
+        <x:v>247.5</x:v>
+      </x:c>
+      <x:c r="K24" s="21" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="21" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B25" s="21" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C25" s="21" t="str">
+        <x:v>7月30日</x:v>
+      </x:c>
+      <x:c r="D25" s="22" t="n">
+        <x:v>7477.31</x:v>
+      </x:c>
+      <x:c r="E25" s="22" t="n">
+        <x:v>7536.49</x:v>
+      </x:c>
+      <x:c r="F25" s="22" t="n">
+        <x:v>7221.95</x:v>
+      </x:c>
+      <x:c r="G25" s="22" t="n">
+        <x:v>7309.58</x:v>
+      </x:c>
+      <x:c r="H25" s="25" t="n">
+        <x:v>-214.9</x:v>
+      </x:c>
+      <x:c r="I25" s="23" t="n">
+        <x:v>-0.028563986226345706</x:v>
+      </x:c>
+      <x:c r="J25" s="27" t="n">
+        <x:f>ROUND(E25-F25,1)</x:f>
+        <x:v>314.5</x:v>
+      </x:c>
+      <x:c r="K25" s="21" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="21" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B26" s="21" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C26" s="21" t="str">
+        <x:v>7月31日</x:v>
+      </x:c>
+      <x:c r="D26" s="22" t="n">
+        <x:v>7537.85</x:v>
+      </x:c>
+      <x:c r="E26" s="22" t="n">
+        <x:v>7638.78</x:v>
+      </x:c>
+      <x:c r="F26" s="22" t="n">
+        <x:v>7487.43</x:v>
+      </x:c>
+      <x:c r="G26" s="22" t="n">
+        <x:v>7493.99</x:v>
+      </x:c>
+      <x:c r="H26" s="25" t="n">
+        <x:v>184.4</x:v>
+      </x:c>
+      <x:c r="I26" s="23" t="n">
+        <x:v>0.025228535702461752</x:v>
+      </x:c>
+      <x:c r="J26" s="22" t="n">
+        <x:f>ROUND(E26-F26,1)</x:f>
+        <x:v>151.3</x:v>
+      </x:c>
+      <x:c r="K26" s="21" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="38" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B23" s="39" t="n">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="C23" s="39"/>
-      <x:c r="D23" s="39"/>
-      <x:c r="E23" s="39"/>
-      <x:c r="F23" s="39"/>
-      <x:c r="G23" s="39"/>
-      <x:c r="H23" s="39"/>
-      <x:c r="I23" s="39"/>
-      <x:c r="J23" s="40" t="n">
-        <x:f>SUM(J4:J20)</x:f>
-        <x:v>4789.299999999999</x:v>
-      </x:c>
-      <x:c r="K23" s="39"/>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="38" t="str">
+      <x:c r="B29" s="39" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="C29" s="39"/>
+      <x:c r="D29" s="39"/>
+      <x:c r="E29" s="39"/>
+      <x:c r="F29" s="39"/>
+      <x:c r="G29" s="39"/>
+      <x:c r="H29" s="39"/>
+      <x:c r="I29" s="39"/>
+      <x:c r="J29" s="40" t="n">
+        <x:f>SUM(J4:J26)</x:f>
+        <x:v>6161.699999999999</x:v>
+      </x:c>
+      <x:c r="K29" s="39"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="38" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B24" s="39"/>
-      <x:c r="C24" s="39"/>
-      <x:c r="D24" s="39"/>
-      <x:c r="E24" s="39"/>
-      <x:c r="F24" s="39"/>
-      <x:c r="G24" s="39"/>
-      <x:c r="H24" s="39"/>
-      <x:c r="I24" s="39"/>
-      <x:c r="J24" s="42" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
-        <x:v>281.7</x:v>
-      </x:c>
-      <x:c r="K24" s="39"/>
+      <x:c r="B30" s="39"/>
+      <x:c r="C30" s="39"/>
+      <x:c r="D30" s="39"/>
+      <x:c r="E30" s="39"/>
+      <x:c r="F30" s="39"/>
+      <x:c r="G30" s="39"/>
+      <x:c r="H30" s="39"/>
+      <x:c r="I30" s="39"/>
+      <x:c r="J30" s="42" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J26),0),1)</x:f>
+        <x:v>267.9</x:v>
+      </x:c>
+      <x:c r="K30" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2323,19 +2755,19 @@
         <x:v>4090.76</x:v>
       </x:c>
       <x:c r="E4" s="22" t="n">
-        <x:v>4143.314</x:v>
+        <x:v>4143.31</x:v>
       </x:c>
       <x:c r="F4" s="22" t="n">
-        <x:v>4087.535</x:v>
+        <x:v>4087.54</x:v>
       </x:c>
       <x:c r="G4" s="22" t="n">
-        <x:v>4112.445</x:v>
+        <x:v>4112.45</x:v>
       </x:c>
       <x:c r="H4" s="22" t="n">
         <x:v>18</x:v>
       </x:c>
       <x:c r="I4" s="23" t="n">
-        <x:v>0.004407975093768224</x:v>
+        <x:v>0.004408460336068787</x:v>
       </x:c>
       <x:c r="J4" s="27" t="n">
         <x:f>ROUND(E4-F4,1)</x:f>
@@ -2356,22 +2788,22 @@
         <x:v>7月2日</x:v>
       </x:c>
       <x:c r="D5" s="22" t="n">
-        <x:v>4054.086</x:v>
+        <x:v>4054.09</x:v>
       </x:c>
       <x:c r="E5" s="22" t="n">
-        <x:v>4093.678</x:v>
+        <x:v>4093.68</x:v>
       </x:c>
       <x:c r="F5" s="22" t="n">
-        <x:v>4019.215</x:v>
+        <x:v>4019.21</x:v>
       </x:c>
       <x:c r="G5" s="22" t="n">
-        <x:v>4028.904</x:v>
+        <x:v>4028.9</x:v>
       </x:c>
       <x:c r="H5" s="22" t="n">
         <x:v>-83.5</x:v>
       </x:c>
       <x:c r="I5" s="23" t="n">
-        <x:v>-0.020314192651816554</x:v>
+        <x:v>-0.02031635642986529</x:v>
       </x:c>
       <x:c r="J5" s="27" t="n">
         <x:f>ROUND(E5-F5,1)</x:f>
@@ -2392,22 +2824,22 @@
         <x:v>7月3日</x:v>
       </x:c>
       <x:c r="D6" s="22" t="n">
-        <x:v>4031.335</x:v>
+        <x:v>4031.34</x:v>
       </x:c>
       <x:c r="E6" s="22" t="n">
         <x:v>4073.88</x:v>
       </x:c>
       <x:c r="F6" s="22" t="n">
-        <x:v>4027.255</x:v>
+        <x:v>4027.26</x:v>
       </x:c>
       <x:c r="G6" s="22" t="n">
-        <x:v>4043.643</x:v>
+        <x:v>4043.64</x:v>
       </x:c>
       <x:c r="H6" s="22" t="n">
         <x:v>14.7</x:v>
       </x:c>
       <x:c r="I6" s="23" t="n">
-        <x:v>0.0036583150156965782</x:v>
+        <x:v>0.0036585668544764083</x:v>
       </x:c>
       <x:c r="J6" s="22" t="n">
         <x:f>ROUND(E6-F6,1)</x:f>
@@ -2428,22 +2860,22 @@
         <x:v>7月6日</x:v>
       </x:c>
       <x:c r="D7" s="22" t="n">
-        <x:v>4059.194</x:v>
+        <x:v>4059.19</x:v>
       </x:c>
       <x:c r="E7" s="22" t="n">
-        <x:v>4060.069</x:v>
+        <x:v>4060.07</x:v>
       </x:c>
       <x:c r="F7" s="22" t="n">
-        <x:v>4005.414</x:v>
+        <x:v>4005.41</x:v>
       </x:c>
       <x:c r="G7" s="22" t="n">
-        <x:v>4041.238</x:v>
+        <x:v>4041.24</x:v>
       </x:c>
       <x:c r="H7" s="22" t="n">
         <x:v>-2.4</x:v>
       </x:c>
       <x:c r="I7" s="23" t="n">
-        <x:v>-0.000594760714533904</x:v>
+        <x:v>-0.0005935246461109545</x:v>
       </x:c>
       <x:c r="J7" s="27" t="n">
         <x:f>ROUND(E7-F7,1)</x:f>
@@ -2464,22 +2896,22 @@
         <x:v>7月7日</x:v>
       </x:c>
       <x:c r="D8" s="22" t="n">
-        <x:v>4019.494</x:v>
+        <x:v>4019.49</x:v>
       </x:c>
       <x:c r="E8" s="22" t="n">
-        <x:v>4028.514</x:v>
+        <x:v>4028.51</x:v>
       </x:c>
       <x:c r="F8" s="22" t="n">
-        <x:v>3971.713</x:v>
+        <x:v>3971.71</x:v>
       </x:c>
       <x:c r="G8" s="22" t="n">
-        <x:v>3990.235</x:v>
+        <x:v>3990.24</x:v>
       </x:c>
       <x:c r="H8" s="22" t="n">
         <x:v>-51</x:v>
       </x:c>
       <x:c r="I8" s="23" t="n">
-        <x:v>-0.01262063753730902</x:v>
+        <x:v>-0.012619888944977231</x:v>
       </x:c>
       <x:c r="J8" s="27" t="n">
         <x:f>ROUND(E8-F8,1)</x:f>
@@ -2500,13 +2932,13 @@
         <x:v>7月8日</x:v>
       </x:c>
       <x:c r="D9" s="22" t="n">
-        <x:v>3996.807</x:v>
+        <x:v>3996.81</x:v>
       </x:c>
       <x:c r="E9" s="22" t="n">
-        <x:v>4016.026</x:v>
+        <x:v>4016.03</x:v>
       </x:c>
       <x:c r="F9" s="22" t="n">
-        <x:v>3967.913</x:v>
+        <x:v>3967.91</x:v>
       </x:c>
       <x:c r="G9" s="22" t="n">
         <x:v>3970.88</x:v>
@@ -2515,7 +2947,7 @@
         <x:v>-19.4</x:v>
       </x:c>
       <x:c r="I9" s="23" t="n">
-        <x:v>-0.004850591506515234</x:v>
+        <x:v>-0.004851838485905535</x:v>
       </x:c>
       <x:c r="J9" s="22" t="n">
         <x:f>ROUND(E9-F9,1)</x:f>
@@ -2536,22 +2968,22 @@
         <x:v>7月9日</x:v>
       </x:c>
       <x:c r="D10" s="22" t="n">
-        <x:v>3977.547</x:v>
+        <x:v>3977.55</x:v>
       </x:c>
       <x:c r="E10" s="22" t="n">
-        <x:v>4040.539</x:v>
+        <x:v>4040.54</x:v>
       </x:c>
       <x:c r="F10" s="22" t="n">
-        <x:v>3938.878</x:v>
+        <x:v>3938.88</x:v>
       </x:c>
       <x:c r="G10" s="22" t="n">
-        <x:v>4036.588</x:v>
+        <x:v>4036.59</x:v>
       </x:c>
       <x:c r="H10" s="22" t="n">
         <x:v>65.7</x:v>
       </x:c>
       <x:c r="I10" s="23" t="n">
-        <x:v>0.01654746554919817</x:v>
+        <x:v>0.016547969215891634</x:v>
       </x:c>
       <x:c r="J10" s="27" t="n">
         <x:f>ROUND(E10-F10,1)</x:f>
@@ -2572,22 +3004,22 @@
         <x:v>7月10日</x:v>
       </x:c>
       <x:c r="D11" s="22" t="n">
-        <x:v>4031.537</x:v>
+        <x:v>4031.54</x:v>
       </x:c>
       <x:c r="E11" s="22" t="n">
-        <x:v>4074.828</x:v>
+        <x:v>4074.83</x:v>
       </x:c>
       <x:c r="F11" s="22" t="n">
-        <x:v>3995.807</x:v>
+        <x:v>3995.81</x:v>
       </x:c>
       <x:c r="G11" s="22" t="n">
-        <x:v>3996.162</x:v>
+        <x:v>3996.16</x:v>
       </x:c>
       <x:c r="H11" s="22" t="n">
         <x:v>-40.4</x:v>
       </x:c>
       <x:c r="I11" s="23" t="n">
-        <x:v>-0.010014893766715938</x:v>
+        <x:v>-0.010015879740077671</x:v>
       </x:c>
       <x:c r="J11" s="27" t="n">
         <x:f>ROUND(E11-F11,1)</x:f>
@@ -2608,22 +3040,22 @@
         <x:v>7月13日</x:v>
       </x:c>
       <x:c r="D12" s="22" t="n">
-        <x:v>3966.023</x:v>
+        <x:v>3966.02</x:v>
       </x:c>
       <x:c r="E12" s="22" t="n">
-        <x:v>3983.054</x:v>
+        <x:v>3983.05</x:v>
       </x:c>
       <x:c r="F12" s="22" t="n">
-        <x:v>3900.668</x:v>
+        <x:v>3900.67</x:v>
       </x:c>
       <x:c r="G12" s="22" t="n">
-        <x:v>3913.794</x:v>
+        <x:v>3913.79</x:v>
       </x:c>
       <x:c r="H12" s="22" t="n">
         <x:v>-82.4</x:v>
       </x:c>
       <x:c r="I12" s="23" t="n">
-        <x:v>-0.020611777000031473</x:v>
+        <x:v>-0.020612287796284434</x:v>
       </x:c>
       <x:c r="J12" s="27" t="n">
         <x:f>ROUND(E12-F12,1)</x:f>
@@ -2644,22 +3076,22 @@
         <x:v>7月14日</x:v>
       </x:c>
       <x:c r="D13" s="22" t="n">
-        <x:v>3909.274</x:v>
+        <x:v>3909.27</x:v>
       </x:c>
       <x:c r="E13" s="22" t="n">
-        <x:v>3967.126</x:v>
+        <x:v>3967.13</x:v>
       </x:c>
       <x:c r="F13" s="22" t="n">
-        <x:v>3869.304</x:v>
+        <x:v>3869.3</x:v>
       </x:c>
       <x:c r="G13" s="22" t="n">
-        <x:v>3967.126</x:v>
+        <x:v>3967.13</x:v>
       </x:c>
       <x:c r="H13" s="22" t="n">
         <x:v>53.3</x:v>
       </x:c>
       <x:c r="I13" s="23" t="n">
-        <x:v>0.01362667529256778</x:v>
+        <x:v>0.013628733273885363</x:v>
       </x:c>
       <x:c r="J13" s="27" t="n">
         <x:f>ROUND(E13-F13,1)</x:f>
@@ -2680,22 +3112,22 @@
         <x:v>7月15日</x:v>
       </x:c>
       <x:c r="D14" s="22" t="n">
-        <x:v>3963.727</x:v>
+        <x:v>3963.73</x:v>
       </x:c>
       <x:c r="E14" s="22" t="n">
-        <x:v>3981.672</x:v>
+        <x:v>3981.67</x:v>
       </x:c>
       <x:c r="F14" s="22" t="n">
-        <x:v>3943.695</x:v>
+        <x:v>3943.7</x:v>
       </x:c>
       <x:c r="G14" s="22" t="n">
-        <x:v>3955.578</x:v>
+        <x:v>3955.58</x:v>
       </x:c>
       <x:c r="H14" s="22" t="n">
-        <x:v>-11.5</x:v>
+        <x:v>-11.6</x:v>
       </x:c>
       <x:c r="I14" s="23" t="n">
-        <x:v>-0.002910923424161549</x:v>
+        <x:v>-0.00291142463191274</x:v>
       </x:c>
       <x:c r="J14" s="22" t="n">
         <x:f>ROUND(E14-F14,1)</x:f>
@@ -2716,22 +3148,22 @@
         <x:v>7月16日</x:v>
       </x:c>
       <x:c r="D15" s="22" t="n">
-        <x:v>3912.381</x:v>
+        <x:v>3912.38</x:v>
       </x:c>
       <x:c r="E15" s="22" t="n">
-        <x:v>3940.451</x:v>
+        <x:v>3940.45</x:v>
       </x:c>
       <x:c r="F15" s="22" t="n">
-        <x:v>3867.601</x:v>
+        <x:v>3867.6</x:v>
       </x:c>
       <x:c r="G15" s="22" t="n">
-        <x:v>3882.413</x:v>
+        <x:v>3882.41</x:v>
       </x:c>
       <x:c r="H15" s="22" t="n">
         <x:v>-73.2</x:v>
       </x:c>
       <x:c r="I15" s="23" t="n">
-        <x:v>-0.01849666470993616</x:v>
+        <x:v>-0.018497919394880213</x:v>
       </x:c>
       <x:c r="J15" s="27" t="n">
         <x:f>ROUND(E15-F15,1)</x:f>
@@ -2752,22 +3184,22 @@
         <x:v>7月17日</x:v>
       </x:c>
       <x:c r="D16" s="32" t="n">
-        <x:v>3865.317</x:v>
+        <x:v>3865.32</x:v>
       </x:c>
       <x:c r="E16" s="32" t="n">
-        <x:v>3869.215</x:v>
+        <x:v>3869.21</x:v>
       </x:c>
       <x:c r="F16" s="32" t="n">
-        <x:v>3745.174</x:v>
+        <x:v>3745.17</x:v>
       </x:c>
       <x:c r="G16" s="32" t="n">
-        <x:v>3764.155</x:v>
+        <x:v>3764.15</x:v>
       </x:c>
       <x:c r="H16" s="32" t="n">
         <x:v>-118.3</x:v>
       </x:c>
       <x:c r="I16" s="33" t="n">
-        <x:v>-0.030459922733619527</x:v>
+        <x:v>-0.030460461414430706</x:v>
       </x:c>
       <x:c r="J16" s="27" t="n">
         <x:f>ROUND(E16-F16,1)</x:f>
@@ -2788,22 +3220,22 @@
         <x:v>7月20日</x:v>
       </x:c>
       <x:c r="D17" s="22" t="n">
-        <x:v>3791.662</x:v>
+        <x:v>3791.66</x:v>
       </x:c>
       <x:c r="E17" s="22" t="n">
-        <x:v>3831.659</x:v>
+        <x:v>3831.66</x:v>
       </x:c>
       <x:c r="F17" s="22" t="n">
         <x:v>3741.11</x:v>
       </x:c>
       <x:c r="G17" s="22" t="n">
-        <x:v>3796.281</x:v>
+        <x:v>3796.28</x:v>
       </x:c>
       <x:c r="H17" s="22" t="n">
         <x:v>32.1</x:v>
       </x:c>
       <x:c r="I17" s="23" t="n">
-        <x:v>0.008534717619226528</x:v>
+        <x:v>0.008535791612980459</x:v>
       </x:c>
       <x:c r="J17" s="27" t="n">
         <x:f>ROUND(E17-F17,1)</x:f>
@@ -2824,7 +3256,7 @@
         <x:v>7月21日</x:v>
       </x:c>
       <x:c r="D18" s="22" t="n">
-        <x:v>3812.162</x:v>
+        <x:v>3812.16</x:v>
       </x:c>
       <x:c r="E18" s="22" t="n">
         <x:v>3864.6</x:v>
@@ -2833,13 +3265,13 @@
         <x:v>3743.36</x:v>
       </x:c>
       <x:c r="G18" s="22" t="n">
-        <x:v>3864.367</x:v>
+        <x:v>3864.37</x:v>
       </x:c>
       <x:c r="H18" s="22" t="n">
         <x:v>68.1</x:v>
       </x:c>
       <x:c r="I18" s="23" t="n">
-        <x:v>0.01793492104509653</x:v>
+        <x:v>0.017935979432496918</x:v>
       </x:c>
       <x:c r="J18" s="27" t="n">
         <x:f>ROUND(E18-F18,1)</x:f>
@@ -2860,22 +3292,22 @@
         <x:v>7月22日</x:v>
       </x:c>
       <x:c r="D19" s="22" t="n">
-        <x:v>3839.665</x:v>
+        <x:v>3839.67</x:v>
       </x:c>
       <x:c r="E19" s="22" t="n">
-        <x:v>3884.435</x:v>
+        <x:v>3884.44</x:v>
       </x:c>
       <x:c r="F19" s="22" t="n">
-        <x:v>3839.665</x:v>
+        <x:v>3839.67</x:v>
       </x:c>
       <x:c r="G19" s="22" t="n">
-        <x:v>3867.034</x:v>
+        <x:v>3867.03</x:v>
       </x:c>
       <x:c r="H19" s="22" t="n">
         <x:v>2.7</x:v>
       </x:c>
       <x:c r="I19" s="23" t="n">
-        <x:v>0.0006901518411681629</x:v>
+        <x:v>0.0006883398846384559</x:v>
       </x:c>
       <x:c r="J19" s="22" t="n">
         <x:f>ROUND(E19-F19,1)</x:f>
@@ -2896,22 +3328,22 @@
         <x:v>7月23日</x:v>
       </x:c>
       <x:c r="D20" s="22" t="n">
-        <x:v>3868.087</x:v>
+        <x:v>3868.09</x:v>
       </x:c>
       <x:c r="E20" s="22" t="n">
-        <x:v>3878.832</x:v>
+        <x:v>3878.83</x:v>
       </x:c>
       <x:c r="F20" s="22" t="n">
-        <x:v>3851.706</x:v>
+        <x:v>3851.71</x:v>
       </x:c>
       <x:c r="G20" s="22" t="n">
-        <x:v>3876.777</x:v>
+        <x:v>3876.78</x:v>
       </x:c>
       <x:c r="H20" s="22" t="n">
-        <x:v>9.7</x:v>
+        <x:v>9.8</x:v>
       </x:c>
       <x:c r="I20" s="23" t="n">
-        <x:v>0.0025195020266177703</x:v>
+        <x:v>0.002521314807487851</x:v>
       </x:c>
       <x:c r="J20" s="22" t="n">
         <x:f>ROUND(E20-F20,1)</x:f>
@@ -2921,43 +3353,259 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="21" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B21" s="21" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C21" s="21" t="str">
+        <x:v>7月24日</x:v>
+      </x:c>
+      <x:c r="D21" s="22" t="n">
+        <x:v>3853.63</x:v>
+      </x:c>
+      <x:c r="E21" s="22" t="n">
+        <x:v>3861.04</x:v>
+      </x:c>
+      <x:c r="F21" s="22" t="n">
+        <x:v>3808.64</x:v>
+      </x:c>
+      <x:c r="G21" s="22" t="n">
+        <x:v>3814.2</x:v>
+      </x:c>
+      <x:c r="H21" s="22" t="n">
+        <x:v>-62.6</x:v>
+      </x:c>
+      <x:c r="I21" s="23" t="n">
+        <x:v>-0.01614226239301697</x:v>
+      </x:c>
+      <x:c r="J21" s="27" t="n">
+        <x:f>ROUND(E21-F21,1)</x:f>
+        <x:v>52.4</x:v>
+      </x:c>
+      <x:c r="K21" s="21" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="21" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B22" s="21" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C22" s="21" t="str">
+        <x:v>7月27日</x:v>
+      </x:c>
+      <x:c r="D22" s="22" t="n">
+        <x:v>3808.9</x:v>
+      </x:c>
+      <x:c r="E22" s="22" t="n">
+        <x:v>3858.31</x:v>
+      </x:c>
+      <x:c r="F22" s="22" t="n">
+        <x:v>3793.45</x:v>
+      </x:c>
+      <x:c r="G22" s="22" t="n">
+        <x:v>3858.25</x:v>
+      </x:c>
+      <x:c r="H22" s="22" t="n">
+        <x:v>44.1</x:v>
+      </x:c>
+      <x:c r="I22" s="23" t="n">
+        <x:v>0.011548948665513148</x:v>
+      </x:c>
+      <x:c r="J22" s="27" t="n">
+        <x:f>ROUND(E22-F22,1)</x:f>
+        <x:v>64.9</x:v>
+      </x:c>
+      <x:c r="K22" s="21" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+    </x:row>
     <x:row r="23">
-      <x:c r="A23" s="38" t="str">
+      <x:c r="A23" s="21" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B23" s="21" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C23" s="21" t="str">
+        <x:v>7月28日</x:v>
+      </x:c>
+      <x:c r="D23" s="22" t="n">
+        <x:v>3823.13</x:v>
+      </x:c>
+      <x:c r="E23" s="22" t="n">
+        <x:v>3844.01</x:v>
+      </x:c>
+      <x:c r="F23" s="22" t="n">
+        <x:v>3797.37</x:v>
+      </x:c>
+      <x:c r="G23" s="22" t="n">
+        <x:v>3813.31</x:v>
+      </x:c>
+      <x:c r="H23" s="22" t="n">
+        <x:v>-44.9</x:v>
+      </x:c>
+      <x:c r="I23" s="23" t="n">
+        <x:v>-0.01164776777036225</x:v>
+      </x:c>
+      <x:c r="J23" s="22" t="n">
+        <x:f>ROUND(E23-F23,1)</x:f>
+        <x:v>46.6</x:v>
+      </x:c>
+      <x:c r="K23" s="21" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="21" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B24" s="21" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C24" s="21" t="str">
+        <x:v>7月29日</x:v>
+      </x:c>
+      <x:c r="D24" s="22" t="n">
+        <x:v>3823.29</x:v>
+      </x:c>
+      <x:c r="E24" s="22" t="n">
+        <x:v>3845.77</x:v>
+      </x:c>
+      <x:c r="F24" s="22" t="n">
+        <x:v>3782.48</x:v>
+      </x:c>
+      <x:c r="G24" s="22" t="n">
+        <x:v>3828.47</x:v>
+      </x:c>
+      <x:c r="H24" s="22" t="n">
+        <x:v>15.2</x:v>
+      </x:c>
+      <x:c r="I24" s="23" t="n">
+        <x:v>0.003975548801435025</x:v>
+      </x:c>
+      <x:c r="J24" s="27" t="n">
+        <x:f>ROUND(E24-F24,1)</x:f>
+        <x:v>63.3</x:v>
+      </x:c>
+      <x:c r="K24" s="21" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="21" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B25" s="21" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C25" s="21" t="str">
+        <x:v>7月30日</x:v>
+      </x:c>
+      <x:c r="D25" s="22" t="n">
+        <x:v>3812.11</x:v>
+      </x:c>
+      <x:c r="E25" s="22" t="n">
+        <x:v>3839.34</x:v>
+      </x:c>
+      <x:c r="F25" s="22" t="n">
+        <x:v>3767.5</x:v>
+      </x:c>
+      <x:c r="G25" s="22" t="n">
+        <x:v>3804.69</x:v>
+      </x:c>
+      <x:c r="H25" s="22" t="n">
+        <x:v>-23.8</x:v>
+      </x:c>
+      <x:c r="I25" s="23" t="n">
+        <x:v>-0.0062113585844997266</x:v>
+      </x:c>
+      <x:c r="J25" s="27" t="n">
+        <x:f>ROUND(E25-F25,1)</x:f>
+        <x:v>71.8</x:v>
+      </x:c>
+      <x:c r="K25" s="21" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="21" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B26" s="21" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C26" s="21" t="str">
+        <x:v>7月31日</x:v>
+      </x:c>
+      <x:c r="D26" s="22" t="n">
+        <x:v>3833.54</x:v>
+      </x:c>
+      <x:c r="E26" s="22" t="n">
+        <x:v>3847.09</x:v>
+      </x:c>
+      <x:c r="F26" s="22" t="n">
+        <x:v>3822.37</x:v>
+      </x:c>
+      <x:c r="G26" s="22" t="n">
+        <x:v>3832.26</x:v>
+      </x:c>
+      <x:c r="H26" s="22" t="n">
+        <x:v>27.6</x:v>
+      </x:c>
+      <x:c r="I26" s="23" t="n">
+        <x:v>0.007246319673876123</x:v>
+      </x:c>
+      <x:c r="J26" s="22" t="n">
+        <x:f>ROUND(E26-F26,1)</x:f>
+        <x:v>24.7</x:v>
+      </x:c>
+      <x:c r="K26" s="21" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="38" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B23" s="39" t="n">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="C23" s="39"/>
-      <x:c r="D23" s="39"/>
-      <x:c r="E23" s="39"/>
-      <x:c r="F23" s="39"/>
-      <x:c r="G23" s="39"/>
-      <x:c r="H23" s="39"/>
-      <x:c r="I23" s="39"/>
-      <x:c r="J23" s="40" t="n">
-        <x:f>SUM(J4:J20)</x:f>
-        <x:v>1215.7999999999997</x:v>
-      </x:c>
-      <x:c r="K23" s="39"/>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="38" t="str">
+      <x:c r="B29" s="39" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="C29" s="39"/>
+      <x:c r="D29" s="39"/>
+      <x:c r="E29" s="39"/>
+      <x:c r="F29" s="39"/>
+      <x:c r="G29" s="39"/>
+      <x:c r="H29" s="39"/>
+      <x:c r="I29" s="39"/>
+      <x:c r="J29" s="40" t="n">
+        <x:f>SUM(J4:J26)</x:f>
+        <x:v>1539.4999999999998</x:v>
+      </x:c>
+      <x:c r="K29" s="39"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="38" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B24" s="39"/>
-      <x:c r="C24" s="39"/>
-      <x:c r="D24" s="39"/>
-      <x:c r="E24" s="39"/>
-      <x:c r="F24" s="39"/>
-      <x:c r="G24" s="39"/>
-      <x:c r="H24" s="39"/>
-      <x:c r="I24" s="39"/>
-      <x:c r="J24" s="42" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
-        <x:v>71.5</x:v>
-      </x:c>
-      <x:c r="K24" s="39"/>
+      <x:c r="B30" s="39"/>
+      <x:c r="C30" s="39"/>
+      <x:c r="D30" s="39"/>
+      <x:c r="E30" s="39"/>
+      <x:c r="F30" s="39"/>
+      <x:c r="G30" s="39"/>
+      <x:c r="H30" s="39"/>
+      <x:c r="I30" s="39"/>
+      <x:c r="J30" s="42" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J26),0),1)</x:f>
+        <x:v>66.9</x:v>
+      </x:c>
+      <x:c r="K30" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3636,43 +4284,259 @@
         <x:v>IM2609</x:v>
       </x:c>
     </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="21" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B21" s="21" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C21" s="21" t="str">
+        <x:v>7月24日</x:v>
+      </x:c>
+      <x:c r="D21" s="22" t="n">
+        <x:v>7000</x:v>
+      </x:c>
+      <x:c r="E21" s="22" t="n">
+        <x:v>7054.8</x:v>
+      </x:c>
+      <x:c r="F21" s="22" t="n">
+        <x:v>6866</x:v>
+      </x:c>
+      <x:c r="G21" s="22" t="n">
+        <x:v>6880.2</x:v>
+      </x:c>
+      <x:c r="H21" s="25" t="n">
+        <x:v>-191.4</x:v>
+      </x:c>
+      <x:c r="I21" s="23" t="n">
+        <x:v>-0.02706601052095714</x:v>
+      </x:c>
+      <x:c r="J21" s="22" t="n">
+        <x:f>ROUND(E21-F21,1)</x:f>
+        <x:v>188.8</x:v>
+      </x:c>
+      <x:c r="K21" s="21" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="21" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B22" s="21" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C22" s="21" t="str">
+        <x:v>7月27日</x:v>
+      </x:c>
+      <x:c r="D22" s="22" t="n">
+        <x:v>6880.4</x:v>
+      </x:c>
+      <x:c r="E22" s="22" t="n">
+        <x:v>7155</x:v>
+      </x:c>
+      <x:c r="F22" s="22" t="n">
+        <x:v>6880.4</x:v>
+      </x:c>
+      <x:c r="G22" s="22" t="n">
+        <x:v>7148.8</x:v>
+      </x:c>
+      <x:c r="H22" s="25" t="n">
+        <x:v>268.6</x:v>
+      </x:c>
+      <x:c r="I22" s="23" t="n">
+        <x:v>0.039039562803407035</x:v>
+      </x:c>
+      <x:c r="J22" s="27" t="n">
+        <x:f>ROUND(E22-F22,1)</x:f>
+        <x:v>274.6</x:v>
+      </x:c>
+      <x:c r="K22" s="21" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+    </x:row>
     <x:row r="23">
-      <x:c r="A23" s="38" t="str">
+      <x:c r="A23" s="21" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B23" s="21" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C23" s="21" t="str">
+        <x:v>7月28日</x:v>
+      </x:c>
+      <x:c r="D23" s="22" t="n">
+        <x:v>7020</x:v>
+      </x:c>
+      <x:c r="E23" s="22" t="n">
+        <x:v>7075.6</x:v>
+      </x:c>
+      <x:c r="F23" s="22" t="n">
+        <x:v>6888.8</x:v>
+      </x:c>
+      <x:c r="G23" s="22" t="n">
+        <x:v>6943.2</x:v>
+      </x:c>
+      <x:c r="H23" s="25" t="n">
+        <x:v>-205.6</x:v>
+      </x:c>
+      <x:c r="I23" s="23" t="n">
+        <x:v>-0.02876007162041183</x:v>
+      </x:c>
+      <x:c r="J23" s="22" t="n">
+        <x:f>ROUND(E23-F23,1)</x:f>
+        <x:v>186.8</x:v>
+      </x:c>
+      <x:c r="K23" s="21" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="21" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B24" s="21" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C24" s="21" t="str">
+        <x:v>7月29日</x:v>
+      </x:c>
+      <x:c r="D24" s="22" t="n">
+        <x:v>6966</x:v>
+      </x:c>
+      <x:c r="E24" s="22" t="n">
+        <x:v>7081</x:v>
+      </x:c>
+      <x:c r="F24" s="22" t="n">
+        <x:v>6825</x:v>
+      </x:c>
+      <x:c r="G24" s="22" t="n">
+        <x:v>7047.2</x:v>
+      </x:c>
+      <x:c r="H24" s="22" t="n">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="I24" s="23" t="n">
+        <x:v>0.014978684180205093</x:v>
+      </x:c>
+      <x:c r="J24" s="27" t="n">
+        <x:f>ROUND(E24-F24,1)</x:f>
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="K24" s="21" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="21" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B25" s="21" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C25" s="21" t="str">
+        <x:v>7月30日</x:v>
+      </x:c>
+      <x:c r="D25" s="22" t="n">
+        <x:v>7033.4</x:v>
+      </x:c>
+      <x:c r="E25" s="22" t="n">
+        <x:v>7088</x:v>
+      </x:c>
+      <x:c r="F25" s="22" t="n">
+        <x:v>6757.6</x:v>
+      </x:c>
+      <x:c r="G25" s="22" t="n">
+        <x:v>6845.2</x:v>
+      </x:c>
+      <x:c r="H25" s="25" t="n">
+        <x:v>-202</x:v>
+      </x:c>
+      <x:c r="I25" s="23" t="n">
+        <x:v>-0.028663866500170276</x:v>
+      </x:c>
+      <x:c r="J25" s="27" t="n">
+        <x:f>ROUND(E25-F25,1)</x:f>
+        <x:v>330.4</x:v>
+      </x:c>
+      <x:c r="K25" s="21" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="21" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B26" s="21" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C26" s="21" t="str">
+        <x:v>7月31日</x:v>
+      </x:c>
+      <x:c r="D26" s="22" t="n">
+        <x:v>7110</x:v>
+      </x:c>
+      <x:c r="E26" s="22" t="n">
+        <x:v>7205</x:v>
+      </x:c>
+      <x:c r="F26" s="22" t="n">
+        <x:v>6986</x:v>
+      </x:c>
+      <x:c r="G26" s="22" t="n">
+        <x:v>6987.8</x:v>
+      </x:c>
+      <x:c r="H26" s="22" t="n">
+        <x:v>142.6</x:v>
+      </x:c>
+      <x:c r="I26" s="23" t="n">
+        <x:v>0.020832115935254025</x:v>
+      </x:c>
+      <x:c r="J26" s="27" t="n">
+        <x:f>ROUND(E26-F26,1)</x:f>
+        <x:v>219</x:v>
+      </x:c>
+      <x:c r="K26" s="21" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="38" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B23" s="39" t="n">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="C23" s="39"/>
-      <x:c r="D23" s="39"/>
-      <x:c r="E23" s="39"/>
-      <x:c r="F23" s="39"/>
-      <x:c r="G23" s="39"/>
-      <x:c r="H23" s="39"/>
-      <x:c r="I23" s="39"/>
-      <x:c r="J23" s="40" t="n">
-        <x:f>SUM(J4:J20)</x:f>
-        <x:v>4631.6</x:v>
-      </x:c>
-      <x:c r="K23" s="39"/>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="38" t="str">
+      <x:c r="B29" s="39" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="C29" s="39"/>
+      <x:c r="D29" s="39"/>
+      <x:c r="E29" s="39"/>
+      <x:c r="F29" s="39"/>
+      <x:c r="G29" s="39"/>
+      <x:c r="H29" s="39"/>
+      <x:c r="I29" s="39"/>
+      <x:c r="J29" s="40" t="n">
+        <x:f>SUM(J4:J26)</x:f>
+        <x:v>6087.200000000001</x:v>
+      </x:c>
+      <x:c r="K29" s="39"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="38" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B24" s="39"/>
-      <x:c r="C24" s="39"/>
-      <x:c r="D24" s="39"/>
-      <x:c r="E24" s="39"/>
-      <x:c r="F24" s="39"/>
-      <x:c r="G24" s="39"/>
-      <x:c r="H24" s="39"/>
-      <x:c r="I24" s="39"/>
-      <x:c r="J24" s="42" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
-        <x:v>272.4</x:v>
-      </x:c>
-      <x:c r="K24" s="39"/>
+      <x:c r="B30" s="39"/>
+      <x:c r="C30" s="39"/>
+      <x:c r="D30" s="39"/>
+      <x:c r="E30" s="39"/>
+      <x:c r="F30" s="39"/>
+      <x:c r="G30" s="39"/>
+      <x:c r="H30" s="39"/>
+      <x:c r="I30" s="39"/>
+      <x:c r="J30" s="42" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J26),0),1)</x:f>
+        <x:v>264.7</x:v>
+      </x:c>
+      <x:c r="K30" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4351,43 +5215,259 @@
         <x:v>IC2609</x:v>
       </x:c>
     </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="21" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B21" s="21" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C21" s="21" t="str">
+        <x:v>7月24日</x:v>
+      </x:c>
+      <x:c r="D21" s="22" t="n">
+        <x:v>7520</x:v>
+      </x:c>
+      <x:c r="E21" s="22" t="n">
+        <x:v>7596</x:v>
+      </x:c>
+      <x:c r="F21" s="22" t="n">
+        <x:v>7410.6</x:v>
+      </x:c>
+      <x:c r="G21" s="22" t="n">
+        <x:v>7416</x:v>
+      </x:c>
+      <x:c r="H21" s="25" t="n">
+        <x:v>-186.6</x:v>
+      </x:c>
+      <x:c r="I21" s="23" t="n">
+        <x:v>-0.024544234867019177</x:v>
+      </x:c>
+      <x:c r="J21" s="27" t="n">
+        <x:f>ROUND(E21-F21,1)</x:f>
+        <x:v>185.4</x:v>
+      </x:c>
+      <x:c r="K21" s="21" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="21" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B22" s="21" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C22" s="21" t="str">
+        <x:v>7月27日</x:v>
+      </x:c>
+      <x:c r="D22" s="22" t="n">
+        <x:v>7447</x:v>
+      </x:c>
+      <x:c r="E22" s="22" t="n">
+        <x:v>7666.6</x:v>
+      </x:c>
+      <x:c r="F22" s="22" t="n">
+        <x:v>7394.2</x:v>
+      </x:c>
+      <x:c r="G22" s="22" t="n">
+        <x:v>7647</x:v>
+      </x:c>
+      <x:c r="H22" s="25" t="n">
+        <x:v>231</x:v>
+      </x:c>
+      <x:c r="I22" s="23" t="n">
+        <x:v>0.03114886731391575</x:v>
+      </x:c>
+      <x:c r="J22" s="27" t="n">
+        <x:f>ROUND(E22-F22,1)</x:f>
+        <x:v>272.4</x:v>
+      </x:c>
+      <x:c r="K22" s="21" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+    </x:row>
     <x:row r="23">
-      <x:c r="A23" s="38" t="str">
+      <x:c r="A23" s="21" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B23" s="21" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C23" s="21" t="str">
+        <x:v>7月28日</x:v>
+      </x:c>
+      <x:c r="D23" s="22" t="n">
+        <x:v>7489</x:v>
+      </x:c>
+      <x:c r="E23" s="22" t="n">
+        <x:v>7535.8</x:v>
+      </x:c>
+      <x:c r="F23" s="22" t="n">
+        <x:v>7285.2</x:v>
+      </x:c>
+      <x:c r="G23" s="22" t="n">
+        <x:v>7352.4</x:v>
+      </x:c>
+      <x:c r="H23" s="25" t="n">
+        <x:v>-294.6</x:v>
+      </x:c>
+      <x:c r="I23" s="23" t="n">
+        <x:v>-0.03852491173009032</x:v>
+      </x:c>
+      <x:c r="J23" s="27" t="n">
+        <x:f>ROUND(E23-F23,1)</x:f>
+        <x:v>250.6</x:v>
+      </x:c>
+      <x:c r="K23" s="21" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="21" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B24" s="21" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C24" s="21" t="str">
+        <x:v>7月29日</x:v>
+      </x:c>
+      <x:c r="D24" s="22" t="n">
+        <x:v>7380</x:v>
+      </x:c>
+      <x:c r="E24" s="22" t="n">
+        <x:v>7514.8</x:v>
+      </x:c>
+      <x:c r="F24" s="22" t="n">
+        <x:v>7260.6</x:v>
+      </x:c>
+      <x:c r="G24" s="22" t="n">
+        <x:v>7454.2</x:v>
+      </x:c>
+      <x:c r="H24" s="22" t="n">
+        <x:v>101.8</x:v>
+      </x:c>
+      <x:c r="I24" s="23" t="n">
+        <x:v>0.013845819052282327</x:v>
+      </x:c>
+      <x:c r="J24" s="27" t="n">
+        <x:f>ROUND(E24-F24,1)</x:f>
+        <x:v>254.2</x:v>
+      </x:c>
+      <x:c r="K24" s="21" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="21" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B25" s="21" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C25" s="21" t="str">
+        <x:v>7月30日</x:v>
+      </x:c>
+      <x:c r="D25" s="22" t="n">
+        <x:v>7405</x:v>
+      </x:c>
+      <x:c r="E25" s="22" t="n">
+        <x:v>7487.6</x:v>
+      </x:c>
+      <x:c r="F25" s="22" t="n">
+        <x:v>7106</x:v>
+      </x:c>
+      <x:c r="G25" s="22" t="n">
+        <x:v>7245.6</x:v>
+      </x:c>
+      <x:c r="H25" s="25" t="n">
+        <x:v>-208.6</x:v>
+      </x:c>
+      <x:c r="I25" s="23" t="n">
+        <x:v>-0.027984223659145102</x:v>
+      </x:c>
+      <x:c r="J25" s="27" t="n">
+        <x:f>ROUND(E25-F25,1)</x:f>
+        <x:v>381.6</x:v>
+      </x:c>
+      <x:c r="K25" s="21" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="21" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B26" s="21" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C26" s="21" t="str">
+        <x:v>7月31日</x:v>
+      </x:c>
+      <x:c r="D26" s="22" t="n">
+        <x:v>7514.8</x:v>
+      </x:c>
+      <x:c r="E26" s="22" t="n">
+        <x:v>7611.8</x:v>
+      </x:c>
+      <x:c r="F26" s="22" t="n">
+        <x:v>7389.6</x:v>
+      </x:c>
+      <x:c r="G26" s="22" t="n">
+        <x:v>7395</x:v>
+      </x:c>
+      <x:c r="H26" s="22" t="n">
+        <x:v>149.4</x:v>
+      </x:c>
+      <x:c r="I26" s="23" t="n">
+        <x:v>0.020619410400794846</x:v>
+      </x:c>
+      <x:c r="J26" s="27" t="n">
+        <x:f>ROUND(E26-F26,1)</x:f>
+        <x:v>222.2</x:v>
+      </x:c>
+      <x:c r="K26" s="21" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="38" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B23" s="39" t="n">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="C23" s="39"/>
-      <x:c r="D23" s="39"/>
-      <x:c r="E23" s="39"/>
-      <x:c r="F23" s="39"/>
-      <x:c r="G23" s="39"/>
-      <x:c r="H23" s="39"/>
-      <x:c r="I23" s="39"/>
-      <x:c r="J23" s="40" t="n">
-        <x:f>SUM(J4:J20)</x:f>
-        <x:v>4697.8</x:v>
-      </x:c>
-      <x:c r="K23" s="39"/>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="38" t="str">
+      <x:c r="B29" s="39" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="C29" s="39"/>
+      <x:c r="D29" s="39"/>
+      <x:c r="E29" s="39"/>
+      <x:c r="F29" s="39"/>
+      <x:c r="G29" s="39"/>
+      <x:c r="H29" s="39"/>
+      <x:c r="I29" s="39"/>
+      <x:c r="J29" s="40" t="n">
+        <x:f>SUM(J4:J26)</x:f>
+        <x:v>6264.2</x:v>
+      </x:c>
+      <x:c r="K29" s="39"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="38" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B24" s="39"/>
-      <x:c r="C24" s="39"/>
-      <x:c r="D24" s="39"/>
-      <x:c r="E24" s="39"/>
-      <x:c r="F24" s="39"/>
-      <x:c r="G24" s="39"/>
-      <x:c r="H24" s="39"/>
-      <x:c r="I24" s="39"/>
-      <x:c r="J24" s="42" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
-        <x:v>276.3</x:v>
-      </x:c>
-      <x:c r="K24" s="39"/>
+      <x:c r="B30" s="39"/>
+      <x:c r="C30" s="39"/>
+      <x:c r="D30" s="39"/>
+      <x:c r="E30" s="39"/>
+      <x:c r="F30" s="39"/>
+      <x:c r="G30" s="39"/>
+      <x:c r="H30" s="39"/>
+      <x:c r="I30" s="39"/>
+      <x:c r="J30" s="42" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J26),0),1)</x:f>
+        <x:v>272.4</x:v>
+      </x:c>
+      <x:c r="K30" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5066,43 +6146,259 @@
         <x:v>IF2609</x:v>
       </x:c>
     </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="21" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B21" s="21" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C21" s="21" t="str">
+        <x:v>7月24日</x:v>
+      </x:c>
+      <x:c r="D21" s="22" t="n">
+        <x:v>4623</x:v>
+      </x:c>
+      <x:c r="E21" s="22" t="n">
+        <x:v>4645</x:v>
+      </x:c>
+      <x:c r="F21" s="22" t="n">
+        <x:v>4576</x:v>
+      </x:c>
+      <x:c r="G21" s="22" t="n">
+        <x:v>4578.2</x:v>
+      </x:c>
+      <x:c r="H21" s="22" t="n">
+        <x:v>-83.2</x:v>
+      </x:c>
+      <x:c r="I21" s="23" t="n">
+        <x:v>-0.017848714978332625</x:v>
+      </x:c>
+      <x:c r="J21" s="22" t="n">
+        <x:f>ROUND(E21-F21,1)</x:f>
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="K21" s="21" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="21" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B22" s="21" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C22" s="21" t="str">
+        <x:v>7月27日</x:v>
+      </x:c>
+      <x:c r="D22" s="22" t="n">
+        <x:v>4589.4</x:v>
+      </x:c>
+      <x:c r="E22" s="22" t="n">
+        <x:v>4652.2</x:v>
+      </x:c>
+      <x:c r="F22" s="22" t="n">
+        <x:v>4572.2</x:v>
+      </x:c>
+      <x:c r="G22" s="22" t="n">
+        <x:v>4651.8</x:v>
+      </x:c>
+      <x:c r="H22" s="22" t="n">
+        <x:v>73.6</x:v>
+      </x:c>
+      <x:c r="I22" s="23" t="n">
+        <x:v>0.01607618714778747</x:v>
+      </x:c>
+      <x:c r="J22" s="22" t="n">
+        <x:f>ROUND(E22-F22,1)</x:f>
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="K22" s="21" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+    </x:row>
     <x:row r="23">
-      <x:c r="A23" s="38" t="str">
+      <x:c r="A23" s="21" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B23" s="21" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C23" s="21" t="str">
+        <x:v>7月28日</x:v>
+      </x:c>
+      <x:c r="D23" s="22" t="n">
+        <x:v>4589</x:v>
+      </x:c>
+      <x:c r="E23" s="22" t="n">
+        <x:v>4594</x:v>
+      </x:c>
+      <x:c r="F23" s="22" t="n">
+        <x:v>4488.2</x:v>
+      </x:c>
+      <x:c r="G23" s="22" t="n">
+        <x:v>4521</x:v>
+      </x:c>
+      <x:c r="H23" s="22" t="n">
+        <x:v>-130.8</x:v>
+      </x:c>
+      <x:c r="I23" s="23" t="n">
+        <x:v>-0.02811814781374955</x:v>
+      </x:c>
+      <x:c r="J23" s="27" t="n">
+        <x:f>ROUND(E23-F23,1)</x:f>
+        <x:v>105.8</x:v>
+      </x:c>
+      <x:c r="K23" s="21" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="21" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B24" s="21" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C24" s="21" t="str">
+        <x:v>7月29日</x:v>
+      </x:c>
+      <x:c r="D24" s="22" t="n">
+        <x:v>4529</x:v>
+      </x:c>
+      <x:c r="E24" s="22" t="n">
+        <x:v>4587.6</x:v>
+      </x:c>
+      <x:c r="F24" s="22" t="n">
+        <x:v>4473.6</x:v>
+      </x:c>
+      <x:c r="G24" s="22" t="n">
+        <x:v>4544.8</x:v>
+      </x:c>
+      <x:c r="H24" s="22" t="n">
+        <x:v>23.8</x:v>
+      </x:c>
+      <x:c r="I24" s="23" t="n">
+        <x:v>0.0052643220526431556</x:v>
+      </x:c>
+      <x:c r="J24" s="27" t="n">
+        <x:f>ROUND(E24-F24,1)</x:f>
+        <x:v>114</x:v>
+      </x:c>
+      <x:c r="K24" s="21" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="21" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B25" s="21" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C25" s="21" t="str">
+        <x:v>7月30日</x:v>
+      </x:c>
+      <x:c r="D25" s="22" t="n">
+        <x:v>4520</x:v>
+      </x:c>
+      <x:c r="E25" s="22" t="n">
+        <x:v>4555.4</x:v>
+      </x:c>
+      <x:c r="F25" s="22" t="n">
+        <x:v>4420</x:v>
+      </x:c>
+      <x:c r="G25" s="22" t="n">
+        <x:v>4508.2</x:v>
+      </x:c>
+      <x:c r="H25" s="22" t="n">
+        <x:v>-36.6</x:v>
+      </x:c>
+      <x:c r="I25" s="23" t="n">
+        <x:v>-0.008053159654990427</x:v>
+      </x:c>
+      <x:c r="J25" s="27" t="n">
+        <x:f>ROUND(E25-F25,1)</x:f>
+        <x:v>135.4</x:v>
+      </x:c>
+      <x:c r="K25" s="21" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="21" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B26" s="21" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C26" s="21" t="str">
+        <x:v>7月31日</x:v>
+      </x:c>
+      <x:c r="D26" s="22" t="n">
+        <x:v>4589.4</x:v>
+      </x:c>
+      <x:c r="E26" s="22" t="n">
+        <x:v>4619.4</x:v>
+      </x:c>
+      <x:c r="F26" s="22" t="n">
+        <x:v>4532.2</x:v>
+      </x:c>
+      <x:c r="G26" s="22" t="n">
+        <x:v>4538</x:v>
+      </x:c>
+      <x:c r="H26" s="22" t="n">
+        <x:v>29.8</x:v>
+      </x:c>
+      <x:c r="I26" s="23" t="n">
+        <x:v>0.0066101770107804825</x:v>
+      </x:c>
+      <x:c r="J26" s="22" t="n">
+        <x:f>ROUND(E26-F26,1)</x:f>
+        <x:v>87.2</x:v>
+      </x:c>
+      <x:c r="K26" s="21" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="38" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B23" s="39" t="n">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="C23" s="39"/>
-      <x:c r="D23" s="39"/>
-      <x:c r="E23" s="39"/>
-      <x:c r="F23" s="39"/>
-      <x:c r="G23" s="39"/>
-      <x:c r="H23" s="39"/>
-      <x:c r="I23" s="39"/>
-      <x:c r="J23" s="40" t="n">
-        <x:f>SUM(J4:J20)</x:f>
-        <x:v>1713</x:v>
-      </x:c>
-      <x:c r="K23" s="39"/>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="38" t="str">
+      <x:c r="B29" s="39" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="C29" s="39"/>
+      <x:c r="D29" s="39"/>
+      <x:c r="E29" s="39"/>
+      <x:c r="F29" s="39"/>
+      <x:c r="G29" s="39"/>
+      <x:c r="H29" s="39"/>
+      <x:c r="I29" s="39"/>
+      <x:c r="J29" s="40" t="n">
+        <x:f>SUM(J4:J26)</x:f>
+        <x:v>2304.4</x:v>
+      </x:c>
+      <x:c r="K29" s="39"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="38" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B24" s="39"/>
-      <x:c r="C24" s="39"/>
-      <x:c r="D24" s="39"/>
-      <x:c r="E24" s="39"/>
-      <x:c r="F24" s="39"/>
-      <x:c r="G24" s="39"/>
-      <x:c r="H24" s="39"/>
-      <x:c r="I24" s="39"/>
-      <x:c r="J24" s="42" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
-        <x:v>100.8</x:v>
-      </x:c>
-      <x:c r="K24" s="39"/>
+      <x:c r="B30" s="39"/>
+      <x:c r="C30" s="39"/>
+      <x:c r="D30" s="39"/>
+      <x:c r="E30" s="39"/>
+      <x:c r="F30" s="39"/>
+      <x:c r="G30" s="39"/>
+      <x:c r="H30" s="39"/>
+      <x:c r="I30" s="39"/>
+      <x:c r="J30" s="42" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J26),0),1)</x:f>
+        <x:v>100.2</x:v>
+      </x:c>
+      <x:c r="K30" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5781,43 +7077,259 @@
         <x:v>IH2609</x:v>
       </x:c>
     </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="21" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B21" s="21" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C21" s="21" t="str">
+        <x:v>7月24日</x:v>
+      </x:c>
+      <x:c r="D21" s="22" t="n">
+        <x:v>2945.8</x:v>
+      </x:c>
+      <x:c r="E21" s="22" t="n">
+        <x:v>2945.8</x:v>
+      </x:c>
+      <x:c r="F21" s="22" t="n">
+        <x:v>2908.4</x:v>
+      </x:c>
+      <x:c r="G21" s="22" t="n">
+        <x:v>2910</x:v>
+      </x:c>
+      <x:c r="H21" s="22" t="n">
+        <x:v>-38.8</x:v>
+      </x:c>
+      <x:c r="I21" s="23" t="n">
+        <x:v>-0.013157894736842146</x:v>
+      </x:c>
+      <x:c r="J21" s="22" t="n">
+        <x:f>ROUND(E21-F21,1)</x:f>
+        <x:v>37.4</x:v>
+      </x:c>
+      <x:c r="K21" s="21" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="21" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B22" s="21" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C22" s="21" t="str">
+        <x:v>7月27日</x:v>
+      </x:c>
+      <x:c r="D22" s="22" t="n">
+        <x:v>2929.6</x:v>
+      </x:c>
+      <x:c r="E22" s="22" t="n">
+        <x:v>2930</x:v>
+      </x:c>
+      <x:c r="F22" s="22" t="n">
+        <x:v>2889.8</x:v>
+      </x:c>
+      <x:c r="G22" s="22" t="n">
+        <x:v>2923</x:v>
+      </x:c>
+      <x:c r="H22" s="22" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="I22" s="23" t="n">
+        <x:v>0.0044673539518900185</x:v>
+      </x:c>
+      <x:c r="J22" s="22" t="n">
+        <x:f>ROUND(E22-F22,1)</x:f>
+        <x:v>40.2</x:v>
+      </x:c>
+      <x:c r="K22" s="21" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+    </x:row>
     <x:row r="23">
-      <x:c r="A23" s="38" t="str">
+      <x:c r="A23" s="21" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B23" s="21" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C23" s="21" t="str">
+        <x:v>7月28日</x:v>
+      </x:c>
+      <x:c r="D23" s="22" t="n">
+        <x:v>2894.6</x:v>
+      </x:c>
+      <x:c r="E23" s="22" t="n">
+        <x:v>2899.4</x:v>
+      </x:c>
+      <x:c r="F23" s="22" t="n">
+        <x:v>2855</x:v>
+      </x:c>
+      <x:c r="G23" s="22" t="n">
+        <x:v>2889.8</x:v>
+      </x:c>
+      <x:c r="H23" s="22" t="n">
+        <x:v>-33.2</x:v>
+      </x:c>
+      <x:c r="I23" s="23" t="n">
+        <x:v>-0.011358193636674563</x:v>
+      </x:c>
+      <x:c r="J23" s="22" t="n">
+        <x:f>ROUND(E23-F23,1)</x:f>
+        <x:v>44.4</x:v>
+      </x:c>
+      <x:c r="K23" s="21" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="21" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B24" s="21" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C24" s="21" t="str">
+        <x:v>7月29日</x:v>
+      </x:c>
+      <x:c r="D24" s="22" t="n">
+        <x:v>2896</x:v>
+      </x:c>
+      <x:c r="E24" s="22" t="n">
+        <x:v>2905.4</x:v>
+      </x:c>
+      <x:c r="F24" s="22" t="n">
+        <x:v>2856.6</x:v>
+      </x:c>
+      <x:c r="G24" s="22" t="n">
+        <x:v>2878.6</x:v>
+      </x:c>
+      <x:c r="H24" s="22" t="n">
+        <x:v>-11.2</x:v>
+      </x:c>
+      <x:c r="I24" s="23" t="n">
+        <x:v>-0.0038757007405357813</x:v>
+      </x:c>
+      <x:c r="J24" s="22" t="n">
+        <x:f>ROUND(E24-F24,1)</x:f>
+        <x:v>48.8</x:v>
+      </x:c>
+      <x:c r="K24" s="21" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="21" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B25" s="21" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C25" s="21" t="str">
+        <x:v>7月30日</x:v>
+      </x:c>
+      <x:c r="D25" s="22" t="n">
+        <x:v>2871</x:v>
+      </x:c>
+      <x:c r="E25" s="22" t="n">
+        <x:v>2901</x:v>
+      </x:c>
+      <x:c r="F25" s="22" t="n">
+        <x:v>2847.2</x:v>
+      </x:c>
+      <x:c r="G25" s="22" t="n">
+        <x:v>2885.8</x:v>
+      </x:c>
+      <x:c r="H25" s="22" t="n">
+        <x:v>7.2</x:v>
+      </x:c>
+      <x:c r="I25" s="23" t="n">
+        <x:v>0.002501215868825124</x:v>
+      </x:c>
+      <x:c r="J25" s="22" t="n">
+        <x:f>ROUND(E25-F25,1)</x:f>
+        <x:v>53.8</x:v>
+      </x:c>
+      <x:c r="K25" s="21" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="21" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B26" s="21" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C26" s="21" t="str">
+        <x:v>7月31日</x:v>
+      </x:c>
+      <x:c r="D26" s="22" t="n">
+        <x:v>2910</x:v>
+      </x:c>
+      <x:c r="E26" s="22" t="n">
+        <x:v>2927</x:v>
+      </x:c>
+      <x:c r="F26" s="22" t="n">
+        <x:v>2886.4</x:v>
+      </x:c>
+      <x:c r="G26" s="22" t="n">
+        <x:v>2891.8</x:v>
+      </x:c>
+      <x:c r="H26" s="22" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="I26" s="23" t="n">
+        <x:v>0.0020791461639753095</x:v>
+      </x:c>
+      <x:c r="J26" s="22" t="n">
+        <x:f>ROUND(E26-F26,1)</x:f>
+        <x:v>40.6</x:v>
+      </x:c>
+      <x:c r="K26" s="21" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="38" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B23" s="39" t="n">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="C23" s="39"/>
-      <x:c r="D23" s="39"/>
-      <x:c r="E23" s="39"/>
-      <x:c r="F23" s="39"/>
-      <x:c r="G23" s="39"/>
-      <x:c r="H23" s="39"/>
-      <x:c r="I23" s="39"/>
-      <x:c r="J23" s="40" t="n">
-        <x:f>SUM(J4:J20)</x:f>
-        <x:v>956.4</x:v>
-      </x:c>
-      <x:c r="K23" s="39"/>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="38" t="str">
+      <x:c r="B29" s="39" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="C29" s="39"/>
+      <x:c r="D29" s="39"/>
+      <x:c r="E29" s="39"/>
+      <x:c r="F29" s="39"/>
+      <x:c r="G29" s="39"/>
+      <x:c r="H29" s="39"/>
+      <x:c r="I29" s="39"/>
+      <x:c r="J29" s="40" t="n">
+        <x:f>SUM(J4:J26)</x:f>
+        <x:v>1221.6</x:v>
+      </x:c>
+      <x:c r="K29" s="39"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="38" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B24" s="39"/>
-      <x:c r="C24" s="39"/>
-      <x:c r="D24" s="39"/>
-      <x:c r="E24" s="39"/>
-      <x:c r="F24" s="39"/>
-      <x:c r="G24" s="39"/>
-      <x:c r="H24" s="39"/>
-      <x:c r="I24" s="39"/>
-      <x:c r="J24" s="42" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
-        <x:v>56.3</x:v>
-      </x:c>
-      <x:c r="K24" s="39"/>
+      <x:c r="B30" s="39"/>
+      <x:c r="C30" s="39"/>
+      <x:c r="D30" s="39"/>
+      <x:c r="E30" s="39"/>
+      <x:c r="F30" s="39"/>
+      <x:c r="G30" s="39"/>
+      <x:c r="H30" s="39"/>
+      <x:c r="I30" s="39"/>
+      <x:c r="J30" s="42" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J26),0),1)</x:f>
+        <x:v>53.1</x:v>
+      </x:c>
+      <x:c r="K30" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-08-03
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R7637537ca1584f80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R197dbeb25c394002"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R6e7345ff714741ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R96eca8515006405c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R125fbfec7e1f4135"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R83a0c2406bbb4657"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Rd6e1f6f5325842ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rda4d290680b34a22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R54052f26d0fb4445"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rb76d4c0392c04dc9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R08e28ae3c6fb4a50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R04779d4a50e84a9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R18f2e8da11f24c66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Rc7aaa2ef17f84940"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R2bf40d6f6520433f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R1d589fb80e244d16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rabfffc7e0d494d59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R24509e4f66ee485d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -133,7 +133,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="36">
+  <x:cellXfs count="35">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -197,9 +197,6 @@
       <x:alignment horizontal="center"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -550,17 +547,27 @@
       <x:c r="A7" s="9" t="str">
         <x:v>IM主力</x:v>
       </x:c>
-      <x:c r="B7" s="9" t="str"/>
-      <x:c r="C7" s="10" t="str"/>
-      <x:c r="D7" s="10" t="str"/>
-      <x:c r="E7" s="12" t="str"/>
+      <x:c r="B7" s="9" t="str">
+        <x:v>2026-08-03</x:v>
+      </x:c>
+      <x:c r="C7" s="10" t="n">
+        <x:v>7064.2</x:v>
+      </x:c>
+      <x:c r="D7" s="10" t="n">
+        <x:v>6976</x:v>
+      </x:c>
+      <x:c r="E7" s="12" t="n">
+        <x:v>88.2</x:v>
+      </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H7" s="10" t="str"/>
+        <x:v>88.2</x:v>
+      </x:c>
+      <x:c r="H7" s="10" t="n">
+        <x:v>88.2</x:v>
+      </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
       </x:c>
@@ -1205,379 +1212,434 @@
       </x:c>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="31" t="str">
-        <x:v>暂无数据</x:v>
-      </x:c>
-      <x:c r="B23" s="31"/>
-      <x:c r="C23" s="31"/>
-      <x:c r="D23" s="31"/>
-      <x:c r="E23" s="31"/>
-      <x:c r="F23" s="31"/>
-      <x:c r="G23" s="31"/>
-      <x:c r="H23" s="31"/>
-      <x:c r="I23" s="31"/>
-      <x:c r="J23" s="31"/>
-      <x:c r="K23" s="31"/>
+      <x:c r="A23" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B23" s="22" t="str">
+        <x:v>8月3日</x:v>
+      </x:c>
+      <x:c r="C23" s="23" t="n">
+        <x:v>7000</x:v>
+      </x:c>
+      <x:c r="D23" s="23" t="n">
+        <x:v>7064.2</x:v>
+      </x:c>
+      <x:c r="E23" s="23" t="n">
+        <x:v>6976</x:v>
+      </x:c>
+      <x:c r="F23" s="23" t="n">
+        <x:v>7023.4</x:v>
+      </x:c>
+      <x:c r="G23" s="23"/>
+      <x:c r="H23" s="24"/>
+      <x:c r="I23" s="23" t="n">
+        <x:f>ROUND(D23-E23,1)</x:f>
+        <x:v>88.2</x:v>
+      </x:c>
+      <x:c r="J23" s="22" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+      <x:c r="K23" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="27" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B24" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C24" s="26"/>
+      <x:c r="D24" s="26"/>
+      <x:c r="E24" s="26"/>
+      <x:c r="F24" s="26"/>
+      <x:c r="G24" s="26"/>
+      <x:c r="H24" s="26"/>
+      <x:c r="I24" s="28" t="n">
+        <x:f>ROUND(SUM(I23:I23),1)</x:f>
+        <x:v>88.2</x:v>
+      </x:c>
+      <x:c r="J24" s="26"/>
+      <x:c r="K24" s="26"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="17" t="str">
+      <x:c r="A25" s="27" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B25" s="26"/>
+      <x:c r="C25" s="26"/>
+      <x:c r="D25" s="26"/>
+      <x:c r="E25" s="26"/>
+      <x:c r="F25" s="26"/>
+      <x:c r="G25" s="26"/>
+      <x:c r="H25" s="26"/>
+      <x:c r="I25" s="30" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I23:I23),0),1)</x:f>
+        <x:v>88.2</x:v>
+      </x:c>
+      <x:c r="J25" s="26"/>
+      <x:c r="K25" s="26"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="17" t="str">
         <x:v>IC主力</x:v>
       </x:c>
-      <x:c r="B25" s="17"/>
-      <x:c r="C25" s="17"/>
-      <x:c r="D25" s="17"/>
-      <x:c r="E25" s="17"/>
-      <x:c r="F25" s="17"/>
-      <x:c r="G25" s="17"/>
-      <x:c r="H25" s="17"/>
-      <x:c r="I25" s="17"/>
-      <x:c r="J25" s="17"/>
-      <x:c r="K25" s="17"/>
-    </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="20" t="str">
+      <x:c r="B27" s="17"/>
+      <x:c r="C27" s="17"/>
+      <x:c r="D27" s="17"/>
+      <x:c r="E27" s="17"/>
+      <x:c r="F27" s="17"/>
+      <x:c r="G27" s="17"/>
+      <x:c r="H27" s="17"/>
+      <x:c r="I27" s="17"/>
+      <x:c r="J27" s="17"/>
+      <x:c r="K27" s="17"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B26" s="20" t="str">
+      <x:c r="B28" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C26" s="20" t="str">
+      <x:c r="C28" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D26" s="20" t="str">
+      <x:c r="D28" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E26" s="20" t="str">
+      <x:c r="E28" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F26" s="20" t="str">
+      <x:c r="F28" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G26" s="20" t="str">
+      <x:c r="G28" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H26" s="20" t="str">
+      <x:c r="H28" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I26" s="20" t="str">
+      <x:c r="I28" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J26" s="20" t="str">
+      <x:c r="J28" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K26" s="20" t="str">
+      <x:c r="K28" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B27" s="22" t="str">
+    <x:row r="29">
+      <x:c r="A29" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B29" s="22" t="str">
         <x:v>8月3日</x:v>
       </x:c>
-      <x:c r="C27" s="23" t="n">
+      <x:c r="C29" s="23" t="n">
         <x:v>7391</x:v>
       </x:c>
-      <x:c r="D27" s="23" t="n">
+      <x:c r="D29" s="23" t="n">
         <x:v>7440</x:v>
       </x:c>
-      <x:c r="E27" s="23" t="n">
+      <x:c r="E29" s="23" t="n">
         <x:v>7335</x:v>
       </x:c>
-      <x:c r="F27" s="23" t="n">
+      <x:c r="F29" s="23" t="n">
         <x:v>7356</x:v>
       </x:c>
-      <x:c r="G27" s="23"/>
-      <x:c r="H27" s="24"/>
-      <x:c r="I27" s="23" t="n">
-        <x:f>ROUND(D27-E27,1)</x:f>
+      <x:c r="G29" s="23"/>
+      <x:c r="H29" s="24"/>
+      <x:c r="I29" s="23" t="n">
+        <x:f>ROUND(D29-E29,1)</x:f>
         <x:v>105</x:v>
       </x:c>
-      <x:c r="J27" s="22" t="str">
+      <x:c r="J29" s="22" t="str">
         <x:v>IC2609</x:v>
       </x:c>
-      <x:c r="K27" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28">
-      <x:c r="A28" s="27" t="str">
+      <x:c r="K29" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="27" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B28" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C28" s="26"/>
-      <x:c r="D28" s="26"/>
-      <x:c r="E28" s="26"/>
-      <x:c r="F28" s="26"/>
-      <x:c r="G28" s="26"/>
-      <x:c r="H28" s="26"/>
-      <x:c r="I28" s="28" t="n">
-        <x:f>ROUND(SUM(I27:I27),1)</x:f>
+      <x:c r="B30" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C30" s="26"/>
+      <x:c r="D30" s="26"/>
+      <x:c r="E30" s="26"/>
+      <x:c r="F30" s="26"/>
+      <x:c r="G30" s="26"/>
+      <x:c r="H30" s="26"/>
+      <x:c r="I30" s="28" t="n">
+        <x:f>ROUND(SUM(I29:I29),1)</x:f>
         <x:v>105</x:v>
       </x:c>
-      <x:c r="J28" s="26"/>
-      <x:c r="K28" s="26"/>
-    </x:row>
-    <x:row r="29">
-      <x:c r="A29" s="27" t="str">
+      <x:c r="J30" s="26"/>
+      <x:c r="K30" s="26"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="27" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B29" s="26"/>
-      <x:c r="C29" s="26"/>
-      <x:c r="D29" s="26"/>
-      <x:c r="E29" s="26"/>
-      <x:c r="F29" s="26"/>
-      <x:c r="G29" s="26"/>
-      <x:c r="H29" s="26"/>
-      <x:c r="I29" s="30" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I27:I27),0),1)</x:f>
+      <x:c r="B31" s="26"/>
+      <x:c r="C31" s="26"/>
+      <x:c r="D31" s="26"/>
+      <x:c r="E31" s="26"/>
+      <x:c r="F31" s="26"/>
+      <x:c r="G31" s="26"/>
+      <x:c r="H31" s="26"/>
+      <x:c r="I31" s="30" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I29:I29),0),1)</x:f>
         <x:v>105</x:v>
       </x:c>
-      <x:c r="J29" s="26"/>
-      <x:c r="K29" s="26"/>
-    </x:row>
-    <x:row r="31">
-      <x:c r="A31" s="17" t="str">
+      <x:c r="J31" s="26"/>
+      <x:c r="K31" s="26"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="17" t="str">
         <x:v>IF主力</x:v>
       </x:c>
-      <x:c r="B31" s="17"/>
-      <x:c r="C31" s="17"/>
-      <x:c r="D31" s="17"/>
-      <x:c r="E31" s="17"/>
-      <x:c r="F31" s="17"/>
-      <x:c r="G31" s="17"/>
-      <x:c r="H31" s="17"/>
-      <x:c r="I31" s="17"/>
-      <x:c r="J31" s="17"/>
-      <x:c r="K31" s="17"/>
-    </x:row>
-    <x:row r="32">
-      <x:c r="A32" s="20" t="str">
+      <x:c r="B33" s="17"/>
+      <x:c r="C33" s="17"/>
+      <x:c r="D33" s="17"/>
+      <x:c r="E33" s="17"/>
+      <x:c r="F33" s="17"/>
+      <x:c r="G33" s="17"/>
+      <x:c r="H33" s="17"/>
+      <x:c r="I33" s="17"/>
+      <x:c r="J33" s="17"/>
+      <x:c r="K33" s="17"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B32" s="20" t="str">
+      <x:c r="B34" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C32" s="20" t="str">
+      <x:c r="C34" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D32" s="20" t="str">
+      <x:c r="D34" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E32" s="20" t="str">
+      <x:c r="E34" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F32" s="20" t="str">
+      <x:c r="F34" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G32" s="20" t="str">
+      <x:c r="G34" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H32" s="20" t="str">
+      <x:c r="H34" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I32" s="20" t="str">
+      <x:c r="I34" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J32" s="20" t="str">
+      <x:c r="J34" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K32" s="20" t="str">
+      <x:c r="K34" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="33">
-      <x:c r="A33" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B33" s="22" t="str">
+    <x:row r="35">
+      <x:c r="A35" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B35" s="22" t="str">
         <x:v>8月3日</x:v>
       </x:c>
-      <x:c r="C33" s="23" t="n">
+      <x:c r="C35" s="23" t="n">
         <x:v>4526.4</x:v>
       </x:c>
-      <x:c r="D33" s="23" t="n">
+      <x:c r="D35" s="23" t="n">
         <x:v>4538</x:v>
       </x:c>
-      <x:c r="E33" s="23" t="n">
+      <x:c r="E35" s="23" t="n">
         <x:v>4494.2</x:v>
       </x:c>
-      <x:c r="F33" s="23" t="n">
+      <x:c r="F35" s="23" t="n">
         <x:v>4512.2</x:v>
       </x:c>
-      <x:c r="G33" s="23"/>
-      <x:c r="H33" s="24"/>
-      <x:c r="I33" s="23" t="n">
-        <x:f>ROUND(D33-E33,1)</x:f>
+      <x:c r="G35" s="23"/>
+      <x:c r="H35" s="24"/>
+      <x:c r="I35" s="23" t="n">
+        <x:f>ROUND(D35-E35,1)</x:f>
         <x:v>43.8</x:v>
       </x:c>
-      <x:c r="J33" s="22" t="str">
+      <x:c r="J35" s="22" t="str">
         <x:v>IF2609</x:v>
       </x:c>
-      <x:c r="K33" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34">
-      <x:c r="A34" s="27" t="str">
+      <x:c r="K35" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="27" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B34" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C34" s="26"/>
-      <x:c r="D34" s="26"/>
-      <x:c r="E34" s="26"/>
-      <x:c r="F34" s="26"/>
-      <x:c r="G34" s="26"/>
-      <x:c r="H34" s="26"/>
-      <x:c r="I34" s="28" t="n">
-        <x:f>ROUND(SUM(I33:I33),1)</x:f>
+      <x:c r="B36" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C36" s="26"/>
+      <x:c r="D36" s="26"/>
+      <x:c r="E36" s="26"/>
+      <x:c r="F36" s="26"/>
+      <x:c r="G36" s="26"/>
+      <x:c r="H36" s="26"/>
+      <x:c r="I36" s="28" t="n">
+        <x:f>ROUND(SUM(I35:I35),1)</x:f>
         <x:v>43.8</x:v>
       </x:c>
-      <x:c r="J34" s="26"/>
-      <x:c r="K34" s="26"/>
-    </x:row>
-    <x:row r="35">
-      <x:c r="A35" s="27" t="str">
+      <x:c r="J36" s="26"/>
+      <x:c r="K36" s="26"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="27" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B35" s="26"/>
-      <x:c r="C35" s="26"/>
-      <x:c r="D35" s="26"/>
-      <x:c r="E35" s="26"/>
-      <x:c r="F35" s="26"/>
-      <x:c r="G35" s="26"/>
-      <x:c r="H35" s="26"/>
-      <x:c r="I35" s="30" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I33:I33),0),1)</x:f>
+      <x:c r="B37" s="26"/>
+      <x:c r="C37" s="26"/>
+      <x:c r="D37" s="26"/>
+      <x:c r="E37" s="26"/>
+      <x:c r="F37" s="26"/>
+      <x:c r="G37" s="26"/>
+      <x:c r="H37" s="26"/>
+      <x:c r="I37" s="30" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I35:I35),0),1)</x:f>
         <x:v>43.8</x:v>
       </x:c>
-      <x:c r="J35" s="26"/>
-      <x:c r="K35" s="26"/>
-    </x:row>
-    <x:row r="37">
-      <x:c r="A37" s="17" t="str">
+      <x:c r="J37" s="26"/>
+      <x:c r="K37" s="26"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="17" t="str">
         <x:v>IH主力</x:v>
       </x:c>
-      <x:c r="B37" s="17"/>
-      <x:c r="C37" s="17"/>
-      <x:c r="D37" s="17"/>
-      <x:c r="E37" s="17"/>
-      <x:c r="F37" s="17"/>
-      <x:c r="G37" s="17"/>
-      <x:c r="H37" s="17"/>
-      <x:c r="I37" s="17"/>
-      <x:c r="J37" s="17"/>
-      <x:c r="K37" s="17"/>
-    </x:row>
-    <x:row r="38">
-      <x:c r="A38" s="20" t="str">
+      <x:c r="B39" s="17"/>
+      <x:c r="C39" s="17"/>
+      <x:c r="D39" s="17"/>
+      <x:c r="E39" s="17"/>
+      <x:c r="F39" s="17"/>
+      <x:c r="G39" s="17"/>
+      <x:c r="H39" s="17"/>
+      <x:c r="I39" s="17"/>
+      <x:c r="J39" s="17"/>
+      <x:c r="K39" s="17"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B38" s="20" t="str">
+      <x:c r="B40" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C38" s="20" t="str">
+      <x:c r="C40" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D38" s="20" t="str">
+      <x:c r="D40" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E38" s="20" t="str">
+      <x:c r="E40" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F38" s="20" t="str">
+      <x:c r="F40" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G38" s="20" t="str">
+      <x:c r="G40" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H38" s="20" t="str">
+      <x:c r="H40" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I38" s="20" t="str">
+      <x:c r="I40" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J38" s="20" t="str">
+      <x:c r="J40" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K38" s="20" t="str">
+      <x:c r="K40" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="39">
-      <x:c r="A39" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B39" s="22" t="str">
+    <x:row r="41">
+      <x:c r="A41" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B41" s="22" t="str">
         <x:v>8月3日</x:v>
       </x:c>
-      <x:c r="C39" s="23" t="n">
+      <x:c r="C41" s="23" t="n">
         <x:v>2882.4</x:v>
       </x:c>
-      <x:c r="D39" s="23" t="n">
+      <x:c r="D41" s="23" t="n">
         <x:v>2890</x:v>
       </x:c>
-      <x:c r="E39" s="23" t="n">
+      <x:c r="E41" s="23" t="n">
         <x:v>2845.8</x:v>
       </x:c>
-      <x:c r="F39" s="23" t="n">
+      <x:c r="F41" s="23" t="n">
         <x:v>2860</x:v>
       </x:c>
-      <x:c r="G39" s="23"/>
-      <x:c r="H39" s="24"/>
-      <x:c r="I39" s="23" t="n">
-        <x:f>ROUND(D39-E39,1)</x:f>
+      <x:c r="G41" s="23"/>
+      <x:c r="H41" s="24"/>
+      <x:c r="I41" s="23" t="n">
+        <x:f>ROUND(D41-E41,1)</x:f>
         <x:v>44.2</x:v>
       </x:c>
-      <x:c r="J39" s="22" t="str">
+      <x:c r="J41" s="22" t="str">
         <x:v>IH2609</x:v>
       </x:c>
-      <x:c r="K39" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40">
-      <x:c r="A40" s="27" t="str">
+      <x:c r="K41" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="27" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B40" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C40" s="26"/>
-      <x:c r="D40" s="26"/>
-      <x:c r="E40" s="26"/>
-      <x:c r="F40" s="26"/>
-      <x:c r="G40" s="26"/>
-      <x:c r="H40" s="26"/>
-      <x:c r="I40" s="28" t="n">
-        <x:f>ROUND(SUM(I39:I39),1)</x:f>
+      <x:c r="B42" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C42" s="26"/>
+      <x:c r="D42" s="26"/>
+      <x:c r="E42" s="26"/>
+      <x:c r="F42" s="26"/>
+      <x:c r="G42" s="26"/>
+      <x:c r="H42" s="26"/>
+      <x:c r="I42" s="28" t="n">
+        <x:f>ROUND(SUM(I41:I41),1)</x:f>
         <x:v>44.2</x:v>
       </x:c>
-      <x:c r="J40" s="26"/>
-      <x:c r="K40" s="26"/>
-    </x:row>
-    <x:row r="41">
-      <x:c r="A41" s="27" t="str">
+      <x:c r="J42" s="26"/>
+      <x:c r="K42" s="26"/>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="27" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B41" s="26"/>
-      <x:c r="C41" s="26"/>
-      <x:c r="D41" s="26"/>
-      <x:c r="E41" s="26"/>
-      <x:c r="F41" s="26"/>
-      <x:c r="G41" s="26"/>
-      <x:c r="H41" s="26"/>
-      <x:c r="I41" s="30" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I39:I39),0),1)</x:f>
+      <x:c r="B43" s="26"/>
+      <x:c r="C43" s="26"/>
+      <x:c r="D43" s="26"/>
+      <x:c r="E43" s="26"/>
+      <x:c r="F43" s="26"/>
+      <x:c r="G43" s="26"/>
+      <x:c r="H43" s="26"/>
+      <x:c r="I43" s="30" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I41:I41),0),1)</x:f>
         <x:v>44.2</x:v>
       </x:c>
-      <x:c r="J41" s="26"/>
-      <x:c r="K41" s="26"/>
+      <x:c r="J43" s="26"/>
+      <x:c r="K43" s="26"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1586,10 +1648,9 @@
     <x:mergeCell ref="A9:K9"/>
     <x:mergeCell ref="A15:K15"/>
     <x:mergeCell ref="A21:K21"/>
-    <x:mergeCell ref="A23:K23"/>
-    <x:mergeCell ref="A25:K25"/>
-    <x:mergeCell ref="A31:K31"/>
-    <x:mergeCell ref="A37:K37"/>
+    <x:mergeCell ref="A27:K27"/>
+    <x:mergeCell ref="A33:K33"/>
+    <x:mergeCell ref="A39:K39"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2070,24 +2131,47 @@
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="22"/>
-      <x:c r="B4" s="22"/>
-      <x:c r="C4" s="22"/>
-      <x:c r="D4" s="23"/>
-      <x:c r="E4" s="23"/>
-      <x:c r="F4" s="23"/>
-      <x:c r="G4" s="23"/>
-      <x:c r="H4" s="23"/>
-      <x:c r="I4" s="24"/>
-      <x:c r="J4" s="23"/>
-      <x:c r="K4" s="22"/>
+      <x:c r="A4" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B4" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C4" s="22" t="str">
+        <x:v>8月3日</x:v>
+      </x:c>
+      <x:c r="D4" s="23" t="n">
+        <x:v>7000</x:v>
+      </x:c>
+      <x:c r="E4" s="23" t="n">
+        <x:v>7064.2</x:v>
+      </x:c>
+      <x:c r="F4" s="23" t="n">
+        <x:v>6976</x:v>
+      </x:c>
+      <x:c r="G4" s="23" t="n">
+        <x:v>7023.4</x:v>
+      </x:c>
+      <x:c r="H4" s="23" t="n">
+        <x:v>35.6</x:v>
+      </x:c>
+      <x:c r="I4" s="24" t="n">
+        <x:v>0.005094593434270989</x:v>
+      </x:c>
+      <x:c r="J4" s="23" t="n">
+        <x:f>ROUND(E4-F4,1)</x:f>
+        <x:v>88.2</x:v>
+      </x:c>
+      <x:c r="K4" s="22" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="27" t="str">
         <x:v>合计</x:v>
       </x:c>
       <x:c r="B7" s="26" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C7" s="26"/>
       <x:c r="D7" s="26"/>
@@ -2098,7 +2182,7 @@
       <x:c r="I7" s="26"/>
       <x:c r="J7" s="28" t="n">
         <x:f>SUM(J4:J4)</x:f>
-        <x:v>0</x:v>
+        <x:v>88.2</x:v>
       </x:c>
       <x:c r="K7" s="26"/>
     </x:row>
@@ -2116,7 +2200,7 @@
       <x:c r="I8" s="26"/>
       <x:c r="J8" s="30" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J4),0),1)</x:f>
-        <x:v>0</x:v>
+        <x:v>88.2</x:v>
       </x:c>
       <x:c r="K8" s="26"/>
     </x:row>

</xml_diff>

<commit_message>
Update amplitude website 2026-08-04
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rb76d4c0392c04dc9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R08e28ae3c6fb4a50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R04779d4a50e84a9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R18f2e8da11f24c66"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Rc7aaa2ef17f84940"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R2bf40d6f6520433f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R1d589fb80e244d16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rabfffc7e0d494d59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R24509e4f66ee485d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Re6f9db915ca84abf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R949830abaa5e4bbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R4ca2be52f1f346a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rbbe73bca31d04fd1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Rc1aa42fc62bd4fe3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R90ac848b832b410c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Rc25682c705d24c55"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Re3355a1891274c35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rb2be9439dff54bed"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25,7 +25,7 @@
     <x:numFmt numFmtId="200" formatCode="General"/>
     <x:numFmt numFmtId="201" formatCode="0.0%"/>
   </x:numFmts>
-  <x:fonts count="8">
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -70,8 +70,14 @@
       <x:color rgb="FFE11D48"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF1D4ED8"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -96,6 +102,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFFF00"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFBFDBFE"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -133,7 +144,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="35">
+  <x:cellXfs count="39">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -183,6 +194,12 @@
     <x:xf numFmtId="201" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="7" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
@@ -207,6 +224,12 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="8" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
@@ -461,25 +484,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-08-03</x:v>
+        <x:v>2026-08-04</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7118.1</x:v>
+        <x:v>7307.17</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7042.89</x:v>
+        <x:v>7102.46</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>75.2</x:v>
+        <x:v>204.7</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>75.2</x:v>
+        <x:v>279.9</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>75.2</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -490,25 +513,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-08-03</x:v>
+        <x:v>2026-08-04</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7499.58</x:v>
+        <x:v>7645.48</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7397.94</x:v>
+        <x:v>7450.32</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>101.6</x:v>
+        <x:v>195.2</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>101.6</x:v>
+        <x:v>296.8</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>101.6</x:v>
+        <x:v>148.4</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -519,25 +542,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-08-03</x:v>
+        <x:v>2026-08-04</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3827.64</x:v>
+        <x:v>3831.94</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3797.64</x:v>
+        <x:v>3799.52</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>30</x:v>
+        <x:v>32.4</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>30</x:v>
+        <x:v>62.4</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>30</x:v>
+        <x:v>31.2</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -548,25 +571,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-08-03</x:v>
+        <x:v>2026-08-04</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>7064.2</x:v>
+        <x:v>7269.8</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>6976</x:v>
+        <x:v>7057.8</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>88.2</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>88.2</x:v>
+        <x:v>300.2</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>88.2</x:v>
+        <x:v>150.1</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -577,25 +600,25 @@
         <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>2026-08-03</x:v>
+        <x:v>2026-08-04</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:v>7440</x:v>
+        <x:v>7599</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>7335</x:v>
+        <x:v>7392.8</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>105</x:v>
+        <x:v>206.2</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>105</x:v>
+        <x:v>311.2</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
-        <x:v>105</x:v>
+        <x:v>155.6</x:v>
       </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
@@ -606,25 +629,25 @@
         <x:v>IF主力</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>2026-08-03</x:v>
+        <x:v>2026-08-04</x:v>
       </x:c>
       <x:c r="C9" s="10" t="n">
-        <x:v>4538</x:v>
+        <x:v>4580.8</x:v>
       </x:c>
       <x:c r="D9" s="10" t="n">
-        <x:v>4494.2</x:v>
+        <x:v>4524.2</x:v>
       </x:c>
       <x:c r="E9" s="12" t="n">
-        <x:v>43.8</x:v>
+        <x:v>56.6</x:v>
       </x:c>
       <x:c r="F9" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G9" s="10" t="n">
-        <x:v>43.8</x:v>
+        <x:v>100.4</x:v>
       </x:c>
       <x:c r="H9" s="10" t="n">
-        <x:v>43.8</x:v>
+        <x:v>50.2</x:v>
       </x:c>
       <x:c r="I9" s="10" t="n">
         <x:v>90</x:v>
@@ -635,25 +658,25 @@
         <x:v>IH主力</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>2026-08-03</x:v>
+        <x:v>2026-08-04</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:v>2890</x:v>
+        <x:v>2872</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
-        <x:v>2845.8</x:v>
+        <x:v>2846.6</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
-        <x:v>44.2</x:v>
+        <x:v>25.4</x:v>
       </x:c>
       <x:c r="F10" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G10" s="10" t="n">
-        <x:v>44.2</x:v>
+        <x:v>69.6</x:v>
       </x:c>
       <x:c r="H10" s="10" t="n">
-        <x:v>44.2</x:v>
+        <x:v>34.8</x:v>
       </x:c>
       <x:c r="I10" s="10" t="n">
         <x:v>60</x:v>
@@ -667,7 +690,7 @@
         <x:v>2026-08-01</x:v>
       </x:c>
       <x:c r="C13" s="14" t="str">
-        <x:v>2026-08-03</x:v>
+        <x:v>2026-08-04</x:v>
       </x:c>
       <x:c r="D13" s="14" t="str">
         <x:v>数据源</x:v>
@@ -856,70 +879,70 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B5" s="22" t="str">
-        <x:v>8月3日</x:v>
+        <x:v>8月3日-8月4日</x:v>
       </x:c>
       <x:c r="C5" s="23" t="n">
         <x:v>7055.27</x:v>
       </x:c>
       <x:c r="D5" s="23" t="n">
-        <x:v>7118.1</x:v>
+        <x:v>7307.17</x:v>
       </x:c>
       <x:c r="E5" s="23" t="n">
         <x:v>7042.89</x:v>
       </x:c>
       <x:c r="F5" s="23" t="n">
-        <x:v>7079.78</x:v>
+        <x:v>7279.19</x:v>
       </x:c>
       <x:c r="G5" s="23"/>
       <x:c r="H5" s="24"/>
-      <x:c r="I5" s="23" t="n">
+      <x:c r="I5" s="26" t="n">
         <x:f>ROUND(D5-E5,1)</x:f>
-        <x:v>75.2</x:v>
+        <x:v>264.3</x:v>
       </x:c>
       <x:c r="J5" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K5" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="29" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B6" s="28" t="n">
         <x:v>1</x:v>
       </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="27" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B6" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C6" s="26"/>
-      <x:c r="D6" s="26"/>
-      <x:c r="E6" s="26"/>
-      <x:c r="F6" s="26"/>
-      <x:c r="G6" s="26"/>
-      <x:c r="H6" s="26"/>
-      <x:c r="I6" s="28" t="n">
+      <x:c r="C6" s="28"/>
+      <x:c r="D6" s="28"/>
+      <x:c r="E6" s="28"/>
+      <x:c r="F6" s="28"/>
+      <x:c r="G6" s="28"/>
+      <x:c r="H6" s="28"/>
+      <x:c r="I6" s="30" t="n">
         <x:f>ROUND(SUM(I5:I5),1)</x:f>
-        <x:v>75.2</x:v>
-      </x:c>
-      <x:c r="J6" s="26"/>
-      <x:c r="K6" s="26"/>
+        <x:v>264.3</x:v>
+      </x:c>
+      <x:c r="J6" s="28"/>
+      <x:c r="K6" s="28"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="27" t="str">
+      <x:c r="A7" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B7" s="26"/>
-      <x:c r="C7" s="26"/>
-      <x:c r="D7" s="26"/>
-      <x:c r="E7" s="26"/>
-      <x:c r="F7" s="26"/>
-      <x:c r="G7" s="26"/>
-      <x:c r="H7" s="26"/>
-      <x:c r="I7" s="30" t="n">
+      <x:c r="B7" s="28"/>
+      <x:c r="C7" s="28"/>
+      <x:c r="D7" s="28"/>
+      <x:c r="E7" s="28"/>
+      <x:c r="F7" s="28"/>
+      <x:c r="G7" s="28"/>
+      <x:c r="H7" s="28"/>
+      <x:c r="I7" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I5),0),1)</x:f>
-        <x:v>75.2</x:v>
-      </x:c>
-      <x:c r="J7" s="26"/>
-      <x:c r="K7" s="26"/>
+        <x:v>264.3</x:v>
+      </x:c>
+      <x:c r="J7" s="28"/>
+      <x:c r="K7" s="28"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="17" t="str">
@@ -976,70 +999,70 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B11" s="22" t="str">
-        <x:v>8月3日</x:v>
+        <x:v>8月3日-8月4日</x:v>
       </x:c>
       <x:c r="C11" s="23" t="n">
         <x:v>7457.12</x:v>
       </x:c>
       <x:c r="D11" s="23" t="n">
-        <x:v>7499.58</x:v>
+        <x:v>7645.48</x:v>
       </x:c>
       <x:c r="E11" s="23" t="n">
         <x:v>7397.94</x:v>
       </x:c>
       <x:c r="F11" s="23" t="n">
-        <x:v>7414.52</x:v>
+        <x:v>7607.49</x:v>
       </x:c>
       <x:c r="G11" s="23"/>
       <x:c r="H11" s="24"/>
-      <x:c r="I11" s="23" t="n">
+      <x:c r="I11" s="26" t="n">
         <x:f>ROUND(D11-E11,1)</x:f>
-        <x:v>101.6</x:v>
+        <x:v>247.5</x:v>
       </x:c>
       <x:c r="J11" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K11" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="29" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B12" s="28" t="n">
         <x:v>1</x:v>
       </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="27" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B12" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C12" s="26"/>
-      <x:c r="D12" s="26"/>
-      <x:c r="E12" s="26"/>
-      <x:c r="F12" s="26"/>
-      <x:c r="G12" s="26"/>
-      <x:c r="H12" s="26"/>
-      <x:c r="I12" s="28" t="n">
+      <x:c r="C12" s="28"/>
+      <x:c r="D12" s="28"/>
+      <x:c r="E12" s="28"/>
+      <x:c r="F12" s="28"/>
+      <x:c r="G12" s="28"/>
+      <x:c r="H12" s="28"/>
+      <x:c r="I12" s="30" t="n">
         <x:f>ROUND(SUM(I11:I11),1)</x:f>
-        <x:v>101.6</x:v>
-      </x:c>
-      <x:c r="J12" s="26"/>
-      <x:c r="K12" s="26"/>
+        <x:v>247.5</x:v>
+      </x:c>
+      <x:c r="J12" s="28"/>
+      <x:c r="K12" s="28"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="27" t="str">
+      <x:c r="A13" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B13" s="26"/>
-      <x:c r="C13" s="26"/>
-      <x:c r="D13" s="26"/>
-      <x:c r="E13" s="26"/>
-      <x:c r="F13" s="26"/>
-      <x:c r="G13" s="26"/>
-      <x:c r="H13" s="26"/>
-      <x:c r="I13" s="30" t="n">
+      <x:c r="B13" s="28"/>
+      <x:c r="C13" s="28"/>
+      <x:c r="D13" s="28"/>
+      <x:c r="E13" s="28"/>
+      <x:c r="F13" s="28"/>
+      <x:c r="G13" s="28"/>
+      <x:c r="H13" s="28"/>
+      <x:c r="I13" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I11:I11),0),1)</x:f>
-        <x:v>101.6</x:v>
-      </x:c>
-      <x:c r="J13" s="26"/>
-      <x:c r="K13" s="26"/>
+        <x:v>247.5</x:v>
+      </x:c>
+      <x:c r="J13" s="28"/>
+      <x:c r="K13" s="28"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="17" t="str">
@@ -1096,70 +1119,70 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B17" s="22" t="str">
-        <x:v>8月3日</x:v>
+        <x:v>8月3日-8月4日</x:v>
       </x:c>
       <x:c r="C17" s="23" t="n">
         <x:v>3812.61</x:v>
       </x:c>
       <x:c r="D17" s="23" t="n">
-        <x:v>3827.64</x:v>
+        <x:v>3831.94</x:v>
       </x:c>
       <x:c r="E17" s="23" t="n">
         <x:v>3797.64</x:v>
       </x:c>
       <x:c r="F17" s="23" t="n">
-        <x:v>3809.66</x:v>
+        <x:v>3822.28</x:v>
       </x:c>
       <x:c r="G17" s="23"/>
       <x:c r="H17" s="24"/>
       <x:c r="I17" s="23" t="n">
         <x:f>ROUND(D17-E17,1)</x:f>
-        <x:v>30</x:v>
+        <x:v>34.3</x:v>
       </x:c>
       <x:c r="J17" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K17" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="29" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B18" s="28" t="n">
         <x:v>1</x:v>
       </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="27" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B18" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C18" s="26"/>
-      <x:c r="D18" s="26"/>
-      <x:c r="E18" s="26"/>
-      <x:c r="F18" s="26"/>
-      <x:c r="G18" s="26"/>
-      <x:c r="H18" s="26"/>
-      <x:c r="I18" s="28" t="n">
+      <x:c r="C18" s="28"/>
+      <x:c r="D18" s="28"/>
+      <x:c r="E18" s="28"/>
+      <x:c r="F18" s="28"/>
+      <x:c r="G18" s="28"/>
+      <x:c r="H18" s="28"/>
+      <x:c r="I18" s="30" t="n">
         <x:f>ROUND(SUM(I17:I17),1)</x:f>
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="J18" s="26"/>
-      <x:c r="K18" s="26"/>
+        <x:v>34.3</x:v>
+      </x:c>
+      <x:c r="J18" s="28"/>
+      <x:c r="K18" s="28"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="27" t="str">
+      <x:c r="A19" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B19" s="26"/>
-      <x:c r="C19" s="26"/>
-      <x:c r="D19" s="26"/>
-      <x:c r="E19" s="26"/>
-      <x:c r="F19" s="26"/>
-      <x:c r="G19" s="26"/>
-      <x:c r="H19" s="26"/>
-      <x:c r="I19" s="30" t="n">
+      <x:c r="B19" s="28"/>
+      <x:c r="C19" s="28"/>
+      <x:c r="D19" s="28"/>
+      <x:c r="E19" s="28"/>
+      <x:c r="F19" s="28"/>
+      <x:c r="G19" s="28"/>
+      <x:c r="H19" s="28"/>
+      <x:c r="I19" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I17:I17),0),1)</x:f>
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="J19" s="26"/>
-      <x:c r="K19" s="26"/>
+        <x:v>34.3</x:v>
+      </x:c>
+      <x:c r="J19" s="28"/>
+      <x:c r="K19" s="28"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="17" t="str">
@@ -1216,70 +1239,70 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B23" s="22" t="str">
-        <x:v>8月3日</x:v>
+        <x:v>8月3日-8月4日</x:v>
       </x:c>
       <x:c r="C23" s="23" t="n">
         <x:v>7000</x:v>
       </x:c>
       <x:c r="D23" s="23" t="n">
-        <x:v>7064.2</x:v>
+        <x:v>7269.8</x:v>
       </x:c>
       <x:c r="E23" s="23" t="n">
         <x:v>6976</x:v>
       </x:c>
       <x:c r="F23" s="23" t="n">
-        <x:v>7023.4</x:v>
+        <x:v>7211.4</x:v>
       </x:c>
       <x:c r="G23" s="23"/>
       <x:c r="H23" s="24"/>
-      <x:c r="I23" s="23" t="n">
+      <x:c r="I23" s="26" t="n">
         <x:f>ROUND(D23-E23,1)</x:f>
-        <x:v>88.2</x:v>
+        <x:v>293.8</x:v>
       </x:c>
       <x:c r="J23" s="22" t="str">
         <x:v>IM2609</x:v>
       </x:c>
       <x:c r="K23" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="29" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B24" s="28" t="n">
         <x:v>1</x:v>
       </x:c>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="27" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B24" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C24" s="26"/>
-      <x:c r="D24" s="26"/>
-      <x:c r="E24" s="26"/>
-      <x:c r="F24" s="26"/>
-      <x:c r="G24" s="26"/>
-      <x:c r="H24" s="26"/>
-      <x:c r="I24" s="28" t="n">
+      <x:c r="C24" s="28"/>
+      <x:c r="D24" s="28"/>
+      <x:c r="E24" s="28"/>
+      <x:c r="F24" s="28"/>
+      <x:c r="G24" s="28"/>
+      <x:c r="H24" s="28"/>
+      <x:c r="I24" s="30" t="n">
         <x:f>ROUND(SUM(I23:I23),1)</x:f>
-        <x:v>88.2</x:v>
-      </x:c>
-      <x:c r="J24" s="26"/>
-      <x:c r="K24" s="26"/>
+        <x:v>293.8</x:v>
+      </x:c>
+      <x:c r="J24" s="28"/>
+      <x:c r="K24" s="28"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="27" t="str">
+      <x:c r="A25" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B25" s="26"/>
-      <x:c r="C25" s="26"/>
-      <x:c r="D25" s="26"/>
-      <x:c r="E25" s="26"/>
-      <x:c r="F25" s="26"/>
-      <x:c r="G25" s="26"/>
-      <x:c r="H25" s="26"/>
-      <x:c r="I25" s="30" t="n">
+      <x:c r="B25" s="28"/>
+      <x:c r="C25" s="28"/>
+      <x:c r="D25" s="28"/>
+      <x:c r="E25" s="28"/>
+      <x:c r="F25" s="28"/>
+      <x:c r="G25" s="28"/>
+      <x:c r="H25" s="28"/>
+      <x:c r="I25" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I23:I23),0),1)</x:f>
-        <x:v>88.2</x:v>
-      </x:c>
-      <x:c r="J25" s="26"/>
-      <x:c r="K25" s="26"/>
+        <x:v>293.8</x:v>
+      </x:c>
+      <x:c r="J25" s="28"/>
+      <x:c r="K25" s="28"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="17" t="str">
@@ -1336,70 +1359,70 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B29" s="22" t="str">
-        <x:v>8月3日</x:v>
+        <x:v>8月3日-8月4日</x:v>
       </x:c>
       <x:c r="C29" s="23" t="n">
         <x:v>7391</x:v>
       </x:c>
       <x:c r="D29" s="23" t="n">
-        <x:v>7440</x:v>
+        <x:v>7599</x:v>
       </x:c>
       <x:c r="E29" s="23" t="n">
         <x:v>7335</x:v>
       </x:c>
       <x:c r="F29" s="23" t="n">
-        <x:v>7356</x:v>
+        <x:v>7529</x:v>
       </x:c>
       <x:c r="G29" s="23"/>
       <x:c r="H29" s="24"/>
-      <x:c r="I29" s="23" t="n">
+      <x:c r="I29" s="26" t="n">
         <x:f>ROUND(D29-E29,1)</x:f>
-        <x:v>105</x:v>
+        <x:v>264</x:v>
       </x:c>
       <x:c r="J29" s="22" t="str">
         <x:v>IC2609</x:v>
       </x:c>
       <x:c r="K29" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="29" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B30" s="28" t="n">
         <x:v>1</x:v>
       </x:c>
-    </x:row>
-    <x:row r="30">
-      <x:c r="A30" s="27" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B30" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C30" s="26"/>
-      <x:c r="D30" s="26"/>
-      <x:c r="E30" s="26"/>
-      <x:c r="F30" s="26"/>
-      <x:c r="G30" s="26"/>
-      <x:c r="H30" s="26"/>
-      <x:c r="I30" s="28" t="n">
+      <x:c r="C30" s="28"/>
+      <x:c r="D30" s="28"/>
+      <x:c r="E30" s="28"/>
+      <x:c r="F30" s="28"/>
+      <x:c r="G30" s="28"/>
+      <x:c r="H30" s="28"/>
+      <x:c r="I30" s="30" t="n">
         <x:f>ROUND(SUM(I29:I29),1)</x:f>
-        <x:v>105</x:v>
-      </x:c>
-      <x:c r="J30" s="26"/>
-      <x:c r="K30" s="26"/>
+        <x:v>264</x:v>
+      </x:c>
+      <x:c r="J30" s="28"/>
+      <x:c r="K30" s="28"/>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="27" t="str">
+      <x:c r="A31" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B31" s="26"/>
-      <x:c r="C31" s="26"/>
-      <x:c r="D31" s="26"/>
-      <x:c r="E31" s="26"/>
-      <x:c r="F31" s="26"/>
-      <x:c r="G31" s="26"/>
-      <x:c r="H31" s="26"/>
-      <x:c r="I31" s="30" t="n">
+      <x:c r="B31" s="28"/>
+      <x:c r="C31" s="28"/>
+      <x:c r="D31" s="28"/>
+      <x:c r="E31" s="28"/>
+      <x:c r="F31" s="28"/>
+      <x:c r="G31" s="28"/>
+      <x:c r="H31" s="28"/>
+      <x:c r="I31" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I29:I29),0),1)</x:f>
-        <x:v>105</x:v>
-      </x:c>
-      <x:c r="J31" s="26"/>
-      <x:c r="K31" s="26"/>
+        <x:v>264</x:v>
+      </x:c>
+      <x:c r="J31" s="28"/>
+      <x:c r="K31" s="28"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="17" t="str">
@@ -1456,70 +1479,70 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B35" s="22" t="str">
-        <x:v>8月3日</x:v>
+        <x:v>8月3日-8月4日</x:v>
       </x:c>
       <x:c r="C35" s="23" t="n">
         <x:v>4526.4</x:v>
       </x:c>
       <x:c r="D35" s="23" t="n">
-        <x:v>4538</x:v>
+        <x:v>4580.8</x:v>
       </x:c>
       <x:c r="E35" s="23" t="n">
         <x:v>4494.2</x:v>
       </x:c>
       <x:c r="F35" s="23" t="n">
-        <x:v>4512.2</x:v>
+        <x:v>4552.8</x:v>
       </x:c>
       <x:c r="G35" s="23"/>
       <x:c r="H35" s="24"/>
       <x:c r="I35" s="23" t="n">
         <x:f>ROUND(D35-E35,1)</x:f>
-        <x:v>43.8</x:v>
+        <x:v>86.6</x:v>
       </x:c>
       <x:c r="J35" s="22" t="str">
         <x:v>IF2609</x:v>
       </x:c>
       <x:c r="K35" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="29" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B36" s="28" t="n">
         <x:v>1</x:v>
       </x:c>
-    </x:row>
-    <x:row r="36">
-      <x:c r="A36" s="27" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B36" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C36" s="26"/>
-      <x:c r="D36" s="26"/>
-      <x:c r="E36" s="26"/>
-      <x:c r="F36" s="26"/>
-      <x:c r="G36" s="26"/>
-      <x:c r="H36" s="26"/>
-      <x:c r="I36" s="28" t="n">
+      <x:c r="C36" s="28"/>
+      <x:c r="D36" s="28"/>
+      <x:c r="E36" s="28"/>
+      <x:c r="F36" s="28"/>
+      <x:c r="G36" s="28"/>
+      <x:c r="H36" s="28"/>
+      <x:c r="I36" s="30" t="n">
         <x:f>ROUND(SUM(I35:I35),1)</x:f>
-        <x:v>43.8</x:v>
-      </x:c>
-      <x:c r="J36" s="26"/>
-      <x:c r="K36" s="26"/>
+        <x:v>86.6</x:v>
+      </x:c>
+      <x:c r="J36" s="28"/>
+      <x:c r="K36" s="28"/>
     </x:row>
     <x:row r="37">
-      <x:c r="A37" s="27" t="str">
+      <x:c r="A37" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B37" s="26"/>
-      <x:c r="C37" s="26"/>
-      <x:c r="D37" s="26"/>
-      <x:c r="E37" s="26"/>
-      <x:c r="F37" s="26"/>
-      <x:c r="G37" s="26"/>
-      <x:c r="H37" s="26"/>
-      <x:c r="I37" s="30" t="n">
+      <x:c r="B37" s="28"/>
+      <x:c r="C37" s="28"/>
+      <x:c r="D37" s="28"/>
+      <x:c r="E37" s="28"/>
+      <x:c r="F37" s="28"/>
+      <x:c r="G37" s="28"/>
+      <x:c r="H37" s="28"/>
+      <x:c r="I37" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I35:I35),0),1)</x:f>
-        <x:v>43.8</x:v>
-      </x:c>
-      <x:c r="J37" s="26"/>
-      <x:c r="K37" s="26"/>
+        <x:v>86.6</x:v>
+      </x:c>
+      <x:c r="J37" s="28"/>
+      <x:c r="K37" s="28"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="17" t="str">
@@ -1576,7 +1599,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B41" s="22" t="str">
-        <x:v>8月3日</x:v>
+        <x:v>8月3日-8月4日</x:v>
       </x:c>
       <x:c r="C41" s="23" t="n">
         <x:v>2882.4</x:v>
@@ -1588,7 +1611,7 @@
         <x:v>2845.8</x:v>
       </x:c>
       <x:c r="F41" s="23" t="n">
-        <x:v>2860</x:v>
+        <x:v>2852.4</x:v>
       </x:c>
       <x:c r="G41" s="23"/>
       <x:c r="H41" s="24"/>
@@ -1600,46 +1623,46 @@
         <x:v>IH2609</x:v>
       </x:c>
       <x:c r="K41" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="29" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B42" s="28" t="n">
         <x:v>1</x:v>
       </x:c>
-    </x:row>
-    <x:row r="42">
-      <x:c r="A42" s="27" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B42" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C42" s="26"/>
-      <x:c r="D42" s="26"/>
-      <x:c r="E42" s="26"/>
-      <x:c r="F42" s="26"/>
-      <x:c r="G42" s="26"/>
-      <x:c r="H42" s="26"/>
-      <x:c r="I42" s="28" t="n">
+      <x:c r="C42" s="28"/>
+      <x:c r="D42" s="28"/>
+      <x:c r="E42" s="28"/>
+      <x:c r="F42" s="28"/>
+      <x:c r="G42" s="28"/>
+      <x:c r="H42" s="28"/>
+      <x:c r="I42" s="30" t="n">
         <x:f>ROUND(SUM(I41:I41),1)</x:f>
         <x:v>44.2</x:v>
       </x:c>
-      <x:c r="J42" s="26"/>
-      <x:c r="K42" s="26"/>
+      <x:c r="J42" s="28"/>
+      <x:c r="K42" s="28"/>
     </x:row>
     <x:row r="43">
-      <x:c r="A43" s="27" t="str">
+      <x:c r="A43" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B43" s="26"/>
-      <x:c r="C43" s="26"/>
-      <x:c r="D43" s="26"/>
-      <x:c r="E43" s="26"/>
-      <x:c r="F43" s="26"/>
-      <x:c r="G43" s="26"/>
-      <x:c r="H43" s="26"/>
-      <x:c r="I43" s="30" t="n">
+      <x:c r="B43" s="28"/>
+      <x:c r="C43" s="28"/>
+      <x:c r="D43" s="28"/>
+      <x:c r="E43" s="28"/>
+      <x:c r="F43" s="28"/>
+      <x:c r="G43" s="28"/>
+      <x:c r="H43" s="28"/>
+      <x:c r="I43" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I41:I41),0),1)</x:f>
         <x:v>44.2</x:v>
       </x:c>
-      <x:c r="J43" s="26"/>
-      <x:c r="K43" s="26"/>
+      <x:c r="J43" s="28"/>
+      <x:c r="K43" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1749,43 +1772,79 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="27" t="str">
+    <x:row r="5">
+      <x:c r="A5" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B5" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C5" s="22" t="str">
+        <x:v>8月4日</x:v>
+      </x:c>
+      <x:c r="D5" s="23" t="n">
+        <x:v>7128.49</x:v>
+      </x:c>
+      <x:c r="E5" s="23" t="n">
+        <x:v>7307.17</x:v>
+      </x:c>
+      <x:c r="F5" s="23" t="n">
+        <x:v>7102.46</x:v>
+      </x:c>
+      <x:c r="G5" s="23" t="n">
+        <x:v>7279.19</x:v>
+      </x:c>
+      <x:c r="H5" s="37" t="n">
+        <x:v>199.4</x:v>
+      </x:c>
+      <x:c r="I5" s="24" t="n">
+        <x:v>0.028166129456000055</x:v>
+      </x:c>
+      <x:c r="J5" s="26" t="n">
+        <x:f>ROUND(E5-F5,1)</x:f>
+        <x:v>204.7</x:v>
+      </x:c>
+      <x:c r="K5" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B7" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C7" s="26"/>
-      <x:c r="D7" s="26"/>
-      <x:c r="E7" s="26"/>
-      <x:c r="F7" s="26"/>
-      <x:c r="G7" s="26"/>
-      <x:c r="H7" s="26"/>
-      <x:c r="I7" s="26"/>
-      <x:c r="J7" s="28" t="n">
-        <x:f>SUM(J4:J4)</x:f>
-        <x:v>75.2</x:v>
-      </x:c>
-      <x:c r="K7" s="26"/>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="27" t="str">
+      <x:c r="B8" s="28" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C8" s="28"/>
+      <x:c r="D8" s="28"/>
+      <x:c r="E8" s="28"/>
+      <x:c r="F8" s="28"/>
+      <x:c r="G8" s="28"/>
+      <x:c r="H8" s="28"/>
+      <x:c r="I8" s="28"/>
+      <x:c r="J8" s="30" t="n">
+        <x:f>SUM(J4:J5)</x:f>
+        <x:v>279.9</x:v>
+      </x:c>
+      <x:c r="K8" s="28"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B8" s="26"/>
-      <x:c r="C8" s="26"/>
-      <x:c r="D8" s="26"/>
-      <x:c r="E8" s="26"/>
-      <x:c r="F8" s="26"/>
-      <x:c r="G8" s="26"/>
-      <x:c r="H8" s="26"/>
-      <x:c r="I8" s="26"/>
-      <x:c r="J8" s="30" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J4),0),1)</x:f>
-        <x:v>75.2</x:v>
-      </x:c>
-      <x:c r="K8" s="26"/>
+      <x:c r="B9" s="28"/>
+      <x:c r="C9" s="28"/>
+      <x:c r="D9" s="28"/>
+      <x:c r="E9" s="28"/>
+      <x:c r="F9" s="28"/>
+      <x:c r="G9" s="28"/>
+      <x:c r="H9" s="28"/>
+      <x:c r="I9" s="28"/>
+      <x:c r="J9" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J5),0),1)</x:f>
+        <x:v>140</x:v>
+      </x:c>
+      <x:c r="K9" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1888,43 +1947,79 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="27" t="str">
+    <x:row r="5">
+      <x:c r="A5" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B5" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C5" s="22" t="str">
+        <x:v>8月4日</x:v>
+      </x:c>
+      <x:c r="D5" s="23" t="n">
+        <x:v>7467.08</x:v>
+      </x:c>
+      <x:c r="E5" s="23" t="n">
+        <x:v>7645.48</x:v>
+      </x:c>
+      <x:c r="F5" s="23" t="n">
+        <x:v>7450.32</x:v>
+      </x:c>
+      <x:c r="G5" s="23" t="n">
+        <x:v>7607.49</x:v>
+      </x:c>
+      <x:c r="H5" s="37" t="n">
+        <x:v>193</x:v>
+      </x:c>
+      <x:c r="I5" s="24" t="n">
+        <x:v>0.02602595987332945</x:v>
+      </x:c>
+      <x:c r="J5" s="26" t="n">
+        <x:f>ROUND(E5-F5,1)</x:f>
+        <x:v>195.2</x:v>
+      </x:c>
+      <x:c r="K5" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B7" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C7" s="26"/>
-      <x:c r="D7" s="26"/>
-      <x:c r="E7" s="26"/>
-      <x:c r="F7" s="26"/>
-      <x:c r="G7" s="26"/>
-      <x:c r="H7" s="26"/>
-      <x:c r="I7" s="26"/>
-      <x:c r="J7" s="28" t="n">
-        <x:f>SUM(J4:J4)</x:f>
-        <x:v>101.6</x:v>
-      </x:c>
-      <x:c r="K7" s="26"/>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="27" t="str">
+      <x:c r="B8" s="28" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C8" s="28"/>
+      <x:c r="D8" s="28"/>
+      <x:c r="E8" s="28"/>
+      <x:c r="F8" s="28"/>
+      <x:c r="G8" s="28"/>
+      <x:c r="H8" s="28"/>
+      <x:c r="I8" s="28"/>
+      <x:c r="J8" s="30" t="n">
+        <x:f>SUM(J4:J5)</x:f>
+        <x:v>296.79999999999995</x:v>
+      </x:c>
+      <x:c r="K8" s="28"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B8" s="26"/>
-      <x:c r="C8" s="26"/>
-      <x:c r="D8" s="26"/>
-      <x:c r="E8" s="26"/>
-      <x:c r="F8" s="26"/>
-      <x:c r="G8" s="26"/>
-      <x:c r="H8" s="26"/>
-      <x:c r="I8" s="26"/>
-      <x:c r="J8" s="30" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J4),0),1)</x:f>
-        <x:v>101.6</x:v>
-      </x:c>
-      <x:c r="K8" s="26"/>
+      <x:c r="B9" s="28"/>
+      <x:c r="C9" s="28"/>
+      <x:c r="D9" s="28"/>
+      <x:c r="E9" s="28"/>
+      <x:c r="F9" s="28"/>
+      <x:c r="G9" s="28"/>
+      <x:c r="H9" s="28"/>
+      <x:c r="I9" s="28"/>
+      <x:c r="J9" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J5),0),1)</x:f>
+        <x:v>148.4</x:v>
+      </x:c>
+      <x:c r="K9" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2027,43 +2122,79 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="27" t="str">
+    <x:row r="5">
+      <x:c r="A5" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B5" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C5" s="22" t="str">
+        <x:v>8月4日</x:v>
+      </x:c>
+      <x:c r="D5" s="23" t="n">
+        <x:v>3816.37</x:v>
+      </x:c>
+      <x:c r="E5" s="23" t="n">
+        <x:v>3831.94</x:v>
+      </x:c>
+      <x:c r="F5" s="23" t="n">
+        <x:v>3799.52</x:v>
+      </x:c>
+      <x:c r="G5" s="23" t="n">
+        <x:v>3822.28</x:v>
+      </x:c>
+      <x:c r="H5" s="23" t="n">
+        <x:v>12.6</x:v>
+      </x:c>
+      <x:c r="I5" s="24" t="n">
+        <x:v>0.0033126315734213208</x:v>
+      </x:c>
+      <x:c r="J5" s="23" t="n">
+        <x:f>ROUND(E5-F5,1)</x:f>
+        <x:v>32.4</x:v>
+      </x:c>
+      <x:c r="K5" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B7" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C7" s="26"/>
-      <x:c r="D7" s="26"/>
-      <x:c r="E7" s="26"/>
-      <x:c r="F7" s="26"/>
-      <x:c r="G7" s="26"/>
-      <x:c r="H7" s="26"/>
-      <x:c r="I7" s="26"/>
-      <x:c r="J7" s="28" t="n">
-        <x:f>SUM(J4:J4)</x:f>
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="K7" s="26"/>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="27" t="str">
+      <x:c r="B8" s="28" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C8" s="28"/>
+      <x:c r="D8" s="28"/>
+      <x:c r="E8" s="28"/>
+      <x:c r="F8" s="28"/>
+      <x:c r="G8" s="28"/>
+      <x:c r="H8" s="28"/>
+      <x:c r="I8" s="28"/>
+      <x:c r="J8" s="30" t="n">
+        <x:f>SUM(J4:J5)</x:f>
+        <x:v>62.4</x:v>
+      </x:c>
+      <x:c r="K8" s="28"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B8" s="26"/>
-      <x:c r="C8" s="26"/>
-      <x:c r="D8" s="26"/>
-      <x:c r="E8" s="26"/>
-      <x:c r="F8" s="26"/>
-      <x:c r="G8" s="26"/>
-      <x:c r="H8" s="26"/>
-      <x:c r="I8" s="26"/>
-      <x:c r="J8" s="30" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J4),0),1)</x:f>
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="K8" s="26"/>
+      <x:c r="B9" s="28"/>
+      <x:c r="C9" s="28"/>
+      <x:c r="D9" s="28"/>
+      <x:c r="E9" s="28"/>
+      <x:c r="F9" s="28"/>
+      <x:c r="G9" s="28"/>
+      <x:c r="H9" s="28"/>
+      <x:c r="I9" s="28"/>
+      <x:c r="J9" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J5),0),1)</x:f>
+        <x:v>31.2</x:v>
+      </x:c>
+      <x:c r="K9" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2166,43 +2297,79 @@
         <x:v>IM2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="27" t="str">
+    <x:row r="5">
+      <x:c r="A5" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B5" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C5" s="22" t="str">
+        <x:v>8月4日</x:v>
+      </x:c>
+      <x:c r="D5" s="23" t="n">
+        <x:v>7073.2</x:v>
+      </x:c>
+      <x:c r="E5" s="23" t="n">
+        <x:v>7269.8</x:v>
+      </x:c>
+      <x:c r="F5" s="23" t="n">
+        <x:v>7057.8</x:v>
+      </x:c>
+      <x:c r="G5" s="23" t="n">
+        <x:v>7211.4</x:v>
+      </x:c>
+      <x:c r="H5" s="37" t="n">
+        <x:v>188</x:v>
+      </x:c>
+      <x:c r="I5" s="24" t="n">
+        <x:v>0.026767662385739133</x:v>
+      </x:c>
+      <x:c r="J5" s="26" t="n">
+        <x:f>ROUND(E5-F5,1)</x:f>
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="K5" s="22" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B7" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C7" s="26"/>
-      <x:c r="D7" s="26"/>
-      <x:c r="E7" s="26"/>
-      <x:c r="F7" s="26"/>
-      <x:c r="G7" s="26"/>
-      <x:c r="H7" s="26"/>
-      <x:c r="I7" s="26"/>
-      <x:c r="J7" s="28" t="n">
-        <x:f>SUM(J4:J4)</x:f>
-        <x:v>88.2</x:v>
-      </x:c>
-      <x:c r="K7" s="26"/>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="27" t="str">
+      <x:c r="B8" s="28" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C8" s="28"/>
+      <x:c r="D8" s="28"/>
+      <x:c r="E8" s="28"/>
+      <x:c r="F8" s="28"/>
+      <x:c r="G8" s="28"/>
+      <x:c r="H8" s="28"/>
+      <x:c r="I8" s="28"/>
+      <x:c r="J8" s="30" t="n">
+        <x:f>SUM(J4:J5)</x:f>
+        <x:v>300.2</x:v>
+      </x:c>
+      <x:c r="K8" s="28"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B8" s="26"/>
-      <x:c r="C8" s="26"/>
-      <x:c r="D8" s="26"/>
-      <x:c r="E8" s="26"/>
-      <x:c r="F8" s="26"/>
-      <x:c r="G8" s="26"/>
-      <x:c r="H8" s="26"/>
-      <x:c r="I8" s="26"/>
-      <x:c r="J8" s="30" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J4),0),1)</x:f>
-        <x:v>88.2</x:v>
-      </x:c>
-      <x:c r="K8" s="26"/>
+      <x:c r="B9" s="28"/>
+      <x:c r="C9" s="28"/>
+      <x:c r="D9" s="28"/>
+      <x:c r="E9" s="28"/>
+      <x:c r="F9" s="28"/>
+      <x:c r="G9" s="28"/>
+      <x:c r="H9" s="28"/>
+      <x:c r="I9" s="28"/>
+      <x:c r="J9" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J5),0),1)</x:f>
+        <x:v>150.1</x:v>
+      </x:c>
+      <x:c r="K9" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2305,43 +2472,79 @@
         <x:v>IC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="27" t="str">
+    <x:row r="5">
+      <x:c r="A5" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B5" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C5" s="22" t="str">
+        <x:v>8月4日</x:v>
+      </x:c>
+      <x:c r="D5" s="23" t="n">
+        <x:v>7406</x:v>
+      </x:c>
+      <x:c r="E5" s="23" t="n">
+        <x:v>7599</x:v>
+      </x:c>
+      <x:c r="F5" s="23" t="n">
+        <x:v>7392.8</x:v>
+      </x:c>
+      <x:c r="G5" s="23" t="n">
+        <x:v>7529</x:v>
+      </x:c>
+      <x:c r="H5" s="37" t="n">
+        <x:v>173</x:v>
+      </x:c>
+      <x:c r="I5" s="24" t="n">
+        <x:v>0.023518216421968496</x:v>
+      </x:c>
+      <x:c r="J5" s="26" t="n">
+        <x:f>ROUND(E5-F5,1)</x:f>
+        <x:v>206.2</x:v>
+      </x:c>
+      <x:c r="K5" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B7" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C7" s="26"/>
-      <x:c r="D7" s="26"/>
-      <x:c r="E7" s="26"/>
-      <x:c r="F7" s="26"/>
-      <x:c r="G7" s="26"/>
-      <x:c r="H7" s="26"/>
-      <x:c r="I7" s="26"/>
-      <x:c r="J7" s="28" t="n">
-        <x:f>SUM(J4:J4)</x:f>
-        <x:v>105</x:v>
-      </x:c>
-      <x:c r="K7" s="26"/>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="27" t="str">
+      <x:c r="B8" s="28" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C8" s="28"/>
+      <x:c r="D8" s="28"/>
+      <x:c r="E8" s="28"/>
+      <x:c r="F8" s="28"/>
+      <x:c r="G8" s="28"/>
+      <x:c r="H8" s="28"/>
+      <x:c r="I8" s="28"/>
+      <x:c r="J8" s="30" t="n">
+        <x:f>SUM(J4:J5)</x:f>
+        <x:v>311.2</x:v>
+      </x:c>
+      <x:c r="K8" s="28"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B8" s="26"/>
-      <x:c r="C8" s="26"/>
-      <x:c r="D8" s="26"/>
-      <x:c r="E8" s="26"/>
-      <x:c r="F8" s="26"/>
-      <x:c r="G8" s="26"/>
-      <x:c r="H8" s="26"/>
-      <x:c r="I8" s="26"/>
-      <x:c r="J8" s="30" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J4),0),1)</x:f>
-        <x:v>105</x:v>
-      </x:c>
-      <x:c r="K8" s="26"/>
+      <x:c r="B9" s="28"/>
+      <x:c r="C9" s="28"/>
+      <x:c r="D9" s="28"/>
+      <x:c r="E9" s="28"/>
+      <x:c r="F9" s="28"/>
+      <x:c r="G9" s="28"/>
+      <x:c r="H9" s="28"/>
+      <x:c r="I9" s="28"/>
+      <x:c r="J9" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J5),0),1)</x:f>
+        <x:v>155.6</x:v>
+      </x:c>
+      <x:c r="K9" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2444,43 +2647,79 @@
         <x:v>IF2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="27" t="str">
+    <x:row r="5">
+      <x:c r="A5" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B5" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C5" s="22" t="str">
+        <x:v>8月4日</x:v>
+      </x:c>
+      <x:c r="D5" s="23" t="n">
+        <x:v>4538</x:v>
+      </x:c>
+      <x:c r="E5" s="23" t="n">
+        <x:v>4580.8</x:v>
+      </x:c>
+      <x:c r="F5" s="23" t="n">
+        <x:v>4524.2</x:v>
+      </x:c>
+      <x:c r="G5" s="23" t="n">
+        <x:v>4552.8</x:v>
+      </x:c>
+      <x:c r="H5" s="23" t="n">
+        <x:v>40.6</x:v>
+      </x:c>
+      <x:c r="I5" s="24" t="n">
+        <x:v>0.00899782811045613</x:v>
+      </x:c>
+      <x:c r="J5" s="23" t="n">
+        <x:f>ROUND(E5-F5,1)</x:f>
+        <x:v>56.6</x:v>
+      </x:c>
+      <x:c r="K5" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B7" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C7" s="26"/>
-      <x:c r="D7" s="26"/>
-      <x:c r="E7" s="26"/>
-      <x:c r="F7" s="26"/>
-      <x:c r="G7" s="26"/>
-      <x:c r="H7" s="26"/>
-      <x:c r="I7" s="26"/>
-      <x:c r="J7" s="28" t="n">
-        <x:f>SUM(J4:J4)</x:f>
-        <x:v>43.8</x:v>
-      </x:c>
-      <x:c r="K7" s="26"/>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="27" t="str">
+      <x:c r="B8" s="28" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C8" s="28"/>
+      <x:c r="D8" s="28"/>
+      <x:c r="E8" s="28"/>
+      <x:c r="F8" s="28"/>
+      <x:c r="G8" s="28"/>
+      <x:c r="H8" s="28"/>
+      <x:c r="I8" s="28"/>
+      <x:c r="J8" s="30" t="n">
+        <x:f>SUM(J4:J5)</x:f>
+        <x:v>100.4</x:v>
+      </x:c>
+      <x:c r="K8" s="28"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B8" s="26"/>
-      <x:c r="C8" s="26"/>
-      <x:c r="D8" s="26"/>
-      <x:c r="E8" s="26"/>
-      <x:c r="F8" s="26"/>
-      <x:c r="G8" s="26"/>
-      <x:c r="H8" s="26"/>
-      <x:c r="I8" s="26"/>
-      <x:c r="J8" s="30" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J4),0),1)</x:f>
-        <x:v>43.8</x:v>
-      </x:c>
-      <x:c r="K8" s="26"/>
+      <x:c r="B9" s="28"/>
+      <x:c r="C9" s="28"/>
+      <x:c r="D9" s="28"/>
+      <x:c r="E9" s="28"/>
+      <x:c r="F9" s="28"/>
+      <x:c r="G9" s="28"/>
+      <x:c r="H9" s="28"/>
+      <x:c r="I9" s="28"/>
+      <x:c r="J9" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J5),0),1)</x:f>
+        <x:v>50.2</x:v>
+      </x:c>
+      <x:c r="K9" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2583,43 +2822,79 @@
         <x:v>IH2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="27" t="str">
+    <x:row r="5">
+      <x:c r="A5" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B5" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C5" s="22" t="str">
+        <x:v>8月4日</x:v>
+      </x:c>
+      <x:c r="D5" s="23" t="n">
+        <x:v>2872</x:v>
+      </x:c>
+      <x:c r="E5" s="23" t="n">
+        <x:v>2872</x:v>
+      </x:c>
+      <x:c r="F5" s="23" t="n">
+        <x:v>2846.6</x:v>
+      </x:c>
+      <x:c r="G5" s="23" t="n">
+        <x:v>2852.4</x:v>
+      </x:c>
+      <x:c r="H5" s="23" t="n">
+        <x:v>-7.6</x:v>
+      </x:c>
+      <x:c r="I5" s="24" t="n">
+        <x:v>-0.0026573426573426318</x:v>
+      </x:c>
+      <x:c r="J5" s="23" t="n">
+        <x:f>ROUND(E5-F5,1)</x:f>
+        <x:v>25.4</x:v>
+      </x:c>
+      <x:c r="K5" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B7" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C7" s="26"/>
-      <x:c r="D7" s="26"/>
-      <x:c r="E7" s="26"/>
-      <x:c r="F7" s="26"/>
-      <x:c r="G7" s="26"/>
-      <x:c r="H7" s="26"/>
-      <x:c r="I7" s="26"/>
-      <x:c r="J7" s="28" t="n">
-        <x:f>SUM(J4:J4)</x:f>
-        <x:v>44.2</x:v>
-      </x:c>
-      <x:c r="K7" s="26"/>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="27" t="str">
+      <x:c r="B8" s="28" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C8" s="28"/>
+      <x:c r="D8" s="28"/>
+      <x:c r="E8" s="28"/>
+      <x:c r="F8" s="28"/>
+      <x:c r="G8" s="28"/>
+      <x:c r="H8" s="28"/>
+      <x:c r="I8" s="28"/>
+      <x:c r="J8" s="30" t="n">
+        <x:f>SUM(J4:J5)</x:f>
+        <x:v>69.6</x:v>
+      </x:c>
+      <x:c r="K8" s="28"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B8" s="26"/>
-      <x:c r="C8" s="26"/>
-      <x:c r="D8" s="26"/>
-      <x:c r="E8" s="26"/>
-      <x:c r="F8" s="26"/>
-      <x:c r="G8" s="26"/>
-      <x:c r="H8" s="26"/>
-      <x:c r="I8" s="26"/>
-      <x:c r="J8" s="30" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J4),0),1)</x:f>
-        <x:v>44.2</x:v>
-      </x:c>
-      <x:c r="K8" s="26"/>
+      <x:c r="B9" s="28"/>
+      <x:c r="C9" s="28"/>
+      <x:c r="D9" s="28"/>
+      <x:c r="E9" s="28"/>
+      <x:c r="F9" s="28"/>
+      <x:c r="G9" s="28"/>
+      <x:c r="H9" s="28"/>
+      <x:c r="I9" s="28"/>
+      <x:c r="J9" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J5),0),1)</x:f>
+        <x:v>34.8</x:v>
+      </x:c>
+      <x:c r="K9" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-08-05
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rede2126f2b7b47ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Raa6ea3672b78409a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Rf54642ce61cc4afe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R24230e6d14f24e99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Rc8abf6fd62c5448f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R5684d792ab514e61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R641d69169b354c0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R8f5d9c818d764978"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R78825a0cde7440ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rbc8ea03a9dc34ec9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Rab15b08a3bd344db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R9998e5128fdb4316"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rdbb16c5fff544497"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R76c36c4b142445f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R65ec3c92713f4819"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R4b8c91c98422466f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Re5ca34c48b154373"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R3095ecf954de4443"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -484,25 +484,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-08-04</x:v>
+        <x:v>2026-08-05</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7307.17</x:v>
+        <x:v>7523.5</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7102.46</x:v>
+        <x:v>7253.22</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>204.7</x:v>
+        <x:v>270.3</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>279.9</x:v>
+        <x:v>550.2</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>140</x:v>
+        <x:v>183.4</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -513,25 +513,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-08-04</x:v>
+        <x:v>2026-08-05</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7645.48</x:v>
+        <x:v>7845.39</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7450.32</x:v>
+        <x:v>7567.96</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>195.2</x:v>
+        <x:v>277.4</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>296.8</x:v>
+        <x:v>574.2</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>148.4</x:v>
+        <x:v>191.4</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -542,25 +542,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-08-04</x:v>
+        <x:v>2026-08-05</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3831.94</x:v>
+        <x:v>3884.4</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3799.52</x:v>
+        <x:v>3815.12</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>32.4</x:v>
+        <x:v>69.3</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>62.4</x:v>
+        <x:v>131.7</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>31.2</x:v>
+        <x:v>43.9</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -571,25 +571,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-08-04</x:v>
+        <x:v>2026-08-05</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>7269.8</x:v>
+        <x:v>7466</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>7057.8</x:v>
+        <x:v>7201.6</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>212</x:v>
+        <x:v>264.4</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>300.2</x:v>
+        <x:v>564.6</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>150.1</x:v>
+        <x:v>188.2</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -690,7 +690,7 @@
         <x:v>2026-08-01</x:v>
       </x:c>
       <x:c r="C13" s="14" t="str">
-        <x:v>2026-08-04</x:v>
+        <x:v>2026-08-05</x:v>
       </x:c>
       <x:c r="D13" s="14" t="str">
         <x:v>数据源</x:v>
@@ -879,31 +879,31 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B5" s="22" t="str">
-        <x:v>8月3日-8月4日</x:v>
+        <x:v>8月3日-8月5日</x:v>
       </x:c>
       <x:c r="C5" s="23" t="n">
         <x:v>7055.27</x:v>
       </x:c>
       <x:c r="D5" s="23" t="n">
-        <x:v>7307.17</x:v>
+        <x:v>7523.5</x:v>
       </x:c>
       <x:c r="E5" s="23" t="n">
         <x:v>7042.89</x:v>
       </x:c>
       <x:c r="F5" s="23" t="n">
-        <x:v>7279.19</x:v>
+        <x:v>7493.05</x:v>
       </x:c>
       <x:c r="G5" s="23"/>
       <x:c r="H5" s="24"/>
       <x:c r="I5" s="26" t="n">
         <x:f>ROUND(D5-E5,1)</x:f>
-        <x:v>264.3</x:v>
+        <x:v>480.6</x:v>
       </x:c>
       <x:c r="J5" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K5" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -921,7 +921,7 @@
       <x:c r="H6" s="28"/>
       <x:c r="I6" s="30" t="n">
         <x:f>ROUND(SUM(I5:I5),1)</x:f>
-        <x:v>264.3</x:v>
+        <x:v>480.6</x:v>
       </x:c>
       <x:c r="J6" s="28"/>
       <x:c r="K6" s="28"/>
@@ -939,7 +939,7 @@
       <x:c r="H7" s="28"/>
       <x:c r="I7" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I5),0),1)</x:f>
-        <x:v>264.3</x:v>
+        <x:v>480.6</x:v>
       </x:c>
       <x:c r="J7" s="28"/>
       <x:c r="K7" s="28"/>
@@ -999,31 +999,31 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B11" s="22" t="str">
-        <x:v>8月3日-8月4日</x:v>
+        <x:v>8月3日-8月5日</x:v>
       </x:c>
       <x:c r="C11" s="23" t="n">
         <x:v>7457.12</x:v>
       </x:c>
       <x:c r="D11" s="23" t="n">
-        <x:v>7645.48</x:v>
+        <x:v>7845.39</x:v>
       </x:c>
       <x:c r="E11" s="23" t="n">
         <x:v>7397.94</x:v>
       </x:c>
       <x:c r="F11" s="23" t="n">
-        <x:v>7607.49</x:v>
+        <x:v>7809.21</x:v>
       </x:c>
       <x:c r="G11" s="23"/>
       <x:c r="H11" s="24"/>
       <x:c r="I11" s="26" t="n">
         <x:f>ROUND(D11-E11,1)</x:f>
-        <x:v>247.5</x:v>
+        <x:v>447.5</x:v>
       </x:c>
       <x:c r="J11" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K11" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -1041,7 +1041,7 @@
       <x:c r="H12" s="28"/>
       <x:c r="I12" s="30" t="n">
         <x:f>ROUND(SUM(I11:I11),1)</x:f>
-        <x:v>247.5</x:v>
+        <x:v>447.5</x:v>
       </x:c>
       <x:c r="J12" s="28"/>
       <x:c r="K12" s="28"/>
@@ -1059,7 +1059,7 @@
       <x:c r="H13" s="28"/>
       <x:c r="I13" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I11:I11),0),1)</x:f>
-        <x:v>247.5</x:v>
+        <x:v>447.5</x:v>
       </x:c>
       <x:c r="J13" s="28"/>
       <x:c r="K13" s="28"/>
@@ -1119,31 +1119,31 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B17" s="22" t="str">
-        <x:v>8月3日-8月4日</x:v>
+        <x:v>8月3日-8月5日</x:v>
       </x:c>
       <x:c r="C17" s="23" t="n">
         <x:v>3812.61</x:v>
       </x:c>
       <x:c r="D17" s="23" t="n">
-        <x:v>3831.94</x:v>
+        <x:v>3884.4</x:v>
       </x:c>
       <x:c r="E17" s="23" t="n">
         <x:v>3797.64</x:v>
       </x:c>
       <x:c r="F17" s="23" t="n">
-        <x:v>3822.28</x:v>
+        <x:v>3878.43</x:v>
       </x:c>
       <x:c r="G17" s="23"/>
       <x:c r="H17" s="24"/>
-      <x:c r="I17" s="23" t="n">
+      <x:c r="I17" s="26" t="n">
         <x:f>ROUND(D17-E17,1)</x:f>
-        <x:v>34.3</x:v>
+        <x:v>86.8</x:v>
       </x:c>
       <x:c r="J17" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K17" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -1161,7 +1161,7 @@
       <x:c r="H18" s="28"/>
       <x:c r="I18" s="30" t="n">
         <x:f>ROUND(SUM(I17:I17),1)</x:f>
-        <x:v>34.3</x:v>
+        <x:v>86.8</x:v>
       </x:c>
       <x:c r="J18" s="28"/>
       <x:c r="K18" s="28"/>
@@ -1179,7 +1179,7 @@
       <x:c r="H19" s="28"/>
       <x:c r="I19" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I17:I17),0),1)</x:f>
-        <x:v>34.3</x:v>
+        <x:v>86.8</x:v>
       </x:c>
       <x:c r="J19" s="28"/>
       <x:c r="K19" s="28"/>
@@ -1239,31 +1239,31 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B23" s="22" t="str">
-        <x:v>8月3日-8月4日</x:v>
+        <x:v>8月3日-8月5日</x:v>
       </x:c>
       <x:c r="C23" s="23" t="n">
         <x:v>7000</x:v>
       </x:c>
       <x:c r="D23" s="23" t="n">
-        <x:v>7269.8</x:v>
+        <x:v>7466</x:v>
       </x:c>
       <x:c r="E23" s="23" t="n">
         <x:v>6976</x:v>
       </x:c>
       <x:c r="F23" s="23" t="n">
-        <x:v>7211.4</x:v>
+        <x:v>7433.8</x:v>
       </x:c>
       <x:c r="G23" s="23"/>
       <x:c r="H23" s="24"/>
       <x:c r="I23" s="26" t="n">
         <x:f>ROUND(D23-E23,1)</x:f>
-        <x:v>293.8</x:v>
+        <x:v>490</x:v>
       </x:c>
       <x:c r="J23" s="22" t="str">
         <x:v>IM2609</x:v>
       </x:c>
       <x:c r="K23" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1281,7 +1281,7 @@
       <x:c r="H24" s="28"/>
       <x:c r="I24" s="30" t="n">
         <x:f>ROUND(SUM(I23:I23),1)</x:f>
-        <x:v>293.8</x:v>
+        <x:v>490</x:v>
       </x:c>
       <x:c r="J24" s="28"/>
       <x:c r="K24" s="28"/>
@@ -1299,7 +1299,7 @@
       <x:c r="H25" s="28"/>
       <x:c r="I25" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I23:I23),0),1)</x:f>
-        <x:v>293.8</x:v>
+        <x:v>490</x:v>
       </x:c>
       <x:c r="J25" s="28"/>
       <x:c r="K25" s="28"/>
@@ -1808,31 +1808,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B8" s="28" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C8" s="28"/>
-      <x:c r="D8" s="28"/>
-      <x:c r="E8" s="28"/>
-      <x:c r="F8" s="28"/>
-      <x:c r="G8" s="28"/>
-      <x:c r="H8" s="28"/>
-      <x:c r="I8" s="28"/>
-      <x:c r="J8" s="30" t="n">
-        <x:f>SUM(J4:J5)</x:f>
-        <x:v>279.9</x:v>
-      </x:c>
-      <x:c r="K8" s="28"/>
+    <x:row r="6">
+      <x:c r="A6" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B6" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C6" s="22" t="str">
+        <x:v>8月5日</x:v>
+      </x:c>
+      <x:c r="D6" s="23" t="n">
+        <x:v>7253.22</x:v>
+      </x:c>
+      <x:c r="E6" s="23" t="n">
+        <x:v>7523.5</x:v>
+      </x:c>
+      <x:c r="F6" s="23" t="n">
+        <x:v>7253.22</x:v>
+      </x:c>
+      <x:c r="G6" s="23" t="n">
+        <x:v>7493.05</x:v>
+      </x:c>
+      <x:c r="H6" s="37" t="n">
+        <x:v>213.9</x:v>
+      </x:c>
+      <x:c r="I6" s="24" t="n">
+        <x:v>0.02937964251517</x:v>
+      </x:c>
+      <x:c r="J6" s="26" t="n">
+        <x:f>ROUND(E6-F6,1)</x:f>
+        <x:v>270.3</x:v>
+      </x:c>
+      <x:c r="K6" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B9" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B9" s="28" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="C9" s="28"/>
       <x:c r="D9" s="28"/>
       <x:c r="E9" s="28"/>
@@ -1840,11 +1858,29 @@
       <x:c r="G9" s="28"/>
       <x:c r="H9" s="28"/>
       <x:c r="I9" s="28"/>
-      <x:c r="J9" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J5),0),1)</x:f>
-        <x:v>140</x:v>
+      <x:c r="J9" s="30" t="n">
+        <x:f>SUM(J4:J6)</x:f>
+        <x:v>550.2</x:v>
       </x:c>
       <x:c r="K9" s="28"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B10" s="28"/>
+      <x:c r="C10" s="28"/>
+      <x:c r="D10" s="28"/>
+      <x:c r="E10" s="28"/>
+      <x:c r="F10" s="28"/>
+      <x:c r="G10" s="28"/>
+      <x:c r="H10" s="28"/>
+      <x:c r="I10" s="28"/>
+      <x:c r="J10" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J6),0),1)</x:f>
+        <x:v>183.4</x:v>
+      </x:c>
+      <x:c r="K10" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1983,31 +2019,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B8" s="28" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C8" s="28"/>
-      <x:c r="D8" s="28"/>
-      <x:c r="E8" s="28"/>
-      <x:c r="F8" s="28"/>
-      <x:c r="G8" s="28"/>
-      <x:c r="H8" s="28"/>
-      <x:c r="I8" s="28"/>
-      <x:c r="J8" s="30" t="n">
-        <x:f>SUM(J4:J5)</x:f>
-        <x:v>296.79999999999995</x:v>
-      </x:c>
-      <x:c r="K8" s="28"/>
+    <x:row r="6">
+      <x:c r="A6" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B6" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C6" s="22" t="str">
+        <x:v>8月5日</x:v>
+      </x:c>
+      <x:c r="D6" s="23" t="n">
+        <x:v>7567.96</x:v>
+      </x:c>
+      <x:c r="E6" s="23" t="n">
+        <x:v>7845.39</x:v>
+      </x:c>
+      <x:c r="F6" s="23" t="n">
+        <x:v>7567.96</x:v>
+      </x:c>
+      <x:c r="G6" s="23" t="n">
+        <x:v>7809.21</x:v>
+      </x:c>
+      <x:c r="H6" s="37" t="n">
+        <x:v>201.7</x:v>
+      </x:c>
+      <x:c r="I6" s="24" t="n">
+        <x:v>0.026515973073904853</x:v>
+      </x:c>
+      <x:c r="J6" s="26" t="n">
+        <x:f>ROUND(E6-F6,1)</x:f>
+        <x:v>277.4</x:v>
+      </x:c>
+      <x:c r="K6" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B9" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B9" s="28" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="C9" s="28"/>
       <x:c r="D9" s="28"/>
       <x:c r="E9" s="28"/>
@@ -2015,11 +2069,29 @@
       <x:c r="G9" s="28"/>
       <x:c r="H9" s="28"/>
       <x:c r="I9" s="28"/>
-      <x:c r="J9" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J5),0),1)</x:f>
-        <x:v>148.4</x:v>
+      <x:c r="J9" s="30" t="n">
+        <x:f>SUM(J4:J6)</x:f>
+        <x:v>574.1999999999999</x:v>
       </x:c>
       <x:c r="K9" s="28"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B10" s="28"/>
+      <x:c r="C10" s="28"/>
+      <x:c r="D10" s="28"/>
+      <x:c r="E10" s="28"/>
+      <x:c r="F10" s="28"/>
+      <x:c r="G10" s="28"/>
+      <x:c r="H10" s="28"/>
+      <x:c r="I10" s="28"/>
+      <x:c r="J10" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J6),0),1)</x:f>
+        <x:v>191.4</x:v>
+      </x:c>
+      <x:c r="K10" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2158,31 +2230,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B8" s="28" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C8" s="28"/>
-      <x:c r="D8" s="28"/>
-      <x:c r="E8" s="28"/>
-      <x:c r="F8" s="28"/>
-      <x:c r="G8" s="28"/>
-      <x:c r="H8" s="28"/>
-      <x:c r="I8" s="28"/>
-      <x:c r="J8" s="30" t="n">
-        <x:f>SUM(J4:J5)</x:f>
-        <x:v>62.4</x:v>
-      </x:c>
-      <x:c r="K8" s="28"/>
+    <x:row r="6">
+      <x:c r="A6" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B6" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C6" s="22" t="str">
+        <x:v>8月5日</x:v>
+      </x:c>
+      <x:c r="D6" s="23" t="n">
+        <x:v>3815.12</x:v>
+      </x:c>
+      <x:c r="E6" s="23" t="n">
+        <x:v>3884.4</x:v>
+      </x:c>
+      <x:c r="F6" s="23" t="n">
+        <x:v>3815.12</x:v>
+      </x:c>
+      <x:c r="G6" s="23" t="n">
+        <x:v>3878.43</x:v>
+      </x:c>
+      <x:c r="H6" s="23" t="n">
+        <x:v>56.1</x:v>
+      </x:c>
+      <x:c r="I6" s="24" t="n">
+        <x:v>0.014690184915809423</x:v>
+      </x:c>
+      <x:c r="J6" s="26" t="n">
+        <x:f>ROUND(E6-F6,1)</x:f>
+        <x:v>69.3</x:v>
+      </x:c>
+      <x:c r="K6" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B9" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B9" s="28" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="C9" s="28"/>
       <x:c r="D9" s="28"/>
       <x:c r="E9" s="28"/>
@@ -2190,11 +2280,29 @@
       <x:c r="G9" s="28"/>
       <x:c r="H9" s="28"/>
       <x:c r="I9" s="28"/>
-      <x:c r="J9" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J5),0),1)</x:f>
-        <x:v>31.2</x:v>
+      <x:c r="J9" s="30" t="n">
+        <x:f>SUM(J4:J6)</x:f>
+        <x:v>131.7</x:v>
       </x:c>
       <x:c r="K9" s="28"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B10" s="28"/>
+      <x:c r="C10" s="28"/>
+      <x:c r="D10" s="28"/>
+      <x:c r="E10" s="28"/>
+      <x:c r="F10" s="28"/>
+      <x:c r="G10" s="28"/>
+      <x:c r="H10" s="28"/>
+      <x:c r="I10" s="28"/>
+      <x:c r="J10" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J6),0),1)</x:f>
+        <x:v>43.9</x:v>
+      </x:c>
+      <x:c r="K10" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2333,31 +2441,49 @@
         <x:v>IM2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B8" s="28" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C8" s="28"/>
-      <x:c r="D8" s="28"/>
-      <x:c r="E8" s="28"/>
-      <x:c r="F8" s="28"/>
-      <x:c r="G8" s="28"/>
-      <x:c r="H8" s="28"/>
-      <x:c r="I8" s="28"/>
-      <x:c r="J8" s="30" t="n">
-        <x:f>SUM(J4:J5)</x:f>
-        <x:v>300.2</x:v>
-      </x:c>
-      <x:c r="K8" s="28"/>
+    <x:row r="6">
+      <x:c r="A6" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B6" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C6" s="22" t="str">
+        <x:v>8月5日</x:v>
+      </x:c>
+      <x:c r="D6" s="23" t="n">
+        <x:v>7206.4</x:v>
+      </x:c>
+      <x:c r="E6" s="23" t="n">
+        <x:v>7466</x:v>
+      </x:c>
+      <x:c r="F6" s="23" t="n">
+        <x:v>7201.6</x:v>
+      </x:c>
+      <x:c r="G6" s="23" t="n">
+        <x:v>7433.8</x:v>
+      </x:c>
+      <x:c r="H6" s="37" t="n">
+        <x:v>222.4</x:v>
+      </x:c>
+      <x:c r="I6" s="24" t="n">
+        <x:v>0.030840058795795544</x:v>
+      </x:c>
+      <x:c r="J6" s="26" t="n">
+        <x:f>ROUND(E6-F6,1)</x:f>
+        <x:v>264.4</x:v>
+      </x:c>
+      <x:c r="K6" s="22" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B9" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B9" s="28" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="C9" s="28"/>
       <x:c r="D9" s="28"/>
       <x:c r="E9" s="28"/>
@@ -2365,11 +2491,29 @@
       <x:c r="G9" s="28"/>
       <x:c r="H9" s="28"/>
       <x:c r="I9" s="28"/>
-      <x:c r="J9" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J5),0),1)</x:f>
-        <x:v>150.1</x:v>
+      <x:c r="J9" s="30" t="n">
+        <x:f>SUM(J4:J6)</x:f>
+        <x:v>564.5999999999999</x:v>
       </x:c>
       <x:c r="K9" s="28"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B10" s="28"/>
+      <x:c r="C10" s="28"/>
+      <x:c r="D10" s="28"/>
+      <x:c r="E10" s="28"/>
+      <x:c r="F10" s="28"/>
+      <x:c r="G10" s="28"/>
+      <x:c r="H10" s="28"/>
+      <x:c r="I10" s="28"/>
+      <x:c r="J10" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J6),0),1)</x:f>
+        <x:v>188.2</x:v>
+      </x:c>
+      <x:c r="K10" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-08-06
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R050e088af8b94d03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R465de9f115cd4521"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R81f1af970a524257"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R25134676a0094044"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R3976291390ee438c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R62b9de4409a14eca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Re6a15c14b38d4385"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Ra8e5b07f1bae44eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R117c9bea0f0c456a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R7d9b43b22a204c28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rb78185570bdd4b20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R5947c31564534f85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R35ec6e0e284d4f69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R05c3b4125aff4efb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Ree85330e447047dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rd875c2d8b275472a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R1953dd6002c4483c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rc9a1dc2c613e48fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rab35406fd874445f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R6e9d04c1d47146e6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -485,25 +485,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-08-05</x:v>
+        <x:v>2026-08-06</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7523.5</x:v>
+        <x:v>7564.69</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7253.22</x:v>
+        <x:v>7434.49</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>270.3</x:v>
+        <x:v>130.2</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>550.2</x:v>
+        <x:v>680.4</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>183.4</x:v>
+        <x:v>170.1</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -514,25 +514,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-08-05</x:v>
+        <x:v>2026-08-06</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7845.39</x:v>
+        <x:v>7868.85</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7567.96</x:v>
+        <x:v>7722.57</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>277.4</x:v>
+        <x:v>146.3</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>574.2</x:v>
+        <x:v>720.5</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>191.4</x:v>
+        <x:v>180.1</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -543,25 +543,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-08-05</x:v>
+        <x:v>2026-08-06</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3884.4</x:v>
+        <x:v>3902.05</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3815.12</x:v>
+        <x:v>3864.27</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>69.3</x:v>
+        <x:v>37.8</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>131.7</x:v>
+        <x:v>169.5</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>43.9</x:v>
+        <x:v>42.4</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -601,25 +601,25 @@
         <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>2026-08-05</x:v>
+        <x:v>2026-08-06</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:v>7775.6</x:v>
+        <x:v>7768</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>7501</x:v>
+        <x:v>7640</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>274.6</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>585.8</x:v>
+        <x:v>713.8</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
-        <x:v>195.3</x:v>
+        <x:v>178.5</x:v>
       </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
@@ -688,25 +688,25 @@
         <x:v>碳酸锂2609</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>2026-08-05</x:v>
+        <x:v>2026-08-06</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:v>144300</x:v>
+        <x:v>143860</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
-        <x:v>138320</x:v>
+        <x:v>139240</x:v>
       </x:c>
       <x:c r="E11" s="12" t="n">
-        <x:v>5980</x:v>
+        <x:v>4620</x:v>
       </x:c>
       <x:c r="F11" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G11" s="10" t="n">
-        <x:v>15280</x:v>
+        <x:v>19900</x:v>
       </x:c>
       <x:c r="H11" s="10" t="n">
-        <x:v>5093.3</x:v>
+        <x:v>4975</x:v>
       </x:c>
       <x:c r="I11" s="10" t="n">
         <x:v>6000</x:v>
@@ -720,7 +720,7 @@
         <x:v>2026-08-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-08-05</x:v>
+        <x:v>2026-08-06</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1011,31 +1011,49 @@
         <x:v>LC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B9" s="28" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C9" s="28"/>
-      <x:c r="D9" s="28"/>
-      <x:c r="E9" s="28"/>
-      <x:c r="F9" s="28"/>
-      <x:c r="G9" s="28"/>
-      <x:c r="H9" s="28"/>
-      <x:c r="I9" s="28"/>
-      <x:c r="J9" s="30" t="n">
-        <x:f>SUM(J4:J6)</x:f>
-        <x:v>15280</x:v>
-      </x:c>
-      <x:c r="K9" s="28"/>
+    <x:row r="7">
+      <x:c r="A7" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C7" s="22" t="str">
+        <x:v>8月6日</x:v>
+      </x:c>
+      <x:c r="D7" s="23" t="n">
+        <x:v>143200</x:v>
+      </x:c>
+      <x:c r="E7" s="23" t="n">
+        <x:v>143860</x:v>
+      </x:c>
+      <x:c r="F7" s="23" t="n">
+        <x:v>139240</x:v>
+      </x:c>
+      <x:c r="G7" s="23" t="n">
+        <x:v>141460</x:v>
+      </x:c>
+      <x:c r="H7" s="37" t="n">
+        <x:v>-1760</x:v>
+      </x:c>
+      <x:c r="I7" s="24" t="n">
+        <x:v>-0.01228878648233489</x:v>
+      </x:c>
+      <x:c r="J7" s="23" t="n">
+        <x:f>ROUND(E7-F7,1)</x:f>
+        <x:v>4620</x:v>
+      </x:c>
+      <x:c r="K7" s="22" t="str">
+        <x:v>LC2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B10" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B10" s="28" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="C10" s="28"/>
       <x:c r="D10" s="28"/>
       <x:c r="E10" s="28"/>
@@ -1043,11 +1061,29 @@
       <x:c r="G10" s="28"/>
       <x:c r="H10" s="28"/>
       <x:c r="I10" s="28"/>
-      <x:c r="J10" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J6),0),1)</x:f>
-        <x:v>5093.3</x:v>
+      <x:c r="J10" s="30" t="n">
+        <x:f>SUM(J4:J7)</x:f>
+        <x:v>19900</x:v>
       </x:c>
       <x:c r="K10" s="28"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B11" s="28"/>
+      <x:c r="C11" s="28"/>
+      <x:c r="D11" s="28"/>
+      <x:c r="E11" s="28"/>
+      <x:c r="F11" s="28"/>
+      <x:c r="G11" s="28"/>
+      <x:c r="H11" s="28"/>
+      <x:c r="I11" s="28"/>
+      <x:c r="J11" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
+        <x:v>4975</x:v>
+      </x:c>
+      <x:c r="K11" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1134,31 +1170,31 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B5" s="22" t="str">
-        <x:v>8月3日-8月5日</x:v>
+        <x:v>8月3日-8月6日</x:v>
       </x:c>
       <x:c r="C5" s="23" t="n">
         <x:v>7055.27</x:v>
       </x:c>
       <x:c r="D5" s="23" t="n">
-        <x:v>7523.5</x:v>
+        <x:v>7564.69</x:v>
       </x:c>
       <x:c r="E5" s="23" t="n">
         <x:v>7042.89</x:v>
       </x:c>
       <x:c r="F5" s="23" t="n">
-        <x:v>7493.05</x:v>
+        <x:v>7530.43</x:v>
       </x:c>
       <x:c r="G5" s="23"/>
       <x:c r="H5" s="24"/>
       <x:c r="I5" s="26" t="n">
         <x:f>ROUND(D5-E5,1)</x:f>
-        <x:v>480.6</x:v>
+        <x:v>521.8</x:v>
       </x:c>
       <x:c r="J5" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K5" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -1176,7 +1212,7 @@
       <x:c r="H6" s="28"/>
       <x:c r="I6" s="30" t="n">
         <x:f>ROUND(SUM(I5:I5),1)</x:f>
-        <x:v>480.6</x:v>
+        <x:v>521.8</x:v>
       </x:c>
       <x:c r="J6" s="28"/>
       <x:c r="K6" s="28"/>
@@ -1194,7 +1230,7 @@
       <x:c r="H7" s="28"/>
       <x:c r="I7" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I5),0),1)</x:f>
-        <x:v>480.6</x:v>
+        <x:v>521.8</x:v>
       </x:c>
       <x:c r="J7" s="28"/>
       <x:c r="K7" s="28"/>
@@ -1254,31 +1290,31 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B11" s="22" t="str">
-        <x:v>8月3日-8月5日</x:v>
+        <x:v>8月3日-8月6日</x:v>
       </x:c>
       <x:c r="C11" s="23" t="n">
         <x:v>7457.12</x:v>
       </x:c>
       <x:c r="D11" s="23" t="n">
-        <x:v>7845.39</x:v>
+        <x:v>7868.85</x:v>
       </x:c>
       <x:c r="E11" s="23" t="n">
         <x:v>7397.94</x:v>
       </x:c>
       <x:c r="F11" s="23" t="n">
-        <x:v>7809.21</x:v>
+        <x:v>7829.36</x:v>
       </x:c>
       <x:c r="G11" s="23"/>
       <x:c r="H11" s="24"/>
       <x:c r="I11" s="26" t="n">
         <x:f>ROUND(D11-E11,1)</x:f>
-        <x:v>447.5</x:v>
+        <x:v>470.9</x:v>
       </x:c>
       <x:c r="J11" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K11" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -1296,7 +1332,7 @@
       <x:c r="H12" s="28"/>
       <x:c r="I12" s="30" t="n">
         <x:f>ROUND(SUM(I11:I11),1)</x:f>
-        <x:v>447.5</x:v>
+        <x:v>470.9</x:v>
       </x:c>
       <x:c r="J12" s="28"/>
       <x:c r="K12" s="28"/>
@@ -1314,7 +1350,7 @@
       <x:c r="H13" s="28"/>
       <x:c r="I13" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I11:I11),0),1)</x:f>
-        <x:v>447.5</x:v>
+        <x:v>470.9</x:v>
       </x:c>
       <x:c r="J13" s="28"/>
       <x:c r="K13" s="28"/>
@@ -1374,31 +1410,31 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B17" s="22" t="str">
-        <x:v>8月3日-8月5日</x:v>
+        <x:v>8月3日-8月6日</x:v>
       </x:c>
       <x:c r="C17" s="23" t="n">
         <x:v>3812.61</x:v>
       </x:c>
       <x:c r="D17" s="23" t="n">
-        <x:v>3884.4</x:v>
+        <x:v>3902.05</x:v>
       </x:c>
       <x:c r="E17" s="23" t="n">
         <x:v>3797.64</x:v>
       </x:c>
       <x:c r="F17" s="23" t="n">
-        <x:v>3878.43</x:v>
+        <x:v>3900.35</x:v>
       </x:c>
       <x:c r="G17" s="23"/>
       <x:c r="H17" s="24"/>
       <x:c r="I17" s="26" t="n">
         <x:f>ROUND(D17-E17,1)</x:f>
-        <x:v>86.8</x:v>
+        <x:v>104.4</x:v>
       </x:c>
       <x:c r="J17" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K17" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -1416,7 +1452,7 @@
       <x:c r="H18" s="28"/>
       <x:c r="I18" s="30" t="n">
         <x:f>ROUND(SUM(I17:I17),1)</x:f>
-        <x:v>86.8</x:v>
+        <x:v>104.4</x:v>
       </x:c>
       <x:c r="J18" s="28"/>
       <x:c r="K18" s="28"/>
@@ -1434,7 +1470,7 @@
       <x:c r="H19" s="28"/>
       <x:c r="I19" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I17:I17),0),1)</x:f>
-        <x:v>86.8</x:v>
+        <x:v>104.4</x:v>
       </x:c>
       <x:c r="J19" s="28"/>
       <x:c r="K19" s="28"/>
@@ -1614,7 +1650,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B29" s="22" t="str">
-        <x:v>8月3日-8月5日</x:v>
+        <x:v>8月3日-8月6日</x:v>
       </x:c>
       <x:c r="C29" s="23" t="n">
         <x:v>7391</x:v>
@@ -1626,7 +1662,7 @@
         <x:v>7335</x:v>
       </x:c>
       <x:c r="F29" s="23" t="n">
-        <x:v>7744.4</x:v>
+        <x:v>7730</x:v>
       </x:c>
       <x:c r="G29" s="23"/>
       <x:c r="H29" s="24"/>
@@ -1638,7 +1674,7 @@
         <x:v>IC2609</x:v>
       </x:c>
       <x:c r="K29" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -1974,7 +2010,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B47" s="22" t="str">
-        <x:v>8月3日-8月5日</x:v>
+        <x:v>8月3日-8月6日</x:v>
       </x:c>
       <x:c r="C47" s="23" t="n">
         <x:v>137500</x:v>
@@ -1986,7 +2022,7 @@
         <x:v>135560</x:v>
       </x:c>
       <x:c r="F47" s="23" t="n">
-        <x:v>143220</x:v>
+        <x:v>141460</x:v>
       </x:c>
       <x:c r="G47" s="23"/>
       <x:c r="H47" s="24"/>
@@ -1998,7 +2034,7 @@
         <x:v>LC2609</x:v>
       </x:c>
       <x:c r="K47" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -2220,31 +2256,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B9" s="28" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C9" s="28"/>
-      <x:c r="D9" s="28"/>
-      <x:c r="E9" s="28"/>
-      <x:c r="F9" s="28"/>
-      <x:c r="G9" s="28"/>
-      <x:c r="H9" s="28"/>
-      <x:c r="I9" s="28"/>
-      <x:c r="J9" s="30" t="n">
-        <x:f>SUM(J4:J6)</x:f>
-        <x:v>550.2</x:v>
-      </x:c>
-      <x:c r="K9" s="28"/>
+    <x:row r="7">
+      <x:c r="A7" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C7" s="22" t="str">
+        <x:v>8月6日</x:v>
+      </x:c>
+      <x:c r="D7" s="23" t="n">
+        <x:v>7440.01</x:v>
+      </x:c>
+      <x:c r="E7" s="23" t="n">
+        <x:v>7564.69</x:v>
+      </x:c>
+      <x:c r="F7" s="23" t="n">
+        <x:v>7434.49</x:v>
+      </x:c>
+      <x:c r="G7" s="23" t="n">
+        <x:v>7530.43</x:v>
+      </x:c>
+      <x:c r="H7" s="23" t="n">
+        <x:v>37.4</x:v>
+      </x:c>
+      <x:c r="I7" s="24" t="n">
+        <x:v>0.004988622790452535</x:v>
+      </x:c>
+      <x:c r="J7" s="23" t="n">
+        <x:f>ROUND(E7-F7,1)</x:f>
+        <x:v>130.2</x:v>
+      </x:c>
+      <x:c r="K7" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B10" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B10" s="28" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="C10" s="28"/>
       <x:c r="D10" s="28"/>
       <x:c r="E10" s="28"/>
@@ -2252,11 +2306,29 @@
       <x:c r="G10" s="28"/>
       <x:c r="H10" s="28"/>
       <x:c r="I10" s="28"/>
-      <x:c r="J10" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J6),0),1)</x:f>
-        <x:v>183.4</x:v>
+      <x:c r="J10" s="30" t="n">
+        <x:f>SUM(J4:J7)</x:f>
+        <x:v>680.4000000000001</x:v>
       </x:c>
       <x:c r="K10" s="28"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B11" s="28"/>
+      <x:c r="C11" s="28"/>
+      <x:c r="D11" s="28"/>
+      <x:c r="E11" s="28"/>
+      <x:c r="F11" s="28"/>
+      <x:c r="G11" s="28"/>
+      <x:c r="H11" s="28"/>
+      <x:c r="I11" s="28"/>
+      <x:c r="J11" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
+        <x:v>170.1</x:v>
+      </x:c>
+      <x:c r="K11" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2431,31 +2503,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B9" s="28" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C9" s="28"/>
-      <x:c r="D9" s="28"/>
-      <x:c r="E9" s="28"/>
-      <x:c r="F9" s="28"/>
-      <x:c r="G9" s="28"/>
-      <x:c r="H9" s="28"/>
-      <x:c r="I9" s="28"/>
-      <x:c r="J9" s="30" t="n">
-        <x:f>SUM(J4:J6)</x:f>
-        <x:v>574.1999999999999</x:v>
-      </x:c>
-      <x:c r="K9" s="28"/>
+    <x:row r="7">
+      <x:c r="A7" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C7" s="22" t="str">
+        <x:v>8月6日</x:v>
+      </x:c>
+      <x:c r="D7" s="23" t="n">
+        <x:v>7737.59</x:v>
+      </x:c>
+      <x:c r="E7" s="23" t="n">
+        <x:v>7868.85</x:v>
+      </x:c>
+      <x:c r="F7" s="23" t="n">
+        <x:v>7722.57</x:v>
+      </x:c>
+      <x:c r="G7" s="23" t="n">
+        <x:v>7829.36</x:v>
+      </x:c>
+      <x:c r="H7" s="23" t="n">
+        <x:v>20.1</x:v>
+      </x:c>
+      <x:c r="I7" s="24" t="n">
+        <x:v>0.0025802866102973</x:v>
+      </x:c>
+      <x:c r="J7" s="23" t="n">
+        <x:f>ROUND(E7-F7,1)</x:f>
+        <x:v>146.3</x:v>
+      </x:c>
+      <x:c r="K7" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B10" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B10" s="28" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="C10" s="28"/>
       <x:c r="D10" s="28"/>
       <x:c r="E10" s="28"/>
@@ -2463,11 +2553,29 @@
       <x:c r="G10" s="28"/>
       <x:c r="H10" s="28"/>
       <x:c r="I10" s="28"/>
-      <x:c r="J10" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J6),0),1)</x:f>
-        <x:v>191.4</x:v>
+      <x:c r="J10" s="30" t="n">
+        <x:f>SUM(J4:J7)</x:f>
+        <x:v>720.5</x:v>
       </x:c>
       <x:c r="K10" s="28"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B11" s="28"/>
+      <x:c r="C11" s="28"/>
+      <x:c r="D11" s="28"/>
+      <x:c r="E11" s="28"/>
+      <x:c r="F11" s="28"/>
+      <x:c r="G11" s="28"/>
+      <x:c r="H11" s="28"/>
+      <x:c r="I11" s="28"/>
+      <x:c r="J11" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
+        <x:v>180.1</x:v>
+      </x:c>
+      <x:c r="K11" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2642,31 +2750,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B9" s="28" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C9" s="28"/>
-      <x:c r="D9" s="28"/>
-      <x:c r="E9" s="28"/>
-      <x:c r="F9" s="28"/>
-      <x:c r="G9" s="28"/>
-      <x:c r="H9" s="28"/>
-      <x:c r="I9" s="28"/>
-      <x:c r="J9" s="30" t="n">
-        <x:f>SUM(J4:J6)</x:f>
-        <x:v>131.7</x:v>
-      </x:c>
-      <x:c r="K9" s="28"/>
+    <x:row r="7">
+      <x:c r="A7" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C7" s="22" t="str">
+        <x:v>8月6日</x:v>
+      </x:c>
+      <x:c r="D7" s="23" t="n">
+        <x:v>3864.27</x:v>
+      </x:c>
+      <x:c r="E7" s="23" t="n">
+        <x:v>3902.05</x:v>
+      </x:c>
+      <x:c r="F7" s="23" t="n">
+        <x:v>3864.27</x:v>
+      </x:c>
+      <x:c r="G7" s="23" t="n">
+        <x:v>3900.35</x:v>
+      </x:c>
+      <x:c r="H7" s="23" t="n">
+        <x:v>21.9</x:v>
+      </x:c>
+      <x:c r="I7" s="24" t="n">
+        <x:v>0.005651771464226574</x:v>
+      </x:c>
+      <x:c r="J7" s="23" t="n">
+        <x:f>ROUND(E7-F7,1)</x:f>
+        <x:v>37.8</x:v>
+      </x:c>
+      <x:c r="K7" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B10" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B10" s="28" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="C10" s="28"/>
       <x:c r="D10" s="28"/>
       <x:c r="E10" s="28"/>
@@ -2674,11 +2800,29 @@
       <x:c r="G10" s="28"/>
       <x:c r="H10" s="28"/>
       <x:c r="I10" s="28"/>
-      <x:c r="J10" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J6),0),1)</x:f>
-        <x:v>43.9</x:v>
+      <x:c r="J10" s="30" t="n">
+        <x:f>SUM(J4:J7)</x:f>
+        <x:v>169.5</x:v>
       </x:c>
       <x:c r="K10" s="28"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B11" s="28"/>
+      <x:c r="C11" s="28"/>
+      <x:c r="D11" s="28"/>
+      <x:c r="E11" s="28"/>
+      <x:c r="F11" s="28"/>
+      <x:c r="G11" s="28"/>
+      <x:c r="H11" s="28"/>
+      <x:c r="I11" s="28"/>
+      <x:c r="J11" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
+        <x:v>42.4</x:v>
+      </x:c>
+      <x:c r="K11" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3064,31 +3208,49 @@
         <x:v>IC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B9" s="28" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C9" s="28"/>
-      <x:c r="D9" s="28"/>
-      <x:c r="E9" s="28"/>
-      <x:c r="F9" s="28"/>
-      <x:c r="G9" s="28"/>
-      <x:c r="H9" s="28"/>
-      <x:c r="I9" s="28"/>
-      <x:c r="J9" s="30" t="n">
-        <x:f>SUM(J4:J6)</x:f>
-        <x:v>585.8</x:v>
-      </x:c>
-      <x:c r="K9" s="28"/>
+    <x:row r="7">
+      <x:c r="A7" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C7" s="22" t="str">
+        <x:v>8月6日</x:v>
+      </x:c>
+      <x:c r="D7" s="23" t="n">
+        <x:v>7680</x:v>
+      </x:c>
+      <x:c r="E7" s="23" t="n">
+        <x:v>7768</x:v>
+      </x:c>
+      <x:c r="F7" s="23" t="n">
+        <x:v>7640</x:v>
+      </x:c>
+      <x:c r="G7" s="23" t="n">
+        <x:v>7730</x:v>
+      </x:c>
+      <x:c r="H7" s="23" t="n">
+        <x:v>-14.4</x:v>
+      </x:c>
+      <x:c r="I7" s="24" t="n">
+        <x:v>-0.0018594080884251074</x:v>
+      </x:c>
+      <x:c r="J7" s="23" t="n">
+        <x:f>ROUND(E7-F7,1)</x:f>
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="K7" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B10" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B10" s="28" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="C10" s="28"/>
       <x:c r="D10" s="28"/>
       <x:c r="E10" s="28"/>
@@ -3096,11 +3258,29 @@
       <x:c r="G10" s="28"/>
       <x:c r="H10" s="28"/>
       <x:c r="I10" s="28"/>
-      <x:c r="J10" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J6),0),1)</x:f>
-        <x:v>195.3</x:v>
+      <x:c r="J10" s="30" t="n">
+        <x:f>SUM(J4:J7)</x:f>
+        <x:v>713.8</x:v>
       </x:c>
       <x:c r="K10" s="28"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B11" s="28"/>
+      <x:c r="C11" s="28"/>
+      <x:c r="D11" s="28"/>
+      <x:c r="E11" s="28"/>
+      <x:c r="F11" s="28"/>
+      <x:c r="G11" s="28"/>
+      <x:c r="H11" s="28"/>
+      <x:c r="I11" s="28"/>
+      <x:c r="J11" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
+        <x:v>178.5</x:v>
+      </x:c>
+      <x:c r="K11" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-08-07
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rd954db5c203b4c23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R63f629d4db004466"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Rc8346addf64e4490"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rbbd1989b967045b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R3ee85475db4e4aa8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R280341ffd4b2417c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Rb492177ff26e4fb6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rca296e2dbc04435c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Re860cb81a6fb43d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R4c27490ccbed44fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R1d2889df289e4ee6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Ra05660a161d049da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R5c528b319b864486"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R5235475ce1774ee4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R711ebb90def1424a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rae8ebbdf65194b63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R4e147531b7f8442f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rb9f85e892ee14271"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R2105fbcfd5a9426f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R610f1ffae85947af"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -485,25 +485,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-08-06</x:v>
+        <x:v>2026-08-07</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7564.69</x:v>
+        <x:v>7685.57</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7434.49</x:v>
+        <x:v>7448.46</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>130.2</x:v>
+        <x:v>237.1</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>680.4</x:v>
+        <x:v>917.5</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>170.1</x:v>
+        <x:v>183.5</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -514,25 +514,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-08-06</x:v>
+        <x:v>2026-08-07</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7868.85</x:v>
+        <x:v>7983.17</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7722.57</x:v>
+        <x:v>7763.53</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>146.3</x:v>
+        <x:v>219.6</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>720.5</x:v>
+        <x:v>940.1</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>180.1</x:v>
+        <x:v>188</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -543,25 +543,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-08-06</x:v>
+        <x:v>2026-08-07</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3902.05</x:v>
+        <x:v>3940.93</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3864.27</x:v>
+        <x:v>3885.62</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>37.8</x:v>
+        <x:v>55.3</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>169.5</x:v>
+        <x:v>224.8</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>42.4</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -572,25 +572,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-08-06</x:v>
+        <x:v>2026-08-07</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>7477</x:v>
+        <x:v>7594.2</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>7352</x:v>
+        <x:v>7369</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>125</x:v>
+        <x:v>225.2</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>689.6</x:v>
+        <x:v>914.8</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>172.4</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -630,25 +630,25 @@
         <x:v>IF主力</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>2026-08-06</x:v>
+        <x:v>2026-08-07</x:v>
       </x:c>
       <x:c r="C9" s="10" t="n">
-        <x:v>4626</x:v>
+        <x:v>4656.2</x:v>
       </x:c>
       <x:c r="D9" s="10" t="n">
-        <x:v>4570.8</x:v>
+        <x:v>4604.6</x:v>
       </x:c>
       <x:c r="E9" s="12" t="n">
-        <x:v>55.2</x:v>
+        <x:v>51.6</x:v>
       </x:c>
       <x:c r="F9" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G9" s="10" t="n">
-        <x:v>276.8</x:v>
+        <x:v>328.4</x:v>
       </x:c>
       <x:c r="H9" s="10" t="n">
-        <x:v>69.2</x:v>
+        <x:v>65.7</x:v>
       </x:c>
       <x:c r="I9" s="10" t="n">
         <x:v>90</x:v>
@@ -659,25 +659,25 @@
         <x:v>IH主力</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>2026-08-06</x:v>
+        <x:v>2026-08-07</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:v>2897.8</x:v>
+        <x:v>2930.6</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
-        <x:v>2879.8</x:v>
+        <x:v>2884</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
-        <x:v>18</x:v>
+        <x:v>46.6</x:v>
       </x:c>
       <x:c r="F10" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G10" s="10" t="n">
-        <x:v>140.2</x:v>
+        <x:v>186.8</x:v>
       </x:c>
       <x:c r="H10" s="10" t="n">
-        <x:v>35.1</x:v>
+        <x:v>37.4</x:v>
       </x:c>
       <x:c r="I10" s="10" t="n">
         <x:v>60</x:v>
@@ -688,25 +688,25 @@
         <x:v>碳酸锂2609</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>2026-08-06</x:v>
+        <x:v>2026-08-07</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:v>143860</x:v>
+        <x:v>144800</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
-        <x:v>139240</x:v>
+        <x:v>139600</x:v>
       </x:c>
       <x:c r="E11" s="12" t="n">
-        <x:v>4620</x:v>
+        <x:v>5200</x:v>
       </x:c>
       <x:c r="F11" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G11" s="10" t="n">
-        <x:v>19900</x:v>
+        <x:v>25100</x:v>
       </x:c>
       <x:c r="H11" s="10" t="n">
-        <x:v>4975</x:v>
+        <x:v>5020</x:v>
       </x:c>
       <x:c r="I11" s="10" t="n">
         <x:v>6000</x:v>
@@ -720,7 +720,7 @@
         <x:v>2026-08-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-08-06</x:v>
+        <x:v>2026-08-07</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1047,31 +1047,49 @@
         <x:v>LC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B10" s="28" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C10" s="28"/>
-      <x:c r="D10" s="28"/>
-      <x:c r="E10" s="28"/>
-      <x:c r="F10" s="28"/>
-      <x:c r="G10" s="28"/>
-      <x:c r="H10" s="28"/>
-      <x:c r="I10" s="28"/>
-      <x:c r="J10" s="30" t="n">
-        <x:f>SUM(J4:J7)</x:f>
-        <x:v>19900</x:v>
-      </x:c>
-      <x:c r="K10" s="28"/>
+    <x:row r="8">
+      <x:c r="A8" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C8" s="22" t="str">
+        <x:v>8月7日</x:v>
+      </x:c>
+      <x:c r="D8" s="23" t="n">
+        <x:v>142920</x:v>
+      </x:c>
+      <x:c r="E8" s="23" t="n">
+        <x:v>144800</x:v>
+      </x:c>
+      <x:c r="F8" s="23" t="n">
+        <x:v>139600</x:v>
+      </x:c>
+      <x:c r="G8" s="23" t="n">
+        <x:v>140000</x:v>
+      </x:c>
+      <x:c r="H8" s="37" t="n">
+        <x:v>-1460</x:v>
+      </x:c>
+      <x:c r="I8" s="24" t="n">
+        <x:v>-0.01032093878128093</x:v>
+      </x:c>
+      <x:c r="J8" s="23" t="n">
+        <x:f>ROUND(E8-F8,1)</x:f>
+        <x:v>5200</x:v>
+      </x:c>
+      <x:c r="K8" s="22" t="str">
+        <x:v>LC2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B11" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B11" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
       <x:c r="C11" s="28"/>
       <x:c r="D11" s="28"/>
       <x:c r="E11" s="28"/>
@@ -1079,11 +1097,29 @@
       <x:c r="G11" s="28"/>
       <x:c r="H11" s="28"/>
       <x:c r="I11" s="28"/>
-      <x:c r="J11" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
-        <x:v>4975</x:v>
+      <x:c r="J11" s="30" t="n">
+        <x:f>SUM(J4:J8)</x:f>
+        <x:v>25100</x:v>
       </x:c>
       <x:c r="K11" s="28"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B12" s="28"/>
+      <x:c r="C12" s="28"/>
+      <x:c r="D12" s="28"/>
+      <x:c r="E12" s="28"/>
+      <x:c r="F12" s="28"/>
+      <x:c r="G12" s="28"/>
+      <x:c r="H12" s="28"/>
+      <x:c r="I12" s="28"/>
+      <x:c r="J12" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
+        <x:v>5020</x:v>
+      </x:c>
+      <x:c r="K12" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1170,31 +1206,31 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B5" s="22" t="str">
-        <x:v>8月3日-8月6日</x:v>
+        <x:v>8月3日-8月7日</x:v>
       </x:c>
       <x:c r="C5" s="23" t="n">
         <x:v>7055.27</x:v>
       </x:c>
       <x:c r="D5" s="23" t="n">
-        <x:v>7564.69</x:v>
+        <x:v>7685.57</x:v>
       </x:c>
       <x:c r="E5" s="23" t="n">
         <x:v>7042.89</x:v>
       </x:c>
       <x:c r="F5" s="23" t="n">
-        <x:v>7530.43</x:v>
+        <x:v>7679.53</x:v>
       </x:c>
       <x:c r="G5" s="23"/>
       <x:c r="H5" s="24"/>
       <x:c r="I5" s="26" t="n">
         <x:f>ROUND(D5-E5,1)</x:f>
-        <x:v>521.8</x:v>
+        <x:v>642.7</x:v>
       </x:c>
       <x:c r="J5" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K5" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -1212,7 +1248,7 @@
       <x:c r="H6" s="28"/>
       <x:c r="I6" s="30" t="n">
         <x:f>ROUND(SUM(I5:I5),1)</x:f>
-        <x:v>521.8</x:v>
+        <x:v>642.7</x:v>
       </x:c>
       <x:c r="J6" s="28"/>
       <x:c r="K6" s="28"/>
@@ -1230,7 +1266,7 @@
       <x:c r="H7" s="28"/>
       <x:c r="I7" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I5),0),1)</x:f>
-        <x:v>521.8</x:v>
+        <x:v>642.7</x:v>
       </x:c>
       <x:c r="J7" s="28"/>
       <x:c r="K7" s="28"/>
@@ -1290,31 +1326,31 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B11" s="22" t="str">
-        <x:v>8月3日-8月6日</x:v>
+        <x:v>8月3日-8月7日</x:v>
       </x:c>
       <x:c r="C11" s="23" t="n">
         <x:v>7457.12</x:v>
       </x:c>
       <x:c r="D11" s="23" t="n">
-        <x:v>7868.85</x:v>
+        <x:v>7983.17</x:v>
       </x:c>
       <x:c r="E11" s="23" t="n">
         <x:v>7397.94</x:v>
       </x:c>
       <x:c r="F11" s="23" t="n">
-        <x:v>7829.36</x:v>
+        <x:v>7980.12</x:v>
       </x:c>
       <x:c r="G11" s="23"/>
       <x:c r="H11" s="24"/>
       <x:c r="I11" s="26" t="n">
         <x:f>ROUND(D11-E11,1)</x:f>
-        <x:v>470.9</x:v>
+        <x:v>585.2</x:v>
       </x:c>
       <x:c r="J11" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K11" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -1332,7 +1368,7 @@
       <x:c r="H12" s="28"/>
       <x:c r="I12" s="30" t="n">
         <x:f>ROUND(SUM(I11:I11),1)</x:f>
-        <x:v>470.9</x:v>
+        <x:v>585.2</x:v>
       </x:c>
       <x:c r="J12" s="28"/>
       <x:c r="K12" s="28"/>
@@ -1350,7 +1386,7 @@
       <x:c r="H13" s="28"/>
       <x:c r="I13" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I11:I11),0),1)</x:f>
-        <x:v>470.9</x:v>
+        <x:v>585.2</x:v>
       </x:c>
       <x:c r="J13" s="28"/>
       <x:c r="K13" s="28"/>
@@ -1410,31 +1446,31 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B17" s="22" t="str">
-        <x:v>8月3日-8月6日</x:v>
+        <x:v>8月3日-8月7日</x:v>
       </x:c>
       <x:c r="C17" s="23" t="n">
         <x:v>3812.61</x:v>
       </x:c>
       <x:c r="D17" s="23" t="n">
-        <x:v>3902.05</x:v>
+        <x:v>3940.93</x:v>
       </x:c>
       <x:c r="E17" s="23" t="n">
         <x:v>3797.64</x:v>
       </x:c>
       <x:c r="F17" s="23" t="n">
-        <x:v>3900.35</x:v>
+        <x:v>3940.04</x:v>
       </x:c>
       <x:c r="G17" s="23"/>
       <x:c r="H17" s="24"/>
       <x:c r="I17" s="26" t="n">
         <x:f>ROUND(D17-E17,1)</x:f>
-        <x:v>104.4</x:v>
+        <x:v>143.3</x:v>
       </x:c>
       <x:c r="J17" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K17" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -1452,7 +1488,7 @@
       <x:c r="H18" s="28"/>
       <x:c r="I18" s="30" t="n">
         <x:f>ROUND(SUM(I17:I17),1)</x:f>
-        <x:v>104.4</x:v>
+        <x:v>143.3</x:v>
       </x:c>
       <x:c r="J18" s="28"/>
       <x:c r="K18" s="28"/>
@@ -1470,7 +1506,7 @@
       <x:c r="H19" s="28"/>
       <x:c r="I19" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I17:I17),0),1)</x:f>
-        <x:v>104.4</x:v>
+        <x:v>143.3</x:v>
       </x:c>
       <x:c r="J19" s="28"/>
       <x:c r="K19" s="28"/>
@@ -1530,31 +1566,31 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B23" s="22" t="str">
-        <x:v>8月3日-8月6日</x:v>
+        <x:v>8月3日-8月7日</x:v>
       </x:c>
       <x:c r="C23" s="23" t="n">
         <x:v>7000</x:v>
       </x:c>
       <x:c r="D23" s="23" t="n">
-        <x:v>7477</x:v>
+        <x:v>7594.2</x:v>
       </x:c>
       <x:c r="E23" s="23" t="n">
         <x:v>6976</x:v>
       </x:c>
       <x:c r="F23" s="23" t="n">
-        <x:v>7451.8</x:v>
+        <x:v>7590.6</x:v>
       </x:c>
       <x:c r="G23" s="23"/>
       <x:c r="H23" s="24"/>
       <x:c r="I23" s="26" t="n">
         <x:f>ROUND(D23-E23,1)</x:f>
-        <x:v>501</x:v>
+        <x:v>618.2</x:v>
       </x:c>
       <x:c r="J23" s="22" t="str">
         <x:v>IM2609</x:v>
       </x:c>
       <x:c r="K23" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1572,7 +1608,7 @@
       <x:c r="H24" s="28"/>
       <x:c r="I24" s="30" t="n">
         <x:f>ROUND(SUM(I23:I23),1)</x:f>
-        <x:v>501</x:v>
+        <x:v>618.2</x:v>
       </x:c>
       <x:c r="J24" s="28"/>
       <x:c r="K24" s="28"/>
@@ -1590,7 +1626,7 @@
       <x:c r="H25" s="28"/>
       <x:c r="I25" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I23:I23),0),1)</x:f>
-        <x:v>501</x:v>
+        <x:v>618.2</x:v>
       </x:c>
       <x:c r="J25" s="28"/>
       <x:c r="K25" s="28"/>
@@ -1770,31 +1806,31 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B35" s="22" t="str">
-        <x:v>8月3日-8月6日</x:v>
+        <x:v>8月3日-8月7日</x:v>
       </x:c>
       <x:c r="C35" s="23" t="n">
         <x:v>4526.4</x:v>
       </x:c>
       <x:c r="D35" s="23" t="n">
-        <x:v>4641.2</x:v>
+        <x:v>4656.2</x:v>
       </x:c>
       <x:c r="E35" s="23" t="n">
         <x:v>4494.2</x:v>
       </x:c>
       <x:c r="F35" s="23" t="n">
-        <x:v>4612</x:v>
+        <x:v>4645.6</x:v>
       </x:c>
       <x:c r="G35" s="23"/>
       <x:c r="H35" s="24"/>
       <x:c r="I35" s="26" t="n">
         <x:f>ROUND(D35-E35,1)</x:f>
-        <x:v>147</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="J35" s="22" t="str">
         <x:v>IF2609</x:v>
       </x:c>
       <x:c r="K35" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -1812,7 +1848,7 @@
       <x:c r="H36" s="28"/>
       <x:c r="I36" s="30" t="n">
         <x:f>ROUND(SUM(I35:I35),1)</x:f>
-        <x:v>147</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="J36" s="28"/>
       <x:c r="K36" s="28"/>
@@ -1830,7 +1866,7 @@
       <x:c r="H37" s="28"/>
       <x:c r="I37" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I35:I35),0),1)</x:f>
-        <x:v>147</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="J37" s="28"/>
       <x:c r="K37" s="28"/>
@@ -1890,31 +1926,31 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B41" s="22" t="str">
-        <x:v>8月3日-8月6日</x:v>
+        <x:v>8月3日-8月7日</x:v>
       </x:c>
       <x:c r="C41" s="23" t="n">
         <x:v>2882.4</x:v>
       </x:c>
       <x:c r="D41" s="23" t="n">
-        <x:v>2907.6</x:v>
+        <x:v>2930.6</x:v>
       </x:c>
       <x:c r="E41" s="23" t="n">
         <x:v>2845.8</x:v>
       </x:c>
       <x:c r="F41" s="23" t="n">
-        <x:v>2897.2</x:v>
+        <x:v>2930</x:v>
       </x:c>
       <x:c r="G41" s="23"/>
       <x:c r="H41" s="24"/>
       <x:c r="I41" s="26" t="n">
         <x:f>ROUND(D41-E41,1)</x:f>
-        <x:v>61.8</x:v>
+        <x:v>84.8</x:v>
       </x:c>
       <x:c r="J41" s="22" t="str">
         <x:v>IH2609</x:v>
       </x:c>
       <x:c r="K41" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -1932,7 +1968,7 @@
       <x:c r="H42" s="28"/>
       <x:c r="I42" s="30" t="n">
         <x:f>ROUND(SUM(I41:I41),1)</x:f>
-        <x:v>61.8</x:v>
+        <x:v>84.8</x:v>
       </x:c>
       <x:c r="J42" s="28"/>
       <x:c r="K42" s="28"/>
@@ -1950,7 +1986,7 @@
       <x:c r="H43" s="28"/>
       <x:c r="I43" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I41:I41),0),1)</x:f>
-        <x:v>61.8</x:v>
+        <x:v>84.8</x:v>
       </x:c>
       <x:c r="J43" s="28"/>
       <x:c r="K43" s="28"/>
@@ -2010,31 +2046,31 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B47" s="22" t="str">
-        <x:v>8月3日-8月6日</x:v>
+        <x:v>8月3日-8月7日</x:v>
       </x:c>
       <x:c r="C47" s="23" t="n">
         <x:v>137500</x:v>
       </x:c>
       <x:c r="D47" s="23" t="n">
-        <x:v>144300</x:v>
+        <x:v>144800</x:v>
       </x:c>
       <x:c r="E47" s="23" t="n">
         <x:v>135560</x:v>
       </x:c>
       <x:c r="F47" s="23" t="n">
-        <x:v>141460</x:v>
+        <x:v>140000</x:v>
       </x:c>
       <x:c r="G47" s="23"/>
       <x:c r="H47" s="24"/>
       <x:c r="I47" s="26" t="n">
         <x:f>ROUND(D47-E47,1)</x:f>
-        <x:v>8740</x:v>
+        <x:v>9240</x:v>
       </x:c>
       <x:c r="J47" s="22" t="str">
         <x:v>LC2609</x:v>
       </x:c>
       <x:c r="K47" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -2052,7 +2088,7 @@
       <x:c r="H48" s="28"/>
       <x:c r="I48" s="30" t="n">
         <x:f>ROUND(SUM(I47:I47),1)</x:f>
-        <x:v>8740</x:v>
+        <x:v>9240</x:v>
       </x:c>
       <x:c r="J48" s="28"/>
       <x:c r="K48" s="28"/>
@@ -2070,7 +2106,7 @@
       <x:c r="H49" s="28"/>
       <x:c r="I49" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I47:I47),0),1)</x:f>
-        <x:v>8740</x:v>
+        <x:v>9240</x:v>
       </x:c>
       <x:c r="J49" s="28"/>
       <x:c r="K49" s="28"/>
@@ -2292,31 +2328,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B10" s="28" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C10" s="28"/>
-      <x:c r="D10" s="28"/>
-      <x:c r="E10" s="28"/>
-      <x:c r="F10" s="28"/>
-      <x:c r="G10" s="28"/>
-      <x:c r="H10" s="28"/>
-      <x:c r="I10" s="28"/>
-      <x:c r="J10" s="30" t="n">
-        <x:f>SUM(J4:J7)</x:f>
-        <x:v>680.4000000000001</x:v>
-      </x:c>
-      <x:c r="K10" s="28"/>
+    <x:row r="8">
+      <x:c r="A8" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C8" s="22" t="str">
+        <x:v>8月7日</x:v>
+      </x:c>
+      <x:c r="D8" s="23" t="n">
+        <x:v>7534.24</x:v>
+      </x:c>
+      <x:c r="E8" s="23" t="n">
+        <x:v>7685.57</x:v>
+      </x:c>
+      <x:c r="F8" s="23" t="n">
+        <x:v>7448.46</x:v>
+      </x:c>
+      <x:c r="G8" s="23" t="n">
+        <x:v>7679.53</x:v>
+      </x:c>
+      <x:c r="H8" s="23" t="n">
+        <x:v>149.1</x:v>
+      </x:c>
+      <x:c r="I8" s="24" t="n">
+        <x:v>0.019799666154522333</x:v>
+      </x:c>
+      <x:c r="J8" s="26" t="n">
+        <x:f>ROUND(E8-F8,1)</x:f>
+        <x:v>237.1</x:v>
+      </x:c>
+      <x:c r="K8" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B11" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B11" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
       <x:c r="C11" s="28"/>
       <x:c r="D11" s="28"/>
       <x:c r="E11" s="28"/>
@@ -2324,11 +2378,29 @@
       <x:c r="G11" s="28"/>
       <x:c r="H11" s="28"/>
       <x:c r="I11" s="28"/>
-      <x:c r="J11" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
-        <x:v>170.1</x:v>
+      <x:c r="J11" s="30" t="n">
+        <x:f>SUM(J4:J8)</x:f>
+        <x:v>917.5000000000001</x:v>
       </x:c>
       <x:c r="K11" s="28"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B12" s="28"/>
+      <x:c r="C12" s="28"/>
+      <x:c r="D12" s="28"/>
+      <x:c r="E12" s="28"/>
+      <x:c r="F12" s="28"/>
+      <x:c r="G12" s="28"/>
+      <x:c r="H12" s="28"/>
+      <x:c r="I12" s="28"/>
+      <x:c r="J12" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
+        <x:v>183.5</x:v>
+      </x:c>
+      <x:c r="K12" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2539,31 +2611,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B10" s="28" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C10" s="28"/>
-      <x:c r="D10" s="28"/>
-      <x:c r="E10" s="28"/>
-      <x:c r="F10" s="28"/>
-      <x:c r="G10" s="28"/>
-      <x:c r="H10" s="28"/>
-      <x:c r="I10" s="28"/>
-      <x:c r="J10" s="30" t="n">
-        <x:f>SUM(J4:J7)</x:f>
-        <x:v>720.5</x:v>
-      </x:c>
-      <x:c r="K10" s="28"/>
+    <x:row r="8">
+      <x:c r="A8" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C8" s="22" t="str">
+        <x:v>8月7日</x:v>
+      </x:c>
+      <x:c r="D8" s="23" t="n">
+        <x:v>7828.79</x:v>
+      </x:c>
+      <x:c r="E8" s="23" t="n">
+        <x:v>7983.17</x:v>
+      </x:c>
+      <x:c r="F8" s="23" t="n">
+        <x:v>7763.53</x:v>
+      </x:c>
+      <x:c r="G8" s="23" t="n">
+        <x:v>7980.12</x:v>
+      </x:c>
+      <x:c r="H8" s="37" t="n">
+        <x:v>150.8</x:v>
+      </x:c>
+      <x:c r="I8" s="24" t="n">
+        <x:v>0.019255724605842683</x:v>
+      </x:c>
+      <x:c r="J8" s="26" t="n">
+        <x:f>ROUND(E8-F8,1)</x:f>
+        <x:v>219.6</x:v>
+      </x:c>
+      <x:c r="K8" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B11" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B11" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
       <x:c r="C11" s="28"/>
       <x:c r="D11" s="28"/>
       <x:c r="E11" s="28"/>
@@ -2571,11 +2661,29 @@
       <x:c r="G11" s="28"/>
       <x:c r="H11" s="28"/>
       <x:c r="I11" s="28"/>
-      <x:c r="J11" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
-        <x:v>180.1</x:v>
+      <x:c r="J11" s="30" t="n">
+        <x:f>SUM(J4:J8)</x:f>
+        <x:v>940.1</x:v>
       </x:c>
       <x:c r="K11" s="28"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B12" s="28"/>
+      <x:c r="C12" s="28"/>
+      <x:c r="D12" s="28"/>
+      <x:c r="E12" s="28"/>
+      <x:c r="F12" s="28"/>
+      <x:c r="G12" s="28"/>
+      <x:c r="H12" s="28"/>
+      <x:c r="I12" s="28"/>
+      <x:c r="J12" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
+        <x:v>188</x:v>
+      </x:c>
+      <x:c r="K12" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2786,31 +2894,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B10" s="28" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C10" s="28"/>
-      <x:c r="D10" s="28"/>
-      <x:c r="E10" s="28"/>
-      <x:c r="F10" s="28"/>
-      <x:c r="G10" s="28"/>
-      <x:c r="H10" s="28"/>
-      <x:c r="I10" s="28"/>
-      <x:c r="J10" s="30" t="n">
-        <x:f>SUM(J4:J7)</x:f>
-        <x:v>169.5</x:v>
-      </x:c>
-      <x:c r="K10" s="28"/>
+    <x:row r="8">
+      <x:c r="A8" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C8" s="22" t="str">
+        <x:v>8月7日</x:v>
+      </x:c>
+      <x:c r="D8" s="23" t="n">
+        <x:v>3896.49</x:v>
+      </x:c>
+      <x:c r="E8" s="23" t="n">
+        <x:v>3940.93</x:v>
+      </x:c>
+      <x:c r="F8" s="23" t="n">
+        <x:v>3885.62</x:v>
+      </x:c>
+      <x:c r="G8" s="23" t="n">
+        <x:v>3940.04</x:v>
+      </x:c>
+      <x:c r="H8" s="23" t="n">
+        <x:v>39.7</x:v>
+      </x:c>
+      <x:c r="I8" s="24" t="n">
+        <x:v>0.01017600984527034</x:v>
+      </x:c>
+      <x:c r="J8" s="26" t="n">
+        <x:f>ROUND(E8-F8,1)</x:f>
+        <x:v>55.3</x:v>
+      </x:c>
+      <x:c r="K8" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B11" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B11" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
       <x:c r="C11" s="28"/>
       <x:c r="D11" s="28"/>
       <x:c r="E11" s="28"/>
@@ -2818,11 +2944,29 @@
       <x:c r="G11" s="28"/>
       <x:c r="H11" s="28"/>
       <x:c r="I11" s="28"/>
-      <x:c r="J11" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
-        <x:v>42.4</x:v>
+      <x:c r="J11" s="30" t="n">
+        <x:f>SUM(J4:J8)</x:f>
+        <x:v>224.8</x:v>
       </x:c>
       <x:c r="K11" s="28"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B12" s="28"/>
+      <x:c r="C12" s="28"/>
+      <x:c r="D12" s="28"/>
+      <x:c r="E12" s="28"/>
+      <x:c r="F12" s="28"/>
+      <x:c r="G12" s="28"/>
+      <x:c r="H12" s="28"/>
+      <x:c r="I12" s="28"/>
+      <x:c r="J12" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="K12" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3033,31 +3177,49 @@
         <x:v>IM2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B10" s="28" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C10" s="28"/>
-      <x:c r="D10" s="28"/>
-      <x:c r="E10" s="28"/>
-      <x:c r="F10" s="28"/>
-      <x:c r="G10" s="28"/>
-      <x:c r="H10" s="28"/>
-      <x:c r="I10" s="28"/>
-      <x:c r="J10" s="30" t="n">
-        <x:f>SUM(J4:J7)</x:f>
-        <x:v>689.5999999999999</x:v>
-      </x:c>
-      <x:c r="K10" s="28"/>
+    <x:row r="8">
+      <x:c r="A8" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C8" s="22" t="str">
+        <x:v>8月7日</x:v>
+      </x:c>
+      <x:c r="D8" s="23" t="n">
+        <x:v>7450</x:v>
+      </x:c>
+      <x:c r="E8" s="23" t="n">
+        <x:v>7594.2</x:v>
+      </x:c>
+      <x:c r="F8" s="23" t="n">
+        <x:v>7369</x:v>
+      </x:c>
+      <x:c r="G8" s="23" t="n">
+        <x:v>7590.6</x:v>
+      </x:c>
+      <x:c r="H8" s="23" t="n">
+        <x:v>138.8</x:v>
+      </x:c>
+      <x:c r="I8" s="24" t="n">
+        <x:v>0.018626372151694826</x:v>
+      </x:c>
+      <x:c r="J8" s="26" t="n">
+        <x:f>ROUND(E8-F8,1)</x:f>
+        <x:v>225.2</x:v>
+      </x:c>
+      <x:c r="K8" s="22" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B11" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B11" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
       <x:c r="C11" s="28"/>
       <x:c r="D11" s="28"/>
       <x:c r="E11" s="28"/>
@@ -3065,11 +3227,29 @@
       <x:c r="G11" s="28"/>
       <x:c r="H11" s="28"/>
       <x:c r="I11" s="28"/>
-      <x:c r="J11" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
-        <x:v>172.4</x:v>
+      <x:c r="J11" s="30" t="n">
+        <x:f>SUM(J4:J8)</x:f>
+        <x:v>914.8</x:v>
       </x:c>
       <x:c r="K11" s="28"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B12" s="28"/>
+      <x:c r="C12" s="28"/>
+      <x:c r="D12" s="28"/>
+      <x:c r="E12" s="28"/>
+      <x:c r="F12" s="28"/>
+      <x:c r="G12" s="28"/>
+      <x:c r="H12" s="28"/>
+      <x:c r="I12" s="28"/>
+      <x:c r="J12" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
+        <x:v>183</x:v>
+      </x:c>
+      <x:c r="K12" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3527,31 +3707,49 @@
         <x:v>IF2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B10" s="28" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C10" s="28"/>
-      <x:c r="D10" s="28"/>
-      <x:c r="E10" s="28"/>
-      <x:c r="F10" s="28"/>
-      <x:c r="G10" s="28"/>
-      <x:c r="H10" s="28"/>
-      <x:c r="I10" s="28"/>
-      <x:c r="J10" s="30" t="n">
-        <x:f>SUM(J4:J7)</x:f>
-        <x:v>276.8</x:v>
-      </x:c>
-      <x:c r="K10" s="28"/>
+    <x:row r="8">
+      <x:c r="A8" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C8" s="22" t="str">
+        <x:v>8月7日</x:v>
+      </x:c>
+      <x:c r="D8" s="23" t="n">
+        <x:v>4620</x:v>
+      </x:c>
+      <x:c r="E8" s="23" t="n">
+        <x:v>4656.2</x:v>
+      </x:c>
+      <x:c r="F8" s="23" t="n">
+        <x:v>4604.6</x:v>
+      </x:c>
+      <x:c r="G8" s="23" t="n">
+        <x:v>4645.6</x:v>
+      </x:c>
+      <x:c r="H8" s="23" t="n">
+        <x:v>33.6</x:v>
+      </x:c>
+      <x:c r="I8" s="24" t="n">
+        <x:v>0.007285342584562038</x:v>
+      </x:c>
+      <x:c r="J8" s="23" t="n">
+        <x:f>ROUND(E8-F8,1)</x:f>
+        <x:v>51.6</x:v>
+      </x:c>
+      <x:c r="K8" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B11" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B11" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
       <x:c r="C11" s="28"/>
       <x:c r="D11" s="28"/>
       <x:c r="E11" s="28"/>
@@ -3559,11 +3757,29 @@
       <x:c r="G11" s="28"/>
       <x:c r="H11" s="28"/>
       <x:c r="I11" s="28"/>
-      <x:c r="J11" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
-        <x:v>69.2</x:v>
+      <x:c r="J11" s="30" t="n">
+        <x:f>SUM(J4:J8)</x:f>
+        <x:v>328.40000000000003</x:v>
       </x:c>
       <x:c r="K11" s="28"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B12" s="28"/>
+      <x:c r="C12" s="28"/>
+      <x:c r="D12" s="28"/>
+      <x:c r="E12" s="28"/>
+      <x:c r="F12" s="28"/>
+      <x:c r="G12" s="28"/>
+      <x:c r="H12" s="28"/>
+      <x:c r="I12" s="28"/>
+      <x:c r="J12" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
+        <x:v>65.7</x:v>
+      </x:c>
+      <x:c r="K12" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3774,31 +3990,49 @@
         <x:v>IH2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B10" s="28" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C10" s="28"/>
-      <x:c r="D10" s="28"/>
-      <x:c r="E10" s="28"/>
-      <x:c r="F10" s="28"/>
-      <x:c r="G10" s="28"/>
-      <x:c r="H10" s="28"/>
-      <x:c r="I10" s="28"/>
-      <x:c r="J10" s="30" t="n">
-        <x:f>SUM(J4:J7)</x:f>
-        <x:v>140.2</x:v>
-      </x:c>
-      <x:c r="K10" s="28"/>
+    <x:row r="8">
+      <x:c r="A8" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C8" s="22" t="str">
+        <x:v>8月7日</x:v>
+      </x:c>
+      <x:c r="D8" s="23" t="n">
+        <x:v>2892.2</x:v>
+      </x:c>
+      <x:c r="E8" s="23" t="n">
+        <x:v>2930.6</x:v>
+      </x:c>
+      <x:c r="F8" s="23" t="n">
+        <x:v>2884</x:v>
+      </x:c>
+      <x:c r="G8" s="23" t="n">
+        <x:v>2930</x:v>
+      </x:c>
+      <x:c r="H8" s="23" t="n">
+        <x:v>32.8</x:v>
+      </x:c>
+      <x:c r="I8" s="24" t="n">
+        <x:v>0.011321275714482937</x:v>
+      </x:c>
+      <x:c r="J8" s="23" t="n">
+        <x:f>ROUND(E8-F8,1)</x:f>
+        <x:v>46.6</x:v>
+      </x:c>
+      <x:c r="K8" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B11" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B11" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
       <x:c r="C11" s="28"/>
       <x:c r="D11" s="28"/>
       <x:c r="E11" s="28"/>
@@ -3806,11 +4040,29 @@
       <x:c r="G11" s="28"/>
       <x:c r="H11" s="28"/>
       <x:c r="I11" s="28"/>
-      <x:c r="J11" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
-        <x:v>35.1</x:v>
+      <x:c r="J11" s="30" t="n">
+        <x:f>SUM(J4:J8)</x:f>
+        <x:v>186.79999999999998</x:v>
       </x:c>
       <x:c r="K11" s="28"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B12" s="28"/>
+      <x:c r="C12" s="28"/>
+      <x:c r="D12" s="28"/>
+      <x:c r="E12" s="28"/>
+      <x:c r="F12" s="28"/>
+      <x:c r="G12" s="28"/>
+      <x:c r="H12" s="28"/>
+      <x:c r="I12" s="28"/>
+      <x:c r="J12" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
+        <x:v>37.4</x:v>
+      </x:c>
+      <x:c r="K12" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-08-10
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R9ac329f9429c4de1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R4245402c00074616"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Rd9967522559e40f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rdf28b6d6a4524c79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Rf9a7ec8ba95d494c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R8e0bfe3e9eac4e47"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R90892f03b50b41f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R44228e5754b24b32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R5b23dd489a484aa8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R5beedbe8a1604bac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rba3221fd35d14075"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R1b63c839501340ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Rfc40bec8f66143d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R2125c6092d9e4211"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Rf33c6e2a146d4a83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rda83f680401e4aee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R082b64e0c3d242e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rcd01c5cdc7d840d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R5949b5edc26f4a1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R94db2b6370d84088"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -485,25 +485,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-08-07</x:v>
+        <x:v>2026-08-10</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7685.57</x:v>
+        <x:v>7736.1</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7448.46</x:v>
+        <x:v>7621.65</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>237.1</x:v>
+        <x:v>114.5</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>917.5</x:v>
+        <x:v>1032</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>183.5</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -514,25 +514,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-08-07</x:v>
+        <x:v>2026-08-10</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7983.17</x:v>
+        <x:v>8031.16</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7763.53</x:v>
+        <x:v>7910.84</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>219.6</x:v>
+        <x:v>120.3</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>940.1</x:v>
+        <x:v>1060.4</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>188</x:v>
+        <x:v>176.7</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -543,25 +543,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-08-07</x:v>
+        <x:v>2026-08-10</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3940.93</x:v>
+        <x:v>3967.59</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3885.62</x:v>
+        <x:v>3938.63</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>55.3</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>224.8</x:v>
+        <x:v>253.8</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>45</x:v>
+        <x:v>42.3</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -572,25 +572,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-08-07</x:v>
+        <x:v>2026-08-10</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>7594.2</x:v>
+        <x:v>7631.2</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>7369</x:v>
+        <x:v>7525</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>225.2</x:v>
+        <x:v>106.2</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>914.8</x:v>
+        <x:v>1021</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>183</x:v>
+        <x:v>170.2</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -720,7 +720,7 @@
         <x:v>2026-08-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-08-07</x:v>
+        <x:v>2026-08-10</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1234,894 +1234,1046 @@
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B6" s="28" t="n">
+      <x:c r="A6" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B6" s="22" t="str">
+        <x:v>8月10日</x:v>
+      </x:c>
+      <x:c r="C6" s="23" t="n">
+        <x:v>7723.38</x:v>
+      </x:c>
+      <x:c r="D6" s="23" t="n">
+        <x:v>7736.1</x:v>
+      </x:c>
+      <x:c r="E6" s="23" t="n">
+        <x:v>7621.65</x:v>
+      </x:c>
+      <x:c r="F6" s="23" t="n">
+        <x:v>7733.9</x:v>
+      </x:c>
+      <x:c r="G6" s="23" t="n">
+        <x:f>ROUND(F6-F5,1)</x:f>
+        <x:v>54.4</x:v>
+      </x:c>
+      <x:c r="H6" s="24" t="n">
+        <x:f>IFERROR(F6/F5-1,"")</x:f>
+        <x:v>0.00707986035603736</x:v>
+      </x:c>
+      <x:c r="I6" s="23" t="n">
+        <x:f>ROUND(D6-E6,1)</x:f>
+        <x:v>114.5</x:v>
+      </x:c>
+      <x:c r="J6" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
+      <x:c r="K6" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C6" s="28"/>
-      <x:c r="D6" s="28"/>
-      <x:c r="E6" s="28"/>
-      <x:c r="F6" s="28"/>
-      <x:c r="G6" s="28"/>
-      <x:c r="H6" s="28"/>
-      <x:c r="I6" s="30" t="n">
-        <x:f>ROUND(SUM(I5:I5),1)</x:f>
-        <x:v>642.7</x:v>
-      </x:c>
-      <x:c r="J6" s="28"/>
-      <x:c r="K6" s="28"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B7" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B7" s="28" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="C7" s="28"/>
       <x:c r="D7" s="28"/>
       <x:c r="E7" s="28"/>
       <x:c r="F7" s="28"/>
       <x:c r="G7" s="28"/>
       <x:c r="H7" s="28"/>
-      <x:c r="I7" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I5:I5),0),1)</x:f>
-        <x:v>642.7</x:v>
+      <x:c r="I7" s="30" t="n">
+        <x:f>ROUND(SUM(I5:I6),1)</x:f>
+        <x:v>757.2</x:v>
       </x:c>
       <x:c r="J7" s="28"/>
       <x:c r="K7" s="28"/>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="17" t="str">
+    <x:row r="8">
+      <x:c r="A8" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B8" s="28"/>
+      <x:c r="C8" s="28"/>
+      <x:c r="D8" s="28"/>
+      <x:c r="E8" s="28"/>
+      <x:c r="F8" s="28"/>
+      <x:c r="G8" s="28"/>
+      <x:c r="H8" s="28"/>
+      <x:c r="I8" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I5:I6),0),1)</x:f>
+        <x:v>378.6</x:v>
+      </x:c>
+      <x:c r="J8" s="28"/>
+      <x:c r="K8" s="28"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="17" t="str">
         <x:v>中证500</x:v>
       </x:c>
-      <x:c r="B9" s="17"/>
-      <x:c r="C9" s="17"/>
-      <x:c r="D9" s="17"/>
-      <x:c r="E9" s="17"/>
-      <x:c r="F9" s="17"/>
-      <x:c r="G9" s="17"/>
-      <x:c r="H9" s="17"/>
-      <x:c r="I9" s="17"/>
-      <x:c r="J9" s="17"/>
-      <x:c r="K9" s="17"/>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="20" t="str">
+      <x:c r="B10" s="17"/>
+      <x:c r="C10" s="17"/>
+      <x:c r="D10" s="17"/>
+      <x:c r="E10" s="17"/>
+      <x:c r="F10" s="17"/>
+      <x:c r="G10" s="17"/>
+      <x:c r="H10" s="17"/>
+      <x:c r="I10" s="17"/>
+      <x:c r="J10" s="17"/>
+      <x:c r="K10" s="17"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B10" s="20" t="str">
+      <x:c r="B11" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C10" s="20" t="str">
+      <x:c r="C11" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D10" s="20" t="str">
+      <x:c r="D11" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E10" s="20" t="str">
+      <x:c r="E11" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F10" s="20" t="str">
+      <x:c r="F11" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G10" s="20" t="str">
+      <x:c r="G11" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H10" s="20" t="str">
+      <x:c r="H11" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I10" s="20" t="str">
+      <x:c r="I11" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J10" s="20" t="str">
+      <x:c r="J11" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K10" s="20" t="str">
+      <x:c r="K11" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="22" t="n">
+    <x:row r="12">
+      <x:c r="A12" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B11" s="22" t="str">
+      <x:c r="B12" s="22" t="str">
         <x:v>8月3日-8月7日</x:v>
       </x:c>
-      <x:c r="C11" s="23" t="n">
+      <x:c r="C12" s="23" t="n">
         <x:v>7457.12</x:v>
       </x:c>
-      <x:c r="D11" s="23" t="n">
+      <x:c r="D12" s="23" t="n">
         <x:v>7983.17</x:v>
       </x:c>
-      <x:c r="E11" s="23" t="n">
+      <x:c r="E12" s="23" t="n">
         <x:v>7397.94</x:v>
       </x:c>
-      <x:c r="F11" s="23" t="n">
+      <x:c r="F12" s="23" t="n">
         <x:v>7980.12</x:v>
       </x:c>
-      <x:c r="G11" s="23"/>
-      <x:c r="H11" s="24"/>
-      <x:c r="I11" s="26" t="n">
-        <x:f>ROUND(D11-E11,1)</x:f>
+      <x:c r="G12" s="23"/>
+      <x:c r="H12" s="24"/>
+      <x:c r="I12" s="26" t="n">
+        <x:f>ROUND(D12-E12,1)</x:f>
         <x:v>585.2</x:v>
       </x:c>
-      <x:c r="J11" s="22" t="str">
+      <x:c r="J12" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
-      <x:c r="K11" s="22" t="n">
+      <x:c r="K12" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="29" t="str">
+    <x:row r="13">
+      <x:c r="A13" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B13" s="22" t="str">
+        <x:v>8月10日</x:v>
+      </x:c>
+      <x:c r="C13" s="23" t="n">
+        <x:v>8003.92</x:v>
+      </x:c>
+      <x:c r="D13" s="23" t="n">
+        <x:v>8031.16</x:v>
+      </x:c>
+      <x:c r="E13" s="23" t="n">
+        <x:v>7910.84</x:v>
+      </x:c>
+      <x:c r="F13" s="23" t="n">
+        <x:v>8030.95</x:v>
+      </x:c>
+      <x:c r="G13" s="23" t="n">
+        <x:f>ROUND(F13-F12,1)</x:f>
+        <x:v>50.8</x:v>
+      </x:c>
+      <x:c r="H13" s="24" t="n">
+        <x:f>IFERROR(F13/F12-1,"")</x:f>
+        <x:v>0.0063695784023298785</x:v>
+      </x:c>
+      <x:c r="I13" s="23" t="n">
+        <x:f>ROUND(D13-E13,1)</x:f>
+        <x:v>120.3</x:v>
+      </x:c>
+      <x:c r="J13" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+      <x:c r="K13" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B12" s="28" t="n">
+      <x:c r="B14" s="28" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C14" s="28"/>
+      <x:c r="D14" s="28"/>
+      <x:c r="E14" s="28"/>
+      <x:c r="F14" s="28"/>
+      <x:c r="G14" s="28"/>
+      <x:c r="H14" s="28"/>
+      <x:c r="I14" s="30" t="n">
+        <x:f>ROUND(SUM(I12:I13),1)</x:f>
+        <x:v>705.5</x:v>
+      </x:c>
+      <x:c r="J14" s="28"/>
+      <x:c r="K14" s="28"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B15" s="28"/>
+      <x:c r="C15" s="28"/>
+      <x:c r="D15" s="28"/>
+      <x:c r="E15" s="28"/>
+      <x:c r="F15" s="28"/>
+      <x:c r="G15" s="28"/>
+      <x:c r="H15" s="28"/>
+      <x:c r="I15" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I12:I13),0),1)</x:f>
+        <x:v>352.8</x:v>
+      </x:c>
+      <x:c r="J15" s="28"/>
+      <x:c r="K15" s="28"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="17" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="B17" s="17"/>
+      <x:c r="C17" s="17"/>
+      <x:c r="D17" s="17"/>
+      <x:c r="E17" s="17"/>
+      <x:c r="F17" s="17"/>
+      <x:c r="G17" s="17"/>
+      <x:c r="H17" s="17"/>
+      <x:c r="I17" s="17"/>
+      <x:c r="J17" s="17"/>
+      <x:c r="K17" s="17"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="20" t="str">
+        <x:v>序号</x:v>
+      </x:c>
+      <x:c r="B18" s="20" t="str">
+        <x:v>周期</x:v>
+      </x:c>
+      <x:c r="C18" s="20" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="D18" s="20" t="str">
+        <x:v>高点</x:v>
+      </x:c>
+      <x:c r="E18" s="20" t="str">
+        <x:v>低点</x:v>
+      </x:c>
+      <x:c r="F18" s="20" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="G18" s="20" t="str">
+        <x:v>涨跌点数</x:v>
+      </x:c>
+      <x:c r="H18" s="20" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I18" s="20" t="str">
+        <x:v>振幅</x:v>
+      </x:c>
+      <x:c r="J18" s="20" t="str">
+        <x:v>标的</x:v>
+      </x:c>
+      <x:c r="K18" s="20" t="str">
+        <x:v>交易日</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C12" s="28"/>
-      <x:c r="D12" s="28"/>
-      <x:c r="E12" s="28"/>
-      <x:c r="F12" s="28"/>
-      <x:c r="G12" s="28"/>
-      <x:c r="H12" s="28"/>
-      <x:c r="I12" s="30" t="n">
-        <x:f>ROUND(SUM(I11:I11),1)</x:f>
-        <x:v>585.2</x:v>
-      </x:c>
-      <x:c r="J12" s="28"/>
-      <x:c r="K12" s="28"/>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="29" t="str">
+      <x:c r="B19" s="22" t="str">
+        <x:v>8月3日-8月7日</x:v>
+      </x:c>
+      <x:c r="C19" s="23" t="n">
+        <x:v>3812.61</x:v>
+      </x:c>
+      <x:c r="D19" s="23" t="n">
+        <x:v>3940.93</x:v>
+      </x:c>
+      <x:c r="E19" s="23" t="n">
+        <x:v>3797.64</x:v>
+      </x:c>
+      <x:c r="F19" s="23" t="n">
+        <x:v>3940.04</x:v>
+      </x:c>
+      <x:c r="G19" s="23"/>
+      <x:c r="H19" s="24"/>
+      <x:c r="I19" s="26" t="n">
+        <x:f>ROUND(D19-E19,1)</x:f>
+        <x:v>143.3</x:v>
+      </x:c>
+      <x:c r="J19" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="K19" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B20" s="22" t="str">
+        <x:v>8月10日</x:v>
+      </x:c>
+      <x:c r="C20" s="23" t="n">
+        <x:v>3943.82</x:v>
+      </x:c>
+      <x:c r="D20" s="23" t="n">
+        <x:v>3967.59</x:v>
+      </x:c>
+      <x:c r="E20" s="23" t="n">
+        <x:v>3938.63</x:v>
+      </x:c>
+      <x:c r="F20" s="23" t="n">
+        <x:v>3966.59</x:v>
+      </x:c>
+      <x:c r="G20" s="23" t="n">
+        <x:f>ROUND(F20-F19,1)</x:f>
+        <x:v>26.6</x:v>
+      </x:c>
+      <x:c r="H20" s="24" t="n">
+        <x:f>IFERROR(F20/F19-1,"")</x:f>
+        <x:v>0.0067385102689312415</x:v>
+      </x:c>
+      <x:c r="I20" s="23" t="n">
+        <x:f>ROUND(D20-E20,1)</x:f>
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="J20" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="K20" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="29" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B21" s="28" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C21" s="28"/>
+      <x:c r="D21" s="28"/>
+      <x:c r="E21" s="28"/>
+      <x:c r="F21" s="28"/>
+      <x:c r="G21" s="28"/>
+      <x:c r="H21" s="28"/>
+      <x:c r="I21" s="30" t="n">
+        <x:f>ROUND(SUM(I19:I20),1)</x:f>
+        <x:v>172.3</x:v>
+      </x:c>
+      <x:c r="J21" s="28"/>
+      <x:c r="K21" s="28"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B13" s="28"/>
-      <x:c r="C13" s="28"/>
-      <x:c r="D13" s="28"/>
-      <x:c r="E13" s="28"/>
-      <x:c r="F13" s="28"/>
-      <x:c r="G13" s="28"/>
-      <x:c r="H13" s="28"/>
-      <x:c r="I13" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I11:I11),0),1)</x:f>
-        <x:v>585.2</x:v>
-      </x:c>
-      <x:c r="J13" s="28"/>
-      <x:c r="K13" s="28"/>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="17" t="str">
-        <x:v>上证指数</x:v>
-      </x:c>
-      <x:c r="B15" s="17"/>
-      <x:c r="C15" s="17"/>
-      <x:c r="D15" s="17"/>
-      <x:c r="E15" s="17"/>
-      <x:c r="F15" s="17"/>
-      <x:c r="G15" s="17"/>
-      <x:c r="H15" s="17"/>
-      <x:c r="I15" s="17"/>
-      <x:c r="J15" s="17"/>
-      <x:c r="K15" s="17"/>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="20" t="str">
+      <x:c r="B22" s="28"/>
+      <x:c r="C22" s="28"/>
+      <x:c r="D22" s="28"/>
+      <x:c r="E22" s="28"/>
+      <x:c r="F22" s="28"/>
+      <x:c r="G22" s="28"/>
+      <x:c r="H22" s="28"/>
+      <x:c r="I22" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I19:I20),0),1)</x:f>
+        <x:v>86.2</x:v>
+      </x:c>
+      <x:c r="J22" s="28"/>
+      <x:c r="K22" s="28"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="17" t="str">
+        <x:v>IM主力</x:v>
+      </x:c>
+      <x:c r="B24" s="17"/>
+      <x:c r="C24" s="17"/>
+      <x:c r="D24" s="17"/>
+      <x:c r="E24" s="17"/>
+      <x:c r="F24" s="17"/>
+      <x:c r="G24" s="17"/>
+      <x:c r="H24" s="17"/>
+      <x:c r="I24" s="17"/>
+      <x:c r="J24" s="17"/>
+      <x:c r="K24" s="17"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B16" s="20" t="str">
+      <x:c r="B25" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C16" s="20" t="str">
+      <x:c r="C25" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D16" s="20" t="str">
+      <x:c r="D25" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E16" s="20" t="str">
+      <x:c r="E25" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F16" s="20" t="str">
+      <x:c r="F25" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G16" s="20" t="str">
+      <x:c r="G25" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H16" s="20" t="str">
+      <x:c r="H25" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I16" s="20" t="str">
+      <x:c r="I25" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J16" s="20" t="str">
+      <x:c r="J25" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K16" s="20" t="str">
+      <x:c r="K25" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="22" t="n">
+    <x:row r="26">
+      <x:c r="A26" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B17" s="22" t="str">
+      <x:c r="B26" s="22" t="str">
         <x:v>8月3日-8月7日</x:v>
       </x:c>
-      <x:c r="C17" s="23" t="n">
-        <x:v>3812.61</x:v>
-      </x:c>
-      <x:c r="D17" s="23" t="n">
-        <x:v>3940.93</x:v>
-      </x:c>
-      <x:c r="E17" s="23" t="n">
-        <x:v>3797.64</x:v>
-      </x:c>
-      <x:c r="F17" s="23" t="n">
-        <x:v>3940.04</x:v>
-      </x:c>
-      <x:c r="G17" s="23"/>
-      <x:c r="H17" s="24"/>
-      <x:c r="I17" s="26" t="n">
-        <x:f>ROUND(D17-E17,1)</x:f>
-        <x:v>143.3</x:v>
-      </x:c>
-      <x:c r="J17" s="22" t="str">
-        <x:v>上证指数</x:v>
-      </x:c>
-      <x:c r="K17" s="22" t="n">
+      <x:c r="C26" s="23" t="n">
+        <x:v>7000</x:v>
+      </x:c>
+      <x:c r="D26" s="23" t="n">
+        <x:v>7594.2</x:v>
+      </x:c>
+      <x:c r="E26" s="23" t="n">
+        <x:v>6976</x:v>
+      </x:c>
+      <x:c r="F26" s="23" t="n">
+        <x:v>7590.6</x:v>
+      </x:c>
+      <x:c r="G26" s="23"/>
+      <x:c r="H26" s="24"/>
+      <x:c r="I26" s="26" t="n">
+        <x:f>ROUND(D26-E26,1)</x:f>
+        <x:v>618.2</x:v>
+      </x:c>
+      <x:c r="J26" s="22" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+      <x:c r="K26" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="29" t="str">
+    <x:row r="27">
+      <x:c r="A27" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B27" s="22" t="str">
+        <x:v>8月10日</x:v>
+      </x:c>
+      <x:c r="C27" s="23" t="n">
+        <x:v>7628.8</x:v>
+      </x:c>
+      <x:c r="D27" s="23" t="n">
+        <x:v>7631.2</x:v>
+      </x:c>
+      <x:c r="E27" s="23" t="n">
+        <x:v>7525</x:v>
+      </x:c>
+      <x:c r="F27" s="23" t="n">
+        <x:v>7607.2</x:v>
+      </x:c>
+      <x:c r="G27" s="23" t="n">
+        <x:f>ROUND(F27-F26,1)</x:f>
+        <x:v>16.6</x:v>
+      </x:c>
+      <x:c r="H27" s="24" t="n">
+        <x:f>IFERROR(F27/F26-1,"")</x:f>
+        <x:v>0.002186915395357314</x:v>
+      </x:c>
+      <x:c r="I27" s="23" t="n">
+        <x:f>ROUND(D27-E27,1)</x:f>
+        <x:v>106.2</x:v>
+      </x:c>
+      <x:c r="J27" s="22" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+      <x:c r="K27" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B18" s="28" t="n">
+      <x:c r="B28" s="28" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C28" s="28"/>
+      <x:c r="D28" s="28"/>
+      <x:c r="E28" s="28"/>
+      <x:c r="F28" s="28"/>
+      <x:c r="G28" s="28"/>
+      <x:c r="H28" s="28"/>
+      <x:c r="I28" s="30" t="n">
+        <x:f>ROUND(SUM(I26:I27),1)</x:f>
+        <x:v>724.4</x:v>
+      </x:c>
+      <x:c r="J28" s="28"/>
+      <x:c r="K28" s="28"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B29" s="28"/>
+      <x:c r="C29" s="28"/>
+      <x:c r="D29" s="28"/>
+      <x:c r="E29" s="28"/>
+      <x:c r="F29" s="28"/>
+      <x:c r="G29" s="28"/>
+      <x:c r="H29" s="28"/>
+      <x:c r="I29" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I26:I27),0),1)</x:f>
+        <x:v>362.2</x:v>
+      </x:c>
+      <x:c r="J29" s="28"/>
+      <x:c r="K29" s="28"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="17" t="str">
+        <x:v>IC主力</x:v>
+      </x:c>
+      <x:c r="B31" s="17"/>
+      <x:c r="C31" s="17"/>
+      <x:c r="D31" s="17"/>
+      <x:c r="E31" s="17"/>
+      <x:c r="F31" s="17"/>
+      <x:c r="G31" s="17"/>
+      <x:c r="H31" s="17"/>
+      <x:c r="I31" s="17"/>
+      <x:c r="J31" s="17"/>
+      <x:c r="K31" s="17"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="20" t="str">
+        <x:v>序号</x:v>
+      </x:c>
+      <x:c r="B32" s="20" t="str">
+        <x:v>周期</x:v>
+      </x:c>
+      <x:c r="C32" s="20" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="D32" s="20" t="str">
+        <x:v>高点</x:v>
+      </x:c>
+      <x:c r="E32" s="20" t="str">
+        <x:v>低点</x:v>
+      </x:c>
+      <x:c r="F32" s="20" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="G32" s="20" t="str">
+        <x:v>涨跌点数</x:v>
+      </x:c>
+      <x:c r="H32" s="20" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I32" s="20" t="str">
+        <x:v>振幅</x:v>
+      </x:c>
+      <x:c r="J32" s="20" t="str">
+        <x:v>标的</x:v>
+      </x:c>
+      <x:c r="K32" s="20" t="str">
+        <x:v>交易日</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C18" s="28"/>
-      <x:c r="D18" s="28"/>
-      <x:c r="E18" s="28"/>
-      <x:c r="F18" s="28"/>
-      <x:c r="G18" s="28"/>
-      <x:c r="H18" s="28"/>
-      <x:c r="I18" s="30" t="n">
-        <x:f>ROUND(SUM(I17:I17),1)</x:f>
-        <x:v>143.3</x:v>
-      </x:c>
-      <x:c r="J18" s="28"/>
-      <x:c r="K18" s="28"/>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="29" t="str">
+      <x:c r="B33" s="22" t="str">
+        <x:v>8月3日-8月7日</x:v>
+      </x:c>
+      <x:c r="C33" s="23" t="n">
+        <x:v>7391</x:v>
+      </x:c>
+      <x:c r="D33" s="23" t="n">
+        <x:v>7882.6</x:v>
+      </x:c>
+      <x:c r="E33" s="23" t="n">
+        <x:v>7335</x:v>
+      </x:c>
+      <x:c r="F33" s="23" t="n">
+        <x:v>7877.8</x:v>
+      </x:c>
+      <x:c r="G33" s="23"/>
+      <x:c r="H33" s="24"/>
+      <x:c r="I33" s="26" t="n">
+        <x:f>ROUND(D33-E33,1)</x:f>
+        <x:v>547.6</x:v>
+      </x:c>
+      <x:c r="J33" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+      <x:c r="K33" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="29" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B34" s="28" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C34" s="28"/>
+      <x:c r="D34" s="28"/>
+      <x:c r="E34" s="28"/>
+      <x:c r="F34" s="28"/>
+      <x:c r="G34" s="28"/>
+      <x:c r="H34" s="28"/>
+      <x:c r="I34" s="30" t="n">
+        <x:f>ROUND(SUM(I33:I33),1)</x:f>
+        <x:v>547.6</x:v>
+      </x:c>
+      <x:c r="J34" s="28"/>
+      <x:c r="K34" s="28"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B19" s="28"/>
-      <x:c r="C19" s="28"/>
-      <x:c r="D19" s="28"/>
-      <x:c r="E19" s="28"/>
-      <x:c r="F19" s="28"/>
-      <x:c r="G19" s="28"/>
-      <x:c r="H19" s="28"/>
-      <x:c r="I19" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I17:I17),0),1)</x:f>
-        <x:v>143.3</x:v>
-      </x:c>
-      <x:c r="J19" s="28"/>
-      <x:c r="K19" s="28"/>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="17" t="str">
-        <x:v>IM主力</x:v>
-      </x:c>
-      <x:c r="B21" s="17"/>
-      <x:c r="C21" s="17"/>
-      <x:c r="D21" s="17"/>
-      <x:c r="E21" s="17"/>
-      <x:c r="F21" s="17"/>
-      <x:c r="G21" s="17"/>
-      <x:c r="H21" s="17"/>
-      <x:c r="I21" s="17"/>
-      <x:c r="J21" s="17"/>
-      <x:c r="K21" s="17"/>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="20" t="str">
+      <x:c r="B35" s="28"/>
+      <x:c r="C35" s="28"/>
+      <x:c r="D35" s="28"/>
+      <x:c r="E35" s="28"/>
+      <x:c r="F35" s="28"/>
+      <x:c r="G35" s="28"/>
+      <x:c r="H35" s="28"/>
+      <x:c r="I35" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I33:I33),0),1)</x:f>
+        <x:v>547.6</x:v>
+      </x:c>
+      <x:c r="J35" s="28"/>
+      <x:c r="K35" s="28"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="17" t="str">
+        <x:v>IF主力</x:v>
+      </x:c>
+      <x:c r="B37" s="17"/>
+      <x:c r="C37" s="17"/>
+      <x:c r="D37" s="17"/>
+      <x:c r="E37" s="17"/>
+      <x:c r="F37" s="17"/>
+      <x:c r="G37" s="17"/>
+      <x:c r="H37" s="17"/>
+      <x:c r="I37" s="17"/>
+      <x:c r="J37" s="17"/>
+      <x:c r="K37" s="17"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B22" s="20" t="str">
+      <x:c r="B38" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C22" s="20" t="str">
+      <x:c r="C38" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D22" s="20" t="str">
+      <x:c r="D38" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E22" s="20" t="str">
+      <x:c r="E38" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F22" s="20" t="str">
+      <x:c r="F38" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G22" s="20" t="str">
+      <x:c r="G38" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H22" s="20" t="str">
+      <x:c r="H38" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I22" s="20" t="str">
+      <x:c r="I38" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J22" s="20" t="str">
+      <x:c r="J38" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K22" s="20" t="str">
+      <x:c r="K38" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="22" t="n">
+    <x:row r="39">
+      <x:c r="A39" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B23" s="22" t="str">
+      <x:c r="B39" s="22" t="str">
         <x:v>8月3日-8月7日</x:v>
       </x:c>
-      <x:c r="C23" s="23" t="n">
-        <x:v>7000</x:v>
-      </x:c>
-      <x:c r="D23" s="23" t="n">
-        <x:v>7594.2</x:v>
-      </x:c>
-      <x:c r="E23" s="23" t="n">
-        <x:v>6976</x:v>
-      </x:c>
-      <x:c r="F23" s="23" t="n">
-        <x:v>7590.6</x:v>
-      </x:c>
-      <x:c r="G23" s="23"/>
-      <x:c r="H23" s="24"/>
-      <x:c r="I23" s="26" t="n">
-        <x:f>ROUND(D23-E23,1)</x:f>
-        <x:v>618.2</x:v>
-      </x:c>
-      <x:c r="J23" s="22" t="str">
-        <x:v>IM2609</x:v>
-      </x:c>
-      <x:c r="K23" s="22" t="n">
+      <x:c r="C39" s="23" t="n">
+        <x:v>4526.4</x:v>
+      </x:c>
+      <x:c r="D39" s="23" t="n">
+        <x:v>4656.2</x:v>
+      </x:c>
+      <x:c r="E39" s="23" t="n">
+        <x:v>4494.2</x:v>
+      </x:c>
+      <x:c r="F39" s="23" t="n">
+        <x:v>4645.6</x:v>
+      </x:c>
+      <x:c r="G39" s="23"/>
+      <x:c r="H39" s="24"/>
+      <x:c r="I39" s="26" t="n">
+        <x:f>ROUND(D39-E39,1)</x:f>
+        <x:v>162</x:v>
+      </x:c>
+      <x:c r="J39" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+      <x:c r="K39" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="29" t="str">
+    <x:row r="40">
+      <x:c r="A40" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B24" s="28" t="n">
+      <x:c r="B40" s="28" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C24" s="28"/>
-      <x:c r="D24" s="28"/>
-      <x:c r="E24" s="28"/>
-      <x:c r="F24" s="28"/>
-      <x:c r="G24" s="28"/>
-      <x:c r="H24" s="28"/>
-      <x:c r="I24" s="30" t="n">
-        <x:f>ROUND(SUM(I23:I23),1)</x:f>
-        <x:v>618.2</x:v>
-      </x:c>
-      <x:c r="J24" s="28"/>
-      <x:c r="K24" s="28"/>
-    </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="29" t="str">
+      <x:c r="C40" s="28"/>
+      <x:c r="D40" s="28"/>
+      <x:c r="E40" s="28"/>
+      <x:c r="F40" s="28"/>
+      <x:c r="G40" s="28"/>
+      <x:c r="H40" s="28"/>
+      <x:c r="I40" s="30" t="n">
+        <x:f>ROUND(SUM(I39:I39),1)</x:f>
+        <x:v>162</x:v>
+      </x:c>
+      <x:c r="J40" s="28"/>
+      <x:c r="K40" s="28"/>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B25" s="28"/>
-      <x:c r="C25" s="28"/>
-      <x:c r="D25" s="28"/>
-      <x:c r="E25" s="28"/>
-      <x:c r="F25" s="28"/>
-      <x:c r="G25" s="28"/>
-      <x:c r="H25" s="28"/>
-      <x:c r="I25" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I23:I23),0),1)</x:f>
-        <x:v>618.2</x:v>
-      </x:c>
-      <x:c r="J25" s="28"/>
-      <x:c r="K25" s="28"/>
-    </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="17" t="str">
-        <x:v>IC主力</x:v>
-      </x:c>
-      <x:c r="B27" s="17"/>
-      <x:c r="C27" s="17"/>
-      <x:c r="D27" s="17"/>
-      <x:c r="E27" s="17"/>
-      <x:c r="F27" s="17"/>
-      <x:c r="G27" s="17"/>
-      <x:c r="H27" s="17"/>
-      <x:c r="I27" s="17"/>
-      <x:c r="J27" s="17"/>
-      <x:c r="K27" s="17"/>
-    </x:row>
-    <x:row r="28">
-      <x:c r="A28" s="20" t="str">
+      <x:c r="B41" s="28"/>
+      <x:c r="C41" s="28"/>
+      <x:c r="D41" s="28"/>
+      <x:c r="E41" s="28"/>
+      <x:c r="F41" s="28"/>
+      <x:c r="G41" s="28"/>
+      <x:c r="H41" s="28"/>
+      <x:c r="I41" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I39:I39),0),1)</x:f>
+        <x:v>162</x:v>
+      </x:c>
+      <x:c r="J41" s="28"/>
+      <x:c r="K41" s="28"/>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="17" t="str">
+        <x:v>IH主力</x:v>
+      </x:c>
+      <x:c r="B43" s="17"/>
+      <x:c r="C43" s="17"/>
+      <x:c r="D43" s="17"/>
+      <x:c r="E43" s="17"/>
+      <x:c r="F43" s="17"/>
+      <x:c r="G43" s="17"/>
+      <x:c r="H43" s="17"/>
+      <x:c r="I43" s="17"/>
+      <x:c r="J43" s="17"/>
+      <x:c r="K43" s="17"/>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B28" s="20" t="str">
+      <x:c r="B44" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C28" s="20" t="str">
+      <x:c r="C44" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D28" s="20" t="str">
+      <x:c r="D44" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E28" s="20" t="str">
+      <x:c r="E44" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F28" s="20" t="str">
+      <x:c r="F44" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G28" s="20" t="str">
+      <x:c r="G44" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H28" s="20" t="str">
+      <x:c r="H44" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I28" s="20" t="str">
+      <x:c r="I44" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J28" s="20" t="str">
+      <x:c r="J44" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K28" s="20" t="str">
+      <x:c r="K44" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="29">
-      <x:c r="A29" s="22" t="n">
+    <x:row r="45">
+      <x:c r="A45" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B29" s="22" t="str">
+      <x:c r="B45" s="22" t="str">
         <x:v>8月3日-8月7日</x:v>
       </x:c>
-      <x:c r="C29" s="23" t="n">
-        <x:v>7391</x:v>
-      </x:c>
-      <x:c r="D29" s="23" t="n">
-        <x:v>7882.6</x:v>
-      </x:c>
-      <x:c r="E29" s="23" t="n">
-        <x:v>7335</x:v>
-      </x:c>
-      <x:c r="F29" s="23" t="n">
-        <x:v>7877.8</x:v>
-      </x:c>
-      <x:c r="G29" s="23"/>
-      <x:c r="H29" s="24"/>
-      <x:c r="I29" s="26" t="n">
-        <x:f>ROUND(D29-E29,1)</x:f>
-        <x:v>547.6</x:v>
-      </x:c>
-      <x:c r="J29" s="22" t="str">
-        <x:v>IC2609</x:v>
-      </x:c>
-      <x:c r="K29" s="22" t="n">
+      <x:c r="C45" s="23" t="n">
+        <x:v>2882.4</x:v>
+      </x:c>
+      <x:c r="D45" s="23" t="n">
+        <x:v>2930.6</x:v>
+      </x:c>
+      <x:c r="E45" s="23" t="n">
+        <x:v>2845.8</x:v>
+      </x:c>
+      <x:c r="F45" s="23" t="n">
+        <x:v>2930</x:v>
+      </x:c>
+      <x:c r="G45" s="23"/>
+      <x:c r="H45" s="24"/>
+      <x:c r="I45" s="26" t="n">
+        <x:f>ROUND(D45-E45,1)</x:f>
+        <x:v>84.8</x:v>
+      </x:c>
+      <x:c r="J45" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+      <x:c r="K45" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="30">
-      <x:c r="A30" s="29" t="str">
+    <x:row r="46">
+      <x:c r="A46" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B30" s="28" t="n">
+      <x:c r="B46" s="28" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C30" s="28"/>
-      <x:c r="D30" s="28"/>
-      <x:c r="E30" s="28"/>
-      <x:c r="F30" s="28"/>
-      <x:c r="G30" s="28"/>
-      <x:c r="H30" s="28"/>
-      <x:c r="I30" s="30" t="n">
-        <x:f>ROUND(SUM(I29:I29),1)</x:f>
-        <x:v>547.6</x:v>
-      </x:c>
-      <x:c r="J30" s="28"/>
-      <x:c r="K30" s="28"/>
-    </x:row>
-    <x:row r="31">
-      <x:c r="A31" s="29" t="str">
+      <x:c r="C46" s="28"/>
+      <x:c r="D46" s="28"/>
+      <x:c r="E46" s="28"/>
+      <x:c r="F46" s="28"/>
+      <x:c r="G46" s="28"/>
+      <x:c r="H46" s="28"/>
+      <x:c r="I46" s="30" t="n">
+        <x:f>ROUND(SUM(I45:I45),1)</x:f>
+        <x:v>84.8</x:v>
+      </x:c>
+      <x:c r="J46" s="28"/>
+      <x:c r="K46" s="28"/>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B31" s="28"/>
-      <x:c r="C31" s="28"/>
-      <x:c r="D31" s="28"/>
-      <x:c r="E31" s="28"/>
-      <x:c r="F31" s="28"/>
-      <x:c r="G31" s="28"/>
-      <x:c r="H31" s="28"/>
-      <x:c r="I31" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I29:I29),0),1)</x:f>
-        <x:v>547.6</x:v>
-      </x:c>
-      <x:c r="J31" s="28"/>
-      <x:c r="K31" s="28"/>
-    </x:row>
-    <x:row r="33">
-      <x:c r="A33" s="17" t="str">
-        <x:v>IF主力</x:v>
-      </x:c>
-      <x:c r="B33" s="17"/>
-      <x:c r="C33" s="17"/>
-      <x:c r="D33" s="17"/>
-      <x:c r="E33" s="17"/>
-      <x:c r="F33" s="17"/>
-      <x:c r="G33" s="17"/>
-      <x:c r="H33" s="17"/>
-      <x:c r="I33" s="17"/>
-      <x:c r="J33" s="17"/>
-      <x:c r="K33" s="17"/>
-    </x:row>
-    <x:row r="34">
-      <x:c r="A34" s="20" t="str">
+      <x:c r="B47" s="28"/>
+      <x:c r="C47" s="28"/>
+      <x:c r="D47" s="28"/>
+      <x:c r="E47" s="28"/>
+      <x:c r="F47" s="28"/>
+      <x:c r="G47" s="28"/>
+      <x:c r="H47" s="28"/>
+      <x:c r="I47" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I45:I45),0),1)</x:f>
+        <x:v>84.8</x:v>
+      </x:c>
+      <x:c r="J47" s="28"/>
+      <x:c r="K47" s="28"/>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="17" t="str">
+        <x:v>碳酸锂2609</x:v>
+      </x:c>
+      <x:c r="B49" s="17"/>
+      <x:c r="C49" s="17"/>
+      <x:c r="D49" s="17"/>
+      <x:c r="E49" s="17"/>
+      <x:c r="F49" s="17"/>
+      <x:c r="G49" s="17"/>
+      <x:c r="H49" s="17"/>
+      <x:c r="I49" s="17"/>
+      <x:c r="J49" s="17"/>
+      <x:c r="K49" s="17"/>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B34" s="20" t="str">
+      <x:c r="B50" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C34" s="20" t="str">
+      <x:c r="C50" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D34" s="20" t="str">
+      <x:c r="D50" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E34" s="20" t="str">
+      <x:c r="E50" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F34" s="20" t="str">
+      <x:c r="F50" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G34" s="20" t="str">
+      <x:c r="G50" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H34" s="20" t="str">
+      <x:c r="H50" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I34" s="20" t="str">
+      <x:c r="I50" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J34" s="20" t="str">
+      <x:c r="J50" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K34" s="20" t="str">
+      <x:c r="K50" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="35">
-      <x:c r="A35" s="22" t="n">
+    <x:row r="51">
+      <x:c r="A51" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B35" s="22" t="str">
+      <x:c r="B51" s="22" t="str">
         <x:v>8月3日-8月7日</x:v>
       </x:c>
-      <x:c r="C35" s="23" t="n">
-        <x:v>4526.4</x:v>
-      </x:c>
-      <x:c r="D35" s="23" t="n">
-        <x:v>4656.2</x:v>
-      </x:c>
-      <x:c r="E35" s="23" t="n">
-        <x:v>4494.2</x:v>
-      </x:c>
-      <x:c r="F35" s="23" t="n">
-        <x:v>4645.6</x:v>
-      </x:c>
-      <x:c r="G35" s="23"/>
-      <x:c r="H35" s="24"/>
-      <x:c r="I35" s="26" t="n">
-        <x:f>ROUND(D35-E35,1)</x:f>
-        <x:v>162</x:v>
-      </x:c>
-      <x:c r="J35" s="22" t="str">
-        <x:v>IF2609</x:v>
-      </x:c>
-      <x:c r="K35" s="22" t="n">
+      <x:c r="C51" s="23" t="n">
+        <x:v>137500</x:v>
+      </x:c>
+      <x:c r="D51" s="23" t="n">
+        <x:v>144800</x:v>
+      </x:c>
+      <x:c r="E51" s="23" t="n">
+        <x:v>135560</x:v>
+      </x:c>
+      <x:c r="F51" s="23" t="n">
+        <x:v>140000</x:v>
+      </x:c>
+      <x:c r="G51" s="23"/>
+      <x:c r="H51" s="24"/>
+      <x:c r="I51" s="26" t="n">
+        <x:f>ROUND(D51-E51,1)</x:f>
+        <x:v>9240</x:v>
+      </x:c>
+      <x:c r="J51" s="22" t="str">
+        <x:v>LC2609</x:v>
+      </x:c>
+      <x:c r="K51" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="36">
-      <x:c r="A36" s="29" t="str">
+    <x:row r="52">
+      <x:c r="A52" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B36" s="28" t="n">
+      <x:c r="B52" s="28" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C36" s="28"/>
-      <x:c r="D36" s="28"/>
-      <x:c r="E36" s="28"/>
-      <x:c r="F36" s="28"/>
-      <x:c r="G36" s="28"/>
-      <x:c r="H36" s="28"/>
-      <x:c r="I36" s="30" t="n">
-        <x:f>ROUND(SUM(I35:I35),1)</x:f>
-        <x:v>162</x:v>
-      </x:c>
-      <x:c r="J36" s="28"/>
-      <x:c r="K36" s="28"/>
-    </x:row>
-    <x:row r="37">
-      <x:c r="A37" s="29" t="str">
+      <x:c r="C52" s="28"/>
+      <x:c r="D52" s="28"/>
+      <x:c r="E52" s="28"/>
+      <x:c r="F52" s="28"/>
+      <x:c r="G52" s="28"/>
+      <x:c r="H52" s="28"/>
+      <x:c r="I52" s="30" t="n">
+        <x:f>ROUND(SUM(I51:I51),1)</x:f>
+        <x:v>9240</x:v>
+      </x:c>
+      <x:c r="J52" s="28"/>
+      <x:c r="K52" s="28"/>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B37" s="28"/>
-      <x:c r="C37" s="28"/>
-      <x:c r="D37" s="28"/>
-      <x:c r="E37" s="28"/>
-      <x:c r="F37" s="28"/>
-      <x:c r="G37" s="28"/>
-      <x:c r="H37" s="28"/>
-      <x:c r="I37" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I35:I35),0),1)</x:f>
-        <x:v>162</x:v>
-      </x:c>
-      <x:c r="J37" s="28"/>
-      <x:c r="K37" s="28"/>
-    </x:row>
-    <x:row r="39">
-      <x:c r="A39" s="17" t="str">
-        <x:v>IH主力</x:v>
-      </x:c>
-      <x:c r="B39" s="17"/>
-      <x:c r="C39" s="17"/>
-      <x:c r="D39" s="17"/>
-      <x:c r="E39" s="17"/>
-      <x:c r="F39" s="17"/>
-      <x:c r="G39" s="17"/>
-      <x:c r="H39" s="17"/>
-      <x:c r="I39" s="17"/>
-      <x:c r="J39" s="17"/>
-      <x:c r="K39" s="17"/>
-    </x:row>
-    <x:row r="40">
-      <x:c r="A40" s="20" t="str">
-        <x:v>序号</x:v>
-      </x:c>
-      <x:c r="B40" s="20" t="str">
-        <x:v>周期</x:v>
-      </x:c>
-      <x:c r="C40" s="20" t="str">
-        <x:v>开盘</x:v>
-      </x:c>
-      <x:c r="D40" s="20" t="str">
-        <x:v>高点</x:v>
-      </x:c>
-      <x:c r="E40" s="20" t="str">
-        <x:v>低点</x:v>
-      </x:c>
-      <x:c r="F40" s="20" t="str">
-        <x:v>收盘</x:v>
-      </x:c>
-      <x:c r="G40" s="20" t="str">
-        <x:v>涨跌点数</x:v>
-      </x:c>
-      <x:c r="H40" s="20" t="str">
-        <x:v>涨幅</x:v>
-      </x:c>
-      <x:c r="I40" s="20" t="str">
-        <x:v>振幅</x:v>
-      </x:c>
-      <x:c r="J40" s="20" t="str">
-        <x:v>标的</x:v>
-      </x:c>
-      <x:c r="K40" s="20" t="str">
-        <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="41">
-      <x:c r="A41" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B41" s="22" t="str">
-        <x:v>8月3日-8月7日</x:v>
-      </x:c>
-      <x:c r="C41" s="23" t="n">
-        <x:v>2882.4</x:v>
-      </x:c>
-      <x:c r="D41" s="23" t="n">
-        <x:v>2930.6</x:v>
-      </x:c>
-      <x:c r="E41" s="23" t="n">
-        <x:v>2845.8</x:v>
-      </x:c>
-      <x:c r="F41" s="23" t="n">
-        <x:v>2930</x:v>
-      </x:c>
-      <x:c r="G41" s="23"/>
-      <x:c r="H41" s="24"/>
-      <x:c r="I41" s="26" t="n">
-        <x:f>ROUND(D41-E41,1)</x:f>
-        <x:v>84.8</x:v>
-      </x:c>
-      <x:c r="J41" s="22" t="str">
-        <x:v>IH2609</x:v>
-      </x:c>
-      <x:c r="K41" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="42">
-      <x:c r="A42" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B42" s="28" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C42" s="28"/>
-      <x:c r="D42" s="28"/>
-      <x:c r="E42" s="28"/>
-      <x:c r="F42" s="28"/>
-      <x:c r="G42" s="28"/>
-      <x:c r="H42" s="28"/>
-      <x:c r="I42" s="30" t="n">
-        <x:f>ROUND(SUM(I41:I41),1)</x:f>
-        <x:v>84.8</x:v>
-      </x:c>
-      <x:c r="J42" s="28"/>
-      <x:c r="K42" s="28"/>
-    </x:row>
-    <x:row r="43">
-      <x:c r="A43" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B43" s="28"/>
-      <x:c r="C43" s="28"/>
-      <x:c r="D43" s="28"/>
-      <x:c r="E43" s="28"/>
-      <x:c r="F43" s="28"/>
-      <x:c r="G43" s="28"/>
-      <x:c r="H43" s="28"/>
-      <x:c r="I43" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I41:I41),0),1)</x:f>
-        <x:v>84.8</x:v>
-      </x:c>
-      <x:c r="J43" s="28"/>
-      <x:c r="K43" s="28"/>
-    </x:row>
-    <x:row r="45">
-      <x:c r="A45" s="17" t="str">
-        <x:v>碳酸锂2609</x:v>
-      </x:c>
-      <x:c r="B45" s="17"/>
-      <x:c r="C45" s="17"/>
-      <x:c r="D45" s="17"/>
-      <x:c r="E45" s="17"/>
-      <x:c r="F45" s="17"/>
-      <x:c r="G45" s="17"/>
-      <x:c r="H45" s="17"/>
-      <x:c r="I45" s="17"/>
-      <x:c r="J45" s="17"/>
-      <x:c r="K45" s="17"/>
-    </x:row>
-    <x:row r="46">
-      <x:c r="A46" s="20" t="str">
-        <x:v>序号</x:v>
-      </x:c>
-      <x:c r="B46" s="20" t="str">
-        <x:v>周期</x:v>
-      </x:c>
-      <x:c r="C46" s="20" t="str">
-        <x:v>开盘</x:v>
-      </x:c>
-      <x:c r="D46" s="20" t="str">
-        <x:v>高点</x:v>
-      </x:c>
-      <x:c r="E46" s="20" t="str">
-        <x:v>低点</x:v>
-      </x:c>
-      <x:c r="F46" s="20" t="str">
-        <x:v>收盘</x:v>
-      </x:c>
-      <x:c r="G46" s="20" t="str">
-        <x:v>涨跌点数</x:v>
-      </x:c>
-      <x:c r="H46" s="20" t="str">
-        <x:v>涨幅</x:v>
-      </x:c>
-      <x:c r="I46" s="20" t="str">
-        <x:v>振幅</x:v>
-      </x:c>
-      <x:c r="J46" s="20" t="str">
-        <x:v>标的</x:v>
-      </x:c>
-      <x:c r="K46" s="20" t="str">
-        <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="47">
-      <x:c r="A47" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B47" s="22" t="str">
-        <x:v>8月3日-8月7日</x:v>
-      </x:c>
-      <x:c r="C47" s="23" t="n">
-        <x:v>137500</x:v>
-      </x:c>
-      <x:c r="D47" s="23" t="n">
-        <x:v>144800</x:v>
-      </x:c>
-      <x:c r="E47" s="23" t="n">
-        <x:v>135560</x:v>
-      </x:c>
-      <x:c r="F47" s="23" t="n">
-        <x:v>140000</x:v>
-      </x:c>
-      <x:c r="G47" s="23"/>
-      <x:c r="H47" s="24"/>
-      <x:c r="I47" s="26" t="n">
-        <x:f>ROUND(D47-E47,1)</x:f>
+      <x:c r="B53" s="28"/>
+      <x:c r="C53" s="28"/>
+      <x:c r="D53" s="28"/>
+      <x:c r="E53" s="28"/>
+      <x:c r="F53" s="28"/>
+      <x:c r="G53" s="28"/>
+      <x:c r="H53" s="28"/>
+      <x:c r="I53" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I51:I51),0),1)</x:f>
         <x:v>9240</x:v>
       </x:c>
-      <x:c r="J47" s="22" t="str">
-        <x:v>LC2609</x:v>
-      </x:c>
-      <x:c r="K47" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="48">
-      <x:c r="A48" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B48" s="28" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C48" s="28"/>
-      <x:c r="D48" s="28"/>
-      <x:c r="E48" s="28"/>
-      <x:c r="F48" s="28"/>
-      <x:c r="G48" s="28"/>
-      <x:c r="H48" s="28"/>
-      <x:c r="I48" s="30" t="n">
-        <x:f>ROUND(SUM(I47:I47),1)</x:f>
-        <x:v>9240</x:v>
-      </x:c>
-      <x:c r="J48" s="28"/>
-      <x:c r="K48" s="28"/>
-    </x:row>
-    <x:row r="49">
-      <x:c r="A49" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B49" s="28"/>
-      <x:c r="C49" s="28"/>
-      <x:c r="D49" s="28"/>
-      <x:c r="E49" s="28"/>
-      <x:c r="F49" s="28"/>
-      <x:c r="G49" s="28"/>
-      <x:c r="H49" s="28"/>
-      <x:c r="I49" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I47:I47),0),1)</x:f>
-        <x:v>9240</x:v>
-      </x:c>
-      <x:c r="J49" s="28"/>
-      <x:c r="K49" s="28"/>
+      <x:c r="J53" s="28"/>
+      <x:c r="K53" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:K1"/>
     <x:mergeCell ref="A3:K3"/>
-    <x:mergeCell ref="A9:K9"/>
-    <x:mergeCell ref="A15:K15"/>
-    <x:mergeCell ref="A21:K21"/>
-    <x:mergeCell ref="A27:K27"/>
-    <x:mergeCell ref="A33:K33"/>
-    <x:mergeCell ref="A39:K39"/>
-    <x:mergeCell ref="A45:K45"/>
+    <x:mergeCell ref="A10:K10"/>
+    <x:mergeCell ref="A17:K17"/>
+    <x:mergeCell ref="A24:K24"/>
+    <x:mergeCell ref="A31:K31"/>
+    <x:mergeCell ref="A37:K37"/>
+    <x:mergeCell ref="A43:K43"/>
+    <x:mergeCell ref="A49:K49"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2364,31 +2516,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B11" s="28" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C11" s="28"/>
-      <x:c r="D11" s="28"/>
-      <x:c r="E11" s="28"/>
-      <x:c r="F11" s="28"/>
-      <x:c r="G11" s="28"/>
-      <x:c r="H11" s="28"/>
-      <x:c r="I11" s="28"/>
-      <x:c r="J11" s="30" t="n">
-        <x:f>SUM(J4:J8)</x:f>
-        <x:v>917.5000000000001</x:v>
-      </x:c>
-      <x:c r="K11" s="28"/>
+    <x:row r="9">
+      <x:c r="A9" s="22" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B9" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C9" s="22" t="str">
+        <x:v>8月10日</x:v>
+      </x:c>
+      <x:c r="D9" s="23" t="n">
+        <x:v>7723.38</x:v>
+      </x:c>
+      <x:c r="E9" s="23" t="n">
+        <x:v>7736.1</x:v>
+      </x:c>
+      <x:c r="F9" s="23" t="n">
+        <x:v>7621.65</x:v>
+      </x:c>
+      <x:c r="G9" s="23" t="n">
+        <x:v>7733.9</x:v>
+      </x:c>
+      <x:c r="H9" s="23" t="n">
+        <x:v>54.4</x:v>
+      </x:c>
+      <x:c r="I9" s="24" t="n">
+        <x:v>0.00707986035603736</x:v>
+      </x:c>
+      <x:c r="J9" s="23" t="n">
+        <x:f>ROUND(E9-F9,1)</x:f>
+        <x:v>114.5</x:v>
+      </x:c>
+      <x:c r="K9" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B12" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B12" s="28" t="n">
+        <x:v>6</x:v>
+      </x:c>
       <x:c r="C12" s="28"/>
       <x:c r="D12" s="28"/>
       <x:c r="E12" s="28"/>
@@ -2396,11 +2566,29 @@
       <x:c r="G12" s="28"/>
       <x:c r="H12" s="28"/>
       <x:c r="I12" s="28"/>
-      <x:c r="J12" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
-        <x:v>183.5</x:v>
+      <x:c r="J12" s="30" t="n">
+        <x:f>SUM(J4:J9)</x:f>
+        <x:v>1032</x:v>
       </x:c>
       <x:c r="K12" s="28"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B13" s="28"/>
+      <x:c r="C13" s="28"/>
+      <x:c r="D13" s="28"/>
+      <x:c r="E13" s="28"/>
+      <x:c r="F13" s="28"/>
+      <x:c r="G13" s="28"/>
+      <x:c r="H13" s="28"/>
+      <x:c r="I13" s="28"/>
+      <x:c r="J13" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J9),0),1)</x:f>
+        <x:v>172</x:v>
+      </x:c>
+      <x:c r="K13" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2647,31 +2835,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B11" s="28" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C11" s="28"/>
-      <x:c r="D11" s="28"/>
-      <x:c r="E11" s="28"/>
-      <x:c r="F11" s="28"/>
-      <x:c r="G11" s="28"/>
-      <x:c r="H11" s="28"/>
-      <x:c r="I11" s="28"/>
-      <x:c r="J11" s="30" t="n">
-        <x:f>SUM(J4:J8)</x:f>
-        <x:v>940.1</x:v>
-      </x:c>
-      <x:c r="K11" s="28"/>
+    <x:row r="9">
+      <x:c r="A9" s="22" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B9" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C9" s="22" t="str">
+        <x:v>8月10日</x:v>
+      </x:c>
+      <x:c r="D9" s="23" t="n">
+        <x:v>8003.92</x:v>
+      </x:c>
+      <x:c r="E9" s="23" t="n">
+        <x:v>8031.16</x:v>
+      </x:c>
+      <x:c r="F9" s="23" t="n">
+        <x:v>7910.84</x:v>
+      </x:c>
+      <x:c r="G9" s="23" t="n">
+        <x:v>8030.95</x:v>
+      </x:c>
+      <x:c r="H9" s="23" t="n">
+        <x:v>50.8</x:v>
+      </x:c>
+      <x:c r="I9" s="24" t="n">
+        <x:v>0.0063695784023298785</x:v>
+      </x:c>
+      <x:c r="J9" s="23" t="n">
+        <x:f>ROUND(E9-F9,1)</x:f>
+        <x:v>120.3</x:v>
+      </x:c>
+      <x:c r="K9" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B12" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B12" s="28" t="n">
+        <x:v>6</x:v>
+      </x:c>
       <x:c r="C12" s="28"/>
       <x:c r="D12" s="28"/>
       <x:c r="E12" s="28"/>
@@ -2679,11 +2885,29 @@
       <x:c r="G12" s="28"/>
       <x:c r="H12" s="28"/>
       <x:c r="I12" s="28"/>
-      <x:c r="J12" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
-        <x:v>188</x:v>
+      <x:c r="J12" s="30" t="n">
+        <x:f>SUM(J4:J9)</x:f>
+        <x:v>1060.4</x:v>
       </x:c>
       <x:c r="K12" s="28"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B13" s="28"/>
+      <x:c r="C13" s="28"/>
+      <x:c r="D13" s="28"/>
+      <x:c r="E13" s="28"/>
+      <x:c r="F13" s="28"/>
+      <x:c r="G13" s="28"/>
+      <x:c r="H13" s="28"/>
+      <x:c r="I13" s="28"/>
+      <x:c r="J13" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J9),0),1)</x:f>
+        <x:v>176.7</x:v>
+      </x:c>
+      <x:c r="K13" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2930,31 +3154,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B11" s="28" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C11" s="28"/>
-      <x:c r="D11" s="28"/>
-      <x:c r="E11" s="28"/>
-      <x:c r="F11" s="28"/>
-      <x:c r="G11" s="28"/>
-      <x:c r="H11" s="28"/>
-      <x:c r="I11" s="28"/>
-      <x:c r="J11" s="30" t="n">
-        <x:f>SUM(J4:J8)</x:f>
-        <x:v>224.8</x:v>
-      </x:c>
-      <x:c r="K11" s="28"/>
+    <x:row r="9">
+      <x:c r="A9" s="22" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B9" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C9" s="22" t="str">
+        <x:v>8月10日</x:v>
+      </x:c>
+      <x:c r="D9" s="23" t="n">
+        <x:v>3943.82</x:v>
+      </x:c>
+      <x:c r="E9" s="23" t="n">
+        <x:v>3967.59</x:v>
+      </x:c>
+      <x:c r="F9" s="23" t="n">
+        <x:v>3938.63</x:v>
+      </x:c>
+      <x:c r="G9" s="23" t="n">
+        <x:v>3966.59</x:v>
+      </x:c>
+      <x:c r="H9" s="23" t="n">
+        <x:v>26.6</x:v>
+      </x:c>
+      <x:c r="I9" s="24" t="n">
+        <x:v>0.0067385102689312415</x:v>
+      </x:c>
+      <x:c r="J9" s="23" t="n">
+        <x:f>ROUND(E9-F9,1)</x:f>
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="K9" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B12" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B12" s="28" t="n">
+        <x:v>6</x:v>
+      </x:c>
       <x:c r="C12" s="28"/>
       <x:c r="D12" s="28"/>
       <x:c r="E12" s="28"/>
@@ -2962,11 +3204,29 @@
       <x:c r="G12" s="28"/>
       <x:c r="H12" s="28"/>
       <x:c r="I12" s="28"/>
-      <x:c r="J12" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
-        <x:v>45</x:v>
+      <x:c r="J12" s="30" t="n">
+        <x:f>SUM(J4:J9)</x:f>
+        <x:v>253.8</x:v>
       </x:c>
       <x:c r="K12" s="28"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B13" s="28"/>
+      <x:c r="C13" s="28"/>
+      <x:c r="D13" s="28"/>
+      <x:c r="E13" s="28"/>
+      <x:c r="F13" s="28"/>
+      <x:c r="G13" s="28"/>
+      <x:c r="H13" s="28"/>
+      <x:c r="I13" s="28"/>
+      <x:c r="J13" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J9),0),1)</x:f>
+        <x:v>42.3</x:v>
+      </x:c>
+      <x:c r="K13" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3213,31 +3473,49 @@
         <x:v>IM2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B11" s="28" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C11" s="28"/>
-      <x:c r="D11" s="28"/>
-      <x:c r="E11" s="28"/>
-      <x:c r="F11" s="28"/>
-      <x:c r="G11" s="28"/>
-      <x:c r="H11" s="28"/>
-      <x:c r="I11" s="28"/>
-      <x:c r="J11" s="30" t="n">
-        <x:f>SUM(J4:J8)</x:f>
-        <x:v>914.8</x:v>
-      </x:c>
-      <x:c r="K11" s="28"/>
+    <x:row r="9">
+      <x:c r="A9" s="22" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B9" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C9" s="22" t="str">
+        <x:v>8月10日</x:v>
+      </x:c>
+      <x:c r="D9" s="23" t="n">
+        <x:v>7628.8</x:v>
+      </x:c>
+      <x:c r="E9" s="23" t="n">
+        <x:v>7631.2</x:v>
+      </x:c>
+      <x:c r="F9" s="23" t="n">
+        <x:v>7525</x:v>
+      </x:c>
+      <x:c r="G9" s="23" t="n">
+        <x:v>7607.2</x:v>
+      </x:c>
+      <x:c r="H9" s="23" t="n">
+        <x:v>16.6</x:v>
+      </x:c>
+      <x:c r="I9" s="24" t="n">
+        <x:v>0.002186915395357314</x:v>
+      </x:c>
+      <x:c r="J9" s="23" t="n">
+        <x:f>ROUND(E9-F9,1)</x:f>
+        <x:v>106.2</x:v>
+      </x:c>
+      <x:c r="K9" s="22" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B12" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B12" s="28" t="n">
+        <x:v>6</x:v>
+      </x:c>
       <x:c r="C12" s="28"/>
       <x:c r="D12" s="28"/>
       <x:c r="E12" s="28"/>
@@ -3245,11 +3523,29 @@
       <x:c r="G12" s="28"/>
       <x:c r="H12" s="28"/>
       <x:c r="I12" s="28"/>
-      <x:c r="J12" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
-        <x:v>183</x:v>
+      <x:c r="J12" s="30" t="n">
+        <x:f>SUM(J4:J9)</x:f>
+        <x:v>1021</x:v>
       </x:c>
       <x:c r="K12" s="28"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B13" s="28"/>
+      <x:c r="C13" s="28"/>
+      <x:c r="D13" s="28"/>
+      <x:c r="E13" s="28"/>
+      <x:c r="F13" s="28"/>
+      <x:c r="G13" s="28"/>
+      <x:c r="H13" s="28"/>
+      <x:c r="I13" s="28"/>
+      <x:c r="J13" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J9),0),1)</x:f>
+        <x:v>170.2</x:v>
+      </x:c>
+      <x:c r="K13" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-08-11
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R572ebea8cd6d4572"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R1d4b8289dd384b0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R5e8e360336934895"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rfacf5e51f26e4ad7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Rf68f9dd31afc432d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R189483cacf0c4fe7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R79fc5639920c465e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R2be4e568adcb4985"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R703f6bbaee8349ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="Raa043f1c35ac4c60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R8f5d80af2dab49f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Ra945f639a3634dfb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Rf25d3aaf1ac54a06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R0f1f1b86064e407e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R5739fa15f46045d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rdb20aafd02fc4d92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Rfbaafecdc5074912"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R265f4d2596de4dd1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Re382ca6ae45a40b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="Rcdb1d6a989f0410b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -485,25 +485,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-08-10</x:v>
+        <x:v>2026-08-11</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7736.1</x:v>
+        <x:v>7789.21</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7621.65</x:v>
+        <x:v>7642.44</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>114.5</x:v>
+        <x:v>146.8</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>1032</x:v>
+        <x:v>1178.8</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>172</x:v>
+        <x:v>168.4</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -514,25 +514,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-08-10</x:v>
+        <x:v>2026-08-11</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>8031.16</x:v>
+        <x:v>8078.36</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7910.84</x:v>
+        <x:v>7947.67</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>120.3</x:v>
+        <x:v>130.7</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>1060.4</x:v>
+        <x:v>1191.1</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>176.7</x:v>
+        <x:v>170.2</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -543,25 +543,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-08-10</x:v>
+        <x:v>2026-08-11</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3967.59</x:v>
+        <x:v>3966.39</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3938.63</x:v>
+        <x:v>3930.64</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>29</x:v>
+        <x:v>35.8</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>253.8</x:v>
+        <x:v>289.6</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>42.3</x:v>
+        <x:v>41.4</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -688,25 +688,25 @@
         <x:v>碳酸锂2609</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>2026-08-10</x:v>
+        <x:v>2026-08-11</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:v>146380</x:v>
+        <x:v>146680</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
-        <x:v>139280</x:v>
+        <x:v>143500</x:v>
       </x:c>
       <x:c r="E11" s="12" t="n">
-        <x:v>7100</x:v>
+        <x:v>3180</x:v>
       </x:c>
       <x:c r="F11" s="9" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G11" s="10" t="n">
-        <x:v>32200</x:v>
+        <x:v>35380</x:v>
       </x:c>
       <x:c r="H11" s="10" t="n">
-        <x:v>5366.7</x:v>
+        <x:v>5054.3</x:v>
       </x:c>
       <x:c r="I11" s="10" t="n">
         <x:v>6000</x:v>
@@ -720,7 +720,7 @@
         <x:v>2026-08-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-08-10</x:v>
+        <x:v>2026-08-11</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1119,31 +1119,49 @@
         <x:v>LC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B12" s="28" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="C12" s="28"/>
-      <x:c r="D12" s="28"/>
-      <x:c r="E12" s="28"/>
-      <x:c r="F12" s="28"/>
-      <x:c r="G12" s="28"/>
-      <x:c r="H12" s="28"/>
-      <x:c r="I12" s="28"/>
-      <x:c r="J12" s="30" t="n">
-        <x:f>SUM(J4:J9)</x:f>
-        <x:v>32200</x:v>
-      </x:c>
-      <x:c r="K12" s="28"/>
+    <x:row r="10">
+      <x:c r="A10" s="22" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B10" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C10" s="22" t="str">
+        <x:v>8月11日</x:v>
+      </x:c>
+      <x:c r="D10" s="23" t="n">
+        <x:v>146500</x:v>
+      </x:c>
+      <x:c r="E10" s="23" t="n">
+        <x:v>146680</x:v>
+      </x:c>
+      <x:c r="F10" s="23" t="n">
+        <x:v>143500</x:v>
+      </x:c>
+      <x:c r="G10" s="23" t="n">
+        <x:v>145860</x:v>
+      </x:c>
+      <x:c r="H10" s="34" t="n">
+        <x:v>-500</x:v>
+      </x:c>
+      <x:c r="I10" s="24" t="n">
+        <x:v>-0.0034162339437004974</x:v>
+      </x:c>
+      <x:c r="J10" s="23" t="n">
+        <x:f>ROUND(E10-F10,1)</x:f>
+        <x:v>3180</x:v>
+      </x:c>
+      <x:c r="K10" s="22" t="str">
+        <x:v>LC2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B13" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B13" s="28" t="n">
+        <x:v>7</x:v>
+      </x:c>
       <x:c r="C13" s="28"/>
       <x:c r="D13" s="28"/>
       <x:c r="E13" s="28"/>
@@ -1151,11 +1169,29 @@
       <x:c r="G13" s="28"/>
       <x:c r="H13" s="28"/>
       <x:c r="I13" s="28"/>
-      <x:c r="J13" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J9),0),1)</x:f>
-        <x:v>5366.7</x:v>
+      <x:c r="J13" s="30" t="n">
+        <x:f>SUM(J4:J10)</x:f>
+        <x:v>35380</x:v>
       </x:c>
       <x:c r="K13" s="28"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B14" s="28"/>
+      <x:c r="C14" s="28"/>
+      <x:c r="D14" s="28"/>
+      <x:c r="E14" s="28"/>
+      <x:c r="F14" s="28"/>
+      <x:c r="G14" s="28"/>
+      <x:c r="H14" s="28"/>
+      <x:c r="I14" s="28"/>
+      <x:c r="J14" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J10),0),1)</x:f>
+        <x:v>5054.3</x:v>
+      </x:c>
+      <x:c r="K14" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1274,37 +1310,37 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B6" s="22" t="str">
-        <x:v>8月10日</x:v>
+        <x:v>8月10日-8月11日</x:v>
       </x:c>
       <x:c r="C6" s="23" t="n">
         <x:v>7723.38</x:v>
       </x:c>
       <x:c r="D6" s="23" t="n">
-        <x:v>7736.1</x:v>
+        <x:v>7789.21</x:v>
       </x:c>
       <x:c r="E6" s="23" t="n">
         <x:v>7621.65</x:v>
       </x:c>
       <x:c r="F6" s="23" t="n">
-        <x:v>7733.9</x:v>
+        <x:v>7698.05</x:v>
       </x:c>
       <x:c r="G6" s="23" t="n">
         <x:f>ROUND(F6-F5,1)</x:f>
-        <x:v>54.4</x:v>
+        <x:v>18.5</x:v>
       </x:c>
       <x:c r="H6" s="24" t="n">
         <x:f>IFERROR(F6/F5-1,"")</x:f>
-        <x:v>0.00707986035603736</x:v>
+        <x:v>0.002411605918591464</x:v>
       </x:c>
       <x:c r="I6" s="23" t="n">
         <x:f>ROUND(D6-E6,1)</x:f>
-        <x:v>114.5</x:v>
+        <x:v>167.6</x:v>
       </x:c>
       <x:c r="J6" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K6" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1322,7 +1358,7 @@
       <x:c r="H7" s="28"/>
       <x:c r="I7" s="30" t="n">
         <x:f>ROUND(SUM(I5:I6),1)</x:f>
-        <x:v>757.2</x:v>
+        <x:v>810.3</x:v>
       </x:c>
       <x:c r="J7" s="28"/>
       <x:c r="K7" s="28"/>
@@ -1340,7 +1376,7 @@
       <x:c r="H8" s="28"/>
       <x:c r="I8" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I6),0),1)</x:f>
-        <x:v>378.6</x:v>
+        <x:v>405.2</x:v>
       </x:c>
       <x:c r="J8" s="28"/>
       <x:c r="K8" s="28"/>
@@ -1432,37 +1468,37 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B13" s="22" t="str">
-        <x:v>8月10日</x:v>
+        <x:v>8月10日-8月11日</x:v>
       </x:c>
       <x:c r="C13" s="23" t="n">
         <x:v>8003.92</x:v>
       </x:c>
       <x:c r="D13" s="23" t="n">
-        <x:v>8031.16</x:v>
+        <x:v>8078.36</x:v>
       </x:c>
       <x:c r="E13" s="23" t="n">
         <x:v>7910.84</x:v>
       </x:c>
       <x:c r="F13" s="23" t="n">
-        <x:v>8030.95</x:v>
+        <x:v>7967.54</x:v>
       </x:c>
       <x:c r="G13" s="23" t="n">
         <x:f>ROUND(F13-F12,1)</x:f>
-        <x:v>50.8</x:v>
+        <x:v>-12.6</x:v>
       </x:c>
       <x:c r="H13" s="24" t="n">
         <x:f>IFERROR(F13/F12-1,"")</x:f>
-        <x:v>0.0063695784023298785</x:v>
-      </x:c>
-      <x:c r="I13" s="23" t="n">
+        <x:v>-0.0015764173972321327</x:v>
+      </x:c>
+      <x:c r="I13" s="26" t="n">
         <x:f>ROUND(D13-E13,1)</x:f>
-        <x:v>120.3</x:v>
+        <x:v>167.5</x:v>
       </x:c>
       <x:c r="J13" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K13" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -1480,7 +1516,7 @@
       <x:c r="H14" s="28"/>
       <x:c r="I14" s="30" t="n">
         <x:f>ROUND(SUM(I12:I13),1)</x:f>
-        <x:v>705.5</x:v>
+        <x:v>752.7</x:v>
       </x:c>
       <x:c r="J14" s="28"/>
       <x:c r="K14" s="28"/>
@@ -1498,7 +1534,7 @@
       <x:c r="H15" s="28"/>
       <x:c r="I15" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I12:I13),0),1)</x:f>
-        <x:v>352.8</x:v>
+        <x:v>376.4</x:v>
       </x:c>
       <x:c r="J15" s="28"/>
       <x:c r="K15" s="28"/>
@@ -1590,7 +1626,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B20" s="22" t="str">
-        <x:v>8月10日</x:v>
+        <x:v>8月10日-8月11日</x:v>
       </x:c>
       <x:c r="C20" s="23" t="n">
         <x:v>3943.82</x:v>
@@ -1599,28 +1635,28 @@
         <x:v>3967.59</x:v>
       </x:c>
       <x:c r="E20" s="23" t="n">
-        <x:v>3938.63</x:v>
+        <x:v>3930.64</x:v>
       </x:c>
       <x:c r="F20" s="23" t="n">
-        <x:v>3966.59</x:v>
+        <x:v>3934.09</x:v>
       </x:c>
       <x:c r="G20" s="23" t="n">
         <x:f>ROUND(F20-F19,1)</x:f>
-        <x:v>26.6</x:v>
+        <x:v>-5.9</x:v>
       </x:c>
       <x:c r="H20" s="24" t="n">
         <x:f>IFERROR(F20/F19-1,"")</x:f>
-        <x:v>0.0067385102689312415</x:v>
+        <x:v>-0.0015101369529242348</x:v>
       </x:c>
       <x:c r="I20" s="23" t="n">
         <x:f>ROUND(D20-E20,1)</x:f>
-        <x:v>29</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="J20" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K20" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -1638,7 +1674,7 @@
       <x:c r="H21" s="28"/>
       <x:c r="I21" s="30" t="n">
         <x:f>ROUND(SUM(I19:I20),1)</x:f>
-        <x:v>172.3</x:v>
+        <x:v>180.3</x:v>
       </x:c>
       <x:c r="J21" s="28"/>
       <x:c r="K21" s="28"/>
@@ -1656,7 +1692,7 @@
       <x:c r="H22" s="28"/>
       <x:c r="I22" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I19:I20),0),1)</x:f>
-        <x:v>86.2</x:v>
+        <x:v>90.2</x:v>
       </x:c>
       <x:c r="J22" s="28"/>
       <x:c r="K22" s="28"/>
@@ -2380,37 +2416,37 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B55" s="22" t="str">
-        <x:v>8月10日</x:v>
+        <x:v>8月10日-8月11日</x:v>
       </x:c>
       <x:c r="C55" s="23" t="n">
         <x:v>140500</x:v>
       </x:c>
       <x:c r="D55" s="23" t="n">
-        <x:v>146380</x:v>
+        <x:v>146680</x:v>
       </x:c>
       <x:c r="E55" s="23" t="n">
         <x:v>139280</x:v>
       </x:c>
       <x:c r="F55" s="23" t="n">
-        <x:v>146360</x:v>
+        <x:v>145860</x:v>
       </x:c>
       <x:c r="G55" s="34" t="n">
         <x:f>ROUND(F55-F54,1)</x:f>
-        <x:v>6360</x:v>
+        <x:v>5860</x:v>
       </x:c>
       <x:c r="H55" s="24" t="n">
         <x:f>IFERROR(F55/F54-1,"")</x:f>
-        <x:v>0.045428571428571374</x:v>
+        <x:v>0.041857142857142815</x:v>
       </x:c>
       <x:c r="I55" s="26" t="n">
         <x:f>ROUND(D55-E55,1)</x:f>
-        <x:v>7100</x:v>
+        <x:v>7400</x:v>
       </x:c>
       <x:c r="J55" s="22" t="str">
         <x:v>LC2609</x:v>
       </x:c>
       <x:c r="K55" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -2428,7 +2464,7 @@
       <x:c r="H56" s="28"/>
       <x:c r="I56" s="30" t="n">
         <x:f>ROUND(SUM(I54:I55),1)</x:f>
-        <x:v>16340</x:v>
+        <x:v>16640</x:v>
       </x:c>
       <x:c r="J56" s="28"/>
       <x:c r="K56" s="28"/>
@@ -2446,7 +2482,7 @@
       <x:c r="H57" s="28"/>
       <x:c r="I57" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I54:I55),0),1)</x:f>
-        <x:v>8170</x:v>
+        <x:v>8320</x:v>
       </x:c>
       <x:c r="J57" s="28"/>
       <x:c r="K57" s="28"/>
@@ -2740,31 +2776,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B12" s="28" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="C12" s="28"/>
-      <x:c r="D12" s="28"/>
-      <x:c r="E12" s="28"/>
-      <x:c r="F12" s="28"/>
-      <x:c r="G12" s="28"/>
-      <x:c r="H12" s="28"/>
-      <x:c r="I12" s="28"/>
-      <x:c r="J12" s="30" t="n">
-        <x:f>SUM(J4:J9)</x:f>
-        <x:v>1032</x:v>
-      </x:c>
-      <x:c r="K12" s="28"/>
+    <x:row r="10">
+      <x:c r="A10" s="22" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B10" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C10" s="22" t="str">
+        <x:v>8月11日</x:v>
+      </x:c>
+      <x:c r="D10" s="23" t="n">
+        <x:v>7686.04</x:v>
+      </x:c>
+      <x:c r="E10" s="23" t="n">
+        <x:v>7789.21</x:v>
+      </x:c>
+      <x:c r="F10" s="23" t="n">
+        <x:v>7642.44</x:v>
+      </x:c>
+      <x:c r="G10" s="23" t="n">
+        <x:v>7698.05</x:v>
+      </x:c>
+      <x:c r="H10" s="23" t="n">
+        <x:v>-35.8</x:v>
+      </x:c>
+      <x:c r="I10" s="24" t="n">
+        <x:v>-0.004635436196485543</x:v>
+      </x:c>
+      <x:c r="J10" s="23" t="n">
+        <x:f>ROUND(E10-F10,1)</x:f>
+        <x:v>146.8</x:v>
+      </x:c>
+      <x:c r="K10" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B13" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B13" s="28" t="n">
+        <x:v>7</x:v>
+      </x:c>
       <x:c r="C13" s="28"/>
       <x:c r="D13" s="28"/>
       <x:c r="E13" s="28"/>
@@ -2772,11 +2826,29 @@
       <x:c r="G13" s="28"/>
       <x:c r="H13" s="28"/>
       <x:c r="I13" s="28"/>
-      <x:c r="J13" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J9),0),1)</x:f>
-        <x:v>172</x:v>
+      <x:c r="J13" s="30" t="n">
+        <x:f>SUM(J4:J10)</x:f>
+        <x:v>1178.8</x:v>
       </x:c>
       <x:c r="K13" s="28"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B14" s="28"/>
+      <x:c r="C14" s="28"/>
+      <x:c r="D14" s="28"/>
+      <x:c r="E14" s="28"/>
+      <x:c r="F14" s="28"/>
+      <x:c r="G14" s="28"/>
+      <x:c r="H14" s="28"/>
+      <x:c r="I14" s="28"/>
+      <x:c r="J14" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J10),0),1)</x:f>
+        <x:v>168.4</x:v>
+      </x:c>
+      <x:c r="K14" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3059,31 +3131,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B12" s="28" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="C12" s="28"/>
-      <x:c r="D12" s="28"/>
-      <x:c r="E12" s="28"/>
-      <x:c r="F12" s="28"/>
-      <x:c r="G12" s="28"/>
-      <x:c r="H12" s="28"/>
-      <x:c r="I12" s="28"/>
-      <x:c r="J12" s="30" t="n">
-        <x:f>SUM(J4:J9)</x:f>
-        <x:v>1060.4</x:v>
-      </x:c>
-      <x:c r="K12" s="28"/>
+    <x:row r="10">
+      <x:c r="A10" s="22" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B10" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C10" s="22" t="str">
+        <x:v>8月11日</x:v>
+      </x:c>
+      <x:c r="D10" s="23" t="n">
+        <x:v>7979.28</x:v>
+      </x:c>
+      <x:c r="E10" s="23" t="n">
+        <x:v>8078.36</x:v>
+      </x:c>
+      <x:c r="F10" s="23" t="n">
+        <x:v>7947.67</x:v>
+      </x:c>
+      <x:c r="G10" s="23" t="n">
+        <x:v>7967.54</x:v>
+      </x:c>
+      <x:c r="H10" s="23" t="n">
+        <x:v>-63.4</x:v>
+      </x:c>
+      <x:c r="I10" s="24" t="n">
+        <x:v>-0.007895703497095563</x:v>
+      </x:c>
+      <x:c r="J10" s="23" t="n">
+        <x:f>ROUND(E10-F10,1)</x:f>
+        <x:v>130.7</x:v>
+      </x:c>
+      <x:c r="K10" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B13" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B13" s="28" t="n">
+        <x:v>7</x:v>
+      </x:c>
       <x:c r="C13" s="28"/>
       <x:c r="D13" s="28"/>
       <x:c r="E13" s="28"/>
@@ -3091,11 +3181,29 @@
       <x:c r="G13" s="28"/>
       <x:c r="H13" s="28"/>
       <x:c r="I13" s="28"/>
-      <x:c r="J13" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J9),0),1)</x:f>
-        <x:v>176.7</x:v>
+      <x:c r="J13" s="30" t="n">
+        <x:f>SUM(J4:J10)</x:f>
+        <x:v>1191.1000000000001</x:v>
       </x:c>
       <x:c r="K13" s="28"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B14" s="28"/>
+      <x:c r="C14" s="28"/>
+      <x:c r="D14" s="28"/>
+      <x:c r="E14" s="28"/>
+      <x:c r="F14" s="28"/>
+      <x:c r="G14" s="28"/>
+      <x:c r="H14" s="28"/>
+      <x:c r="I14" s="28"/>
+      <x:c r="J14" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J10),0),1)</x:f>
+        <x:v>170.2</x:v>
+      </x:c>
+      <x:c r="K14" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3378,31 +3486,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B12" s="28" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="C12" s="28"/>
-      <x:c r="D12" s="28"/>
-      <x:c r="E12" s="28"/>
-      <x:c r="F12" s="28"/>
-      <x:c r="G12" s="28"/>
-      <x:c r="H12" s="28"/>
-      <x:c r="I12" s="28"/>
-      <x:c r="J12" s="30" t="n">
-        <x:f>SUM(J4:J9)</x:f>
-        <x:v>253.8</x:v>
-      </x:c>
-      <x:c r="K12" s="28"/>
+    <x:row r="10">
+      <x:c r="A10" s="22" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B10" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C10" s="22" t="str">
+        <x:v>8月11日</x:v>
+      </x:c>
+      <x:c r="D10" s="23" t="n">
+        <x:v>3950.71</x:v>
+      </x:c>
+      <x:c r="E10" s="23" t="n">
+        <x:v>3966.39</x:v>
+      </x:c>
+      <x:c r="F10" s="23" t="n">
+        <x:v>3930.64</x:v>
+      </x:c>
+      <x:c r="G10" s="23" t="n">
+        <x:v>3934.09</x:v>
+      </x:c>
+      <x:c r="H10" s="23" t="n">
+        <x:v>-32.5</x:v>
+      </x:c>
+      <x:c r="I10" s="24" t="n">
+        <x:v>-0.008193435671445704</x:v>
+      </x:c>
+      <x:c r="J10" s="23" t="n">
+        <x:f>ROUND(E10-F10,1)</x:f>
+        <x:v>35.8</x:v>
+      </x:c>
+      <x:c r="K10" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B13" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B13" s="28" t="n">
+        <x:v>7</x:v>
+      </x:c>
       <x:c r="C13" s="28"/>
       <x:c r="D13" s="28"/>
       <x:c r="E13" s="28"/>
@@ -3410,11 +3536,29 @@
       <x:c r="G13" s="28"/>
       <x:c r="H13" s="28"/>
       <x:c r="I13" s="28"/>
-      <x:c r="J13" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J9),0),1)</x:f>
-        <x:v>42.3</x:v>
+      <x:c r="J13" s="30" t="n">
+        <x:f>SUM(J4:J10)</x:f>
+        <x:v>289.6</x:v>
       </x:c>
       <x:c r="K13" s="28"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B14" s="28"/>
+      <x:c r="C14" s="28"/>
+      <x:c r="D14" s="28"/>
+      <x:c r="E14" s="28"/>
+      <x:c r="F14" s="28"/>
+      <x:c r="G14" s="28"/>
+      <x:c r="H14" s="28"/>
+      <x:c r="I14" s="28"/>
+      <x:c r="J14" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J10),0),1)</x:f>
+        <x:v>41.4</x:v>
+      </x:c>
+      <x:c r="K14" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-08-12
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rcabbdbddd3ba4918"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Rc858fb77e43f4bd8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Rb753c2e673544334"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R7763ee952ea04ee5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Ra3945aa68ff64132"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R8d457db0e5e846f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R35451bab023c4241"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rfdbe59e4ef8a438c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R488e612d4e584964"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R948015195afe4481"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R5b8fc48de09c4777"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R2a97bf1645b84953"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Rc0a2b9296d3a4d94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rbb8e02c1a8d846c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R9ceb2ba781f14468"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rd6646227e1374f9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Rb6f5714077ff4147"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R4f69930df5a94d7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R997f1229234b4a0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R3111d0df69b0448d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -485,25 +485,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-08-11</x:v>
+        <x:v>2026-08-12</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7789.21</x:v>
+        <x:v>7805.27</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7642.44</x:v>
+        <x:v>7692.44</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>146.8</x:v>
+        <x:v>112.8</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>1178.8</x:v>
+        <x:v>1291.6</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>168.4</x:v>
+        <x:v>161.5</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -514,25 +514,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-08-11</x:v>
+        <x:v>2026-08-12</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>8078.36</x:v>
+        <x:v>8067.53</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7947.67</x:v>
+        <x:v>7961.83</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>130.7</x:v>
+        <x:v>105.7</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>1191.1</x:v>
+        <x:v>1296.8</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>170.2</x:v>
+        <x:v>162.1</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -543,25 +543,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-08-11</x:v>
+        <x:v>2026-08-12</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3966.39</x:v>
+        <x:v>3950.62</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3930.64</x:v>
+        <x:v>3927.55</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>35.8</x:v>
+        <x:v>23.1</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>289.6</x:v>
+        <x:v>312.7</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>41.4</x:v>
+        <x:v>39.1</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -572,25 +572,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-08-11</x:v>
+        <x:v>2026-08-12</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>7692</x:v>
+        <x:v>7712.8</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>7547.2</x:v>
+        <x:v>7600</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>144.8</x:v>
+        <x:v>112.8</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>1165.8</x:v>
+        <x:v>1278.6</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>166.5</x:v>
+        <x:v>159.8</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -720,7 +720,7 @@
         <x:v>2026-08-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-08-11</x:v>
+        <x:v>2026-08-12</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1310,37 +1310,37 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B6" s="22" t="str">
-        <x:v>8月10日-8月11日</x:v>
+        <x:v>8月10日-8月12日</x:v>
       </x:c>
       <x:c r="C6" s="23" t="n">
         <x:v>7723.38</x:v>
       </x:c>
       <x:c r="D6" s="23" t="n">
-        <x:v>7789.21</x:v>
+        <x:v>7805.27</x:v>
       </x:c>
       <x:c r="E6" s="23" t="n">
         <x:v>7621.65</x:v>
       </x:c>
       <x:c r="F6" s="23" t="n">
-        <x:v>7698.05</x:v>
+        <x:v>7793.72</x:v>
       </x:c>
       <x:c r="G6" s="23" t="n">
         <x:f>ROUND(F6-F5,1)</x:f>
-        <x:v>18.5</x:v>
+        <x:v>114.2</x:v>
       </x:c>
       <x:c r="H6" s="24" t="n">
         <x:f>IFERROR(F6/F5-1,"")</x:f>
-        <x:v>0.002411605918591464</x:v>
-      </x:c>
-      <x:c r="I6" s="23" t="n">
+        <x:v>0.014869399559608532</x:v>
+      </x:c>
+      <x:c r="I6" s="26" t="n">
         <x:f>ROUND(D6-E6,1)</x:f>
-        <x:v>167.6</x:v>
+        <x:v>183.6</x:v>
       </x:c>
       <x:c r="J6" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K6" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1358,7 +1358,7 @@
       <x:c r="H7" s="28"/>
       <x:c r="I7" s="30" t="n">
         <x:f>ROUND(SUM(I5:I6),1)</x:f>
-        <x:v>810.3</x:v>
+        <x:v>826.3</x:v>
       </x:c>
       <x:c r="J7" s="28"/>
       <x:c r="K7" s="28"/>
@@ -1376,7 +1376,7 @@
       <x:c r="H8" s="28"/>
       <x:c r="I8" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I6),0),1)</x:f>
-        <x:v>405.2</x:v>
+        <x:v>413.2</x:v>
       </x:c>
       <x:c r="J8" s="28"/>
       <x:c r="K8" s="28"/>
@@ -1468,7 +1468,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B13" s="22" t="str">
-        <x:v>8月10日-8月11日</x:v>
+        <x:v>8月10日-8月12日</x:v>
       </x:c>
       <x:c r="C13" s="23" t="n">
         <x:v>8003.92</x:v>
@@ -1480,15 +1480,15 @@
         <x:v>7910.84</x:v>
       </x:c>
       <x:c r="F13" s="23" t="n">
-        <x:v>7967.54</x:v>
+        <x:v>8045.31</x:v>
       </x:c>
       <x:c r="G13" s="23" t="n">
         <x:f>ROUND(F13-F12,1)</x:f>
-        <x:v>-12.6</x:v>
+        <x:v>65.2</x:v>
       </x:c>
       <x:c r="H13" s="24" t="n">
         <x:f>IFERROR(F13/F12-1,"")</x:f>
-        <x:v>-0.0015764173972321327</x:v>
+        <x:v>0.00816905008947244</x:v>
       </x:c>
       <x:c r="I13" s="26" t="n">
         <x:f>ROUND(D13-E13,1)</x:f>
@@ -1498,7 +1498,7 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K13" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -1626,7 +1626,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B20" s="22" t="str">
-        <x:v>8月10日-8月11日</x:v>
+        <x:v>8月10日-8月12日</x:v>
       </x:c>
       <x:c r="C20" s="23" t="n">
         <x:v>3943.82</x:v>
@@ -1635,28 +1635,28 @@
         <x:v>3967.59</x:v>
       </x:c>
       <x:c r="E20" s="23" t="n">
-        <x:v>3930.64</x:v>
+        <x:v>3927.55</x:v>
       </x:c>
       <x:c r="F20" s="23" t="n">
-        <x:v>3934.09</x:v>
+        <x:v>3946.68</x:v>
       </x:c>
       <x:c r="G20" s="23" t="n">
         <x:f>ROUND(F20-F19,1)</x:f>
-        <x:v>-5.9</x:v>
+        <x:v>6.6</x:v>
       </x:c>
       <x:c r="H20" s="24" t="n">
         <x:f>IFERROR(F20/F19-1,"")</x:f>
-        <x:v>-0.0015101369529242348</x:v>
+        <x:v>0.001685262078557459</x:v>
       </x:c>
       <x:c r="I20" s="23" t="n">
         <x:f>ROUND(D20-E20,1)</x:f>
-        <x:v>37</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="J20" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K20" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -1674,7 +1674,7 @@
       <x:c r="H21" s="28"/>
       <x:c r="I21" s="30" t="n">
         <x:f>ROUND(SUM(I19:I20),1)</x:f>
-        <x:v>180.3</x:v>
+        <x:v>183.3</x:v>
       </x:c>
       <x:c r="J21" s="28"/>
       <x:c r="K21" s="28"/>
@@ -1692,7 +1692,7 @@
       <x:c r="H22" s="28"/>
       <x:c r="I22" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I19:I20),0),1)</x:f>
-        <x:v>90.2</x:v>
+        <x:v>91.7</x:v>
       </x:c>
       <x:c r="J22" s="28"/>
       <x:c r="K22" s="28"/>
@@ -1784,37 +1784,37 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B27" s="22" t="str">
-        <x:v>8月10日-8月11日</x:v>
+        <x:v>8月10日-8月12日</x:v>
       </x:c>
       <x:c r="C27" s="23" t="n">
         <x:v>7628.8</x:v>
       </x:c>
       <x:c r="D27" s="23" t="n">
-        <x:v>7692</x:v>
+        <x:v>7712.8</x:v>
       </x:c>
       <x:c r="E27" s="23" t="n">
         <x:v>7525</x:v>
       </x:c>
       <x:c r="F27" s="23" t="n">
-        <x:v>7613.2</x:v>
+        <x:v>7677.4</x:v>
       </x:c>
       <x:c r="G27" s="23" t="n">
         <x:f>ROUND(F27-F26,1)</x:f>
-        <x:v>22.6</x:v>
+        <x:v>86.8</x:v>
       </x:c>
       <x:c r="H27" s="24" t="n">
         <x:f>IFERROR(F27/F26-1,"")</x:f>
-        <x:v>0.0029773667430768036</x:v>
+        <x:v>0.011435196163676054</x:v>
       </x:c>
       <x:c r="I27" s="23" t="n">
         <x:f>ROUND(D27-E27,1)</x:f>
-        <x:v>167</x:v>
+        <x:v>187.8</x:v>
       </x:c>
       <x:c r="J27" s="22" t="str">
         <x:v>IM2609</x:v>
       </x:c>
       <x:c r="K27" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -1832,7 +1832,7 @@
       <x:c r="H28" s="28"/>
       <x:c r="I28" s="30" t="n">
         <x:f>ROUND(SUM(I26:I27),1)</x:f>
-        <x:v>785.2</x:v>
+        <x:v>806</x:v>
       </x:c>
       <x:c r="J28" s="28"/>
       <x:c r="K28" s="28"/>
@@ -1850,7 +1850,7 @@
       <x:c r="H29" s="28"/>
       <x:c r="I29" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I26:I27),0),1)</x:f>
-        <x:v>392.6</x:v>
+        <x:v>403</x:v>
       </x:c>
       <x:c r="J29" s="28"/>
       <x:c r="K29" s="28"/>
@@ -2812,31 +2812,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B13" s="28" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C13" s="28"/>
-      <x:c r="D13" s="28"/>
-      <x:c r="E13" s="28"/>
-      <x:c r="F13" s="28"/>
-      <x:c r="G13" s="28"/>
-      <x:c r="H13" s="28"/>
-      <x:c r="I13" s="28"/>
-      <x:c r="J13" s="30" t="n">
-        <x:f>SUM(J4:J10)</x:f>
-        <x:v>1178.8</x:v>
-      </x:c>
-      <x:c r="K13" s="28"/>
+    <x:row r="11">
+      <x:c r="A11" s="22" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B11" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C11" s="22" t="str">
+        <x:v>8月12日</x:v>
+      </x:c>
+      <x:c r="D11" s="23" t="n">
+        <x:v>7704.96</x:v>
+      </x:c>
+      <x:c r="E11" s="23" t="n">
+        <x:v>7805.27</x:v>
+      </x:c>
+      <x:c r="F11" s="23" t="n">
+        <x:v>7692.44</x:v>
+      </x:c>
+      <x:c r="G11" s="23" t="n">
+        <x:v>7793.72</x:v>
+      </x:c>
+      <x:c r="H11" s="23" t="n">
+        <x:v>95.7</x:v>
+      </x:c>
+      <x:c r="I11" s="24" t="n">
+        <x:v>0.012427822630406427</x:v>
+      </x:c>
+      <x:c r="J11" s="23" t="n">
+        <x:f>ROUND(E11-F11,1)</x:f>
+        <x:v>112.8</x:v>
+      </x:c>
+      <x:c r="K11" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B14" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B14" s="28" t="n">
+        <x:v>8</x:v>
+      </x:c>
       <x:c r="C14" s="28"/>
       <x:c r="D14" s="28"/>
       <x:c r="E14" s="28"/>
@@ -2844,11 +2862,29 @@
       <x:c r="G14" s="28"/>
       <x:c r="H14" s="28"/>
       <x:c r="I14" s="28"/>
-      <x:c r="J14" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J10),0),1)</x:f>
-        <x:v>168.4</x:v>
+      <x:c r="J14" s="30" t="n">
+        <x:f>SUM(J4:J11)</x:f>
+        <x:v>1291.6</x:v>
       </x:c>
       <x:c r="K14" s="28"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B15" s="28"/>
+      <x:c r="C15" s="28"/>
+      <x:c r="D15" s="28"/>
+      <x:c r="E15" s="28"/>
+      <x:c r="F15" s="28"/>
+      <x:c r="G15" s="28"/>
+      <x:c r="H15" s="28"/>
+      <x:c r="I15" s="28"/>
+      <x:c r="J15" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
+        <x:v>161.5</x:v>
+      </x:c>
+      <x:c r="K15" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3167,31 +3203,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B13" s="28" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C13" s="28"/>
-      <x:c r="D13" s="28"/>
-      <x:c r="E13" s="28"/>
-      <x:c r="F13" s="28"/>
-      <x:c r="G13" s="28"/>
-      <x:c r="H13" s="28"/>
-      <x:c r="I13" s="28"/>
-      <x:c r="J13" s="30" t="n">
-        <x:f>SUM(J4:J10)</x:f>
-        <x:v>1191.1000000000001</x:v>
-      </x:c>
-      <x:c r="K13" s="28"/>
+    <x:row r="11">
+      <x:c r="A11" s="22" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B11" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C11" s="22" t="str">
+        <x:v>8月12日</x:v>
+      </x:c>
+      <x:c r="D11" s="23" t="n">
+        <x:v>7978.04</x:v>
+      </x:c>
+      <x:c r="E11" s="23" t="n">
+        <x:v>8067.53</x:v>
+      </x:c>
+      <x:c r="F11" s="23" t="n">
+        <x:v>7961.83</x:v>
+      </x:c>
+      <x:c r="G11" s="23" t="n">
+        <x:v>8045.31</x:v>
+      </x:c>
+      <x:c r="H11" s="23" t="n">
+        <x:v>77.8</x:v>
+      </x:c>
+      <x:c r="I11" s="24" t="n">
+        <x:v>0.009760854667814733</x:v>
+      </x:c>
+      <x:c r="J11" s="23" t="n">
+        <x:f>ROUND(E11-F11,1)</x:f>
+        <x:v>105.7</x:v>
+      </x:c>
+      <x:c r="K11" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B14" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B14" s="28" t="n">
+        <x:v>8</x:v>
+      </x:c>
       <x:c r="C14" s="28"/>
       <x:c r="D14" s="28"/>
       <x:c r="E14" s="28"/>
@@ -3199,11 +3253,29 @@
       <x:c r="G14" s="28"/>
       <x:c r="H14" s="28"/>
       <x:c r="I14" s="28"/>
-      <x:c r="J14" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J10),0),1)</x:f>
-        <x:v>170.2</x:v>
+      <x:c r="J14" s="30" t="n">
+        <x:f>SUM(J4:J11)</x:f>
+        <x:v>1296.8000000000002</x:v>
       </x:c>
       <x:c r="K14" s="28"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B15" s="28"/>
+      <x:c r="C15" s="28"/>
+      <x:c r="D15" s="28"/>
+      <x:c r="E15" s="28"/>
+      <x:c r="F15" s="28"/>
+      <x:c r="G15" s="28"/>
+      <x:c r="H15" s="28"/>
+      <x:c r="I15" s="28"/>
+      <x:c r="J15" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
+        <x:v>162.1</x:v>
+      </x:c>
+      <x:c r="K15" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3522,31 +3594,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B13" s="28" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C13" s="28"/>
-      <x:c r="D13" s="28"/>
-      <x:c r="E13" s="28"/>
-      <x:c r="F13" s="28"/>
-      <x:c r="G13" s="28"/>
-      <x:c r="H13" s="28"/>
-      <x:c r="I13" s="28"/>
-      <x:c r="J13" s="30" t="n">
-        <x:f>SUM(J4:J10)</x:f>
-        <x:v>289.6</x:v>
-      </x:c>
-      <x:c r="K13" s="28"/>
+    <x:row r="11">
+      <x:c r="A11" s="22" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B11" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C11" s="22" t="str">
+        <x:v>8月12日</x:v>
+      </x:c>
+      <x:c r="D11" s="23" t="n">
+        <x:v>3933.55</x:v>
+      </x:c>
+      <x:c r="E11" s="23" t="n">
+        <x:v>3950.62</x:v>
+      </x:c>
+      <x:c r="F11" s="23" t="n">
+        <x:v>3927.55</x:v>
+      </x:c>
+      <x:c r="G11" s="23" t="n">
+        <x:v>3946.68</x:v>
+      </x:c>
+      <x:c r="H11" s="23" t="n">
+        <x:v>12.6</x:v>
+      </x:c>
+      <x:c r="I11" s="24" t="n">
+        <x:v>0.0032002318198107726</x:v>
+      </x:c>
+      <x:c r="J11" s="23" t="n">
+        <x:f>ROUND(E11-F11,1)</x:f>
+        <x:v>23.1</x:v>
+      </x:c>
+      <x:c r="K11" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B14" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B14" s="28" t="n">
+        <x:v>8</x:v>
+      </x:c>
       <x:c r="C14" s="28"/>
       <x:c r="D14" s="28"/>
       <x:c r="E14" s="28"/>
@@ -3554,11 +3644,29 @@
       <x:c r="G14" s="28"/>
       <x:c r="H14" s="28"/>
       <x:c r="I14" s="28"/>
-      <x:c r="J14" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J10),0),1)</x:f>
-        <x:v>41.4</x:v>
+      <x:c r="J14" s="30" t="n">
+        <x:f>SUM(J4:J11)</x:f>
+        <x:v>312.70000000000005</x:v>
       </x:c>
       <x:c r="K14" s="28"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B15" s="28"/>
+      <x:c r="C15" s="28"/>
+      <x:c r="D15" s="28"/>
+      <x:c r="E15" s="28"/>
+      <x:c r="F15" s="28"/>
+      <x:c r="G15" s="28"/>
+      <x:c r="H15" s="28"/>
+      <x:c r="I15" s="28"/>
+      <x:c r="J15" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
+        <x:v>39.1</x:v>
+      </x:c>
+      <x:c r="K15" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3877,31 +3985,49 @@
         <x:v>IM2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B13" s="28" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C13" s="28"/>
-      <x:c r="D13" s="28"/>
-      <x:c r="E13" s="28"/>
-      <x:c r="F13" s="28"/>
-      <x:c r="G13" s="28"/>
-      <x:c r="H13" s="28"/>
-      <x:c r="I13" s="28"/>
-      <x:c r="J13" s="30" t="n">
-        <x:f>SUM(J4:J10)</x:f>
-        <x:v>1165.8</x:v>
-      </x:c>
-      <x:c r="K13" s="28"/>
+    <x:row r="11">
+      <x:c r="A11" s="22" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B11" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C11" s="22" t="str">
+        <x:v>8月12日</x:v>
+      </x:c>
+      <x:c r="D11" s="23" t="n">
+        <x:v>7633.2</x:v>
+      </x:c>
+      <x:c r="E11" s="23" t="n">
+        <x:v>7712.8</x:v>
+      </x:c>
+      <x:c r="F11" s="23" t="n">
+        <x:v>7600</x:v>
+      </x:c>
+      <x:c r="G11" s="23" t="n">
+        <x:v>7677.4</x:v>
+      </x:c>
+      <x:c r="H11" s="23" t="n">
+        <x:v>64.2</x:v>
+      </x:c>
+      <x:c r="I11" s="24" t="n">
+        <x:v>0.008432722114222635</x:v>
+      </x:c>
+      <x:c r="J11" s="23" t="n">
+        <x:f>ROUND(E11-F11,1)</x:f>
+        <x:v>112.8</x:v>
+      </x:c>
+      <x:c r="K11" s="22" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B14" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B14" s="28" t="n">
+        <x:v>8</x:v>
+      </x:c>
       <x:c r="C14" s="28"/>
       <x:c r="D14" s="28"/>
       <x:c r="E14" s="28"/>
@@ -3909,11 +4035,29 @@
       <x:c r="G14" s="28"/>
       <x:c r="H14" s="28"/>
       <x:c r="I14" s="28"/>
-      <x:c r="J14" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J10),0),1)</x:f>
-        <x:v>166.5</x:v>
+      <x:c r="J14" s="30" t="n">
+        <x:f>SUM(J4:J11)</x:f>
+        <x:v>1278.6</x:v>
       </x:c>
       <x:c r="K14" s="28"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B15" s="28"/>
+      <x:c r="C15" s="28"/>
+      <x:c r="D15" s="28"/>
+      <x:c r="E15" s="28"/>
+      <x:c r="F15" s="28"/>
+      <x:c r="G15" s="28"/>
+      <x:c r="H15" s="28"/>
+      <x:c r="I15" s="28"/>
+      <x:c r="J15" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
+        <x:v>159.8</x:v>
+      </x:c>
+      <x:c r="K15" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-08-13
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R9a8ff22e8dc94244"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R0cf001af684548fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R3e93012ee91347d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rb539a8b5a9424e5b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Rb3e515278ddd487d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R5f97c2299580417e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Ra1897964a0c44123"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R4dc47a7850184cbd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R3b2f575769984c12"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="Rf6655e10dca74c6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rd51b45a790b84d2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Rcdd4882aaba34b3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R3ce1582d9d0f4299"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R6fec732ed89f48c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R3d45191dbd864252"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rdb23ff2ce1f742e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Rd831feebf80f477b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R71f515c3f3c844fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R279216c5040349e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R22eeee18f0234e9f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -485,25 +485,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-08-12</x:v>
+        <x:v>2026-08-13</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7805.27</x:v>
+        <x:v>7880.22</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7692.44</x:v>
+        <x:v>7714.37</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>112.8</x:v>
+        <x:v>165.9</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>1291.6</x:v>
+        <x:v>1457.5</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>161.5</x:v>
+        <x:v>161.9</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -514,25 +514,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-08-12</x:v>
+        <x:v>2026-08-13</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>8067.53</x:v>
+        <x:v>8142.33</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7961.83</x:v>
+        <x:v>7966.87</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>105.7</x:v>
+        <x:v>175.5</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>1296.8</x:v>
+        <x:v>1472.3</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>162.1</x:v>
+        <x:v>163.6</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -543,25 +543,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-08-12</x:v>
+        <x:v>2026-08-13</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3950.62</x:v>
+        <x:v>3968.48</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3927.55</x:v>
+        <x:v>3924.64</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>23.1</x:v>
+        <x:v>43.8</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>312.7</x:v>
+        <x:v>356.5</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>39.1</x:v>
+        <x:v>39.6</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -688,25 +688,25 @@
         <x:v>碳酸锂2609</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>2026-08-12</x:v>
+        <x:v>2026-08-13</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:v>150880</x:v>
+        <x:v>152440</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
-        <x:v>146060</x:v>
+        <x:v>147100</x:v>
       </x:c>
       <x:c r="E11" s="12" t="n">
-        <x:v>4820</x:v>
+        <x:v>5340</x:v>
       </x:c>
       <x:c r="F11" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G11" s="10" t="n">
-        <x:v>40200</x:v>
+        <x:v>45540</x:v>
       </x:c>
       <x:c r="H11" s="10" t="n">
-        <x:v>5025</x:v>
+        <x:v>5060</x:v>
       </x:c>
       <x:c r="I11" s="10" t="n">
         <x:v>6000</x:v>
@@ -720,7 +720,7 @@
         <x:v>2026-08-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-08-12</x:v>
+        <x:v>2026-08-13</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1191,31 +1191,49 @@
         <x:v>LC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B14" s="28" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C14" s="28"/>
-      <x:c r="D14" s="28"/>
-      <x:c r="E14" s="28"/>
-      <x:c r="F14" s="28"/>
-      <x:c r="G14" s="28"/>
-      <x:c r="H14" s="28"/>
-      <x:c r="I14" s="28"/>
-      <x:c r="J14" s="30" t="n">
-        <x:f>SUM(J4:J11)</x:f>
-        <x:v>40200</x:v>
-      </x:c>
-      <x:c r="K14" s="28"/>
+    <x:row r="12">
+      <x:c r="A12" s="22" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B12" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C12" s="22" t="str">
+        <x:v>8月13日</x:v>
+      </x:c>
+      <x:c r="D12" s="23" t="n">
+        <x:v>150100</x:v>
+      </x:c>
+      <x:c r="E12" s="23" t="n">
+        <x:v>152440</x:v>
+      </x:c>
+      <x:c r="F12" s="23" t="n">
+        <x:v>147100</x:v>
+      </x:c>
+      <x:c r="G12" s="23" t="n">
+        <x:v>151420</x:v>
+      </x:c>
+      <x:c r="H12" s="34" t="n">
+        <x:v>1720</x:v>
+      </x:c>
+      <x:c r="I12" s="24" t="n">
+        <x:v>0.011489645958583816</x:v>
+      </x:c>
+      <x:c r="J12" s="23" t="n">
+        <x:f>ROUND(E12-F12,1)</x:f>
+        <x:v>5340</x:v>
+      </x:c>
+      <x:c r="K12" s="22" t="str">
+        <x:v>LC2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B15" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B15" s="28" t="n">
+        <x:v>9</x:v>
+      </x:c>
       <x:c r="C15" s="28"/>
       <x:c r="D15" s="28"/>
       <x:c r="E15" s="28"/>
@@ -1223,11 +1241,29 @@
       <x:c r="G15" s="28"/>
       <x:c r="H15" s="28"/>
       <x:c r="I15" s="28"/>
-      <x:c r="J15" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
-        <x:v>5025</x:v>
+      <x:c r="J15" s="30" t="n">
+        <x:f>SUM(J4:J12)</x:f>
+        <x:v>45540</x:v>
       </x:c>
       <x:c r="K15" s="28"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B16" s="28"/>
+      <x:c r="C16" s="28"/>
+      <x:c r="D16" s="28"/>
+      <x:c r="E16" s="28"/>
+      <x:c r="F16" s="28"/>
+      <x:c r="G16" s="28"/>
+      <x:c r="H16" s="28"/>
+      <x:c r="I16" s="28"/>
+      <x:c r="J16" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J12),0),1)</x:f>
+        <x:v>5060</x:v>
+      </x:c>
+      <x:c r="K16" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1346,37 +1382,37 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B6" s="22" t="str">
-        <x:v>8月10日-8月12日</x:v>
+        <x:v>8月10日-8月13日</x:v>
       </x:c>
       <x:c r="C6" s="23" t="n">
         <x:v>7723.38</x:v>
       </x:c>
       <x:c r="D6" s="23" t="n">
-        <x:v>7805.27</x:v>
+        <x:v>7880.22</x:v>
       </x:c>
       <x:c r="E6" s="23" t="n">
         <x:v>7621.65</x:v>
       </x:c>
       <x:c r="F6" s="23" t="n">
-        <x:v>7793.72</x:v>
+        <x:v>7715.89</x:v>
       </x:c>
       <x:c r="G6" s="23" t="n">
         <x:f>ROUND(F6-F5,1)</x:f>
-        <x:v>114.2</x:v>
+        <x:v>36.4</x:v>
       </x:c>
       <x:c r="H6" s="24" t="n">
         <x:f>IFERROR(F6/F5-1,"")</x:f>
-        <x:v>0.014869399559608532</x:v>
+        <x:v>0.0047346647516191</x:v>
       </x:c>
       <x:c r="I6" s="26" t="n">
         <x:f>ROUND(D6-E6,1)</x:f>
-        <x:v>183.6</x:v>
+        <x:v>258.6</x:v>
       </x:c>
       <x:c r="J6" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K6" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1394,7 +1430,7 @@
       <x:c r="H7" s="28"/>
       <x:c r="I7" s="30" t="n">
         <x:f>ROUND(SUM(I5:I6),1)</x:f>
-        <x:v>826.3</x:v>
+        <x:v>901.3</x:v>
       </x:c>
       <x:c r="J7" s="28"/>
       <x:c r="K7" s="28"/>
@@ -1412,7 +1448,7 @@
       <x:c r="H8" s="28"/>
       <x:c r="I8" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I6),0),1)</x:f>
-        <x:v>413.2</x:v>
+        <x:v>450.7</x:v>
       </x:c>
       <x:c r="J8" s="28"/>
       <x:c r="K8" s="28"/>
@@ -1504,37 +1540,37 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B13" s="22" t="str">
-        <x:v>8月10日-8月12日</x:v>
+        <x:v>8月10日-8月13日</x:v>
       </x:c>
       <x:c r="C13" s="23" t="n">
         <x:v>8003.92</x:v>
       </x:c>
       <x:c r="D13" s="23" t="n">
-        <x:v>8078.36</x:v>
+        <x:v>8142.33</x:v>
       </x:c>
       <x:c r="E13" s="23" t="n">
         <x:v>7910.84</x:v>
       </x:c>
       <x:c r="F13" s="23" t="n">
-        <x:v>8045.31</x:v>
+        <x:v>7968.38</x:v>
       </x:c>
       <x:c r="G13" s="23" t="n">
         <x:f>ROUND(F13-F12,1)</x:f>
-        <x:v>65.2</x:v>
+        <x:v>-11.7</x:v>
       </x:c>
       <x:c r="H13" s="24" t="n">
         <x:f>IFERROR(F13/F12-1,"")</x:f>
-        <x:v>0.00816905008947244</x:v>
+        <x:v>-0.0014711558222182397</x:v>
       </x:c>
       <x:c r="I13" s="26" t="n">
         <x:f>ROUND(D13-E13,1)</x:f>
-        <x:v>167.5</x:v>
+        <x:v>231.5</x:v>
       </x:c>
       <x:c r="J13" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K13" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -1552,7 +1588,7 @@
       <x:c r="H14" s="28"/>
       <x:c r="I14" s="30" t="n">
         <x:f>ROUND(SUM(I12:I13),1)</x:f>
-        <x:v>752.7</x:v>
+        <x:v>816.7</x:v>
       </x:c>
       <x:c r="J14" s="28"/>
       <x:c r="K14" s="28"/>
@@ -1570,7 +1606,7 @@
       <x:c r="H15" s="28"/>
       <x:c r="I15" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I12:I13),0),1)</x:f>
-        <x:v>376.4</x:v>
+        <x:v>408.4</x:v>
       </x:c>
       <x:c r="J15" s="28"/>
       <x:c r="K15" s="28"/>
@@ -1662,37 +1698,37 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B20" s="22" t="str">
-        <x:v>8月10日-8月12日</x:v>
+        <x:v>8月10日-8月13日</x:v>
       </x:c>
       <x:c r="C20" s="23" t="n">
         <x:v>3943.82</x:v>
       </x:c>
       <x:c r="D20" s="23" t="n">
-        <x:v>3967.59</x:v>
+        <x:v>3968.48</x:v>
       </x:c>
       <x:c r="E20" s="23" t="n">
-        <x:v>3927.55</x:v>
+        <x:v>3924.64</x:v>
       </x:c>
       <x:c r="F20" s="23" t="n">
-        <x:v>3946.68</x:v>
+        <x:v>3926.96</x:v>
       </x:c>
       <x:c r="G20" s="23" t="n">
         <x:f>ROUND(F20-F19,1)</x:f>
-        <x:v>6.6</x:v>
+        <x:v>-13.1</x:v>
       </x:c>
       <x:c r="H20" s="24" t="n">
         <x:f>IFERROR(F20/F19-1,"")</x:f>
-        <x:v>0.001685262078557459</x:v>
+        <x:v>-0.0033197632511344777</x:v>
       </x:c>
       <x:c r="I20" s="23" t="n">
         <x:f>ROUND(D20-E20,1)</x:f>
-        <x:v>40</x:v>
+        <x:v>43.8</x:v>
       </x:c>
       <x:c r="J20" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K20" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -1710,7 +1746,7 @@
       <x:c r="H21" s="28"/>
       <x:c r="I21" s="30" t="n">
         <x:f>ROUND(SUM(I19:I20),1)</x:f>
-        <x:v>183.3</x:v>
+        <x:v>187.1</x:v>
       </x:c>
       <x:c r="J21" s="28"/>
       <x:c r="K21" s="28"/>
@@ -1728,7 +1764,7 @@
       <x:c r="H22" s="28"/>
       <x:c r="I22" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I19:I20),0),1)</x:f>
-        <x:v>91.7</x:v>
+        <x:v>93.6</x:v>
       </x:c>
       <x:c r="J22" s="28"/>
       <x:c r="K22" s="28"/>
@@ -2452,37 +2488,37 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B55" s="22" t="str">
-        <x:v>8月10日-8月12日</x:v>
+        <x:v>8月10日-8月13日</x:v>
       </x:c>
       <x:c r="C55" s="23" t="n">
         <x:v>140500</x:v>
       </x:c>
       <x:c r="D55" s="23" t="n">
-        <x:v>150880</x:v>
+        <x:v>152440</x:v>
       </x:c>
       <x:c r="E55" s="23" t="n">
         <x:v>139280</x:v>
       </x:c>
       <x:c r="F55" s="23" t="n">
-        <x:v>149700</x:v>
+        <x:v>151420</x:v>
       </x:c>
       <x:c r="G55" s="34" t="n">
         <x:f>ROUND(F55-F54,1)</x:f>
-        <x:v>9700</x:v>
+        <x:v>11420</x:v>
       </x:c>
       <x:c r="H55" s="24" t="n">
         <x:f>IFERROR(F55/F54-1,"")</x:f>
-        <x:v>0.0692857142857144</x:v>
+        <x:v>0.08157142857142863</x:v>
       </x:c>
       <x:c r="I55" s="26" t="n">
         <x:f>ROUND(D55-E55,1)</x:f>
-        <x:v>11600</x:v>
+        <x:v>13160</x:v>
       </x:c>
       <x:c r="J55" s="22" t="str">
         <x:v>LC2609</x:v>
       </x:c>
       <x:c r="K55" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -2500,7 +2536,7 @@
       <x:c r="H56" s="28"/>
       <x:c r="I56" s="30" t="n">
         <x:f>ROUND(SUM(I54:I55),1)</x:f>
-        <x:v>20840</x:v>
+        <x:v>22400</x:v>
       </x:c>
       <x:c r="J56" s="28"/>
       <x:c r="K56" s="28"/>
@@ -2518,7 +2554,7 @@
       <x:c r="H57" s="28"/>
       <x:c r="I57" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I54:I55),0),1)</x:f>
-        <x:v>10420</x:v>
+        <x:v>11200</x:v>
       </x:c>
       <x:c r="J57" s="28"/>
       <x:c r="K57" s="28"/>
@@ -2884,31 +2920,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B14" s="28" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C14" s="28"/>
-      <x:c r="D14" s="28"/>
-      <x:c r="E14" s="28"/>
-      <x:c r="F14" s="28"/>
-      <x:c r="G14" s="28"/>
-      <x:c r="H14" s="28"/>
-      <x:c r="I14" s="28"/>
-      <x:c r="J14" s="30" t="n">
-        <x:f>SUM(J4:J11)</x:f>
-        <x:v>1291.6</x:v>
-      </x:c>
-      <x:c r="K14" s="28"/>
+    <x:row r="12">
+      <x:c r="A12" s="22" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B12" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C12" s="22" t="str">
+        <x:v>8月13日</x:v>
+      </x:c>
+      <x:c r="D12" s="23" t="n">
+        <x:v>7847.24</x:v>
+      </x:c>
+      <x:c r="E12" s="23" t="n">
+        <x:v>7880.22</x:v>
+      </x:c>
+      <x:c r="F12" s="23" t="n">
+        <x:v>7714.37</x:v>
+      </x:c>
+      <x:c r="G12" s="23" t="n">
+        <x:v>7715.89</x:v>
+      </x:c>
+      <x:c r="H12" s="23" t="n">
+        <x:v>-77.8</x:v>
+      </x:c>
+      <x:c r="I12" s="24" t="n">
+        <x:v>-0.009986245335988464</x:v>
+      </x:c>
+      <x:c r="J12" s="23" t="n">
+        <x:f>ROUND(E12-F12,1)</x:f>
+        <x:v>165.9</x:v>
+      </x:c>
+      <x:c r="K12" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B15" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B15" s="28" t="n">
+        <x:v>9</x:v>
+      </x:c>
       <x:c r="C15" s="28"/>
       <x:c r="D15" s="28"/>
       <x:c r="E15" s="28"/>
@@ -2916,11 +2970,29 @@
       <x:c r="G15" s="28"/>
       <x:c r="H15" s="28"/>
       <x:c r="I15" s="28"/>
-      <x:c r="J15" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
-        <x:v>161.5</x:v>
+      <x:c r="J15" s="30" t="n">
+        <x:f>SUM(J4:J12)</x:f>
+        <x:v>1457.5</x:v>
       </x:c>
       <x:c r="K15" s="28"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B16" s="28"/>
+      <x:c r="C16" s="28"/>
+      <x:c r="D16" s="28"/>
+      <x:c r="E16" s="28"/>
+      <x:c r="F16" s="28"/>
+      <x:c r="G16" s="28"/>
+      <x:c r="H16" s="28"/>
+      <x:c r="I16" s="28"/>
+      <x:c r="J16" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J12),0),1)</x:f>
+        <x:v>161.9</x:v>
+      </x:c>
+      <x:c r="K16" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3275,31 +3347,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B14" s="28" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C14" s="28"/>
-      <x:c r="D14" s="28"/>
-      <x:c r="E14" s="28"/>
-      <x:c r="F14" s="28"/>
-      <x:c r="G14" s="28"/>
-      <x:c r="H14" s="28"/>
-      <x:c r="I14" s="28"/>
-      <x:c r="J14" s="30" t="n">
-        <x:f>SUM(J4:J11)</x:f>
-        <x:v>1296.8000000000002</x:v>
-      </x:c>
-      <x:c r="K14" s="28"/>
+    <x:row r="12">
+      <x:c r="A12" s="22" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B12" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C12" s="22" t="str">
+        <x:v>8月13日</x:v>
+      </x:c>
+      <x:c r="D12" s="23" t="n">
+        <x:v>8096.85</x:v>
+      </x:c>
+      <x:c r="E12" s="23" t="n">
+        <x:v>8142.33</x:v>
+      </x:c>
+      <x:c r="F12" s="23" t="n">
+        <x:v>7966.87</x:v>
+      </x:c>
+      <x:c r="G12" s="23" t="n">
+        <x:v>7968.38</x:v>
+      </x:c>
+      <x:c r="H12" s="23" t="n">
+        <x:v>-76.9</x:v>
+      </x:c>
+      <x:c r="I12" s="24" t="n">
+        <x:v>-0.009562092697484648</x:v>
+      </x:c>
+      <x:c r="J12" s="26" t="n">
+        <x:f>ROUND(E12-F12,1)</x:f>
+        <x:v>175.5</x:v>
+      </x:c>
+      <x:c r="K12" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B15" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B15" s="28" t="n">
+        <x:v>9</x:v>
+      </x:c>
       <x:c r="C15" s="28"/>
       <x:c r="D15" s="28"/>
       <x:c r="E15" s="28"/>
@@ -3307,11 +3397,29 @@
       <x:c r="G15" s="28"/>
       <x:c r="H15" s="28"/>
       <x:c r="I15" s="28"/>
-      <x:c r="J15" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
-        <x:v>162.1</x:v>
+      <x:c r="J15" s="30" t="n">
+        <x:f>SUM(J4:J12)</x:f>
+        <x:v>1472.3000000000002</x:v>
       </x:c>
       <x:c r="K15" s="28"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B16" s="28"/>
+      <x:c r="C16" s="28"/>
+      <x:c r="D16" s="28"/>
+      <x:c r="E16" s="28"/>
+      <x:c r="F16" s="28"/>
+      <x:c r="G16" s="28"/>
+      <x:c r="H16" s="28"/>
+      <x:c r="I16" s="28"/>
+      <x:c r="J16" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J12),0),1)</x:f>
+        <x:v>163.6</x:v>
+      </x:c>
+      <x:c r="K16" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3666,31 +3774,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B14" s="28" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C14" s="28"/>
-      <x:c r="D14" s="28"/>
-      <x:c r="E14" s="28"/>
-      <x:c r="F14" s="28"/>
-      <x:c r="G14" s="28"/>
-      <x:c r="H14" s="28"/>
-      <x:c r="I14" s="28"/>
-      <x:c r="J14" s="30" t="n">
-        <x:f>SUM(J4:J11)</x:f>
-        <x:v>312.70000000000005</x:v>
-      </x:c>
-      <x:c r="K14" s="28"/>
+    <x:row r="12">
+      <x:c r="A12" s="22" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B12" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C12" s="22" t="str">
+        <x:v>8月13日</x:v>
+      </x:c>
+      <x:c r="D12" s="23" t="n">
+        <x:v>3957.16</x:v>
+      </x:c>
+      <x:c r="E12" s="23" t="n">
+        <x:v>3968.48</x:v>
+      </x:c>
+      <x:c r="F12" s="23" t="n">
+        <x:v>3924.64</x:v>
+      </x:c>
+      <x:c r="G12" s="23" t="n">
+        <x:v>3926.96</x:v>
+      </x:c>
+      <x:c r="H12" s="23" t="n">
+        <x:v>-19.7</x:v>
+      </x:c>
+      <x:c r="I12" s="24" t="n">
+        <x:v>-0.004996604741200117</x:v>
+      </x:c>
+      <x:c r="J12" s="23" t="n">
+        <x:f>ROUND(E12-F12,1)</x:f>
+        <x:v>43.8</x:v>
+      </x:c>
+      <x:c r="K12" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B15" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B15" s="28" t="n">
+        <x:v>9</x:v>
+      </x:c>
       <x:c r="C15" s="28"/>
       <x:c r="D15" s="28"/>
       <x:c r="E15" s="28"/>
@@ -3698,11 +3824,29 @@
       <x:c r="G15" s="28"/>
       <x:c r="H15" s="28"/>
       <x:c r="I15" s="28"/>
-      <x:c r="J15" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
-        <x:v>39.1</x:v>
+      <x:c r="J15" s="30" t="n">
+        <x:f>SUM(J4:J12)</x:f>
+        <x:v>356.50000000000006</x:v>
       </x:c>
       <x:c r="K15" s="28"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B16" s="28"/>
+      <x:c r="C16" s="28"/>
+      <x:c r="D16" s="28"/>
+      <x:c r="E16" s="28"/>
+      <x:c r="F16" s="28"/>
+      <x:c r="G16" s="28"/>
+      <x:c r="H16" s="28"/>
+      <x:c r="I16" s="28"/>
+      <x:c r="J16" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J12),0),1)</x:f>
+        <x:v>39.6</x:v>
+      </x:c>
+      <x:c r="K16" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-08-14
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R4b9ef206c0f146d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R20feab403e444b19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Ra8bc42e3a77041f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Re19a1c486a8b4d53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R0ce48e760ece49f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Raf435f7664a94105"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Rad0642f144a44883"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Re3ba3f0ccbaf4693"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R332df9c349434197"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="Rc0c63f7a556d4bf0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R5937932bd6294397"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R652d8e098f1444ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R65ac4658fd3a4bab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R981ce712eb31422f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R4ec76fa4e71e4034"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R64134fac3f434e26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Rc22b03b219c34a98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R31d08eca958949b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R81c399a2237046d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="Rdee9a5e54edf4a59"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -485,25 +485,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-08-13</x:v>
+        <x:v>2026-08-14</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7880.22</x:v>
+        <x:v>7784.38</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7714.37</x:v>
+        <x:v>7673.44</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>165.9</x:v>
+        <x:v>110.9</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>1457.5</x:v>
+        <x:v>1568.4</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>161.9</x:v>
+        <x:v>156.8</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -514,25 +514,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-08-13</x:v>
+        <x:v>2026-08-14</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>8142.33</x:v>
+        <x:v>8005.15</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7966.87</x:v>
+        <x:v>7897.24</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>175.5</x:v>
+        <x:v>107.9</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>1472.3</x:v>
+        <x:v>1580.2</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>163.6</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -543,25 +543,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-08-13</x:v>
+        <x:v>2026-08-14</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3968.48</x:v>
+        <x:v>3932.64</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3924.64</x:v>
+        <x:v>3903.7</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>43.8</x:v>
+        <x:v>28.9</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>356.5</x:v>
+        <x:v>385.4</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>39.6</x:v>
+        <x:v>38.5</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -572,25 +572,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-08-13</x:v>
+        <x:v>2026-08-14</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>7776</x:v>
+        <x:v>7695</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>7627</x:v>
+        <x:v>7597.6</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>149</x:v>
+        <x:v>97.4</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>1427.6</x:v>
+        <x:v>1525</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>158.6</x:v>
+        <x:v>152.5</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -601,25 +601,25 @@
         <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>2026-08-13</x:v>
+        <x:v>2026-08-14</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:v>8024</x:v>
+        <x:v>7914</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>7860.8</x:v>
+        <x:v>7802</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>163.2</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>1461</x:v>
+        <x:v>1573</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
-        <x:v>162.3</x:v>
+        <x:v>157.3</x:v>
       </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
@@ -659,25 +659,25 @@
         <x:v>IH主力</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>2026-08-13</x:v>
+        <x:v>2026-08-14</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:v>2933.6</x:v>
+        <x:v>2910.2</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
-        <x:v>2900.6</x:v>
+        <x:v>2877</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
-        <x:v>33</x:v>
+        <x:v>33.2</x:v>
       </x:c>
       <x:c r="F10" s="9" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G10" s="10" t="n">
-        <x:v>295.6</x:v>
+        <x:v>328.8</x:v>
       </x:c>
       <x:c r="H10" s="10" t="n">
-        <x:v>32.8</x:v>
+        <x:v>32.9</x:v>
       </x:c>
       <x:c r="I10" s="10" t="n">
         <x:v>60</x:v>
@@ -720,7 +720,7 @@
         <x:v>2026-08-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-08-13</x:v>
+        <x:v>2026-08-14</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1382,7 +1382,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B6" s="22" t="str">
-        <x:v>8月10日-8月13日</x:v>
+        <x:v>8月10日-8月14日</x:v>
       </x:c>
       <x:c r="C6" s="23" t="n">
         <x:v>7723.38</x:v>
@@ -1394,15 +1394,15 @@
         <x:v>7621.65</x:v>
       </x:c>
       <x:c r="F6" s="23" t="n">
-        <x:v>7715.89</x:v>
+        <x:v>7769.82</x:v>
       </x:c>
       <x:c r="G6" s="23" t="n">
         <x:f>ROUND(F6-F5,1)</x:f>
-        <x:v>36.4</x:v>
+        <x:v>90.3</x:v>
       </x:c>
       <x:c r="H6" s="24" t="n">
         <x:f>IFERROR(F6/F5-1,"")</x:f>
-        <x:v>0.0047346647516191</x:v>
+        <x:v>0.011757229934644453</x:v>
       </x:c>
       <x:c r="I6" s="26" t="n">
         <x:f>ROUND(D6-E6,1)</x:f>
@@ -1412,7 +1412,7 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K6" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1540,7 +1540,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B13" s="22" t="str">
-        <x:v>8月10日-8月13日</x:v>
+        <x:v>8月10日-8月14日</x:v>
       </x:c>
       <x:c r="C13" s="23" t="n">
         <x:v>8003.92</x:v>
@@ -1549,28 +1549,28 @@
         <x:v>8142.33</x:v>
       </x:c>
       <x:c r="E13" s="23" t="n">
-        <x:v>7910.84</x:v>
+        <x:v>7897.24</x:v>
       </x:c>
       <x:c r="F13" s="23" t="n">
-        <x:v>7968.38</x:v>
+        <x:v>7990.33</x:v>
       </x:c>
       <x:c r="G13" s="23" t="n">
         <x:f>ROUND(F13-F12,1)</x:f>
-        <x:v>-11.7</x:v>
+        <x:v>10.2</x:v>
       </x:c>
       <x:c r="H13" s="24" t="n">
         <x:f>IFERROR(F13/F12-1,"")</x:f>
-        <x:v>-0.0014711558222182397</x:v>
+        <x:v>0.0012794293820144187</x:v>
       </x:c>
       <x:c r="I13" s="26" t="n">
         <x:f>ROUND(D13-E13,1)</x:f>
-        <x:v>231.5</x:v>
+        <x:v>245.1</x:v>
       </x:c>
       <x:c r="J13" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K13" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -1588,7 +1588,7 @@
       <x:c r="H14" s="28"/>
       <x:c r="I14" s="30" t="n">
         <x:f>ROUND(SUM(I12:I13),1)</x:f>
-        <x:v>816.7</x:v>
+        <x:v>830.3</x:v>
       </x:c>
       <x:c r="J14" s="28"/>
       <x:c r="K14" s="28"/>
@@ -1606,7 +1606,7 @@
       <x:c r="H15" s="28"/>
       <x:c r="I15" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I12:I13),0),1)</x:f>
-        <x:v>408.4</x:v>
+        <x:v>415.2</x:v>
       </x:c>
       <x:c r="J15" s="28"/>
       <x:c r="K15" s="28"/>
@@ -1698,7 +1698,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B20" s="22" t="str">
-        <x:v>8月10日-8月13日</x:v>
+        <x:v>8月10日-8月14日</x:v>
       </x:c>
       <x:c r="C20" s="23" t="n">
         <x:v>3943.82</x:v>
@@ -1707,28 +1707,28 @@
         <x:v>3968.48</x:v>
       </x:c>
       <x:c r="E20" s="23" t="n">
-        <x:v>3924.64</x:v>
+        <x:v>3903.7</x:v>
       </x:c>
       <x:c r="F20" s="23" t="n">
-        <x:v>3926.96</x:v>
+        <x:v>3927.18</x:v>
       </x:c>
       <x:c r="G20" s="23" t="n">
         <x:f>ROUND(F20-F19,1)</x:f>
-        <x:v>-13.1</x:v>
+        <x:v>-12.9</x:v>
       </x:c>
       <x:c r="H20" s="24" t="n">
         <x:f>IFERROR(F20/F19-1,"")</x:f>
-        <x:v>-0.0033197632511344777</x:v>
-      </x:c>
-      <x:c r="I20" s="23" t="n">
+        <x:v>-0.003263926254555849</x:v>
+      </x:c>
+      <x:c r="I20" s="26" t="n">
         <x:f>ROUND(D20-E20,1)</x:f>
-        <x:v>43.8</x:v>
+        <x:v>64.8</x:v>
       </x:c>
       <x:c r="J20" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K20" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -1746,7 +1746,7 @@
       <x:c r="H21" s="28"/>
       <x:c r="I21" s="30" t="n">
         <x:f>ROUND(SUM(I19:I20),1)</x:f>
-        <x:v>187.1</x:v>
+        <x:v>208.1</x:v>
       </x:c>
       <x:c r="J21" s="28"/>
       <x:c r="K21" s="28"/>
@@ -1764,7 +1764,7 @@
       <x:c r="H22" s="28"/>
       <x:c r="I22" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I19:I20),0),1)</x:f>
-        <x:v>93.6</x:v>
+        <x:v>104.1</x:v>
       </x:c>
       <x:c r="J22" s="28"/>
       <x:c r="K22" s="28"/>
@@ -1856,7 +1856,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B27" s="22" t="str">
-        <x:v>8月10日-8月13日</x:v>
+        <x:v>8月10日-8月14日</x:v>
       </x:c>
       <x:c r="C27" s="23" t="n">
         <x:v>7628.8</x:v>
@@ -1868,15 +1868,15 @@
         <x:v>7525</x:v>
       </x:c>
       <x:c r="F27" s="23" t="n">
-        <x:v>7634.2</x:v>
+        <x:v>7650.2</x:v>
       </x:c>
       <x:c r="G27" s="23" t="n">
         <x:f>ROUND(F27-F26,1)</x:f>
-        <x:v>43.6</x:v>
+        <x:v>59.6</x:v>
       </x:c>
       <x:c r="H27" s="24" t="n">
         <x:f>IFERROR(F27/F26-1,"")</x:f>
-        <x:v>0.0057439464600952395</x:v>
+        <x:v>0.007851816720680693</x:v>
       </x:c>
       <x:c r="I27" s="26" t="n">
         <x:f>ROUND(D27-E27,1)</x:f>
@@ -1886,7 +1886,7 @@
         <x:v>IM2609</x:v>
       </x:c>
       <x:c r="K27" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -2014,7 +2014,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B34" s="22" t="str">
-        <x:v>8月10日-8月13日</x:v>
+        <x:v>8月10日-8月14日</x:v>
       </x:c>
       <x:c r="C34" s="23" t="n">
         <x:v>7888</x:v>
@@ -2026,15 +2026,15 @@
         <x:v>7795.8</x:v>
       </x:c>
       <x:c r="F34" s="23" t="n">
-        <x:v>7866.2</x:v>
+        <x:v>7861.2</x:v>
       </x:c>
       <x:c r="G34" s="23" t="n">
         <x:f>ROUND(F34-F33,1)</x:f>
-        <x:v>-11.6</x:v>
+        <x:v>-16.6</x:v>
       </x:c>
       <x:c r="H34" s="24" t="n">
         <x:f>IFERROR(F34/F33-1,"")</x:f>
-        <x:v>-0.0014724923201909768</x:v>
+        <x:v>-0.0021071872857905127</x:v>
       </x:c>
       <x:c r="I34" s="26" t="n">
         <x:f>ROUND(D34-E34,1)</x:f>
@@ -2044,7 +2044,7 @@
         <x:v>IC2609</x:v>
       </x:c>
       <x:c r="K34" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -2330,7 +2330,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B48" s="22" t="str">
-        <x:v>8月10日-8月13日</x:v>
+        <x:v>8月10日-8月14日</x:v>
       </x:c>
       <x:c r="C48" s="23" t="n">
         <x:v>2930</x:v>
@@ -2339,28 +2339,28 @@
         <x:v>2949.6</x:v>
       </x:c>
       <x:c r="E48" s="23" t="n">
-        <x:v>2900.6</x:v>
+        <x:v>2877</x:v>
       </x:c>
       <x:c r="F48" s="23" t="n">
-        <x:v>2902.6</x:v>
+        <x:v>2890</x:v>
       </x:c>
       <x:c r="G48" s="23" t="n">
         <x:f>ROUND(F48-F47,1)</x:f>
-        <x:v>-27.4</x:v>
+        <x:v>-40</x:v>
       </x:c>
       <x:c r="H48" s="24" t="n">
         <x:f>IFERROR(F48/F47-1,"")</x:f>
-        <x:v>-0.009351535836177538</x:v>
-      </x:c>
-      <x:c r="I48" s="23" t="n">
+        <x:v>-0.013651877133105783</x:v>
+      </x:c>
+      <x:c r="I48" s="26" t="n">
         <x:f>ROUND(D48-E48,1)</x:f>
-        <x:v>49</x:v>
+        <x:v>72.6</x:v>
       </x:c>
       <x:c r="J48" s="22" t="str">
         <x:v>IH2609</x:v>
       </x:c>
       <x:c r="K48" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -2378,7 +2378,7 @@
       <x:c r="H49" s="28"/>
       <x:c r="I49" s="30" t="n">
         <x:f>ROUND(SUM(I47:I48),1)</x:f>
-        <x:v>133.8</x:v>
+        <x:v>157.4</x:v>
       </x:c>
       <x:c r="J49" s="28"/>
       <x:c r="K49" s="28"/>
@@ -2396,7 +2396,7 @@
       <x:c r="H50" s="28"/>
       <x:c r="I50" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I47:I48),0),1)</x:f>
-        <x:v>66.9</x:v>
+        <x:v>78.7</x:v>
       </x:c>
       <x:c r="J50" s="28"/>
       <x:c r="K50" s="28"/>
@@ -2956,31 +2956,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B15" s="28" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="C15" s="28"/>
-      <x:c r="D15" s="28"/>
-      <x:c r="E15" s="28"/>
-      <x:c r="F15" s="28"/>
-      <x:c r="G15" s="28"/>
-      <x:c r="H15" s="28"/>
-      <x:c r="I15" s="28"/>
-      <x:c r="J15" s="30" t="n">
-        <x:f>SUM(J4:J12)</x:f>
-        <x:v>1457.5</x:v>
-      </x:c>
-      <x:c r="K15" s="28"/>
+    <x:row r="13">
+      <x:c r="A13" s="22" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B13" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C13" s="22" t="str">
+        <x:v>8月14日</x:v>
+      </x:c>
+      <x:c r="D13" s="23" t="n">
+        <x:v>7750.99</x:v>
+      </x:c>
+      <x:c r="E13" s="23" t="n">
+        <x:v>7784.38</x:v>
+      </x:c>
+      <x:c r="F13" s="23" t="n">
+        <x:v>7673.44</x:v>
+      </x:c>
+      <x:c r="G13" s="23" t="n">
+        <x:v>7769.82</x:v>
+      </x:c>
+      <x:c r="H13" s="23" t="n">
+        <x:v>53.9</x:v>
+      </x:c>
+      <x:c r="I13" s="24" t="n">
+        <x:v>0.0069894723745413945</x:v>
+      </x:c>
+      <x:c r="J13" s="23" t="n">
+        <x:f>ROUND(E13-F13,1)</x:f>
+        <x:v>110.9</x:v>
+      </x:c>
+      <x:c r="K13" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B16" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B16" s="28" t="n">
+        <x:v>10</x:v>
+      </x:c>
       <x:c r="C16" s="28"/>
       <x:c r="D16" s="28"/>
       <x:c r="E16" s="28"/>
@@ -2988,11 +3006,29 @@
       <x:c r="G16" s="28"/>
       <x:c r="H16" s="28"/>
       <x:c r="I16" s="28"/>
-      <x:c r="J16" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J12),0),1)</x:f>
-        <x:v>161.9</x:v>
+      <x:c r="J16" s="30" t="n">
+        <x:f>SUM(J4:J13)</x:f>
+        <x:v>1568.4</x:v>
       </x:c>
       <x:c r="K16" s="28"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B17" s="28"/>
+      <x:c r="C17" s="28"/>
+      <x:c r="D17" s="28"/>
+      <x:c r="E17" s="28"/>
+      <x:c r="F17" s="28"/>
+      <x:c r="G17" s="28"/>
+      <x:c r="H17" s="28"/>
+      <x:c r="I17" s="28"/>
+      <x:c r="J17" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
+        <x:v>156.8</x:v>
+      </x:c>
+      <x:c r="K17" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3383,31 +3419,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B15" s="28" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="C15" s="28"/>
-      <x:c r="D15" s="28"/>
-      <x:c r="E15" s="28"/>
-      <x:c r="F15" s="28"/>
-      <x:c r="G15" s="28"/>
-      <x:c r="H15" s="28"/>
-      <x:c r="I15" s="28"/>
-      <x:c r="J15" s="30" t="n">
-        <x:f>SUM(J4:J12)</x:f>
-        <x:v>1472.3000000000002</x:v>
-      </x:c>
-      <x:c r="K15" s="28"/>
+    <x:row r="13">
+      <x:c r="A13" s="22" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B13" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C13" s="22" t="str">
+        <x:v>8月14日</x:v>
+      </x:c>
+      <x:c r="D13" s="23" t="n">
+        <x:v>7989.65</x:v>
+      </x:c>
+      <x:c r="E13" s="23" t="n">
+        <x:v>8005.15</x:v>
+      </x:c>
+      <x:c r="F13" s="23" t="n">
+        <x:v>7897.24</x:v>
+      </x:c>
+      <x:c r="G13" s="23" t="n">
+        <x:v>7990.33</x:v>
+      </x:c>
+      <x:c r="H13" s="23" t="n">
+        <x:v>21.9</x:v>
+      </x:c>
+      <x:c r="I13" s="24" t="n">
+        <x:v>0.0027546377055311932</x:v>
+      </x:c>
+      <x:c r="J13" s="23" t="n">
+        <x:f>ROUND(E13-F13,1)</x:f>
+        <x:v>107.9</x:v>
+      </x:c>
+      <x:c r="K13" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B16" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B16" s="28" t="n">
+        <x:v>10</x:v>
+      </x:c>
       <x:c r="C16" s="28"/>
       <x:c r="D16" s="28"/>
       <x:c r="E16" s="28"/>
@@ -3415,11 +3469,29 @@
       <x:c r="G16" s="28"/>
       <x:c r="H16" s="28"/>
       <x:c r="I16" s="28"/>
-      <x:c r="J16" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J12),0),1)</x:f>
-        <x:v>163.6</x:v>
+      <x:c r="J16" s="30" t="n">
+        <x:f>SUM(J4:J13)</x:f>
+        <x:v>1580.2000000000003</x:v>
       </x:c>
       <x:c r="K16" s="28"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B17" s="28"/>
+      <x:c r="C17" s="28"/>
+      <x:c r="D17" s="28"/>
+      <x:c r="E17" s="28"/>
+      <x:c r="F17" s="28"/>
+      <x:c r="G17" s="28"/>
+      <x:c r="H17" s="28"/>
+      <x:c r="I17" s="28"/>
+      <x:c r="J17" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
+        <x:v>158</x:v>
+      </x:c>
+      <x:c r="K17" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3810,31 +3882,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B15" s="28" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="C15" s="28"/>
-      <x:c r="D15" s="28"/>
-      <x:c r="E15" s="28"/>
-      <x:c r="F15" s="28"/>
-      <x:c r="G15" s="28"/>
-      <x:c r="H15" s="28"/>
-      <x:c r="I15" s="28"/>
-      <x:c r="J15" s="30" t="n">
-        <x:f>SUM(J4:J12)</x:f>
-        <x:v>356.50000000000006</x:v>
-      </x:c>
-      <x:c r="K15" s="28"/>
+    <x:row r="13">
+      <x:c r="A13" s="22" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B13" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C13" s="22" t="str">
+        <x:v>8月14日</x:v>
+      </x:c>
+      <x:c r="D13" s="23" t="n">
+        <x:v>3930.02</x:v>
+      </x:c>
+      <x:c r="E13" s="23" t="n">
+        <x:v>3932.64</x:v>
+      </x:c>
+      <x:c r="F13" s="23" t="n">
+        <x:v>3903.7</x:v>
+      </x:c>
+      <x:c r="G13" s="23" t="n">
+        <x:v>3927.18</x:v>
+      </x:c>
+      <x:c r="H13" s="23" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="I13" s="24" t="n">
+        <x:v>0.00005602297960760616</x:v>
+      </x:c>
+      <x:c r="J13" s="23" t="n">
+        <x:f>ROUND(E13-F13,1)</x:f>
+        <x:v>28.9</x:v>
+      </x:c>
+      <x:c r="K13" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B16" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B16" s="28" t="n">
+        <x:v>10</x:v>
+      </x:c>
       <x:c r="C16" s="28"/>
       <x:c r="D16" s="28"/>
       <x:c r="E16" s="28"/>
@@ -3842,11 +3932,29 @@
       <x:c r="G16" s="28"/>
       <x:c r="H16" s="28"/>
       <x:c r="I16" s="28"/>
-      <x:c r="J16" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J12),0),1)</x:f>
-        <x:v>39.6</x:v>
+      <x:c r="J16" s="30" t="n">
+        <x:f>SUM(J4:J13)</x:f>
+        <x:v>385.40000000000003</x:v>
       </x:c>
       <x:c r="K16" s="28"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B17" s="28"/>
+      <x:c r="C17" s="28"/>
+      <x:c r="D17" s="28"/>
+      <x:c r="E17" s="28"/>
+      <x:c r="F17" s="28"/>
+      <x:c r="G17" s="28"/>
+      <x:c r="H17" s="28"/>
+      <x:c r="I17" s="28"/>
+      <x:c r="J17" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
+        <x:v>38.5</x:v>
+      </x:c>
+      <x:c r="K17" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4237,31 +4345,49 @@
         <x:v>IM2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B15" s="28" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="C15" s="28"/>
-      <x:c r="D15" s="28"/>
-      <x:c r="E15" s="28"/>
-      <x:c r="F15" s="28"/>
-      <x:c r="G15" s="28"/>
-      <x:c r="H15" s="28"/>
-      <x:c r="I15" s="28"/>
-      <x:c r="J15" s="30" t="n">
-        <x:f>SUM(J4:J12)</x:f>
-        <x:v>1427.6</x:v>
-      </x:c>
-      <x:c r="K15" s="28"/>
+    <x:row r="13">
+      <x:c r="A13" s="22" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B13" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C13" s="22" t="str">
+        <x:v>8月14日</x:v>
+      </x:c>
+      <x:c r="D13" s="23" t="n">
+        <x:v>7670</x:v>
+      </x:c>
+      <x:c r="E13" s="23" t="n">
+        <x:v>7695</x:v>
+      </x:c>
+      <x:c r="F13" s="23" t="n">
+        <x:v>7597.6</x:v>
+      </x:c>
+      <x:c r="G13" s="23" t="n">
+        <x:v>7650.2</x:v>
+      </x:c>
+      <x:c r="H13" s="23" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="I13" s="24" t="n">
+        <x:v>0.0020958319142805326</x:v>
+      </x:c>
+      <x:c r="J13" s="23" t="n">
+        <x:f>ROUND(E13-F13,1)</x:f>
+        <x:v>97.4</x:v>
+      </x:c>
+      <x:c r="K13" s="22" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B16" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B16" s="28" t="n">
+        <x:v>10</x:v>
+      </x:c>
       <x:c r="C16" s="28"/>
       <x:c r="D16" s="28"/>
       <x:c r="E16" s="28"/>
@@ -4269,11 +4395,29 @@
       <x:c r="G16" s="28"/>
       <x:c r="H16" s="28"/>
       <x:c r="I16" s="28"/>
-      <x:c r="J16" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J12),0),1)</x:f>
-        <x:v>158.6</x:v>
+      <x:c r="J16" s="30" t="n">
+        <x:f>SUM(J4:J13)</x:f>
+        <x:v>1525</x:v>
       </x:c>
       <x:c r="K16" s="28"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B17" s="28"/>
+      <x:c r="C17" s="28"/>
+      <x:c r="D17" s="28"/>
+      <x:c r="E17" s="28"/>
+      <x:c r="F17" s="28"/>
+      <x:c r="G17" s="28"/>
+      <x:c r="H17" s="28"/>
+      <x:c r="I17" s="28"/>
+      <x:c r="J17" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
+        <x:v>152.5</x:v>
+      </x:c>
+      <x:c r="K17" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4664,31 +4808,49 @@
         <x:v>IC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B15" s="28" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="C15" s="28"/>
-      <x:c r="D15" s="28"/>
-      <x:c r="E15" s="28"/>
-      <x:c r="F15" s="28"/>
-      <x:c r="G15" s="28"/>
-      <x:c r="H15" s="28"/>
-      <x:c r="I15" s="28"/>
-      <x:c r="J15" s="30" t="n">
-        <x:f>SUM(J4:J12)</x:f>
-        <x:v>1461</x:v>
-      </x:c>
-      <x:c r="K15" s="28"/>
+    <x:row r="13">
+      <x:c r="A13" s="22" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B13" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C13" s="22" t="str">
+        <x:v>8月14日</x:v>
+      </x:c>
+      <x:c r="D13" s="23" t="n">
+        <x:v>7905</x:v>
+      </x:c>
+      <x:c r="E13" s="23" t="n">
+        <x:v>7914</x:v>
+      </x:c>
+      <x:c r="F13" s="23" t="n">
+        <x:v>7802</x:v>
+      </x:c>
+      <x:c r="G13" s="23" t="n">
+        <x:v>7861.2</x:v>
+      </x:c>
+      <x:c r="H13" s="23" t="n">
+        <x:v>-5</x:v>
+      </x:c>
+      <x:c r="I13" s="24" t="n">
+        <x:v>-0.0006356309272583793</x:v>
+      </x:c>
+      <x:c r="J13" s="23" t="n">
+        <x:f>ROUND(E13-F13,1)</x:f>
+        <x:v>112</x:v>
+      </x:c>
+      <x:c r="K13" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B16" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B16" s="28" t="n">
+        <x:v>10</x:v>
+      </x:c>
       <x:c r="C16" s="28"/>
       <x:c r="D16" s="28"/>
       <x:c r="E16" s="28"/>
@@ -4696,11 +4858,29 @@
       <x:c r="G16" s="28"/>
       <x:c r="H16" s="28"/>
       <x:c r="I16" s="28"/>
-      <x:c r="J16" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J12),0),1)</x:f>
-        <x:v>162.3</x:v>
+      <x:c r="J16" s="30" t="n">
+        <x:f>SUM(J4:J13)</x:f>
+        <x:v>1573</x:v>
       </x:c>
       <x:c r="K16" s="28"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B17" s="28"/>
+      <x:c r="C17" s="28"/>
+      <x:c r="D17" s="28"/>
+      <x:c r="E17" s="28"/>
+      <x:c r="F17" s="28"/>
+      <x:c r="G17" s="28"/>
+      <x:c r="H17" s="28"/>
+      <x:c r="I17" s="28"/>
+      <x:c r="J17" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
+        <x:v>157.3</x:v>
+      </x:c>
+      <x:c r="K17" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5518,31 +5698,49 @@
         <x:v>IH2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B15" s="28" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="C15" s="28"/>
-      <x:c r="D15" s="28"/>
-      <x:c r="E15" s="28"/>
-      <x:c r="F15" s="28"/>
-      <x:c r="G15" s="28"/>
-      <x:c r="H15" s="28"/>
-      <x:c r="I15" s="28"/>
-      <x:c r="J15" s="30" t="n">
-        <x:f>SUM(J4:J12)</x:f>
-        <x:v>295.6</x:v>
-      </x:c>
-      <x:c r="K15" s="28"/>
+    <x:row r="13">
+      <x:c r="A13" s="22" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B13" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C13" s="22" t="str">
+        <x:v>8月14日</x:v>
+      </x:c>
+      <x:c r="D13" s="23" t="n">
+        <x:v>2905.6</x:v>
+      </x:c>
+      <x:c r="E13" s="23" t="n">
+        <x:v>2910.2</x:v>
+      </x:c>
+      <x:c r="F13" s="23" t="n">
+        <x:v>2877</x:v>
+      </x:c>
+      <x:c r="G13" s="23" t="n">
+        <x:v>2890</x:v>
+      </x:c>
+      <x:c r="H13" s="23" t="n">
+        <x:v>-12.6</x:v>
+      </x:c>
+      <x:c r="I13" s="24" t="n">
+        <x:v>-0.004340935712809135</x:v>
+      </x:c>
+      <x:c r="J13" s="23" t="n">
+        <x:f>ROUND(E13-F13,1)</x:f>
+        <x:v>33.2</x:v>
+      </x:c>
+      <x:c r="K13" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B16" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B16" s="28" t="n">
+        <x:v>10</x:v>
+      </x:c>
       <x:c r="C16" s="28"/>
       <x:c r="D16" s="28"/>
       <x:c r="E16" s="28"/>
@@ -5550,11 +5748,29 @@
       <x:c r="G16" s="28"/>
       <x:c r="H16" s="28"/>
       <x:c r="I16" s="28"/>
-      <x:c r="J16" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J12),0),1)</x:f>
-        <x:v>32.8</x:v>
+      <x:c r="J16" s="30" t="n">
+        <x:f>SUM(J4:J13)</x:f>
+        <x:v>328.8</x:v>
       </x:c>
       <x:c r="K16" s="28"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B17" s="28"/>
+      <x:c r="C17" s="28"/>
+      <x:c r="D17" s="28"/>
+      <x:c r="E17" s="28"/>
+      <x:c r="F17" s="28"/>
+      <x:c r="G17" s="28"/>
+      <x:c r="H17" s="28"/>
+      <x:c r="I17" s="28"/>
+      <x:c r="J17" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
+        <x:v>32.9</x:v>
+      </x:c>
+      <x:c r="K17" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-08-17
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rece6efb3ae584476"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R93ccbdd884374289"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Rdd95cafc9d5845a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R94c6a8a217984c45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R9b717868e0d047e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R0f37a08119c840d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Rb4830dacfb1e492d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R03512f125eb2465d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R2eb6141901bf4fd3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R32a387899d904942"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R1d1f068488684b2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Re7e6d556698145dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R7daa132653714ded"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R6e67cbe7636c48d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Rba3ba5fc066a415c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R80847e72e40f49dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Rd6fb8a1fc73c44f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R2d776c6d3aa54908"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R45447e35c16544e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R9cc8930fc0094358"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -201,6 +201,12 @@
     <x:xf numFmtId="200" fontId="7" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="8" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
@@ -216,12 +222,6 @@
     </x:xf>
     <x:xf numFmtId="200" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="8" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
@@ -485,25 +485,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-08-14</x:v>
+        <x:v>2026-08-17</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7784.38</x:v>
+        <x:v>7968.38</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7673.44</x:v>
+        <x:v>7750.43</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>110.9</x:v>
+        <x:v>217.9</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>1568.4</x:v>
+        <x:v>1786.3</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>156.8</x:v>
+        <x:v>162.4</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -514,25 +514,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-08-14</x:v>
+        <x:v>2026-08-17</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>8005.15</x:v>
+        <x:v>8184.64</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7897.24</x:v>
+        <x:v>7992.36</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>107.9</x:v>
+        <x:v>192.3</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>1580.2</x:v>
+        <x:v>1772.5</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>158</x:v>
+        <x:v>161.1</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -543,25 +543,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-08-14</x:v>
+        <x:v>2026-08-17</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3932.64</x:v>
+        <x:v>3983.51</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3903.7</x:v>
+        <x:v>3924.47</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>28.9</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>385.4</x:v>
+        <x:v>444.4</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>38.5</x:v>
+        <x:v>40.4</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -720,7 +720,7 @@
         <x:v>2026-08-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-08-14</x:v>
+        <x:v>2026-08-17</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -925,7 +925,7 @@
       <x:c r="G4" s="23" t="n">
         <x:v>138900</x:v>
       </x:c>
-      <x:c r="H4" s="34" t="n">
+      <x:c r="H4" s="28" t="n">
         <x:v>1140</x:v>
       </x:c>
       <x:c r="I4" s="24" t="n">
@@ -961,7 +961,7 @@
       <x:c r="G5" s="23" t="n">
         <x:v>139380</x:v>
       </x:c>
-      <x:c r="H5" s="34" t="n">
+      <x:c r="H5" s="28" t="n">
         <x:v>480</x:v>
       </x:c>
       <x:c r="I5" s="24" t="n">
@@ -997,7 +997,7 @@
       <x:c r="G6" s="23" t="n">
         <x:v>143220</x:v>
       </x:c>
-      <x:c r="H6" s="34" t="n">
+      <x:c r="H6" s="28" t="n">
         <x:v>3840</x:v>
       </x:c>
       <x:c r="I6" s="24" t="n">
@@ -1033,7 +1033,7 @@
       <x:c r="G7" s="23" t="n">
         <x:v>141460</x:v>
       </x:c>
-      <x:c r="H7" s="34" t="n">
+      <x:c r="H7" s="28" t="n">
         <x:v>-1760</x:v>
       </x:c>
       <x:c r="I7" s="24" t="n">
@@ -1069,7 +1069,7 @@
       <x:c r="G8" s="23" t="n">
         <x:v>140000</x:v>
       </x:c>
-      <x:c r="H8" s="34" t="n">
+      <x:c r="H8" s="28" t="n">
         <x:v>-1460</x:v>
       </x:c>
       <x:c r="I8" s="24" t="n">
@@ -1105,7 +1105,7 @@
       <x:c r="G9" s="23" t="n">
         <x:v>146360</x:v>
       </x:c>
-      <x:c r="H9" s="34" t="n">
+      <x:c r="H9" s="28" t="n">
         <x:v>6360</x:v>
       </x:c>
       <x:c r="I9" s="24" t="n">
@@ -1141,7 +1141,7 @@
       <x:c r="G10" s="23" t="n">
         <x:v>145860</x:v>
       </x:c>
-      <x:c r="H10" s="34" t="n">
+      <x:c r="H10" s="28" t="n">
         <x:v>-500</x:v>
       </x:c>
       <x:c r="I10" s="24" t="n">
@@ -1177,7 +1177,7 @@
       <x:c r="G11" s="23" t="n">
         <x:v>149700</x:v>
       </x:c>
-      <x:c r="H11" s="34" t="n">
+      <x:c r="H11" s="28" t="n">
         <x:v>3840</x:v>
       </x:c>
       <x:c r="I11" s="24" t="n">
@@ -1213,7 +1213,7 @@
       <x:c r="G12" s="23" t="n">
         <x:v>151420</x:v>
       </x:c>
-      <x:c r="H12" s="34" t="n">
+      <x:c r="H12" s="28" t="n">
         <x:v>1720</x:v>
       </x:c>
       <x:c r="I12" s="24" t="n">
@@ -1249,7 +1249,7 @@
       <x:c r="G13" s="23" t="n">
         <x:v>153940</x:v>
       </x:c>
-      <x:c r="H13" s="34" t="n">
+      <x:c r="H13" s="28" t="n">
         <x:v>2520</x:v>
       </x:c>
       <x:c r="I13" s="24" t="n">
@@ -1264,42 +1264,42 @@
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="29" t="str">
+      <x:c r="A16" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B16" s="28" t="n">
+      <x:c r="B16" s="30" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C16" s="28"/>
-      <x:c r="D16" s="28"/>
-      <x:c r="E16" s="28"/>
-      <x:c r="F16" s="28"/>
-      <x:c r="G16" s="28"/>
-      <x:c r="H16" s="28"/>
-      <x:c r="I16" s="28"/>
-      <x:c r="J16" s="30" t="n">
+      <x:c r="C16" s="30"/>
+      <x:c r="D16" s="30"/>
+      <x:c r="E16" s="30"/>
+      <x:c r="F16" s="30"/>
+      <x:c r="G16" s="30"/>
+      <x:c r="H16" s="30"/>
+      <x:c r="I16" s="30"/>
+      <x:c r="J16" s="32" t="n">
         <x:f>SUM(J4:J13)</x:f>
         <x:v>50340</x:v>
       </x:c>
-      <x:c r="K16" s="28"/>
+      <x:c r="K16" s="30"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="29" t="str">
+      <x:c r="A17" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B17" s="28"/>
-      <x:c r="C17" s="28"/>
-      <x:c r="D17" s="28"/>
-      <x:c r="E17" s="28"/>
-      <x:c r="F17" s="28"/>
-      <x:c r="G17" s="28"/>
-      <x:c r="H17" s="28"/>
-      <x:c r="I17" s="28"/>
-      <x:c r="J17" s="32" t="n">
+      <x:c r="B17" s="30"/>
+      <x:c r="C17" s="30"/>
+      <x:c r="D17" s="30"/>
+      <x:c r="E17" s="30"/>
+      <x:c r="F17" s="30"/>
+      <x:c r="G17" s="30"/>
+      <x:c r="H17" s="30"/>
+      <x:c r="I17" s="30"/>
+      <x:c r="J17" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
         <x:v>5034</x:v>
       </x:c>
-      <x:c r="K17" s="28"/>
+      <x:c r="K17" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1452,155 +1452,155 @@
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="29" t="str">
+      <x:c r="A7" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B7" s="22" t="str">
+        <x:v>8月17日</x:v>
+      </x:c>
+      <x:c r="C7" s="23" t="n">
+        <x:v>7797.18</x:v>
+      </x:c>
+      <x:c r="D7" s="23" t="n">
+        <x:v>7968.38</x:v>
+      </x:c>
+      <x:c r="E7" s="23" t="n">
+        <x:v>7750.43</x:v>
+      </x:c>
+      <x:c r="F7" s="23" t="n">
+        <x:v>7968.38</x:v>
+      </x:c>
+      <x:c r="G7" s="28" t="n">
+        <x:f>ROUND(F7-F6,1)</x:f>
+        <x:v>198.6</x:v>
+      </x:c>
+      <x:c r="H7" s="24" t="n">
+        <x:f>IFERROR(F7/F6-1,"")</x:f>
+        <x:v>0.02555528956912778</x:v>
+      </x:c>
+      <x:c r="I7" s="26" t="n">
+        <x:f>ROUND(D7-E7,1)</x:f>
+        <x:v>217.9</x:v>
+      </x:c>
+      <x:c r="J7" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
+      <x:c r="K7" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B7" s="28" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C7" s="28"/>
-      <x:c r="D7" s="28"/>
-      <x:c r="E7" s="28"/>
-      <x:c r="F7" s="28"/>
-      <x:c r="G7" s="28"/>
-      <x:c r="H7" s="28"/>
-      <x:c r="I7" s="30" t="n">
-        <x:f>ROUND(SUM(I5:I6),1)</x:f>
-        <x:v>901.3</x:v>
-      </x:c>
-      <x:c r="J7" s="28"/>
-      <x:c r="K7" s="28"/>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="29" t="str">
+      <x:c r="B8" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C8" s="30"/>
+      <x:c r="D8" s="30"/>
+      <x:c r="E8" s="30"/>
+      <x:c r="F8" s="30"/>
+      <x:c r="G8" s="30"/>
+      <x:c r="H8" s="30"/>
+      <x:c r="I8" s="32" t="n">
+        <x:f>ROUND(SUM(I5:I7),1)</x:f>
+        <x:v>1119.2</x:v>
+      </x:c>
+      <x:c r="J8" s="30"/>
+      <x:c r="K8" s="30"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B8" s="28"/>
-      <x:c r="C8" s="28"/>
-      <x:c r="D8" s="28"/>
-      <x:c r="E8" s="28"/>
-      <x:c r="F8" s="28"/>
-      <x:c r="G8" s="28"/>
-      <x:c r="H8" s="28"/>
-      <x:c r="I8" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I5:I6),0),1)</x:f>
-        <x:v>450.7</x:v>
-      </x:c>
-      <x:c r="J8" s="28"/>
-      <x:c r="K8" s="28"/>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="17" t="str">
+      <x:c r="B9" s="30"/>
+      <x:c r="C9" s="30"/>
+      <x:c r="D9" s="30"/>
+      <x:c r="E9" s="30"/>
+      <x:c r="F9" s="30"/>
+      <x:c r="G9" s="30"/>
+      <x:c r="H9" s="30"/>
+      <x:c r="I9" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I5:I7),0),1)</x:f>
+        <x:v>373.1</x:v>
+      </x:c>
+      <x:c r="J9" s="30"/>
+      <x:c r="K9" s="30"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="17" t="str">
         <x:v>中证500</x:v>
       </x:c>
-      <x:c r="B10" s="17"/>
-      <x:c r="C10" s="17"/>
-      <x:c r="D10" s="17"/>
-      <x:c r="E10" s="17"/>
-      <x:c r="F10" s="17"/>
-      <x:c r="G10" s="17"/>
-      <x:c r="H10" s="17"/>
-      <x:c r="I10" s="17"/>
-      <x:c r="J10" s="17"/>
-      <x:c r="K10" s="17"/>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="20" t="str">
+      <x:c r="B11" s="17"/>
+      <x:c r="C11" s="17"/>
+      <x:c r="D11" s="17"/>
+      <x:c r="E11" s="17"/>
+      <x:c r="F11" s="17"/>
+      <x:c r="G11" s="17"/>
+      <x:c r="H11" s="17"/>
+      <x:c r="I11" s="17"/>
+      <x:c r="J11" s="17"/>
+      <x:c r="K11" s="17"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B11" s="20" t="str">
+      <x:c r="B12" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C11" s="20" t="str">
+      <x:c r="C12" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D11" s="20" t="str">
+      <x:c r="D12" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E11" s="20" t="str">
+      <x:c r="E12" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F11" s="20" t="str">
+      <x:c r="F12" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G11" s="20" t="str">
+      <x:c r="G12" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H11" s="20" t="str">
+      <x:c r="H12" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I11" s="20" t="str">
+      <x:c r="I12" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J11" s="20" t="str">
+      <x:c r="J12" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K11" s="20" t="str">
+      <x:c r="K12" s="20" t="str">
         <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B12" s="22" t="str">
-        <x:v>8月3日-8月7日</x:v>
-      </x:c>
-      <x:c r="C12" s="23" t="n">
-        <x:v>7457.12</x:v>
-      </x:c>
-      <x:c r="D12" s="23" t="n">
-        <x:v>7983.17</x:v>
-      </x:c>
-      <x:c r="E12" s="23" t="n">
-        <x:v>7397.94</x:v>
-      </x:c>
-      <x:c r="F12" s="23" t="n">
-        <x:v>7980.12</x:v>
-      </x:c>
-      <x:c r="G12" s="23"/>
-      <x:c r="H12" s="24"/>
-      <x:c r="I12" s="26" t="n">
-        <x:f>ROUND(D12-E12,1)</x:f>
-        <x:v>585.2</x:v>
-      </x:c>
-      <x:c r="J12" s="22" t="str">
-        <x:v>中证500</x:v>
-      </x:c>
-      <x:c r="K12" s="22" t="n">
-        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="B13" s="22" t="str">
-        <x:v>8月10日-8月14日</x:v>
+        <x:v>8月3日-8月7日</x:v>
       </x:c>
       <x:c r="C13" s="23" t="n">
-        <x:v>8003.92</x:v>
+        <x:v>7457.12</x:v>
       </x:c>
       <x:c r="D13" s="23" t="n">
-        <x:v>8142.33</x:v>
+        <x:v>7983.17</x:v>
       </x:c>
       <x:c r="E13" s="23" t="n">
-        <x:v>7897.24</x:v>
+        <x:v>7397.94</x:v>
       </x:c>
       <x:c r="F13" s="23" t="n">
-        <x:v>7990.33</x:v>
-      </x:c>
-      <x:c r="G13" s="23" t="n">
-        <x:f>ROUND(F13-F12,1)</x:f>
-        <x:v>10.2</x:v>
-      </x:c>
-      <x:c r="H13" s="24" t="n">
-        <x:f>IFERROR(F13/F12-1,"")</x:f>
-        <x:v>0.0012794293820144187</x:v>
-      </x:c>
+        <x:v>7980.12</x:v>
+      </x:c>
+      <x:c r="G13" s="23"/>
+      <x:c r="H13" s="24"/>
       <x:c r="I13" s="26" t="n">
         <x:f>ROUND(D13-E13,1)</x:f>
-        <x:v>245.1</x:v>
+        <x:v>585.2</x:v>
       </x:c>
       <x:c r="J13" s="22" t="str">
         <x:v>中证500</x:v>
@@ -1610,1002 +1610,1116 @@
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="29" t="str">
+      <x:c r="A14" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B14" s="22" t="str">
+        <x:v>8月10日-8月14日</x:v>
+      </x:c>
+      <x:c r="C14" s="23" t="n">
+        <x:v>8003.92</x:v>
+      </x:c>
+      <x:c r="D14" s="23" t="n">
+        <x:v>8142.33</x:v>
+      </x:c>
+      <x:c r="E14" s="23" t="n">
+        <x:v>7897.24</x:v>
+      </x:c>
+      <x:c r="F14" s="23" t="n">
+        <x:v>7990.33</x:v>
+      </x:c>
+      <x:c r="G14" s="23" t="n">
+        <x:f>ROUND(F14-F13,1)</x:f>
+        <x:v>10.2</x:v>
+      </x:c>
+      <x:c r="H14" s="24" t="n">
+        <x:f>IFERROR(F14/F13-1,"")</x:f>
+        <x:v>0.0012794293820144187</x:v>
+      </x:c>
+      <x:c r="I14" s="26" t="n">
+        <x:f>ROUND(D14-E14,1)</x:f>
+        <x:v>245.1</x:v>
+      </x:c>
+      <x:c r="J14" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+      <x:c r="K14" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B15" s="22" t="str">
+        <x:v>8月17日</x:v>
+      </x:c>
+      <x:c r="C15" s="23" t="n">
+        <x:v>8007.87</x:v>
+      </x:c>
+      <x:c r="D15" s="23" t="n">
+        <x:v>8184.64</x:v>
+      </x:c>
+      <x:c r="E15" s="23" t="n">
+        <x:v>7992.36</x:v>
+      </x:c>
+      <x:c r="F15" s="23" t="n">
+        <x:v>8184.64</x:v>
+      </x:c>
+      <x:c r="G15" s="28" t="n">
+        <x:f>ROUND(F15-F14,1)</x:f>
+        <x:v>194.3</x:v>
+      </x:c>
+      <x:c r="H15" s="24" t="n">
+        <x:f>IFERROR(F15/F14-1,"")</x:f>
+        <x:v>0.02431814455723358</x:v>
+      </x:c>
+      <x:c r="I15" s="26" t="n">
+        <x:f>ROUND(D15-E15,1)</x:f>
+        <x:v>192.3</x:v>
+      </x:c>
+      <x:c r="J15" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+      <x:c r="K15" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B14" s="28" t="n">
+      <x:c r="B16" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C16" s="30"/>
+      <x:c r="D16" s="30"/>
+      <x:c r="E16" s="30"/>
+      <x:c r="F16" s="30"/>
+      <x:c r="G16" s="30"/>
+      <x:c r="H16" s="30"/>
+      <x:c r="I16" s="32" t="n">
+        <x:f>ROUND(SUM(I13:I15),1)</x:f>
+        <x:v>1022.6</x:v>
+      </x:c>
+      <x:c r="J16" s="30"/>
+      <x:c r="K16" s="30"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B17" s="30"/>
+      <x:c r="C17" s="30"/>
+      <x:c r="D17" s="30"/>
+      <x:c r="E17" s="30"/>
+      <x:c r="F17" s="30"/>
+      <x:c r="G17" s="30"/>
+      <x:c r="H17" s="30"/>
+      <x:c r="I17" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I13:I15),0),1)</x:f>
+        <x:v>340.9</x:v>
+      </x:c>
+      <x:c r="J17" s="30"/>
+      <x:c r="K17" s="30"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="17" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="B19" s="17"/>
+      <x:c r="C19" s="17"/>
+      <x:c r="D19" s="17"/>
+      <x:c r="E19" s="17"/>
+      <x:c r="F19" s="17"/>
+      <x:c r="G19" s="17"/>
+      <x:c r="H19" s="17"/>
+      <x:c r="I19" s="17"/>
+      <x:c r="J19" s="17"/>
+      <x:c r="K19" s="17"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="20" t="str">
+        <x:v>序号</x:v>
+      </x:c>
+      <x:c r="B20" s="20" t="str">
+        <x:v>周期</x:v>
+      </x:c>
+      <x:c r="C20" s="20" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="D20" s="20" t="str">
+        <x:v>高点</x:v>
+      </x:c>
+      <x:c r="E20" s="20" t="str">
+        <x:v>低点</x:v>
+      </x:c>
+      <x:c r="F20" s="20" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="G20" s="20" t="str">
+        <x:v>涨跌点数</x:v>
+      </x:c>
+      <x:c r="H20" s="20" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I20" s="20" t="str">
+        <x:v>振幅</x:v>
+      </x:c>
+      <x:c r="J20" s="20" t="str">
+        <x:v>标的</x:v>
+      </x:c>
+      <x:c r="K20" s="20" t="str">
+        <x:v>交易日</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B21" s="22" t="str">
+        <x:v>8月3日-8月7日</x:v>
+      </x:c>
+      <x:c r="C21" s="23" t="n">
+        <x:v>3812.61</x:v>
+      </x:c>
+      <x:c r="D21" s="23" t="n">
+        <x:v>3940.93</x:v>
+      </x:c>
+      <x:c r="E21" s="23" t="n">
+        <x:v>3797.64</x:v>
+      </x:c>
+      <x:c r="F21" s="23" t="n">
+        <x:v>3940.04</x:v>
+      </x:c>
+      <x:c r="G21" s="23"/>
+      <x:c r="H21" s="24"/>
+      <x:c r="I21" s="26" t="n">
+        <x:f>ROUND(D21-E21,1)</x:f>
+        <x:v>143.3</x:v>
+      </x:c>
+      <x:c r="J21" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="K21" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C14" s="28"/>
-      <x:c r="D14" s="28"/>
-      <x:c r="E14" s="28"/>
-      <x:c r="F14" s="28"/>
-      <x:c r="G14" s="28"/>
-      <x:c r="H14" s="28"/>
-      <x:c r="I14" s="30" t="n">
-        <x:f>ROUND(SUM(I12:I13),1)</x:f>
-        <x:v>830.3</x:v>
-      </x:c>
-      <x:c r="J14" s="28"/>
-      <x:c r="K14" s="28"/>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="29" t="str">
+      <x:c r="B22" s="22" t="str">
+        <x:v>8月10日-8月14日</x:v>
+      </x:c>
+      <x:c r="C22" s="23" t="n">
+        <x:v>3943.82</x:v>
+      </x:c>
+      <x:c r="D22" s="23" t="n">
+        <x:v>3968.48</x:v>
+      </x:c>
+      <x:c r="E22" s="23" t="n">
+        <x:v>3903.7</x:v>
+      </x:c>
+      <x:c r="F22" s="23" t="n">
+        <x:v>3927.18</x:v>
+      </x:c>
+      <x:c r="G22" s="23" t="n">
+        <x:f>ROUND(F22-F21,1)</x:f>
+        <x:v>-12.9</x:v>
+      </x:c>
+      <x:c r="H22" s="24" t="n">
+        <x:f>IFERROR(F22/F21-1,"")</x:f>
+        <x:v>-0.003263926254555849</x:v>
+      </x:c>
+      <x:c r="I22" s="26" t="n">
+        <x:f>ROUND(D22-E22,1)</x:f>
+        <x:v>64.8</x:v>
+      </x:c>
+      <x:c r="J22" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="K22" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B23" s="22" t="str">
+        <x:v>8月17日</x:v>
+      </x:c>
+      <x:c r="C23" s="23" t="n">
+        <x:v>3930.1</x:v>
+      </x:c>
+      <x:c r="D23" s="23" t="n">
+        <x:v>3983.51</x:v>
+      </x:c>
+      <x:c r="E23" s="23" t="n">
+        <x:v>3924.47</x:v>
+      </x:c>
+      <x:c r="F23" s="23" t="n">
+        <x:v>3982.65</x:v>
+      </x:c>
+      <x:c r="G23" s="23" t="n">
+        <x:f>ROUND(F23-F22,1)</x:f>
+        <x:v>55.5</x:v>
+      </x:c>
+      <x:c r="H23" s="24" t="n">
+        <x:f>IFERROR(F23/F22-1,"")</x:f>
+        <x:v>0.014124639053977761</x:v>
+      </x:c>
+      <x:c r="I23" s="26" t="n">
+        <x:f>ROUND(D23-E23,1)</x:f>
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="J23" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="K23" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="31" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B24" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C24" s="30"/>
+      <x:c r="D24" s="30"/>
+      <x:c r="E24" s="30"/>
+      <x:c r="F24" s="30"/>
+      <x:c r="G24" s="30"/>
+      <x:c r="H24" s="30"/>
+      <x:c r="I24" s="32" t="n">
+        <x:f>ROUND(SUM(I21:I23),1)</x:f>
+        <x:v>267.1</x:v>
+      </x:c>
+      <x:c r="J24" s="30"/>
+      <x:c r="K24" s="30"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B15" s="28"/>
-      <x:c r="C15" s="28"/>
-      <x:c r="D15" s="28"/>
-      <x:c r="E15" s="28"/>
-      <x:c r="F15" s="28"/>
-      <x:c r="G15" s="28"/>
-      <x:c r="H15" s="28"/>
-      <x:c r="I15" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I12:I13),0),1)</x:f>
-        <x:v>415.2</x:v>
-      </x:c>
-      <x:c r="J15" s="28"/>
-      <x:c r="K15" s="28"/>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="17" t="str">
-        <x:v>上证指数</x:v>
-      </x:c>
-      <x:c r="B17" s="17"/>
-      <x:c r="C17" s="17"/>
-      <x:c r="D17" s="17"/>
-      <x:c r="E17" s="17"/>
-      <x:c r="F17" s="17"/>
-      <x:c r="G17" s="17"/>
-      <x:c r="H17" s="17"/>
-      <x:c r="I17" s="17"/>
-      <x:c r="J17" s="17"/>
-      <x:c r="K17" s="17"/>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="20" t="str">
+      <x:c r="B25" s="30"/>
+      <x:c r="C25" s="30"/>
+      <x:c r="D25" s="30"/>
+      <x:c r="E25" s="30"/>
+      <x:c r="F25" s="30"/>
+      <x:c r="G25" s="30"/>
+      <x:c r="H25" s="30"/>
+      <x:c r="I25" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I21:I23),0),1)</x:f>
+        <x:v>89</x:v>
+      </x:c>
+      <x:c r="J25" s="30"/>
+      <x:c r="K25" s="30"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="17" t="str">
+        <x:v>IM主力</x:v>
+      </x:c>
+      <x:c r="B27" s="17"/>
+      <x:c r="C27" s="17"/>
+      <x:c r="D27" s="17"/>
+      <x:c r="E27" s="17"/>
+      <x:c r="F27" s="17"/>
+      <x:c r="G27" s="17"/>
+      <x:c r="H27" s="17"/>
+      <x:c r="I27" s="17"/>
+      <x:c r="J27" s="17"/>
+      <x:c r="K27" s="17"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B18" s="20" t="str">
+      <x:c r="B28" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C18" s="20" t="str">
+      <x:c r="C28" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D18" s="20" t="str">
+      <x:c r="D28" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E18" s="20" t="str">
+      <x:c r="E28" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F18" s="20" t="str">
+      <x:c r="F28" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G18" s="20" t="str">
+      <x:c r="G28" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H18" s="20" t="str">
+      <x:c r="H28" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I18" s="20" t="str">
+      <x:c r="I28" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J18" s="20" t="str">
+      <x:c r="J28" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K18" s="20" t="str">
+      <x:c r="K28" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="22" t="n">
+    <x:row r="29">
+      <x:c r="A29" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B19" s="22" t="str">
+      <x:c r="B29" s="22" t="str">
         <x:v>8月3日-8月7日</x:v>
       </x:c>
-      <x:c r="C19" s="23" t="n">
-        <x:v>3812.61</x:v>
-      </x:c>
-      <x:c r="D19" s="23" t="n">
-        <x:v>3940.93</x:v>
-      </x:c>
-      <x:c r="E19" s="23" t="n">
-        <x:v>3797.64</x:v>
-      </x:c>
-      <x:c r="F19" s="23" t="n">
-        <x:v>3940.04</x:v>
-      </x:c>
-      <x:c r="G19" s="23"/>
-      <x:c r="H19" s="24"/>
-      <x:c r="I19" s="26" t="n">
-        <x:f>ROUND(D19-E19,1)</x:f>
-        <x:v>143.3</x:v>
-      </x:c>
-      <x:c r="J19" s="22" t="str">
-        <x:v>上证指数</x:v>
-      </x:c>
-      <x:c r="K19" s="22" t="n">
+      <x:c r="C29" s="23" t="n">
+        <x:v>7000</x:v>
+      </x:c>
+      <x:c r="D29" s="23" t="n">
+        <x:v>7594.2</x:v>
+      </x:c>
+      <x:c r="E29" s="23" t="n">
+        <x:v>6976</x:v>
+      </x:c>
+      <x:c r="F29" s="23" t="n">
+        <x:v>7590.6</x:v>
+      </x:c>
+      <x:c r="G29" s="23"/>
+      <x:c r="H29" s="24"/>
+      <x:c r="I29" s="26" t="n">
+        <x:f>ROUND(D29-E29,1)</x:f>
+        <x:v>618.2</x:v>
+      </x:c>
+      <x:c r="J29" s="22" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+      <x:c r="K29" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="22" t="n">
+    <x:row r="30">
+      <x:c r="A30" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B20" s="22" t="str">
+      <x:c r="B30" s="22" t="str">
         <x:v>8月10日-8月14日</x:v>
       </x:c>
-      <x:c r="C20" s="23" t="n">
-        <x:v>3943.82</x:v>
-      </x:c>
-      <x:c r="D20" s="23" t="n">
-        <x:v>3968.48</x:v>
-      </x:c>
-      <x:c r="E20" s="23" t="n">
-        <x:v>3903.7</x:v>
-      </x:c>
-      <x:c r="F20" s="23" t="n">
-        <x:v>3927.18</x:v>
-      </x:c>
-      <x:c r="G20" s="23" t="n">
-        <x:f>ROUND(F20-F19,1)</x:f>
-        <x:v>-12.9</x:v>
-      </x:c>
-      <x:c r="H20" s="24" t="n">
-        <x:f>IFERROR(F20/F19-1,"")</x:f>
-        <x:v>-0.003263926254555849</x:v>
-      </x:c>
-      <x:c r="I20" s="26" t="n">
-        <x:f>ROUND(D20-E20,1)</x:f>
-        <x:v>64.8</x:v>
-      </x:c>
-      <x:c r="J20" s="22" t="str">
-        <x:v>上证指数</x:v>
-      </x:c>
-      <x:c r="K20" s="22" t="n">
+      <x:c r="C30" s="23" t="n">
+        <x:v>7628.8</x:v>
+      </x:c>
+      <x:c r="D30" s="23" t="n">
+        <x:v>7776</x:v>
+      </x:c>
+      <x:c r="E30" s="23" t="n">
+        <x:v>7525</x:v>
+      </x:c>
+      <x:c r="F30" s="23" t="n">
+        <x:v>7650.2</x:v>
+      </x:c>
+      <x:c r="G30" s="23" t="n">
+        <x:f>ROUND(F30-F29,1)</x:f>
+        <x:v>59.6</x:v>
+      </x:c>
+      <x:c r="H30" s="24" t="n">
+        <x:f>IFERROR(F30/F29-1,"")</x:f>
+        <x:v>0.007851816720680693</x:v>
+      </x:c>
+      <x:c r="I30" s="26" t="n">
+        <x:f>ROUND(D30-E30,1)</x:f>
+        <x:v>251</x:v>
+      </x:c>
+      <x:c r="J30" s="22" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+      <x:c r="K30" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="29" t="str">
+    <x:row r="31">
+      <x:c r="A31" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B21" s="28" t="n">
+      <x:c r="B31" s="30" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C21" s="28"/>
-      <x:c r="D21" s="28"/>
-      <x:c r="E21" s="28"/>
-      <x:c r="F21" s="28"/>
-      <x:c r="G21" s="28"/>
-      <x:c r="H21" s="28"/>
-      <x:c r="I21" s="30" t="n">
-        <x:f>ROUND(SUM(I19:I20),1)</x:f>
-        <x:v>208.1</x:v>
-      </x:c>
-      <x:c r="J21" s="28"/>
-      <x:c r="K21" s="28"/>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="29" t="str">
+      <x:c r="C31" s="30"/>
+      <x:c r="D31" s="30"/>
+      <x:c r="E31" s="30"/>
+      <x:c r="F31" s="30"/>
+      <x:c r="G31" s="30"/>
+      <x:c r="H31" s="30"/>
+      <x:c r="I31" s="32" t="n">
+        <x:f>ROUND(SUM(I29:I30),1)</x:f>
+        <x:v>869.2</x:v>
+      </x:c>
+      <x:c r="J31" s="30"/>
+      <x:c r="K31" s="30"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B22" s="28"/>
-      <x:c r="C22" s="28"/>
-      <x:c r="D22" s="28"/>
-      <x:c r="E22" s="28"/>
-      <x:c r="F22" s="28"/>
-      <x:c r="G22" s="28"/>
-      <x:c r="H22" s="28"/>
-      <x:c r="I22" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I19:I20),0),1)</x:f>
-        <x:v>104.1</x:v>
-      </x:c>
-      <x:c r="J22" s="28"/>
-      <x:c r="K22" s="28"/>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="17" t="str">
-        <x:v>IM主力</x:v>
-      </x:c>
-      <x:c r="B24" s="17"/>
-      <x:c r="C24" s="17"/>
-      <x:c r="D24" s="17"/>
-      <x:c r="E24" s="17"/>
-      <x:c r="F24" s="17"/>
-      <x:c r="G24" s="17"/>
-      <x:c r="H24" s="17"/>
-      <x:c r="I24" s="17"/>
-      <x:c r="J24" s="17"/>
-      <x:c r="K24" s="17"/>
-    </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="20" t="str">
+      <x:c r="B32" s="30"/>
+      <x:c r="C32" s="30"/>
+      <x:c r="D32" s="30"/>
+      <x:c r="E32" s="30"/>
+      <x:c r="F32" s="30"/>
+      <x:c r="G32" s="30"/>
+      <x:c r="H32" s="30"/>
+      <x:c r="I32" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I29:I30),0),1)</x:f>
+        <x:v>434.6</x:v>
+      </x:c>
+      <x:c r="J32" s="30"/>
+      <x:c r="K32" s="30"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="17" t="str">
+        <x:v>IC主力</x:v>
+      </x:c>
+      <x:c r="B34" s="17"/>
+      <x:c r="C34" s="17"/>
+      <x:c r="D34" s="17"/>
+      <x:c r="E34" s="17"/>
+      <x:c r="F34" s="17"/>
+      <x:c r="G34" s="17"/>
+      <x:c r="H34" s="17"/>
+      <x:c r="I34" s="17"/>
+      <x:c r="J34" s="17"/>
+      <x:c r="K34" s="17"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B25" s="20" t="str">
+      <x:c r="B35" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C25" s="20" t="str">
+      <x:c r="C35" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D25" s="20" t="str">
+      <x:c r="D35" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E25" s="20" t="str">
+      <x:c r="E35" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F25" s="20" t="str">
+      <x:c r="F35" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G25" s="20" t="str">
+      <x:c r="G35" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H25" s="20" t="str">
+      <x:c r="H35" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I25" s="20" t="str">
+      <x:c r="I35" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J25" s="20" t="str">
+      <x:c r="J35" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K25" s="20" t="str">
+      <x:c r="K35" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="22" t="n">
+    <x:row r="36">
+      <x:c r="A36" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B26" s="22" t="str">
+      <x:c r="B36" s="22" t="str">
         <x:v>8月3日-8月7日</x:v>
       </x:c>
-      <x:c r="C26" s="23" t="n">
-        <x:v>7000</x:v>
-      </x:c>
-      <x:c r="D26" s="23" t="n">
-        <x:v>7594.2</x:v>
-      </x:c>
-      <x:c r="E26" s="23" t="n">
-        <x:v>6976</x:v>
-      </x:c>
-      <x:c r="F26" s="23" t="n">
-        <x:v>7590.6</x:v>
-      </x:c>
-      <x:c r="G26" s="23"/>
-      <x:c r="H26" s="24"/>
-      <x:c r="I26" s="26" t="n">
-        <x:f>ROUND(D26-E26,1)</x:f>
-        <x:v>618.2</x:v>
-      </x:c>
-      <x:c r="J26" s="22" t="str">
-        <x:v>IM2609</x:v>
-      </x:c>
-      <x:c r="K26" s="22" t="n">
+      <x:c r="C36" s="23" t="n">
+        <x:v>7391</x:v>
+      </x:c>
+      <x:c r="D36" s="23" t="n">
+        <x:v>7882.6</x:v>
+      </x:c>
+      <x:c r="E36" s="23" t="n">
+        <x:v>7335</x:v>
+      </x:c>
+      <x:c r="F36" s="23" t="n">
+        <x:v>7877.8</x:v>
+      </x:c>
+      <x:c r="G36" s="23"/>
+      <x:c r="H36" s="24"/>
+      <x:c r="I36" s="26" t="n">
+        <x:f>ROUND(D36-E36,1)</x:f>
+        <x:v>547.6</x:v>
+      </x:c>
+      <x:c r="J36" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+      <x:c r="K36" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="22" t="n">
+    <x:row r="37">
+      <x:c r="A37" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B27" s="22" t="str">
+      <x:c r="B37" s="22" t="str">
         <x:v>8月10日-8月14日</x:v>
       </x:c>
-      <x:c r="C27" s="23" t="n">
-        <x:v>7628.8</x:v>
-      </x:c>
-      <x:c r="D27" s="23" t="n">
-        <x:v>7776</x:v>
-      </x:c>
-      <x:c r="E27" s="23" t="n">
-        <x:v>7525</x:v>
-      </x:c>
-      <x:c r="F27" s="23" t="n">
-        <x:v>7650.2</x:v>
-      </x:c>
-      <x:c r="G27" s="23" t="n">
-        <x:f>ROUND(F27-F26,1)</x:f>
-        <x:v>59.6</x:v>
-      </x:c>
-      <x:c r="H27" s="24" t="n">
-        <x:f>IFERROR(F27/F26-1,"")</x:f>
-        <x:v>0.007851816720680693</x:v>
-      </x:c>
-      <x:c r="I27" s="26" t="n">
-        <x:f>ROUND(D27-E27,1)</x:f>
-        <x:v>251</x:v>
-      </x:c>
-      <x:c r="J27" s="22" t="str">
-        <x:v>IM2609</x:v>
-      </x:c>
-      <x:c r="K27" s="22" t="n">
+      <x:c r="C37" s="23" t="n">
+        <x:v>7888</x:v>
+      </x:c>
+      <x:c r="D37" s="23" t="n">
+        <x:v>8024</x:v>
+      </x:c>
+      <x:c r="E37" s="23" t="n">
+        <x:v>7795.8</x:v>
+      </x:c>
+      <x:c r="F37" s="23" t="n">
+        <x:v>7861.2</x:v>
+      </x:c>
+      <x:c r="G37" s="23" t="n">
+        <x:f>ROUND(F37-F36,1)</x:f>
+        <x:v>-16.6</x:v>
+      </x:c>
+      <x:c r="H37" s="24" t="n">
+        <x:f>IFERROR(F37/F36-1,"")</x:f>
+        <x:v>-0.0021071872857905127</x:v>
+      </x:c>
+      <x:c r="I37" s="26" t="n">
+        <x:f>ROUND(D37-E37,1)</x:f>
+        <x:v>228.2</x:v>
+      </x:c>
+      <x:c r="J37" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+      <x:c r="K37" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="28">
-      <x:c r="A28" s="29" t="str">
+    <x:row r="38">
+      <x:c r="A38" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B28" s="28" t="n">
+      <x:c r="B38" s="30" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C28" s="28"/>
-      <x:c r="D28" s="28"/>
-      <x:c r="E28" s="28"/>
-      <x:c r="F28" s="28"/>
-      <x:c r="G28" s="28"/>
-      <x:c r="H28" s="28"/>
-      <x:c r="I28" s="30" t="n">
-        <x:f>ROUND(SUM(I26:I27),1)</x:f>
-        <x:v>869.2</x:v>
-      </x:c>
-      <x:c r="J28" s="28"/>
-      <x:c r="K28" s="28"/>
-    </x:row>
-    <x:row r="29">
-      <x:c r="A29" s="29" t="str">
+      <x:c r="C38" s="30"/>
+      <x:c r="D38" s="30"/>
+      <x:c r="E38" s="30"/>
+      <x:c r="F38" s="30"/>
+      <x:c r="G38" s="30"/>
+      <x:c r="H38" s="30"/>
+      <x:c r="I38" s="32" t="n">
+        <x:f>ROUND(SUM(I36:I37),1)</x:f>
+        <x:v>775.8</x:v>
+      </x:c>
+      <x:c r="J38" s="30"/>
+      <x:c r="K38" s="30"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B29" s="28"/>
-      <x:c r="C29" s="28"/>
-      <x:c r="D29" s="28"/>
-      <x:c r="E29" s="28"/>
-      <x:c r="F29" s="28"/>
-      <x:c r="G29" s="28"/>
-      <x:c r="H29" s="28"/>
-      <x:c r="I29" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I26:I27),0),1)</x:f>
-        <x:v>434.6</x:v>
-      </x:c>
-      <x:c r="J29" s="28"/>
-      <x:c r="K29" s="28"/>
-    </x:row>
-    <x:row r="31">
-      <x:c r="A31" s="17" t="str">
-        <x:v>IC主力</x:v>
-      </x:c>
-      <x:c r="B31" s="17"/>
-      <x:c r="C31" s="17"/>
-      <x:c r="D31" s="17"/>
-      <x:c r="E31" s="17"/>
-      <x:c r="F31" s="17"/>
-      <x:c r="G31" s="17"/>
-      <x:c r="H31" s="17"/>
-      <x:c r="I31" s="17"/>
-      <x:c r="J31" s="17"/>
-      <x:c r="K31" s="17"/>
-    </x:row>
-    <x:row r="32">
-      <x:c r="A32" s="20" t="str">
+      <x:c r="B39" s="30"/>
+      <x:c r="C39" s="30"/>
+      <x:c r="D39" s="30"/>
+      <x:c r="E39" s="30"/>
+      <x:c r="F39" s="30"/>
+      <x:c r="G39" s="30"/>
+      <x:c r="H39" s="30"/>
+      <x:c r="I39" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I36:I37),0),1)</x:f>
+        <x:v>387.9</x:v>
+      </x:c>
+      <x:c r="J39" s="30"/>
+      <x:c r="K39" s="30"/>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="17" t="str">
+        <x:v>IF主力</x:v>
+      </x:c>
+      <x:c r="B41" s="17"/>
+      <x:c r="C41" s="17"/>
+      <x:c r="D41" s="17"/>
+      <x:c r="E41" s="17"/>
+      <x:c r="F41" s="17"/>
+      <x:c r="G41" s="17"/>
+      <x:c r="H41" s="17"/>
+      <x:c r="I41" s="17"/>
+      <x:c r="J41" s="17"/>
+      <x:c r="K41" s="17"/>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B32" s="20" t="str">
+      <x:c r="B42" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C32" s="20" t="str">
+      <x:c r="C42" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D32" s="20" t="str">
+      <x:c r="D42" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E32" s="20" t="str">
+      <x:c r="E42" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F32" s="20" t="str">
+      <x:c r="F42" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G32" s="20" t="str">
+      <x:c r="G42" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H32" s="20" t="str">
+      <x:c r="H42" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I32" s="20" t="str">
+      <x:c r="I42" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J32" s="20" t="str">
+      <x:c r="J42" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K32" s="20" t="str">
+      <x:c r="K42" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="33">
-      <x:c r="A33" s="22" t="n">
+    <x:row r="43">
+      <x:c r="A43" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B33" s="22" t="str">
+      <x:c r="B43" s="22" t="str">
         <x:v>8月3日-8月7日</x:v>
       </x:c>
-      <x:c r="C33" s="23" t="n">
-        <x:v>7391</x:v>
-      </x:c>
-      <x:c r="D33" s="23" t="n">
-        <x:v>7882.6</x:v>
-      </x:c>
-      <x:c r="E33" s="23" t="n">
-        <x:v>7335</x:v>
-      </x:c>
-      <x:c r="F33" s="23" t="n">
-        <x:v>7877.8</x:v>
-      </x:c>
-      <x:c r="G33" s="23"/>
-      <x:c r="H33" s="24"/>
-      <x:c r="I33" s="26" t="n">
-        <x:f>ROUND(D33-E33,1)</x:f>
-        <x:v>547.6</x:v>
-      </x:c>
-      <x:c r="J33" s="22" t="str">
-        <x:v>IC2609</x:v>
-      </x:c>
-      <x:c r="K33" s="22" t="n">
+      <x:c r="C43" s="23" t="n">
+        <x:v>4526.4</x:v>
+      </x:c>
+      <x:c r="D43" s="23" t="n">
+        <x:v>4656.2</x:v>
+      </x:c>
+      <x:c r="E43" s="23" t="n">
+        <x:v>4494.2</x:v>
+      </x:c>
+      <x:c r="F43" s="23" t="n">
+        <x:v>4645.6</x:v>
+      </x:c>
+      <x:c r="G43" s="23"/>
+      <x:c r="H43" s="24"/>
+      <x:c r="I43" s="26" t="n">
+        <x:f>ROUND(D43-E43,1)</x:f>
+        <x:v>162</x:v>
+      </x:c>
+      <x:c r="J43" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+      <x:c r="K43" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="34">
-      <x:c r="A34" s="22" t="n">
+    <x:row r="44">
+      <x:c r="A44" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B34" s="22" t="str">
+      <x:c r="B44" s="22" t="str">
         <x:v>8月10日-8月14日</x:v>
       </x:c>
-      <x:c r="C34" s="23" t="n">
-        <x:v>7888</x:v>
-      </x:c>
-      <x:c r="D34" s="23" t="n">
-        <x:v>8024</x:v>
-      </x:c>
-      <x:c r="E34" s="23" t="n">
-        <x:v>7795.8</x:v>
-      </x:c>
-      <x:c r="F34" s="23" t="n">
-        <x:v>7861.2</x:v>
-      </x:c>
-      <x:c r="G34" s="23" t="n">
-        <x:f>ROUND(F34-F33,1)</x:f>
-        <x:v>-16.6</x:v>
-      </x:c>
-      <x:c r="H34" s="24" t="n">
-        <x:f>IFERROR(F34/F33-1,"")</x:f>
-        <x:v>-0.0021071872857905127</x:v>
-      </x:c>
-      <x:c r="I34" s="26" t="n">
-        <x:f>ROUND(D34-E34,1)</x:f>
-        <x:v>228.2</x:v>
-      </x:c>
-      <x:c r="J34" s="22" t="str">
-        <x:v>IC2609</x:v>
-      </x:c>
-      <x:c r="K34" s="22" t="n">
+      <x:c r="C44" s="23" t="n">
+        <x:v>4656.8</x:v>
+      </x:c>
+      <x:c r="D44" s="23" t="n">
+        <x:v>4681</x:v>
+      </x:c>
+      <x:c r="E44" s="23" t="n">
+        <x:v>4598</x:v>
+      </x:c>
+      <x:c r="F44" s="23" t="n">
+        <x:v>4620.4</x:v>
+      </x:c>
+      <x:c r="G44" s="23" t="n">
+        <x:f>ROUND(F44-F43,1)</x:f>
+        <x:v>-25.2</x:v>
+      </x:c>
+      <x:c r="H44" s="24" t="n">
+        <x:f>IFERROR(F44/F43-1,"")</x:f>
+        <x:v>-0.005424487687274104</x:v>
+      </x:c>
+      <x:c r="I44" s="23" t="n">
+        <x:f>ROUND(D44-E44,1)</x:f>
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="J44" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+      <x:c r="K44" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="35">
-      <x:c r="A35" s="29" t="str">
+    <x:row r="45">
+      <x:c r="A45" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B35" s="28" t="n">
+      <x:c r="B45" s="30" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C35" s="28"/>
-      <x:c r="D35" s="28"/>
-      <x:c r="E35" s="28"/>
-      <x:c r="F35" s="28"/>
-      <x:c r="G35" s="28"/>
-      <x:c r="H35" s="28"/>
-      <x:c r="I35" s="30" t="n">
-        <x:f>ROUND(SUM(I33:I34),1)</x:f>
-        <x:v>775.8</x:v>
-      </x:c>
-      <x:c r="J35" s="28"/>
-      <x:c r="K35" s="28"/>
-    </x:row>
-    <x:row r="36">
-      <x:c r="A36" s="29" t="str">
+      <x:c r="C45" s="30"/>
+      <x:c r="D45" s="30"/>
+      <x:c r="E45" s="30"/>
+      <x:c r="F45" s="30"/>
+      <x:c r="G45" s="30"/>
+      <x:c r="H45" s="30"/>
+      <x:c r="I45" s="32" t="n">
+        <x:f>ROUND(SUM(I43:I44),1)</x:f>
+        <x:v>245</x:v>
+      </x:c>
+      <x:c r="J45" s="30"/>
+      <x:c r="K45" s="30"/>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B36" s="28"/>
-      <x:c r="C36" s="28"/>
-      <x:c r="D36" s="28"/>
-      <x:c r="E36" s="28"/>
-      <x:c r="F36" s="28"/>
-      <x:c r="G36" s="28"/>
-      <x:c r="H36" s="28"/>
-      <x:c r="I36" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I33:I34),0),1)</x:f>
-        <x:v>387.9</x:v>
-      </x:c>
-      <x:c r="J36" s="28"/>
-      <x:c r="K36" s="28"/>
-    </x:row>
-    <x:row r="38">
-      <x:c r="A38" s="17" t="str">
-        <x:v>IF主力</x:v>
-      </x:c>
-      <x:c r="B38" s="17"/>
-      <x:c r="C38" s="17"/>
-      <x:c r="D38" s="17"/>
-      <x:c r="E38" s="17"/>
-      <x:c r="F38" s="17"/>
-      <x:c r="G38" s="17"/>
-      <x:c r="H38" s="17"/>
-      <x:c r="I38" s="17"/>
-      <x:c r="J38" s="17"/>
-      <x:c r="K38" s="17"/>
-    </x:row>
-    <x:row r="39">
-      <x:c r="A39" s="20" t="str">
+      <x:c r="B46" s="30"/>
+      <x:c r="C46" s="30"/>
+      <x:c r="D46" s="30"/>
+      <x:c r="E46" s="30"/>
+      <x:c r="F46" s="30"/>
+      <x:c r="G46" s="30"/>
+      <x:c r="H46" s="30"/>
+      <x:c r="I46" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I43:I44),0),1)</x:f>
+        <x:v>122.5</x:v>
+      </x:c>
+      <x:c r="J46" s="30"/>
+      <x:c r="K46" s="30"/>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="17" t="str">
+        <x:v>IH主力</x:v>
+      </x:c>
+      <x:c r="B48" s="17"/>
+      <x:c r="C48" s="17"/>
+      <x:c r="D48" s="17"/>
+      <x:c r="E48" s="17"/>
+      <x:c r="F48" s="17"/>
+      <x:c r="G48" s="17"/>
+      <x:c r="H48" s="17"/>
+      <x:c r="I48" s="17"/>
+      <x:c r="J48" s="17"/>
+      <x:c r="K48" s="17"/>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B39" s="20" t="str">
+      <x:c r="B49" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C39" s="20" t="str">
+      <x:c r="C49" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D39" s="20" t="str">
+      <x:c r="D49" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E39" s="20" t="str">
+      <x:c r="E49" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F39" s="20" t="str">
+      <x:c r="F49" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G39" s="20" t="str">
+      <x:c r="G49" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H39" s="20" t="str">
+      <x:c r="H49" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I39" s="20" t="str">
+      <x:c r="I49" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J39" s="20" t="str">
+      <x:c r="J49" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K39" s="20" t="str">
+      <x:c r="K49" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="40">
-      <x:c r="A40" s="22" t="n">
+    <x:row r="50">
+      <x:c r="A50" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B40" s="22" t="str">
+      <x:c r="B50" s="22" t="str">
         <x:v>8月3日-8月7日</x:v>
       </x:c>
-      <x:c r="C40" s="23" t="n">
-        <x:v>4526.4</x:v>
-      </x:c>
-      <x:c r="D40" s="23" t="n">
-        <x:v>4656.2</x:v>
-      </x:c>
-      <x:c r="E40" s="23" t="n">
-        <x:v>4494.2</x:v>
-      </x:c>
-      <x:c r="F40" s="23" t="n">
-        <x:v>4645.6</x:v>
-      </x:c>
-      <x:c r="G40" s="23"/>
-      <x:c r="H40" s="24"/>
-      <x:c r="I40" s="26" t="n">
-        <x:f>ROUND(D40-E40,1)</x:f>
-        <x:v>162</x:v>
-      </x:c>
-      <x:c r="J40" s="22" t="str">
-        <x:v>IF2609</x:v>
-      </x:c>
-      <x:c r="K40" s="22" t="n">
+      <x:c r="C50" s="23" t="n">
+        <x:v>2882.4</x:v>
+      </x:c>
+      <x:c r="D50" s="23" t="n">
+        <x:v>2930.6</x:v>
+      </x:c>
+      <x:c r="E50" s="23" t="n">
+        <x:v>2845.8</x:v>
+      </x:c>
+      <x:c r="F50" s="23" t="n">
+        <x:v>2930</x:v>
+      </x:c>
+      <x:c r="G50" s="23"/>
+      <x:c r="H50" s="24"/>
+      <x:c r="I50" s="26" t="n">
+        <x:f>ROUND(D50-E50,1)</x:f>
+        <x:v>84.8</x:v>
+      </x:c>
+      <x:c r="J50" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+      <x:c r="K50" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="41">
-      <x:c r="A41" s="22" t="n">
+    <x:row r="51">
+      <x:c r="A51" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B41" s="22" t="str">
+      <x:c r="B51" s="22" t="str">
         <x:v>8月10日-8月14日</x:v>
       </x:c>
-      <x:c r="C41" s="23" t="n">
-        <x:v>4656.8</x:v>
-      </x:c>
-      <x:c r="D41" s="23" t="n">
-        <x:v>4681</x:v>
-      </x:c>
-      <x:c r="E41" s="23" t="n">
-        <x:v>4598</x:v>
-      </x:c>
-      <x:c r="F41" s="23" t="n">
-        <x:v>4620.4</x:v>
-      </x:c>
-      <x:c r="G41" s="23" t="n">
-        <x:f>ROUND(F41-F40,1)</x:f>
-        <x:v>-25.2</x:v>
-      </x:c>
-      <x:c r="H41" s="24" t="n">
-        <x:f>IFERROR(F41/F40-1,"")</x:f>
-        <x:v>-0.005424487687274104</x:v>
-      </x:c>
-      <x:c r="I41" s="23" t="n">
-        <x:f>ROUND(D41-E41,1)</x:f>
-        <x:v>83</x:v>
-      </x:c>
-      <x:c r="J41" s="22" t="str">
-        <x:v>IF2609</x:v>
-      </x:c>
-      <x:c r="K41" s="22" t="n">
+      <x:c r="C51" s="23" t="n">
+        <x:v>2930</x:v>
+      </x:c>
+      <x:c r="D51" s="23" t="n">
+        <x:v>2949.6</x:v>
+      </x:c>
+      <x:c r="E51" s="23" t="n">
+        <x:v>2877</x:v>
+      </x:c>
+      <x:c r="F51" s="23" t="n">
+        <x:v>2890</x:v>
+      </x:c>
+      <x:c r="G51" s="23" t="n">
+        <x:f>ROUND(F51-F50,1)</x:f>
+        <x:v>-40</x:v>
+      </x:c>
+      <x:c r="H51" s="24" t="n">
+        <x:f>IFERROR(F51/F50-1,"")</x:f>
+        <x:v>-0.013651877133105783</x:v>
+      </x:c>
+      <x:c r="I51" s="26" t="n">
+        <x:f>ROUND(D51-E51,1)</x:f>
+        <x:v>72.6</x:v>
+      </x:c>
+      <x:c r="J51" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+      <x:c r="K51" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="42">
-      <x:c r="A42" s="29" t="str">
+    <x:row r="52">
+      <x:c r="A52" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B42" s="28" t="n">
+      <x:c r="B52" s="30" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C42" s="28"/>
-      <x:c r="D42" s="28"/>
-      <x:c r="E42" s="28"/>
-      <x:c r="F42" s="28"/>
-      <x:c r="G42" s="28"/>
-      <x:c r="H42" s="28"/>
-      <x:c r="I42" s="30" t="n">
-        <x:f>ROUND(SUM(I40:I41),1)</x:f>
-        <x:v>245</x:v>
-      </x:c>
-      <x:c r="J42" s="28"/>
-      <x:c r="K42" s="28"/>
-    </x:row>
-    <x:row r="43">
-      <x:c r="A43" s="29" t="str">
+      <x:c r="C52" s="30"/>
+      <x:c r="D52" s="30"/>
+      <x:c r="E52" s="30"/>
+      <x:c r="F52" s="30"/>
+      <x:c r="G52" s="30"/>
+      <x:c r="H52" s="30"/>
+      <x:c r="I52" s="32" t="n">
+        <x:f>ROUND(SUM(I50:I51),1)</x:f>
+        <x:v>157.4</x:v>
+      </x:c>
+      <x:c r="J52" s="30"/>
+      <x:c r="K52" s="30"/>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B43" s="28"/>
-      <x:c r="C43" s="28"/>
-      <x:c r="D43" s="28"/>
-      <x:c r="E43" s="28"/>
-      <x:c r="F43" s="28"/>
-      <x:c r="G43" s="28"/>
-      <x:c r="H43" s="28"/>
-      <x:c r="I43" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I40:I41),0),1)</x:f>
-        <x:v>122.5</x:v>
-      </x:c>
-      <x:c r="J43" s="28"/>
-      <x:c r="K43" s="28"/>
-    </x:row>
-    <x:row r="45">
-      <x:c r="A45" s="17" t="str">
-        <x:v>IH主力</x:v>
-      </x:c>
-      <x:c r="B45" s="17"/>
-      <x:c r="C45" s="17"/>
-      <x:c r="D45" s="17"/>
-      <x:c r="E45" s="17"/>
-      <x:c r="F45" s="17"/>
-      <x:c r="G45" s="17"/>
-      <x:c r="H45" s="17"/>
-      <x:c r="I45" s="17"/>
-      <x:c r="J45" s="17"/>
-      <x:c r="K45" s="17"/>
-    </x:row>
-    <x:row r="46">
-      <x:c r="A46" s="20" t="str">
+      <x:c r="B53" s="30"/>
+      <x:c r="C53" s="30"/>
+      <x:c r="D53" s="30"/>
+      <x:c r="E53" s="30"/>
+      <x:c r="F53" s="30"/>
+      <x:c r="G53" s="30"/>
+      <x:c r="H53" s="30"/>
+      <x:c r="I53" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I50:I51),0),1)</x:f>
+        <x:v>78.7</x:v>
+      </x:c>
+      <x:c r="J53" s="30"/>
+      <x:c r="K53" s="30"/>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="17" t="str">
+        <x:v>碳酸锂2609</x:v>
+      </x:c>
+      <x:c r="B55" s="17"/>
+      <x:c r="C55" s="17"/>
+      <x:c r="D55" s="17"/>
+      <x:c r="E55" s="17"/>
+      <x:c r="F55" s="17"/>
+      <x:c r="G55" s="17"/>
+      <x:c r="H55" s="17"/>
+      <x:c r="I55" s="17"/>
+      <x:c r="J55" s="17"/>
+      <x:c r="K55" s="17"/>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B46" s="20" t="str">
+      <x:c r="B56" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C46" s="20" t="str">
+      <x:c r="C56" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D46" s="20" t="str">
+      <x:c r="D56" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E46" s="20" t="str">
+      <x:c r="E56" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F46" s="20" t="str">
+      <x:c r="F56" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G46" s="20" t="str">
+      <x:c r="G56" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H46" s="20" t="str">
+      <x:c r="H56" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I46" s="20" t="str">
+      <x:c r="I56" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J46" s="20" t="str">
+      <x:c r="J56" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K46" s="20" t="str">
+      <x:c r="K56" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="47">
-      <x:c r="A47" s="22" t="n">
+    <x:row r="57">
+      <x:c r="A57" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B47" s="22" t="str">
+      <x:c r="B57" s="22" t="str">
         <x:v>8月3日-8月7日</x:v>
       </x:c>
-      <x:c r="C47" s="23" t="n">
-        <x:v>2882.4</x:v>
-      </x:c>
-      <x:c r="D47" s="23" t="n">
-        <x:v>2930.6</x:v>
-      </x:c>
-      <x:c r="E47" s="23" t="n">
-        <x:v>2845.8</x:v>
-      </x:c>
-      <x:c r="F47" s="23" t="n">
-        <x:v>2930</x:v>
-      </x:c>
-      <x:c r="G47" s="23"/>
-      <x:c r="H47" s="24"/>
-      <x:c r="I47" s="26" t="n">
-        <x:f>ROUND(D47-E47,1)</x:f>
-        <x:v>84.8</x:v>
-      </x:c>
-      <x:c r="J47" s="22" t="str">
-        <x:v>IH2609</x:v>
-      </x:c>
-      <x:c r="K47" s="22" t="n">
+      <x:c r="C57" s="23" t="n">
+        <x:v>137500</x:v>
+      </x:c>
+      <x:c r="D57" s="23" t="n">
+        <x:v>144800</x:v>
+      </x:c>
+      <x:c r="E57" s="23" t="n">
+        <x:v>135560</x:v>
+      </x:c>
+      <x:c r="F57" s="23" t="n">
+        <x:v>140000</x:v>
+      </x:c>
+      <x:c r="G57" s="23"/>
+      <x:c r="H57" s="24"/>
+      <x:c r="I57" s="26" t="n">
+        <x:f>ROUND(D57-E57,1)</x:f>
+        <x:v>9240</x:v>
+      </x:c>
+      <x:c r="J57" s="22" t="str">
+        <x:v>LC2609</x:v>
+      </x:c>
+      <x:c r="K57" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="48">
-      <x:c r="A48" s="22" t="n">
+    <x:row r="58">
+      <x:c r="A58" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B48" s="22" t="str">
+      <x:c r="B58" s="22" t="str">
         <x:v>8月10日-8月14日</x:v>
       </x:c>
-      <x:c r="C48" s="23" t="n">
-        <x:v>2930</x:v>
-      </x:c>
-      <x:c r="D48" s="23" t="n">
-        <x:v>2949.6</x:v>
-      </x:c>
-      <x:c r="E48" s="23" t="n">
-        <x:v>2877</x:v>
-      </x:c>
-      <x:c r="F48" s="23" t="n">
-        <x:v>2890</x:v>
-      </x:c>
-      <x:c r="G48" s="23" t="n">
-        <x:f>ROUND(F48-F47,1)</x:f>
-        <x:v>-40</x:v>
-      </x:c>
-      <x:c r="H48" s="24" t="n">
-        <x:f>IFERROR(F48/F47-1,"")</x:f>
-        <x:v>-0.013651877133105783</x:v>
-      </x:c>
-      <x:c r="I48" s="26" t="n">
-        <x:f>ROUND(D48-E48,1)</x:f>
-        <x:v>72.6</x:v>
-      </x:c>
-      <x:c r="J48" s="22" t="str">
-        <x:v>IH2609</x:v>
-      </x:c>
-      <x:c r="K48" s="22" t="n">
+      <x:c r="C58" s="23" t="n">
+        <x:v>140500</x:v>
+      </x:c>
+      <x:c r="D58" s="23" t="n">
+        <x:v>154500</x:v>
+      </x:c>
+      <x:c r="E58" s="23" t="n">
+        <x:v>139280</x:v>
+      </x:c>
+      <x:c r="F58" s="23" t="n">
+        <x:v>153940</x:v>
+      </x:c>
+      <x:c r="G58" s="28" t="n">
+        <x:f>ROUND(F58-F57,1)</x:f>
+        <x:v>13940</x:v>
+      </x:c>
+      <x:c r="H58" s="24" t="n">
+        <x:f>IFERROR(F58/F57-1,"")</x:f>
+        <x:v>0.09957142857142864</x:v>
+      </x:c>
+      <x:c r="I58" s="26" t="n">
+        <x:f>ROUND(D58-E58,1)</x:f>
+        <x:v>15220</x:v>
+      </x:c>
+      <x:c r="J58" s="22" t="str">
+        <x:v>LC2609</x:v>
+      </x:c>
+      <x:c r="K58" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="49">
-      <x:c r="A49" s="29" t="str">
+    <x:row r="59">
+      <x:c r="A59" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B49" s="28" t="n">
+      <x:c r="B59" s="30" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C49" s="28"/>
-      <x:c r="D49" s="28"/>
-      <x:c r="E49" s="28"/>
-      <x:c r="F49" s="28"/>
-      <x:c r="G49" s="28"/>
-      <x:c r="H49" s="28"/>
-      <x:c r="I49" s="30" t="n">
-        <x:f>ROUND(SUM(I47:I48),1)</x:f>
-        <x:v>157.4</x:v>
-      </x:c>
-      <x:c r="J49" s="28"/>
-      <x:c r="K49" s="28"/>
-    </x:row>
-    <x:row r="50">
-      <x:c r="A50" s="29" t="str">
+      <x:c r="C59" s="30"/>
+      <x:c r="D59" s="30"/>
+      <x:c r="E59" s="30"/>
+      <x:c r="F59" s="30"/>
+      <x:c r="G59" s="30"/>
+      <x:c r="H59" s="30"/>
+      <x:c r="I59" s="32" t="n">
+        <x:f>ROUND(SUM(I57:I58),1)</x:f>
+        <x:v>24460</x:v>
+      </x:c>
+      <x:c r="J59" s="30"/>
+      <x:c r="K59" s="30"/>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B50" s="28"/>
-      <x:c r="C50" s="28"/>
-      <x:c r="D50" s="28"/>
-      <x:c r="E50" s="28"/>
-      <x:c r="F50" s="28"/>
-      <x:c r="G50" s="28"/>
-      <x:c r="H50" s="28"/>
-      <x:c r="I50" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I47:I48),0),1)</x:f>
-        <x:v>78.7</x:v>
-      </x:c>
-      <x:c r="J50" s="28"/>
-      <x:c r="K50" s="28"/>
-    </x:row>
-    <x:row r="52">
-      <x:c r="A52" s="17" t="str">
-        <x:v>碳酸锂2609</x:v>
-      </x:c>
-      <x:c r="B52" s="17"/>
-      <x:c r="C52" s="17"/>
-      <x:c r="D52" s="17"/>
-      <x:c r="E52" s="17"/>
-      <x:c r="F52" s="17"/>
-      <x:c r="G52" s="17"/>
-      <x:c r="H52" s="17"/>
-      <x:c r="I52" s="17"/>
-      <x:c r="J52" s="17"/>
-      <x:c r="K52" s="17"/>
-    </x:row>
-    <x:row r="53">
-      <x:c r="A53" s="20" t="str">
-        <x:v>序号</x:v>
-      </x:c>
-      <x:c r="B53" s="20" t="str">
-        <x:v>周期</x:v>
-      </x:c>
-      <x:c r="C53" s="20" t="str">
-        <x:v>开盘</x:v>
-      </x:c>
-      <x:c r="D53" s="20" t="str">
-        <x:v>高点</x:v>
-      </x:c>
-      <x:c r="E53" s="20" t="str">
-        <x:v>低点</x:v>
-      </x:c>
-      <x:c r="F53" s="20" t="str">
-        <x:v>收盘</x:v>
-      </x:c>
-      <x:c r="G53" s="20" t="str">
-        <x:v>涨跌点数</x:v>
-      </x:c>
-      <x:c r="H53" s="20" t="str">
-        <x:v>涨幅</x:v>
-      </x:c>
-      <x:c r="I53" s="20" t="str">
-        <x:v>振幅</x:v>
-      </x:c>
-      <x:c r="J53" s="20" t="str">
-        <x:v>标的</x:v>
-      </x:c>
-      <x:c r="K53" s="20" t="str">
-        <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="54">
-      <x:c r="A54" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B54" s="22" t="str">
-        <x:v>8月3日-8月7日</x:v>
-      </x:c>
-      <x:c r="C54" s="23" t="n">
-        <x:v>137500</x:v>
-      </x:c>
-      <x:c r="D54" s="23" t="n">
-        <x:v>144800</x:v>
-      </x:c>
-      <x:c r="E54" s="23" t="n">
-        <x:v>135560</x:v>
-      </x:c>
-      <x:c r="F54" s="23" t="n">
-        <x:v>140000</x:v>
-      </x:c>
-      <x:c r="G54" s="23"/>
-      <x:c r="H54" s="24"/>
-      <x:c r="I54" s="26" t="n">
-        <x:f>ROUND(D54-E54,1)</x:f>
-        <x:v>9240</x:v>
-      </x:c>
-      <x:c r="J54" s="22" t="str">
-        <x:v>LC2609</x:v>
-      </x:c>
-      <x:c r="K54" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="55">
-      <x:c r="A55" s="22" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B55" s="22" t="str">
-        <x:v>8月10日-8月14日</x:v>
-      </x:c>
-      <x:c r="C55" s="23" t="n">
-        <x:v>140500</x:v>
-      </x:c>
-      <x:c r="D55" s="23" t="n">
-        <x:v>154500</x:v>
-      </x:c>
-      <x:c r="E55" s="23" t="n">
-        <x:v>139280</x:v>
-      </x:c>
-      <x:c r="F55" s="23" t="n">
-        <x:v>153940</x:v>
-      </x:c>
-      <x:c r="G55" s="34" t="n">
-        <x:f>ROUND(F55-F54,1)</x:f>
-        <x:v>13940</x:v>
-      </x:c>
-      <x:c r="H55" s="24" t="n">
-        <x:f>IFERROR(F55/F54-1,"")</x:f>
-        <x:v>0.09957142857142864</x:v>
-      </x:c>
-      <x:c r="I55" s="26" t="n">
-        <x:f>ROUND(D55-E55,1)</x:f>
-        <x:v>15220</x:v>
-      </x:c>
-      <x:c r="J55" s="22" t="str">
-        <x:v>LC2609</x:v>
-      </x:c>
-      <x:c r="K55" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="56">
-      <x:c r="A56" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B56" s="28" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C56" s="28"/>
-      <x:c r="D56" s="28"/>
-      <x:c r="E56" s="28"/>
-      <x:c r="F56" s="28"/>
-      <x:c r="G56" s="28"/>
-      <x:c r="H56" s="28"/>
-      <x:c r="I56" s="30" t="n">
-        <x:f>ROUND(SUM(I54:I55),1)</x:f>
-        <x:v>24460</x:v>
-      </x:c>
-      <x:c r="J56" s="28"/>
-      <x:c r="K56" s="28"/>
-    </x:row>
-    <x:row r="57">
-      <x:c r="A57" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B57" s="28"/>
-      <x:c r="C57" s="28"/>
-      <x:c r="D57" s="28"/>
-      <x:c r="E57" s="28"/>
-      <x:c r="F57" s="28"/>
-      <x:c r="G57" s="28"/>
-      <x:c r="H57" s="28"/>
-      <x:c r="I57" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I54:I55),0),1)</x:f>
+      <x:c r="B60" s="30"/>
+      <x:c r="C60" s="30"/>
+      <x:c r="D60" s="30"/>
+      <x:c r="E60" s="30"/>
+      <x:c r="F60" s="30"/>
+      <x:c r="G60" s="30"/>
+      <x:c r="H60" s="30"/>
+      <x:c r="I60" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I57:I58),0),1)</x:f>
         <x:v>12230</x:v>
       </x:c>
-      <x:c r="J57" s="28"/>
-      <x:c r="K57" s="28"/>
+      <x:c r="J60" s="30"/>
+      <x:c r="K60" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:K1"/>
     <x:mergeCell ref="A3:K3"/>
-    <x:mergeCell ref="A10:K10"/>
-    <x:mergeCell ref="A17:K17"/>
-    <x:mergeCell ref="A24:K24"/>
-    <x:mergeCell ref="A31:K31"/>
-    <x:mergeCell ref="A38:K38"/>
-    <x:mergeCell ref="A45:K45"/>
-    <x:mergeCell ref="A52:K52"/>
+    <x:mergeCell ref="A11:K11"/>
+    <x:mergeCell ref="A19:K19"/>
+    <x:mergeCell ref="A27:K27"/>
+    <x:mergeCell ref="A34:K34"/>
+    <x:mergeCell ref="A41:K41"/>
+    <x:mergeCell ref="A48:K48"/>
+    <x:mergeCell ref="A55:K55"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2726,7 +2840,7 @@
       <x:c r="G5" s="23" t="n">
         <x:v>7279.19</x:v>
       </x:c>
-      <x:c r="H5" s="34" t="n">
+      <x:c r="H5" s="28" t="n">
         <x:v>199.4</x:v>
       </x:c>
       <x:c r="I5" s="24" t="n">
@@ -2762,7 +2876,7 @@
       <x:c r="G6" s="23" t="n">
         <x:v>7493.05</x:v>
       </x:c>
-      <x:c r="H6" s="34" t="n">
+      <x:c r="H6" s="28" t="n">
         <x:v>213.9</x:v>
       </x:c>
       <x:c r="I6" s="24" t="n">
@@ -3028,43 +3142,79 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="29" t="str">
+    <x:row r="14">
+      <x:c r="A14" s="22" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B14" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C14" s="22" t="str">
+        <x:v>8月17日</x:v>
+      </x:c>
+      <x:c r="D14" s="23" t="n">
+        <x:v>7797.18</x:v>
+      </x:c>
+      <x:c r="E14" s="23" t="n">
+        <x:v>7968.38</x:v>
+      </x:c>
+      <x:c r="F14" s="23" t="n">
+        <x:v>7750.43</x:v>
+      </x:c>
+      <x:c r="G14" s="23" t="n">
+        <x:v>7968.38</x:v>
+      </x:c>
+      <x:c r="H14" s="28" t="n">
+        <x:v>198.6</x:v>
+      </x:c>
+      <x:c r="I14" s="24" t="n">
+        <x:v>0.02555528956912778</x:v>
+      </x:c>
+      <x:c r="J14" s="26" t="n">
+        <x:f>ROUND(E14-F14,1)</x:f>
+        <x:v>217.9</x:v>
+      </x:c>
+      <x:c r="K14" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B16" s="28" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="C16" s="28"/>
-      <x:c r="D16" s="28"/>
-      <x:c r="E16" s="28"/>
-      <x:c r="F16" s="28"/>
-      <x:c r="G16" s="28"/>
-      <x:c r="H16" s="28"/>
-      <x:c r="I16" s="28"/>
-      <x:c r="J16" s="30" t="n">
-        <x:f>SUM(J4:J13)</x:f>
-        <x:v>1568.4</x:v>
-      </x:c>
-      <x:c r="K16" s="28"/>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="29" t="str">
+      <x:c r="B17" s="30" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C17" s="30"/>
+      <x:c r="D17" s="30"/>
+      <x:c r="E17" s="30"/>
+      <x:c r="F17" s="30"/>
+      <x:c r="G17" s="30"/>
+      <x:c r="H17" s="30"/>
+      <x:c r="I17" s="30"/>
+      <x:c r="J17" s="32" t="n">
+        <x:f>SUM(J4:J14)</x:f>
+        <x:v>1786.3000000000002</x:v>
+      </x:c>
+      <x:c r="K17" s="30"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B17" s="28"/>
-      <x:c r="C17" s="28"/>
-      <x:c r="D17" s="28"/>
-      <x:c r="E17" s="28"/>
-      <x:c r="F17" s="28"/>
-      <x:c r="G17" s="28"/>
-      <x:c r="H17" s="28"/>
-      <x:c r="I17" s="28"/>
-      <x:c r="J17" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
-        <x:v>156.8</x:v>
-      </x:c>
-      <x:c r="K17" s="28"/>
+      <x:c r="B18" s="30"/>
+      <x:c r="C18" s="30"/>
+      <x:c r="D18" s="30"/>
+      <x:c r="E18" s="30"/>
+      <x:c r="F18" s="30"/>
+      <x:c r="G18" s="30"/>
+      <x:c r="H18" s="30"/>
+      <x:c r="I18" s="30"/>
+      <x:c r="J18" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J14),0),1)</x:f>
+        <x:v>162.4</x:v>
+      </x:c>
+      <x:c r="K18" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3189,7 +3339,7 @@
       <x:c r="G5" s="23" t="n">
         <x:v>7607.49</x:v>
       </x:c>
-      <x:c r="H5" s="34" t="n">
+      <x:c r="H5" s="28" t="n">
         <x:v>193</x:v>
       </x:c>
       <x:c r="I5" s="24" t="n">
@@ -3225,7 +3375,7 @@
       <x:c r="G6" s="23" t="n">
         <x:v>7809.21</x:v>
       </x:c>
-      <x:c r="H6" s="34" t="n">
+      <x:c r="H6" s="28" t="n">
         <x:v>201.7</x:v>
       </x:c>
       <x:c r="I6" s="24" t="n">
@@ -3297,7 +3447,7 @@
       <x:c r="G8" s="23" t="n">
         <x:v>7980.12</x:v>
       </x:c>
-      <x:c r="H8" s="34" t="n">
+      <x:c r="H8" s="28" t="n">
         <x:v>150.8</x:v>
       </x:c>
       <x:c r="I8" s="24" t="n">
@@ -3491,43 +3641,79 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="29" t="str">
+    <x:row r="14">
+      <x:c r="A14" s="22" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B14" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C14" s="22" t="str">
+        <x:v>8月17日</x:v>
+      </x:c>
+      <x:c r="D14" s="23" t="n">
+        <x:v>8007.87</x:v>
+      </x:c>
+      <x:c r="E14" s="23" t="n">
+        <x:v>8184.64</x:v>
+      </x:c>
+      <x:c r="F14" s="23" t="n">
+        <x:v>7992.36</x:v>
+      </x:c>
+      <x:c r="G14" s="23" t="n">
+        <x:v>8184.64</x:v>
+      </x:c>
+      <x:c r="H14" s="28" t="n">
+        <x:v>194.3</x:v>
+      </x:c>
+      <x:c r="I14" s="24" t="n">
+        <x:v>0.02431814455723358</x:v>
+      </x:c>
+      <x:c r="J14" s="26" t="n">
+        <x:f>ROUND(E14-F14,1)</x:f>
+        <x:v>192.3</x:v>
+      </x:c>
+      <x:c r="K14" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B16" s="28" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="C16" s="28"/>
-      <x:c r="D16" s="28"/>
-      <x:c r="E16" s="28"/>
-      <x:c r="F16" s="28"/>
-      <x:c r="G16" s="28"/>
-      <x:c r="H16" s="28"/>
-      <x:c r="I16" s="28"/>
-      <x:c r="J16" s="30" t="n">
-        <x:f>SUM(J4:J13)</x:f>
-        <x:v>1580.2000000000003</x:v>
-      </x:c>
-      <x:c r="K16" s="28"/>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="29" t="str">
+      <x:c r="B17" s="30" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C17" s="30"/>
+      <x:c r="D17" s="30"/>
+      <x:c r="E17" s="30"/>
+      <x:c r="F17" s="30"/>
+      <x:c r="G17" s="30"/>
+      <x:c r="H17" s="30"/>
+      <x:c r="I17" s="30"/>
+      <x:c r="J17" s="32" t="n">
+        <x:f>SUM(J4:J14)</x:f>
+        <x:v>1772.5000000000002</x:v>
+      </x:c>
+      <x:c r="K17" s="30"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B17" s="28"/>
-      <x:c r="C17" s="28"/>
-      <x:c r="D17" s="28"/>
-      <x:c r="E17" s="28"/>
-      <x:c r="F17" s="28"/>
-      <x:c r="G17" s="28"/>
-      <x:c r="H17" s="28"/>
-      <x:c r="I17" s="28"/>
-      <x:c r="J17" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
-        <x:v>158</x:v>
-      </x:c>
-      <x:c r="K17" s="28"/>
+      <x:c r="B18" s="30"/>
+      <x:c r="C18" s="30"/>
+      <x:c r="D18" s="30"/>
+      <x:c r="E18" s="30"/>
+      <x:c r="F18" s="30"/>
+      <x:c r="G18" s="30"/>
+      <x:c r="H18" s="30"/>
+      <x:c r="I18" s="30"/>
+      <x:c r="J18" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J14),0),1)</x:f>
+        <x:v>161.1</x:v>
+      </x:c>
+      <x:c r="K18" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3954,43 +4140,79 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="29" t="str">
+    <x:row r="14">
+      <x:c r="A14" s="22" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B14" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C14" s="22" t="str">
+        <x:v>8月17日</x:v>
+      </x:c>
+      <x:c r="D14" s="23" t="n">
+        <x:v>3930.1</x:v>
+      </x:c>
+      <x:c r="E14" s="23" t="n">
+        <x:v>3983.51</x:v>
+      </x:c>
+      <x:c r="F14" s="23" t="n">
+        <x:v>3924.47</x:v>
+      </x:c>
+      <x:c r="G14" s="23" t="n">
+        <x:v>3982.65</x:v>
+      </x:c>
+      <x:c r="H14" s="23" t="n">
+        <x:v>55.5</x:v>
+      </x:c>
+      <x:c r="I14" s="24" t="n">
+        <x:v>0.014124639053977761</x:v>
+      </x:c>
+      <x:c r="J14" s="26" t="n">
+        <x:f>ROUND(E14-F14,1)</x:f>
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="K14" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B16" s="28" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="C16" s="28"/>
-      <x:c r="D16" s="28"/>
-      <x:c r="E16" s="28"/>
-      <x:c r="F16" s="28"/>
-      <x:c r="G16" s="28"/>
-      <x:c r="H16" s="28"/>
-      <x:c r="I16" s="28"/>
-      <x:c r="J16" s="30" t="n">
-        <x:f>SUM(J4:J13)</x:f>
-        <x:v>385.40000000000003</x:v>
-      </x:c>
-      <x:c r="K16" s="28"/>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="29" t="str">
+      <x:c r="B17" s="30" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C17" s="30"/>
+      <x:c r="D17" s="30"/>
+      <x:c r="E17" s="30"/>
+      <x:c r="F17" s="30"/>
+      <x:c r="G17" s="30"/>
+      <x:c r="H17" s="30"/>
+      <x:c r="I17" s="30"/>
+      <x:c r="J17" s="32" t="n">
+        <x:f>SUM(J4:J14)</x:f>
+        <x:v>444.40000000000003</x:v>
+      </x:c>
+      <x:c r="K17" s="30"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B17" s="28"/>
-      <x:c r="C17" s="28"/>
-      <x:c r="D17" s="28"/>
-      <x:c r="E17" s="28"/>
-      <x:c r="F17" s="28"/>
-      <x:c r="G17" s="28"/>
-      <x:c r="H17" s="28"/>
-      <x:c r="I17" s="28"/>
-      <x:c r="J17" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
-        <x:v>38.5</x:v>
-      </x:c>
-      <x:c r="K17" s="28"/>
+      <x:c r="B18" s="30"/>
+      <x:c r="C18" s="30"/>
+      <x:c r="D18" s="30"/>
+      <x:c r="E18" s="30"/>
+      <x:c r="F18" s="30"/>
+      <x:c r="G18" s="30"/>
+      <x:c r="H18" s="30"/>
+      <x:c r="I18" s="30"/>
+      <x:c r="J18" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J14),0),1)</x:f>
+        <x:v>40.4</x:v>
+      </x:c>
+      <x:c r="K18" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4115,7 +4337,7 @@
       <x:c r="G5" s="23" t="n">
         <x:v>7211.4</x:v>
       </x:c>
-      <x:c r="H5" s="34" t="n">
+      <x:c r="H5" s="28" t="n">
         <x:v>188</x:v>
       </x:c>
       <x:c r="I5" s="24" t="n">
@@ -4151,7 +4373,7 @@
       <x:c r="G6" s="23" t="n">
         <x:v>7433.8</x:v>
       </x:c>
-      <x:c r="H6" s="34" t="n">
+      <x:c r="H6" s="28" t="n">
         <x:v>222.4</x:v>
       </x:c>
       <x:c r="I6" s="24" t="n">
@@ -4418,42 +4640,42 @@
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="29" t="str">
+      <x:c r="A16" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B16" s="28" t="n">
+      <x:c r="B16" s="30" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C16" s="28"/>
-      <x:c r="D16" s="28"/>
-      <x:c r="E16" s="28"/>
-      <x:c r="F16" s="28"/>
-      <x:c r="G16" s="28"/>
-      <x:c r="H16" s="28"/>
-      <x:c r="I16" s="28"/>
-      <x:c r="J16" s="30" t="n">
+      <x:c r="C16" s="30"/>
+      <x:c r="D16" s="30"/>
+      <x:c r="E16" s="30"/>
+      <x:c r="F16" s="30"/>
+      <x:c r="G16" s="30"/>
+      <x:c r="H16" s="30"/>
+      <x:c r="I16" s="30"/>
+      <x:c r="J16" s="32" t="n">
         <x:f>SUM(J4:J13)</x:f>
         <x:v>1525</x:v>
       </x:c>
-      <x:c r="K16" s="28"/>
+      <x:c r="K16" s="30"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="29" t="str">
+      <x:c r="A17" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B17" s="28"/>
-      <x:c r="C17" s="28"/>
-      <x:c r="D17" s="28"/>
-      <x:c r="E17" s="28"/>
-      <x:c r="F17" s="28"/>
-      <x:c r="G17" s="28"/>
-      <x:c r="H17" s="28"/>
-      <x:c r="I17" s="28"/>
-      <x:c r="J17" s="32" t="n">
+      <x:c r="B17" s="30"/>
+      <x:c r="C17" s="30"/>
+      <x:c r="D17" s="30"/>
+      <x:c r="E17" s="30"/>
+      <x:c r="F17" s="30"/>
+      <x:c r="G17" s="30"/>
+      <x:c r="H17" s="30"/>
+      <x:c r="I17" s="30"/>
+      <x:c r="J17" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
         <x:v>152.5</x:v>
       </x:c>
-      <x:c r="K17" s="28"/>
+      <x:c r="K17" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4578,7 +4800,7 @@
       <x:c r="G5" s="23" t="n">
         <x:v>7529</x:v>
       </x:c>
-      <x:c r="H5" s="34" t="n">
+      <x:c r="H5" s="28" t="n">
         <x:v>173</x:v>
       </x:c>
       <x:c r="I5" s="24" t="n">
@@ -4614,7 +4836,7 @@
       <x:c r="G6" s="23" t="n">
         <x:v>7744.4</x:v>
       </x:c>
-      <x:c r="H6" s="34" t="n">
+      <x:c r="H6" s="28" t="n">
         <x:v>215.4</x:v>
       </x:c>
       <x:c r="I6" s="24" t="n">
@@ -4881,42 +5103,42 @@
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="29" t="str">
+      <x:c r="A16" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B16" s="28" t="n">
+      <x:c r="B16" s="30" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C16" s="28"/>
-      <x:c r="D16" s="28"/>
-      <x:c r="E16" s="28"/>
-      <x:c r="F16" s="28"/>
-      <x:c r="G16" s="28"/>
-      <x:c r="H16" s="28"/>
-      <x:c r="I16" s="28"/>
-      <x:c r="J16" s="30" t="n">
+      <x:c r="C16" s="30"/>
+      <x:c r="D16" s="30"/>
+      <x:c r="E16" s="30"/>
+      <x:c r="F16" s="30"/>
+      <x:c r="G16" s="30"/>
+      <x:c r="H16" s="30"/>
+      <x:c r="I16" s="30"/>
+      <x:c r="J16" s="32" t="n">
         <x:f>SUM(J4:J13)</x:f>
         <x:v>1573</x:v>
       </x:c>
-      <x:c r="K16" s="28"/>
+      <x:c r="K16" s="30"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="29" t="str">
+      <x:c r="A17" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B17" s="28"/>
-      <x:c r="C17" s="28"/>
-      <x:c r="D17" s="28"/>
-      <x:c r="E17" s="28"/>
-      <x:c r="F17" s="28"/>
-      <x:c r="G17" s="28"/>
-      <x:c r="H17" s="28"/>
-      <x:c r="I17" s="28"/>
-      <x:c r="J17" s="32" t="n">
+      <x:c r="B17" s="30"/>
+      <x:c r="C17" s="30"/>
+      <x:c r="D17" s="30"/>
+      <x:c r="E17" s="30"/>
+      <x:c r="F17" s="30"/>
+      <x:c r="G17" s="30"/>
+      <x:c r="H17" s="30"/>
+      <x:c r="I17" s="30"/>
+      <x:c r="J17" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
         <x:v>157.3</x:v>
       </x:c>
-      <x:c r="K17" s="28"/>
+      <x:c r="K17" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5344,42 +5566,42 @@
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="29" t="str">
+      <x:c r="A16" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B16" s="28" t="n">
+      <x:c r="B16" s="30" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C16" s="28"/>
-      <x:c r="D16" s="28"/>
-      <x:c r="E16" s="28"/>
-      <x:c r="F16" s="28"/>
-      <x:c r="G16" s="28"/>
-      <x:c r="H16" s="28"/>
-      <x:c r="I16" s="28"/>
-      <x:c r="J16" s="30" t="n">
+      <x:c r="C16" s="30"/>
+      <x:c r="D16" s="30"/>
+      <x:c r="E16" s="30"/>
+      <x:c r="F16" s="30"/>
+      <x:c r="G16" s="30"/>
+      <x:c r="H16" s="30"/>
+      <x:c r="I16" s="30"/>
+      <x:c r="J16" s="32" t="n">
         <x:f>SUM(J4:J13)</x:f>
         <x:v>569.8000000000001</x:v>
       </x:c>
-      <x:c r="K16" s="28"/>
+      <x:c r="K16" s="30"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="29" t="str">
+      <x:c r="A17" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B17" s="28"/>
-      <x:c r="C17" s="28"/>
-      <x:c r="D17" s="28"/>
-      <x:c r="E17" s="28"/>
-      <x:c r="F17" s="28"/>
-      <x:c r="G17" s="28"/>
-      <x:c r="H17" s="28"/>
-      <x:c r="I17" s="28"/>
-      <x:c r="J17" s="32" t="n">
+      <x:c r="B17" s="30"/>
+      <x:c r="C17" s="30"/>
+      <x:c r="D17" s="30"/>
+      <x:c r="E17" s="30"/>
+      <x:c r="F17" s="30"/>
+      <x:c r="G17" s="30"/>
+      <x:c r="H17" s="30"/>
+      <x:c r="I17" s="30"/>
+      <x:c r="J17" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
         <x:v>57</x:v>
       </x:c>
-      <x:c r="K17" s="28"/>
+      <x:c r="K17" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5807,42 +6029,42 @@
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="29" t="str">
+      <x:c r="A16" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B16" s="28" t="n">
+      <x:c r="B16" s="30" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C16" s="28"/>
-      <x:c r="D16" s="28"/>
-      <x:c r="E16" s="28"/>
-      <x:c r="F16" s="28"/>
-      <x:c r="G16" s="28"/>
-      <x:c r="H16" s="28"/>
-      <x:c r="I16" s="28"/>
-      <x:c r="J16" s="30" t="n">
+      <x:c r="C16" s="30"/>
+      <x:c r="D16" s="30"/>
+      <x:c r="E16" s="30"/>
+      <x:c r="F16" s="30"/>
+      <x:c r="G16" s="30"/>
+      <x:c r="H16" s="30"/>
+      <x:c r="I16" s="30"/>
+      <x:c r="J16" s="32" t="n">
         <x:f>SUM(J4:J13)</x:f>
         <x:v>328.8</x:v>
       </x:c>
-      <x:c r="K16" s="28"/>
+      <x:c r="K16" s="30"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="29" t="str">
+      <x:c r="A17" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B17" s="28"/>
-      <x:c r="C17" s="28"/>
-      <x:c r="D17" s="28"/>
-      <x:c r="E17" s="28"/>
-      <x:c r="F17" s="28"/>
-      <x:c r="G17" s="28"/>
-      <x:c r="H17" s="28"/>
-      <x:c r="I17" s="28"/>
-      <x:c r="J17" s="32" t="n">
+      <x:c r="B17" s="30"/>
+      <x:c r="C17" s="30"/>
+      <x:c r="D17" s="30"/>
+      <x:c r="E17" s="30"/>
+      <x:c r="F17" s="30"/>
+      <x:c r="G17" s="30"/>
+      <x:c r="H17" s="30"/>
+      <x:c r="I17" s="30"/>
+      <x:c r="J17" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
         <x:v>32.9</x:v>
       </x:c>
-      <x:c r="K17" s="28"/>
+      <x:c r="K17" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-08-18
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R3aa4d78a21ef46fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R17b625d48af94cb3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R68c7ee0974544ef3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rf0c89dbb064d45b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R7d69b028550a4f39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R8a7589935f034123"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R8f8caecfd4ba4b1a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R9950f2828eb94ac3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rc27f73596f4543e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="Rfcd21540b53e4323"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Re2f15c6de7a94162"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R2fa9e9c3ad3a4457"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Ra20c5a69122c4aa2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R14685a50f5954261"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R52b55768cc5644cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R5463e55e7bb74a93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R4642f1f217db45c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R8466b126876b46b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R838d94a1107d4fc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="Rd28a79bac6e74ee5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -485,25 +485,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-08-17</x:v>
+        <x:v>2026-08-18</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7968.38</x:v>
+        <x:v>7995.5</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7750.43</x:v>
+        <x:v>7842.25</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>217.9</x:v>
+        <x:v>153.3</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>1786.3</x:v>
+        <x:v>1939.6</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>162.4</x:v>
+        <x:v>161.6</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -514,25 +514,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-08-17</x:v>
+        <x:v>2026-08-18</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>8184.64</x:v>
+        <x:v>8211.31</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7992.36</x:v>
+        <x:v>8069.82</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>192.3</x:v>
+        <x:v>141.5</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>1772.5</x:v>
+        <x:v>1914</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>161.1</x:v>
+        <x:v>159.5</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -543,25 +543,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-08-17</x:v>
+        <x:v>2026-08-18</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3983.51</x:v>
+        <x:v>3994.18</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3924.47</x:v>
+        <x:v>3955.6</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>59</x:v>
+        <x:v>38.6</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>444.4</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>40.4</x:v>
+        <x:v>40.3</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -601,25 +601,25 @@
         <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>2026-08-17</x:v>
+        <x:v>2026-08-18</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:v>8086</x:v>
+        <x:v>8091.8</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>7869</x:v>
+        <x:v>7932.4</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>217</x:v>
+        <x:v>159.4</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>1790</x:v>
+        <x:v>1949.4</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
-        <x:v>162.7</x:v>
+        <x:v>162.5</x:v>
       </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
@@ -688,25 +688,25 @@
         <x:v>碳酸锂2609</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>2026-08-17</x:v>
+        <x:v>2026-08-18</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:v>155220</x:v>
+        <x:v>155980</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
-        <x:v>150520</x:v>
+        <x:v>151520</x:v>
       </x:c>
       <x:c r="E11" s="12" t="n">
-        <x:v>4700</x:v>
+        <x:v>4460</x:v>
       </x:c>
       <x:c r="F11" s="9" t="n">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G11" s="10" t="n">
-        <x:v>55040</x:v>
+        <x:v>59500</x:v>
       </x:c>
       <x:c r="H11" s="10" t="n">
-        <x:v>5003.6</x:v>
+        <x:v>4958.3</x:v>
       </x:c>
       <x:c r="I11" s="10" t="n">
         <x:v>6000</x:v>
@@ -720,7 +720,7 @@
         <x:v>2026-08-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-08-17</x:v>
+        <x:v>2026-08-18</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1299,31 +1299,49 @@
         <x:v>LC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B17" s="30" t="n">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="C17" s="30"/>
-      <x:c r="D17" s="30"/>
-      <x:c r="E17" s="30"/>
-      <x:c r="F17" s="30"/>
-      <x:c r="G17" s="30"/>
-      <x:c r="H17" s="30"/>
-      <x:c r="I17" s="30"/>
-      <x:c r="J17" s="32" t="n">
-        <x:f>SUM(J4:J14)</x:f>
-        <x:v>55040</x:v>
-      </x:c>
-      <x:c r="K17" s="30"/>
+    <x:row r="15">
+      <x:c r="A15" s="22" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B15" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C15" s="22" t="str">
+        <x:v>8月18日</x:v>
+      </x:c>
+      <x:c r="D15" s="23" t="n">
+        <x:v>153500</x:v>
+      </x:c>
+      <x:c r="E15" s="23" t="n">
+        <x:v>155980</x:v>
+      </x:c>
+      <x:c r="F15" s="23" t="n">
+        <x:v>151520</x:v>
+      </x:c>
+      <x:c r="G15" s="23" t="n">
+        <x:v>153940</x:v>
+      </x:c>
+      <x:c r="H15" s="28" t="n">
+        <x:v>1080</x:v>
+      </x:c>
+      <x:c r="I15" s="24" t="n">
+        <x:v>0.007065288499280342</x:v>
+      </x:c>
+      <x:c r="J15" s="23" t="n">
+        <x:f>ROUND(E15-F15,1)</x:f>
+        <x:v>4460</x:v>
+      </x:c>
+      <x:c r="K15" s="22" t="str">
+        <x:v>LC2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B18" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B18" s="30" t="n">
+        <x:v>12</x:v>
+      </x:c>
       <x:c r="C18" s="30"/>
       <x:c r="D18" s="30"/>
       <x:c r="E18" s="30"/>
@@ -1331,11 +1349,29 @@
       <x:c r="G18" s="30"/>
       <x:c r="H18" s="30"/>
       <x:c r="I18" s="30"/>
-      <x:c r="J18" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J14),0),1)</x:f>
-        <x:v>5003.6</x:v>
+      <x:c r="J18" s="32" t="n">
+        <x:f>SUM(J4:J15)</x:f>
+        <x:v>59500</x:v>
       </x:c>
       <x:c r="K18" s="30"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B19" s="30"/>
+      <x:c r="C19" s="30"/>
+      <x:c r="D19" s="30"/>
+      <x:c r="E19" s="30"/>
+      <x:c r="F19" s="30"/>
+      <x:c r="G19" s="30"/>
+      <x:c r="H19" s="30"/>
+      <x:c r="I19" s="30"/>
+      <x:c r="J19" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
+        <x:v>4958.3</x:v>
+      </x:c>
+      <x:c r="K19" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1492,37 +1528,37 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B7" s="22" t="str">
-        <x:v>8月17日</x:v>
+        <x:v>8月17日-8月18日</x:v>
       </x:c>
       <x:c r="C7" s="23" t="n">
         <x:v>7797.18</x:v>
       </x:c>
       <x:c r="D7" s="23" t="n">
-        <x:v>7968.38</x:v>
+        <x:v>7995.5</x:v>
       </x:c>
       <x:c r="E7" s="23" t="n">
         <x:v>7750.43</x:v>
       </x:c>
       <x:c r="F7" s="23" t="n">
-        <x:v>7968.38</x:v>
+        <x:v>7945.96</x:v>
       </x:c>
       <x:c r="G7" s="28" t="n">
         <x:f>ROUND(F7-F6,1)</x:f>
-        <x:v>198.6</x:v>
+        <x:v>176.1</x:v>
       </x:c>
       <x:c r="H7" s="24" t="n">
         <x:f>IFERROR(F7/F6-1,"")</x:f>
-        <x:v>0.02555528956912778</x:v>
+        <x:v>0.022669765837561195</x:v>
       </x:c>
       <x:c r="I7" s="26" t="n">
         <x:f>ROUND(D7-E7,1)</x:f>
-        <x:v>217.9</x:v>
+        <x:v>245.1</x:v>
       </x:c>
       <x:c r="J7" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K7" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -1540,7 +1576,7 @@
       <x:c r="H8" s="30"/>
       <x:c r="I8" s="32" t="n">
         <x:f>ROUND(SUM(I5:I7),1)</x:f>
-        <x:v>1119.2</x:v>
+        <x:v>1146.4</x:v>
       </x:c>
       <x:c r="J8" s="30"/>
       <x:c r="K8" s="30"/>
@@ -1558,7 +1594,7 @@
       <x:c r="H9" s="30"/>
       <x:c r="I9" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I7),0),1)</x:f>
-        <x:v>373.1</x:v>
+        <x:v>382.1</x:v>
       </x:c>
       <x:c r="J9" s="30"/>
       <x:c r="K9" s="30"/>
@@ -1688,37 +1724,37 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B15" s="22" t="str">
-        <x:v>8月17日</x:v>
+        <x:v>8月17日-8月18日</x:v>
       </x:c>
       <x:c r="C15" s="23" t="n">
         <x:v>8007.87</x:v>
       </x:c>
       <x:c r="D15" s="23" t="n">
-        <x:v>8184.64</x:v>
+        <x:v>8211.31</x:v>
       </x:c>
       <x:c r="E15" s="23" t="n">
         <x:v>7992.36</x:v>
       </x:c>
       <x:c r="F15" s="23" t="n">
-        <x:v>8184.64</x:v>
+        <x:v>8177.18</x:v>
       </x:c>
       <x:c r="G15" s="28" t="n">
         <x:f>ROUND(F15-F14,1)</x:f>
-        <x:v>194.3</x:v>
+        <x:v>186.9</x:v>
       </x:c>
       <x:c r="H15" s="24" t="n">
         <x:f>IFERROR(F15/F14-1,"")</x:f>
-        <x:v>0.02431814455723358</x:v>
+        <x:v>0.023384516033755798</x:v>
       </x:c>
       <x:c r="I15" s="26" t="n">
         <x:f>ROUND(D15-E15,1)</x:f>
-        <x:v>192.3</x:v>
+        <x:v>218.9</x:v>
       </x:c>
       <x:c r="J15" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K15" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1736,7 +1772,7 @@
       <x:c r="H16" s="30"/>
       <x:c r="I16" s="32" t="n">
         <x:f>ROUND(SUM(I13:I15),1)</x:f>
-        <x:v>1022.6</x:v>
+        <x:v>1049.2</x:v>
       </x:c>
       <x:c r="J16" s="30"/>
       <x:c r="K16" s="30"/>
@@ -1754,7 +1790,7 @@
       <x:c r="H17" s="30"/>
       <x:c r="I17" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I13:I15),0),1)</x:f>
-        <x:v>340.9</x:v>
+        <x:v>349.7</x:v>
       </x:c>
       <x:c r="J17" s="30"/>
       <x:c r="K17" s="30"/>
@@ -1884,37 +1920,37 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B23" s="22" t="str">
-        <x:v>8月17日</x:v>
+        <x:v>8月17日-8月18日</x:v>
       </x:c>
       <x:c r="C23" s="23" t="n">
         <x:v>3930.1</x:v>
       </x:c>
       <x:c r="D23" s="23" t="n">
-        <x:v>3983.51</x:v>
+        <x:v>3994.18</x:v>
       </x:c>
       <x:c r="E23" s="23" t="n">
         <x:v>3924.47</x:v>
       </x:c>
       <x:c r="F23" s="23" t="n">
-        <x:v>3982.65</x:v>
+        <x:v>3990.3</x:v>
       </x:c>
       <x:c r="G23" s="23" t="n">
         <x:f>ROUND(F23-F22,1)</x:f>
-        <x:v>55.5</x:v>
+        <x:v>63.1</x:v>
       </x:c>
       <x:c r="H23" s="24" t="n">
         <x:f>IFERROR(F23/F22-1,"")</x:f>
-        <x:v>0.014124639053977761</x:v>
+        <x:v>0.016072601714207213</x:v>
       </x:c>
       <x:c r="I23" s="26" t="n">
         <x:f>ROUND(D23-E23,1)</x:f>
-        <x:v>59</x:v>
+        <x:v>69.7</x:v>
       </x:c>
       <x:c r="J23" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K23" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1932,7 +1968,7 @@
       <x:c r="H24" s="30"/>
       <x:c r="I24" s="32" t="n">
         <x:f>ROUND(SUM(I21:I23),1)</x:f>
-        <x:v>267.1</x:v>
+        <x:v>277.8</x:v>
       </x:c>
       <x:c r="J24" s="30"/>
       <x:c r="K24" s="30"/>
@@ -1950,7 +1986,7 @@
       <x:c r="H25" s="30"/>
       <x:c r="I25" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I21:I23),0),1)</x:f>
-        <x:v>89</x:v>
+        <x:v>92.6</x:v>
       </x:c>
       <x:c r="J25" s="30"/>
       <x:c r="K25" s="30"/>
@@ -2276,37 +2312,37 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B39" s="22" t="str">
-        <x:v>8月17日</x:v>
+        <x:v>8月17日-8月18日</x:v>
       </x:c>
       <x:c r="C39" s="23" t="n">
         <x:v>7885</x:v>
       </x:c>
       <x:c r="D39" s="23" t="n">
-        <x:v>8086</x:v>
+        <x:v>8091.8</x:v>
       </x:c>
       <x:c r="E39" s="23" t="n">
         <x:v>7869</x:v>
       </x:c>
       <x:c r="F39" s="23" t="n">
-        <x:v>8082</x:v>
+        <x:v>8022.6</x:v>
       </x:c>
       <x:c r="G39" s="28" t="n">
         <x:f>ROUND(F39-F38,1)</x:f>
-        <x:v>220.8</x:v>
+        <x:v>161.4</x:v>
       </x:c>
       <x:c r="H39" s="24" t="n">
         <x:f>IFERROR(F39/F38-1,"")</x:f>
-        <x:v>0.028087314913753714</x:v>
+        <x:v>0.020531216608151492</x:v>
       </x:c>
       <x:c r="I39" s="26" t="n">
         <x:f>ROUND(D39-E39,1)</x:f>
-        <x:v>217</x:v>
+        <x:v>222.8</x:v>
       </x:c>
       <x:c r="J39" s="22" t="str">
         <x:v>IC2609</x:v>
       </x:c>
       <x:c r="K39" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -2324,7 +2360,7 @@
       <x:c r="H40" s="30"/>
       <x:c r="I40" s="32" t="n">
         <x:f>ROUND(SUM(I37:I39),1)</x:f>
-        <x:v>992.8</x:v>
+        <x:v>998.6</x:v>
       </x:c>
       <x:c r="J40" s="30"/>
       <x:c r="K40" s="30"/>
@@ -2342,7 +2378,7 @@
       <x:c r="H41" s="30"/>
       <x:c r="I41" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I37:I39),0),1)</x:f>
-        <x:v>330.9</x:v>
+        <x:v>332.9</x:v>
       </x:c>
       <x:c r="J41" s="30"/>
       <x:c r="K41" s="30"/>
@@ -2864,37 +2900,37 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B63" s="22" t="str">
-        <x:v>8月17日</x:v>
+        <x:v>8月17日-8月18日</x:v>
       </x:c>
       <x:c r="C63" s="23" t="n">
         <x:v>154300</x:v>
       </x:c>
       <x:c r="D63" s="23" t="n">
-        <x:v>155220</x:v>
+        <x:v>155980</x:v>
       </x:c>
       <x:c r="E63" s="23" t="n">
         <x:v>150520</x:v>
       </x:c>
       <x:c r="F63" s="23" t="n">
-        <x:v>152860</x:v>
-      </x:c>
-      <x:c r="G63" s="28" t="n">
+        <x:v>153940</x:v>
+      </x:c>
+      <x:c r="G63" s="23" t="n">
         <x:f>ROUND(F63-F62,1)</x:f>
-        <x:v>-1080</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H63" s="24" t="n">
         <x:f>IFERROR(F63/F62-1,"")</x:f>
-        <x:v>-0.007015720410549542</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I63" s="23" t="n">
         <x:f>ROUND(D63-E63,1)</x:f>
-        <x:v>4700</x:v>
+        <x:v>5460</x:v>
       </x:c>
       <x:c r="J63" s="22" t="str">
         <x:v>LC2609</x:v>
       </x:c>
       <x:c r="K63" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
@@ -2912,7 +2948,7 @@
       <x:c r="H64" s="30"/>
       <x:c r="I64" s="32" t="n">
         <x:f>ROUND(SUM(I61:I63),1)</x:f>
-        <x:v>29160</x:v>
+        <x:v>29920</x:v>
       </x:c>
       <x:c r="J64" s="30"/>
       <x:c r="K64" s="30"/>
@@ -2930,7 +2966,7 @@
       <x:c r="H65" s="30"/>
       <x:c r="I65" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I61:I63),0),1)</x:f>
-        <x:v>9720</x:v>
+        <x:v>9973.3</x:v>
       </x:c>
       <x:c r="J65" s="30"/>
       <x:c r="K65" s="30"/>
@@ -3404,31 +3440,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B17" s="30" t="n">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="C17" s="30"/>
-      <x:c r="D17" s="30"/>
-      <x:c r="E17" s="30"/>
-      <x:c r="F17" s="30"/>
-      <x:c r="G17" s="30"/>
-      <x:c r="H17" s="30"/>
-      <x:c r="I17" s="30"/>
-      <x:c r="J17" s="32" t="n">
-        <x:f>SUM(J4:J14)</x:f>
-        <x:v>1786.3000000000002</x:v>
-      </x:c>
-      <x:c r="K17" s="30"/>
+    <x:row r="15">
+      <x:c r="A15" s="22" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B15" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C15" s="22" t="str">
+        <x:v>8月18日</x:v>
+      </x:c>
+      <x:c r="D15" s="23" t="n">
+        <x:v>7969.37</x:v>
+      </x:c>
+      <x:c r="E15" s="23" t="n">
+        <x:v>7995.5</x:v>
+      </x:c>
+      <x:c r="F15" s="23" t="n">
+        <x:v>7842.25</x:v>
+      </x:c>
+      <x:c r="G15" s="23" t="n">
+        <x:v>7945.96</x:v>
+      </x:c>
+      <x:c r="H15" s="23" t="n">
+        <x:v>-22.4</x:v>
+      </x:c>
+      <x:c r="I15" s="24" t="n">
+        <x:v>-0.0028136208363557236</x:v>
+      </x:c>
+      <x:c r="J15" s="23" t="n">
+        <x:f>ROUND(E15-F15,1)</x:f>
+        <x:v>153.3</x:v>
+      </x:c>
+      <x:c r="K15" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B18" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B18" s="30" t="n">
+        <x:v>12</x:v>
+      </x:c>
       <x:c r="C18" s="30"/>
       <x:c r="D18" s="30"/>
       <x:c r="E18" s="30"/>
@@ -3436,11 +3490,29 @@
       <x:c r="G18" s="30"/>
       <x:c r="H18" s="30"/>
       <x:c r="I18" s="30"/>
-      <x:c r="J18" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J14),0),1)</x:f>
-        <x:v>162.4</x:v>
+      <x:c r="J18" s="32" t="n">
+        <x:f>SUM(J4:J15)</x:f>
+        <x:v>1939.6000000000001</x:v>
       </x:c>
       <x:c r="K18" s="30"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B19" s="30"/>
+      <x:c r="C19" s="30"/>
+      <x:c r="D19" s="30"/>
+      <x:c r="E19" s="30"/>
+      <x:c r="F19" s="30"/>
+      <x:c r="G19" s="30"/>
+      <x:c r="H19" s="30"/>
+      <x:c r="I19" s="30"/>
+      <x:c r="J19" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
+        <x:v>161.6</x:v>
+      </x:c>
+      <x:c r="K19" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3903,31 +3975,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B17" s="30" t="n">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="C17" s="30"/>
-      <x:c r="D17" s="30"/>
-      <x:c r="E17" s="30"/>
-      <x:c r="F17" s="30"/>
-      <x:c r="G17" s="30"/>
-      <x:c r="H17" s="30"/>
-      <x:c r="I17" s="30"/>
-      <x:c r="J17" s="32" t="n">
-        <x:f>SUM(J4:J14)</x:f>
-        <x:v>1772.5000000000002</x:v>
-      </x:c>
-      <x:c r="K17" s="30"/>
+    <x:row r="15">
+      <x:c r="A15" s="22" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B15" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C15" s="22" t="str">
+        <x:v>8月18日</x:v>
+      </x:c>
+      <x:c r="D15" s="23" t="n">
+        <x:v>8178.84</x:v>
+      </x:c>
+      <x:c r="E15" s="23" t="n">
+        <x:v>8211.31</x:v>
+      </x:c>
+      <x:c r="F15" s="23" t="n">
+        <x:v>8069.82</x:v>
+      </x:c>
+      <x:c r="G15" s="23" t="n">
+        <x:v>8177.18</x:v>
+      </x:c>
+      <x:c r="H15" s="23" t="n">
+        <x:v>-7.5</x:v>
+      </x:c>
+      <x:c r="I15" s="24" t="n">
+        <x:v>-0.0009114634241701447</x:v>
+      </x:c>
+      <x:c r="J15" s="23" t="n">
+        <x:f>ROUND(E15-F15,1)</x:f>
+        <x:v>141.5</x:v>
+      </x:c>
+      <x:c r="K15" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B18" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B18" s="30" t="n">
+        <x:v>12</x:v>
+      </x:c>
       <x:c r="C18" s="30"/>
       <x:c r="D18" s="30"/>
       <x:c r="E18" s="30"/>
@@ -3935,11 +4025,29 @@
       <x:c r="G18" s="30"/>
       <x:c r="H18" s="30"/>
       <x:c r="I18" s="30"/>
-      <x:c r="J18" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J14),0),1)</x:f>
-        <x:v>161.1</x:v>
+      <x:c r="J18" s="32" t="n">
+        <x:f>SUM(J4:J15)</x:f>
+        <x:v>1914.0000000000002</x:v>
       </x:c>
       <x:c r="K18" s="30"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B19" s="30"/>
+      <x:c r="C19" s="30"/>
+      <x:c r="D19" s="30"/>
+      <x:c r="E19" s="30"/>
+      <x:c r="F19" s="30"/>
+      <x:c r="G19" s="30"/>
+      <x:c r="H19" s="30"/>
+      <x:c r="I19" s="30"/>
+      <x:c r="J19" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
+        <x:v>159.5</x:v>
+      </x:c>
+      <x:c r="K19" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4402,31 +4510,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B17" s="30" t="n">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="C17" s="30"/>
-      <x:c r="D17" s="30"/>
-      <x:c r="E17" s="30"/>
-      <x:c r="F17" s="30"/>
-      <x:c r="G17" s="30"/>
-      <x:c r="H17" s="30"/>
-      <x:c r="I17" s="30"/>
-      <x:c r="J17" s="32" t="n">
-        <x:f>SUM(J4:J14)</x:f>
-        <x:v>444.40000000000003</x:v>
-      </x:c>
-      <x:c r="K17" s="30"/>
+    <x:row r="15">
+      <x:c r="A15" s="22" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B15" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C15" s="22" t="str">
+        <x:v>8月18日</x:v>
+      </x:c>
+      <x:c r="D15" s="23" t="n">
+        <x:v>3979.49</x:v>
+      </x:c>
+      <x:c r="E15" s="23" t="n">
+        <x:v>3994.18</x:v>
+      </x:c>
+      <x:c r="F15" s="23" t="n">
+        <x:v>3955.6</x:v>
+      </x:c>
+      <x:c r="G15" s="23" t="n">
+        <x:v>3990.3</x:v>
+      </x:c>
+      <x:c r="H15" s="23" t="n">
+        <x:v>7.7</x:v>
+      </x:c>
+      <x:c r="I15" s="24" t="n">
+        <x:v>0.0019208316070957743</x:v>
+      </x:c>
+      <x:c r="J15" s="23" t="n">
+        <x:f>ROUND(E15-F15,1)</x:f>
+        <x:v>38.6</x:v>
+      </x:c>
+      <x:c r="K15" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B18" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B18" s="30" t="n">
+        <x:v>12</x:v>
+      </x:c>
       <x:c r="C18" s="30"/>
       <x:c r="D18" s="30"/>
       <x:c r="E18" s="30"/>
@@ -4434,11 +4560,29 @@
       <x:c r="G18" s="30"/>
       <x:c r="H18" s="30"/>
       <x:c r="I18" s="30"/>
-      <x:c r="J18" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J14),0),1)</x:f>
-        <x:v>40.4</x:v>
+      <x:c r="J18" s="32" t="n">
+        <x:f>SUM(J4:J15)</x:f>
+        <x:v>483.00000000000006</x:v>
       </x:c>
       <x:c r="K18" s="30"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B19" s="30"/>
+      <x:c r="C19" s="30"/>
+      <x:c r="D19" s="30"/>
+      <x:c r="E19" s="30"/>
+      <x:c r="F19" s="30"/>
+      <x:c r="G19" s="30"/>
+      <x:c r="H19" s="30"/>
+      <x:c r="I19" s="30"/>
+      <x:c r="J19" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
+        <x:v>40.3</x:v>
+      </x:c>
+      <x:c r="K19" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5400,31 +5544,49 @@
         <x:v>IC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B17" s="30" t="n">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="C17" s="30"/>
-      <x:c r="D17" s="30"/>
-      <x:c r="E17" s="30"/>
-      <x:c r="F17" s="30"/>
-      <x:c r="G17" s="30"/>
-      <x:c r="H17" s="30"/>
-      <x:c r="I17" s="30"/>
-      <x:c r="J17" s="32" t="n">
-        <x:f>SUM(J4:J14)</x:f>
-        <x:v>1790</x:v>
-      </x:c>
-      <x:c r="K17" s="30"/>
+    <x:row r="15">
+      <x:c r="A15" s="22" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B15" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C15" s="22" t="str">
+        <x:v>8月18日</x:v>
+      </x:c>
+      <x:c r="D15" s="23" t="n">
+        <x:v>8078</x:v>
+      </x:c>
+      <x:c r="E15" s="23" t="n">
+        <x:v>8091.8</x:v>
+      </x:c>
+      <x:c r="F15" s="23" t="n">
+        <x:v>7932.4</x:v>
+      </x:c>
+      <x:c r="G15" s="23" t="n">
+        <x:v>8022.6</x:v>
+      </x:c>
+      <x:c r="H15" s="23" t="n">
+        <x:v>-59.4</x:v>
+      </x:c>
+      <x:c r="I15" s="24" t="n">
+        <x:v>-0.007349665924276105</x:v>
+      </x:c>
+      <x:c r="J15" s="26" t="n">
+        <x:f>ROUND(E15-F15,1)</x:f>
+        <x:v>159.4</x:v>
+      </x:c>
+      <x:c r="K15" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B18" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B18" s="30" t="n">
+        <x:v>12</x:v>
+      </x:c>
       <x:c r="C18" s="30"/>
       <x:c r="D18" s="30"/>
       <x:c r="E18" s="30"/>
@@ -5432,11 +5594,29 @@
       <x:c r="G18" s="30"/>
       <x:c r="H18" s="30"/>
       <x:c r="I18" s="30"/>
-      <x:c r="J18" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J14),0),1)</x:f>
-        <x:v>162.7</x:v>
+      <x:c r="J18" s="32" t="n">
+        <x:f>SUM(J4:J15)</x:f>
+        <x:v>1949.4</x:v>
       </x:c>
       <x:c r="K18" s="30"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B19" s="30"/>
+      <x:c r="C19" s="30"/>
+      <x:c r="D19" s="30"/>
+      <x:c r="E19" s="30"/>
+      <x:c r="F19" s="30"/>
+      <x:c r="G19" s="30"/>
+      <x:c r="H19" s="30"/>
+      <x:c r="I19" s="30"/>
+      <x:c r="J19" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
+        <x:v>162.5</x:v>
+      </x:c>
+      <x:c r="K19" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-08-19
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R396c411b4cd94c6e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R2c548669cbc84f7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Rdf3b68350f1846c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R295c863f0a574ffe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R4ecc195a387745ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R6196fcd87b084475"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Rfe856ec9b0814ad6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R6866db6e61974e95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R12330a02bb0f46a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R3f95fc804ee04d24"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R7f5eec1627ab40cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R0c38fb4191f24d70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R466a218776224151"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R072d8bedfb5e4dd7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R04fbc5f5eeb14965"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R2f4aabc4a289433e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R1d67f1acceab4a78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R46b9ce609681449d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rf6508b3f6a0b4a6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R349c41ef922e4780"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -485,25 +485,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-08-18</x:v>
+        <x:v>2026-08-19</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7995.5</x:v>
+        <x:v>7821.18</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7842.25</x:v>
+        <x:v>7490.21</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>153.3</x:v>
+        <x:v>331</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>1939.6</x:v>
+        <x:v>2270.6</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>161.6</x:v>
+        <x:v>174.7</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -514,25 +514,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-08-18</x:v>
+        <x:v>2026-08-19</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>8211.31</x:v>
+        <x:v>8050.08</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>8069.82</x:v>
+        <x:v>7762.29</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>141.5</x:v>
+        <x:v>287.8</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>1914</x:v>
+        <x:v>2201.8</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>159.5</x:v>
+        <x:v>169.4</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -543,25 +543,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-08-18</x:v>
+        <x:v>2026-08-19</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3994.18</x:v>
+        <x:v>3961.14</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3955.6</x:v>
+        <x:v>3879.58</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>38.6</x:v>
+        <x:v>81.6</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>483</x:v>
+        <x:v>564.6</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>40.3</x:v>
+        <x:v>43.4</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -572,25 +572,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-08-18</x:v>
+        <x:v>2026-08-19</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>7882.8</x:v>
+        <x:v>7734.6</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>7725</x:v>
+        <x:v>7430</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>157.8</x:v>
+        <x:v>304.6</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>1926.4</x:v>
+        <x:v>2231</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>160.5</x:v>
+        <x:v>171.6</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -630,25 +630,25 @@
         <x:v>IF主力</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>2026-08-18</x:v>
+        <x:v>2026-08-19</x:v>
       </x:c>
       <x:c r="C9" s="10" t="n">
-        <x:v>4698.2</x:v>
+        <x:v>4624.2</x:v>
       </x:c>
       <x:c r="D9" s="10" t="n">
-        <x:v>4633.2</x:v>
+        <x:v>4531.8</x:v>
       </x:c>
       <x:c r="E9" s="12" t="n">
-        <x:v>65</x:v>
+        <x:v>92.4</x:v>
       </x:c>
       <x:c r="F9" s="9" t="n">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G9" s="10" t="n">
-        <x:v>715.6</x:v>
+        <x:v>808</x:v>
       </x:c>
       <x:c r="H9" s="10" t="n">
-        <x:v>59.6</x:v>
+        <x:v>62.2</x:v>
       </x:c>
       <x:c r="I9" s="10" t="n">
         <x:v>90</x:v>
@@ -720,7 +720,7 @@
         <x:v>2026-08-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-08-18</x:v>
+        <x:v>2026-08-19</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1528,7 +1528,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B7" s="22" t="str">
-        <x:v>8月17日-8月18日</x:v>
+        <x:v>8月17日-8月19日</x:v>
       </x:c>
       <x:c r="C7" s="23" t="n">
         <x:v>7797.18</x:v>
@@ -1537,28 +1537,28 @@
         <x:v>7995.5</x:v>
       </x:c>
       <x:c r="E7" s="23" t="n">
-        <x:v>7750.43</x:v>
+        <x:v>7490.21</x:v>
       </x:c>
       <x:c r="F7" s="23" t="n">
-        <x:v>7945.96</x:v>
+        <x:v>7517.77</x:v>
       </x:c>
       <x:c r="G7" s="28" t="n">
         <x:f>ROUND(F7-F6,1)</x:f>
-        <x:v>176.1</x:v>
+        <x:v>-252</x:v>
       </x:c>
       <x:c r="H7" s="24" t="n">
         <x:f>IFERROR(F7/F6-1,"")</x:f>
-        <x:v>0.022669765837561195</x:v>
+        <x:v>-0.03243961893583114</x:v>
       </x:c>
       <x:c r="I7" s="26" t="n">
         <x:f>ROUND(D7-E7,1)</x:f>
-        <x:v>245.1</x:v>
+        <x:v>505.3</x:v>
       </x:c>
       <x:c r="J7" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K7" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -1576,7 +1576,7 @@
       <x:c r="H8" s="30"/>
       <x:c r="I8" s="32" t="n">
         <x:f>ROUND(SUM(I5:I7),1)</x:f>
-        <x:v>1146.4</x:v>
+        <x:v>1406.6</x:v>
       </x:c>
       <x:c r="J8" s="30"/>
       <x:c r="K8" s="30"/>
@@ -1594,7 +1594,7 @@
       <x:c r="H9" s="30"/>
       <x:c r="I9" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I7),0),1)</x:f>
-        <x:v>382.1</x:v>
+        <x:v>468.9</x:v>
       </x:c>
       <x:c r="J9" s="30"/>
       <x:c r="K9" s="30"/>
@@ -1724,7 +1724,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B15" s="22" t="str">
-        <x:v>8月17日-8月18日</x:v>
+        <x:v>8月17日-8月19日</x:v>
       </x:c>
       <x:c r="C15" s="23" t="n">
         <x:v>8007.87</x:v>
@@ -1733,28 +1733,28 @@
         <x:v>8211.31</x:v>
       </x:c>
       <x:c r="E15" s="23" t="n">
-        <x:v>7992.36</x:v>
+        <x:v>7762.29</x:v>
       </x:c>
       <x:c r="F15" s="23" t="n">
-        <x:v>8177.18</x:v>
+        <x:v>7783.46</x:v>
       </x:c>
       <x:c r="G15" s="28" t="n">
         <x:f>ROUND(F15-F14,1)</x:f>
-        <x:v>186.9</x:v>
+        <x:v>-206.9</x:v>
       </x:c>
       <x:c r="H15" s="24" t="n">
         <x:f>IFERROR(F15/F14-1,"")</x:f>
-        <x:v>0.023384516033755798</x:v>
+        <x:v>-0.025890044591399874</x:v>
       </x:c>
       <x:c r="I15" s="26" t="n">
         <x:f>ROUND(D15-E15,1)</x:f>
-        <x:v>218.9</x:v>
+        <x:v>449</x:v>
       </x:c>
       <x:c r="J15" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K15" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1772,7 +1772,7 @@
       <x:c r="H16" s="30"/>
       <x:c r="I16" s="32" t="n">
         <x:f>ROUND(SUM(I13:I15),1)</x:f>
-        <x:v>1049.2</x:v>
+        <x:v>1279.3</x:v>
       </x:c>
       <x:c r="J16" s="30"/>
       <x:c r="K16" s="30"/>
@@ -1790,7 +1790,7 @@
       <x:c r="H17" s="30"/>
       <x:c r="I17" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I13:I15),0),1)</x:f>
-        <x:v>349.7</x:v>
+        <x:v>426.4</x:v>
       </x:c>
       <x:c r="J17" s="30"/>
       <x:c r="K17" s="30"/>
@@ -1920,7 +1920,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B23" s="22" t="str">
-        <x:v>8月17日-8月18日</x:v>
+        <x:v>8月17日-8月19日</x:v>
       </x:c>
       <x:c r="C23" s="23" t="n">
         <x:v>3930.1</x:v>
@@ -1929,28 +1929,28 @@
         <x:v>3994.18</x:v>
       </x:c>
       <x:c r="E23" s="23" t="n">
-        <x:v>3924.47</x:v>
+        <x:v>3879.58</x:v>
       </x:c>
       <x:c r="F23" s="23" t="n">
-        <x:v>3990.3</x:v>
+        <x:v>3894.42</x:v>
       </x:c>
       <x:c r="G23" s="23" t="n">
         <x:f>ROUND(F23-F22,1)</x:f>
-        <x:v>63.1</x:v>
+        <x:v>-32.8</x:v>
       </x:c>
       <x:c r="H23" s="24" t="n">
         <x:f>IFERROR(F23/F22-1,"")</x:f>
-        <x:v>0.016072601714207213</x:v>
+        <x:v>-0.008341863627335577</x:v>
       </x:c>
       <x:c r="I23" s="26" t="n">
         <x:f>ROUND(D23-E23,1)</x:f>
-        <x:v>69.7</x:v>
+        <x:v>114.6</x:v>
       </x:c>
       <x:c r="J23" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K23" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1968,7 +1968,7 @@
       <x:c r="H24" s="30"/>
       <x:c r="I24" s="32" t="n">
         <x:f>ROUND(SUM(I21:I23),1)</x:f>
-        <x:v>277.8</x:v>
+        <x:v>322.7</x:v>
       </x:c>
       <x:c r="J24" s="30"/>
       <x:c r="K24" s="30"/>
@@ -1986,7 +1986,7 @@
       <x:c r="H25" s="30"/>
       <x:c r="I25" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I21:I23),0),1)</x:f>
-        <x:v>92.6</x:v>
+        <x:v>107.6</x:v>
       </x:c>
       <x:c r="J25" s="30"/>
       <x:c r="K25" s="30"/>
@@ -2116,7 +2116,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B31" s="22" t="str">
-        <x:v>8月17日-8月18日</x:v>
+        <x:v>8月17日-8月19日</x:v>
       </x:c>
       <x:c r="C31" s="23" t="n">
         <x:v>7675</x:v>
@@ -2125,28 +2125,28 @@
         <x:v>7882.8</x:v>
       </x:c>
       <x:c r="E31" s="23" t="n">
-        <x:v>7631.4</x:v>
+        <x:v>7430</x:v>
       </x:c>
       <x:c r="F31" s="23" t="n">
-        <x:v>7807</x:v>
+        <x:v>7468.8</x:v>
       </x:c>
       <x:c r="G31" s="28" t="n">
         <x:f>ROUND(F31-F30,1)</x:f>
-        <x:v>156.8</x:v>
+        <x:v>-181.4</x:v>
       </x:c>
       <x:c r="H31" s="24" t="n">
         <x:f>IFERROR(F31/F30-1,"")</x:f>
-        <x:v>0.02049619617787779</x:v>
+        <x:v>-0.023711798384355887</x:v>
       </x:c>
       <x:c r="I31" s="26" t="n">
         <x:f>ROUND(D31-E31,1)</x:f>
-        <x:v>251.4</x:v>
+        <x:v>452.8</x:v>
       </x:c>
       <x:c r="J31" s="22" t="str">
         <x:v>IM2609</x:v>
       </x:c>
       <x:c r="K31" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -2164,7 +2164,7 @@
       <x:c r="H32" s="30"/>
       <x:c r="I32" s="32" t="n">
         <x:f>ROUND(SUM(I29:I31),1)</x:f>
-        <x:v>1120.6</x:v>
+        <x:v>1322</x:v>
       </x:c>
       <x:c r="J32" s="30"/>
       <x:c r="K32" s="30"/>
@@ -2182,7 +2182,7 @@
       <x:c r="H33" s="30"/>
       <x:c r="I33" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I29:I31),0),1)</x:f>
-        <x:v>373.5</x:v>
+        <x:v>440.7</x:v>
       </x:c>
       <x:c r="J33" s="30"/>
       <x:c r="K33" s="30"/>
@@ -2508,7 +2508,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B47" s="22" t="str">
-        <x:v>8月17日-8月18日</x:v>
+        <x:v>8月17日-8月19日</x:v>
       </x:c>
       <x:c r="C47" s="23" t="n">
         <x:v>4624</x:v>
@@ -2517,28 +2517,28 @@
         <x:v>4700.6</x:v>
       </x:c>
       <x:c r="E47" s="23" t="n">
-        <x:v>4619.8</x:v>
+        <x:v>4531.8</x:v>
       </x:c>
       <x:c r="F47" s="23" t="n">
-        <x:v>4670.2</x:v>
+        <x:v>4554.2</x:v>
       </x:c>
       <x:c r="G47" s="23" t="n">
         <x:f>ROUND(F47-F46,1)</x:f>
-        <x:v>49.8</x:v>
+        <x:v>-66.2</x:v>
       </x:c>
       <x:c r="H47" s="24" t="n">
         <x:f>IFERROR(F47/F46-1,"")</x:f>
-        <x:v>0.010778287594147784</x:v>
-      </x:c>
-      <x:c r="I47" s="23" t="n">
+        <x:v>-0.014327763829971363</x:v>
+      </x:c>
+      <x:c r="I47" s="26" t="n">
         <x:f>ROUND(D47-E47,1)</x:f>
-        <x:v>80.8</x:v>
+        <x:v>168.8</x:v>
       </x:c>
       <x:c r="J47" s="22" t="str">
         <x:v>IF2609</x:v>
       </x:c>
       <x:c r="K47" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -2556,7 +2556,7 @@
       <x:c r="H48" s="30"/>
       <x:c r="I48" s="32" t="n">
         <x:f>ROUND(SUM(I45:I47),1)</x:f>
-        <x:v>325.8</x:v>
+        <x:v>413.8</x:v>
       </x:c>
       <x:c r="J48" s="30"/>
       <x:c r="K48" s="30"/>
@@ -2574,7 +2574,7 @@
       <x:c r="H49" s="30"/>
       <x:c r="I49" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I45:I47),0),1)</x:f>
-        <x:v>108.6</x:v>
+        <x:v>137.9</x:v>
       </x:c>
       <x:c r="J49" s="30"/>
       <x:c r="K49" s="30"/>
@@ -3476,31 +3476,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B18" s="30" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="C18" s="30"/>
-      <x:c r="D18" s="30"/>
-      <x:c r="E18" s="30"/>
-      <x:c r="F18" s="30"/>
-      <x:c r="G18" s="30"/>
-      <x:c r="H18" s="30"/>
-      <x:c r="I18" s="30"/>
-      <x:c r="J18" s="32" t="n">
-        <x:f>SUM(J4:J15)</x:f>
-        <x:v>1939.6000000000001</x:v>
-      </x:c>
-      <x:c r="K18" s="30"/>
+    <x:row r="16">
+      <x:c r="A16" s="22" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B16" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C16" s="22" t="str">
+        <x:v>8月19日</x:v>
+      </x:c>
+      <x:c r="D16" s="23" t="n">
+        <x:v>7795.26</x:v>
+      </x:c>
+      <x:c r="E16" s="23" t="n">
+        <x:v>7821.18</x:v>
+      </x:c>
+      <x:c r="F16" s="23" t="n">
+        <x:v>7490.21</x:v>
+      </x:c>
+      <x:c r="G16" s="23" t="n">
+        <x:v>7517.77</x:v>
+      </x:c>
+      <x:c r="H16" s="28" t="n">
+        <x:v>-428.2</x:v>
+      </x:c>
+      <x:c r="I16" s="24" t="n">
+        <x:v>-0.0538877618311695</x:v>
+      </x:c>
+      <x:c r="J16" s="26" t="n">
+        <x:f>ROUND(E16-F16,1)</x:f>
+        <x:v>331</x:v>
+      </x:c>
+      <x:c r="K16" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B19" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B19" s="30" t="n">
+        <x:v>13</x:v>
+      </x:c>
       <x:c r="C19" s="30"/>
       <x:c r="D19" s="30"/>
       <x:c r="E19" s="30"/>
@@ -3508,11 +3526,29 @@
       <x:c r="G19" s="30"/>
       <x:c r="H19" s="30"/>
       <x:c r="I19" s="30"/>
-      <x:c r="J19" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
-        <x:v>161.6</x:v>
+      <x:c r="J19" s="32" t="n">
+        <x:f>SUM(J4:J16)</x:f>
+        <x:v>2270.6000000000004</x:v>
       </x:c>
       <x:c r="K19" s="30"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B20" s="30"/>
+      <x:c r="C20" s="30"/>
+      <x:c r="D20" s="30"/>
+      <x:c r="E20" s="30"/>
+      <x:c r="F20" s="30"/>
+      <x:c r="G20" s="30"/>
+      <x:c r="H20" s="30"/>
+      <x:c r="I20" s="30"/>
+      <x:c r="J20" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
+        <x:v>174.7</x:v>
+      </x:c>
+      <x:c r="K20" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4011,31 +4047,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B18" s="30" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="C18" s="30"/>
-      <x:c r="D18" s="30"/>
-      <x:c r="E18" s="30"/>
-      <x:c r="F18" s="30"/>
-      <x:c r="G18" s="30"/>
-      <x:c r="H18" s="30"/>
-      <x:c r="I18" s="30"/>
-      <x:c r="J18" s="32" t="n">
-        <x:f>SUM(J4:J15)</x:f>
-        <x:v>1914.0000000000002</x:v>
-      </x:c>
-      <x:c r="K18" s="30"/>
+    <x:row r="16">
+      <x:c r="A16" s="22" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B16" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C16" s="22" t="str">
+        <x:v>8月19日</x:v>
+      </x:c>
+      <x:c r="D16" s="23" t="n">
+        <x:v>8029.52</x:v>
+      </x:c>
+      <x:c r="E16" s="23" t="n">
+        <x:v>8050.08</x:v>
+      </x:c>
+      <x:c r="F16" s="23" t="n">
+        <x:v>7762.29</x:v>
+      </x:c>
+      <x:c r="G16" s="23" t="n">
+        <x:v>7783.46</x:v>
+      </x:c>
+      <x:c r="H16" s="28" t="n">
+        <x:v>-393.7</x:v>
+      </x:c>
+      <x:c r="I16" s="24" t="n">
+        <x:v>-0.04814862825570676</x:v>
+      </x:c>
+      <x:c r="J16" s="26" t="n">
+        <x:f>ROUND(E16-F16,1)</x:f>
+        <x:v>287.8</x:v>
+      </x:c>
+      <x:c r="K16" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B19" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B19" s="30" t="n">
+        <x:v>13</x:v>
+      </x:c>
       <x:c r="C19" s="30"/>
       <x:c r="D19" s="30"/>
       <x:c r="E19" s="30"/>
@@ -4043,11 +4097,29 @@
       <x:c r="G19" s="30"/>
       <x:c r="H19" s="30"/>
       <x:c r="I19" s="30"/>
-      <x:c r="J19" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
-        <x:v>159.5</x:v>
+      <x:c r="J19" s="32" t="n">
+        <x:f>SUM(J4:J16)</x:f>
+        <x:v>2201.8</x:v>
       </x:c>
       <x:c r="K19" s="30"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B20" s="30"/>
+      <x:c r="C20" s="30"/>
+      <x:c r="D20" s="30"/>
+      <x:c r="E20" s="30"/>
+      <x:c r="F20" s="30"/>
+      <x:c r="G20" s="30"/>
+      <x:c r="H20" s="30"/>
+      <x:c r="I20" s="30"/>
+      <x:c r="J20" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
+        <x:v>169.4</x:v>
+      </x:c>
+      <x:c r="K20" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4546,31 +4618,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B18" s="30" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="C18" s="30"/>
-      <x:c r="D18" s="30"/>
-      <x:c r="E18" s="30"/>
-      <x:c r="F18" s="30"/>
-      <x:c r="G18" s="30"/>
-      <x:c r="H18" s="30"/>
-      <x:c r="I18" s="30"/>
-      <x:c r="J18" s="32" t="n">
-        <x:f>SUM(J4:J15)</x:f>
-        <x:v>483.00000000000006</x:v>
-      </x:c>
-      <x:c r="K18" s="30"/>
+    <x:row r="16">
+      <x:c r="A16" s="22" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B16" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C16" s="22" t="str">
+        <x:v>8月19日</x:v>
+      </x:c>
+      <x:c r="D16" s="23" t="n">
+        <x:v>3952.12</x:v>
+      </x:c>
+      <x:c r="E16" s="23" t="n">
+        <x:v>3961.14</x:v>
+      </x:c>
+      <x:c r="F16" s="23" t="n">
+        <x:v>3879.58</x:v>
+      </x:c>
+      <x:c r="G16" s="23" t="n">
+        <x:v>3894.42</x:v>
+      </x:c>
+      <x:c r="H16" s="23" t="n">
+        <x:v>-95.9</x:v>
+      </x:c>
+      <x:c r="I16" s="24" t="n">
+        <x:v>-0.024028268551236742</x:v>
+      </x:c>
+      <x:c r="J16" s="26" t="n">
+        <x:f>ROUND(E16-F16,1)</x:f>
+        <x:v>81.6</x:v>
+      </x:c>
+      <x:c r="K16" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B19" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B19" s="30" t="n">
+        <x:v>13</x:v>
+      </x:c>
       <x:c r="C19" s="30"/>
       <x:c r="D19" s="30"/>
       <x:c r="E19" s="30"/>
@@ -4578,11 +4668,29 @@
       <x:c r="G19" s="30"/>
       <x:c r="H19" s="30"/>
       <x:c r="I19" s="30"/>
-      <x:c r="J19" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
-        <x:v>40.3</x:v>
+      <x:c r="J19" s="32" t="n">
+        <x:f>SUM(J4:J16)</x:f>
+        <x:v>564.6</x:v>
       </x:c>
       <x:c r="K19" s="30"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B20" s="30"/>
+      <x:c r="C20" s="30"/>
+      <x:c r="D20" s="30"/>
+      <x:c r="E20" s="30"/>
+      <x:c r="F20" s="30"/>
+      <x:c r="G20" s="30"/>
+      <x:c r="H20" s="30"/>
+      <x:c r="I20" s="30"/>
+      <x:c r="J20" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
+        <x:v>43.4</x:v>
+      </x:c>
+      <x:c r="K20" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5081,31 +5189,49 @@
         <x:v>IM2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B18" s="30" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="C18" s="30"/>
-      <x:c r="D18" s="30"/>
-      <x:c r="E18" s="30"/>
-      <x:c r="F18" s="30"/>
-      <x:c r="G18" s="30"/>
-      <x:c r="H18" s="30"/>
-      <x:c r="I18" s="30"/>
-      <x:c r="J18" s="32" t="n">
-        <x:f>SUM(J4:J15)</x:f>
-        <x:v>1926.3999999999999</x:v>
-      </x:c>
-      <x:c r="K18" s="30"/>
+    <x:row r="16">
+      <x:c r="A16" s="22" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B16" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C16" s="22" t="str">
+        <x:v>8月19日</x:v>
+      </x:c>
+      <x:c r="D16" s="23" t="n">
+        <x:v>7711</x:v>
+      </x:c>
+      <x:c r="E16" s="23" t="n">
+        <x:v>7734.6</x:v>
+      </x:c>
+      <x:c r="F16" s="23" t="n">
+        <x:v>7430</x:v>
+      </x:c>
+      <x:c r="G16" s="23" t="n">
+        <x:v>7468.8</x:v>
+      </x:c>
+      <x:c r="H16" s="28" t="n">
+        <x:v>-338.2</x:v>
+      </x:c>
+      <x:c r="I16" s="24" t="n">
+        <x:v>-0.04332009734853337</x:v>
+      </x:c>
+      <x:c r="J16" s="26" t="n">
+        <x:f>ROUND(E16-F16,1)</x:f>
+        <x:v>304.6</x:v>
+      </x:c>
+      <x:c r="K16" s="22" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B19" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B19" s="30" t="n">
+        <x:v>13</x:v>
+      </x:c>
       <x:c r="C19" s="30"/>
       <x:c r="D19" s="30"/>
       <x:c r="E19" s="30"/>
@@ -5113,11 +5239,29 @@
       <x:c r="G19" s="30"/>
       <x:c r="H19" s="30"/>
       <x:c r="I19" s="30"/>
-      <x:c r="J19" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
-        <x:v>160.5</x:v>
+      <x:c r="J19" s="32" t="n">
+        <x:f>SUM(J4:J16)</x:f>
+        <x:v>2231</x:v>
       </x:c>
       <x:c r="K19" s="30"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B20" s="30"/>
+      <x:c r="C20" s="30"/>
+      <x:c r="D20" s="30"/>
+      <x:c r="E20" s="30"/>
+      <x:c r="F20" s="30"/>
+      <x:c r="G20" s="30"/>
+      <x:c r="H20" s="30"/>
+      <x:c r="I20" s="30"/>
+      <x:c r="J20" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
+        <x:v>171.6</x:v>
+      </x:c>
+      <x:c r="K20" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -6151,31 +6295,49 @@
         <x:v>IF2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B18" s="30" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="C18" s="30"/>
-      <x:c r="D18" s="30"/>
-      <x:c r="E18" s="30"/>
-      <x:c r="F18" s="30"/>
-      <x:c r="G18" s="30"/>
-      <x:c r="H18" s="30"/>
-      <x:c r="I18" s="30"/>
-      <x:c r="J18" s="32" t="n">
-        <x:f>SUM(J4:J15)</x:f>
-        <x:v>715.6</x:v>
-      </x:c>
-      <x:c r="K18" s="30"/>
+    <x:row r="16">
+      <x:c r="A16" s="22" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B16" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C16" s="22" t="str">
+        <x:v>8月19日</x:v>
+      </x:c>
+      <x:c r="D16" s="23" t="n">
+        <x:v>4605.2</x:v>
+      </x:c>
+      <x:c r="E16" s="23" t="n">
+        <x:v>4624.2</x:v>
+      </x:c>
+      <x:c r="F16" s="23" t="n">
+        <x:v>4531.8</x:v>
+      </x:c>
+      <x:c r="G16" s="23" t="n">
+        <x:v>4554.2</x:v>
+      </x:c>
+      <x:c r="H16" s="23" t="n">
+        <x:v>-116</x:v>
+      </x:c>
+      <x:c r="I16" s="24" t="n">
+        <x:v>-0.024838336687936224</x:v>
+      </x:c>
+      <x:c r="J16" s="26" t="n">
+        <x:f>ROUND(E16-F16,1)</x:f>
+        <x:v>92.4</x:v>
+      </x:c>
+      <x:c r="K16" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B19" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B19" s="30" t="n">
+        <x:v>13</x:v>
+      </x:c>
       <x:c r="C19" s="30"/>
       <x:c r="D19" s="30"/>
       <x:c r="E19" s="30"/>
@@ -6183,11 +6345,29 @@
       <x:c r="G19" s="30"/>
       <x:c r="H19" s="30"/>
       <x:c r="I19" s="30"/>
-      <x:c r="J19" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
-        <x:v>59.6</x:v>
+      <x:c r="J19" s="32" t="n">
+        <x:f>SUM(J4:J16)</x:f>
+        <x:v>808</x:v>
       </x:c>
       <x:c r="K19" s="30"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B20" s="30"/>
+      <x:c r="C20" s="30"/>
+      <x:c r="D20" s="30"/>
+      <x:c r="E20" s="30"/>
+      <x:c r="F20" s="30"/>
+      <x:c r="G20" s="30"/>
+      <x:c r="H20" s="30"/>
+      <x:c r="I20" s="30"/>
+      <x:c r="J20" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
+        <x:v>62.2</x:v>
+      </x:c>
+      <x:c r="K20" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-08-20
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rd418f97594d847bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Rfd7eed2e836244b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R4c4c92b8a77b4b88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Raba8b872eac4437b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R0c49162d4b5d4b61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R0aa4650891c741ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R7855e487bb374707"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R51da8536474f4dfd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rb5ae3d432e81416d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R01326f9ecd79413e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R4a5b12bc46554601"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R8d30350ffba349b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Rdbb833f7578b4100"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Red5998c2fdfb4abf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Rfb3ba3911ec048e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R207a5e7b00654af1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Rb656bc74e13943f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R15a291394f8f4ea6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Ra08391cdf3be40c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="Rfb9112c03ccd47e2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -485,25 +485,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-08-19</x:v>
+        <x:v>2026-08-20</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7821.18</x:v>
+        <x:v>7656.61</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7490.21</x:v>
+        <x:v>7541.48</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>331</x:v>
+        <x:v>115.1</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>2270.6</x:v>
+        <x:v>2385.7</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>174.7</x:v>
+        <x:v>170.4</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -514,25 +514,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-08-19</x:v>
+        <x:v>2026-08-20</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>8050.08</x:v>
+        <x:v>7923.91</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7762.29</x:v>
+        <x:v>7796.28</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>287.8</x:v>
+        <x:v>127.6</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>2201.8</x:v>
+        <x:v>2329.4</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>169.4</x:v>
+        <x:v>166.4</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -543,25 +543,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-08-19</x:v>
+        <x:v>2026-08-20</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3961.14</x:v>
+        <x:v>3925.06</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3879.58</x:v>
+        <x:v>3888.1</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>81.6</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>564.6</x:v>
+        <x:v>601.6</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>43.4</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -601,25 +601,25 @@
         <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>2026-08-19</x:v>
+        <x:v>2026-08-20</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:v>7939.8</x:v>
+        <x:v>7811</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>7680.2</x:v>
+        <x:v>7713</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>259.6</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>2209</x:v>
+        <x:v>2307</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
-        <x:v>169.9</x:v>
+        <x:v>164.8</x:v>
       </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
@@ -630,25 +630,25 @@
         <x:v>IF主力</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>2026-08-19</x:v>
+        <x:v>2026-08-20</x:v>
       </x:c>
       <x:c r="C9" s="10" t="n">
-        <x:v>4624.2</x:v>
+        <x:v>4585</x:v>
       </x:c>
       <x:c r="D9" s="10" t="n">
-        <x:v>4531.8</x:v>
+        <x:v>4532.4</x:v>
       </x:c>
       <x:c r="E9" s="12" t="n">
-        <x:v>92.4</x:v>
+        <x:v>52.6</x:v>
       </x:c>
       <x:c r="F9" s="9" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G9" s="10" t="n">
-        <x:v>808</x:v>
+        <x:v>860.6</x:v>
       </x:c>
       <x:c r="H9" s="10" t="n">
-        <x:v>62.2</x:v>
+        <x:v>61.5</x:v>
       </x:c>
       <x:c r="I9" s="10" t="n">
         <x:v>90</x:v>
@@ -688,25 +688,25 @@
         <x:v>碳酸锂2609</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>2026-08-19</x:v>
+        <x:v>2026-08-20</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:v>153220</x:v>
+        <x:v>152600</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
-        <x:v>148400</x:v>
+        <x:v>149800</x:v>
       </x:c>
       <x:c r="E11" s="12" t="n">
-        <x:v>4820</x:v>
+        <x:v>2800</x:v>
       </x:c>
       <x:c r="F11" s="9" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G11" s="10" t="n">
-        <x:v>64320</x:v>
+        <x:v>67120</x:v>
       </x:c>
       <x:c r="H11" s="10" t="n">
-        <x:v>4947.7</x:v>
+        <x:v>4794.3</x:v>
       </x:c>
       <x:c r="I11" s="10" t="n">
         <x:v>6000</x:v>
@@ -720,7 +720,7 @@
         <x:v>2026-08-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-08-19</x:v>
+        <x:v>2026-08-20</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1371,31 +1371,49 @@
         <x:v>LC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B19" s="30" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C19" s="30"/>
-      <x:c r="D19" s="30"/>
-      <x:c r="E19" s="30"/>
-      <x:c r="F19" s="30"/>
-      <x:c r="G19" s="30"/>
-      <x:c r="H19" s="30"/>
-      <x:c r="I19" s="30"/>
-      <x:c r="J19" s="32" t="n">
-        <x:f>SUM(J4:J16)</x:f>
-        <x:v>64320</x:v>
-      </x:c>
-      <x:c r="K19" s="30"/>
+    <x:row r="17">
+      <x:c r="A17" s="22" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B17" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C17" s="22" t="str">
+        <x:v>8月20日</x:v>
+      </x:c>
+      <x:c r="D17" s="23" t="n">
+        <x:v>150800</x:v>
+      </x:c>
+      <x:c r="E17" s="23" t="n">
+        <x:v>152600</x:v>
+      </x:c>
+      <x:c r="F17" s="23" t="n">
+        <x:v>149800</x:v>
+      </x:c>
+      <x:c r="G17" s="23" t="n">
+        <x:v>151500</x:v>
+      </x:c>
+      <x:c r="H17" s="28" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="I17" s="24" t="n">
+        <x:v>0.013513513513513598</x:v>
+      </x:c>
+      <x:c r="J17" s="23" t="n">
+        <x:f>ROUND(E17-F17,1)</x:f>
+        <x:v>2800</x:v>
+      </x:c>
+      <x:c r="K17" s="22" t="str">
+        <x:v>LC2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B20" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B20" s="30" t="n">
+        <x:v>14</x:v>
+      </x:c>
       <x:c r="C20" s="30"/>
       <x:c r="D20" s="30"/>
       <x:c r="E20" s="30"/>
@@ -1403,11 +1421,29 @@
       <x:c r="G20" s="30"/>
       <x:c r="H20" s="30"/>
       <x:c r="I20" s="30"/>
-      <x:c r="J20" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
-        <x:v>4947.7</x:v>
+      <x:c r="J20" s="32" t="n">
+        <x:f>SUM(J4:J17)</x:f>
+        <x:v>67120</x:v>
       </x:c>
       <x:c r="K20" s="30"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B21" s="30"/>
+      <x:c r="C21" s="30"/>
+      <x:c r="D21" s="30"/>
+      <x:c r="E21" s="30"/>
+      <x:c r="F21" s="30"/>
+      <x:c r="G21" s="30"/>
+      <x:c r="H21" s="30"/>
+      <x:c r="I21" s="30"/>
+      <x:c r="J21" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
+        <x:v>4794.3</x:v>
+      </x:c>
+      <x:c r="K21" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1564,7 +1600,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B7" s="22" t="str">
-        <x:v>8月17日-8月19日</x:v>
+        <x:v>8月17日-8月20日</x:v>
       </x:c>
       <x:c r="C7" s="23" t="n">
         <x:v>7797.18</x:v>
@@ -1576,15 +1612,15 @@
         <x:v>7490.21</x:v>
       </x:c>
       <x:c r="F7" s="23" t="n">
-        <x:v>7517.77</x:v>
+        <x:v>7589.78</x:v>
       </x:c>
       <x:c r="G7" s="28" t="n">
         <x:f>ROUND(F7-F6,1)</x:f>
-        <x:v>-252</x:v>
+        <x:v>-180</x:v>
       </x:c>
       <x:c r="H7" s="24" t="n">
         <x:f>IFERROR(F7/F6-1,"")</x:f>
-        <x:v>-0.03243961893583114</x:v>
+        <x:v>-0.023171707967494792</x:v>
       </x:c>
       <x:c r="I7" s="26" t="n">
         <x:f>ROUND(D7-E7,1)</x:f>
@@ -1594,7 +1630,7 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K7" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -1760,7 +1796,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B15" s="22" t="str">
-        <x:v>8月17日-8月19日</x:v>
+        <x:v>8月17日-8月20日</x:v>
       </x:c>
       <x:c r="C15" s="23" t="n">
         <x:v>8007.87</x:v>
@@ -1772,15 +1808,15 @@
         <x:v>7762.29</x:v>
       </x:c>
       <x:c r="F15" s="23" t="n">
-        <x:v>7783.46</x:v>
-      </x:c>
-      <x:c r="G15" s="28" t="n">
+        <x:v>7850.4</x:v>
+      </x:c>
+      <x:c r="G15" s="23" t="n">
         <x:f>ROUND(F15-F14,1)</x:f>
-        <x:v>-206.9</x:v>
+        <x:v>-139.9</x:v>
       </x:c>
       <x:c r="H15" s="24" t="n">
         <x:f>IFERROR(F15/F14-1,"")</x:f>
-        <x:v>-0.025890044591399874</x:v>
+        <x:v>-0.01751241813542126</x:v>
       </x:c>
       <x:c r="I15" s="26" t="n">
         <x:f>ROUND(D15-E15,1)</x:f>
@@ -1790,7 +1826,7 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K15" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1956,7 +1992,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B23" s="22" t="str">
-        <x:v>8月17日-8月19日</x:v>
+        <x:v>8月17日-8月20日</x:v>
       </x:c>
       <x:c r="C23" s="23" t="n">
         <x:v>3930.1</x:v>
@@ -1968,15 +2004,15 @@
         <x:v>3879.58</x:v>
       </x:c>
       <x:c r="F23" s="23" t="n">
-        <x:v>3894.42</x:v>
+        <x:v>3903.72</x:v>
       </x:c>
       <x:c r="G23" s="23" t="n">
         <x:f>ROUND(F23-F22,1)</x:f>
-        <x:v>-32.8</x:v>
+        <x:v>-23.5</x:v>
       </x:c>
       <x:c r="H23" s="24" t="n">
         <x:f>IFERROR(F23/F22-1,"")</x:f>
-        <x:v>-0.008341863627335577</x:v>
+        <x:v>-0.005973752158037082</x:v>
       </x:c>
       <x:c r="I23" s="26" t="n">
         <x:f>ROUND(D23-E23,1)</x:f>
@@ -1986,7 +2022,7 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K23" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -2348,7 +2384,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B39" s="22" t="str">
-        <x:v>8月17日-8月19日</x:v>
+        <x:v>8月17日-8月20日</x:v>
       </x:c>
       <x:c r="C39" s="23" t="n">
         <x:v>7885</x:v>
@@ -2360,15 +2396,15 @@
         <x:v>7680.2</x:v>
       </x:c>
       <x:c r="F39" s="23" t="n">
-        <x:v>7712</x:v>
+        <x:v>7761</x:v>
       </x:c>
       <x:c r="G39" s="23" t="n">
         <x:f>ROUND(F39-F38,1)</x:f>
-        <x:v>-149.2</x:v>
+        <x:v>-100.2</x:v>
       </x:c>
       <x:c r="H39" s="24" t="n">
         <x:f>IFERROR(F39/F38-1,"")</x:f>
-        <x:v>-0.01897929069353277</x:v>
+        <x:v>-0.012746145626621908</x:v>
       </x:c>
       <x:c r="I39" s="26" t="n">
         <x:f>ROUND(D39-E39,1)</x:f>
@@ -2378,7 +2414,7 @@
         <x:v>IC2609</x:v>
       </x:c>
       <x:c r="K39" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -2544,7 +2580,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B47" s="22" t="str">
-        <x:v>8月17日-8月19日</x:v>
+        <x:v>8月17日-8月20日</x:v>
       </x:c>
       <x:c r="C47" s="23" t="n">
         <x:v>4624</x:v>
@@ -2556,15 +2592,15 @@
         <x:v>4531.8</x:v>
       </x:c>
       <x:c r="F47" s="23" t="n">
-        <x:v>4554.2</x:v>
+        <x:v>4554</x:v>
       </x:c>
       <x:c r="G47" s="23" t="n">
         <x:f>ROUND(F47-F46,1)</x:f>
-        <x:v>-66.2</x:v>
+        <x:v>-66.4</x:v>
       </x:c>
       <x:c r="H47" s="24" t="n">
         <x:f>IFERROR(F47/F46-1,"")</x:f>
-        <x:v>-0.014327763829971363</x:v>
+        <x:v>-0.014371050125530194</x:v>
       </x:c>
       <x:c r="I47" s="26" t="n">
         <x:f>ROUND(D47-E47,1)</x:f>
@@ -2574,7 +2610,7 @@
         <x:v>IF2609</x:v>
       </x:c>
       <x:c r="K47" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -2936,7 +2972,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B63" s="22" t="str">
-        <x:v>8月17日-8月19日</x:v>
+        <x:v>8月17日-8月20日</x:v>
       </x:c>
       <x:c r="C63" s="23" t="n">
         <x:v>154300</x:v>
@@ -2948,15 +2984,15 @@
         <x:v>148400</x:v>
       </x:c>
       <x:c r="F63" s="23" t="n">
-        <x:v>149480</x:v>
+        <x:v>151500</x:v>
       </x:c>
       <x:c r="G63" s="28" t="n">
         <x:f>ROUND(F63-F62,1)</x:f>
-        <x:v>-4460</x:v>
+        <x:v>-2440</x:v>
       </x:c>
       <x:c r="H63" s="24" t="n">
         <x:f>IFERROR(F63/F62-1,"")</x:f>
-        <x:v>-0.028972326880602806</x:v>
+        <x:v>-0.01585033129790825</x:v>
       </x:c>
       <x:c r="I63" s="26" t="n">
         <x:f>ROUND(D63-E63,1)</x:f>
@@ -2966,7 +3002,7 @@
         <x:v>LC2609</x:v>
       </x:c>
       <x:c r="K63" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
@@ -3548,31 +3584,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B19" s="30" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C19" s="30"/>
-      <x:c r="D19" s="30"/>
-      <x:c r="E19" s="30"/>
-      <x:c r="F19" s="30"/>
-      <x:c r="G19" s="30"/>
-      <x:c r="H19" s="30"/>
-      <x:c r="I19" s="30"/>
-      <x:c r="J19" s="32" t="n">
-        <x:f>SUM(J4:J16)</x:f>
-        <x:v>2270.6000000000004</x:v>
-      </x:c>
-      <x:c r="K19" s="30"/>
+    <x:row r="17">
+      <x:c r="A17" s="22" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B17" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C17" s="22" t="str">
+        <x:v>8月20日</x:v>
+      </x:c>
+      <x:c r="D17" s="23" t="n">
+        <x:v>7602.5</x:v>
+      </x:c>
+      <x:c r="E17" s="23" t="n">
+        <x:v>7656.61</x:v>
+      </x:c>
+      <x:c r="F17" s="23" t="n">
+        <x:v>7541.48</x:v>
+      </x:c>
+      <x:c r="G17" s="23" t="n">
+        <x:v>7589.78</x:v>
+      </x:c>
+      <x:c r="H17" s="23" t="n">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="I17" s="24" t="n">
+        <x:v>0.009578638346211532</x:v>
+      </x:c>
+      <x:c r="J17" s="23" t="n">
+        <x:f>ROUND(E17-F17,1)</x:f>
+        <x:v>115.1</x:v>
+      </x:c>
+      <x:c r="K17" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B20" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B20" s="30" t="n">
+        <x:v>14</x:v>
+      </x:c>
       <x:c r="C20" s="30"/>
       <x:c r="D20" s="30"/>
       <x:c r="E20" s="30"/>
@@ -3580,11 +3634,29 @@
       <x:c r="G20" s="30"/>
       <x:c r="H20" s="30"/>
       <x:c r="I20" s="30"/>
-      <x:c r="J20" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
-        <x:v>174.7</x:v>
+      <x:c r="J20" s="32" t="n">
+        <x:f>SUM(J4:J17)</x:f>
+        <x:v>2385.7000000000003</x:v>
       </x:c>
       <x:c r="K20" s="30"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B21" s="30"/>
+      <x:c r="C21" s="30"/>
+      <x:c r="D21" s="30"/>
+      <x:c r="E21" s="30"/>
+      <x:c r="F21" s="30"/>
+      <x:c r="G21" s="30"/>
+      <x:c r="H21" s="30"/>
+      <x:c r="I21" s="30"/>
+      <x:c r="J21" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
+        <x:v>170.4</x:v>
+      </x:c>
+      <x:c r="K21" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4119,31 +4191,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B19" s="30" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C19" s="30"/>
-      <x:c r="D19" s="30"/>
-      <x:c r="E19" s="30"/>
-      <x:c r="F19" s="30"/>
-      <x:c r="G19" s="30"/>
-      <x:c r="H19" s="30"/>
-      <x:c r="I19" s="30"/>
-      <x:c r="J19" s="32" t="n">
-        <x:f>SUM(J4:J16)</x:f>
-        <x:v>2201.8</x:v>
-      </x:c>
-      <x:c r="K19" s="30"/>
+    <x:row r="17">
+      <x:c r="A17" s="22" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B17" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C17" s="22" t="str">
+        <x:v>8月20日</x:v>
+      </x:c>
+      <x:c r="D17" s="23" t="n">
+        <x:v>7864.68</x:v>
+      </x:c>
+      <x:c r="E17" s="23" t="n">
+        <x:v>7923.91</x:v>
+      </x:c>
+      <x:c r="F17" s="23" t="n">
+        <x:v>7796.28</x:v>
+      </x:c>
+      <x:c r="G17" s="23" t="n">
+        <x:v>7850.4</x:v>
+      </x:c>
+      <x:c r="H17" s="23" t="n">
+        <x:v>66.9</x:v>
+      </x:c>
+      <x:c r="I17" s="24" t="n">
+        <x:v>0.008600288303659331</x:v>
+      </x:c>
+      <x:c r="J17" s="23" t="n">
+        <x:f>ROUND(E17-F17,1)</x:f>
+        <x:v>127.6</x:v>
+      </x:c>
+      <x:c r="K17" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B20" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B20" s="30" t="n">
+        <x:v>14</x:v>
+      </x:c>
       <x:c r="C20" s="30"/>
       <x:c r="D20" s="30"/>
       <x:c r="E20" s="30"/>
@@ -4151,11 +4241,29 @@
       <x:c r="G20" s="30"/>
       <x:c r="H20" s="30"/>
       <x:c r="I20" s="30"/>
-      <x:c r="J20" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
-        <x:v>169.4</x:v>
+      <x:c r="J20" s="32" t="n">
+        <x:f>SUM(J4:J17)</x:f>
+        <x:v>2329.4</x:v>
       </x:c>
       <x:c r="K20" s="30"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B21" s="30"/>
+      <x:c r="C21" s="30"/>
+      <x:c r="D21" s="30"/>
+      <x:c r="E21" s="30"/>
+      <x:c r="F21" s="30"/>
+      <x:c r="G21" s="30"/>
+      <x:c r="H21" s="30"/>
+      <x:c r="I21" s="30"/>
+      <x:c r="J21" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
+        <x:v>166.4</x:v>
+      </x:c>
+      <x:c r="K21" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4690,31 +4798,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B19" s="30" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C19" s="30"/>
-      <x:c r="D19" s="30"/>
-      <x:c r="E19" s="30"/>
-      <x:c r="F19" s="30"/>
-      <x:c r="G19" s="30"/>
-      <x:c r="H19" s="30"/>
-      <x:c r="I19" s="30"/>
-      <x:c r="J19" s="32" t="n">
-        <x:f>SUM(J4:J16)</x:f>
-        <x:v>564.6</x:v>
-      </x:c>
-      <x:c r="K19" s="30"/>
+    <x:row r="17">
+      <x:c r="A17" s="22" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B17" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C17" s="22" t="str">
+        <x:v>8月20日</x:v>
+      </x:c>
+      <x:c r="D17" s="23" t="n">
+        <x:v>3907.21</x:v>
+      </x:c>
+      <x:c r="E17" s="23" t="n">
+        <x:v>3925.06</x:v>
+      </x:c>
+      <x:c r="F17" s="23" t="n">
+        <x:v>3888.1</x:v>
+      </x:c>
+      <x:c r="G17" s="23" t="n">
+        <x:v>3903.72</x:v>
+      </x:c>
+      <x:c r="H17" s="23" t="n">
+        <x:v>9.3</x:v>
+      </x:c>
+      <x:c r="I17" s="24" t="n">
+        <x:v>0.002388032107476734</x:v>
+      </x:c>
+      <x:c r="J17" s="23" t="n">
+        <x:f>ROUND(E17-F17,1)</x:f>
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="K17" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B20" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B20" s="30" t="n">
+        <x:v>14</x:v>
+      </x:c>
       <x:c r="C20" s="30"/>
       <x:c r="D20" s="30"/>
       <x:c r="E20" s="30"/>
@@ -4722,11 +4848,29 @@
       <x:c r="G20" s="30"/>
       <x:c r="H20" s="30"/>
       <x:c r="I20" s="30"/>
-      <x:c r="J20" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
-        <x:v>43.4</x:v>
+      <x:c r="J20" s="32" t="n">
+        <x:f>SUM(J4:J17)</x:f>
+        <x:v>601.6</x:v>
       </x:c>
       <x:c r="K20" s="30"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B21" s="30"/>
+      <x:c r="C21" s="30"/>
+      <x:c r="D21" s="30"/>
+      <x:c r="E21" s="30"/>
+      <x:c r="F21" s="30"/>
+      <x:c r="G21" s="30"/>
+      <x:c r="H21" s="30"/>
+      <x:c r="I21" s="30"/>
+      <x:c r="J21" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="K21" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5832,31 +5976,49 @@
         <x:v>IC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B19" s="30" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C19" s="30"/>
-      <x:c r="D19" s="30"/>
-      <x:c r="E19" s="30"/>
-      <x:c r="F19" s="30"/>
-      <x:c r="G19" s="30"/>
-      <x:c r="H19" s="30"/>
-      <x:c r="I19" s="30"/>
-      <x:c r="J19" s="32" t="n">
-        <x:f>SUM(J4:J16)</x:f>
-        <x:v>2209</x:v>
-      </x:c>
-      <x:c r="K19" s="30"/>
+    <x:row r="17">
+      <x:c r="A17" s="22" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B17" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C17" s="22" t="str">
+        <x:v>8月20日</x:v>
+      </x:c>
+      <x:c r="D17" s="23" t="n">
+        <x:v>7789.6</x:v>
+      </x:c>
+      <x:c r="E17" s="23" t="n">
+        <x:v>7811</x:v>
+      </x:c>
+      <x:c r="F17" s="23" t="n">
+        <x:v>7713</x:v>
+      </x:c>
+      <x:c r="G17" s="23" t="n">
+        <x:v>7761</x:v>
+      </x:c>
+      <x:c r="H17" s="23" t="n">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="I17" s="24" t="n">
+        <x:v>0.006353734439834113</x:v>
+      </x:c>
+      <x:c r="J17" s="23" t="n">
+        <x:f>ROUND(E17-F17,1)</x:f>
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="K17" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B20" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B20" s="30" t="n">
+        <x:v>14</x:v>
+      </x:c>
       <x:c r="C20" s="30"/>
       <x:c r="D20" s="30"/>
       <x:c r="E20" s="30"/>
@@ -5864,11 +6026,29 @@
       <x:c r="G20" s="30"/>
       <x:c r="H20" s="30"/>
       <x:c r="I20" s="30"/>
-      <x:c r="J20" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
-        <x:v>169.9</x:v>
+      <x:c r="J20" s="32" t="n">
+        <x:f>SUM(J4:J17)</x:f>
+        <x:v>2307</x:v>
       </x:c>
       <x:c r="K20" s="30"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B21" s="30"/>
+      <x:c r="C21" s="30"/>
+      <x:c r="D21" s="30"/>
+      <x:c r="E21" s="30"/>
+      <x:c r="F21" s="30"/>
+      <x:c r="G21" s="30"/>
+      <x:c r="H21" s="30"/>
+      <x:c r="I21" s="30"/>
+      <x:c r="J21" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
+        <x:v>164.8</x:v>
+      </x:c>
+      <x:c r="K21" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -6403,31 +6583,49 @@
         <x:v>IF2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B19" s="30" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C19" s="30"/>
-      <x:c r="D19" s="30"/>
-      <x:c r="E19" s="30"/>
-      <x:c r="F19" s="30"/>
-      <x:c r="G19" s="30"/>
-      <x:c r="H19" s="30"/>
-      <x:c r="I19" s="30"/>
-      <x:c r="J19" s="32" t="n">
-        <x:f>SUM(J4:J16)</x:f>
-        <x:v>808</x:v>
-      </x:c>
-      <x:c r="K19" s="30"/>
+    <x:row r="17">
+      <x:c r="A17" s="22" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B17" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C17" s="22" t="str">
+        <x:v>8月20日</x:v>
+      </x:c>
+      <x:c r="D17" s="23" t="n">
+        <x:v>4580</x:v>
+      </x:c>
+      <x:c r="E17" s="23" t="n">
+        <x:v>4585</x:v>
+      </x:c>
+      <x:c r="F17" s="23" t="n">
+        <x:v>4532.4</x:v>
+      </x:c>
+      <x:c r="G17" s="23" t="n">
+        <x:v>4554</x:v>
+      </x:c>
+      <x:c r="H17" s="23" t="n">
+        <x:v>-0.2</x:v>
+      </x:c>
+      <x:c r="I17" s="24" t="n">
+        <x:v>-0.000043915506565350704</x:v>
+      </x:c>
+      <x:c r="J17" s="23" t="n">
+        <x:f>ROUND(E17-F17,1)</x:f>
+        <x:v>52.6</x:v>
+      </x:c>
+      <x:c r="K17" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B20" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B20" s="30" t="n">
+        <x:v>14</x:v>
+      </x:c>
       <x:c r="C20" s="30"/>
       <x:c r="D20" s="30"/>
       <x:c r="E20" s="30"/>
@@ -6435,11 +6633,29 @@
       <x:c r="G20" s="30"/>
       <x:c r="H20" s="30"/>
       <x:c r="I20" s="30"/>
-      <x:c r="J20" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
-        <x:v>62.2</x:v>
+      <x:c r="J20" s="32" t="n">
+        <x:f>SUM(J4:J17)</x:f>
+        <x:v>860.6</x:v>
       </x:c>
       <x:c r="K20" s="30"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B21" s="30"/>
+      <x:c r="C21" s="30"/>
+      <x:c r="D21" s="30"/>
+      <x:c r="E21" s="30"/>
+      <x:c r="F21" s="30"/>
+      <x:c r="G21" s="30"/>
+      <x:c r="H21" s="30"/>
+      <x:c r="I21" s="30"/>
+      <x:c r="J21" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
+        <x:v>61.5</x:v>
+      </x:c>
+      <x:c r="K21" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-08-21
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R1aa1fb9242504593"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Rcee977c0358a494c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Rfbf2772f8ee443f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R1fe7ad66b0ad4637"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R41feceb005914592"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R13f26005b5654395"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R8dc54ded5feb492e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rd6504beba4d34e5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Racab647f61fa4e70"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R48b107f67af44035"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R5b68d53e0cc743fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R113afc4f93ed4be8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Rda78812c1cf143ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rdaeca1abd9c34fca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R40b3d909f50e4c43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Ra3c55fdfbbb648de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Raf1b3dfd22d0412a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R9c3b3f775c794233"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Red132be2df254248"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="Rd6ff078e4e724cd1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -26,7 +26,7 @@
     <x:numFmt numFmtId="200" formatCode="General"/>
     <x:numFmt numFmtId="201" formatCode="0.0%"/>
   </x:numFmts>
-  <x:fonts count="9">
+  <x:fonts count="10">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -77,8 +77,14 @@
       <x:color rgb="FF1D4ED8"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF1E3A8A"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -108,6 +114,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFBFDBFE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDBEAFE"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -145,7 +156,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="39">
+  <x:cellXfs count="47">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -232,7 +243,31 @@
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="6" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="9" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="9" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="9" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="9" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -485,25 +520,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-08-20</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7656.61</x:v>
+        <x:v>7634.08</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7541.48</x:v>
+        <x:v>7472.49</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>115.1</x:v>
+        <x:v>161.6</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>2385.7</x:v>
+        <x:v>2547.3</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>170.4</x:v>
+        <x:v>169.8</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -514,25 +549,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-08-20</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7923.91</x:v>
+        <x:v>7877.34</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7796.28</x:v>
+        <x:v>7756.28</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>127.6</x:v>
+        <x:v>121.1</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>2329.4</x:v>
+        <x:v>2450.5</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>166.4</x:v>
+        <x:v>163.4</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -543,25 +578,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-08-20</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3925.06</x:v>
+        <x:v>3912.13</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3888.1</x:v>
+        <x:v>3883.79</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>37</x:v>
+        <x:v>28.3</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>601.6</x:v>
+        <x:v>629.9</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>43</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -572,25 +607,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-08-20</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>7582.2</x:v>
+        <x:v>7575</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>7482.8</x:v>
+        <x:v>7410</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>99.4</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>2330.4</x:v>
+        <x:v>2495.4</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>166.5</x:v>
+        <x:v>166.4</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -688,25 +723,25 @@
         <x:v>碳酸锂2609</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>2026-08-20</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:v>152600</x:v>
+        <x:v>157000</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
-        <x:v>149800</x:v>
+        <x:v>150020</x:v>
       </x:c>
       <x:c r="E11" s="12" t="n">
-        <x:v>2800</x:v>
+        <x:v>6980</x:v>
       </x:c>
       <x:c r="F11" s="9" t="n">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G11" s="10" t="n">
-        <x:v>67120</x:v>
+        <x:v>74100</x:v>
       </x:c>
       <x:c r="H11" s="10" t="n">
-        <x:v>4794.3</x:v>
+        <x:v>4940</x:v>
       </x:c>
       <x:c r="I11" s="10" t="n">
         <x:v>6000</x:v>
@@ -720,7 +755,7 @@
         <x:v>2026-08-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-08-20</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1407,31 +1442,49 @@
         <x:v>LC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B20" s="30" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C20" s="30"/>
-      <x:c r="D20" s="30"/>
-      <x:c r="E20" s="30"/>
-      <x:c r="F20" s="30"/>
-      <x:c r="G20" s="30"/>
-      <x:c r="H20" s="30"/>
-      <x:c r="I20" s="30"/>
-      <x:c r="J20" s="32" t="n">
-        <x:f>SUM(J4:J17)</x:f>
-        <x:v>67120</x:v>
-      </x:c>
-      <x:c r="K20" s="30"/>
+    <x:row r="18">
+      <x:c r="A18" s="41" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B18" s="41" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C18" s="41" t="str">
+        <x:v>8月21日</x:v>
+      </x:c>
+      <x:c r="D18" s="42" t="n">
+        <x:v>151500</x:v>
+      </x:c>
+      <x:c r="E18" s="42" t="n">
+        <x:v>157000</x:v>
+      </x:c>
+      <x:c r="F18" s="42" t="n">
+        <x:v>150020</x:v>
+      </x:c>
+      <x:c r="G18" s="42" t="n">
+        <x:v>156140</x:v>
+      </x:c>
+      <x:c r="H18" s="28" t="n">
+        <x:v>4640</x:v>
+      </x:c>
+      <x:c r="I18" s="43" t="n">
+        <x:v>0.03062706270627058</x:v>
+      </x:c>
+      <x:c r="J18" s="26" t="n">
+        <x:f>ROUND(E18-F18,1)</x:f>
+        <x:v>6980</x:v>
+      </x:c>
+      <x:c r="K18" s="41" t="str">
+        <x:v>LC2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B21" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B21" s="30" t="n">
+        <x:v>15</x:v>
+      </x:c>
       <x:c r="C21" s="30"/>
       <x:c r="D21" s="30"/>
       <x:c r="E21" s="30"/>
@@ -1439,11 +1492,29 @@
       <x:c r="G21" s="30"/>
       <x:c r="H21" s="30"/>
       <x:c r="I21" s="30"/>
-      <x:c r="J21" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
-        <x:v>4794.3</x:v>
+      <x:c r="J21" s="32" t="n">
+        <x:f>SUM(J4:J18)</x:f>
+        <x:v>74100</x:v>
       </x:c>
       <x:c r="K21" s="30"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B22" s="30"/>
+      <x:c r="C22" s="30"/>
+      <x:c r="D22" s="30"/>
+      <x:c r="E22" s="30"/>
+      <x:c r="F22" s="30"/>
+      <x:c r="G22" s="30"/>
+      <x:c r="H22" s="30"/>
+      <x:c r="I22" s="30"/>
+      <x:c r="J22" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
+        <x:v>4940</x:v>
+      </x:c>
+      <x:c r="K22" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1600,7 +1671,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B7" s="22" t="str">
-        <x:v>8月17日-8月20日</x:v>
+        <x:v>8月17日-8月21日</x:v>
       </x:c>
       <x:c r="C7" s="23" t="n">
         <x:v>7797.18</x:v>
@@ -1609,28 +1680,28 @@
         <x:v>7995.5</x:v>
       </x:c>
       <x:c r="E7" s="23" t="n">
-        <x:v>7490.21</x:v>
+        <x:v>7472.49</x:v>
       </x:c>
       <x:c r="F7" s="23" t="n">
-        <x:v>7589.78</x:v>
+        <x:v>7601.8</x:v>
       </x:c>
       <x:c r="G7" s="28" t="n">
         <x:f>ROUND(F7-F6,1)</x:f>
-        <x:v>-180</x:v>
+        <x:v>-168</x:v>
       </x:c>
       <x:c r="H7" s="24" t="n">
         <x:f>IFERROR(F7/F6-1,"")</x:f>
-        <x:v>-0.023171707967494792</x:v>
+        <x:v>-0.021624696582417502</x:v>
       </x:c>
       <x:c r="I7" s="26" t="n">
         <x:f>ROUND(D7-E7,1)</x:f>
-        <x:v>505.3</x:v>
+        <x:v>523</x:v>
       </x:c>
       <x:c r="J7" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K7" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -1648,7 +1719,7 @@
       <x:c r="H8" s="30"/>
       <x:c r="I8" s="32" t="n">
         <x:f>ROUND(SUM(I5:I7),1)</x:f>
-        <x:v>1406.6</x:v>
+        <x:v>1424.3</x:v>
       </x:c>
       <x:c r="J8" s="30"/>
       <x:c r="K8" s="30"/>
@@ -1666,7 +1737,7 @@
       <x:c r="H9" s="30"/>
       <x:c r="I9" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I7),0),1)</x:f>
-        <x:v>468.9</x:v>
+        <x:v>474.8</x:v>
       </x:c>
       <x:c r="J9" s="30"/>
       <x:c r="K9" s="30"/>
@@ -1796,7 +1867,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B15" s="22" t="str">
-        <x:v>8月17日-8月20日</x:v>
+        <x:v>8月17日-8月21日</x:v>
       </x:c>
       <x:c r="C15" s="23" t="n">
         <x:v>8007.87</x:v>
@@ -1805,28 +1876,28 @@
         <x:v>8211.31</x:v>
       </x:c>
       <x:c r="E15" s="23" t="n">
-        <x:v>7762.29</x:v>
+        <x:v>7756.28</x:v>
       </x:c>
       <x:c r="F15" s="23" t="n">
-        <x:v>7850.4</x:v>
+        <x:v>7854.33</x:v>
       </x:c>
       <x:c r="G15" s="23" t="n">
         <x:f>ROUND(F15-F14,1)</x:f>
-        <x:v>-139.9</x:v>
+        <x:v>-136</x:v>
       </x:c>
       <x:c r="H15" s="24" t="n">
         <x:f>IFERROR(F15/F14-1,"")</x:f>
-        <x:v>-0.01751241813542126</x:v>
+        <x:v>-0.01702057361836118</x:v>
       </x:c>
       <x:c r="I15" s="26" t="n">
         <x:f>ROUND(D15-E15,1)</x:f>
-        <x:v>449</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="J15" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K15" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1844,7 +1915,7 @@
       <x:c r="H16" s="30"/>
       <x:c r="I16" s="32" t="n">
         <x:f>ROUND(SUM(I13:I15),1)</x:f>
-        <x:v>1279.3</x:v>
+        <x:v>1285.3</x:v>
       </x:c>
       <x:c r="J16" s="30"/>
       <x:c r="K16" s="30"/>
@@ -1862,7 +1933,7 @@
       <x:c r="H17" s="30"/>
       <x:c r="I17" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I13:I15),0),1)</x:f>
-        <x:v>426.4</x:v>
+        <x:v>428.4</x:v>
       </x:c>
       <x:c r="J17" s="30"/>
       <x:c r="K17" s="30"/>
@@ -1992,7 +2063,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B23" s="22" t="str">
-        <x:v>8月17日-8月20日</x:v>
+        <x:v>8月17日-8月21日</x:v>
       </x:c>
       <x:c r="C23" s="23" t="n">
         <x:v>3930.1</x:v>
@@ -2004,15 +2075,15 @@
         <x:v>3879.58</x:v>
       </x:c>
       <x:c r="F23" s="23" t="n">
-        <x:v>3903.72</x:v>
+        <x:v>3905.2</x:v>
       </x:c>
       <x:c r="G23" s="23" t="n">
         <x:f>ROUND(F23-F22,1)</x:f>
-        <x:v>-23.5</x:v>
+        <x:v>-22</x:v>
       </x:c>
       <x:c r="H23" s="24" t="n">
         <x:f>IFERROR(F23/F22-1,"")</x:f>
-        <x:v>-0.005973752158037082</x:v>
+        <x:v>-0.00559689140808417</x:v>
       </x:c>
       <x:c r="I23" s="26" t="n">
         <x:f>ROUND(D23-E23,1)</x:f>
@@ -2022,7 +2093,7 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K23" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -2188,7 +2259,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B31" s="22" t="str">
-        <x:v>8月17日-8月20日</x:v>
+        <x:v>8月17日-8月21日</x:v>
       </x:c>
       <x:c r="C31" s="23" t="n">
         <x:v>7675</x:v>
@@ -2197,28 +2268,28 @@
         <x:v>7882.8</x:v>
       </x:c>
       <x:c r="E31" s="23" t="n">
-        <x:v>7430</x:v>
+        <x:v>7410</x:v>
       </x:c>
       <x:c r="F31" s="23" t="n">
-        <x:v>7516.2</x:v>
+        <x:v>7527</x:v>
       </x:c>
       <x:c r="G31" s="23" t="n">
         <x:f>ROUND(F31-F30,1)</x:f>
-        <x:v>-134</x:v>
+        <x:v>-123.2</x:v>
       </x:c>
       <x:c r="H31" s="24" t="n">
         <x:f>IFERROR(F31/F30-1,"")</x:f>
-        <x:v>-0.01751588193772713</x:v>
+        <x:v>-0.016104154139761073</x:v>
       </x:c>
       <x:c r="I31" s="26" t="n">
         <x:f>ROUND(D31-E31,1)</x:f>
-        <x:v>452.8</x:v>
+        <x:v>472.8</x:v>
       </x:c>
       <x:c r="J31" s="22" t="str">
         <x:v>IM2609</x:v>
       </x:c>
       <x:c r="K31" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -2236,7 +2307,7 @@
       <x:c r="H32" s="30"/>
       <x:c r="I32" s="32" t="n">
         <x:f>ROUND(SUM(I29:I31),1)</x:f>
-        <x:v>1322</x:v>
+        <x:v>1342</x:v>
       </x:c>
       <x:c r="J32" s="30"/>
       <x:c r="K32" s="30"/>
@@ -2254,7 +2325,7 @@
       <x:c r="H33" s="30"/>
       <x:c r="I33" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I29:I31),0),1)</x:f>
-        <x:v>440.7</x:v>
+        <x:v>447.3</x:v>
       </x:c>
       <x:c r="J33" s="30"/>
       <x:c r="K33" s="30"/>
@@ -2972,37 +3043,37 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B63" s="22" t="str">
-        <x:v>8月17日-8月20日</x:v>
+        <x:v>8月17日-8月21日</x:v>
       </x:c>
       <x:c r="C63" s="23" t="n">
         <x:v>154300</x:v>
       </x:c>
       <x:c r="D63" s="23" t="n">
-        <x:v>155980</x:v>
+        <x:v>157000</x:v>
       </x:c>
       <x:c r="E63" s="23" t="n">
         <x:v>148400</x:v>
       </x:c>
       <x:c r="F63" s="23" t="n">
-        <x:v>151500</x:v>
+        <x:v>156140</x:v>
       </x:c>
       <x:c r="G63" s="28" t="n">
         <x:f>ROUND(F63-F62,1)</x:f>
-        <x:v>-2440</x:v>
+        <x:v>2200</x:v>
       </x:c>
       <x:c r="H63" s="24" t="n">
         <x:f>IFERROR(F63/F62-1,"")</x:f>
-        <x:v>-0.01585033129790825</x:v>
+        <x:v>0.014291282317786091</x:v>
       </x:c>
       <x:c r="I63" s="26" t="n">
         <x:f>ROUND(D63-E63,1)</x:f>
-        <x:v>7580</x:v>
+        <x:v>8600</x:v>
       </x:c>
       <x:c r="J63" s="22" t="str">
         <x:v>LC2609</x:v>
       </x:c>
       <x:c r="K63" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
@@ -3020,7 +3091,7 @@
       <x:c r="H64" s="30"/>
       <x:c r="I64" s="32" t="n">
         <x:f>ROUND(SUM(I61:I63),1)</x:f>
-        <x:v>32040</x:v>
+        <x:v>33060</x:v>
       </x:c>
       <x:c r="J64" s="30"/>
       <x:c r="K64" s="30"/>
@@ -3038,7 +3109,7 @@
       <x:c r="H65" s="30"/>
       <x:c r="I65" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I61:I63),0),1)</x:f>
-        <x:v>10680</x:v>
+        <x:v>11020</x:v>
       </x:c>
       <x:c r="J65" s="30"/>
       <x:c r="K65" s="30"/>
@@ -3620,31 +3691,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B20" s="30" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C20" s="30"/>
-      <x:c r="D20" s="30"/>
-      <x:c r="E20" s="30"/>
-      <x:c r="F20" s="30"/>
-      <x:c r="G20" s="30"/>
-      <x:c r="H20" s="30"/>
-      <x:c r="I20" s="30"/>
-      <x:c r="J20" s="32" t="n">
-        <x:f>SUM(J4:J17)</x:f>
-        <x:v>2385.7000000000003</x:v>
-      </x:c>
-      <x:c r="K20" s="30"/>
+    <x:row r="18">
+      <x:c r="A18" s="41" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B18" s="41" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C18" s="41" t="str">
+        <x:v>8月21日</x:v>
+      </x:c>
+      <x:c r="D18" s="42" t="n">
+        <x:v>7555.55</x:v>
+      </x:c>
+      <x:c r="E18" s="42" t="n">
+        <x:v>7634.08</x:v>
+      </x:c>
+      <x:c r="F18" s="42" t="n">
+        <x:v>7472.49</x:v>
+      </x:c>
+      <x:c r="G18" s="42" t="n">
+        <x:v>7601.8</x:v>
+      </x:c>
+      <x:c r="H18" s="42" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="I18" s="43" t="n">
+        <x:v>0.0015837086186951677</x:v>
+      </x:c>
+      <x:c r="J18" s="42" t="n">
+        <x:f>ROUND(E18-F18,1)</x:f>
+        <x:v>161.6</x:v>
+      </x:c>
+      <x:c r="K18" s="41" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B21" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B21" s="30" t="n">
+        <x:v>15</x:v>
+      </x:c>
       <x:c r="C21" s="30"/>
       <x:c r="D21" s="30"/>
       <x:c r="E21" s="30"/>
@@ -3652,11 +3741,29 @@
       <x:c r="G21" s="30"/>
       <x:c r="H21" s="30"/>
       <x:c r="I21" s="30"/>
-      <x:c r="J21" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
-        <x:v>170.4</x:v>
+      <x:c r="J21" s="32" t="n">
+        <x:f>SUM(J4:J18)</x:f>
+        <x:v>2547.3</x:v>
       </x:c>
       <x:c r="K21" s="30"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B22" s="30"/>
+      <x:c r="C22" s="30"/>
+      <x:c r="D22" s="30"/>
+      <x:c r="E22" s="30"/>
+      <x:c r="F22" s="30"/>
+      <x:c r="G22" s="30"/>
+      <x:c r="H22" s="30"/>
+      <x:c r="I22" s="30"/>
+      <x:c r="J22" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
+        <x:v>169.8</x:v>
+      </x:c>
+      <x:c r="K22" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4227,31 +4334,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B20" s="30" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C20" s="30"/>
-      <x:c r="D20" s="30"/>
-      <x:c r="E20" s="30"/>
-      <x:c r="F20" s="30"/>
-      <x:c r="G20" s="30"/>
-      <x:c r="H20" s="30"/>
-      <x:c r="I20" s="30"/>
-      <x:c r="J20" s="32" t="n">
-        <x:f>SUM(J4:J17)</x:f>
-        <x:v>2329.4</x:v>
-      </x:c>
-      <x:c r="K20" s="30"/>
+    <x:row r="18">
+      <x:c r="A18" s="41" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B18" s="41" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C18" s="41" t="str">
+        <x:v>8月21日</x:v>
+      </x:c>
+      <x:c r="D18" s="42" t="n">
+        <x:v>7812.26</x:v>
+      </x:c>
+      <x:c r="E18" s="42" t="n">
+        <x:v>7877.34</x:v>
+      </x:c>
+      <x:c r="F18" s="42" t="n">
+        <x:v>7756.28</x:v>
+      </x:c>
+      <x:c r="G18" s="42" t="n">
+        <x:v>7854.33</x:v>
+      </x:c>
+      <x:c r="H18" s="42" t="n">
+        <x:v>3.9</x:v>
+      </x:c>
+      <x:c r="I18" s="43" t="n">
+        <x:v>0.0005006114338124146</x:v>
+      </x:c>
+      <x:c r="J18" s="42" t="n">
+        <x:f>ROUND(E18-F18,1)</x:f>
+        <x:v>121.1</x:v>
+      </x:c>
+      <x:c r="K18" s="41" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B21" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B21" s="30" t="n">
+        <x:v>15</x:v>
+      </x:c>
       <x:c r="C21" s="30"/>
       <x:c r="D21" s="30"/>
       <x:c r="E21" s="30"/>
@@ -4259,11 +4384,29 @@
       <x:c r="G21" s="30"/>
       <x:c r="H21" s="30"/>
       <x:c r="I21" s="30"/>
-      <x:c r="J21" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
-        <x:v>166.4</x:v>
+      <x:c r="J21" s="32" t="n">
+        <x:f>SUM(J4:J18)</x:f>
+        <x:v>2450.5</x:v>
       </x:c>
       <x:c r="K21" s="30"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B22" s="30"/>
+      <x:c r="C22" s="30"/>
+      <x:c r="D22" s="30"/>
+      <x:c r="E22" s="30"/>
+      <x:c r="F22" s="30"/>
+      <x:c r="G22" s="30"/>
+      <x:c r="H22" s="30"/>
+      <x:c r="I22" s="30"/>
+      <x:c r="J22" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
+        <x:v>163.4</x:v>
+      </x:c>
+      <x:c r="K22" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4834,31 +4977,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B20" s="30" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C20" s="30"/>
-      <x:c r="D20" s="30"/>
-      <x:c r="E20" s="30"/>
-      <x:c r="F20" s="30"/>
-      <x:c r="G20" s="30"/>
-      <x:c r="H20" s="30"/>
-      <x:c r="I20" s="30"/>
-      <x:c r="J20" s="32" t="n">
-        <x:f>SUM(J4:J17)</x:f>
-        <x:v>601.6</x:v>
-      </x:c>
-      <x:c r="K20" s="30"/>
+    <x:row r="18">
+      <x:c r="A18" s="41" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B18" s="41" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C18" s="41" t="str">
+        <x:v>8月21日</x:v>
+      </x:c>
+      <x:c r="D18" s="42" t="n">
+        <x:v>3891.18</x:v>
+      </x:c>
+      <x:c r="E18" s="42" t="n">
+        <x:v>3912.13</x:v>
+      </x:c>
+      <x:c r="F18" s="42" t="n">
+        <x:v>3883.79</x:v>
+      </x:c>
+      <x:c r="G18" s="42" t="n">
+        <x:v>3905.2</x:v>
+      </x:c>
+      <x:c r="H18" s="42" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="I18" s="43" t="n">
+        <x:v>0.0003791255520375625</x:v>
+      </x:c>
+      <x:c r="J18" s="42" t="n">
+        <x:f>ROUND(E18-F18,1)</x:f>
+        <x:v>28.3</x:v>
+      </x:c>
+      <x:c r="K18" s="41" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B21" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B21" s="30" t="n">
+        <x:v>15</x:v>
+      </x:c>
       <x:c r="C21" s="30"/>
       <x:c r="D21" s="30"/>
       <x:c r="E21" s="30"/>
@@ -4866,11 +5027,29 @@
       <x:c r="G21" s="30"/>
       <x:c r="H21" s="30"/>
       <x:c r="I21" s="30"/>
-      <x:c r="J21" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
-        <x:v>43</x:v>
+      <x:c r="J21" s="32" t="n">
+        <x:f>SUM(J4:J18)</x:f>
+        <x:v>629.9</x:v>
       </x:c>
       <x:c r="K21" s="30"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B22" s="30"/>
+      <x:c r="C22" s="30"/>
+      <x:c r="D22" s="30"/>
+      <x:c r="E22" s="30"/>
+      <x:c r="F22" s="30"/>
+      <x:c r="G22" s="30"/>
+      <x:c r="H22" s="30"/>
+      <x:c r="I22" s="30"/>
+      <x:c r="J22" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="K22" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5441,31 +5620,49 @@
         <x:v>IM2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B20" s="30" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C20" s="30"/>
-      <x:c r="D20" s="30"/>
-      <x:c r="E20" s="30"/>
-      <x:c r="F20" s="30"/>
-      <x:c r="G20" s="30"/>
-      <x:c r="H20" s="30"/>
-      <x:c r="I20" s="30"/>
-      <x:c r="J20" s="32" t="n">
-        <x:f>SUM(J4:J17)</x:f>
-        <x:v>2330.4</x:v>
-      </x:c>
-      <x:c r="K20" s="30"/>
+    <x:row r="18">
+      <x:c r="A18" s="41" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B18" s="41" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C18" s="41" t="str">
+        <x:v>8月21日</x:v>
+      </x:c>
+      <x:c r="D18" s="42" t="n">
+        <x:v>7500</x:v>
+      </x:c>
+      <x:c r="E18" s="42" t="n">
+        <x:v>7575</x:v>
+      </x:c>
+      <x:c r="F18" s="42" t="n">
+        <x:v>7410</x:v>
+      </x:c>
+      <x:c r="G18" s="42" t="n">
+        <x:v>7527</x:v>
+      </x:c>
+      <x:c r="H18" s="42" t="n">
+        <x:v>10.8</x:v>
+      </x:c>
+      <x:c r="I18" s="43" t="n">
+        <x:v>0.0014368963039834703</x:v>
+      </x:c>
+      <x:c r="J18" s="42" t="n">
+        <x:f>ROUND(E18-F18,1)</x:f>
+        <x:v>165</x:v>
+      </x:c>
+      <x:c r="K18" s="41" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B21" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B21" s="30" t="n">
+        <x:v>15</x:v>
+      </x:c>
       <x:c r="C21" s="30"/>
       <x:c r="D21" s="30"/>
       <x:c r="E21" s="30"/>
@@ -5473,11 +5670,29 @@
       <x:c r="G21" s="30"/>
       <x:c r="H21" s="30"/>
       <x:c r="I21" s="30"/>
-      <x:c r="J21" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
-        <x:v>166.5</x:v>
+      <x:c r="J21" s="32" t="n">
+        <x:f>SUM(J4:J18)</x:f>
+        <x:v>2495.4</x:v>
       </x:c>
       <x:c r="K21" s="30"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B22" s="30"/>
+      <x:c r="C22" s="30"/>
+      <x:c r="D22" s="30"/>
+      <x:c r="E22" s="30"/>
+      <x:c r="F22" s="30"/>
+      <x:c r="G22" s="30"/>
+      <x:c r="H22" s="30"/>
+      <x:c r="I22" s="30"/>
+      <x:c r="J22" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
+        <x:v>166.4</x:v>
+      </x:c>
+      <x:c r="K22" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-08-24
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R9041b47191a545b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R37be7772ec88469a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R1392dc21084a4a91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rb355b0d9ff9749aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Rbe4c998fde4d4cc4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R82710720a50b4989"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R86e17db1d8c94523"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R560f009bbba4459d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rae4b220002794082"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R680f6ddcb2814664"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R3342cb50a6244bd6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R5e46c218d3f94309"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Rb5f1158e97ca4969"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R56eeea034f5c411b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R33c8a99264e9493b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R1ffd55d13c7440ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Reecbc1b6ccfe447b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R9577debbf1054023"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rbcfd2782d0fe4839"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="Rbef552fdff6e47c6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -520,25 +520,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-08-21</x:v>
+        <x:v>2026-08-24</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7634.08</x:v>
+        <x:v>7633.34</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7472.49</x:v>
+        <x:v>7377.72</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>161.6</x:v>
+        <x:v>255.6</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>2547.3</x:v>
+        <x:v>2802.9</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>169.8</x:v>
+        <x:v>175.2</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -549,25 +549,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-08-21</x:v>
+        <x:v>2026-08-24</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7877.34</x:v>
+        <x:v>7865.54</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7756.28</x:v>
+        <x:v>7615.45</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>121.1</x:v>
+        <x:v>250.1</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>2450.5</x:v>
+        <x:v>2700.6</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>163.4</x:v>
+        <x:v>168.8</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -578,25 +578,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-08-21</x:v>
+        <x:v>2026-08-24</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3912.13</x:v>
+        <x:v>3910.24</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3883.79</x:v>
+        <x:v>3855.35</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>28.3</x:v>
+        <x:v>54.9</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>629.9</x:v>
+        <x:v>684.8</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>42</x:v>
+        <x:v>42.8</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -636,25 +636,25 @@
         <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>2026-08-21</x:v>
+        <x:v>2026-08-24</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:v>7797.2</x:v>
+        <x:v>7764.4</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>7669.6</x:v>
+        <x:v>7514.4</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>127.6</x:v>
+        <x:v>250</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>2434.6</x:v>
+        <x:v>2684.6</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
-        <x:v>162.3</x:v>
+        <x:v>167.8</x:v>
       </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
@@ -665,25 +665,25 @@
         <x:v>IF主力</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>2026-08-21</x:v>
+        <x:v>2026-08-24</x:v>
       </x:c>
       <x:c r="C9" s="10" t="n">
-        <x:v>4595.8</x:v>
+        <x:v>4607.4</x:v>
       </x:c>
       <x:c r="D9" s="10" t="n">
-        <x:v>4542.4</x:v>
+        <x:v>4486.4</x:v>
       </x:c>
       <x:c r="E9" s="12" t="n">
-        <x:v>53.4</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="F9" s="9" t="n">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G9" s="10" t="n">
-        <x:v>914</x:v>
+        <x:v>1035</x:v>
       </x:c>
       <x:c r="H9" s="10" t="n">
-        <x:v>60.9</x:v>
+        <x:v>64.7</x:v>
       </x:c>
       <x:c r="I9" s="10" t="n">
         <x:v>90</x:v>
@@ -694,25 +694,25 @@
         <x:v>IH主力</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>2026-08-21</x:v>
+        <x:v>2026-08-24</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:v>2873</x:v>
+        <x:v>2866.8</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
-        <x:v>2847.2</x:v>
+        <x:v>2837.4</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
-        <x:v>25.8</x:v>
+        <x:v>29.4</x:v>
       </x:c>
       <x:c r="F10" s="9" t="n">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G10" s="10" t="n">
-        <x:v>508.6</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="H10" s="10" t="n">
-        <x:v>33.9</x:v>
+        <x:v>33.6</x:v>
       </x:c>
       <x:c r="I10" s="10" t="n">
         <x:v>60</x:v>
@@ -723,25 +723,25 @@
         <x:v>碳酸锂2609</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>2026-08-21</x:v>
+        <x:v>2026-08-24</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:v>157000</x:v>
+        <x:v>160000</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
-        <x:v>150020</x:v>
+        <x:v>154280</x:v>
       </x:c>
       <x:c r="E11" s="12" t="n">
-        <x:v>6980</x:v>
+        <x:v>5720</x:v>
       </x:c>
       <x:c r="F11" s="9" t="n">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G11" s="10" t="n">
-        <x:v>74100</x:v>
+        <x:v>79820</x:v>
       </x:c>
       <x:c r="H11" s="10" t="n">
-        <x:v>4940</x:v>
+        <x:v>4988.8</x:v>
       </x:c>
       <x:c r="I11" s="10" t="n">
         <x:v>6000</x:v>
@@ -755,7 +755,7 @@
         <x:v>2026-08-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-08-21</x:v>
+        <x:v>2026-08-24</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1478,31 +1478,49 @@
         <x:v>LC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B21" s="30" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C21" s="30"/>
-      <x:c r="D21" s="30"/>
-      <x:c r="E21" s="30"/>
-      <x:c r="F21" s="30"/>
-      <x:c r="G21" s="30"/>
-      <x:c r="H21" s="30"/>
-      <x:c r="I21" s="30"/>
-      <x:c r="J21" s="32" t="n">
-        <x:f>SUM(J4:J18)</x:f>
-        <x:v>74100</x:v>
-      </x:c>
-      <x:c r="K21" s="30"/>
+    <x:row r="19">
+      <x:c r="A19" s="22" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B19" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C19" s="22" t="str">
+        <x:v>8月24日</x:v>
+      </x:c>
+      <x:c r="D19" s="23" t="n">
+        <x:v>158500</x:v>
+      </x:c>
+      <x:c r="E19" s="23" t="n">
+        <x:v>160000</x:v>
+      </x:c>
+      <x:c r="F19" s="23" t="n">
+        <x:v>154280</x:v>
+      </x:c>
+      <x:c r="G19" s="23" t="n">
+        <x:v>157000</x:v>
+      </x:c>
+      <x:c r="H19" s="28" t="n">
+        <x:v>860</x:v>
+      </x:c>
+      <x:c r="I19" s="24" t="n">
+        <x:v>0.005507877545792184</x:v>
+      </x:c>
+      <x:c r="J19" s="23" t="n">
+        <x:f>ROUND(E19-F19,1)</x:f>
+        <x:v>5720</x:v>
+      </x:c>
+      <x:c r="K19" s="22" t="str">
+        <x:v>LC2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B22" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B22" s="30" t="n">
+        <x:v>16</x:v>
+      </x:c>
       <x:c r="C22" s="30"/>
       <x:c r="D22" s="30"/>
       <x:c r="E22" s="30"/>
@@ -1510,11 +1528,29 @@
       <x:c r="G22" s="30"/>
       <x:c r="H22" s="30"/>
       <x:c r="I22" s="30"/>
-      <x:c r="J22" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
-        <x:v>4940</x:v>
+      <x:c r="J22" s="32" t="n">
+        <x:f>SUM(J4:J19)</x:f>
+        <x:v>79820</x:v>
       </x:c>
       <x:c r="K22" s="30"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B23" s="30"/>
+      <x:c r="C23" s="30"/>
+      <x:c r="D23" s="30"/>
+      <x:c r="E23" s="30"/>
+      <x:c r="F23" s="30"/>
+      <x:c r="G23" s="30"/>
+      <x:c r="H23" s="30"/>
+      <x:c r="I23" s="30"/>
+      <x:c r="J23" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
+        <x:v>4988.8</x:v>
+      </x:c>
+      <x:c r="K23" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1705,155 +1741,155 @@
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B8" s="30" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C8" s="30"/>
-      <x:c r="D8" s="30"/>
-      <x:c r="E8" s="30"/>
-      <x:c r="F8" s="30"/>
-      <x:c r="G8" s="30"/>
-      <x:c r="H8" s="30"/>
-      <x:c r="I8" s="32" t="n">
-        <x:f>ROUND(SUM(I5:I7),1)</x:f>
-        <x:v>1424.3</x:v>
-      </x:c>
-      <x:c r="J8" s="30"/>
-      <x:c r="K8" s="30"/>
+      <x:c r="A8" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B8" s="22" t="str">
+        <x:v>8月24日</x:v>
+      </x:c>
+      <x:c r="C8" s="23" t="n">
+        <x:v>7614.89</x:v>
+      </x:c>
+      <x:c r="D8" s="23" t="n">
+        <x:v>7633.34</x:v>
+      </x:c>
+      <x:c r="E8" s="23" t="n">
+        <x:v>7377.72</x:v>
+      </x:c>
+      <x:c r="F8" s="23" t="n">
+        <x:v>7491.49</x:v>
+      </x:c>
+      <x:c r="G8" s="23" t="n">
+        <x:f>ROUND(F8-F7,1)</x:f>
+        <x:v>-110.3</x:v>
+      </x:c>
+      <x:c r="H8" s="24" t="n">
+        <x:f>IFERROR(F8/F7-1,"")</x:f>
+        <x:v>-0.014511036859691129</x:v>
+      </x:c>
+      <x:c r="I8" s="26" t="n">
+        <x:f>ROUND(D8-E8,1)</x:f>
+        <x:v>255.6</x:v>
+      </x:c>
+      <x:c r="J8" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
+      <x:c r="K8" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B9" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B9" s="30" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="C9" s="30"/>
       <x:c r="D9" s="30"/>
       <x:c r="E9" s="30"/>
       <x:c r="F9" s="30"/>
       <x:c r="G9" s="30"/>
       <x:c r="H9" s="30"/>
-      <x:c r="I9" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I5:I7),0),1)</x:f>
-        <x:v>474.8</x:v>
+      <x:c r="I9" s="32" t="n">
+        <x:f>ROUND(SUM(I5:I8),1)</x:f>
+        <x:v>1679.9</x:v>
       </x:c>
       <x:c r="J9" s="30"/>
       <x:c r="K9" s="30"/>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="17" t="str">
+    <x:row r="10">
+      <x:c r="A10" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B10" s="30"/>
+      <x:c r="C10" s="30"/>
+      <x:c r="D10" s="30"/>
+      <x:c r="E10" s="30"/>
+      <x:c r="F10" s="30"/>
+      <x:c r="G10" s="30"/>
+      <x:c r="H10" s="30"/>
+      <x:c r="I10" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I5:I8),0),1)</x:f>
+        <x:v>420</x:v>
+      </x:c>
+      <x:c r="J10" s="30"/>
+      <x:c r="K10" s="30"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="17" t="str">
         <x:v>中证500</x:v>
       </x:c>
-      <x:c r="B11" s="17"/>
-      <x:c r="C11" s="17"/>
-      <x:c r="D11" s="17"/>
-      <x:c r="E11" s="17"/>
-      <x:c r="F11" s="17"/>
-      <x:c r="G11" s="17"/>
-      <x:c r="H11" s="17"/>
-      <x:c r="I11" s="17"/>
-      <x:c r="J11" s="17"/>
-      <x:c r="K11" s="17"/>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="20" t="str">
+      <x:c r="B12" s="17"/>
+      <x:c r="C12" s="17"/>
+      <x:c r="D12" s="17"/>
+      <x:c r="E12" s="17"/>
+      <x:c r="F12" s="17"/>
+      <x:c r="G12" s="17"/>
+      <x:c r="H12" s="17"/>
+      <x:c r="I12" s="17"/>
+      <x:c r="J12" s="17"/>
+      <x:c r="K12" s="17"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B12" s="20" t="str">
+      <x:c r="B13" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C12" s="20" t="str">
+      <x:c r="C13" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D12" s="20" t="str">
+      <x:c r="D13" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E12" s="20" t="str">
+      <x:c r="E13" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F12" s="20" t="str">
+      <x:c r="F13" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G12" s="20" t="str">
+      <x:c r="G13" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H12" s="20" t="str">
+      <x:c r="H13" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I12" s="20" t="str">
+      <x:c r="I13" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J12" s="20" t="str">
+      <x:c r="J13" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K12" s="20" t="str">
+      <x:c r="K13" s="20" t="str">
         <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B13" s="22" t="str">
-        <x:v>8月3日-8月7日</x:v>
-      </x:c>
-      <x:c r="C13" s="23" t="n">
-        <x:v>7457.12</x:v>
-      </x:c>
-      <x:c r="D13" s="23" t="n">
-        <x:v>7983.17</x:v>
-      </x:c>
-      <x:c r="E13" s="23" t="n">
-        <x:v>7397.94</x:v>
-      </x:c>
-      <x:c r="F13" s="23" t="n">
-        <x:v>7980.12</x:v>
-      </x:c>
-      <x:c r="G13" s="23"/>
-      <x:c r="H13" s="24"/>
-      <x:c r="I13" s="26" t="n">
-        <x:f>ROUND(D13-E13,1)</x:f>
-        <x:v>585.2</x:v>
-      </x:c>
-      <x:c r="J13" s="22" t="str">
-        <x:v>中证500</x:v>
-      </x:c>
-      <x:c r="K13" s="22" t="n">
-        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="B14" s="22" t="str">
-        <x:v>8月10日-8月14日</x:v>
+        <x:v>8月3日-8月7日</x:v>
       </x:c>
       <x:c r="C14" s="23" t="n">
-        <x:v>8003.92</x:v>
+        <x:v>7457.12</x:v>
       </x:c>
       <x:c r="D14" s="23" t="n">
-        <x:v>8142.33</x:v>
+        <x:v>7983.17</x:v>
       </x:c>
       <x:c r="E14" s="23" t="n">
-        <x:v>7897.24</x:v>
+        <x:v>7397.94</x:v>
       </x:c>
       <x:c r="F14" s="23" t="n">
-        <x:v>7990.33</x:v>
-      </x:c>
-      <x:c r="G14" s="23" t="n">
-        <x:f>ROUND(F14-F13,1)</x:f>
-        <x:v>10.2</x:v>
-      </x:c>
-      <x:c r="H14" s="24" t="n">
-        <x:f>IFERROR(F14/F13-1,"")</x:f>
-        <x:v>0.0012794293820144187</x:v>
-      </x:c>
+        <x:v>7980.12</x:v>
+      </x:c>
+      <x:c r="G14" s="23"/>
+      <x:c r="H14" s="24"/>
       <x:c r="I14" s="26" t="n">
         <x:f>ROUND(D14-E14,1)</x:f>
-        <x:v>245.1</x:v>
+        <x:v>585.2</x:v>
       </x:c>
       <x:c r="J14" s="22" t="str">
         <x:v>中证500</x:v>
@@ -1864,34 +1900,34 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="B15" s="22" t="str">
-        <x:v>8月17日-8月21日</x:v>
+        <x:v>8月10日-8月14日</x:v>
       </x:c>
       <x:c r="C15" s="23" t="n">
-        <x:v>8007.87</x:v>
+        <x:v>8003.92</x:v>
       </x:c>
       <x:c r="D15" s="23" t="n">
-        <x:v>8211.31</x:v>
+        <x:v>8142.33</x:v>
       </x:c>
       <x:c r="E15" s="23" t="n">
-        <x:v>7756.28</x:v>
+        <x:v>7897.24</x:v>
       </x:c>
       <x:c r="F15" s="23" t="n">
-        <x:v>7854.33</x:v>
+        <x:v>7990.33</x:v>
       </x:c>
       <x:c r="G15" s="23" t="n">
         <x:f>ROUND(F15-F14,1)</x:f>
-        <x:v>-136</x:v>
+        <x:v>10.2</x:v>
       </x:c>
       <x:c r="H15" s="24" t="n">
         <x:f>IFERROR(F15/F14-1,"")</x:f>
-        <x:v>-0.01702057361836118</x:v>
+        <x:v>0.0012794293820144187</x:v>
       </x:c>
       <x:c r="I15" s="26" t="n">
         <x:f>ROUND(D15-E15,1)</x:f>
-        <x:v>455</x:v>
+        <x:v>245.1</x:v>
       </x:c>
       <x:c r="J15" s="22" t="str">
         <x:v>中证500</x:v>
@@ -1901,193 +1937,193 @@
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="31" t="str">
+      <x:c r="A16" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B16" s="22" t="str">
+        <x:v>8月17日-8月21日</x:v>
+      </x:c>
+      <x:c r="C16" s="23" t="n">
+        <x:v>8007.87</x:v>
+      </x:c>
+      <x:c r="D16" s="23" t="n">
+        <x:v>8211.31</x:v>
+      </x:c>
+      <x:c r="E16" s="23" t="n">
+        <x:v>7756.28</x:v>
+      </x:c>
+      <x:c r="F16" s="23" t="n">
+        <x:v>7854.33</x:v>
+      </x:c>
+      <x:c r="G16" s="23" t="n">
+        <x:f>ROUND(F16-F15,1)</x:f>
+        <x:v>-136</x:v>
+      </x:c>
+      <x:c r="H16" s="24" t="n">
+        <x:f>IFERROR(F16/F15-1,"")</x:f>
+        <x:v>-0.01702057361836118</x:v>
+      </x:c>
+      <x:c r="I16" s="26" t="n">
+        <x:f>ROUND(D16-E16,1)</x:f>
+        <x:v>455</x:v>
+      </x:c>
+      <x:c r="J16" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+      <x:c r="K16" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B17" s="22" t="str">
+        <x:v>8月24日</x:v>
+      </x:c>
+      <x:c r="C17" s="23" t="n">
+        <x:v>7861.05</x:v>
+      </x:c>
+      <x:c r="D17" s="23" t="n">
+        <x:v>7865.54</x:v>
+      </x:c>
+      <x:c r="E17" s="23" t="n">
+        <x:v>7615.45</x:v>
+      </x:c>
+      <x:c r="F17" s="23" t="n">
+        <x:v>7717.09</x:v>
+      </x:c>
+      <x:c r="G17" s="23" t="n">
+        <x:f>ROUND(F17-F16,1)</x:f>
+        <x:v>-137.2</x:v>
+      </x:c>
+      <x:c r="H17" s="24" t="n">
+        <x:f>IFERROR(F17/F16-1,"")</x:f>
+        <x:v>-0.017473164483794212</x:v>
+      </x:c>
+      <x:c r="I17" s="26" t="n">
+        <x:f>ROUND(D17-E17,1)</x:f>
+        <x:v>250.1</x:v>
+      </x:c>
+      <x:c r="J17" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+      <x:c r="K17" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B16" s="30" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C16" s="30"/>
-      <x:c r="D16" s="30"/>
-      <x:c r="E16" s="30"/>
-      <x:c r="F16" s="30"/>
-      <x:c r="G16" s="30"/>
-      <x:c r="H16" s="30"/>
-      <x:c r="I16" s="32" t="n">
-        <x:f>ROUND(SUM(I13:I15),1)</x:f>
-        <x:v>1285.3</x:v>
-      </x:c>
-      <x:c r="J16" s="30"/>
-      <x:c r="K16" s="30"/>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="31" t="str">
+      <x:c r="B18" s="30" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C18" s="30"/>
+      <x:c r="D18" s="30"/>
+      <x:c r="E18" s="30"/>
+      <x:c r="F18" s="30"/>
+      <x:c r="G18" s="30"/>
+      <x:c r="H18" s="30"/>
+      <x:c r="I18" s="32" t="n">
+        <x:f>ROUND(SUM(I14:I17),1)</x:f>
+        <x:v>1535.4</x:v>
+      </x:c>
+      <x:c r="J18" s="30"/>
+      <x:c r="K18" s="30"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B17" s="30"/>
-      <x:c r="C17" s="30"/>
-      <x:c r="D17" s="30"/>
-      <x:c r="E17" s="30"/>
-      <x:c r="F17" s="30"/>
-      <x:c r="G17" s="30"/>
-      <x:c r="H17" s="30"/>
-      <x:c r="I17" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I13:I15),0),1)</x:f>
-        <x:v>428.4</x:v>
-      </x:c>
-      <x:c r="J17" s="30"/>
-      <x:c r="K17" s="30"/>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="17" t="str">
+      <x:c r="B19" s="30"/>
+      <x:c r="C19" s="30"/>
+      <x:c r="D19" s="30"/>
+      <x:c r="E19" s="30"/>
+      <x:c r="F19" s="30"/>
+      <x:c r="G19" s="30"/>
+      <x:c r="H19" s="30"/>
+      <x:c r="I19" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I14:I17),0),1)</x:f>
+        <x:v>383.9</x:v>
+      </x:c>
+      <x:c r="J19" s="30"/>
+      <x:c r="K19" s="30"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="17" t="str">
         <x:v>上证指数</x:v>
       </x:c>
-      <x:c r="B19" s="17"/>
-      <x:c r="C19" s="17"/>
-      <x:c r="D19" s="17"/>
-      <x:c r="E19" s="17"/>
-      <x:c r="F19" s="17"/>
-      <x:c r="G19" s="17"/>
-      <x:c r="H19" s="17"/>
-      <x:c r="I19" s="17"/>
-      <x:c r="J19" s="17"/>
-      <x:c r="K19" s="17"/>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="20" t="str">
+      <x:c r="B21" s="17"/>
+      <x:c r="C21" s="17"/>
+      <x:c r="D21" s="17"/>
+      <x:c r="E21" s="17"/>
+      <x:c r="F21" s="17"/>
+      <x:c r="G21" s="17"/>
+      <x:c r="H21" s="17"/>
+      <x:c r="I21" s="17"/>
+      <x:c r="J21" s="17"/>
+      <x:c r="K21" s="17"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B20" s="20" t="str">
+      <x:c r="B22" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C20" s="20" t="str">
+      <x:c r="C22" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D20" s="20" t="str">
+      <x:c r="D22" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E20" s="20" t="str">
+      <x:c r="E22" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F20" s="20" t="str">
+      <x:c r="F22" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G20" s="20" t="str">
+      <x:c r="G22" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H20" s="20" t="str">
+      <x:c r="H22" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I20" s="20" t="str">
+      <x:c r="I22" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J20" s="20" t="str">
+      <x:c r="J22" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K20" s="20" t="str">
+      <x:c r="K22" s="20" t="str">
         <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B21" s="22" t="str">
-        <x:v>8月3日-8月7日</x:v>
-      </x:c>
-      <x:c r="C21" s="23" t="n">
-        <x:v>3812.61</x:v>
-      </x:c>
-      <x:c r="D21" s="23" t="n">
-        <x:v>3940.93</x:v>
-      </x:c>
-      <x:c r="E21" s="23" t="n">
-        <x:v>3797.64</x:v>
-      </x:c>
-      <x:c r="F21" s="23" t="n">
-        <x:v>3940.04</x:v>
-      </x:c>
-      <x:c r="G21" s="23"/>
-      <x:c r="H21" s="24"/>
-      <x:c r="I21" s="26" t="n">
-        <x:f>ROUND(D21-E21,1)</x:f>
-        <x:v>143.3</x:v>
-      </x:c>
-      <x:c r="J21" s="22" t="str">
-        <x:v>上证指数</x:v>
-      </x:c>
-      <x:c r="K21" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="22" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B22" s="22" t="str">
-        <x:v>8月10日-8月14日</x:v>
-      </x:c>
-      <x:c r="C22" s="23" t="n">
-        <x:v>3943.82</x:v>
-      </x:c>
-      <x:c r="D22" s="23" t="n">
-        <x:v>3968.48</x:v>
-      </x:c>
-      <x:c r="E22" s="23" t="n">
-        <x:v>3903.7</x:v>
-      </x:c>
-      <x:c r="F22" s="23" t="n">
-        <x:v>3927.18</x:v>
-      </x:c>
-      <x:c r="G22" s="23" t="n">
-        <x:f>ROUND(F22-F21,1)</x:f>
-        <x:v>-12.9</x:v>
-      </x:c>
-      <x:c r="H22" s="24" t="n">
-        <x:f>IFERROR(F22/F21-1,"")</x:f>
-        <x:v>-0.003263926254555849</x:v>
-      </x:c>
-      <x:c r="I22" s="26" t="n">
-        <x:f>ROUND(D22-E22,1)</x:f>
-        <x:v>64.8</x:v>
-      </x:c>
-      <x:c r="J22" s="22" t="str">
-        <x:v>上证指数</x:v>
-      </x:c>
-      <x:c r="K22" s="22" t="n">
-        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="B23" s="22" t="str">
-        <x:v>8月17日-8月21日</x:v>
+        <x:v>8月3日-8月7日</x:v>
       </x:c>
       <x:c r="C23" s="23" t="n">
-        <x:v>3930.1</x:v>
+        <x:v>3812.61</x:v>
       </x:c>
       <x:c r="D23" s="23" t="n">
-        <x:v>3994.18</x:v>
+        <x:v>3940.93</x:v>
       </x:c>
       <x:c r="E23" s="23" t="n">
-        <x:v>3879.58</x:v>
+        <x:v>3797.64</x:v>
       </x:c>
       <x:c r="F23" s="23" t="n">
-        <x:v>3905.2</x:v>
-      </x:c>
-      <x:c r="G23" s="23" t="n">
-        <x:f>ROUND(F23-F22,1)</x:f>
-        <x:v>-22</x:v>
-      </x:c>
-      <x:c r="H23" s="24" t="n">
-        <x:f>IFERROR(F23/F22-1,"")</x:f>
-        <x:v>-0.00559689140808417</x:v>
-      </x:c>
+        <x:v>3940.04</x:v>
+      </x:c>
+      <x:c r="G23" s="23"/>
+      <x:c r="H23" s="24"/>
       <x:c r="I23" s="26" t="n">
         <x:f>ROUND(D23-E23,1)</x:f>
-        <x:v>114.6</x:v>
+        <x:v>143.3</x:v>
       </x:c>
       <x:c r="J23" s="22" t="str">
         <x:v>上证指数</x:v>
@@ -2097,1034 +2133,1300 @@
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="31" t="str">
+      <x:c r="A24" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B24" s="22" t="str">
+        <x:v>8月10日-8月14日</x:v>
+      </x:c>
+      <x:c r="C24" s="23" t="n">
+        <x:v>3943.82</x:v>
+      </x:c>
+      <x:c r="D24" s="23" t="n">
+        <x:v>3968.48</x:v>
+      </x:c>
+      <x:c r="E24" s="23" t="n">
+        <x:v>3903.7</x:v>
+      </x:c>
+      <x:c r="F24" s="23" t="n">
+        <x:v>3927.18</x:v>
+      </x:c>
+      <x:c r="G24" s="23" t="n">
+        <x:f>ROUND(F24-F23,1)</x:f>
+        <x:v>-12.9</x:v>
+      </x:c>
+      <x:c r="H24" s="24" t="n">
+        <x:f>IFERROR(F24/F23-1,"")</x:f>
+        <x:v>-0.003263926254555849</x:v>
+      </x:c>
+      <x:c r="I24" s="26" t="n">
+        <x:f>ROUND(D24-E24,1)</x:f>
+        <x:v>64.8</x:v>
+      </x:c>
+      <x:c r="J24" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="K24" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B25" s="22" t="str">
+        <x:v>8月17日-8月21日</x:v>
+      </x:c>
+      <x:c r="C25" s="23" t="n">
+        <x:v>3930.1</x:v>
+      </x:c>
+      <x:c r="D25" s="23" t="n">
+        <x:v>3994.18</x:v>
+      </x:c>
+      <x:c r="E25" s="23" t="n">
+        <x:v>3879.58</x:v>
+      </x:c>
+      <x:c r="F25" s="23" t="n">
+        <x:v>3905.2</x:v>
+      </x:c>
+      <x:c r="G25" s="23" t="n">
+        <x:f>ROUND(F25-F24,1)</x:f>
+        <x:v>-22</x:v>
+      </x:c>
+      <x:c r="H25" s="24" t="n">
+        <x:f>IFERROR(F25/F24-1,"")</x:f>
+        <x:v>-0.00559689140808417</x:v>
+      </x:c>
+      <x:c r="I25" s="26" t="n">
+        <x:f>ROUND(D25-E25,1)</x:f>
+        <x:v>114.6</x:v>
+      </x:c>
+      <x:c r="J25" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="K25" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B26" s="22" t="str">
+        <x:v>8月24日</x:v>
+      </x:c>
+      <x:c r="C26" s="23" t="n">
+        <x:v>3902.7</x:v>
+      </x:c>
+      <x:c r="D26" s="23" t="n">
+        <x:v>3910.24</x:v>
+      </x:c>
+      <x:c r="E26" s="23" t="n">
+        <x:v>3855.35</x:v>
+      </x:c>
+      <x:c r="F26" s="23" t="n">
+        <x:v>3882.01</x:v>
+      </x:c>
+      <x:c r="G26" s="23" t="n">
+        <x:f>ROUND(F26-F25,1)</x:f>
+        <x:v>-23.2</x:v>
+      </x:c>
+      <x:c r="H26" s="24" t="n">
+        <x:f>IFERROR(F26/F25-1,"")</x:f>
+        <x:v>-0.005938236197889912</x:v>
+      </x:c>
+      <x:c r="I26" s="26" t="n">
+        <x:f>ROUND(D26-E26,1)</x:f>
+        <x:v>54.9</x:v>
+      </x:c>
+      <x:c r="J26" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="K26" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B24" s="30" t="n">
+      <x:c r="B27" s="30" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C27" s="30"/>
+      <x:c r="D27" s="30"/>
+      <x:c r="E27" s="30"/>
+      <x:c r="F27" s="30"/>
+      <x:c r="G27" s="30"/>
+      <x:c r="H27" s="30"/>
+      <x:c r="I27" s="32" t="n">
+        <x:f>ROUND(SUM(I23:I26),1)</x:f>
+        <x:v>377.6</x:v>
+      </x:c>
+      <x:c r="J27" s="30"/>
+      <x:c r="K27" s="30"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B28" s="30"/>
+      <x:c r="C28" s="30"/>
+      <x:c r="D28" s="30"/>
+      <x:c r="E28" s="30"/>
+      <x:c r="F28" s="30"/>
+      <x:c r="G28" s="30"/>
+      <x:c r="H28" s="30"/>
+      <x:c r="I28" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I23:I26),0),1)</x:f>
+        <x:v>94.4</x:v>
+      </x:c>
+      <x:c r="J28" s="30"/>
+      <x:c r="K28" s="30"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="17" t="str">
+        <x:v>IM主力</x:v>
+      </x:c>
+      <x:c r="B30" s="17"/>
+      <x:c r="C30" s="17"/>
+      <x:c r="D30" s="17"/>
+      <x:c r="E30" s="17"/>
+      <x:c r="F30" s="17"/>
+      <x:c r="G30" s="17"/>
+      <x:c r="H30" s="17"/>
+      <x:c r="I30" s="17"/>
+      <x:c r="J30" s="17"/>
+      <x:c r="K30" s="17"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="20" t="str">
+        <x:v>序号</x:v>
+      </x:c>
+      <x:c r="B31" s="20" t="str">
+        <x:v>周期</x:v>
+      </x:c>
+      <x:c r="C31" s="20" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="D31" s="20" t="str">
+        <x:v>高点</x:v>
+      </x:c>
+      <x:c r="E31" s="20" t="str">
+        <x:v>低点</x:v>
+      </x:c>
+      <x:c r="F31" s="20" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="G31" s="20" t="str">
+        <x:v>涨跌点数</x:v>
+      </x:c>
+      <x:c r="H31" s="20" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I31" s="20" t="str">
+        <x:v>振幅</x:v>
+      </x:c>
+      <x:c r="J31" s="20" t="str">
+        <x:v>标的</x:v>
+      </x:c>
+      <x:c r="K31" s="20" t="str">
+        <x:v>交易日</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B32" s="22" t="str">
+        <x:v>8月3日-8月7日</x:v>
+      </x:c>
+      <x:c r="C32" s="23" t="n">
+        <x:v>7000</x:v>
+      </x:c>
+      <x:c r="D32" s="23" t="n">
+        <x:v>7594.2</x:v>
+      </x:c>
+      <x:c r="E32" s="23" t="n">
+        <x:v>6976</x:v>
+      </x:c>
+      <x:c r="F32" s="23" t="n">
+        <x:v>7590.6</x:v>
+      </x:c>
+      <x:c r="G32" s="23"/>
+      <x:c r="H32" s="24"/>
+      <x:c r="I32" s="26" t="n">
+        <x:f>ROUND(D32-E32,1)</x:f>
+        <x:v>618.2</x:v>
+      </x:c>
+      <x:c r="J32" s="22" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+      <x:c r="K32" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B33" s="22" t="str">
+        <x:v>8月10日-8月14日</x:v>
+      </x:c>
+      <x:c r="C33" s="23" t="n">
+        <x:v>7628.8</x:v>
+      </x:c>
+      <x:c r="D33" s="23" t="n">
+        <x:v>7776</x:v>
+      </x:c>
+      <x:c r="E33" s="23" t="n">
+        <x:v>7525</x:v>
+      </x:c>
+      <x:c r="F33" s="23" t="n">
+        <x:v>7650.2</x:v>
+      </x:c>
+      <x:c r="G33" s="23" t="n">
+        <x:f>ROUND(F33-F32,1)</x:f>
+        <x:v>59.6</x:v>
+      </x:c>
+      <x:c r="H33" s="24" t="n">
+        <x:f>IFERROR(F33/F32-1,"")</x:f>
+        <x:v>0.007851816720680693</x:v>
+      </x:c>
+      <x:c r="I33" s="26" t="n">
+        <x:f>ROUND(D33-E33,1)</x:f>
+        <x:v>251</x:v>
+      </x:c>
+      <x:c r="J33" s="22" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+      <x:c r="K33" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="22" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C24" s="30"/>
-      <x:c r="D24" s="30"/>
-      <x:c r="E24" s="30"/>
-      <x:c r="F24" s="30"/>
-      <x:c r="G24" s="30"/>
-      <x:c r="H24" s="30"/>
-      <x:c r="I24" s="32" t="n">
-        <x:f>ROUND(SUM(I21:I23),1)</x:f>
-        <x:v>322.7</x:v>
-      </x:c>
-      <x:c r="J24" s="30"/>
-      <x:c r="K24" s="30"/>
-    </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="31" t="str">
+      <x:c r="B34" s="22" t="str">
+        <x:v>8月17日-8月21日</x:v>
+      </x:c>
+      <x:c r="C34" s="23" t="n">
+        <x:v>7675</x:v>
+      </x:c>
+      <x:c r="D34" s="23" t="n">
+        <x:v>7882.8</x:v>
+      </x:c>
+      <x:c r="E34" s="23" t="n">
+        <x:v>7410</x:v>
+      </x:c>
+      <x:c r="F34" s="23" t="n">
+        <x:v>7527</x:v>
+      </x:c>
+      <x:c r="G34" s="23" t="n">
+        <x:f>ROUND(F34-F33,1)</x:f>
+        <x:v>-123.2</x:v>
+      </x:c>
+      <x:c r="H34" s="24" t="n">
+        <x:f>IFERROR(F34/F33-1,"")</x:f>
+        <x:v>-0.016104154139761073</x:v>
+      </x:c>
+      <x:c r="I34" s="26" t="n">
+        <x:f>ROUND(D34-E34,1)</x:f>
+        <x:v>472.8</x:v>
+      </x:c>
+      <x:c r="J34" s="22" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+      <x:c r="K34" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="31" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B35" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C35" s="30"/>
+      <x:c r="D35" s="30"/>
+      <x:c r="E35" s="30"/>
+      <x:c r="F35" s="30"/>
+      <x:c r="G35" s="30"/>
+      <x:c r="H35" s="30"/>
+      <x:c r="I35" s="32" t="n">
+        <x:f>ROUND(SUM(I32:I34),1)</x:f>
+        <x:v>1342</x:v>
+      </x:c>
+      <x:c r="J35" s="30"/>
+      <x:c r="K35" s="30"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B25" s="30"/>
-      <x:c r="C25" s="30"/>
-      <x:c r="D25" s="30"/>
-      <x:c r="E25" s="30"/>
-      <x:c r="F25" s="30"/>
-      <x:c r="G25" s="30"/>
-      <x:c r="H25" s="30"/>
-      <x:c r="I25" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I21:I23),0),1)</x:f>
-        <x:v>107.6</x:v>
-      </x:c>
-      <x:c r="J25" s="30"/>
-      <x:c r="K25" s="30"/>
-    </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="17" t="str">
-        <x:v>IM主力</x:v>
-      </x:c>
-      <x:c r="B27" s="17"/>
-      <x:c r="C27" s="17"/>
-      <x:c r="D27" s="17"/>
-      <x:c r="E27" s="17"/>
-      <x:c r="F27" s="17"/>
-      <x:c r="G27" s="17"/>
-      <x:c r="H27" s="17"/>
-      <x:c r="I27" s="17"/>
-      <x:c r="J27" s="17"/>
-      <x:c r="K27" s="17"/>
-    </x:row>
-    <x:row r="28">
-      <x:c r="A28" s="20" t="str">
+      <x:c r="B36" s="30"/>
+      <x:c r="C36" s="30"/>
+      <x:c r="D36" s="30"/>
+      <x:c r="E36" s="30"/>
+      <x:c r="F36" s="30"/>
+      <x:c r="G36" s="30"/>
+      <x:c r="H36" s="30"/>
+      <x:c r="I36" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I32:I34),0),1)</x:f>
+        <x:v>447.3</x:v>
+      </x:c>
+      <x:c r="J36" s="30"/>
+      <x:c r="K36" s="30"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="17" t="str">
+        <x:v>IC主力</x:v>
+      </x:c>
+      <x:c r="B38" s="17"/>
+      <x:c r="C38" s="17"/>
+      <x:c r="D38" s="17"/>
+      <x:c r="E38" s="17"/>
+      <x:c r="F38" s="17"/>
+      <x:c r="G38" s="17"/>
+      <x:c r="H38" s="17"/>
+      <x:c r="I38" s="17"/>
+      <x:c r="J38" s="17"/>
+      <x:c r="K38" s="17"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B28" s="20" t="str">
+      <x:c r="B39" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C28" s="20" t="str">
+      <x:c r="C39" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D28" s="20" t="str">
+      <x:c r="D39" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E28" s="20" t="str">
+      <x:c r="E39" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F28" s="20" t="str">
+      <x:c r="F39" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G28" s="20" t="str">
+      <x:c r="G39" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H28" s="20" t="str">
+      <x:c r="H39" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I28" s="20" t="str">
+      <x:c r="I39" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J28" s="20" t="str">
+      <x:c r="J39" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K28" s="20" t="str">
+      <x:c r="K39" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="29">
-      <x:c r="A29" s="22" t="n">
+    <x:row r="40">
+      <x:c r="A40" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B29" s="22" t="str">
+      <x:c r="B40" s="22" t="str">
         <x:v>8月3日-8月7日</x:v>
       </x:c>
-      <x:c r="C29" s="23" t="n">
-        <x:v>7000</x:v>
-      </x:c>
-      <x:c r="D29" s="23" t="n">
-        <x:v>7594.2</x:v>
-      </x:c>
-      <x:c r="E29" s="23" t="n">
-        <x:v>6976</x:v>
-      </x:c>
-      <x:c r="F29" s="23" t="n">
-        <x:v>7590.6</x:v>
-      </x:c>
-      <x:c r="G29" s="23"/>
-      <x:c r="H29" s="24"/>
-      <x:c r="I29" s="26" t="n">
-        <x:f>ROUND(D29-E29,1)</x:f>
-        <x:v>618.2</x:v>
-      </x:c>
-      <x:c r="J29" s="22" t="str">
-        <x:v>IM2609</x:v>
-      </x:c>
-      <x:c r="K29" s="22" t="n">
+      <x:c r="C40" s="23" t="n">
+        <x:v>7391</x:v>
+      </x:c>
+      <x:c r="D40" s="23" t="n">
+        <x:v>7882.6</x:v>
+      </x:c>
+      <x:c r="E40" s="23" t="n">
+        <x:v>7335</x:v>
+      </x:c>
+      <x:c r="F40" s="23" t="n">
+        <x:v>7877.8</x:v>
+      </x:c>
+      <x:c r="G40" s="23"/>
+      <x:c r="H40" s="24"/>
+      <x:c r="I40" s="26" t="n">
+        <x:f>ROUND(D40-E40,1)</x:f>
+        <x:v>547.6</x:v>
+      </x:c>
+      <x:c r="J40" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+      <x:c r="K40" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="30">
-      <x:c r="A30" s="22" t="n">
+    <x:row r="41">
+      <x:c r="A41" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B30" s="22" t="str">
+      <x:c r="B41" s="22" t="str">
         <x:v>8月10日-8月14日</x:v>
       </x:c>
-      <x:c r="C30" s="23" t="n">
-        <x:v>7628.8</x:v>
-      </x:c>
-      <x:c r="D30" s="23" t="n">
-        <x:v>7776</x:v>
-      </x:c>
-      <x:c r="E30" s="23" t="n">
-        <x:v>7525</x:v>
-      </x:c>
-      <x:c r="F30" s="23" t="n">
-        <x:v>7650.2</x:v>
-      </x:c>
-      <x:c r="G30" s="23" t="n">
-        <x:f>ROUND(F30-F29,1)</x:f>
-        <x:v>59.6</x:v>
-      </x:c>
-      <x:c r="H30" s="24" t="n">
-        <x:f>IFERROR(F30/F29-1,"")</x:f>
-        <x:v>0.007851816720680693</x:v>
-      </x:c>
-      <x:c r="I30" s="26" t="n">
-        <x:f>ROUND(D30-E30,1)</x:f>
-        <x:v>251</x:v>
-      </x:c>
-      <x:c r="J30" s="22" t="str">
-        <x:v>IM2609</x:v>
-      </x:c>
-      <x:c r="K30" s="22" t="n">
+      <x:c r="C41" s="23" t="n">
+        <x:v>7888</x:v>
+      </x:c>
+      <x:c r="D41" s="23" t="n">
+        <x:v>8024</x:v>
+      </x:c>
+      <x:c r="E41" s="23" t="n">
+        <x:v>7795.8</x:v>
+      </x:c>
+      <x:c r="F41" s="23" t="n">
+        <x:v>7861.2</x:v>
+      </x:c>
+      <x:c r="G41" s="23" t="n">
+        <x:f>ROUND(F41-F40,1)</x:f>
+        <x:v>-16.6</x:v>
+      </x:c>
+      <x:c r="H41" s="24" t="n">
+        <x:f>IFERROR(F41/F40-1,"")</x:f>
+        <x:v>-0.0021071872857905127</x:v>
+      </x:c>
+      <x:c r="I41" s="26" t="n">
+        <x:f>ROUND(D41-E41,1)</x:f>
+        <x:v>228.2</x:v>
+      </x:c>
+      <x:c r="J41" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+      <x:c r="K41" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="31">
-      <x:c r="A31" s="22" t="n">
+    <x:row r="42">
+      <x:c r="A42" s="22" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B31" s="22" t="str">
+      <x:c r="B42" s="22" t="str">
         <x:v>8月17日-8月21日</x:v>
       </x:c>
-      <x:c r="C31" s="23" t="n">
-        <x:v>7675</x:v>
-      </x:c>
-      <x:c r="D31" s="23" t="n">
-        <x:v>7882.8</x:v>
-      </x:c>
-      <x:c r="E31" s="23" t="n">
-        <x:v>7410</x:v>
-      </x:c>
-      <x:c r="F31" s="23" t="n">
-        <x:v>7527</x:v>
-      </x:c>
-      <x:c r="G31" s="23" t="n">
-        <x:f>ROUND(F31-F30,1)</x:f>
-        <x:v>-123.2</x:v>
-      </x:c>
-      <x:c r="H31" s="24" t="n">
-        <x:f>IFERROR(F31/F30-1,"")</x:f>
-        <x:v>-0.016104154139761073</x:v>
-      </x:c>
-      <x:c r="I31" s="26" t="n">
-        <x:f>ROUND(D31-E31,1)</x:f>
-        <x:v>472.8</x:v>
-      </x:c>
-      <x:c r="J31" s="22" t="str">
-        <x:v>IM2609</x:v>
-      </x:c>
-      <x:c r="K31" s="22" t="n">
+      <x:c r="C42" s="23" t="n">
+        <x:v>7885</x:v>
+      </x:c>
+      <x:c r="D42" s="23" t="n">
+        <x:v>8091.8</x:v>
+      </x:c>
+      <x:c r="E42" s="23" t="n">
+        <x:v>7669.6</x:v>
+      </x:c>
+      <x:c r="F42" s="23" t="n">
+        <x:v>7762</x:v>
+      </x:c>
+      <x:c r="G42" s="23" t="n">
+        <x:f>ROUND(F42-F41,1)</x:f>
+        <x:v>-99.2</x:v>
+      </x:c>
+      <x:c r="H42" s="24" t="n">
+        <x:f>IFERROR(F42/F41-1,"")</x:f>
+        <x:v>-0.012618938584439965</x:v>
+      </x:c>
+      <x:c r="I42" s="26" t="n">
+        <x:f>ROUND(D42-E42,1)</x:f>
+        <x:v>422.2</x:v>
+      </x:c>
+      <x:c r="J42" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+      <x:c r="K42" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="32">
-      <x:c r="A32" s="31" t="str">
+    <x:row r="43">
+      <x:c r="A43" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B43" s="22" t="str">
+        <x:v>8月24日</x:v>
+      </x:c>
+      <x:c r="C43" s="23" t="n">
+        <x:v>7757</x:v>
+      </x:c>
+      <x:c r="D43" s="23" t="n">
+        <x:v>7764.4</x:v>
+      </x:c>
+      <x:c r="E43" s="23" t="n">
+        <x:v>7514.4</x:v>
+      </x:c>
+      <x:c r="F43" s="23" t="n">
+        <x:v>7628.4</x:v>
+      </x:c>
+      <x:c r="G43" s="23" t="n">
+        <x:f>ROUND(F43-F42,1)</x:f>
+        <x:v>-133.6</x:v>
+      </x:c>
+      <x:c r="H43" s="24" t="n">
+        <x:f>IFERROR(F43/F42-1,"")</x:f>
+        <x:v>-0.01721205874774545</x:v>
+      </x:c>
+      <x:c r="I43" s="26" t="n">
+        <x:f>ROUND(D43-E43,1)</x:f>
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="J43" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+      <x:c r="K43" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B32" s="30" t="n">
+      <x:c r="B44" s="30" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C44" s="30"/>
+      <x:c r="D44" s="30"/>
+      <x:c r="E44" s="30"/>
+      <x:c r="F44" s="30"/>
+      <x:c r="G44" s="30"/>
+      <x:c r="H44" s="30"/>
+      <x:c r="I44" s="32" t="n">
+        <x:f>ROUND(SUM(I40:I43),1)</x:f>
+        <x:v>1448</x:v>
+      </x:c>
+      <x:c r="J44" s="30"/>
+      <x:c r="K44" s="30"/>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B45" s="30"/>
+      <x:c r="C45" s="30"/>
+      <x:c r="D45" s="30"/>
+      <x:c r="E45" s="30"/>
+      <x:c r="F45" s="30"/>
+      <x:c r="G45" s="30"/>
+      <x:c r="H45" s="30"/>
+      <x:c r="I45" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I40:I43),0),1)</x:f>
+        <x:v>362</x:v>
+      </x:c>
+      <x:c r="J45" s="30"/>
+      <x:c r="K45" s="30"/>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="17" t="str">
+        <x:v>IF主力</x:v>
+      </x:c>
+      <x:c r="B47" s="17"/>
+      <x:c r="C47" s="17"/>
+      <x:c r="D47" s="17"/>
+      <x:c r="E47" s="17"/>
+      <x:c r="F47" s="17"/>
+      <x:c r="G47" s="17"/>
+      <x:c r="H47" s="17"/>
+      <x:c r="I47" s="17"/>
+      <x:c r="J47" s="17"/>
+      <x:c r="K47" s="17"/>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="20" t="str">
+        <x:v>序号</x:v>
+      </x:c>
+      <x:c r="B48" s="20" t="str">
+        <x:v>周期</x:v>
+      </x:c>
+      <x:c r="C48" s="20" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="D48" s="20" t="str">
+        <x:v>高点</x:v>
+      </x:c>
+      <x:c r="E48" s="20" t="str">
+        <x:v>低点</x:v>
+      </x:c>
+      <x:c r="F48" s="20" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="G48" s="20" t="str">
+        <x:v>涨跌点数</x:v>
+      </x:c>
+      <x:c r="H48" s="20" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I48" s="20" t="str">
+        <x:v>振幅</x:v>
+      </x:c>
+      <x:c r="J48" s="20" t="str">
+        <x:v>标的</x:v>
+      </x:c>
+      <x:c r="K48" s="20" t="str">
+        <x:v>交易日</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B49" s="22" t="str">
+        <x:v>8月3日-8月7日</x:v>
+      </x:c>
+      <x:c r="C49" s="23" t="n">
+        <x:v>4526.4</x:v>
+      </x:c>
+      <x:c r="D49" s="23" t="n">
+        <x:v>4656.2</x:v>
+      </x:c>
+      <x:c r="E49" s="23" t="n">
+        <x:v>4494.2</x:v>
+      </x:c>
+      <x:c r="F49" s="23" t="n">
+        <x:v>4645.6</x:v>
+      </x:c>
+      <x:c r="G49" s="23"/>
+      <x:c r="H49" s="24"/>
+      <x:c r="I49" s="26" t="n">
+        <x:f>ROUND(D49-E49,1)</x:f>
+        <x:v>162</x:v>
+      </x:c>
+      <x:c r="J49" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+      <x:c r="K49" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B50" s="22" t="str">
+        <x:v>8月10日-8月14日</x:v>
+      </x:c>
+      <x:c r="C50" s="23" t="n">
+        <x:v>4656.8</x:v>
+      </x:c>
+      <x:c r="D50" s="23" t="n">
+        <x:v>4681</x:v>
+      </x:c>
+      <x:c r="E50" s="23" t="n">
+        <x:v>4598</x:v>
+      </x:c>
+      <x:c r="F50" s="23" t="n">
+        <x:v>4620.4</x:v>
+      </x:c>
+      <x:c r="G50" s="23" t="n">
+        <x:f>ROUND(F50-F49,1)</x:f>
+        <x:v>-25.2</x:v>
+      </x:c>
+      <x:c r="H50" s="24" t="n">
+        <x:f>IFERROR(F50/F49-1,"")</x:f>
+        <x:v>-0.005424487687274104</x:v>
+      </x:c>
+      <x:c r="I50" s="23" t="n">
+        <x:f>ROUND(D50-E50,1)</x:f>
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="J50" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+      <x:c r="K50" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="22" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C32" s="30"/>
-      <x:c r="D32" s="30"/>
-      <x:c r="E32" s="30"/>
-      <x:c r="F32" s="30"/>
-      <x:c r="G32" s="30"/>
-      <x:c r="H32" s="30"/>
-      <x:c r="I32" s="32" t="n">
-        <x:f>ROUND(SUM(I29:I31),1)</x:f>
-        <x:v>1342</x:v>
-      </x:c>
-      <x:c r="J32" s="30"/>
-      <x:c r="K32" s="30"/>
-    </x:row>
-    <x:row r="33">
-      <x:c r="A33" s="31" t="str">
+      <x:c r="B51" s="22" t="str">
+        <x:v>8月17日-8月21日</x:v>
+      </x:c>
+      <x:c r="C51" s="23" t="n">
+        <x:v>4624</x:v>
+      </x:c>
+      <x:c r="D51" s="23" t="n">
+        <x:v>4700.6</x:v>
+      </x:c>
+      <x:c r="E51" s="23" t="n">
+        <x:v>4531.8</x:v>
+      </x:c>
+      <x:c r="F51" s="23" t="n">
+        <x:v>4576</x:v>
+      </x:c>
+      <x:c r="G51" s="23" t="n">
+        <x:f>ROUND(F51-F50,1)</x:f>
+        <x:v>-44.4</x:v>
+      </x:c>
+      <x:c r="H51" s="24" t="n">
+        <x:f>IFERROR(F51/F50-1,"")</x:f>
+        <x:v>-0.00960955761405935</x:v>
+      </x:c>
+      <x:c r="I51" s="26" t="n">
+        <x:f>ROUND(D51-E51,1)</x:f>
+        <x:v>168.8</x:v>
+      </x:c>
+      <x:c r="J51" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+      <x:c r="K51" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B52" s="22" t="str">
+        <x:v>8月24日</x:v>
+      </x:c>
+      <x:c r="C52" s="23" t="n">
+        <x:v>4607.4</x:v>
+      </x:c>
+      <x:c r="D52" s="23" t="n">
+        <x:v>4607.4</x:v>
+      </x:c>
+      <x:c r="E52" s="23" t="n">
+        <x:v>4486.4</x:v>
+      </x:c>
+      <x:c r="F52" s="23" t="n">
+        <x:v>4526.4</x:v>
+      </x:c>
+      <x:c r="G52" s="23" t="n">
+        <x:f>ROUND(F52-F51,1)</x:f>
+        <x:v>-49.6</x:v>
+      </x:c>
+      <x:c r="H52" s="24" t="n">
+        <x:f>IFERROR(F52/F51-1,"")</x:f>
+        <x:v>-0.010839160839160922</x:v>
+      </x:c>
+      <x:c r="I52" s="26" t="n">
+        <x:f>ROUND(D52-E52,1)</x:f>
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="J52" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+      <x:c r="K52" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="31" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B53" s="30" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C53" s="30"/>
+      <x:c r="D53" s="30"/>
+      <x:c r="E53" s="30"/>
+      <x:c r="F53" s="30"/>
+      <x:c r="G53" s="30"/>
+      <x:c r="H53" s="30"/>
+      <x:c r="I53" s="32" t="n">
+        <x:f>ROUND(SUM(I49:I52),1)</x:f>
+        <x:v>534.8</x:v>
+      </x:c>
+      <x:c r="J53" s="30"/>
+      <x:c r="K53" s="30"/>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B33" s="30"/>
-      <x:c r="C33" s="30"/>
-      <x:c r="D33" s="30"/>
-      <x:c r="E33" s="30"/>
-      <x:c r="F33" s="30"/>
-      <x:c r="G33" s="30"/>
-      <x:c r="H33" s="30"/>
-      <x:c r="I33" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I29:I31),0),1)</x:f>
-        <x:v>447.3</x:v>
-      </x:c>
-      <x:c r="J33" s="30"/>
-      <x:c r="K33" s="30"/>
-    </x:row>
-    <x:row r="35">
-      <x:c r="A35" s="17" t="str">
-        <x:v>IC主力</x:v>
-      </x:c>
-      <x:c r="B35" s="17"/>
-      <x:c r="C35" s="17"/>
-      <x:c r="D35" s="17"/>
-      <x:c r="E35" s="17"/>
-      <x:c r="F35" s="17"/>
-      <x:c r="G35" s="17"/>
-      <x:c r="H35" s="17"/>
-      <x:c r="I35" s="17"/>
-      <x:c r="J35" s="17"/>
-      <x:c r="K35" s="17"/>
-    </x:row>
-    <x:row r="36">
-      <x:c r="A36" s="20" t="str">
+      <x:c r="B54" s="30"/>
+      <x:c r="C54" s="30"/>
+      <x:c r="D54" s="30"/>
+      <x:c r="E54" s="30"/>
+      <x:c r="F54" s="30"/>
+      <x:c r="G54" s="30"/>
+      <x:c r="H54" s="30"/>
+      <x:c r="I54" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I49:I52),0),1)</x:f>
+        <x:v>133.7</x:v>
+      </x:c>
+      <x:c r="J54" s="30"/>
+      <x:c r="K54" s="30"/>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="17" t="str">
+        <x:v>IH主力</x:v>
+      </x:c>
+      <x:c r="B56" s="17"/>
+      <x:c r="C56" s="17"/>
+      <x:c r="D56" s="17"/>
+      <x:c r="E56" s="17"/>
+      <x:c r="F56" s="17"/>
+      <x:c r="G56" s="17"/>
+      <x:c r="H56" s="17"/>
+      <x:c r="I56" s="17"/>
+      <x:c r="J56" s="17"/>
+      <x:c r="K56" s="17"/>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B36" s="20" t="str">
+      <x:c r="B57" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C36" s="20" t="str">
+      <x:c r="C57" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D36" s="20" t="str">
+      <x:c r="D57" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E36" s="20" t="str">
+      <x:c r="E57" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F36" s="20" t="str">
+      <x:c r="F57" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G36" s="20" t="str">
+      <x:c r="G57" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H36" s="20" t="str">
+      <x:c r="H57" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I36" s="20" t="str">
+      <x:c r="I57" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J36" s="20" t="str">
+      <x:c r="J57" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K36" s="20" t="str">
+      <x:c r="K57" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="37">
-      <x:c r="A37" s="22" t="n">
+    <x:row r="58">
+      <x:c r="A58" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B37" s="22" t="str">
+      <x:c r="B58" s="22" t="str">
         <x:v>8月3日-8月7日</x:v>
       </x:c>
-      <x:c r="C37" s="23" t="n">
-        <x:v>7391</x:v>
-      </x:c>
-      <x:c r="D37" s="23" t="n">
-        <x:v>7882.6</x:v>
-      </x:c>
-      <x:c r="E37" s="23" t="n">
-        <x:v>7335</x:v>
-      </x:c>
-      <x:c r="F37" s="23" t="n">
-        <x:v>7877.8</x:v>
-      </x:c>
-      <x:c r="G37" s="23"/>
-      <x:c r="H37" s="24"/>
-      <x:c r="I37" s="26" t="n">
-        <x:f>ROUND(D37-E37,1)</x:f>
-        <x:v>547.6</x:v>
-      </x:c>
-      <x:c r="J37" s="22" t="str">
-        <x:v>IC2609</x:v>
-      </x:c>
-      <x:c r="K37" s="22" t="n">
+      <x:c r="C58" s="23" t="n">
+        <x:v>2882.4</x:v>
+      </x:c>
+      <x:c r="D58" s="23" t="n">
+        <x:v>2930.6</x:v>
+      </x:c>
+      <x:c r="E58" s="23" t="n">
+        <x:v>2845.8</x:v>
+      </x:c>
+      <x:c r="F58" s="23" t="n">
+        <x:v>2930</x:v>
+      </x:c>
+      <x:c r="G58" s="23"/>
+      <x:c r="H58" s="24"/>
+      <x:c r="I58" s="26" t="n">
+        <x:f>ROUND(D58-E58,1)</x:f>
+        <x:v>84.8</x:v>
+      </x:c>
+      <x:c r="J58" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+      <x:c r="K58" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="38">
-      <x:c r="A38" s="22" t="n">
+    <x:row r="59">
+      <x:c r="A59" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B38" s="22" t="str">
+      <x:c r="B59" s="22" t="str">
         <x:v>8月10日-8月14日</x:v>
       </x:c>
-      <x:c r="C38" s="23" t="n">
-        <x:v>7888</x:v>
-      </x:c>
-      <x:c r="D38" s="23" t="n">
-        <x:v>8024</x:v>
-      </x:c>
-      <x:c r="E38" s="23" t="n">
-        <x:v>7795.8</x:v>
-      </x:c>
-      <x:c r="F38" s="23" t="n">
-        <x:v>7861.2</x:v>
-      </x:c>
-      <x:c r="G38" s="23" t="n">
-        <x:f>ROUND(F38-F37,1)</x:f>
-        <x:v>-16.6</x:v>
-      </x:c>
-      <x:c r="H38" s="24" t="n">
-        <x:f>IFERROR(F38/F37-1,"")</x:f>
-        <x:v>-0.0021071872857905127</x:v>
-      </x:c>
-      <x:c r="I38" s="26" t="n">
-        <x:f>ROUND(D38-E38,1)</x:f>
-        <x:v>228.2</x:v>
-      </x:c>
-      <x:c r="J38" s="22" t="str">
-        <x:v>IC2609</x:v>
-      </x:c>
-      <x:c r="K38" s="22" t="n">
+      <x:c r="C59" s="23" t="n">
+        <x:v>2930</x:v>
+      </x:c>
+      <x:c r="D59" s="23" t="n">
+        <x:v>2949.6</x:v>
+      </x:c>
+      <x:c r="E59" s="23" t="n">
+        <x:v>2877</x:v>
+      </x:c>
+      <x:c r="F59" s="23" t="n">
+        <x:v>2890</x:v>
+      </x:c>
+      <x:c r="G59" s="23" t="n">
+        <x:f>ROUND(F59-F58,1)</x:f>
+        <x:v>-40</x:v>
+      </x:c>
+      <x:c r="H59" s="24" t="n">
+        <x:f>IFERROR(F59/F58-1,"")</x:f>
+        <x:v>-0.013651877133105783</x:v>
+      </x:c>
+      <x:c r="I59" s="26" t="n">
+        <x:f>ROUND(D59-E59,1)</x:f>
+        <x:v>72.6</x:v>
+      </x:c>
+      <x:c r="J59" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+      <x:c r="K59" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="39">
-      <x:c r="A39" s="22" t="n">
+    <x:row r="60">
+      <x:c r="A60" s="22" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B39" s="22" t="str">
+      <x:c r="B60" s="22" t="str">
         <x:v>8月17日-8月21日</x:v>
       </x:c>
-      <x:c r="C39" s="23" t="n">
-        <x:v>7885</x:v>
-      </x:c>
-      <x:c r="D39" s="23" t="n">
-        <x:v>8091.8</x:v>
-      </x:c>
-      <x:c r="E39" s="23" t="n">
-        <x:v>7669.6</x:v>
-      </x:c>
-      <x:c r="F39" s="23" t="n">
-        <x:v>7762</x:v>
-      </x:c>
-      <x:c r="G39" s="23" t="n">
-        <x:f>ROUND(F39-F38,1)</x:f>
-        <x:v>-99.2</x:v>
-      </x:c>
-      <x:c r="H39" s="24" t="n">
-        <x:f>IFERROR(F39/F38-1,"")</x:f>
-        <x:v>-0.012618938584439965</x:v>
-      </x:c>
-      <x:c r="I39" s="26" t="n">
-        <x:f>ROUND(D39-E39,1)</x:f>
-        <x:v>422.2</x:v>
-      </x:c>
-      <x:c r="J39" s="22" t="str">
-        <x:v>IC2609</x:v>
-      </x:c>
-      <x:c r="K39" s="22" t="n">
+      <x:c r="C60" s="23" t="n">
+        <x:v>2886</x:v>
+      </x:c>
+      <x:c r="D60" s="23" t="n">
+        <x:v>2921.2</x:v>
+      </x:c>
+      <x:c r="E60" s="23" t="n">
+        <x:v>2843</x:v>
+      </x:c>
+      <x:c r="F60" s="23" t="n">
+        <x:v>2861</x:v>
+      </x:c>
+      <x:c r="G60" s="23" t="n">
+        <x:f>ROUND(F60-F59,1)</x:f>
+        <x:v>-29</x:v>
+      </x:c>
+      <x:c r="H60" s="24" t="n">
+        <x:f>IFERROR(F60/F59-1,"")</x:f>
+        <x:v>-0.01003460207612461</x:v>
+      </x:c>
+      <x:c r="I60" s="26" t="n">
+        <x:f>ROUND(D60-E60,1)</x:f>
+        <x:v>78.2</x:v>
+      </x:c>
+      <x:c r="J60" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+      <x:c r="K60" s="22" t="n">
         <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40">
-      <x:c r="A40" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B40" s="30" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C40" s="30"/>
-      <x:c r="D40" s="30"/>
-      <x:c r="E40" s="30"/>
-      <x:c r="F40" s="30"/>
-      <x:c r="G40" s="30"/>
-      <x:c r="H40" s="30"/>
-      <x:c r="I40" s="32" t="n">
-        <x:f>ROUND(SUM(I37:I39),1)</x:f>
-        <x:v>1198</x:v>
-      </x:c>
-      <x:c r="J40" s="30"/>
-      <x:c r="K40" s="30"/>
-    </x:row>
-    <x:row r="41">
-      <x:c r="A41" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B41" s="30"/>
-      <x:c r="C41" s="30"/>
-      <x:c r="D41" s="30"/>
-      <x:c r="E41" s="30"/>
-      <x:c r="F41" s="30"/>
-      <x:c r="G41" s="30"/>
-      <x:c r="H41" s="30"/>
-      <x:c r="I41" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I37:I39),0),1)</x:f>
-        <x:v>399.3</x:v>
-      </x:c>
-      <x:c r="J41" s="30"/>
-      <x:c r="K41" s="30"/>
-    </x:row>
-    <x:row r="43">
-      <x:c r="A43" s="17" t="str">
-        <x:v>IF主力</x:v>
-      </x:c>
-      <x:c r="B43" s="17"/>
-      <x:c r="C43" s="17"/>
-      <x:c r="D43" s="17"/>
-      <x:c r="E43" s="17"/>
-      <x:c r="F43" s="17"/>
-      <x:c r="G43" s="17"/>
-      <x:c r="H43" s="17"/>
-      <x:c r="I43" s="17"/>
-      <x:c r="J43" s="17"/>
-      <x:c r="K43" s="17"/>
-    </x:row>
-    <x:row r="44">
-      <x:c r="A44" s="20" t="str">
-        <x:v>序号</x:v>
-      </x:c>
-      <x:c r="B44" s="20" t="str">
-        <x:v>周期</x:v>
-      </x:c>
-      <x:c r="C44" s="20" t="str">
-        <x:v>开盘</x:v>
-      </x:c>
-      <x:c r="D44" s="20" t="str">
-        <x:v>高点</x:v>
-      </x:c>
-      <x:c r="E44" s="20" t="str">
-        <x:v>低点</x:v>
-      </x:c>
-      <x:c r="F44" s="20" t="str">
-        <x:v>收盘</x:v>
-      </x:c>
-      <x:c r="G44" s="20" t="str">
-        <x:v>涨跌点数</x:v>
-      </x:c>
-      <x:c r="H44" s="20" t="str">
-        <x:v>涨幅</x:v>
-      </x:c>
-      <x:c r="I44" s="20" t="str">
-        <x:v>振幅</x:v>
-      </x:c>
-      <x:c r="J44" s="20" t="str">
-        <x:v>标的</x:v>
-      </x:c>
-      <x:c r="K44" s="20" t="str">
-        <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="45">
-      <x:c r="A45" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B45" s="22" t="str">
-        <x:v>8月3日-8月7日</x:v>
-      </x:c>
-      <x:c r="C45" s="23" t="n">
-        <x:v>4526.4</x:v>
-      </x:c>
-      <x:c r="D45" s="23" t="n">
-        <x:v>4656.2</x:v>
-      </x:c>
-      <x:c r="E45" s="23" t="n">
-        <x:v>4494.2</x:v>
-      </x:c>
-      <x:c r="F45" s="23" t="n">
-        <x:v>4645.6</x:v>
-      </x:c>
-      <x:c r="G45" s="23"/>
-      <x:c r="H45" s="24"/>
-      <x:c r="I45" s="26" t="n">
-        <x:f>ROUND(D45-E45,1)</x:f>
-        <x:v>162</x:v>
-      </x:c>
-      <x:c r="J45" s="22" t="str">
-        <x:v>IF2609</x:v>
-      </x:c>
-      <x:c r="K45" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="46">
-      <x:c r="A46" s="22" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B46" s="22" t="str">
-        <x:v>8月10日-8月14日</x:v>
-      </x:c>
-      <x:c r="C46" s="23" t="n">
-        <x:v>4656.8</x:v>
-      </x:c>
-      <x:c r="D46" s="23" t="n">
-        <x:v>4681</x:v>
-      </x:c>
-      <x:c r="E46" s="23" t="n">
-        <x:v>4598</x:v>
-      </x:c>
-      <x:c r="F46" s="23" t="n">
-        <x:v>4620.4</x:v>
-      </x:c>
-      <x:c r="G46" s="23" t="n">
-        <x:f>ROUND(F46-F45,1)</x:f>
-        <x:v>-25.2</x:v>
-      </x:c>
-      <x:c r="H46" s="24" t="n">
-        <x:f>IFERROR(F46/F45-1,"")</x:f>
-        <x:v>-0.005424487687274104</x:v>
-      </x:c>
-      <x:c r="I46" s="23" t="n">
-        <x:f>ROUND(D46-E46,1)</x:f>
-        <x:v>83</x:v>
-      </x:c>
-      <x:c r="J46" s="22" t="str">
-        <x:v>IF2609</x:v>
-      </x:c>
-      <x:c r="K46" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="47">
-      <x:c r="A47" s="22" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B47" s="22" t="str">
-        <x:v>8月17日-8月21日</x:v>
-      </x:c>
-      <x:c r="C47" s="23" t="n">
-        <x:v>4624</x:v>
-      </x:c>
-      <x:c r="D47" s="23" t="n">
-        <x:v>4700.6</x:v>
-      </x:c>
-      <x:c r="E47" s="23" t="n">
-        <x:v>4531.8</x:v>
-      </x:c>
-      <x:c r="F47" s="23" t="n">
-        <x:v>4576</x:v>
-      </x:c>
-      <x:c r="G47" s="23" t="n">
-        <x:f>ROUND(F47-F46,1)</x:f>
-        <x:v>-44.4</x:v>
-      </x:c>
-      <x:c r="H47" s="24" t="n">
-        <x:f>IFERROR(F47/F46-1,"")</x:f>
-        <x:v>-0.00960955761405935</x:v>
-      </x:c>
-      <x:c r="I47" s="26" t="n">
-        <x:f>ROUND(D47-E47,1)</x:f>
-        <x:v>168.8</x:v>
-      </x:c>
-      <x:c r="J47" s="22" t="str">
-        <x:v>IF2609</x:v>
-      </x:c>
-      <x:c r="K47" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="48">
-      <x:c r="A48" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B48" s="30" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C48" s="30"/>
-      <x:c r="D48" s="30"/>
-      <x:c r="E48" s="30"/>
-      <x:c r="F48" s="30"/>
-      <x:c r="G48" s="30"/>
-      <x:c r="H48" s="30"/>
-      <x:c r="I48" s="32" t="n">
-        <x:f>ROUND(SUM(I45:I47),1)</x:f>
-        <x:v>413.8</x:v>
-      </x:c>
-      <x:c r="J48" s="30"/>
-      <x:c r="K48" s="30"/>
-    </x:row>
-    <x:row r="49">
-      <x:c r="A49" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B49" s="30"/>
-      <x:c r="C49" s="30"/>
-      <x:c r="D49" s="30"/>
-      <x:c r="E49" s="30"/>
-      <x:c r="F49" s="30"/>
-      <x:c r="G49" s="30"/>
-      <x:c r="H49" s="30"/>
-      <x:c r="I49" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I45:I47),0),1)</x:f>
-        <x:v>137.9</x:v>
-      </x:c>
-      <x:c r="J49" s="30"/>
-      <x:c r="K49" s="30"/>
-    </x:row>
-    <x:row r="51">
-      <x:c r="A51" s="17" t="str">
-        <x:v>IH主力</x:v>
-      </x:c>
-      <x:c r="B51" s="17"/>
-      <x:c r="C51" s="17"/>
-      <x:c r="D51" s="17"/>
-      <x:c r="E51" s="17"/>
-      <x:c r="F51" s="17"/>
-      <x:c r="G51" s="17"/>
-      <x:c r="H51" s="17"/>
-      <x:c r="I51" s="17"/>
-      <x:c r="J51" s="17"/>
-      <x:c r="K51" s="17"/>
-    </x:row>
-    <x:row r="52">
-      <x:c r="A52" s="20" t="str">
-        <x:v>序号</x:v>
-      </x:c>
-      <x:c r="B52" s="20" t="str">
-        <x:v>周期</x:v>
-      </x:c>
-      <x:c r="C52" s="20" t="str">
-        <x:v>开盘</x:v>
-      </x:c>
-      <x:c r="D52" s="20" t="str">
-        <x:v>高点</x:v>
-      </x:c>
-      <x:c r="E52" s="20" t="str">
-        <x:v>低点</x:v>
-      </x:c>
-      <x:c r="F52" s="20" t="str">
-        <x:v>收盘</x:v>
-      </x:c>
-      <x:c r="G52" s="20" t="str">
-        <x:v>涨跌点数</x:v>
-      </x:c>
-      <x:c r="H52" s="20" t="str">
-        <x:v>涨幅</x:v>
-      </x:c>
-      <x:c r="I52" s="20" t="str">
-        <x:v>振幅</x:v>
-      </x:c>
-      <x:c r="J52" s="20" t="str">
-        <x:v>标的</x:v>
-      </x:c>
-      <x:c r="K52" s="20" t="str">
-        <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="53">
-      <x:c r="A53" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B53" s="22" t="str">
-        <x:v>8月3日-8月7日</x:v>
-      </x:c>
-      <x:c r="C53" s="23" t="n">
-        <x:v>2882.4</x:v>
-      </x:c>
-      <x:c r="D53" s="23" t="n">
-        <x:v>2930.6</x:v>
-      </x:c>
-      <x:c r="E53" s="23" t="n">
-        <x:v>2845.8</x:v>
-      </x:c>
-      <x:c r="F53" s="23" t="n">
-        <x:v>2930</x:v>
-      </x:c>
-      <x:c r="G53" s="23"/>
-      <x:c r="H53" s="24"/>
-      <x:c r="I53" s="26" t="n">
-        <x:f>ROUND(D53-E53,1)</x:f>
-        <x:v>84.8</x:v>
-      </x:c>
-      <x:c r="J53" s="22" t="str">
-        <x:v>IH2609</x:v>
-      </x:c>
-      <x:c r="K53" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="54">
-      <x:c r="A54" s="22" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B54" s="22" t="str">
-        <x:v>8月10日-8月14日</x:v>
-      </x:c>
-      <x:c r="C54" s="23" t="n">
-        <x:v>2930</x:v>
-      </x:c>
-      <x:c r="D54" s="23" t="n">
-        <x:v>2949.6</x:v>
-      </x:c>
-      <x:c r="E54" s="23" t="n">
-        <x:v>2877</x:v>
-      </x:c>
-      <x:c r="F54" s="23" t="n">
-        <x:v>2890</x:v>
-      </x:c>
-      <x:c r="G54" s="23" t="n">
-        <x:f>ROUND(F54-F53,1)</x:f>
-        <x:v>-40</x:v>
-      </x:c>
-      <x:c r="H54" s="24" t="n">
-        <x:f>IFERROR(F54/F53-1,"")</x:f>
-        <x:v>-0.013651877133105783</x:v>
-      </x:c>
-      <x:c r="I54" s="26" t="n">
-        <x:f>ROUND(D54-E54,1)</x:f>
-        <x:v>72.6</x:v>
-      </x:c>
-      <x:c r="J54" s="22" t="str">
-        <x:v>IH2609</x:v>
-      </x:c>
-      <x:c r="K54" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="55">
-      <x:c r="A55" s="22" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B55" s="22" t="str">
-        <x:v>8月17日-8月21日</x:v>
-      </x:c>
-      <x:c r="C55" s="23" t="n">
-        <x:v>2886</x:v>
-      </x:c>
-      <x:c r="D55" s="23" t="n">
-        <x:v>2921.2</x:v>
-      </x:c>
-      <x:c r="E55" s="23" t="n">
-        <x:v>2843</x:v>
-      </x:c>
-      <x:c r="F55" s="23" t="n">
-        <x:v>2861</x:v>
-      </x:c>
-      <x:c r="G55" s="23" t="n">
-        <x:f>ROUND(F55-F54,1)</x:f>
-        <x:v>-29</x:v>
-      </x:c>
-      <x:c r="H55" s="24" t="n">
-        <x:f>IFERROR(F55/F54-1,"")</x:f>
-        <x:v>-0.01003460207612461</x:v>
-      </x:c>
-      <x:c r="I55" s="26" t="n">
-        <x:f>ROUND(D55-E55,1)</x:f>
-        <x:v>78.2</x:v>
-      </x:c>
-      <x:c r="J55" s="22" t="str">
-        <x:v>IH2609</x:v>
-      </x:c>
-      <x:c r="K55" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="56">
-      <x:c r="A56" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B56" s="30" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C56" s="30"/>
-      <x:c r="D56" s="30"/>
-      <x:c r="E56" s="30"/>
-      <x:c r="F56" s="30"/>
-      <x:c r="G56" s="30"/>
-      <x:c r="H56" s="30"/>
-      <x:c r="I56" s="32" t="n">
-        <x:f>ROUND(SUM(I53:I55),1)</x:f>
-        <x:v>235.6</x:v>
-      </x:c>
-      <x:c r="J56" s="30"/>
-      <x:c r="K56" s="30"/>
-    </x:row>
-    <x:row r="57">
-      <x:c r="A57" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B57" s="30"/>
-      <x:c r="C57" s="30"/>
-      <x:c r="D57" s="30"/>
-      <x:c r="E57" s="30"/>
-      <x:c r="F57" s="30"/>
-      <x:c r="G57" s="30"/>
-      <x:c r="H57" s="30"/>
-      <x:c r="I57" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I53:I55),0),1)</x:f>
-        <x:v>78.5</x:v>
-      </x:c>
-      <x:c r="J57" s="30"/>
-      <x:c r="K57" s="30"/>
-    </x:row>
-    <x:row r="59">
-      <x:c r="A59" s="17" t="str">
-        <x:v>碳酸锂2609</x:v>
-      </x:c>
-      <x:c r="B59" s="17"/>
-      <x:c r="C59" s="17"/>
-      <x:c r="D59" s="17"/>
-      <x:c r="E59" s="17"/>
-      <x:c r="F59" s="17"/>
-      <x:c r="G59" s="17"/>
-      <x:c r="H59" s="17"/>
-      <x:c r="I59" s="17"/>
-      <x:c r="J59" s="17"/>
-      <x:c r="K59" s="17"/>
-    </x:row>
-    <x:row r="60">
-      <x:c r="A60" s="20" t="str">
-        <x:v>序号</x:v>
-      </x:c>
-      <x:c r="B60" s="20" t="str">
-        <x:v>周期</x:v>
-      </x:c>
-      <x:c r="C60" s="20" t="str">
-        <x:v>开盘</x:v>
-      </x:c>
-      <x:c r="D60" s="20" t="str">
-        <x:v>高点</x:v>
-      </x:c>
-      <x:c r="E60" s="20" t="str">
-        <x:v>低点</x:v>
-      </x:c>
-      <x:c r="F60" s="20" t="str">
-        <x:v>收盘</x:v>
-      </x:c>
-      <x:c r="G60" s="20" t="str">
-        <x:v>涨跌点数</x:v>
-      </x:c>
-      <x:c r="H60" s="20" t="str">
-        <x:v>涨幅</x:v>
-      </x:c>
-      <x:c r="I60" s="20" t="str">
-        <x:v>振幅</x:v>
-      </x:c>
-      <x:c r="J60" s="20" t="str">
-        <x:v>标的</x:v>
-      </x:c>
-      <x:c r="K60" s="20" t="str">
-        <x:v>交易日</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B61" s="22" t="str">
+        <x:v>8月24日</x:v>
+      </x:c>
+      <x:c r="C61" s="23" t="n">
+        <x:v>2856.4</x:v>
+      </x:c>
+      <x:c r="D61" s="23" t="n">
+        <x:v>2866.8</x:v>
+      </x:c>
+      <x:c r="E61" s="23" t="n">
+        <x:v>2837.4</x:v>
+      </x:c>
+      <x:c r="F61" s="23" t="n">
+        <x:v>2851</x:v>
+      </x:c>
+      <x:c r="G61" s="23" t="n">
+        <x:f>ROUND(F61-F60,1)</x:f>
+        <x:v>-10</x:v>
+      </x:c>
+      <x:c r="H61" s="24" t="n">
+        <x:f>IFERROR(F61/F60-1,"")</x:f>
+        <x:v>-0.003495281370150316</x:v>
+      </x:c>
+      <x:c r="I61" s="23" t="n">
+        <x:f>ROUND(D61-E61,1)</x:f>
+        <x:v>29.4</x:v>
+      </x:c>
+      <x:c r="J61" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+      <x:c r="K61" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B61" s="22" t="str">
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="31" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B62" s="30" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C62" s="30"/>
+      <x:c r="D62" s="30"/>
+      <x:c r="E62" s="30"/>
+      <x:c r="F62" s="30"/>
+      <x:c r="G62" s="30"/>
+      <x:c r="H62" s="30"/>
+      <x:c r="I62" s="32" t="n">
+        <x:f>ROUND(SUM(I58:I61),1)</x:f>
+        <x:v>265</x:v>
+      </x:c>
+      <x:c r="J62" s="30"/>
+      <x:c r="K62" s="30"/>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B63" s="30"/>
+      <x:c r="C63" s="30"/>
+      <x:c r="D63" s="30"/>
+      <x:c r="E63" s="30"/>
+      <x:c r="F63" s="30"/>
+      <x:c r="G63" s="30"/>
+      <x:c r="H63" s="30"/>
+      <x:c r="I63" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I58:I61),0),1)</x:f>
+        <x:v>66.2</x:v>
+      </x:c>
+      <x:c r="J63" s="30"/>
+      <x:c r="K63" s="30"/>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="17" t="str">
+        <x:v>碳酸锂2609</x:v>
+      </x:c>
+      <x:c r="B65" s="17"/>
+      <x:c r="C65" s="17"/>
+      <x:c r="D65" s="17"/>
+      <x:c r="E65" s="17"/>
+      <x:c r="F65" s="17"/>
+      <x:c r="G65" s="17"/>
+      <x:c r="H65" s="17"/>
+      <x:c r="I65" s="17"/>
+      <x:c r="J65" s="17"/>
+      <x:c r="K65" s="17"/>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" s="20" t="str">
+        <x:v>序号</x:v>
+      </x:c>
+      <x:c r="B66" s="20" t="str">
+        <x:v>周期</x:v>
+      </x:c>
+      <x:c r="C66" s="20" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="D66" s="20" t="str">
+        <x:v>高点</x:v>
+      </x:c>
+      <x:c r="E66" s="20" t="str">
+        <x:v>低点</x:v>
+      </x:c>
+      <x:c r="F66" s="20" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="G66" s="20" t="str">
+        <x:v>涨跌点数</x:v>
+      </x:c>
+      <x:c r="H66" s="20" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I66" s="20" t="str">
+        <x:v>振幅</x:v>
+      </x:c>
+      <x:c r="J66" s="20" t="str">
+        <x:v>标的</x:v>
+      </x:c>
+      <x:c r="K66" s="20" t="str">
+        <x:v>交易日</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B67" s="22" t="str">
         <x:v>8月3日-8月7日</x:v>
       </x:c>
-      <x:c r="C61" s="23" t="n">
+      <x:c r="C67" s="23" t="n">
         <x:v>137500</x:v>
       </x:c>
-      <x:c r="D61" s="23" t="n">
+      <x:c r="D67" s="23" t="n">
         <x:v>144800</x:v>
       </x:c>
-      <x:c r="E61" s="23" t="n">
+      <x:c r="E67" s="23" t="n">
         <x:v>135560</x:v>
       </x:c>
-      <x:c r="F61" s="23" t="n">
+      <x:c r="F67" s="23" t="n">
         <x:v>140000</x:v>
       </x:c>
-      <x:c r="G61" s="23"/>
-      <x:c r="H61" s="24"/>
-      <x:c r="I61" s="26" t="n">
-        <x:f>ROUND(D61-E61,1)</x:f>
+      <x:c r="G67" s="23"/>
+      <x:c r="H67" s="24"/>
+      <x:c r="I67" s="26" t="n">
+        <x:f>ROUND(D67-E67,1)</x:f>
         <x:v>9240</x:v>
       </x:c>
-      <x:c r="J61" s="22" t="str">
+      <x:c r="J67" s="22" t="str">
         <x:v>LC2609</x:v>
       </x:c>
-      <x:c r="K61" s="22" t="n">
+      <x:c r="K67" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="62">
-      <x:c r="A62" s="22" t="n">
+    <x:row r="68">
+      <x:c r="A68" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B62" s="22" t="str">
+      <x:c r="B68" s="22" t="str">
         <x:v>8月10日-8月14日</x:v>
       </x:c>
-      <x:c r="C62" s="23" t="n">
+      <x:c r="C68" s="23" t="n">
         <x:v>140500</x:v>
       </x:c>
-      <x:c r="D62" s="23" t="n">
+      <x:c r="D68" s="23" t="n">
         <x:v>154500</x:v>
       </x:c>
-      <x:c r="E62" s="23" t="n">
+      <x:c r="E68" s="23" t="n">
         <x:v>139280</x:v>
       </x:c>
-      <x:c r="F62" s="23" t="n">
+      <x:c r="F68" s="23" t="n">
         <x:v>153940</x:v>
       </x:c>
-      <x:c r="G62" s="28" t="n">
-        <x:f>ROUND(F62-F61,1)</x:f>
+      <x:c r="G68" s="28" t="n">
+        <x:f>ROUND(F68-F67,1)</x:f>
         <x:v>13940</x:v>
       </x:c>
-      <x:c r="H62" s="24" t="n">
-        <x:f>IFERROR(F62/F61-1,"")</x:f>
+      <x:c r="H68" s="24" t="n">
+        <x:f>IFERROR(F68/F67-1,"")</x:f>
         <x:v>0.09957142857142864</x:v>
       </x:c>
-      <x:c r="I62" s="26" t="n">
-        <x:f>ROUND(D62-E62,1)</x:f>
+      <x:c r="I68" s="26" t="n">
+        <x:f>ROUND(D68-E68,1)</x:f>
         <x:v>15220</x:v>
       </x:c>
-      <x:c r="J62" s="22" t="str">
+      <x:c r="J68" s="22" t="str">
         <x:v>LC2609</x:v>
       </x:c>
-      <x:c r="K62" s="22" t="n">
+      <x:c r="K68" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="63">
-      <x:c r="A63" s="22" t="n">
+    <x:row r="69">
+      <x:c r="A69" s="22" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B63" s="22" t="str">
+      <x:c r="B69" s="22" t="str">
         <x:v>8月17日-8月21日</x:v>
       </x:c>
-      <x:c r="C63" s="23" t="n">
+      <x:c r="C69" s="23" t="n">
         <x:v>154300</x:v>
       </x:c>
-      <x:c r="D63" s="23" t="n">
+      <x:c r="D69" s="23" t="n">
         <x:v>157000</x:v>
       </x:c>
-      <x:c r="E63" s="23" t="n">
+      <x:c r="E69" s="23" t="n">
         <x:v>148400</x:v>
       </x:c>
-      <x:c r="F63" s="23" t="n">
+      <x:c r="F69" s="23" t="n">
         <x:v>156140</x:v>
       </x:c>
-      <x:c r="G63" s="28" t="n">
-        <x:f>ROUND(F63-F62,1)</x:f>
+      <x:c r="G69" s="28" t="n">
+        <x:f>ROUND(F69-F68,1)</x:f>
         <x:v>2200</x:v>
       </x:c>
-      <x:c r="H63" s="24" t="n">
-        <x:f>IFERROR(F63/F62-1,"")</x:f>
+      <x:c r="H69" s="24" t="n">
+        <x:f>IFERROR(F69/F68-1,"")</x:f>
         <x:v>0.014291282317786091</x:v>
       </x:c>
-      <x:c r="I63" s="26" t="n">
-        <x:f>ROUND(D63-E63,1)</x:f>
+      <x:c r="I69" s="26" t="n">
+        <x:f>ROUND(D69-E69,1)</x:f>
         <x:v>8600</x:v>
       </x:c>
-      <x:c r="J63" s="22" t="str">
+      <x:c r="J69" s="22" t="str">
         <x:v>LC2609</x:v>
       </x:c>
-      <x:c r="K63" s="22" t="n">
+      <x:c r="K69" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="64">
-      <x:c r="A64" s="31" t="str">
+    <x:row r="70">
+      <x:c r="A70" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B70" s="22" t="str">
+        <x:v>8月24日</x:v>
+      </x:c>
+      <x:c r="C70" s="23" t="n">
+        <x:v>158500</x:v>
+      </x:c>
+      <x:c r="D70" s="23" t="n">
+        <x:v>160000</x:v>
+      </x:c>
+      <x:c r="E70" s="23" t="n">
+        <x:v>154280</x:v>
+      </x:c>
+      <x:c r="F70" s="23" t="n">
+        <x:v>157000</x:v>
+      </x:c>
+      <x:c r="G70" s="28" t="n">
+        <x:f>ROUND(F70-F69,1)</x:f>
+        <x:v>860</x:v>
+      </x:c>
+      <x:c r="H70" s="24" t="n">
+        <x:f>IFERROR(F70/F69-1,"")</x:f>
+        <x:v>0.005507877545792184</x:v>
+      </x:c>
+      <x:c r="I70" s="23" t="n">
+        <x:f>ROUND(D70-E70,1)</x:f>
+        <x:v>5720</x:v>
+      </x:c>
+      <x:c r="J70" s="22" t="str">
+        <x:v>LC2609</x:v>
+      </x:c>
+      <x:c r="K70" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B64" s="30" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C64" s="30"/>
-      <x:c r="D64" s="30"/>
-      <x:c r="E64" s="30"/>
-      <x:c r="F64" s="30"/>
-      <x:c r="G64" s="30"/>
-      <x:c r="H64" s="30"/>
-      <x:c r="I64" s="32" t="n">
-        <x:f>ROUND(SUM(I61:I63),1)</x:f>
-        <x:v>33060</x:v>
-      </x:c>
-      <x:c r="J64" s="30"/>
-      <x:c r="K64" s="30"/>
-    </x:row>
-    <x:row r="65">
-      <x:c r="A65" s="31" t="str">
+      <x:c r="B71" s="30" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C71" s="30"/>
+      <x:c r="D71" s="30"/>
+      <x:c r="E71" s="30"/>
+      <x:c r="F71" s="30"/>
+      <x:c r="G71" s="30"/>
+      <x:c r="H71" s="30"/>
+      <x:c r="I71" s="32" t="n">
+        <x:f>ROUND(SUM(I67:I70),1)</x:f>
+        <x:v>38780</x:v>
+      </x:c>
+      <x:c r="J71" s="30"/>
+      <x:c r="K71" s="30"/>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B65" s="30"/>
-      <x:c r="C65" s="30"/>
-      <x:c r="D65" s="30"/>
-      <x:c r="E65" s="30"/>
-      <x:c r="F65" s="30"/>
-      <x:c r="G65" s="30"/>
-      <x:c r="H65" s="30"/>
-      <x:c r="I65" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I61:I63),0),1)</x:f>
-        <x:v>11020</x:v>
-      </x:c>
-      <x:c r="J65" s="30"/>
-      <x:c r="K65" s="30"/>
+      <x:c r="B72" s="30"/>
+      <x:c r="C72" s="30"/>
+      <x:c r="D72" s="30"/>
+      <x:c r="E72" s="30"/>
+      <x:c r="F72" s="30"/>
+      <x:c r="G72" s="30"/>
+      <x:c r="H72" s="30"/>
+      <x:c r="I72" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I67:I70),0),1)</x:f>
+        <x:v>9695</x:v>
+      </x:c>
+      <x:c r="J72" s="30"/>
+      <x:c r="K72" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:K1"/>
     <x:mergeCell ref="A3:K3"/>
-    <x:mergeCell ref="A11:K11"/>
-    <x:mergeCell ref="A19:K19"/>
-    <x:mergeCell ref="A27:K27"/>
-    <x:mergeCell ref="A35:K35"/>
-    <x:mergeCell ref="A43:K43"/>
-    <x:mergeCell ref="A51:K51"/>
-    <x:mergeCell ref="A59:K59"/>
+    <x:mergeCell ref="A12:K12"/>
+    <x:mergeCell ref="A21:K21"/>
+    <x:mergeCell ref="A30:K30"/>
+    <x:mergeCell ref="A38:K38"/>
+    <x:mergeCell ref="A47:K47"/>
+    <x:mergeCell ref="A56:K56"/>
+    <x:mergeCell ref="A65:K65"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -3727,31 +4029,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B21" s="30" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C21" s="30"/>
-      <x:c r="D21" s="30"/>
-      <x:c r="E21" s="30"/>
-      <x:c r="F21" s="30"/>
-      <x:c r="G21" s="30"/>
-      <x:c r="H21" s="30"/>
-      <x:c r="I21" s="30"/>
-      <x:c r="J21" s="32" t="n">
-        <x:f>SUM(J4:J18)</x:f>
-        <x:v>2547.3</x:v>
-      </x:c>
-      <x:c r="K21" s="30"/>
+    <x:row r="19">
+      <x:c r="A19" s="22" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B19" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C19" s="22" t="str">
+        <x:v>8月24日</x:v>
+      </x:c>
+      <x:c r="D19" s="23" t="n">
+        <x:v>7614.89</x:v>
+      </x:c>
+      <x:c r="E19" s="23" t="n">
+        <x:v>7633.34</x:v>
+      </x:c>
+      <x:c r="F19" s="23" t="n">
+        <x:v>7377.72</x:v>
+      </x:c>
+      <x:c r="G19" s="23" t="n">
+        <x:v>7491.49</x:v>
+      </x:c>
+      <x:c r="H19" s="23" t="n">
+        <x:v>-110.3</x:v>
+      </x:c>
+      <x:c r="I19" s="24" t="n">
+        <x:v>-0.014511036859691129</x:v>
+      </x:c>
+      <x:c r="J19" s="26" t="n">
+        <x:f>ROUND(E19-F19,1)</x:f>
+        <x:v>255.6</x:v>
+      </x:c>
+      <x:c r="K19" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B22" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B22" s="30" t="n">
+        <x:v>16</x:v>
+      </x:c>
       <x:c r="C22" s="30"/>
       <x:c r="D22" s="30"/>
       <x:c r="E22" s="30"/>
@@ -3759,11 +4079,29 @@
       <x:c r="G22" s="30"/>
       <x:c r="H22" s="30"/>
       <x:c r="I22" s="30"/>
-      <x:c r="J22" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
-        <x:v>169.8</x:v>
+      <x:c r="J22" s="32" t="n">
+        <x:f>SUM(J4:J19)</x:f>
+        <x:v>2802.9</x:v>
       </x:c>
       <x:c r="K22" s="30"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B23" s="30"/>
+      <x:c r="C23" s="30"/>
+      <x:c r="D23" s="30"/>
+      <x:c r="E23" s="30"/>
+      <x:c r="F23" s="30"/>
+      <x:c r="G23" s="30"/>
+      <x:c r="H23" s="30"/>
+      <x:c r="I23" s="30"/>
+      <x:c r="J23" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
+        <x:v>175.2</x:v>
+      </x:c>
+      <x:c r="K23" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4370,31 +4708,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B21" s="30" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C21" s="30"/>
-      <x:c r="D21" s="30"/>
-      <x:c r="E21" s="30"/>
-      <x:c r="F21" s="30"/>
-      <x:c r="G21" s="30"/>
-      <x:c r="H21" s="30"/>
-      <x:c r="I21" s="30"/>
-      <x:c r="J21" s="32" t="n">
-        <x:f>SUM(J4:J18)</x:f>
-        <x:v>2450.5</x:v>
-      </x:c>
-      <x:c r="K21" s="30"/>
+    <x:row r="19">
+      <x:c r="A19" s="22" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B19" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C19" s="22" t="str">
+        <x:v>8月24日</x:v>
+      </x:c>
+      <x:c r="D19" s="23" t="n">
+        <x:v>7861.05</x:v>
+      </x:c>
+      <x:c r="E19" s="23" t="n">
+        <x:v>7865.54</x:v>
+      </x:c>
+      <x:c r="F19" s="23" t="n">
+        <x:v>7615.45</x:v>
+      </x:c>
+      <x:c r="G19" s="23" t="n">
+        <x:v>7717.09</x:v>
+      </x:c>
+      <x:c r="H19" s="23" t="n">
+        <x:v>-137.2</x:v>
+      </x:c>
+      <x:c r="I19" s="24" t="n">
+        <x:v>-0.017473164483794212</x:v>
+      </x:c>
+      <x:c r="J19" s="26" t="n">
+        <x:f>ROUND(E19-F19,1)</x:f>
+        <x:v>250.1</x:v>
+      </x:c>
+      <x:c r="K19" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B22" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B22" s="30" t="n">
+        <x:v>16</x:v>
+      </x:c>
       <x:c r="C22" s="30"/>
       <x:c r="D22" s="30"/>
       <x:c r="E22" s="30"/>
@@ -4402,11 +4758,29 @@
       <x:c r="G22" s="30"/>
       <x:c r="H22" s="30"/>
       <x:c r="I22" s="30"/>
-      <x:c r="J22" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
-        <x:v>163.4</x:v>
+      <x:c r="J22" s="32" t="n">
+        <x:f>SUM(J4:J19)</x:f>
+        <x:v>2700.6</x:v>
       </x:c>
       <x:c r="K22" s="30"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B23" s="30"/>
+      <x:c r="C23" s="30"/>
+      <x:c r="D23" s="30"/>
+      <x:c r="E23" s="30"/>
+      <x:c r="F23" s="30"/>
+      <x:c r="G23" s="30"/>
+      <x:c r="H23" s="30"/>
+      <x:c r="I23" s="30"/>
+      <x:c r="J23" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
+        <x:v>168.8</x:v>
+      </x:c>
+      <x:c r="K23" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5013,31 +5387,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B21" s="30" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C21" s="30"/>
-      <x:c r="D21" s="30"/>
-      <x:c r="E21" s="30"/>
-      <x:c r="F21" s="30"/>
-      <x:c r="G21" s="30"/>
-      <x:c r="H21" s="30"/>
-      <x:c r="I21" s="30"/>
-      <x:c r="J21" s="32" t="n">
-        <x:f>SUM(J4:J18)</x:f>
-        <x:v>629.9</x:v>
-      </x:c>
-      <x:c r="K21" s="30"/>
+    <x:row r="19">
+      <x:c r="A19" s="22" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B19" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C19" s="22" t="str">
+        <x:v>8月24日</x:v>
+      </x:c>
+      <x:c r="D19" s="23" t="n">
+        <x:v>3902.7</x:v>
+      </x:c>
+      <x:c r="E19" s="23" t="n">
+        <x:v>3910.24</x:v>
+      </x:c>
+      <x:c r="F19" s="23" t="n">
+        <x:v>3855.35</x:v>
+      </x:c>
+      <x:c r="G19" s="23" t="n">
+        <x:v>3882.01</x:v>
+      </x:c>
+      <x:c r="H19" s="23" t="n">
+        <x:v>-23.2</x:v>
+      </x:c>
+      <x:c r="I19" s="24" t="n">
+        <x:v>-0.005938236197889912</x:v>
+      </x:c>
+      <x:c r="J19" s="26" t="n">
+        <x:f>ROUND(E19-F19,1)</x:f>
+        <x:v>54.9</x:v>
+      </x:c>
+      <x:c r="K19" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B22" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B22" s="30" t="n">
+        <x:v>16</x:v>
+      </x:c>
       <x:c r="C22" s="30"/>
       <x:c r="D22" s="30"/>
       <x:c r="E22" s="30"/>
@@ -5045,11 +5437,29 @@
       <x:c r="G22" s="30"/>
       <x:c r="H22" s="30"/>
       <x:c r="I22" s="30"/>
-      <x:c r="J22" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
-        <x:v>42</x:v>
+      <x:c r="J22" s="32" t="n">
+        <x:f>SUM(J4:J19)</x:f>
+        <x:v>684.8</x:v>
       </x:c>
       <x:c r="K22" s="30"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B23" s="30"/>
+      <x:c r="C23" s="30"/>
+      <x:c r="D23" s="30"/>
+      <x:c r="E23" s="30"/>
+      <x:c r="F23" s="30"/>
+      <x:c r="G23" s="30"/>
+      <x:c r="H23" s="30"/>
+      <x:c r="I23" s="30"/>
+      <x:c r="J23" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
+        <x:v>42.8</x:v>
+      </x:c>
+      <x:c r="K23" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -6299,31 +6709,49 @@
         <x:v>IC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B21" s="30" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C21" s="30"/>
-      <x:c r="D21" s="30"/>
-      <x:c r="E21" s="30"/>
-      <x:c r="F21" s="30"/>
-      <x:c r="G21" s="30"/>
-      <x:c r="H21" s="30"/>
-      <x:c r="I21" s="30"/>
-      <x:c r="J21" s="32" t="n">
-        <x:f>SUM(J4:J18)</x:f>
-        <x:v>2434.6</x:v>
-      </x:c>
-      <x:c r="K21" s="30"/>
+    <x:row r="19">
+      <x:c r="A19" s="22" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B19" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C19" s="22" t="str">
+        <x:v>8月24日</x:v>
+      </x:c>
+      <x:c r="D19" s="23" t="n">
+        <x:v>7757</x:v>
+      </x:c>
+      <x:c r="E19" s="23" t="n">
+        <x:v>7764.4</x:v>
+      </x:c>
+      <x:c r="F19" s="23" t="n">
+        <x:v>7514.4</x:v>
+      </x:c>
+      <x:c r="G19" s="23" t="n">
+        <x:v>7628.4</x:v>
+      </x:c>
+      <x:c r="H19" s="23" t="n">
+        <x:v>-133.6</x:v>
+      </x:c>
+      <x:c r="I19" s="24" t="n">
+        <x:v>-0.01721205874774545</x:v>
+      </x:c>
+      <x:c r="J19" s="26" t="n">
+        <x:f>ROUND(E19-F19,1)</x:f>
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="K19" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B22" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B22" s="30" t="n">
+        <x:v>16</x:v>
+      </x:c>
       <x:c r="C22" s="30"/>
       <x:c r="D22" s="30"/>
       <x:c r="E22" s="30"/>
@@ -6331,11 +6759,29 @@
       <x:c r="G22" s="30"/>
       <x:c r="H22" s="30"/>
       <x:c r="I22" s="30"/>
-      <x:c r="J22" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
-        <x:v>162.3</x:v>
+      <x:c r="J22" s="32" t="n">
+        <x:f>SUM(J4:J19)</x:f>
+        <x:v>2684.6</x:v>
       </x:c>
       <x:c r="K22" s="30"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B23" s="30"/>
+      <x:c r="C23" s="30"/>
+      <x:c r="D23" s="30"/>
+      <x:c r="E23" s="30"/>
+      <x:c r="F23" s="30"/>
+      <x:c r="G23" s="30"/>
+      <x:c r="H23" s="30"/>
+      <x:c r="I23" s="30"/>
+      <x:c r="J23" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
+        <x:v>167.8</x:v>
+      </x:c>
+      <x:c r="K23" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -6942,31 +7388,49 @@
         <x:v>IF2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B21" s="30" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C21" s="30"/>
-      <x:c r="D21" s="30"/>
-      <x:c r="E21" s="30"/>
-      <x:c r="F21" s="30"/>
-      <x:c r="G21" s="30"/>
-      <x:c r="H21" s="30"/>
-      <x:c r="I21" s="30"/>
-      <x:c r="J21" s="32" t="n">
-        <x:f>SUM(J4:J18)</x:f>
-        <x:v>914</x:v>
-      </x:c>
-      <x:c r="K21" s="30"/>
+    <x:row r="19">
+      <x:c r="A19" s="22" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B19" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C19" s="22" t="str">
+        <x:v>8月24日</x:v>
+      </x:c>
+      <x:c r="D19" s="23" t="n">
+        <x:v>4607.4</x:v>
+      </x:c>
+      <x:c r="E19" s="23" t="n">
+        <x:v>4607.4</x:v>
+      </x:c>
+      <x:c r="F19" s="23" t="n">
+        <x:v>4486.4</x:v>
+      </x:c>
+      <x:c r="G19" s="23" t="n">
+        <x:v>4526.4</x:v>
+      </x:c>
+      <x:c r="H19" s="23" t="n">
+        <x:v>-49.6</x:v>
+      </x:c>
+      <x:c r="I19" s="24" t="n">
+        <x:v>-0.010839160839160922</x:v>
+      </x:c>
+      <x:c r="J19" s="26" t="n">
+        <x:f>ROUND(E19-F19,1)</x:f>
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="K19" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B22" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B22" s="30" t="n">
+        <x:v>16</x:v>
+      </x:c>
       <x:c r="C22" s="30"/>
       <x:c r="D22" s="30"/>
       <x:c r="E22" s="30"/>
@@ -6974,11 +7438,29 @@
       <x:c r="G22" s="30"/>
       <x:c r="H22" s="30"/>
       <x:c r="I22" s="30"/>
-      <x:c r="J22" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
-        <x:v>60.9</x:v>
+      <x:c r="J22" s="32" t="n">
+        <x:f>SUM(J4:J19)</x:f>
+        <x:v>1035</x:v>
       </x:c>
       <x:c r="K22" s="30"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B23" s="30"/>
+      <x:c r="C23" s="30"/>
+      <x:c r="D23" s="30"/>
+      <x:c r="E23" s="30"/>
+      <x:c r="F23" s="30"/>
+      <x:c r="G23" s="30"/>
+      <x:c r="H23" s="30"/>
+      <x:c r="I23" s="30"/>
+      <x:c r="J23" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
+        <x:v>64.7</x:v>
+      </x:c>
+      <x:c r="K23" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -7585,31 +8067,49 @@
         <x:v>IH2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B21" s="30" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C21" s="30"/>
-      <x:c r="D21" s="30"/>
-      <x:c r="E21" s="30"/>
-      <x:c r="F21" s="30"/>
-      <x:c r="G21" s="30"/>
-      <x:c r="H21" s="30"/>
-      <x:c r="I21" s="30"/>
-      <x:c r="J21" s="32" t="n">
-        <x:f>SUM(J4:J18)</x:f>
-        <x:v>508.6000000000001</x:v>
-      </x:c>
-      <x:c r="K21" s="30"/>
+    <x:row r="19">
+      <x:c r="A19" s="22" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B19" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C19" s="22" t="str">
+        <x:v>8月24日</x:v>
+      </x:c>
+      <x:c r="D19" s="23" t="n">
+        <x:v>2856.4</x:v>
+      </x:c>
+      <x:c r="E19" s="23" t="n">
+        <x:v>2866.8</x:v>
+      </x:c>
+      <x:c r="F19" s="23" t="n">
+        <x:v>2837.4</x:v>
+      </x:c>
+      <x:c r="G19" s="23" t="n">
+        <x:v>2851</x:v>
+      </x:c>
+      <x:c r="H19" s="23" t="n">
+        <x:v>-10</x:v>
+      </x:c>
+      <x:c r="I19" s="24" t="n">
+        <x:v>-0.003495281370150316</x:v>
+      </x:c>
+      <x:c r="J19" s="23" t="n">
+        <x:f>ROUND(E19-F19,1)</x:f>
+        <x:v>29.4</x:v>
+      </x:c>
+      <x:c r="K19" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B22" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B22" s="30" t="n">
+        <x:v>16</x:v>
+      </x:c>
       <x:c r="C22" s="30"/>
       <x:c r="D22" s="30"/>
       <x:c r="E22" s="30"/>
@@ -7617,11 +8117,29 @@
       <x:c r="G22" s="30"/>
       <x:c r="H22" s="30"/>
       <x:c r="I22" s="30"/>
-      <x:c r="J22" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
-        <x:v>33.9</x:v>
+      <x:c r="J22" s="32" t="n">
+        <x:f>SUM(J4:J19)</x:f>
+        <x:v>538.0000000000001</x:v>
       </x:c>
       <x:c r="K22" s="30"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B23" s="30"/>
+      <x:c r="C23" s="30"/>
+      <x:c r="D23" s="30"/>
+      <x:c r="E23" s="30"/>
+      <x:c r="F23" s="30"/>
+      <x:c r="G23" s="30"/>
+      <x:c r="H23" s="30"/>
+      <x:c r="I23" s="30"/>
+      <x:c r="J23" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
+        <x:v>33.6</x:v>
+      </x:c>
+      <x:c r="K23" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-08-25
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rdc74d2f7b45d4fb4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R64a30d6e771d42de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Rbe3f9846e9d544b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R92c3bfeba51b4f86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R841eb197c2f349f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rc32209c1f2894e89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R5f378fb7ce9c4bd4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rab5d28d83e844f34"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rcc51f00593704333"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R45f1925038ce4a42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R79cd2c97656c4a02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Red00d5f211724efd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R1507a17ebb8d4b0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rc9fe7dc461434811"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R2b8a2528e2ad47f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R2d2ac5cc2c064bed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Rd7bec770a9b74ef3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rac01e62827b84ffb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rc27ff46bbbfb44a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R0b280c99f85d4c50"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -520,25 +520,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7633.34</x:v>
+        <x:v>7556.07</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7377.72</x:v>
+        <x:v>7347.95</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>255.6</x:v>
+        <x:v>208.1</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>2802.9</x:v>
+        <x:v>3011</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>175.2</x:v>
+        <x:v>177.1</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -549,25 +549,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7865.54</x:v>
+        <x:v>7755.72</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7615.45</x:v>
+        <x:v>7572.86</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>250.1</x:v>
+        <x:v>182.9</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>2700.6</x:v>
+        <x:v>2883.5</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>168.8</x:v>
+        <x:v>169.6</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -578,25 +578,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3910.24</x:v>
+        <x:v>3896.21</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3855.35</x:v>
+        <x:v>3850.86</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>54.9</x:v>
+        <x:v>45.3</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>684.8</x:v>
+        <x:v>730.1</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>42.8</x:v>
+        <x:v>42.9</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -755,7 +755,7 @@
         <x:v>2026-08-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1745,7 +1745,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B8" s="22" t="str">
-        <x:v>8月24日</x:v>
+        <x:v>8月24日-8月25日</x:v>
       </x:c>
       <x:c r="C8" s="23" t="n">
         <x:v>7614.89</x:v>
@@ -1754,28 +1754,28 @@
         <x:v>7633.34</x:v>
       </x:c>
       <x:c r="E8" s="23" t="n">
-        <x:v>7377.72</x:v>
+        <x:v>7347.95</x:v>
       </x:c>
       <x:c r="F8" s="23" t="n">
-        <x:v>7491.49</x:v>
+        <x:v>7527.5</x:v>
       </x:c>
       <x:c r="G8" s="23" t="n">
         <x:f>ROUND(F8-F7,1)</x:f>
-        <x:v>-110.3</x:v>
+        <x:v>-74.3</x:v>
       </x:c>
       <x:c r="H8" s="24" t="n">
         <x:f>IFERROR(F8/F7-1,"")</x:f>
-        <x:v>-0.014511036859691129</x:v>
+        <x:v>-0.009774000894524959</x:v>
       </x:c>
       <x:c r="I8" s="26" t="n">
         <x:f>ROUND(D8-E8,1)</x:f>
-        <x:v>255.6</x:v>
+        <x:v>285.4</x:v>
       </x:c>
       <x:c r="J8" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K8" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1793,7 +1793,7 @@
       <x:c r="H9" s="30"/>
       <x:c r="I9" s="32" t="n">
         <x:f>ROUND(SUM(I5:I8),1)</x:f>
-        <x:v>1679.9</x:v>
+        <x:v>1709.7</x:v>
       </x:c>
       <x:c r="J9" s="30"/>
       <x:c r="K9" s="30"/>
@@ -1811,7 +1811,7 @@
       <x:c r="H10" s="30"/>
       <x:c r="I10" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I8),0),1)</x:f>
-        <x:v>420</x:v>
+        <x:v>427.4</x:v>
       </x:c>
       <x:c r="J10" s="30"/>
       <x:c r="K10" s="30"/>
@@ -1979,7 +1979,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B17" s="22" t="str">
-        <x:v>8月24日</x:v>
+        <x:v>8月24日-8月25日</x:v>
       </x:c>
       <x:c r="C17" s="23" t="n">
         <x:v>7861.05</x:v>
@@ -1988,28 +1988,28 @@
         <x:v>7865.54</x:v>
       </x:c>
       <x:c r="E17" s="23" t="n">
-        <x:v>7615.45</x:v>
+        <x:v>7572.86</x:v>
       </x:c>
       <x:c r="F17" s="23" t="n">
-        <x:v>7717.09</x:v>
+        <x:v>7710.94</x:v>
       </x:c>
       <x:c r="G17" s="23" t="n">
         <x:f>ROUND(F17-F16,1)</x:f>
-        <x:v>-137.2</x:v>
+        <x:v>-143.4</x:v>
       </x:c>
       <x:c r="H17" s="24" t="n">
         <x:f>IFERROR(F17/F16-1,"")</x:f>
-        <x:v>-0.017473164483794212</x:v>
+        <x:v>-0.018256172073238597</x:v>
       </x:c>
       <x:c r="I17" s="26" t="n">
         <x:f>ROUND(D17-E17,1)</x:f>
-        <x:v>250.1</x:v>
+        <x:v>292.7</x:v>
       </x:c>
       <x:c r="J17" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K17" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -2027,7 +2027,7 @@
       <x:c r="H18" s="30"/>
       <x:c r="I18" s="32" t="n">
         <x:f>ROUND(SUM(I14:I17),1)</x:f>
-        <x:v>1535.4</x:v>
+        <x:v>1578</x:v>
       </x:c>
       <x:c r="J18" s="30"/>
       <x:c r="K18" s="30"/>
@@ -2045,7 +2045,7 @@
       <x:c r="H19" s="30"/>
       <x:c r="I19" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I14:I17),0),1)</x:f>
-        <x:v>383.9</x:v>
+        <x:v>394.5</x:v>
       </x:c>
       <x:c r="J19" s="30"/>
       <x:c r="K19" s="30"/>
@@ -2213,7 +2213,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B26" s="22" t="str">
-        <x:v>8月24日</x:v>
+        <x:v>8月24日-8月25日</x:v>
       </x:c>
       <x:c r="C26" s="23" t="n">
         <x:v>3902.7</x:v>
@@ -2222,28 +2222,28 @@
         <x:v>3910.24</x:v>
       </x:c>
       <x:c r="E26" s="23" t="n">
-        <x:v>3855.35</x:v>
+        <x:v>3850.86</x:v>
       </x:c>
       <x:c r="F26" s="23" t="n">
-        <x:v>3882.01</x:v>
+        <x:v>3889.44</x:v>
       </x:c>
       <x:c r="G26" s="23" t="n">
         <x:f>ROUND(F26-F25,1)</x:f>
-        <x:v>-23.2</x:v>
+        <x:v>-15.8</x:v>
       </x:c>
       <x:c r="H26" s="24" t="n">
         <x:f>IFERROR(F26/F25-1,"")</x:f>
-        <x:v>-0.005938236197889912</x:v>
+        <x:v>-0.004035644781317127</x:v>
       </x:c>
       <x:c r="I26" s="26" t="n">
         <x:f>ROUND(D26-E26,1)</x:f>
-        <x:v>54.9</x:v>
+        <x:v>59.4</x:v>
       </x:c>
       <x:c r="J26" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K26" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -2261,7 +2261,7 @@
       <x:c r="H27" s="30"/>
       <x:c r="I27" s="32" t="n">
         <x:f>ROUND(SUM(I23:I26),1)</x:f>
-        <x:v>377.6</x:v>
+        <x:v>382.1</x:v>
       </x:c>
       <x:c r="J27" s="30"/>
       <x:c r="K27" s="30"/>
@@ -2279,7 +2279,7 @@
       <x:c r="H28" s="30"/>
       <x:c r="I28" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I23:I26),0),1)</x:f>
-        <x:v>94.4</x:v>
+        <x:v>95.5</x:v>
       </x:c>
       <x:c r="J28" s="30"/>
       <x:c r="K28" s="30"/>
@@ -4103,31 +4103,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B22" s="30" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="C22" s="30"/>
-      <x:c r="D22" s="30"/>
-      <x:c r="E22" s="30"/>
-      <x:c r="F22" s="30"/>
-      <x:c r="G22" s="30"/>
-      <x:c r="H22" s="30"/>
-      <x:c r="I22" s="30"/>
-      <x:c r="J22" s="32" t="n">
-        <x:f>SUM(J4:J19)</x:f>
-        <x:v>2802.9</x:v>
-      </x:c>
-      <x:c r="K22" s="30"/>
+    <x:row r="20">
+      <x:c r="A20" s="22" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B20" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C20" s="22" t="str">
+        <x:v>8月25日</x:v>
+      </x:c>
+      <x:c r="D20" s="23" t="n">
+        <x:v>7420.77</x:v>
+      </x:c>
+      <x:c r="E20" s="23" t="n">
+        <x:v>7556.07</x:v>
+      </x:c>
+      <x:c r="F20" s="23" t="n">
+        <x:v>7347.95</x:v>
+      </x:c>
+      <x:c r="G20" s="23" t="n">
+        <x:v>7527.5</x:v>
+      </x:c>
+      <x:c r="H20" s="23" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="I20" s="24" t="n">
+        <x:v>0.004806787434809445</x:v>
+      </x:c>
+      <x:c r="J20" s="26" t="n">
+        <x:f>ROUND(E20-F20,1)</x:f>
+        <x:v>208.1</x:v>
+      </x:c>
+      <x:c r="K20" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B23" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B23" s="30" t="n">
+        <x:v>17</x:v>
+      </x:c>
       <x:c r="C23" s="30"/>
       <x:c r="D23" s="30"/>
       <x:c r="E23" s="30"/>
@@ -4135,11 +4153,29 @@
       <x:c r="G23" s="30"/>
       <x:c r="H23" s="30"/>
       <x:c r="I23" s="30"/>
-      <x:c r="J23" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
-        <x:v>175.2</x:v>
+      <x:c r="J23" s="32" t="n">
+        <x:f>SUM(J4:J20)</x:f>
+        <x:v>3011</x:v>
       </x:c>
       <x:c r="K23" s="30"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B24" s="30"/>
+      <x:c r="C24" s="30"/>
+      <x:c r="D24" s="30"/>
+      <x:c r="E24" s="30"/>
+      <x:c r="F24" s="30"/>
+      <x:c r="G24" s="30"/>
+      <x:c r="H24" s="30"/>
+      <x:c r="I24" s="30"/>
+      <x:c r="J24" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
+        <x:v>177.1</x:v>
+      </x:c>
+      <x:c r="K24" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4782,31 +4818,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B22" s="30" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="C22" s="30"/>
-      <x:c r="D22" s="30"/>
-      <x:c r="E22" s="30"/>
-      <x:c r="F22" s="30"/>
-      <x:c r="G22" s="30"/>
-      <x:c r="H22" s="30"/>
-      <x:c r="I22" s="30"/>
-      <x:c r="J22" s="32" t="n">
-        <x:f>SUM(J4:J19)</x:f>
-        <x:v>2700.6</x:v>
-      </x:c>
-      <x:c r="K22" s="30"/>
+    <x:row r="20">
+      <x:c r="A20" s="22" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B20" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C20" s="22" t="str">
+        <x:v>8月25日</x:v>
+      </x:c>
+      <x:c r="D20" s="23" t="n">
+        <x:v>7644.2</x:v>
+      </x:c>
+      <x:c r="E20" s="23" t="n">
+        <x:v>7755.72</x:v>
+      </x:c>
+      <x:c r="F20" s="23" t="n">
+        <x:v>7572.86</x:v>
+      </x:c>
+      <x:c r="G20" s="23" t="n">
+        <x:v>7710.94</x:v>
+      </x:c>
+      <x:c r="H20" s="23" t="n">
+        <x:v>-6.2</x:v>
+      </x:c>
+      <x:c r="I20" s="24" t="n">
+        <x:v>-0.0007969325224923551</x:v>
+      </x:c>
+      <x:c r="J20" s="26" t="n">
+        <x:f>ROUND(E20-F20,1)</x:f>
+        <x:v>182.9</x:v>
+      </x:c>
+      <x:c r="K20" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B23" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B23" s="30" t="n">
+        <x:v>17</x:v>
+      </x:c>
       <x:c r="C23" s="30"/>
       <x:c r="D23" s="30"/>
       <x:c r="E23" s="30"/>
@@ -4814,11 +4868,29 @@
       <x:c r="G23" s="30"/>
       <x:c r="H23" s="30"/>
       <x:c r="I23" s="30"/>
-      <x:c r="J23" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
-        <x:v>168.8</x:v>
+      <x:c r="J23" s="32" t="n">
+        <x:f>SUM(J4:J20)</x:f>
+        <x:v>2883.5</x:v>
       </x:c>
       <x:c r="K23" s="30"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B24" s="30"/>
+      <x:c r="C24" s="30"/>
+      <x:c r="D24" s="30"/>
+      <x:c r="E24" s="30"/>
+      <x:c r="F24" s="30"/>
+      <x:c r="G24" s="30"/>
+      <x:c r="H24" s="30"/>
+      <x:c r="I24" s="30"/>
+      <x:c r="J24" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
+        <x:v>169.6</x:v>
+      </x:c>
+      <x:c r="K24" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5461,31 +5533,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B22" s="30" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="C22" s="30"/>
-      <x:c r="D22" s="30"/>
-      <x:c r="E22" s="30"/>
-      <x:c r="F22" s="30"/>
-      <x:c r="G22" s="30"/>
-      <x:c r="H22" s="30"/>
-      <x:c r="I22" s="30"/>
-      <x:c r="J22" s="32" t="n">
-        <x:f>SUM(J4:J19)</x:f>
-        <x:v>684.8</x:v>
-      </x:c>
-      <x:c r="K22" s="30"/>
+    <x:row r="20">
+      <x:c r="A20" s="22" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B20" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C20" s="22" t="str">
+        <x:v>8月25日</x:v>
+      </x:c>
+      <x:c r="D20" s="23" t="n">
+        <x:v>3863.37</x:v>
+      </x:c>
+      <x:c r="E20" s="23" t="n">
+        <x:v>3896.21</x:v>
+      </x:c>
+      <x:c r="F20" s="23" t="n">
+        <x:v>3850.86</x:v>
+      </x:c>
+      <x:c r="G20" s="23" t="n">
+        <x:v>3889.44</x:v>
+      </x:c>
+      <x:c r="H20" s="23" t="n">
+        <x:v>7.4</x:v>
+      </x:c>
+      <x:c r="I20" s="24" t="n">
+        <x:v>0.0019139569449846405</x:v>
+      </x:c>
+      <x:c r="J20" s="23" t="n">
+        <x:f>ROUND(E20-F20,1)</x:f>
+        <x:v>45.3</x:v>
+      </x:c>
+      <x:c r="K20" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B23" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B23" s="30" t="n">
+        <x:v>17</x:v>
+      </x:c>
       <x:c r="C23" s="30"/>
       <x:c r="D23" s="30"/>
       <x:c r="E23" s="30"/>
@@ -5493,11 +5583,29 @@
       <x:c r="G23" s="30"/>
       <x:c r="H23" s="30"/>
       <x:c r="I23" s="30"/>
-      <x:c r="J23" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
-        <x:v>42.8</x:v>
+      <x:c r="J23" s="32" t="n">
+        <x:f>SUM(J4:J20)</x:f>
+        <x:v>730.0999999999999</x:v>
       </x:c>
       <x:c r="K23" s="30"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B24" s="30"/>
+      <x:c r="C24" s="30"/>
+      <x:c r="D24" s="30"/>
+      <x:c r="E24" s="30"/>
+      <x:c r="F24" s="30"/>
+      <x:c r="G24" s="30"/>
+      <x:c r="H24" s="30"/>
+      <x:c r="I24" s="30"/>
+      <x:c r="J24" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
+        <x:v>42.9</x:v>
+      </x:c>
+      <x:c r="K24" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-08-26
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Ra317229e523c4888"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R6e8e898930624d1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Reb779522f1bc4f2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R04bb01c5f804473d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R032424ba5a7941de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R6d50ea67166a4789"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Rec4225b24ea14707"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R90fbfc7a1c784b5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Radf3ed5b01744b4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="Rb663e5ec84a24fb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rcc0a534f1afa48a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R2c8e19e23abc4b60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Rb133448646dd4f09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rf1c8bf6da86e4c3e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R1b645c0efc2c4e7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rd3265af2c18146d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R1e5af7a7149c41c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R4e89afa6042142d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rfa0e623106174454"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="Rb4e7f5c887524a9c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -520,25 +520,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-08-25</x:v>
+        <x:v>2026-08-26</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7556.07</x:v>
+        <x:v>7601.84</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7347.95</x:v>
+        <x:v>7467.41</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>208.1</x:v>
+        <x:v>134.4</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>3011</x:v>
+        <x:v>3145.4</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>177.1</x:v>
+        <x:v>174.7</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -549,25 +549,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-08-25</x:v>
+        <x:v>2026-08-26</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7755.72</x:v>
+        <x:v>7833.6</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7572.86</x:v>
+        <x:v>7699.42</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>182.9</x:v>
+        <x:v>134.2</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>2883.5</x:v>
+        <x:v>3017.7</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>169.6</x:v>
+        <x:v>167.6</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -578,25 +578,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-08-25</x:v>
+        <x:v>2026-08-26</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3896.21</x:v>
+        <x:v>3926.44</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3850.86</x:v>
+        <x:v>3881.74</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>45.3</x:v>
+        <x:v>44.7</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>730.1</x:v>
+        <x:v>774.8</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>42.9</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -636,25 +636,25 @@
         <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>2026-08-25</x:v>
+        <x:v>2026-08-26</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:v>7687.8</x:v>
+        <x:v>7783.2</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>7496</x:v>
+        <x:v>7604</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>191.8</x:v>
+        <x:v>179.2</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>2876.4</x:v>
+        <x:v>3055.6</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
-        <x:v>169.2</x:v>
+        <x:v>169.8</x:v>
       </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
@@ -694,25 +694,25 @@
         <x:v>IH主力</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>2026-08-25</x:v>
+        <x:v>2026-08-26</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:v>2864.4</x:v>
+        <x:v>2903.8</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
-        <x:v>2840</x:v>
+        <x:v>2850</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
-        <x:v>24.4</x:v>
+        <x:v>53.8</x:v>
       </x:c>
       <x:c r="F10" s="9" t="n">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="G10" s="10" t="n">
-        <x:v>562.4</x:v>
+        <x:v>616.2</x:v>
       </x:c>
       <x:c r="H10" s="10" t="n">
-        <x:v>33.1</x:v>
+        <x:v>34.2</x:v>
       </x:c>
       <x:c r="I10" s="10" t="n">
         <x:v>60</x:v>
@@ -723,25 +723,25 @@
         <x:v>碳酸锂2609</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>2026-08-25</x:v>
+        <x:v>2026-08-26</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:v>157980</x:v>
+        <x:v>153380</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
-        <x:v>149300</x:v>
+        <x:v>147000</x:v>
       </x:c>
       <x:c r="E11" s="12" t="n">
-        <x:v>8680</x:v>
+        <x:v>6380</x:v>
       </x:c>
       <x:c r="F11" s="9" t="n">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="G11" s="10" t="n">
-        <x:v>88500</x:v>
+        <x:v>94880</x:v>
       </x:c>
       <x:c r="H11" s="10" t="n">
-        <x:v>5205.9</x:v>
+        <x:v>5271.1</x:v>
       </x:c>
       <x:c r="I11" s="10" t="n">
         <x:v>6000</x:v>
@@ -755,7 +755,7 @@
         <x:v>2026-08-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-08-25</x:v>
+        <x:v>2026-08-26</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1550,31 +1550,49 @@
         <x:v>LC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B23" s="30" t="n">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="C23" s="30"/>
-      <x:c r="D23" s="30"/>
-      <x:c r="E23" s="30"/>
-      <x:c r="F23" s="30"/>
-      <x:c r="G23" s="30"/>
-      <x:c r="H23" s="30"/>
-      <x:c r="I23" s="30"/>
-      <x:c r="J23" s="32" t="n">
-        <x:f>SUM(J4:J20)</x:f>
-        <x:v>88500</x:v>
-      </x:c>
-      <x:c r="K23" s="30"/>
+    <x:row r="21">
+      <x:c r="A21" s="22" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B21" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C21" s="22" t="str">
+        <x:v>8月26日</x:v>
+      </x:c>
+      <x:c r="D21" s="23" t="n">
+        <x:v>147000</x:v>
+      </x:c>
+      <x:c r="E21" s="23" t="n">
+        <x:v>153380</x:v>
+      </x:c>
+      <x:c r="F21" s="23" t="n">
+        <x:v>147000</x:v>
+      </x:c>
+      <x:c r="G21" s="23" t="n">
+        <x:v>150580</x:v>
+      </x:c>
+      <x:c r="H21" s="28" t="n">
+        <x:v>1280</x:v>
+      </x:c>
+      <x:c r="I21" s="24" t="n">
+        <x:v>0.008573342263898276</x:v>
+      </x:c>
+      <x:c r="J21" s="26" t="n">
+        <x:f>ROUND(E21-F21,1)</x:f>
+        <x:v>6380</x:v>
+      </x:c>
+      <x:c r="K21" s="22" t="str">
+        <x:v>LC2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B24" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B24" s="30" t="n">
+        <x:v>18</x:v>
+      </x:c>
       <x:c r="C24" s="30"/>
       <x:c r="D24" s="30"/>
       <x:c r="E24" s="30"/>
@@ -1582,11 +1600,29 @@
       <x:c r="G24" s="30"/>
       <x:c r="H24" s="30"/>
       <x:c r="I24" s="30"/>
-      <x:c r="J24" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
-        <x:v>5205.9</x:v>
+      <x:c r="J24" s="32" t="n">
+        <x:f>SUM(J4:J21)</x:f>
+        <x:v>94880</x:v>
       </x:c>
       <x:c r="K24" s="30"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B25" s="30"/>
+      <x:c r="C25" s="30"/>
+      <x:c r="D25" s="30"/>
+      <x:c r="E25" s="30"/>
+      <x:c r="F25" s="30"/>
+      <x:c r="G25" s="30"/>
+      <x:c r="H25" s="30"/>
+      <x:c r="I25" s="30"/>
+      <x:c r="J25" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J21),0),1)</x:f>
+        <x:v>5271.1</x:v>
+      </x:c>
+      <x:c r="K25" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1781,7 +1817,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B8" s="22" t="str">
-        <x:v>8月24日-8月25日</x:v>
+        <x:v>8月24日-8月26日</x:v>
       </x:c>
       <x:c r="C8" s="23" t="n">
         <x:v>7614.89</x:v>
@@ -1793,15 +1829,15 @@
         <x:v>7347.95</x:v>
       </x:c>
       <x:c r="F8" s="23" t="n">
-        <x:v>7527.5</x:v>
+        <x:v>7544.67</x:v>
       </x:c>
       <x:c r="G8" s="23" t="n">
         <x:f>ROUND(F8-F7,1)</x:f>
-        <x:v>-74.3</x:v>
+        <x:v>-57.1</x:v>
       </x:c>
       <x:c r="H8" s="24" t="n">
         <x:f>IFERROR(F8/F7-1,"")</x:f>
-        <x:v>-0.009774000894524959</x:v>
+        <x:v>-0.007515325317687949</x:v>
       </x:c>
       <x:c r="I8" s="26" t="n">
         <x:f>ROUND(D8-E8,1)</x:f>
@@ -1811,7 +1847,7 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K8" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -2015,7 +2051,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B17" s="22" t="str">
-        <x:v>8月24日-8月25日</x:v>
+        <x:v>8月24日-8月26日</x:v>
       </x:c>
       <x:c r="C17" s="23" t="n">
         <x:v>7861.05</x:v>
@@ -2027,15 +2063,15 @@
         <x:v>7572.86</x:v>
       </x:c>
       <x:c r="F17" s="23" t="n">
-        <x:v>7710.94</x:v>
+        <x:v>7770.53</x:v>
       </x:c>
       <x:c r="G17" s="23" t="n">
         <x:f>ROUND(F17-F16,1)</x:f>
-        <x:v>-143.4</x:v>
+        <x:v>-83.8</x:v>
       </x:c>
       <x:c r="H17" s="24" t="n">
         <x:f>IFERROR(F17/F16-1,"")</x:f>
-        <x:v>-0.018256172073238597</x:v>
+        <x:v>-0.010669274145598706</x:v>
       </x:c>
       <x:c r="I17" s="26" t="n">
         <x:f>ROUND(D17-E17,1)</x:f>
@@ -2045,7 +2081,7 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K17" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -2249,37 +2285,37 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B26" s="22" t="str">
-        <x:v>8月24日-8月25日</x:v>
+        <x:v>8月24日-8月26日</x:v>
       </x:c>
       <x:c r="C26" s="23" t="n">
         <x:v>3902.7</x:v>
       </x:c>
       <x:c r="D26" s="23" t="n">
-        <x:v>3910.24</x:v>
+        <x:v>3926.44</x:v>
       </x:c>
       <x:c r="E26" s="23" t="n">
         <x:v>3850.86</x:v>
       </x:c>
       <x:c r="F26" s="23" t="n">
-        <x:v>3889.44</x:v>
+        <x:v>3912.52</x:v>
       </x:c>
       <x:c r="G26" s="23" t="n">
         <x:f>ROUND(F26-F25,1)</x:f>
-        <x:v>-15.8</x:v>
+        <x:v>7.3</x:v>
       </x:c>
       <x:c r="H26" s="24" t="n">
         <x:f>IFERROR(F26/F25-1,"")</x:f>
-        <x:v>-0.004035644781317127</x:v>
+        <x:v>0.0018744238451295914</x:v>
       </x:c>
       <x:c r="I26" s="26" t="n">
         <x:f>ROUND(D26-E26,1)</x:f>
-        <x:v>59.4</x:v>
+        <x:v>75.6</x:v>
       </x:c>
       <x:c r="J26" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K26" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -2297,7 +2333,7 @@
       <x:c r="H27" s="30"/>
       <x:c r="I27" s="32" t="n">
         <x:f>ROUND(SUM(I23:I26),1)</x:f>
-        <x:v>382.1</x:v>
+        <x:v>398.3</x:v>
       </x:c>
       <x:c r="J27" s="30"/>
       <x:c r="K27" s="30"/>
@@ -2315,7 +2351,7 @@
       <x:c r="H28" s="30"/>
       <x:c r="I28" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I23:I26),0),1)</x:f>
-        <x:v>95.5</x:v>
+        <x:v>99.6</x:v>
       </x:c>
       <x:c r="J28" s="30"/>
       <x:c r="K28" s="30"/>
@@ -2717,37 +2753,37 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B44" s="22" t="str">
-        <x:v>8月24日-8月25日</x:v>
+        <x:v>8月24日-8月26日</x:v>
       </x:c>
       <x:c r="C44" s="23" t="n">
         <x:v>7757</x:v>
       </x:c>
       <x:c r="D44" s="23" t="n">
-        <x:v>7764.4</x:v>
+        <x:v>7783.2</x:v>
       </x:c>
       <x:c r="E44" s="23" t="n">
         <x:v>7496</x:v>
       </x:c>
       <x:c r="F44" s="23" t="n">
-        <x:v>7637</x:v>
+        <x:v>7708.8</x:v>
       </x:c>
       <x:c r="G44" s="23" t="n">
         <x:f>ROUND(F44-F43,1)</x:f>
-        <x:v>-125</x:v>
+        <x:v>-53.2</x:v>
       </x:c>
       <x:c r="H44" s="24" t="n">
         <x:f>IFERROR(F44/F43-1,"")</x:f>
-        <x:v>-0.0161040968822469</x:v>
+        <x:v>-0.006853903633084246</x:v>
       </x:c>
       <x:c r="I44" s="26" t="n">
         <x:f>ROUND(D44-E44,1)</x:f>
-        <x:v>268.4</x:v>
+        <x:v>287.2</x:v>
       </x:c>
       <x:c r="J44" s="22" t="str">
         <x:v>IC2609</x:v>
       </x:c>
       <x:c r="K44" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -2765,7 +2801,7 @@
       <x:c r="H45" s="30"/>
       <x:c r="I45" s="32" t="n">
         <x:f>ROUND(SUM(I41:I44),1)</x:f>
-        <x:v>1466.4</x:v>
+        <x:v>1485.2</x:v>
       </x:c>
       <x:c r="J45" s="30"/>
       <x:c r="K45" s="30"/>
@@ -2783,7 +2819,7 @@
       <x:c r="H46" s="30"/>
       <x:c r="I46" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I41:I44),0),1)</x:f>
-        <x:v>366.6</x:v>
+        <x:v>371.3</x:v>
       </x:c>
       <x:c r="J46" s="30"/>
       <x:c r="K46" s="30"/>
@@ -3185,37 +3221,37 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B62" s="22" t="str">
-        <x:v>8月24日-8月25日</x:v>
+        <x:v>8月24日-8月26日</x:v>
       </x:c>
       <x:c r="C62" s="23" t="n">
         <x:v>2856.4</x:v>
       </x:c>
       <x:c r="D62" s="23" t="n">
-        <x:v>2866.8</x:v>
+        <x:v>2903.8</x:v>
       </x:c>
       <x:c r="E62" s="23" t="n">
         <x:v>2837.4</x:v>
       </x:c>
       <x:c r="F62" s="23" t="n">
-        <x:v>2855.2</x:v>
+        <x:v>2888.8</x:v>
       </x:c>
       <x:c r="G62" s="23" t="n">
         <x:f>ROUND(F62-F61,1)</x:f>
-        <x:v>-5.8</x:v>
+        <x:v>27.8</x:v>
       </x:c>
       <x:c r="H62" s="24" t="n">
         <x:f>IFERROR(F62/F61-1,"")</x:f>
-        <x:v>-0.0020272631946872677</x:v>
-      </x:c>
-      <x:c r="I62" s="23" t="n">
+        <x:v>0.009716882209017896</x:v>
+      </x:c>
+      <x:c r="I62" s="26" t="n">
         <x:f>ROUND(D62-E62,1)</x:f>
-        <x:v>29.4</x:v>
+        <x:v>66.4</x:v>
       </x:c>
       <x:c r="J62" s="22" t="str">
         <x:v>IH2609</x:v>
       </x:c>
       <x:c r="K62" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
@@ -3233,7 +3269,7 @@
       <x:c r="H63" s="30"/>
       <x:c r="I63" s="32" t="n">
         <x:f>ROUND(SUM(I59:I62),1)</x:f>
-        <x:v>265</x:v>
+        <x:v>302</x:v>
       </x:c>
       <x:c r="J63" s="30"/>
       <x:c r="K63" s="30"/>
@@ -3251,7 +3287,7 @@
       <x:c r="H64" s="30"/>
       <x:c r="I64" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I59:I62),0),1)</x:f>
-        <x:v>66.2</x:v>
+        <x:v>75.5</x:v>
       </x:c>
       <x:c r="J64" s="30"/>
       <x:c r="K64" s="30"/>
@@ -3419,7 +3455,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B71" s="22" t="str">
-        <x:v>8月24日-8月25日</x:v>
+        <x:v>8月24日-8月26日</x:v>
       </x:c>
       <x:c r="C71" s="23" t="n">
         <x:v>158500</x:v>
@@ -3428,28 +3464,28 @@
         <x:v>160000</x:v>
       </x:c>
       <x:c r="E71" s="23" t="n">
-        <x:v>149300</x:v>
+        <x:v>147000</x:v>
       </x:c>
       <x:c r="F71" s="23" t="n">
-        <x:v>149300</x:v>
+        <x:v>150580</x:v>
       </x:c>
       <x:c r="G71" s="28" t="n">
         <x:f>ROUND(F71-F70,1)</x:f>
-        <x:v>-6840</x:v>
+        <x:v>-5560</x:v>
       </x:c>
       <x:c r="H71" s="24" t="n">
         <x:f>IFERROR(F71/F70-1,"")</x:f>
-        <x:v>-0.04380684001537083</x:v>
+        <x:v>-0.03560906878442427</x:v>
       </x:c>
       <x:c r="I71" s="26" t="n">
         <x:f>ROUND(D71-E71,1)</x:f>
-        <x:v>10700</x:v>
+        <x:v>13000</x:v>
       </x:c>
       <x:c r="J71" s="22" t="str">
         <x:v>LC2609</x:v>
       </x:c>
       <x:c r="K71" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
@@ -3467,7 +3503,7 @@
       <x:c r="H72" s="30"/>
       <x:c r="I72" s="32" t="n">
         <x:f>ROUND(SUM(I68:I71),1)</x:f>
-        <x:v>43760</x:v>
+        <x:v>46060</x:v>
       </x:c>
       <x:c r="J72" s="30"/>
       <x:c r="K72" s="30"/>
@@ -3485,7 +3521,7 @@
       <x:c r="H73" s="30"/>
       <x:c r="I73" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I68:I71),0),1)</x:f>
-        <x:v>10940</x:v>
+        <x:v>11515</x:v>
       </x:c>
       <x:c r="J73" s="30"/>
       <x:c r="K73" s="30"/>
@@ -4175,31 +4211,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B23" s="30" t="n">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="C23" s="30"/>
-      <x:c r="D23" s="30"/>
-      <x:c r="E23" s="30"/>
-      <x:c r="F23" s="30"/>
-      <x:c r="G23" s="30"/>
-      <x:c r="H23" s="30"/>
-      <x:c r="I23" s="30"/>
-      <x:c r="J23" s="32" t="n">
-        <x:f>SUM(J4:J20)</x:f>
-        <x:v>3011</x:v>
-      </x:c>
-      <x:c r="K23" s="30"/>
+    <x:row r="21">
+      <x:c r="A21" s="22" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B21" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C21" s="22" t="str">
+        <x:v>8月26日</x:v>
+      </x:c>
+      <x:c r="D21" s="23" t="n">
+        <x:v>7536.37</x:v>
+      </x:c>
+      <x:c r="E21" s="23" t="n">
+        <x:v>7601.84</x:v>
+      </x:c>
+      <x:c r="F21" s="23" t="n">
+        <x:v>7467.41</x:v>
+      </x:c>
+      <x:c r="G21" s="23" t="n">
+        <x:v>7544.67</x:v>
+      </x:c>
+      <x:c r="H21" s="23" t="n">
+        <x:v>17.2</x:v>
+      </x:c>
+      <x:c r="I21" s="24" t="n">
+        <x:v>0.0022809697774826</x:v>
+      </x:c>
+      <x:c r="J21" s="23" t="n">
+        <x:f>ROUND(E21-F21,1)</x:f>
+        <x:v>134.4</x:v>
+      </x:c>
+      <x:c r="K21" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B24" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B24" s="30" t="n">
+        <x:v>18</x:v>
+      </x:c>
       <x:c r="C24" s="30"/>
       <x:c r="D24" s="30"/>
       <x:c r="E24" s="30"/>
@@ -4207,11 +4261,29 @@
       <x:c r="G24" s="30"/>
       <x:c r="H24" s="30"/>
       <x:c r="I24" s="30"/>
-      <x:c r="J24" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
-        <x:v>177.1</x:v>
+      <x:c r="J24" s="32" t="n">
+        <x:f>SUM(J4:J21)</x:f>
+        <x:v>3145.4</x:v>
       </x:c>
       <x:c r="K24" s="30"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B25" s="30"/>
+      <x:c r="C25" s="30"/>
+      <x:c r="D25" s="30"/>
+      <x:c r="E25" s="30"/>
+      <x:c r="F25" s="30"/>
+      <x:c r="G25" s="30"/>
+      <x:c r="H25" s="30"/>
+      <x:c r="I25" s="30"/>
+      <x:c r="J25" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J21),0),1)</x:f>
+        <x:v>174.7</x:v>
+      </x:c>
+      <x:c r="K25" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4890,31 +4962,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B23" s="30" t="n">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="C23" s="30"/>
-      <x:c r="D23" s="30"/>
-      <x:c r="E23" s="30"/>
-      <x:c r="F23" s="30"/>
-      <x:c r="G23" s="30"/>
-      <x:c r="H23" s="30"/>
-      <x:c r="I23" s="30"/>
-      <x:c r="J23" s="32" t="n">
-        <x:f>SUM(J4:J20)</x:f>
-        <x:v>2883.5</x:v>
-      </x:c>
-      <x:c r="K23" s="30"/>
+    <x:row r="21">
+      <x:c r="A21" s="22" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B21" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C21" s="22" t="str">
+        <x:v>8月26日</x:v>
+      </x:c>
+      <x:c r="D21" s="23" t="n">
+        <x:v>7714.84</x:v>
+      </x:c>
+      <x:c r="E21" s="23" t="n">
+        <x:v>7833.6</x:v>
+      </x:c>
+      <x:c r="F21" s="23" t="n">
+        <x:v>7699.42</x:v>
+      </x:c>
+      <x:c r="G21" s="23" t="n">
+        <x:v>7770.53</x:v>
+      </x:c>
+      <x:c r="H21" s="23" t="n">
+        <x:v>59.6</x:v>
+      </x:c>
+      <x:c r="I21" s="24" t="n">
+        <x:v>0.007727981283734531</x:v>
+      </x:c>
+      <x:c r="J21" s="23" t="n">
+        <x:f>ROUND(E21-F21,1)</x:f>
+        <x:v>134.2</x:v>
+      </x:c>
+      <x:c r="K21" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B24" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B24" s="30" t="n">
+        <x:v>18</x:v>
+      </x:c>
       <x:c r="C24" s="30"/>
       <x:c r="D24" s="30"/>
       <x:c r="E24" s="30"/>
@@ -4922,11 +5012,29 @@
       <x:c r="G24" s="30"/>
       <x:c r="H24" s="30"/>
       <x:c r="I24" s="30"/>
-      <x:c r="J24" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
-        <x:v>169.6</x:v>
+      <x:c r="J24" s="32" t="n">
+        <x:f>SUM(J4:J21)</x:f>
+        <x:v>3017.7</x:v>
       </x:c>
       <x:c r="K24" s="30"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B25" s="30"/>
+      <x:c r="C25" s="30"/>
+      <x:c r="D25" s="30"/>
+      <x:c r="E25" s="30"/>
+      <x:c r="F25" s="30"/>
+      <x:c r="G25" s="30"/>
+      <x:c r="H25" s="30"/>
+      <x:c r="I25" s="30"/>
+      <x:c r="J25" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J21),0),1)</x:f>
+        <x:v>167.6</x:v>
+      </x:c>
+      <x:c r="K25" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5605,31 +5713,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B23" s="30" t="n">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="C23" s="30"/>
-      <x:c r="D23" s="30"/>
-      <x:c r="E23" s="30"/>
-      <x:c r="F23" s="30"/>
-      <x:c r="G23" s="30"/>
-      <x:c r="H23" s="30"/>
-      <x:c r="I23" s="30"/>
-      <x:c r="J23" s="32" t="n">
-        <x:f>SUM(J4:J20)</x:f>
-        <x:v>730.0999999999999</x:v>
-      </x:c>
-      <x:c r="K23" s="30"/>
+    <x:row r="21">
+      <x:c r="A21" s="22" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B21" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C21" s="22" t="str">
+        <x:v>8月26日</x:v>
+      </x:c>
+      <x:c r="D21" s="23" t="n">
+        <x:v>3881.74</x:v>
+      </x:c>
+      <x:c r="E21" s="23" t="n">
+        <x:v>3926.44</x:v>
+      </x:c>
+      <x:c r="F21" s="23" t="n">
+        <x:v>3881.74</x:v>
+      </x:c>
+      <x:c r="G21" s="23" t="n">
+        <x:v>3912.52</x:v>
+      </x:c>
+      <x:c r="H21" s="23" t="n">
+        <x:v>23.1</x:v>
+      </x:c>
+      <x:c r="I21" s="24" t="n">
+        <x:v>0.005934016207988835</x:v>
+      </x:c>
+      <x:c r="J21" s="23" t="n">
+        <x:f>ROUND(E21-F21,1)</x:f>
+        <x:v>44.7</x:v>
+      </x:c>
+      <x:c r="K21" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B24" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B24" s="30" t="n">
+        <x:v>18</x:v>
+      </x:c>
       <x:c r="C24" s="30"/>
       <x:c r="D24" s="30"/>
       <x:c r="E24" s="30"/>
@@ -5637,11 +5763,29 @@
       <x:c r="G24" s="30"/>
       <x:c r="H24" s="30"/>
       <x:c r="I24" s="30"/>
-      <x:c r="J24" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
-        <x:v>42.9</x:v>
+      <x:c r="J24" s="32" t="n">
+        <x:f>SUM(J4:J21)</x:f>
+        <x:v>774.8</x:v>
       </x:c>
       <x:c r="K24" s="30"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B25" s="30"/>
+      <x:c r="C25" s="30"/>
+      <x:c r="D25" s="30"/>
+      <x:c r="E25" s="30"/>
+      <x:c r="F25" s="30"/>
+      <x:c r="G25" s="30"/>
+      <x:c r="H25" s="30"/>
+      <x:c r="I25" s="30"/>
+      <x:c r="J25" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J21),0),1)</x:f>
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="K25" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -7035,31 +7179,49 @@
         <x:v>IC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B23" s="30" t="n">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="C23" s="30"/>
-      <x:c r="D23" s="30"/>
-      <x:c r="E23" s="30"/>
-      <x:c r="F23" s="30"/>
-      <x:c r="G23" s="30"/>
-      <x:c r="H23" s="30"/>
-      <x:c r="I23" s="30"/>
-      <x:c r="J23" s="32" t="n">
-        <x:f>SUM(J4:J20)</x:f>
-        <x:v>2876.4</x:v>
-      </x:c>
-      <x:c r="K23" s="30"/>
+    <x:row r="21">
+      <x:c r="A21" s="22" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B21" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C21" s="22" t="str">
+        <x:v>8月26日</x:v>
+      </x:c>
+      <x:c r="D21" s="23" t="n">
+        <x:v>7633.8</x:v>
+      </x:c>
+      <x:c r="E21" s="23" t="n">
+        <x:v>7783.2</x:v>
+      </x:c>
+      <x:c r="F21" s="23" t="n">
+        <x:v>7604</x:v>
+      </x:c>
+      <x:c r="G21" s="23" t="n">
+        <x:v>7708.8</x:v>
+      </x:c>
+      <x:c r="H21" s="23" t="n">
+        <x:v>71.8</x:v>
+      </x:c>
+      <x:c r="I21" s="24" t="n">
+        <x:v>0.00940159748592384</x:v>
+      </x:c>
+      <x:c r="J21" s="26" t="n">
+        <x:f>ROUND(E21-F21,1)</x:f>
+        <x:v>179.2</x:v>
+      </x:c>
+      <x:c r="K21" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B24" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B24" s="30" t="n">
+        <x:v>18</x:v>
+      </x:c>
       <x:c r="C24" s="30"/>
       <x:c r="D24" s="30"/>
       <x:c r="E24" s="30"/>
@@ -7067,11 +7229,29 @@
       <x:c r="G24" s="30"/>
       <x:c r="H24" s="30"/>
       <x:c r="I24" s="30"/>
-      <x:c r="J24" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
-        <x:v>169.2</x:v>
+      <x:c r="J24" s="32" t="n">
+        <x:f>SUM(J4:J21)</x:f>
+        <x:v>3055.6</x:v>
       </x:c>
       <x:c r="K24" s="30"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B25" s="30"/>
+      <x:c r="C25" s="30"/>
+      <x:c r="D25" s="30"/>
+      <x:c r="E25" s="30"/>
+      <x:c r="F25" s="30"/>
+      <x:c r="G25" s="30"/>
+      <x:c r="H25" s="30"/>
+      <x:c r="I25" s="30"/>
+      <x:c r="J25" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J21),0),1)</x:f>
+        <x:v>169.8</x:v>
+      </x:c>
+      <x:c r="K25" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -8465,31 +8645,49 @@
         <x:v>IH2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B23" s="30" t="n">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="C23" s="30"/>
-      <x:c r="D23" s="30"/>
-      <x:c r="E23" s="30"/>
-      <x:c r="F23" s="30"/>
-      <x:c r="G23" s="30"/>
-      <x:c r="H23" s="30"/>
-      <x:c r="I23" s="30"/>
-      <x:c r="J23" s="32" t="n">
-        <x:f>SUM(J4:J20)</x:f>
-        <x:v>562.4000000000001</x:v>
-      </x:c>
-      <x:c r="K23" s="30"/>
+    <x:row r="21">
+      <x:c r="A21" s="22" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B21" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C21" s="22" t="str">
+        <x:v>8月26日</x:v>
+      </x:c>
+      <x:c r="D21" s="23" t="n">
+        <x:v>2850</x:v>
+      </x:c>
+      <x:c r="E21" s="23" t="n">
+        <x:v>2903.8</x:v>
+      </x:c>
+      <x:c r="F21" s="23" t="n">
+        <x:v>2850</x:v>
+      </x:c>
+      <x:c r="G21" s="23" t="n">
+        <x:v>2888.8</x:v>
+      </x:c>
+      <x:c r="H21" s="23" t="n">
+        <x:v>33.6</x:v>
+      </x:c>
+      <x:c r="I21" s="24" t="n">
+        <x:v>0.0117680022415243</x:v>
+      </x:c>
+      <x:c r="J21" s="23" t="n">
+        <x:f>ROUND(E21-F21,1)</x:f>
+        <x:v>53.8</x:v>
+      </x:c>
+      <x:c r="K21" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B24" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B24" s="30" t="n">
+        <x:v>18</x:v>
+      </x:c>
       <x:c r="C24" s="30"/>
       <x:c r="D24" s="30"/>
       <x:c r="E24" s="30"/>
@@ -8497,11 +8695,29 @@
       <x:c r="G24" s="30"/>
       <x:c r="H24" s="30"/>
       <x:c r="I24" s="30"/>
-      <x:c r="J24" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
-        <x:v>33.1</x:v>
+      <x:c r="J24" s="32" t="n">
+        <x:f>SUM(J4:J21)</x:f>
+        <x:v>616.2</x:v>
       </x:c>
       <x:c r="K24" s="30"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B25" s="30"/>
+      <x:c r="C25" s="30"/>
+      <x:c r="D25" s="30"/>
+      <x:c r="E25" s="30"/>
+      <x:c r="F25" s="30"/>
+      <x:c r="G25" s="30"/>
+      <x:c r="H25" s="30"/>
+      <x:c r="I25" s="30"/>
+      <x:c r="J25" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J21),0),1)</x:f>
+        <x:v>34.2</x:v>
+      </x:c>
+      <x:c r="K25" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-08-27
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R37e217b39da94260"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R5239e188f9e8483f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R71658e28c3dd4ff8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Re4e73ae44ed34db5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Re6d214f3b9c345b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rb2984efd1d524edd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Rd60ae79767674939"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R6e33dce0b8834083"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R9b2dfe13664c4c63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R7c99fe8ab28b4945"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R30c312f536874f9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Rcd7381a9fd744f94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Rc4399d309aa249f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Re210cfc3f87f4056"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R2c5f0cd816bb4b5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Re6f0e39e93a5443b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R5692245066024be1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R2afd88d404944147"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R9440f040348b4d52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R3270b954ebe74271"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -520,25 +520,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-08-26</x:v>
+        <x:v>2026-08-27</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7601.84</x:v>
+        <x:v>7734.31</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7467.41</x:v>
+        <x:v>7531.78</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>134.4</x:v>
+        <x:v>202.5</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>3145.4</x:v>
+        <x:v>3347.9</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>174.7</x:v>
+        <x:v>176.2</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -549,25 +549,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-08-26</x:v>
+        <x:v>2026-08-27</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7833.6</x:v>
+        <x:v>7951.05</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7699.42</x:v>
+        <x:v>7763.98</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>134.2</x:v>
+        <x:v>187.1</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>3017.7</x:v>
+        <x:v>3204.8</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>167.6</x:v>
+        <x:v>168.7</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -578,25 +578,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-08-26</x:v>
+        <x:v>2026-08-27</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3926.44</x:v>
+        <x:v>3958.03</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3881.74</x:v>
+        <x:v>3909.31</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>44.7</x:v>
+        <x:v>48.7</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>774.8</x:v>
+        <x:v>823.5</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>43</x:v>
+        <x:v>43.3</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -607,25 +607,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-08-26</x:v>
+        <x:v>2026-08-27</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>7558</x:v>
+        <x:v>7696</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>7395</x:v>
+        <x:v>7472</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>163</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>3108</x:v>
+        <x:v>3332</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>172.7</x:v>
+        <x:v>175.4</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -636,25 +636,25 @@
         <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>2026-08-26</x:v>
+        <x:v>2026-08-27</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:v>7783.2</x:v>
+        <x:v>7907</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>7604</x:v>
+        <x:v>7700</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>179.2</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>3055.6</x:v>
+        <x:v>3262.6</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
-        <x:v>169.8</x:v>
+        <x:v>171.7</x:v>
       </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
@@ -665,25 +665,25 @@
         <x:v>IF主力</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>2026-08-26</x:v>
+        <x:v>2026-08-27</x:v>
       </x:c>
       <x:c r="C9" s="10" t="n">
-        <x:v>4593.6</x:v>
+        <x:v>4608.2</x:v>
       </x:c>
       <x:c r="D9" s="10" t="n">
-        <x:v>4515.6</x:v>
+        <x:v>4561.8</x:v>
       </x:c>
       <x:c r="E9" s="12" t="n">
-        <x:v>78</x:v>
+        <x:v>46.4</x:v>
       </x:c>
       <x:c r="F9" s="9" t="n">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="G9" s="10" t="n">
-        <x:v>1169.2</x:v>
+        <x:v>1215.6</x:v>
       </x:c>
       <x:c r="H9" s="10" t="n">
-        <x:v>65</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="I9" s="10" t="n">
         <x:v>90</x:v>
@@ -694,25 +694,25 @@
         <x:v>IH主力</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>2026-08-26</x:v>
+        <x:v>2026-08-27</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:v>2903.8</x:v>
+        <x:v>2916.2</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
-        <x:v>2850</x:v>
+        <x:v>2890.4</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
-        <x:v>53.8</x:v>
+        <x:v>25.8</x:v>
       </x:c>
       <x:c r="F10" s="9" t="n">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="G10" s="10" t="n">
-        <x:v>616.2</x:v>
+        <x:v>642</x:v>
       </x:c>
       <x:c r="H10" s="10" t="n">
-        <x:v>34.2</x:v>
+        <x:v>33.8</x:v>
       </x:c>
       <x:c r="I10" s="10" t="n">
         <x:v>60</x:v>
@@ -755,7 +755,7 @@
         <x:v>2026-08-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-08-26</x:v>
+        <x:v>2026-08-27</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1817,37 +1817,37 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B8" s="22" t="str">
-        <x:v>8月24日-8月26日</x:v>
+        <x:v>8月24日-8月27日</x:v>
       </x:c>
       <x:c r="C8" s="23" t="n">
         <x:v>7614.89</x:v>
       </x:c>
       <x:c r="D8" s="23" t="n">
-        <x:v>7633.34</x:v>
+        <x:v>7734.31</x:v>
       </x:c>
       <x:c r="E8" s="23" t="n">
         <x:v>7347.95</x:v>
       </x:c>
       <x:c r="F8" s="23" t="n">
-        <x:v>7544.67</x:v>
+        <x:v>7732.95</x:v>
       </x:c>
       <x:c r="G8" s="23" t="n">
         <x:f>ROUND(F8-F7,1)</x:f>
-        <x:v>-57.1</x:v>
+        <x:v>131.1</x:v>
       </x:c>
       <x:c r="H8" s="24" t="n">
         <x:f>IFERROR(F8/F7-1,"")</x:f>
-        <x:v>-0.007515325317687949</x:v>
+        <x:v>0.017252492830645227</x:v>
       </x:c>
       <x:c r="I8" s="26" t="n">
         <x:f>ROUND(D8-E8,1)</x:f>
-        <x:v>285.4</x:v>
+        <x:v>386.4</x:v>
       </x:c>
       <x:c r="J8" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K8" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1865,7 +1865,7 @@
       <x:c r="H9" s="30"/>
       <x:c r="I9" s="32" t="n">
         <x:f>ROUND(SUM(I5:I8),1)</x:f>
-        <x:v>1709.7</x:v>
+        <x:v>1810.7</x:v>
       </x:c>
       <x:c r="J9" s="30"/>
       <x:c r="K9" s="30"/>
@@ -1883,7 +1883,7 @@
       <x:c r="H10" s="30"/>
       <x:c r="I10" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I8),0),1)</x:f>
-        <x:v>427.4</x:v>
+        <x:v>452.7</x:v>
       </x:c>
       <x:c r="J10" s="30"/>
       <x:c r="K10" s="30"/>
@@ -2051,37 +2051,37 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B17" s="22" t="str">
-        <x:v>8月24日-8月26日</x:v>
+        <x:v>8月24日-8月27日</x:v>
       </x:c>
       <x:c r="C17" s="23" t="n">
         <x:v>7861.05</x:v>
       </x:c>
       <x:c r="D17" s="23" t="n">
-        <x:v>7865.54</x:v>
+        <x:v>7951.05</x:v>
       </x:c>
       <x:c r="E17" s="23" t="n">
         <x:v>7572.86</x:v>
       </x:c>
       <x:c r="F17" s="23" t="n">
-        <x:v>7770.53</x:v>
+        <x:v>7946.33</x:v>
       </x:c>
       <x:c r="G17" s="23" t="n">
         <x:f>ROUND(F17-F16,1)</x:f>
-        <x:v>-83.8</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="H17" s="24" t="n">
         <x:f>IFERROR(F17/F16-1,"")</x:f>
-        <x:v>-0.010669274145598706</x:v>
+        <x:v>0.011713284264857737</x:v>
       </x:c>
       <x:c r="I17" s="26" t="n">
         <x:f>ROUND(D17-E17,1)</x:f>
-        <x:v>292.7</x:v>
+        <x:v>378.2</x:v>
       </x:c>
       <x:c r="J17" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K17" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -2099,7 +2099,7 @@
       <x:c r="H18" s="30"/>
       <x:c r="I18" s="32" t="n">
         <x:f>ROUND(SUM(I14:I17),1)</x:f>
-        <x:v>1578</x:v>
+        <x:v>1663.5</x:v>
       </x:c>
       <x:c r="J18" s="30"/>
       <x:c r="K18" s="30"/>
@@ -2117,7 +2117,7 @@
       <x:c r="H19" s="30"/>
       <x:c r="I19" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I14:I17),0),1)</x:f>
-        <x:v>394.5</x:v>
+        <x:v>415.9</x:v>
       </x:c>
       <x:c r="J19" s="30"/>
       <x:c r="K19" s="30"/>
@@ -2285,37 +2285,37 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B26" s="22" t="str">
-        <x:v>8月24日-8月26日</x:v>
+        <x:v>8月24日-8月27日</x:v>
       </x:c>
       <x:c r="C26" s="23" t="n">
         <x:v>3902.7</x:v>
       </x:c>
       <x:c r="D26" s="23" t="n">
-        <x:v>3926.44</x:v>
+        <x:v>3958.03</x:v>
       </x:c>
       <x:c r="E26" s="23" t="n">
         <x:v>3850.86</x:v>
       </x:c>
       <x:c r="F26" s="23" t="n">
-        <x:v>3912.52</x:v>
+        <x:v>3956.57</x:v>
       </x:c>
       <x:c r="G26" s="23" t="n">
         <x:f>ROUND(F26-F25,1)</x:f>
-        <x:v>7.3</x:v>
+        <x:v>51.4</x:v>
       </x:c>
       <x:c r="H26" s="24" t="n">
         <x:f>IFERROR(F26/F25-1,"")</x:f>
-        <x:v>0.0018744238451295914</x:v>
+        <x:v>0.013154255863976339</x:v>
       </x:c>
       <x:c r="I26" s="26" t="n">
         <x:f>ROUND(D26-E26,1)</x:f>
-        <x:v>75.6</x:v>
+        <x:v>107.2</x:v>
       </x:c>
       <x:c r="J26" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K26" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -2333,7 +2333,7 @@
       <x:c r="H27" s="30"/>
       <x:c r="I27" s="32" t="n">
         <x:f>ROUND(SUM(I23:I26),1)</x:f>
-        <x:v>398.3</x:v>
+        <x:v>429.9</x:v>
       </x:c>
       <x:c r="J27" s="30"/>
       <x:c r="K27" s="30"/>
@@ -2351,7 +2351,7 @@
       <x:c r="H28" s="30"/>
       <x:c r="I28" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I23:I26),0),1)</x:f>
-        <x:v>99.6</x:v>
+        <x:v>107.5</x:v>
       </x:c>
       <x:c r="J28" s="30"/>
       <x:c r="K28" s="30"/>
@@ -2519,37 +2519,37 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B35" s="22" t="str">
-        <x:v>8月24日-8月26日</x:v>
+        <x:v>8月24日-8月27日</x:v>
       </x:c>
       <x:c r="C35" s="23" t="n">
         <x:v>7534.8</x:v>
       </x:c>
       <x:c r="D35" s="23" t="n">
-        <x:v>7558</x:v>
+        <x:v>7696</x:v>
       </x:c>
       <x:c r="E35" s="23" t="n">
         <x:v>7300.2</x:v>
       </x:c>
       <x:c r="F35" s="23" t="n">
-        <x:v>7491.8</x:v>
-      </x:c>
-      <x:c r="G35" s="23" t="n">
+        <x:v>7686.6</x:v>
+      </x:c>
+      <x:c r="G35" s="28" t="n">
         <x:f>ROUND(F35-F34,1)</x:f>
-        <x:v>-35.2</x:v>
+        <x:v>159.6</x:v>
       </x:c>
       <x:c r="H35" s="24" t="n">
         <x:f>IFERROR(F35/F34-1,"")</x:f>
-        <x:v>-0.004676497940746649</x:v>
+        <x:v>0.02120366679952168</x:v>
       </x:c>
       <x:c r="I35" s="26" t="n">
         <x:f>ROUND(D35-E35,1)</x:f>
-        <x:v>257.8</x:v>
+        <x:v>395.8</x:v>
       </x:c>
       <x:c r="J35" s="22" t="str">
         <x:v>IM2609</x:v>
       </x:c>
       <x:c r="K35" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -2567,7 +2567,7 @@
       <x:c r="H36" s="30"/>
       <x:c r="I36" s="32" t="n">
         <x:f>ROUND(SUM(I32:I35),1)</x:f>
-        <x:v>1599.8</x:v>
+        <x:v>1737.8</x:v>
       </x:c>
       <x:c r="J36" s="30"/>
       <x:c r="K36" s="30"/>
@@ -2585,7 +2585,7 @@
       <x:c r="H37" s="30"/>
       <x:c r="I37" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I32:I35),0),1)</x:f>
-        <x:v>400</x:v>
+        <x:v>434.5</x:v>
       </x:c>
       <x:c r="J37" s="30"/>
       <x:c r="K37" s="30"/>
@@ -2753,37 +2753,37 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B44" s="22" t="str">
-        <x:v>8月24日-8月26日</x:v>
+        <x:v>8月24日-8月27日</x:v>
       </x:c>
       <x:c r="C44" s="23" t="n">
         <x:v>7757</x:v>
       </x:c>
       <x:c r="D44" s="23" t="n">
-        <x:v>7783.2</x:v>
+        <x:v>7907</x:v>
       </x:c>
       <x:c r="E44" s="23" t="n">
         <x:v>7496</x:v>
       </x:c>
       <x:c r="F44" s="23" t="n">
-        <x:v>7708.8</x:v>
+        <x:v>7903</x:v>
       </x:c>
       <x:c r="G44" s="23" t="n">
         <x:f>ROUND(F44-F43,1)</x:f>
-        <x:v>-53.2</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="H44" s="24" t="n">
         <x:f>IFERROR(F44/F43-1,"")</x:f>
-        <x:v>-0.006853903633084246</x:v>
+        <x:v>0.018165421283174332</x:v>
       </x:c>
       <x:c r="I44" s="26" t="n">
         <x:f>ROUND(D44-E44,1)</x:f>
-        <x:v>287.2</x:v>
+        <x:v>411</x:v>
       </x:c>
       <x:c r="J44" s="22" t="str">
         <x:v>IC2609</x:v>
       </x:c>
       <x:c r="K44" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -2801,7 +2801,7 @@
       <x:c r="H45" s="30"/>
       <x:c r="I45" s="32" t="n">
         <x:f>ROUND(SUM(I41:I44),1)</x:f>
-        <x:v>1485.2</x:v>
+        <x:v>1609</x:v>
       </x:c>
       <x:c r="J45" s="30"/>
       <x:c r="K45" s="30"/>
@@ -2819,7 +2819,7 @@
       <x:c r="H46" s="30"/>
       <x:c r="I46" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I41:I44),0),1)</x:f>
-        <x:v>371.3</x:v>
+        <x:v>402.3</x:v>
       </x:c>
       <x:c r="J46" s="30"/>
       <x:c r="K46" s="30"/>
@@ -2987,37 +2987,37 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B53" s="22" t="str">
-        <x:v>8月24日-8月26日</x:v>
+        <x:v>8月24日-8月27日</x:v>
       </x:c>
       <x:c r="C53" s="23" t="n">
         <x:v>4607.4</x:v>
       </x:c>
       <x:c r="D53" s="23" t="n">
-        <x:v>4607.4</x:v>
+        <x:v>4608.2</x:v>
       </x:c>
       <x:c r="E53" s="23" t="n">
         <x:v>4486.4</x:v>
       </x:c>
       <x:c r="F53" s="23" t="n">
-        <x:v>4566.8</x:v>
+        <x:v>4604.8</x:v>
       </x:c>
       <x:c r="G53" s="23" t="n">
         <x:f>ROUND(F53-F52,1)</x:f>
-        <x:v>-9.2</x:v>
+        <x:v>28.8</x:v>
       </x:c>
       <x:c r="H53" s="24" t="n">
         <x:f>IFERROR(F53/F52-1,"")</x:f>
-        <x:v>-0.0020104895104894327</x:v>
+        <x:v>0.0062937062937062915</x:v>
       </x:c>
       <x:c r="I53" s="26" t="n">
         <x:f>ROUND(D53-E53,1)</x:f>
-        <x:v>121</x:v>
+        <x:v>121.8</x:v>
       </x:c>
       <x:c r="J53" s="22" t="str">
         <x:v>IF2609</x:v>
       </x:c>
       <x:c r="K53" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -3035,7 +3035,7 @@
       <x:c r="H54" s="30"/>
       <x:c r="I54" s="32" t="n">
         <x:f>ROUND(SUM(I50:I53),1)</x:f>
-        <x:v>534.8</x:v>
+        <x:v>535.6</x:v>
       </x:c>
       <x:c r="J54" s="30"/>
       <x:c r="K54" s="30"/>
@@ -3053,7 +3053,7 @@
       <x:c r="H55" s="30"/>
       <x:c r="I55" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I50:I53),0),1)</x:f>
-        <x:v>133.7</x:v>
+        <x:v>133.9</x:v>
       </x:c>
       <x:c r="J55" s="30"/>
       <x:c r="K55" s="30"/>
@@ -3221,37 +3221,37 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B62" s="22" t="str">
-        <x:v>8月24日-8月26日</x:v>
+        <x:v>8月24日-8月27日</x:v>
       </x:c>
       <x:c r="C62" s="23" t="n">
         <x:v>2856.4</x:v>
       </x:c>
       <x:c r="D62" s="23" t="n">
-        <x:v>2903.8</x:v>
+        <x:v>2916.2</x:v>
       </x:c>
       <x:c r="E62" s="23" t="n">
         <x:v>2837.4</x:v>
       </x:c>
       <x:c r="F62" s="23" t="n">
-        <x:v>2888.8</x:v>
+        <x:v>2914</x:v>
       </x:c>
       <x:c r="G62" s="23" t="n">
         <x:f>ROUND(F62-F61,1)</x:f>
-        <x:v>27.8</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="H62" s="24" t="n">
         <x:f>IFERROR(F62/F61-1,"")</x:f>
-        <x:v>0.009716882209017896</x:v>
+        <x:v>0.01852499126179663</x:v>
       </x:c>
       <x:c r="I62" s="26" t="n">
         <x:f>ROUND(D62-E62,1)</x:f>
-        <x:v>66.4</x:v>
+        <x:v>78.8</x:v>
       </x:c>
       <x:c r="J62" s="22" t="str">
         <x:v>IH2609</x:v>
       </x:c>
       <x:c r="K62" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
@@ -3269,7 +3269,7 @@
       <x:c r="H63" s="30"/>
       <x:c r="I63" s="32" t="n">
         <x:f>ROUND(SUM(I59:I62),1)</x:f>
-        <x:v>302</x:v>
+        <x:v>314.4</x:v>
       </x:c>
       <x:c r="J63" s="30"/>
       <x:c r="K63" s="30"/>
@@ -3287,7 +3287,7 @@
       <x:c r="H64" s="30"/>
       <x:c r="I64" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I59:I62),0),1)</x:f>
-        <x:v>75.5</x:v>
+        <x:v>78.6</x:v>
       </x:c>
       <x:c r="J64" s="30"/>
       <x:c r="K64" s="30"/>
@@ -4247,31 +4247,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B24" s="30" t="n">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C24" s="30"/>
-      <x:c r="D24" s="30"/>
-      <x:c r="E24" s="30"/>
-      <x:c r="F24" s="30"/>
-      <x:c r="G24" s="30"/>
-      <x:c r="H24" s="30"/>
-      <x:c r="I24" s="30"/>
-      <x:c r="J24" s="32" t="n">
-        <x:f>SUM(J4:J21)</x:f>
-        <x:v>3145.4</x:v>
-      </x:c>
-      <x:c r="K24" s="30"/>
+    <x:row r="22">
+      <x:c r="A22" s="22" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B22" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C22" s="22" t="str">
+        <x:v>8月27日</x:v>
+      </x:c>
+      <x:c r="D22" s="23" t="n">
+        <x:v>7551.44</x:v>
+      </x:c>
+      <x:c r="E22" s="23" t="n">
+        <x:v>7734.31</x:v>
+      </x:c>
+      <x:c r="F22" s="23" t="n">
+        <x:v>7531.78</x:v>
+      </x:c>
+      <x:c r="G22" s="23" t="n">
+        <x:v>7732.95</x:v>
+      </x:c>
+      <x:c r="H22" s="28" t="n">
+        <x:v>188.3</x:v>
+      </x:c>
+      <x:c r="I22" s="24" t="n">
+        <x:v>0.024955365841050625</x:v>
+      </x:c>
+      <x:c r="J22" s="26" t="n">
+        <x:f>ROUND(E22-F22,1)</x:f>
+        <x:v>202.5</x:v>
+      </x:c>
+      <x:c r="K22" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B25" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B25" s="30" t="n">
+        <x:v>19</x:v>
+      </x:c>
       <x:c r="C25" s="30"/>
       <x:c r="D25" s="30"/>
       <x:c r="E25" s="30"/>
@@ -4279,11 +4297,29 @@
       <x:c r="G25" s="30"/>
       <x:c r="H25" s="30"/>
       <x:c r="I25" s="30"/>
-      <x:c r="J25" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J21),0),1)</x:f>
-        <x:v>174.7</x:v>
+      <x:c r="J25" s="32" t="n">
+        <x:f>SUM(J4:J22)</x:f>
+        <x:v>3347.9</x:v>
       </x:c>
       <x:c r="K25" s="30"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B26" s="30"/>
+      <x:c r="C26" s="30"/>
+      <x:c r="D26" s="30"/>
+      <x:c r="E26" s="30"/>
+      <x:c r="F26" s="30"/>
+      <x:c r="G26" s="30"/>
+      <x:c r="H26" s="30"/>
+      <x:c r="I26" s="30"/>
+      <x:c r="J26" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J22),0),1)</x:f>
+        <x:v>176.2</x:v>
+      </x:c>
+      <x:c r="K26" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4998,31 +5034,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B24" s="30" t="n">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C24" s="30"/>
-      <x:c r="D24" s="30"/>
-      <x:c r="E24" s="30"/>
-      <x:c r="F24" s="30"/>
-      <x:c r="G24" s="30"/>
-      <x:c r="H24" s="30"/>
-      <x:c r="I24" s="30"/>
-      <x:c r="J24" s="32" t="n">
-        <x:f>SUM(J4:J21)</x:f>
-        <x:v>3017.7</x:v>
-      </x:c>
-      <x:c r="K24" s="30"/>
+    <x:row r="22">
+      <x:c r="A22" s="22" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B22" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C22" s="22" t="str">
+        <x:v>8月27日</x:v>
+      </x:c>
+      <x:c r="D22" s="23" t="n">
+        <x:v>7786.69</x:v>
+      </x:c>
+      <x:c r="E22" s="23" t="n">
+        <x:v>7951.05</x:v>
+      </x:c>
+      <x:c r="F22" s="23" t="n">
+        <x:v>7763.98</x:v>
+      </x:c>
+      <x:c r="G22" s="23" t="n">
+        <x:v>7946.33</x:v>
+      </x:c>
+      <x:c r="H22" s="28" t="n">
+        <x:v>175.8</x:v>
+      </x:c>
+      <x:c r="I22" s="24" t="n">
+        <x:v>0.02262393942240748</x:v>
+      </x:c>
+      <x:c r="J22" s="26" t="n">
+        <x:f>ROUND(E22-F22,1)</x:f>
+        <x:v>187.1</x:v>
+      </x:c>
+      <x:c r="K22" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B25" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B25" s="30" t="n">
+        <x:v>19</x:v>
+      </x:c>
       <x:c r="C25" s="30"/>
       <x:c r="D25" s="30"/>
       <x:c r="E25" s="30"/>
@@ -5030,11 +5084,29 @@
       <x:c r="G25" s="30"/>
       <x:c r="H25" s="30"/>
       <x:c r="I25" s="30"/>
-      <x:c r="J25" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J21),0),1)</x:f>
-        <x:v>167.6</x:v>
+      <x:c r="J25" s="32" t="n">
+        <x:f>SUM(J4:J22)</x:f>
+        <x:v>3204.7999999999997</x:v>
       </x:c>
       <x:c r="K25" s="30"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B26" s="30"/>
+      <x:c r="C26" s="30"/>
+      <x:c r="D26" s="30"/>
+      <x:c r="E26" s="30"/>
+      <x:c r="F26" s="30"/>
+      <x:c r="G26" s="30"/>
+      <x:c r="H26" s="30"/>
+      <x:c r="I26" s="30"/>
+      <x:c r="J26" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J22),0),1)</x:f>
+        <x:v>168.7</x:v>
+      </x:c>
+      <x:c r="K26" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5749,31 +5821,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B24" s="30" t="n">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C24" s="30"/>
-      <x:c r="D24" s="30"/>
-      <x:c r="E24" s="30"/>
-      <x:c r="F24" s="30"/>
-      <x:c r="G24" s="30"/>
-      <x:c r="H24" s="30"/>
-      <x:c r="I24" s="30"/>
-      <x:c r="J24" s="32" t="n">
-        <x:f>SUM(J4:J21)</x:f>
-        <x:v>774.8</x:v>
-      </x:c>
-      <x:c r="K24" s="30"/>
+    <x:row r="22">
+      <x:c r="A22" s="22" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B22" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C22" s="22" t="str">
+        <x:v>8月27日</x:v>
+      </x:c>
+      <x:c r="D22" s="23" t="n">
+        <x:v>3911.89</x:v>
+      </x:c>
+      <x:c r="E22" s="23" t="n">
+        <x:v>3958.03</x:v>
+      </x:c>
+      <x:c r="F22" s="23" t="n">
+        <x:v>3909.31</x:v>
+      </x:c>
+      <x:c r="G22" s="23" t="n">
+        <x:v>3956.57</x:v>
+      </x:c>
+      <x:c r="H22" s="23" t="n">
+        <x:v>44.1</x:v>
+      </x:c>
+      <x:c r="I22" s="24" t="n">
+        <x:v>0.01125872838988684</x:v>
+      </x:c>
+      <x:c r="J22" s="23" t="n">
+        <x:f>ROUND(E22-F22,1)</x:f>
+        <x:v>48.7</x:v>
+      </x:c>
+      <x:c r="K22" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B25" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B25" s="30" t="n">
+        <x:v>19</x:v>
+      </x:c>
       <x:c r="C25" s="30"/>
       <x:c r="D25" s="30"/>
       <x:c r="E25" s="30"/>
@@ -5781,11 +5871,29 @@
       <x:c r="G25" s="30"/>
       <x:c r="H25" s="30"/>
       <x:c r="I25" s="30"/>
-      <x:c r="J25" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J21),0),1)</x:f>
-        <x:v>43</x:v>
+      <x:c r="J25" s="32" t="n">
+        <x:f>SUM(J4:J22)</x:f>
+        <x:v>823.5</x:v>
       </x:c>
       <x:c r="K25" s="30"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B26" s="30"/>
+      <x:c r="C26" s="30"/>
+      <x:c r="D26" s="30"/>
+      <x:c r="E26" s="30"/>
+      <x:c r="F26" s="30"/>
+      <x:c r="G26" s="30"/>
+      <x:c r="H26" s="30"/>
+      <x:c r="I26" s="30"/>
+      <x:c r="J26" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J22),0),1)</x:f>
+        <x:v>43.3</x:v>
+      </x:c>
+      <x:c r="K26" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -6500,31 +6608,49 @@
         <x:v>IM2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B24" s="30" t="n">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C24" s="30"/>
-      <x:c r="D24" s="30"/>
-      <x:c r="E24" s="30"/>
-      <x:c r="F24" s="30"/>
-      <x:c r="G24" s="30"/>
-      <x:c r="H24" s="30"/>
-      <x:c r="I24" s="30"/>
-      <x:c r="J24" s="32" t="n">
-        <x:f>SUM(J4:J21)</x:f>
-        <x:v>3108</x:v>
-      </x:c>
-      <x:c r="K24" s="30"/>
+    <x:row r="22">
+      <x:c r="A22" s="22" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B22" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C22" s="22" t="str">
+        <x:v>8月27日</x:v>
+      </x:c>
+      <x:c r="D22" s="23" t="n">
+        <x:v>7511</x:v>
+      </x:c>
+      <x:c r="E22" s="23" t="n">
+        <x:v>7696</x:v>
+      </x:c>
+      <x:c r="F22" s="23" t="n">
+        <x:v>7472</x:v>
+      </x:c>
+      <x:c r="G22" s="23" t="n">
+        <x:v>7686.6</x:v>
+      </x:c>
+      <x:c r="H22" s="28" t="n">
+        <x:v>194.8</x:v>
+      </x:c>
+      <x:c r="I22" s="24" t="n">
+        <x:v>0.026001761926372824</x:v>
+      </x:c>
+      <x:c r="J22" s="26" t="n">
+        <x:f>ROUND(E22-F22,1)</x:f>
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="K22" s="22" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B25" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B25" s="30" t="n">
+        <x:v>19</x:v>
+      </x:c>
       <x:c r="C25" s="30"/>
       <x:c r="D25" s="30"/>
       <x:c r="E25" s="30"/>
@@ -6532,11 +6658,29 @@
       <x:c r="G25" s="30"/>
       <x:c r="H25" s="30"/>
       <x:c r="I25" s="30"/>
-      <x:c r="J25" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J21),0),1)</x:f>
-        <x:v>172.7</x:v>
+      <x:c r="J25" s="32" t="n">
+        <x:f>SUM(J4:J22)</x:f>
+        <x:v>3332</x:v>
       </x:c>
       <x:c r="K25" s="30"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B26" s="30"/>
+      <x:c r="C26" s="30"/>
+      <x:c r="D26" s="30"/>
+      <x:c r="E26" s="30"/>
+      <x:c r="F26" s="30"/>
+      <x:c r="G26" s="30"/>
+      <x:c r="H26" s="30"/>
+      <x:c r="I26" s="30"/>
+      <x:c r="J26" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J22),0),1)</x:f>
+        <x:v>175.4</x:v>
+      </x:c>
+      <x:c r="K26" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -7251,31 +7395,49 @@
         <x:v>IC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B24" s="30" t="n">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C24" s="30"/>
-      <x:c r="D24" s="30"/>
-      <x:c r="E24" s="30"/>
-      <x:c r="F24" s="30"/>
-      <x:c r="G24" s="30"/>
-      <x:c r="H24" s="30"/>
-      <x:c r="I24" s="30"/>
-      <x:c r="J24" s="32" t="n">
-        <x:f>SUM(J4:J21)</x:f>
-        <x:v>3055.6</x:v>
-      </x:c>
-      <x:c r="K24" s="30"/>
+    <x:row r="22">
+      <x:c r="A22" s="22" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B22" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C22" s="22" t="str">
+        <x:v>8月27日</x:v>
+      </x:c>
+      <x:c r="D22" s="23" t="n">
+        <x:v>7730.6</x:v>
+      </x:c>
+      <x:c r="E22" s="23" t="n">
+        <x:v>7907</x:v>
+      </x:c>
+      <x:c r="F22" s="23" t="n">
+        <x:v>7700</x:v>
+      </x:c>
+      <x:c r="G22" s="23" t="n">
+        <x:v>7903</x:v>
+      </x:c>
+      <x:c r="H22" s="28" t="n">
+        <x:v>194.2</x:v>
+      </x:c>
+      <x:c r="I22" s="24" t="n">
+        <x:v>0.025191988376919827</x:v>
+      </x:c>
+      <x:c r="J22" s="26" t="n">
+        <x:f>ROUND(E22-F22,1)</x:f>
+        <x:v>207</x:v>
+      </x:c>
+      <x:c r="K22" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B25" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B25" s="30" t="n">
+        <x:v>19</x:v>
+      </x:c>
       <x:c r="C25" s="30"/>
       <x:c r="D25" s="30"/>
       <x:c r="E25" s="30"/>
@@ -7283,11 +7445,29 @@
       <x:c r="G25" s="30"/>
       <x:c r="H25" s="30"/>
       <x:c r="I25" s="30"/>
-      <x:c r="J25" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J21),0),1)</x:f>
-        <x:v>169.8</x:v>
+      <x:c r="J25" s="32" t="n">
+        <x:f>SUM(J4:J22)</x:f>
+        <x:v>3262.6</x:v>
       </x:c>
       <x:c r="K25" s="30"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B26" s="30"/>
+      <x:c r="C26" s="30"/>
+      <x:c r="D26" s="30"/>
+      <x:c r="E26" s="30"/>
+      <x:c r="F26" s="30"/>
+      <x:c r="G26" s="30"/>
+      <x:c r="H26" s="30"/>
+      <x:c r="I26" s="30"/>
+      <x:c r="J26" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J22),0),1)</x:f>
+        <x:v>171.7</x:v>
+      </x:c>
+      <x:c r="K26" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -8002,31 +8182,49 @@
         <x:v>IF2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B24" s="30" t="n">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C24" s="30"/>
-      <x:c r="D24" s="30"/>
-      <x:c r="E24" s="30"/>
-      <x:c r="F24" s="30"/>
-      <x:c r="G24" s="30"/>
-      <x:c r="H24" s="30"/>
-      <x:c r="I24" s="30"/>
-      <x:c r="J24" s="32" t="n">
-        <x:f>SUM(J4:J21)</x:f>
-        <x:v>1169.2</x:v>
-      </x:c>
-      <x:c r="K24" s="30"/>
+    <x:row r="22">
+      <x:c r="A22" s="22" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B22" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C22" s="22" t="str">
+        <x:v>8月27日</x:v>
+      </x:c>
+      <x:c r="D22" s="23" t="n">
+        <x:v>4577.2</x:v>
+      </x:c>
+      <x:c r="E22" s="23" t="n">
+        <x:v>4608.2</x:v>
+      </x:c>
+      <x:c r="F22" s="23" t="n">
+        <x:v>4561.8</x:v>
+      </x:c>
+      <x:c r="G22" s="23" t="n">
+        <x:v>4604.8</x:v>
+      </x:c>
+      <x:c r="H22" s="23" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="I22" s="24" t="n">
+        <x:v>0.008320924936498164</x:v>
+      </x:c>
+      <x:c r="J22" s="23" t="n">
+        <x:f>ROUND(E22-F22,1)</x:f>
+        <x:v>46.4</x:v>
+      </x:c>
+      <x:c r="K22" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B25" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B25" s="30" t="n">
+        <x:v>19</x:v>
+      </x:c>
       <x:c r="C25" s="30"/>
       <x:c r="D25" s="30"/>
       <x:c r="E25" s="30"/>
@@ -8034,11 +8232,29 @@
       <x:c r="G25" s="30"/>
       <x:c r="H25" s="30"/>
       <x:c r="I25" s="30"/>
-      <x:c r="J25" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J21),0),1)</x:f>
-        <x:v>65</x:v>
+      <x:c r="J25" s="32" t="n">
+        <x:f>SUM(J4:J22)</x:f>
+        <x:v>1215.6000000000001</x:v>
       </x:c>
       <x:c r="K25" s="30"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B26" s="30"/>
+      <x:c r="C26" s="30"/>
+      <x:c r="D26" s="30"/>
+      <x:c r="E26" s="30"/>
+      <x:c r="F26" s="30"/>
+      <x:c r="G26" s="30"/>
+      <x:c r="H26" s="30"/>
+      <x:c r="I26" s="30"/>
+      <x:c r="J26" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J22),0),1)</x:f>
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="K26" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -8753,31 +8969,49 @@
         <x:v>IH2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B24" s="30" t="n">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C24" s="30"/>
-      <x:c r="D24" s="30"/>
-      <x:c r="E24" s="30"/>
-      <x:c r="F24" s="30"/>
-      <x:c r="G24" s="30"/>
-      <x:c r="H24" s="30"/>
-      <x:c r="I24" s="30"/>
-      <x:c r="J24" s="32" t="n">
-        <x:f>SUM(J4:J21)</x:f>
-        <x:v>616.2</x:v>
-      </x:c>
-      <x:c r="K24" s="30"/>
+    <x:row r="22">
+      <x:c r="A22" s="22" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B22" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C22" s="22" t="str">
+        <x:v>8月27日</x:v>
+      </x:c>
+      <x:c r="D22" s="23" t="n">
+        <x:v>2895</x:v>
+      </x:c>
+      <x:c r="E22" s="23" t="n">
+        <x:v>2916.2</x:v>
+      </x:c>
+      <x:c r="F22" s="23" t="n">
+        <x:v>2890.4</x:v>
+      </x:c>
+      <x:c r="G22" s="23" t="n">
+        <x:v>2914</x:v>
+      </x:c>
+      <x:c r="H22" s="23" t="n">
+        <x:v>25.2</x:v>
+      </x:c>
+      <x:c r="I22" s="24" t="n">
+        <x:v>0.008723345333702559</x:v>
+      </x:c>
+      <x:c r="J22" s="23" t="n">
+        <x:f>ROUND(E22-F22,1)</x:f>
+        <x:v>25.8</x:v>
+      </x:c>
+      <x:c r="K22" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B25" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B25" s="30" t="n">
+        <x:v>19</x:v>
+      </x:c>
       <x:c r="C25" s="30"/>
       <x:c r="D25" s="30"/>
       <x:c r="E25" s="30"/>
@@ -8785,11 +9019,29 @@
       <x:c r="G25" s="30"/>
       <x:c r="H25" s="30"/>
       <x:c r="I25" s="30"/>
-      <x:c r="J25" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J21),0),1)</x:f>
-        <x:v>34.2</x:v>
+      <x:c r="J25" s="32" t="n">
+        <x:f>SUM(J4:J22)</x:f>
+        <x:v>642</x:v>
       </x:c>
       <x:c r="K25" s="30"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B26" s="30"/>
+      <x:c r="C26" s="30"/>
+      <x:c r="D26" s="30"/>
+      <x:c r="E26" s="30"/>
+      <x:c r="F26" s="30"/>
+      <x:c r="G26" s="30"/>
+      <x:c r="H26" s="30"/>
+      <x:c r="I26" s="30"/>
+      <x:c r="J26" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J22),0),1)</x:f>
+        <x:v>33.8</x:v>
+      </x:c>
+      <x:c r="K26" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-08-28
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Re16f2bda53824bad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R30fb7ffb01fb4fba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Rdf01c1f2ea274b0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rf1da7476a61a4eb7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R40233dd5380b4540"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R1abc07c6812d446f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R85c9b2c209f74bb8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R522c1c2254da4cb2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R99a30a5bf5c34258"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R8614dfc1111d4290"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R5eefbb8af0db4832"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Ra214988800514d64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Rb64f1f4852254cf6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R4cfd520273514074"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R91ea1b9b801c4a1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rec6a2ac136684ca4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R8820b99811b94e28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R6f5ef3ac4417458a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R3586f63882574bb4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R61f7afe4b5d14fec"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -520,25 +520,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-08-27</x:v>
+        <x:v>2026-08-28</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7734.31</x:v>
+        <x:v>7802.55</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7531.78</x:v>
+        <x:v>7702.18</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>202.5</x:v>
+        <x:v>100.4</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>3347.9</x:v>
+        <x:v>3448.3</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>176.2</x:v>
+        <x:v>172.4</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -549,25 +549,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-08-27</x:v>
+        <x:v>2026-08-28</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7951.05</x:v>
+        <x:v>7986.43</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7763.98</x:v>
+        <x:v>7892.51</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>187.1</x:v>
+        <x:v>93.9</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>3204.8</x:v>
+        <x:v>3298.7</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>168.7</x:v>
+        <x:v>164.9</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -578,25 +578,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-08-27</x:v>
+        <x:v>2026-08-28</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3958.03</x:v>
+        <x:v>3970.31</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3909.31</x:v>
+        <x:v>3947.8</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>48.7</x:v>
+        <x:v>22.5</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>823.5</x:v>
+        <x:v>846</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>43.3</x:v>
+        <x:v>42.3</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -694,25 +694,25 @@
         <x:v>IH主力</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>2026-08-27</x:v>
+        <x:v>2026-08-28</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:v>2916.2</x:v>
+        <x:v>2918.2</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
-        <x:v>2890.4</x:v>
+        <x:v>2905.2</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
-        <x:v>25.8</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="F10" s="9" t="n">
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="G10" s="10" t="n">
-        <x:v>642</x:v>
+        <x:v>655</x:v>
       </x:c>
       <x:c r="H10" s="10" t="n">
-        <x:v>33.8</x:v>
+        <x:v>32.8</x:v>
       </x:c>
       <x:c r="I10" s="10" t="n">
         <x:v>60</x:v>
@@ -755,7 +755,7 @@
         <x:v>2026-08-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-08-27</x:v>
+        <x:v>2026-08-28</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1853,37 +1853,37 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B8" s="22" t="str">
-        <x:v>8月24日-8月27日</x:v>
+        <x:v>8月24日-8月28日</x:v>
       </x:c>
       <x:c r="C8" s="23" t="n">
         <x:v>7614.89</x:v>
       </x:c>
       <x:c r="D8" s="23" t="n">
-        <x:v>7734.31</x:v>
+        <x:v>7802.55</x:v>
       </x:c>
       <x:c r="E8" s="23" t="n">
         <x:v>7347.95</x:v>
       </x:c>
       <x:c r="F8" s="23" t="n">
-        <x:v>7732.95</x:v>
+        <x:v>7705.03</x:v>
       </x:c>
       <x:c r="G8" s="23" t="n">
         <x:f>ROUND(F8-F7,1)</x:f>
-        <x:v>131.1</x:v>
+        <x:v>103.2</x:v>
       </x:c>
       <x:c r="H8" s="24" t="n">
         <x:f>IFERROR(F8/F7-1,"")</x:f>
-        <x:v>0.017252492830645227</x:v>
+        <x:v>0.013579678497197989</x:v>
       </x:c>
       <x:c r="I8" s="26" t="n">
         <x:f>ROUND(D8-E8,1)</x:f>
-        <x:v>386.4</x:v>
+        <x:v>454.6</x:v>
       </x:c>
       <x:c r="J8" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K8" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1901,7 +1901,7 @@
       <x:c r="H9" s="30"/>
       <x:c r="I9" s="32" t="n">
         <x:f>ROUND(SUM(I5:I8),1)</x:f>
-        <x:v>1810.7</x:v>
+        <x:v>1878.9</x:v>
       </x:c>
       <x:c r="J9" s="30"/>
       <x:c r="K9" s="30"/>
@@ -1919,7 +1919,7 @@
       <x:c r="H10" s="30"/>
       <x:c r="I10" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I8),0),1)</x:f>
-        <x:v>452.7</x:v>
+        <x:v>469.7</x:v>
       </x:c>
       <x:c r="J10" s="30"/>
       <x:c r="K10" s="30"/>
@@ -2087,37 +2087,37 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B17" s="22" t="str">
-        <x:v>8月24日-8月27日</x:v>
+        <x:v>8月24日-8月28日</x:v>
       </x:c>
       <x:c r="C17" s="23" t="n">
         <x:v>7861.05</x:v>
       </x:c>
       <x:c r="D17" s="23" t="n">
-        <x:v>7951.05</x:v>
+        <x:v>7986.43</x:v>
       </x:c>
       <x:c r="E17" s="23" t="n">
         <x:v>7572.86</x:v>
       </x:c>
       <x:c r="F17" s="23" t="n">
-        <x:v>7946.33</x:v>
+        <x:v>7895.45</x:v>
       </x:c>
       <x:c r="G17" s="23" t="n">
         <x:f>ROUND(F17-F16,1)</x:f>
-        <x:v>92</x:v>
+        <x:v>41.1</x:v>
       </x:c>
       <x:c r="H17" s="24" t="n">
         <x:f>IFERROR(F17/F16-1,"")</x:f>
-        <x:v>0.011713284264857737</x:v>
+        <x:v>0.005235328793162575</x:v>
       </x:c>
       <x:c r="I17" s="26" t="n">
         <x:f>ROUND(D17-E17,1)</x:f>
-        <x:v>378.2</x:v>
+        <x:v>413.6</x:v>
       </x:c>
       <x:c r="J17" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K17" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -2135,7 +2135,7 @@
       <x:c r="H18" s="30"/>
       <x:c r="I18" s="32" t="n">
         <x:f>ROUND(SUM(I14:I17),1)</x:f>
-        <x:v>1663.5</x:v>
+        <x:v>1698.9</x:v>
       </x:c>
       <x:c r="J18" s="30"/>
       <x:c r="K18" s="30"/>
@@ -2153,7 +2153,7 @@
       <x:c r="H19" s="30"/>
       <x:c r="I19" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I14:I17),0),1)</x:f>
-        <x:v>415.9</x:v>
+        <x:v>424.7</x:v>
       </x:c>
       <x:c r="J19" s="30"/>
       <x:c r="K19" s="30"/>
@@ -2321,37 +2321,37 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B26" s="22" t="str">
-        <x:v>8月24日-8月27日</x:v>
+        <x:v>8月24日-8月28日</x:v>
       </x:c>
       <x:c r="C26" s="23" t="n">
         <x:v>3902.7</x:v>
       </x:c>
       <x:c r="D26" s="23" t="n">
-        <x:v>3958.03</x:v>
+        <x:v>3970.31</x:v>
       </x:c>
       <x:c r="E26" s="23" t="n">
         <x:v>3850.86</x:v>
       </x:c>
       <x:c r="F26" s="23" t="n">
-        <x:v>3956.57</x:v>
+        <x:v>3952.18</x:v>
       </x:c>
       <x:c r="G26" s="23" t="n">
         <x:f>ROUND(F26-F25,1)</x:f>
-        <x:v>51.4</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="H26" s="24" t="n">
         <x:f>IFERROR(F26/F25-1,"")</x:f>
-        <x:v>0.013154255863976339</x:v>
+        <x:v>0.012030113694561084</x:v>
       </x:c>
       <x:c r="I26" s="26" t="n">
         <x:f>ROUND(D26-E26,1)</x:f>
-        <x:v>107.2</x:v>
+        <x:v>119.4</x:v>
       </x:c>
       <x:c r="J26" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K26" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -2369,7 +2369,7 @@
       <x:c r="H27" s="30"/>
       <x:c r="I27" s="32" t="n">
         <x:f>ROUND(SUM(I23:I26),1)</x:f>
-        <x:v>429.9</x:v>
+        <x:v>442.1</x:v>
       </x:c>
       <x:c r="J27" s="30"/>
       <x:c r="K27" s="30"/>
@@ -2387,7 +2387,7 @@
       <x:c r="H28" s="30"/>
       <x:c r="I28" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I23:I26),0),1)</x:f>
-        <x:v>107.5</x:v>
+        <x:v>110.5</x:v>
       </x:c>
       <x:c r="J28" s="30"/>
       <x:c r="K28" s="30"/>
@@ -3257,37 +3257,37 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B62" s="22" t="str">
-        <x:v>8月24日-8月27日</x:v>
+        <x:v>8月24日-8月28日</x:v>
       </x:c>
       <x:c r="C62" s="23" t="n">
         <x:v>2856.4</x:v>
       </x:c>
       <x:c r="D62" s="23" t="n">
-        <x:v>2916.2</x:v>
+        <x:v>2918.2</x:v>
       </x:c>
       <x:c r="E62" s="23" t="n">
         <x:v>2837.4</x:v>
       </x:c>
       <x:c r="F62" s="23" t="n">
-        <x:v>2914</x:v>
+        <x:v>2911.4</x:v>
       </x:c>
       <x:c r="G62" s="23" t="n">
         <x:f>ROUND(F62-F61,1)</x:f>
-        <x:v>53</x:v>
+        <x:v>50.4</x:v>
       </x:c>
       <x:c r="H62" s="24" t="n">
         <x:f>IFERROR(F62/F61-1,"")</x:f>
-        <x:v>0.01852499126179663</x:v>
+        <x:v>0.01761621810555747</x:v>
       </x:c>
       <x:c r="I62" s="26" t="n">
         <x:f>ROUND(D62-E62,1)</x:f>
-        <x:v>78.8</x:v>
+        <x:v>80.8</x:v>
       </x:c>
       <x:c r="J62" s="22" t="str">
         <x:v>IH2609</x:v>
       </x:c>
       <x:c r="K62" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
@@ -3305,7 +3305,7 @@
       <x:c r="H63" s="30"/>
       <x:c r="I63" s="32" t="n">
         <x:f>ROUND(SUM(I59:I62),1)</x:f>
-        <x:v>314.4</x:v>
+        <x:v>316.4</x:v>
       </x:c>
       <x:c r="J63" s="30"/>
       <x:c r="K63" s="30"/>
@@ -3323,7 +3323,7 @@
       <x:c r="H64" s="30"/>
       <x:c r="I64" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I59:I62),0),1)</x:f>
-        <x:v>78.6</x:v>
+        <x:v>79.1</x:v>
       </x:c>
       <x:c r="J64" s="30"/>
       <x:c r="K64" s="30"/>
@@ -4319,31 +4319,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B25" s="30" t="n">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="C25" s="30"/>
-      <x:c r="D25" s="30"/>
-      <x:c r="E25" s="30"/>
-      <x:c r="F25" s="30"/>
-      <x:c r="G25" s="30"/>
-      <x:c r="H25" s="30"/>
-      <x:c r="I25" s="30"/>
-      <x:c r="J25" s="32" t="n">
-        <x:f>SUM(J4:J22)</x:f>
-        <x:v>3347.9</x:v>
-      </x:c>
-      <x:c r="K25" s="30"/>
+    <x:row r="23">
+      <x:c r="A23" s="22" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B23" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C23" s="22" t="str">
+        <x:v>8月28日</x:v>
+      </x:c>
+      <x:c r="D23" s="23" t="n">
+        <x:v>7734.19</x:v>
+      </x:c>
+      <x:c r="E23" s="23" t="n">
+        <x:v>7802.55</x:v>
+      </x:c>
+      <x:c r="F23" s="23" t="n">
+        <x:v>7702.18</x:v>
+      </x:c>
+      <x:c r="G23" s="23" t="n">
+        <x:v>7705.03</x:v>
+      </x:c>
+      <x:c r="H23" s="23" t="n">
+        <x:v>-27.9</x:v>
+      </x:c>
+      <x:c r="I23" s="24" t="n">
+        <x:v>-0.0036105237975158078</x:v>
+      </x:c>
+      <x:c r="J23" s="23" t="n">
+        <x:f>ROUND(E23-F23,1)</x:f>
+        <x:v>100.4</x:v>
+      </x:c>
+      <x:c r="K23" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B26" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B26" s="30" t="n">
+        <x:v>20</x:v>
+      </x:c>
       <x:c r="C26" s="30"/>
       <x:c r="D26" s="30"/>
       <x:c r="E26" s="30"/>
@@ -4351,11 +4369,29 @@
       <x:c r="G26" s="30"/>
       <x:c r="H26" s="30"/>
       <x:c r="I26" s="30"/>
-      <x:c r="J26" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J22),0),1)</x:f>
-        <x:v>176.2</x:v>
+      <x:c r="J26" s="32" t="n">
+        <x:f>SUM(J4:J23)</x:f>
+        <x:v>3448.3</x:v>
       </x:c>
       <x:c r="K26" s="30"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B27" s="30"/>
+      <x:c r="C27" s="30"/>
+      <x:c r="D27" s="30"/>
+      <x:c r="E27" s="30"/>
+      <x:c r="F27" s="30"/>
+      <x:c r="G27" s="30"/>
+      <x:c r="H27" s="30"/>
+      <x:c r="I27" s="30"/>
+      <x:c r="J27" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J23),0),1)</x:f>
+        <x:v>172.4</x:v>
+      </x:c>
+      <x:c r="K27" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5106,31 +5142,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B25" s="30" t="n">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="C25" s="30"/>
-      <x:c r="D25" s="30"/>
-      <x:c r="E25" s="30"/>
-      <x:c r="F25" s="30"/>
-      <x:c r="G25" s="30"/>
-      <x:c r="H25" s="30"/>
-      <x:c r="I25" s="30"/>
-      <x:c r="J25" s="32" t="n">
-        <x:f>SUM(J4:J22)</x:f>
-        <x:v>3204.7999999999997</x:v>
-      </x:c>
-      <x:c r="K25" s="30"/>
+    <x:row r="23">
+      <x:c r="A23" s="22" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B23" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C23" s="22" t="str">
+        <x:v>8月28日</x:v>
+      </x:c>
+      <x:c r="D23" s="23" t="n">
+        <x:v>7939.45</x:v>
+      </x:c>
+      <x:c r="E23" s="23" t="n">
+        <x:v>7986.43</x:v>
+      </x:c>
+      <x:c r="F23" s="23" t="n">
+        <x:v>7892.51</x:v>
+      </x:c>
+      <x:c r="G23" s="23" t="n">
+        <x:v>7895.45</x:v>
+      </x:c>
+      <x:c r="H23" s="23" t="n">
+        <x:v>-50.9</x:v>
+      </x:c>
+      <x:c r="I23" s="24" t="n">
+        <x:v>-0.006402955829924006</x:v>
+      </x:c>
+      <x:c r="J23" s="23" t="n">
+        <x:f>ROUND(E23-F23,1)</x:f>
+        <x:v>93.9</x:v>
+      </x:c>
+      <x:c r="K23" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B26" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B26" s="30" t="n">
+        <x:v>20</x:v>
+      </x:c>
       <x:c r="C26" s="30"/>
       <x:c r="D26" s="30"/>
       <x:c r="E26" s="30"/>
@@ -5138,11 +5192,29 @@
       <x:c r="G26" s="30"/>
       <x:c r="H26" s="30"/>
       <x:c r="I26" s="30"/>
-      <x:c r="J26" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J22),0),1)</x:f>
-        <x:v>168.7</x:v>
+      <x:c r="J26" s="32" t="n">
+        <x:f>SUM(J4:J23)</x:f>
+        <x:v>3298.7</x:v>
       </x:c>
       <x:c r="K26" s="30"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B27" s="30"/>
+      <x:c r="C27" s="30"/>
+      <x:c r="D27" s="30"/>
+      <x:c r="E27" s="30"/>
+      <x:c r="F27" s="30"/>
+      <x:c r="G27" s="30"/>
+      <x:c r="H27" s="30"/>
+      <x:c r="I27" s="30"/>
+      <x:c r="J27" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J23),0),1)</x:f>
+        <x:v>164.9</x:v>
+      </x:c>
+      <x:c r="K27" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5893,31 +5965,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B25" s="30" t="n">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="C25" s="30"/>
-      <x:c r="D25" s="30"/>
-      <x:c r="E25" s="30"/>
-      <x:c r="F25" s="30"/>
-      <x:c r="G25" s="30"/>
-      <x:c r="H25" s="30"/>
-      <x:c r="I25" s="30"/>
-      <x:c r="J25" s="32" t="n">
-        <x:f>SUM(J4:J22)</x:f>
-        <x:v>823.5</x:v>
-      </x:c>
-      <x:c r="K25" s="30"/>
+    <x:row r="23">
+      <x:c r="A23" s="22" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B23" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C23" s="22" t="str">
+        <x:v>8月28日</x:v>
+      </x:c>
+      <x:c r="D23" s="23" t="n">
+        <x:v>3950.24</x:v>
+      </x:c>
+      <x:c r="E23" s="23" t="n">
+        <x:v>3970.31</x:v>
+      </x:c>
+      <x:c r="F23" s="23" t="n">
+        <x:v>3947.8</x:v>
+      </x:c>
+      <x:c r="G23" s="23" t="n">
+        <x:v>3952.18</x:v>
+      </x:c>
+      <x:c r="H23" s="23" t="n">
+        <x:v>-4.4</x:v>
+      </x:c>
+      <x:c r="I23" s="24" t="n">
+        <x:v>-0.0011095469055268925</x:v>
+      </x:c>
+      <x:c r="J23" s="23" t="n">
+        <x:f>ROUND(E23-F23,1)</x:f>
+        <x:v>22.5</x:v>
+      </x:c>
+      <x:c r="K23" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B26" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B26" s="30" t="n">
+        <x:v>20</x:v>
+      </x:c>
       <x:c r="C26" s="30"/>
       <x:c r="D26" s="30"/>
       <x:c r="E26" s="30"/>
@@ -5925,11 +6015,29 @@
       <x:c r="G26" s="30"/>
       <x:c r="H26" s="30"/>
       <x:c r="I26" s="30"/>
-      <x:c r="J26" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J22),0),1)</x:f>
-        <x:v>43.3</x:v>
+      <x:c r="J26" s="32" t="n">
+        <x:f>SUM(J4:J23)</x:f>
+        <x:v>846</x:v>
       </x:c>
       <x:c r="K26" s="30"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B27" s="30"/>
+      <x:c r="C27" s="30"/>
+      <x:c r="D27" s="30"/>
+      <x:c r="E27" s="30"/>
+      <x:c r="F27" s="30"/>
+      <x:c r="G27" s="30"/>
+      <x:c r="H27" s="30"/>
+      <x:c r="I27" s="30"/>
+      <x:c r="J27" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J23),0),1)</x:f>
+        <x:v>42.3</x:v>
+      </x:c>
+      <x:c r="K27" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -9041,31 +9149,49 @@
         <x:v>IH2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B25" s="30" t="n">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="C25" s="30"/>
-      <x:c r="D25" s="30"/>
-      <x:c r="E25" s="30"/>
-      <x:c r="F25" s="30"/>
-      <x:c r="G25" s="30"/>
-      <x:c r="H25" s="30"/>
-      <x:c r="I25" s="30"/>
-      <x:c r="J25" s="32" t="n">
-        <x:f>SUM(J4:J22)</x:f>
-        <x:v>642</x:v>
-      </x:c>
-      <x:c r="K25" s="30"/>
+    <x:row r="23">
+      <x:c r="A23" s="22" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B23" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C23" s="22" t="str">
+        <x:v>8月28日</x:v>
+      </x:c>
+      <x:c r="D23" s="23" t="n">
+        <x:v>2909</x:v>
+      </x:c>
+      <x:c r="E23" s="23" t="n">
+        <x:v>2918.2</x:v>
+      </x:c>
+      <x:c r="F23" s="23" t="n">
+        <x:v>2905.2</x:v>
+      </x:c>
+      <x:c r="G23" s="23" t="n">
+        <x:v>2911.4</x:v>
+      </x:c>
+      <x:c r="H23" s="23" t="n">
+        <x:v>-2.6</x:v>
+      </x:c>
+      <x:c r="I23" s="24" t="n">
+        <x:v>-0.0008922443376800926</x:v>
+      </x:c>
+      <x:c r="J23" s="23" t="n">
+        <x:f>ROUND(E23-F23,1)</x:f>
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="K23" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B26" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B26" s="30" t="n">
+        <x:v>20</x:v>
+      </x:c>
       <x:c r="C26" s="30"/>
       <x:c r="D26" s="30"/>
       <x:c r="E26" s="30"/>
@@ -9073,11 +9199,29 @@
       <x:c r="G26" s="30"/>
       <x:c r="H26" s="30"/>
       <x:c r="I26" s="30"/>
-      <x:c r="J26" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J22),0),1)</x:f>
-        <x:v>33.8</x:v>
+      <x:c r="J26" s="32" t="n">
+        <x:f>SUM(J4:J23)</x:f>
+        <x:v>655</x:v>
       </x:c>
       <x:c r="K26" s="30"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B27" s="30"/>
+      <x:c r="C27" s="30"/>
+      <x:c r="D27" s="30"/>
+      <x:c r="E27" s="30"/>
+      <x:c r="F27" s="30"/>
+      <x:c r="G27" s="30"/>
+      <x:c r="H27" s="30"/>
+      <x:c r="I27" s="30"/>
+      <x:c r="J27" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J23),0),1)</x:f>
+        <x:v>32.8</x:v>
+      </x:c>
+      <x:c r="K27" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-08-31
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R7c0e6143f5944460"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Rccfb8d8a8a314ea8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R9968d3768a224516"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rcbbf8a5a4a064d66"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R7a7533a6326a41e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R51faefcba87a4534"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Rd09af5f598ee410d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R24dc1220db984c0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R8a7f71541c3243f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="Rc77f4c167729473d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rdb9c22eb5c03432f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R062a1809195946fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R8e5db369f40448c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R985e1fb240724ab0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R6b79f082cddf43ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R719883118ce74723"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Ra3ce8d9a021a4749"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Re39118ad37c0432e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rd3899b201a0b4b49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R95edff9b06ce4194"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -520,25 +520,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-08-28</x:v>
+        <x:v>2026-08-31</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7802.55</x:v>
+        <x:v>7771.55</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7702.18</x:v>
+        <x:v>7604.95</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>100.4</x:v>
+        <x:v>166.6</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>3448.3</x:v>
+        <x:v>3614.9</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>172.4</x:v>
+        <x:v>172.1</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -549,25 +549,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-08-28</x:v>
+        <x:v>2026-08-31</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7986.43</x:v>
+        <x:v>7953.93</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7892.51</x:v>
+        <x:v>7764.98</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>93.9</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>3298.7</x:v>
+        <x:v>3487.7</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>164.9</x:v>
+        <x:v>166.1</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -578,25 +578,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-08-28</x:v>
+        <x:v>2026-08-31</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3970.31</x:v>
+        <x:v>3986.3</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3947.8</x:v>
+        <x:v>3926.5</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>22.5</x:v>
+        <x:v>59.8</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>846</x:v>
+        <x:v>905.8</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>42.3</x:v>
+        <x:v>43.1</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -665,25 +665,25 @@
         <x:v>IF主力</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>2026-08-28</x:v>
+        <x:v>2026-08-31</x:v>
       </x:c>
       <x:c r="C9" s="10" t="n">
-        <x:v>4620</x:v>
+        <x:v>4608.6</x:v>
       </x:c>
       <x:c r="D9" s="10" t="n">
-        <x:v>4587.2</x:v>
+        <x:v>4530</x:v>
       </x:c>
       <x:c r="E9" s="12" t="n">
-        <x:v>32.8</x:v>
+        <x:v>78.6</x:v>
       </x:c>
       <x:c r="F9" s="9" t="n">
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="G9" s="10" t="n">
-        <x:v>1248.4</x:v>
+        <x:v>1327</x:v>
       </x:c>
       <x:c r="H9" s="10" t="n">
-        <x:v>62.4</x:v>
+        <x:v>63.2</x:v>
       </x:c>
       <x:c r="I9" s="10" t="n">
         <x:v>90</x:v>
@@ -755,7 +755,7 @@
         <x:v>2026-08-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-08-28</x:v>
+        <x:v>2026-08-31</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1923,155 +1923,155 @@
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B9" s="30" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C9" s="30"/>
-      <x:c r="D9" s="30"/>
-      <x:c r="E9" s="30"/>
-      <x:c r="F9" s="30"/>
-      <x:c r="G9" s="30"/>
-      <x:c r="H9" s="30"/>
-      <x:c r="I9" s="32" t="n">
-        <x:f>ROUND(SUM(I5:I8),1)</x:f>
-        <x:v>1878.9</x:v>
-      </x:c>
-      <x:c r="J9" s="30"/>
-      <x:c r="K9" s="30"/>
+      <x:c r="A9" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B9" s="22" t="str">
+        <x:v>8月31日</x:v>
+      </x:c>
+      <x:c r="C9" s="23" t="n">
+        <x:v>7607.23</x:v>
+      </x:c>
+      <x:c r="D9" s="23" t="n">
+        <x:v>7771.55</x:v>
+      </x:c>
+      <x:c r="E9" s="23" t="n">
+        <x:v>7604.95</x:v>
+      </x:c>
+      <x:c r="F9" s="23" t="n">
+        <x:v>7770.42</x:v>
+      </x:c>
+      <x:c r="G9" s="23" t="n">
+        <x:f>ROUND(F9-F8,1)</x:f>
+        <x:v>65.4</x:v>
+      </x:c>
+      <x:c r="H9" s="24" t="n">
+        <x:f>IFERROR(F9/F8-1,"")</x:f>
+        <x:v>0.00848666390656505</x:v>
+      </x:c>
+      <x:c r="I9" s="23" t="n">
+        <x:f>ROUND(D9-E9,1)</x:f>
+        <x:v>166.6</x:v>
+      </x:c>
+      <x:c r="J9" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
+      <x:c r="K9" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B10" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B10" s="30" t="n">
+        <x:v>5</x:v>
+      </x:c>
       <x:c r="C10" s="30"/>
       <x:c r="D10" s="30"/>
       <x:c r="E10" s="30"/>
       <x:c r="F10" s="30"/>
       <x:c r="G10" s="30"/>
       <x:c r="H10" s="30"/>
-      <x:c r="I10" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I5:I8),0),1)</x:f>
-        <x:v>469.7</x:v>
+      <x:c r="I10" s="32" t="n">
+        <x:f>ROUND(SUM(I5:I9),1)</x:f>
+        <x:v>2045.5</x:v>
       </x:c>
       <x:c r="J10" s="30"/>
       <x:c r="K10" s="30"/>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="17" t="str">
+    <x:row r="11">
+      <x:c r="A11" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B11" s="30"/>
+      <x:c r="C11" s="30"/>
+      <x:c r="D11" s="30"/>
+      <x:c r="E11" s="30"/>
+      <x:c r="F11" s="30"/>
+      <x:c r="G11" s="30"/>
+      <x:c r="H11" s="30"/>
+      <x:c r="I11" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I5:I9),0),1)</x:f>
+        <x:v>409.1</x:v>
+      </x:c>
+      <x:c r="J11" s="30"/>
+      <x:c r="K11" s="30"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="17" t="str">
         <x:v>中证500</x:v>
       </x:c>
-      <x:c r="B12" s="17"/>
-      <x:c r="C12" s="17"/>
-      <x:c r="D12" s="17"/>
-      <x:c r="E12" s="17"/>
-      <x:c r="F12" s="17"/>
-      <x:c r="G12" s="17"/>
-      <x:c r="H12" s="17"/>
-      <x:c r="I12" s="17"/>
-      <x:c r="J12" s="17"/>
-      <x:c r="K12" s="17"/>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="20" t="str">
+      <x:c r="B13" s="17"/>
+      <x:c r="C13" s="17"/>
+      <x:c r="D13" s="17"/>
+      <x:c r="E13" s="17"/>
+      <x:c r="F13" s="17"/>
+      <x:c r="G13" s="17"/>
+      <x:c r="H13" s="17"/>
+      <x:c r="I13" s="17"/>
+      <x:c r="J13" s="17"/>
+      <x:c r="K13" s="17"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B13" s="20" t="str">
+      <x:c r="B14" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C13" s="20" t="str">
+      <x:c r="C14" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D13" s="20" t="str">
+      <x:c r="D14" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E13" s="20" t="str">
+      <x:c r="E14" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F13" s="20" t="str">
+      <x:c r="F14" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G13" s="20" t="str">
+      <x:c r="G14" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H13" s="20" t="str">
+      <x:c r="H14" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I13" s="20" t="str">
+      <x:c r="I14" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J13" s="20" t="str">
+      <x:c r="J14" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K13" s="20" t="str">
+      <x:c r="K14" s="20" t="str">
         <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B14" s="22" t="str">
-        <x:v>8月3日-8月7日</x:v>
-      </x:c>
-      <x:c r="C14" s="23" t="n">
-        <x:v>7457.12</x:v>
-      </x:c>
-      <x:c r="D14" s="23" t="n">
-        <x:v>7983.17</x:v>
-      </x:c>
-      <x:c r="E14" s="23" t="n">
-        <x:v>7397.94</x:v>
-      </x:c>
-      <x:c r="F14" s="23" t="n">
-        <x:v>7980.12</x:v>
-      </x:c>
-      <x:c r="G14" s="23"/>
-      <x:c r="H14" s="24"/>
-      <x:c r="I14" s="26" t="n">
-        <x:f>ROUND(D14-E14,1)</x:f>
-        <x:v>585.2</x:v>
-      </x:c>
-      <x:c r="J14" s="22" t="str">
-        <x:v>中证500</x:v>
-      </x:c>
-      <x:c r="K14" s="22" t="n">
-        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="B15" s="22" t="str">
-        <x:v>8月10日-8月14日</x:v>
+        <x:v>8月3日-8月7日</x:v>
       </x:c>
       <x:c r="C15" s="23" t="n">
-        <x:v>8003.92</x:v>
+        <x:v>7457.12</x:v>
       </x:c>
       <x:c r="D15" s="23" t="n">
-        <x:v>8142.33</x:v>
+        <x:v>7983.17</x:v>
       </x:c>
       <x:c r="E15" s="23" t="n">
-        <x:v>7897.24</x:v>
+        <x:v>7397.94</x:v>
       </x:c>
       <x:c r="F15" s="23" t="n">
-        <x:v>7990.33</x:v>
-      </x:c>
-      <x:c r="G15" s="23" t="n">
-        <x:f>ROUND(F15-F14,1)</x:f>
-        <x:v>10.2</x:v>
-      </x:c>
-      <x:c r="H15" s="24" t="n">
-        <x:f>IFERROR(F15/F14-1,"")</x:f>
-        <x:v>0.0012794293820144187</x:v>
-      </x:c>
+        <x:v>7980.12</x:v>
+      </x:c>
+      <x:c r="G15" s="23"/>
+      <x:c r="H15" s="24"/>
       <x:c r="I15" s="26" t="n">
         <x:f>ROUND(D15-E15,1)</x:f>
-        <x:v>245.1</x:v>
+        <x:v>585.2</x:v>
       </x:c>
       <x:c r="J15" s="22" t="str">
         <x:v>中证500</x:v>
@@ -2082,34 +2082,34 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="B16" s="22" t="str">
-        <x:v>8月17日-8月21日</x:v>
+        <x:v>8月10日-8月14日</x:v>
       </x:c>
       <x:c r="C16" s="23" t="n">
-        <x:v>8007.87</x:v>
+        <x:v>8003.92</x:v>
       </x:c>
       <x:c r="D16" s="23" t="n">
-        <x:v>8211.31</x:v>
+        <x:v>8142.33</x:v>
       </x:c>
       <x:c r="E16" s="23" t="n">
-        <x:v>7756.28</x:v>
+        <x:v>7897.24</x:v>
       </x:c>
       <x:c r="F16" s="23" t="n">
-        <x:v>7854.33</x:v>
+        <x:v>7990.33</x:v>
       </x:c>
       <x:c r="G16" s="23" t="n">
         <x:f>ROUND(F16-F15,1)</x:f>
-        <x:v>-136</x:v>
+        <x:v>10.2</x:v>
       </x:c>
       <x:c r="H16" s="24" t="n">
         <x:f>IFERROR(F16/F15-1,"")</x:f>
-        <x:v>-0.01702057361836118</x:v>
+        <x:v>0.0012794293820144187</x:v>
       </x:c>
       <x:c r="I16" s="26" t="n">
         <x:f>ROUND(D16-E16,1)</x:f>
-        <x:v>455</x:v>
+        <x:v>245.1</x:v>
       </x:c>
       <x:c r="J16" s="22" t="str">
         <x:v>中证500</x:v>
@@ -2120,34 +2120,34 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="B17" s="22" t="str">
-        <x:v>8月24日-8月28日</x:v>
+        <x:v>8月17日-8月21日</x:v>
       </x:c>
       <x:c r="C17" s="23" t="n">
-        <x:v>7861.05</x:v>
+        <x:v>8007.87</x:v>
       </x:c>
       <x:c r="D17" s="23" t="n">
-        <x:v>7986.43</x:v>
+        <x:v>8211.31</x:v>
       </x:c>
       <x:c r="E17" s="23" t="n">
-        <x:v>7572.86</x:v>
+        <x:v>7756.28</x:v>
       </x:c>
       <x:c r="F17" s="23" t="n">
-        <x:v>7895.45</x:v>
+        <x:v>7854.33</x:v>
       </x:c>
       <x:c r="G17" s="23" t="n">
         <x:f>ROUND(F17-F16,1)</x:f>
-        <x:v>41.1</x:v>
+        <x:v>-136</x:v>
       </x:c>
       <x:c r="H17" s="24" t="n">
         <x:f>IFERROR(F17/F16-1,"")</x:f>
-        <x:v>0.005235328793162575</x:v>
+        <x:v>-0.01702057361836118</x:v>
       </x:c>
       <x:c r="I17" s="26" t="n">
         <x:f>ROUND(D17-E17,1)</x:f>
-        <x:v>413.6</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="J17" s="22" t="str">
         <x:v>中证500</x:v>
@@ -2157,193 +2157,193 @@
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="31" t="str">
+      <x:c r="A18" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B18" s="22" t="str">
+        <x:v>8月24日-8月28日</x:v>
+      </x:c>
+      <x:c r="C18" s="23" t="n">
+        <x:v>7861.05</x:v>
+      </x:c>
+      <x:c r="D18" s="23" t="n">
+        <x:v>7986.43</x:v>
+      </x:c>
+      <x:c r="E18" s="23" t="n">
+        <x:v>7572.86</x:v>
+      </x:c>
+      <x:c r="F18" s="23" t="n">
+        <x:v>7895.45</x:v>
+      </x:c>
+      <x:c r="G18" s="23" t="n">
+        <x:f>ROUND(F18-F17,1)</x:f>
+        <x:v>41.1</x:v>
+      </x:c>
+      <x:c r="H18" s="24" t="n">
+        <x:f>IFERROR(F18/F17-1,"")</x:f>
+        <x:v>0.005235328793162575</x:v>
+      </x:c>
+      <x:c r="I18" s="26" t="n">
+        <x:f>ROUND(D18-E18,1)</x:f>
+        <x:v>413.6</x:v>
+      </x:c>
+      <x:c r="J18" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+      <x:c r="K18" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B19" s="22" t="str">
+        <x:v>8月31日</x:v>
+      </x:c>
+      <x:c r="C19" s="23" t="n">
+        <x:v>7797.23</x:v>
+      </x:c>
+      <x:c r="D19" s="23" t="n">
+        <x:v>7953.93</x:v>
+      </x:c>
+      <x:c r="E19" s="23" t="n">
+        <x:v>7764.98</x:v>
+      </x:c>
+      <x:c r="F19" s="23" t="n">
+        <x:v>7952.1</x:v>
+      </x:c>
+      <x:c r="G19" s="23" t="n">
+        <x:f>ROUND(F19-F18,1)</x:f>
+        <x:v>56.7</x:v>
+      </x:c>
+      <x:c r="H19" s="24" t="n">
+        <x:f>IFERROR(F19/F18-1,"")</x:f>
+        <x:v>0.007175018523326804</x:v>
+      </x:c>
+      <x:c r="I19" s="26" t="n">
+        <x:f>ROUND(D19-E19,1)</x:f>
+        <x:v>189</x:v>
+      </x:c>
+      <x:c r="J19" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+      <x:c r="K19" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B18" s="30" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C18" s="30"/>
-      <x:c r="D18" s="30"/>
-      <x:c r="E18" s="30"/>
-      <x:c r="F18" s="30"/>
-      <x:c r="G18" s="30"/>
-      <x:c r="H18" s="30"/>
-      <x:c r="I18" s="32" t="n">
-        <x:f>ROUND(SUM(I14:I17),1)</x:f>
-        <x:v>1698.9</x:v>
-      </x:c>
-      <x:c r="J18" s="30"/>
-      <x:c r="K18" s="30"/>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="31" t="str">
+      <x:c r="B20" s="30" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C20" s="30"/>
+      <x:c r="D20" s="30"/>
+      <x:c r="E20" s="30"/>
+      <x:c r="F20" s="30"/>
+      <x:c r="G20" s="30"/>
+      <x:c r="H20" s="30"/>
+      <x:c r="I20" s="32" t="n">
+        <x:f>ROUND(SUM(I15:I19),1)</x:f>
+        <x:v>1887.9</x:v>
+      </x:c>
+      <x:c r="J20" s="30"/>
+      <x:c r="K20" s="30"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B19" s="30"/>
-      <x:c r="C19" s="30"/>
-      <x:c r="D19" s="30"/>
-      <x:c r="E19" s="30"/>
-      <x:c r="F19" s="30"/>
-      <x:c r="G19" s="30"/>
-      <x:c r="H19" s="30"/>
-      <x:c r="I19" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I14:I17),0),1)</x:f>
-        <x:v>424.7</x:v>
-      </x:c>
-      <x:c r="J19" s="30"/>
-      <x:c r="K19" s="30"/>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="17" t="str">
+      <x:c r="B21" s="30"/>
+      <x:c r="C21" s="30"/>
+      <x:c r="D21" s="30"/>
+      <x:c r="E21" s="30"/>
+      <x:c r="F21" s="30"/>
+      <x:c r="G21" s="30"/>
+      <x:c r="H21" s="30"/>
+      <x:c r="I21" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I15:I19),0),1)</x:f>
+        <x:v>377.6</x:v>
+      </x:c>
+      <x:c r="J21" s="30"/>
+      <x:c r="K21" s="30"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="17" t="str">
         <x:v>上证指数</x:v>
       </x:c>
-      <x:c r="B21" s="17"/>
-      <x:c r="C21" s="17"/>
-      <x:c r="D21" s="17"/>
-      <x:c r="E21" s="17"/>
-      <x:c r="F21" s="17"/>
-      <x:c r="G21" s="17"/>
-      <x:c r="H21" s="17"/>
-      <x:c r="I21" s="17"/>
-      <x:c r="J21" s="17"/>
-      <x:c r="K21" s="17"/>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="20" t="str">
+      <x:c r="B23" s="17"/>
+      <x:c r="C23" s="17"/>
+      <x:c r="D23" s="17"/>
+      <x:c r="E23" s="17"/>
+      <x:c r="F23" s="17"/>
+      <x:c r="G23" s="17"/>
+      <x:c r="H23" s="17"/>
+      <x:c r="I23" s="17"/>
+      <x:c r="J23" s="17"/>
+      <x:c r="K23" s="17"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B22" s="20" t="str">
+      <x:c r="B24" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C22" s="20" t="str">
+      <x:c r="C24" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D22" s="20" t="str">
+      <x:c r="D24" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E22" s="20" t="str">
+      <x:c r="E24" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F22" s="20" t="str">
+      <x:c r="F24" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G22" s="20" t="str">
+      <x:c r="G24" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H22" s="20" t="str">
+      <x:c r="H24" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I22" s="20" t="str">
+      <x:c r="I24" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J22" s="20" t="str">
+      <x:c r="J24" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K22" s="20" t="str">
+      <x:c r="K24" s="20" t="str">
         <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B23" s="22" t="str">
-        <x:v>8月3日-8月7日</x:v>
-      </x:c>
-      <x:c r="C23" s="23" t="n">
-        <x:v>3812.61</x:v>
-      </x:c>
-      <x:c r="D23" s="23" t="n">
-        <x:v>3940.93</x:v>
-      </x:c>
-      <x:c r="E23" s="23" t="n">
-        <x:v>3797.64</x:v>
-      </x:c>
-      <x:c r="F23" s="23" t="n">
-        <x:v>3940.04</x:v>
-      </x:c>
-      <x:c r="G23" s="23"/>
-      <x:c r="H23" s="24"/>
-      <x:c r="I23" s="26" t="n">
-        <x:f>ROUND(D23-E23,1)</x:f>
-        <x:v>143.3</x:v>
-      </x:c>
-      <x:c r="J23" s="22" t="str">
-        <x:v>上证指数</x:v>
-      </x:c>
-      <x:c r="K23" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="22" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B24" s="22" t="str">
-        <x:v>8月10日-8月14日</x:v>
-      </x:c>
-      <x:c r="C24" s="23" t="n">
-        <x:v>3943.82</x:v>
-      </x:c>
-      <x:c r="D24" s="23" t="n">
-        <x:v>3968.48</x:v>
-      </x:c>
-      <x:c r="E24" s="23" t="n">
-        <x:v>3903.7</x:v>
-      </x:c>
-      <x:c r="F24" s="23" t="n">
-        <x:v>3927.18</x:v>
-      </x:c>
-      <x:c r="G24" s="23" t="n">
-        <x:f>ROUND(F24-F23,1)</x:f>
-        <x:v>-12.9</x:v>
-      </x:c>
-      <x:c r="H24" s="24" t="n">
-        <x:f>IFERROR(F24/F23-1,"")</x:f>
-        <x:v>-0.003263926254555849</x:v>
-      </x:c>
-      <x:c r="I24" s="26" t="n">
-        <x:f>ROUND(D24-E24,1)</x:f>
-        <x:v>64.8</x:v>
-      </x:c>
-      <x:c r="J24" s="22" t="str">
-        <x:v>上证指数</x:v>
-      </x:c>
-      <x:c r="K24" s="22" t="n">
-        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="B25" s="22" t="str">
-        <x:v>8月17日-8月21日</x:v>
+        <x:v>8月3日-8月7日</x:v>
       </x:c>
       <x:c r="C25" s="23" t="n">
-        <x:v>3930.1</x:v>
+        <x:v>3812.61</x:v>
       </x:c>
       <x:c r="D25" s="23" t="n">
-        <x:v>3994.18</x:v>
+        <x:v>3940.93</x:v>
       </x:c>
       <x:c r="E25" s="23" t="n">
-        <x:v>3879.58</x:v>
+        <x:v>3797.64</x:v>
       </x:c>
       <x:c r="F25" s="23" t="n">
-        <x:v>3905.2</x:v>
-      </x:c>
-      <x:c r="G25" s="23" t="n">
-        <x:f>ROUND(F25-F24,1)</x:f>
-        <x:v>-22</x:v>
-      </x:c>
-      <x:c r="H25" s="24" t="n">
-        <x:f>IFERROR(F25/F24-1,"")</x:f>
-        <x:v>-0.00559689140808417</x:v>
-      </x:c>
+        <x:v>3940.04</x:v>
+      </x:c>
+      <x:c r="G25" s="23"/>
+      <x:c r="H25" s="24"/>
       <x:c r="I25" s="26" t="n">
         <x:f>ROUND(D25-E25,1)</x:f>
-        <x:v>114.6</x:v>
+        <x:v>143.3</x:v>
       </x:c>
       <x:c r="J25" s="22" t="str">
         <x:v>上证指数</x:v>
@@ -2354,34 +2354,34 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="B26" s="22" t="str">
-        <x:v>8月24日-8月28日</x:v>
+        <x:v>8月10日-8月14日</x:v>
       </x:c>
       <x:c r="C26" s="23" t="n">
-        <x:v>3902.7</x:v>
+        <x:v>3943.82</x:v>
       </x:c>
       <x:c r="D26" s="23" t="n">
-        <x:v>3970.31</x:v>
+        <x:v>3968.48</x:v>
       </x:c>
       <x:c r="E26" s="23" t="n">
-        <x:v>3850.86</x:v>
+        <x:v>3903.7</x:v>
       </x:c>
       <x:c r="F26" s="23" t="n">
-        <x:v>3952.18</x:v>
+        <x:v>3927.18</x:v>
       </x:c>
       <x:c r="G26" s="23" t="n">
         <x:f>ROUND(F26-F25,1)</x:f>
-        <x:v>47</x:v>
+        <x:v>-12.9</x:v>
       </x:c>
       <x:c r="H26" s="24" t="n">
         <x:f>IFERROR(F26/F25-1,"")</x:f>
-        <x:v>0.012030113694561084</x:v>
+        <x:v>-0.003263926254555849</x:v>
       </x:c>
       <x:c r="I26" s="26" t="n">
         <x:f>ROUND(D26-E26,1)</x:f>
-        <x:v>119.4</x:v>
+        <x:v>64.8</x:v>
       </x:c>
       <x:c r="J26" s="22" t="str">
         <x:v>上证指数</x:v>
@@ -2391,231 +2391,231 @@
       </x:c>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="31" t="str">
+      <x:c r="A27" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B27" s="22" t="str">
+        <x:v>8月17日-8月21日</x:v>
+      </x:c>
+      <x:c r="C27" s="23" t="n">
+        <x:v>3930.1</x:v>
+      </x:c>
+      <x:c r="D27" s="23" t="n">
+        <x:v>3994.18</x:v>
+      </x:c>
+      <x:c r="E27" s="23" t="n">
+        <x:v>3879.58</x:v>
+      </x:c>
+      <x:c r="F27" s="23" t="n">
+        <x:v>3905.2</x:v>
+      </x:c>
+      <x:c r="G27" s="23" t="n">
+        <x:f>ROUND(F27-F26,1)</x:f>
+        <x:v>-22</x:v>
+      </x:c>
+      <x:c r="H27" s="24" t="n">
+        <x:f>IFERROR(F27/F26-1,"")</x:f>
+        <x:v>-0.00559689140808417</x:v>
+      </x:c>
+      <x:c r="I27" s="26" t="n">
+        <x:f>ROUND(D27-E27,1)</x:f>
+        <x:v>114.6</x:v>
+      </x:c>
+      <x:c r="J27" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="K27" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B28" s="22" t="str">
+        <x:v>8月24日-8月28日</x:v>
+      </x:c>
+      <x:c r="C28" s="23" t="n">
+        <x:v>3902.7</x:v>
+      </x:c>
+      <x:c r="D28" s="23" t="n">
+        <x:v>3970.31</x:v>
+      </x:c>
+      <x:c r="E28" s="23" t="n">
+        <x:v>3850.86</x:v>
+      </x:c>
+      <x:c r="F28" s="23" t="n">
+        <x:v>3952.18</x:v>
+      </x:c>
+      <x:c r="G28" s="23" t="n">
+        <x:f>ROUND(F28-F27,1)</x:f>
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="H28" s="24" t="n">
+        <x:f>IFERROR(F28/F27-1,"")</x:f>
+        <x:v>0.012030113694561084</x:v>
+      </x:c>
+      <x:c r="I28" s="26" t="n">
+        <x:f>ROUND(D28-E28,1)</x:f>
+        <x:v>119.4</x:v>
+      </x:c>
+      <x:c r="J28" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="K28" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B29" s="22" t="str">
+        <x:v>8月31日</x:v>
+      </x:c>
+      <x:c r="C29" s="23" t="n">
+        <x:v>3926.53</x:v>
+      </x:c>
+      <x:c r="D29" s="23" t="n">
+        <x:v>3986.3</x:v>
+      </x:c>
+      <x:c r="E29" s="23" t="n">
+        <x:v>3926.5</x:v>
+      </x:c>
+      <x:c r="F29" s="23" t="n">
+        <x:v>3986.3</x:v>
+      </x:c>
+      <x:c r="G29" s="23" t="n">
+        <x:f>ROUND(F29-F28,1)</x:f>
+        <x:v>34.1</x:v>
+      </x:c>
+      <x:c r="H29" s="24" t="n">
+        <x:f>IFERROR(F29/F28-1,"")</x:f>
+        <x:v>0.008633210025859261</x:v>
+      </x:c>
+      <x:c r="I29" s="26" t="n">
+        <x:f>ROUND(D29-E29,1)</x:f>
+        <x:v>59.8</x:v>
+      </x:c>
+      <x:c r="J29" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="K29" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B27" s="30" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C27" s="30"/>
-      <x:c r="D27" s="30"/>
-      <x:c r="E27" s="30"/>
-      <x:c r="F27" s="30"/>
-      <x:c r="G27" s="30"/>
-      <x:c r="H27" s="30"/>
-      <x:c r="I27" s="32" t="n">
-        <x:f>ROUND(SUM(I23:I26),1)</x:f>
-        <x:v>442.1</x:v>
-      </x:c>
-      <x:c r="J27" s="30"/>
-      <x:c r="K27" s="30"/>
-    </x:row>
-    <x:row r="28">
-      <x:c r="A28" s="31" t="str">
+      <x:c r="B30" s="30" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C30" s="30"/>
+      <x:c r="D30" s="30"/>
+      <x:c r="E30" s="30"/>
+      <x:c r="F30" s="30"/>
+      <x:c r="G30" s="30"/>
+      <x:c r="H30" s="30"/>
+      <x:c r="I30" s="32" t="n">
+        <x:f>ROUND(SUM(I25:I29),1)</x:f>
+        <x:v>501.9</x:v>
+      </x:c>
+      <x:c r="J30" s="30"/>
+      <x:c r="K30" s="30"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B28" s="30"/>
-      <x:c r="C28" s="30"/>
-      <x:c r="D28" s="30"/>
-      <x:c r="E28" s="30"/>
-      <x:c r="F28" s="30"/>
-      <x:c r="G28" s="30"/>
-      <x:c r="H28" s="30"/>
-      <x:c r="I28" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I23:I26),0),1)</x:f>
-        <x:v>110.5</x:v>
-      </x:c>
-      <x:c r="J28" s="30"/>
-      <x:c r="K28" s="30"/>
-    </x:row>
-    <x:row r="30">
-      <x:c r="A30" s="17" t="str">
+      <x:c r="B31" s="30"/>
+      <x:c r="C31" s="30"/>
+      <x:c r="D31" s="30"/>
+      <x:c r="E31" s="30"/>
+      <x:c r="F31" s="30"/>
+      <x:c r="G31" s="30"/>
+      <x:c r="H31" s="30"/>
+      <x:c r="I31" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I25:I29),0),1)</x:f>
+        <x:v>100.4</x:v>
+      </x:c>
+      <x:c r="J31" s="30"/>
+      <x:c r="K31" s="30"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="17" t="str">
         <x:v>IM主力</x:v>
       </x:c>
-      <x:c r="B30" s="17"/>
-      <x:c r="C30" s="17"/>
-      <x:c r="D30" s="17"/>
-      <x:c r="E30" s="17"/>
-      <x:c r="F30" s="17"/>
-      <x:c r="G30" s="17"/>
-      <x:c r="H30" s="17"/>
-      <x:c r="I30" s="17"/>
-      <x:c r="J30" s="17"/>
-      <x:c r="K30" s="17"/>
-    </x:row>
-    <x:row r="31">
-      <x:c r="A31" s="20" t="str">
+      <x:c r="B33" s="17"/>
+      <x:c r="C33" s="17"/>
+      <x:c r="D33" s="17"/>
+      <x:c r="E33" s="17"/>
+      <x:c r="F33" s="17"/>
+      <x:c r="G33" s="17"/>
+      <x:c r="H33" s="17"/>
+      <x:c r="I33" s="17"/>
+      <x:c r="J33" s="17"/>
+      <x:c r="K33" s="17"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B31" s="20" t="str">
+      <x:c r="B34" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C31" s="20" t="str">
+      <x:c r="C34" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D31" s="20" t="str">
+      <x:c r="D34" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E31" s="20" t="str">
+      <x:c r="E34" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F31" s="20" t="str">
+      <x:c r="F34" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G31" s="20" t="str">
+      <x:c r="G34" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H31" s="20" t="str">
+      <x:c r="H34" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I31" s="20" t="str">
+      <x:c r="I34" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J31" s="20" t="str">
+      <x:c r="J34" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K31" s="20" t="str">
+      <x:c r="K34" s="20" t="str">
         <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32">
-      <x:c r="A32" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B32" s="22" t="str">
-        <x:v>8月3日-8月7日</x:v>
-      </x:c>
-      <x:c r="C32" s="23" t="n">
-        <x:v>7000</x:v>
-      </x:c>
-      <x:c r="D32" s="23" t="n">
-        <x:v>7594.2</x:v>
-      </x:c>
-      <x:c r="E32" s="23" t="n">
-        <x:v>6976</x:v>
-      </x:c>
-      <x:c r="F32" s="23" t="n">
-        <x:v>7590.6</x:v>
-      </x:c>
-      <x:c r="G32" s="23"/>
-      <x:c r="H32" s="24"/>
-      <x:c r="I32" s="26" t="n">
-        <x:f>ROUND(D32-E32,1)</x:f>
-        <x:v>618.2</x:v>
-      </x:c>
-      <x:c r="J32" s="22" t="str">
-        <x:v>IM2609</x:v>
-      </x:c>
-      <x:c r="K32" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33">
-      <x:c r="A33" s="22" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B33" s="22" t="str">
-        <x:v>8月10日-8月14日</x:v>
-      </x:c>
-      <x:c r="C33" s="23" t="n">
-        <x:v>7628.8</x:v>
-      </x:c>
-      <x:c r="D33" s="23" t="n">
-        <x:v>7776</x:v>
-      </x:c>
-      <x:c r="E33" s="23" t="n">
-        <x:v>7525</x:v>
-      </x:c>
-      <x:c r="F33" s="23" t="n">
-        <x:v>7650.2</x:v>
-      </x:c>
-      <x:c r="G33" s="23" t="n">
-        <x:f>ROUND(F33-F32,1)</x:f>
-        <x:v>59.6</x:v>
-      </x:c>
-      <x:c r="H33" s="24" t="n">
-        <x:f>IFERROR(F33/F32-1,"")</x:f>
-        <x:v>0.007851816720680693</x:v>
-      </x:c>
-      <x:c r="I33" s="26" t="n">
-        <x:f>ROUND(D33-E33,1)</x:f>
-        <x:v>251</x:v>
-      </x:c>
-      <x:c r="J33" s="22" t="str">
-        <x:v>IM2609</x:v>
-      </x:c>
-      <x:c r="K33" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34">
-      <x:c r="A34" s="22" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B34" s="22" t="str">
-        <x:v>8月17日-8月21日</x:v>
-      </x:c>
-      <x:c r="C34" s="23" t="n">
-        <x:v>7675</x:v>
-      </x:c>
-      <x:c r="D34" s="23" t="n">
-        <x:v>7882.8</x:v>
-      </x:c>
-      <x:c r="E34" s="23" t="n">
-        <x:v>7410</x:v>
-      </x:c>
-      <x:c r="F34" s="23" t="n">
-        <x:v>7527</x:v>
-      </x:c>
-      <x:c r="G34" s="23" t="n">
-        <x:f>ROUND(F34-F33,1)</x:f>
-        <x:v>-123.2</x:v>
-      </x:c>
-      <x:c r="H34" s="24" t="n">
-        <x:f>IFERROR(F34/F33-1,"")</x:f>
-        <x:v>-0.016104154139761073</x:v>
-      </x:c>
-      <x:c r="I34" s="26" t="n">
-        <x:f>ROUND(D34-E34,1)</x:f>
-        <x:v>472.8</x:v>
-      </x:c>
-      <x:c r="J34" s="22" t="str">
-        <x:v>IM2609</x:v>
-      </x:c>
-      <x:c r="K34" s="22" t="n">
-        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="B35" s="22" t="str">
-        <x:v>8月24日-8月28日</x:v>
+        <x:v>8月3日-8月7日</x:v>
       </x:c>
       <x:c r="C35" s="23" t="n">
-        <x:v>7534.8</x:v>
+        <x:v>7000</x:v>
       </x:c>
       <x:c r="D35" s="23" t="n">
-        <x:v>7753.8</x:v>
+        <x:v>7594.2</x:v>
       </x:c>
       <x:c r="E35" s="23" t="n">
-        <x:v>7300.2</x:v>
+        <x:v>6976</x:v>
       </x:c>
       <x:c r="F35" s="23" t="n">
-        <x:v>7666.6</x:v>
-      </x:c>
-      <x:c r="G35" s="23" t="n">
-        <x:f>ROUND(F35-F34,1)</x:f>
-        <x:v>139.6</x:v>
-      </x:c>
-      <x:c r="H35" s="24" t="n">
-        <x:f>IFERROR(F35/F34-1,"")</x:f>
-        <x:v>0.01854656569682489</x:v>
-      </x:c>
+        <x:v>7590.6</x:v>
+      </x:c>
+      <x:c r="G35" s="23"/>
+      <x:c r="H35" s="24"/>
       <x:c r="I35" s="26" t="n">
         <x:f>ROUND(D35-E35,1)</x:f>
-        <x:v>453.6</x:v>
+        <x:v>618.2</x:v>
       </x:c>
       <x:c r="J35" s="22" t="str">
         <x:v>IM2609</x:v>
@@ -2625,231 +2625,231 @@
       </x:c>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="31" t="str">
+      <x:c r="A36" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B36" s="22" t="str">
+        <x:v>8月10日-8月14日</x:v>
+      </x:c>
+      <x:c r="C36" s="23" t="n">
+        <x:v>7628.8</x:v>
+      </x:c>
+      <x:c r="D36" s="23" t="n">
+        <x:v>7776</x:v>
+      </x:c>
+      <x:c r="E36" s="23" t="n">
+        <x:v>7525</x:v>
+      </x:c>
+      <x:c r="F36" s="23" t="n">
+        <x:v>7650.2</x:v>
+      </x:c>
+      <x:c r="G36" s="23" t="n">
+        <x:f>ROUND(F36-F35,1)</x:f>
+        <x:v>59.6</x:v>
+      </x:c>
+      <x:c r="H36" s="24" t="n">
+        <x:f>IFERROR(F36/F35-1,"")</x:f>
+        <x:v>0.007851816720680693</x:v>
+      </x:c>
+      <x:c r="I36" s="26" t="n">
+        <x:f>ROUND(D36-E36,1)</x:f>
+        <x:v>251</x:v>
+      </x:c>
+      <x:c r="J36" s="22" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+      <x:c r="K36" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B37" s="22" t="str">
+        <x:v>8月17日-8月21日</x:v>
+      </x:c>
+      <x:c r="C37" s="23" t="n">
+        <x:v>7675</x:v>
+      </x:c>
+      <x:c r="D37" s="23" t="n">
+        <x:v>7882.8</x:v>
+      </x:c>
+      <x:c r="E37" s="23" t="n">
+        <x:v>7410</x:v>
+      </x:c>
+      <x:c r="F37" s="23" t="n">
+        <x:v>7527</x:v>
+      </x:c>
+      <x:c r="G37" s="23" t="n">
+        <x:f>ROUND(F37-F36,1)</x:f>
+        <x:v>-123.2</x:v>
+      </x:c>
+      <x:c r="H37" s="24" t="n">
+        <x:f>IFERROR(F37/F36-1,"")</x:f>
+        <x:v>-0.016104154139761073</x:v>
+      </x:c>
+      <x:c r="I37" s="26" t="n">
+        <x:f>ROUND(D37-E37,1)</x:f>
+        <x:v>472.8</x:v>
+      </x:c>
+      <x:c r="J37" s="22" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+      <x:c r="K37" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B38" s="22" t="str">
+        <x:v>8月24日-8月28日</x:v>
+      </x:c>
+      <x:c r="C38" s="23" t="n">
+        <x:v>7534.8</x:v>
+      </x:c>
+      <x:c r="D38" s="23" t="n">
+        <x:v>7753.8</x:v>
+      </x:c>
+      <x:c r="E38" s="23" t="n">
+        <x:v>7300.2</x:v>
+      </x:c>
+      <x:c r="F38" s="23" t="n">
+        <x:v>7666.6</x:v>
+      </x:c>
+      <x:c r="G38" s="23" t="n">
+        <x:f>ROUND(F38-F37,1)</x:f>
+        <x:v>139.6</x:v>
+      </x:c>
+      <x:c r="H38" s="24" t="n">
+        <x:f>IFERROR(F38/F37-1,"")</x:f>
+        <x:v>0.01854656569682489</x:v>
+      </x:c>
+      <x:c r="I38" s="26" t="n">
+        <x:f>ROUND(D38-E38,1)</x:f>
+        <x:v>453.6</x:v>
+      </x:c>
+      <x:c r="J38" s="22" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+      <x:c r="K38" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B36" s="30" t="n">
+      <x:c r="B39" s="30" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C36" s="30"/>
-      <x:c r="D36" s="30"/>
-      <x:c r="E36" s="30"/>
-      <x:c r="F36" s="30"/>
-      <x:c r="G36" s="30"/>
-      <x:c r="H36" s="30"/>
-      <x:c r="I36" s="32" t="n">
-        <x:f>ROUND(SUM(I32:I35),1)</x:f>
+      <x:c r="C39" s="30"/>
+      <x:c r="D39" s="30"/>
+      <x:c r="E39" s="30"/>
+      <x:c r="F39" s="30"/>
+      <x:c r="G39" s="30"/>
+      <x:c r="H39" s="30"/>
+      <x:c r="I39" s="32" t="n">
+        <x:f>ROUND(SUM(I35:I38),1)</x:f>
         <x:v>1795.6</x:v>
       </x:c>
-      <x:c r="J36" s="30"/>
-      <x:c r="K36" s="30"/>
-    </x:row>
-    <x:row r="37">
-      <x:c r="A37" s="31" t="str">
+      <x:c r="J39" s="30"/>
+      <x:c r="K39" s="30"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B37" s="30"/>
-      <x:c r="C37" s="30"/>
-      <x:c r="D37" s="30"/>
-      <x:c r="E37" s="30"/>
-      <x:c r="F37" s="30"/>
-      <x:c r="G37" s="30"/>
-      <x:c r="H37" s="30"/>
-      <x:c r="I37" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I32:I35),0),1)</x:f>
+      <x:c r="B40" s="30"/>
+      <x:c r="C40" s="30"/>
+      <x:c r="D40" s="30"/>
+      <x:c r="E40" s="30"/>
+      <x:c r="F40" s="30"/>
+      <x:c r="G40" s="30"/>
+      <x:c r="H40" s="30"/>
+      <x:c r="I40" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I35:I38),0),1)</x:f>
         <x:v>448.9</x:v>
       </x:c>
-      <x:c r="J37" s="30"/>
-      <x:c r="K37" s="30"/>
-    </x:row>
-    <x:row r="39">
-      <x:c r="A39" s="17" t="str">
+      <x:c r="J40" s="30"/>
+      <x:c r="K40" s="30"/>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="17" t="str">
         <x:v>IC主力</x:v>
       </x:c>
-      <x:c r="B39" s="17"/>
-      <x:c r="C39" s="17"/>
-      <x:c r="D39" s="17"/>
-      <x:c r="E39" s="17"/>
-      <x:c r="F39" s="17"/>
-      <x:c r="G39" s="17"/>
-      <x:c r="H39" s="17"/>
-      <x:c r="I39" s="17"/>
-      <x:c r="J39" s="17"/>
-      <x:c r="K39" s="17"/>
-    </x:row>
-    <x:row r="40">
-      <x:c r="A40" s="20" t="str">
+      <x:c r="B42" s="17"/>
+      <x:c r="C42" s="17"/>
+      <x:c r="D42" s="17"/>
+      <x:c r="E42" s="17"/>
+      <x:c r="F42" s="17"/>
+      <x:c r="G42" s="17"/>
+      <x:c r="H42" s="17"/>
+      <x:c r="I42" s="17"/>
+      <x:c r="J42" s="17"/>
+      <x:c r="K42" s="17"/>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B40" s="20" t="str">
+      <x:c r="B43" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C40" s="20" t="str">
+      <x:c r="C43" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D40" s="20" t="str">
+      <x:c r="D43" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E40" s="20" t="str">
+      <x:c r="E43" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F40" s="20" t="str">
+      <x:c r="F43" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G40" s="20" t="str">
+      <x:c r="G43" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H40" s="20" t="str">
+      <x:c r="H43" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I40" s="20" t="str">
+      <x:c r="I43" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J40" s="20" t="str">
+      <x:c r="J43" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K40" s="20" t="str">
+      <x:c r="K43" s="20" t="str">
         <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="41">
-      <x:c r="A41" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B41" s="22" t="str">
-        <x:v>8月3日-8月7日</x:v>
-      </x:c>
-      <x:c r="C41" s="23" t="n">
-        <x:v>7391</x:v>
-      </x:c>
-      <x:c r="D41" s="23" t="n">
-        <x:v>7882.6</x:v>
-      </x:c>
-      <x:c r="E41" s="23" t="n">
-        <x:v>7335</x:v>
-      </x:c>
-      <x:c r="F41" s="23" t="n">
-        <x:v>7877.8</x:v>
-      </x:c>
-      <x:c r="G41" s="23"/>
-      <x:c r="H41" s="24"/>
-      <x:c r="I41" s="26" t="n">
-        <x:f>ROUND(D41-E41,1)</x:f>
-        <x:v>547.6</x:v>
-      </x:c>
-      <x:c r="J41" s="22" t="str">
-        <x:v>IC2609</x:v>
-      </x:c>
-      <x:c r="K41" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="42">
-      <x:c r="A42" s="22" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B42" s="22" t="str">
-        <x:v>8月10日-8月14日</x:v>
-      </x:c>
-      <x:c r="C42" s="23" t="n">
-        <x:v>7888</x:v>
-      </x:c>
-      <x:c r="D42" s="23" t="n">
-        <x:v>8024</x:v>
-      </x:c>
-      <x:c r="E42" s="23" t="n">
-        <x:v>7795.8</x:v>
-      </x:c>
-      <x:c r="F42" s="23" t="n">
-        <x:v>7861.2</x:v>
-      </x:c>
-      <x:c r="G42" s="23" t="n">
-        <x:f>ROUND(F42-F41,1)</x:f>
-        <x:v>-16.6</x:v>
-      </x:c>
-      <x:c r="H42" s="24" t="n">
-        <x:f>IFERROR(F42/F41-1,"")</x:f>
-        <x:v>-0.0021071872857905127</x:v>
-      </x:c>
-      <x:c r="I42" s="26" t="n">
-        <x:f>ROUND(D42-E42,1)</x:f>
-        <x:v>228.2</x:v>
-      </x:c>
-      <x:c r="J42" s="22" t="str">
-        <x:v>IC2609</x:v>
-      </x:c>
-      <x:c r="K42" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="43">
-      <x:c r="A43" s="22" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B43" s="22" t="str">
-        <x:v>8月17日-8月21日</x:v>
-      </x:c>
-      <x:c r="C43" s="23" t="n">
-        <x:v>7885</x:v>
-      </x:c>
-      <x:c r="D43" s="23" t="n">
-        <x:v>8091.8</x:v>
-      </x:c>
-      <x:c r="E43" s="23" t="n">
-        <x:v>7669.6</x:v>
-      </x:c>
-      <x:c r="F43" s="23" t="n">
-        <x:v>7762</x:v>
-      </x:c>
-      <x:c r="G43" s="23" t="n">
-        <x:f>ROUND(F43-F42,1)</x:f>
-        <x:v>-99.2</x:v>
-      </x:c>
-      <x:c r="H43" s="24" t="n">
-        <x:f>IFERROR(F43/F42-1,"")</x:f>
-        <x:v>-0.012618938584439965</x:v>
-      </x:c>
-      <x:c r="I43" s="26" t="n">
-        <x:f>ROUND(D43-E43,1)</x:f>
-        <x:v>422.2</x:v>
-      </x:c>
-      <x:c r="J43" s="22" t="str">
-        <x:v>IC2609</x:v>
-      </x:c>
-      <x:c r="K43" s="22" t="n">
-        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="B44" s="22" t="str">
-        <x:v>8月24日-8月28日</x:v>
+        <x:v>8月3日-8月7日</x:v>
       </x:c>
       <x:c r="C44" s="23" t="n">
-        <x:v>7757</x:v>
+        <x:v>7391</x:v>
       </x:c>
       <x:c r="D44" s="23" t="n">
-        <x:v>7931</x:v>
+        <x:v>7882.6</x:v>
       </x:c>
       <x:c r="E44" s="23" t="n">
-        <x:v>7496</x:v>
+        <x:v>7335</x:v>
       </x:c>
       <x:c r="F44" s="23" t="n">
-        <x:v>7853.8</x:v>
-      </x:c>
-      <x:c r="G44" s="23" t="n">
-        <x:f>ROUND(F44-F43,1)</x:f>
-        <x:v>91.8</x:v>
-      </x:c>
-      <x:c r="H44" s="24" t="n">
-        <x:f>IFERROR(F44/F43-1,"")</x:f>
-        <x:v>0.011826848750322139</x:v>
-      </x:c>
+        <x:v>7877.8</x:v>
+      </x:c>
+      <x:c r="G44" s="23"/>
+      <x:c r="H44" s="24"/>
       <x:c r="I44" s="26" t="n">
         <x:f>ROUND(D44-E44,1)</x:f>
-        <x:v>435</x:v>
+        <x:v>547.6</x:v>
       </x:c>
       <x:c r="J44" s="22" t="str">
         <x:v>IC2609</x:v>
@@ -2859,231 +2859,231 @@
       </x:c>
     </x:row>
     <x:row r="45">
-      <x:c r="A45" s="31" t="str">
+      <x:c r="A45" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B45" s="22" t="str">
+        <x:v>8月10日-8月14日</x:v>
+      </x:c>
+      <x:c r="C45" s="23" t="n">
+        <x:v>7888</x:v>
+      </x:c>
+      <x:c r="D45" s="23" t="n">
+        <x:v>8024</x:v>
+      </x:c>
+      <x:c r="E45" s="23" t="n">
+        <x:v>7795.8</x:v>
+      </x:c>
+      <x:c r="F45" s="23" t="n">
+        <x:v>7861.2</x:v>
+      </x:c>
+      <x:c r="G45" s="23" t="n">
+        <x:f>ROUND(F45-F44,1)</x:f>
+        <x:v>-16.6</x:v>
+      </x:c>
+      <x:c r="H45" s="24" t="n">
+        <x:f>IFERROR(F45/F44-1,"")</x:f>
+        <x:v>-0.0021071872857905127</x:v>
+      </x:c>
+      <x:c r="I45" s="26" t="n">
+        <x:f>ROUND(D45-E45,1)</x:f>
+        <x:v>228.2</x:v>
+      </x:c>
+      <x:c r="J45" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+      <x:c r="K45" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B46" s="22" t="str">
+        <x:v>8月17日-8月21日</x:v>
+      </x:c>
+      <x:c r="C46" s="23" t="n">
+        <x:v>7885</x:v>
+      </x:c>
+      <x:c r="D46" s="23" t="n">
+        <x:v>8091.8</x:v>
+      </x:c>
+      <x:c r="E46" s="23" t="n">
+        <x:v>7669.6</x:v>
+      </x:c>
+      <x:c r="F46" s="23" t="n">
+        <x:v>7762</x:v>
+      </x:c>
+      <x:c r="G46" s="23" t="n">
+        <x:f>ROUND(F46-F45,1)</x:f>
+        <x:v>-99.2</x:v>
+      </x:c>
+      <x:c r="H46" s="24" t="n">
+        <x:f>IFERROR(F46/F45-1,"")</x:f>
+        <x:v>-0.012618938584439965</x:v>
+      </x:c>
+      <x:c r="I46" s="26" t="n">
+        <x:f>ROUND(D46-E46,1)</x:f>
+        <x:v>422.2</x:v>
+      </x:c>
+      <x:c r="J46" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+      <x:c r="K46" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B47" s="22" t="str">
+        <x:v>8月24日-8月28日</x:v>
+      </x:c>
+      <x:c r="C47" s="23" t="n">
+        <x:v>7757</x:v>
+      </x:c>
+      <x:c r="D47" s="23" t="n">
+        <x:v>7931</x:v>
+      </x:c>
+      <x:c r="E47" s="23" t="n">
+        <x:v>7496</x:v>
+      </x:c>
+      <x:c r="F47" s="23" t="n">
+        <x:v>7853.8</x:v>
+      </x:c>
+      <x:c r="G47" s="23" t="n">
+        <x:f>ROUND(F47-F46,1)</x:f>
+        <x:v>91.8</x:v>
+      </x:c>
+      <x:c r="H47" s="24" t="n">
+        <x:f>IFERROR(F47/F46-1,"")</x:f>
+        <x:v>0.011826848750322139</x:v>
+      </x:c>
+      <x:c r="I47" s="26" t="n">
+        <x:f>ROUND(D47-E47,1)</x:f>
+        <x:v>435</x:v>
+      </x:c>
+      <x:c r="J47" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+      <x:c r="K47" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B45" s="30" t="n">
+      <x:c r="B48" s="30" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C45" s="30"/>
-      <x:c r="D45" s="30"/>
-      <x:c r="E45" s="30"/>
-      <x:c r="F45" s="30"/>
-      <x:c r="G45" s="30"/>
-      <x:c r="H45" s="30"/>
-      <x:c r="I45" s="32" t="n">
-        <x:f>ROUND(SUM(I41:I44),1)</x:f>
+      <x:c r="C48" s="30"/>
+      <x:c r="D48" s="30"/>
+      <x:c r="E48" s="30"/>
+      <x:c r="F48" s="30"/>
+      <x:c r="G48" s="30"/>
+      <x:c r="H48" s="30"/>
+      <x:c r="I48" s="32" t="n">
+        <x:f>ROUND(SUM(I44:I47),1)</x:f>
         <x:v>1633</x:v>
       </x:c>
-      <x:c r="J45" s="30"/>
-      <x:c r="K45" s="30"/>
-    </x:row>
-    <x:row r="46">
-      <x:c r="A46" s="31" t="str">
+      <x:c r="J48" s="30"/>
+      <x:c r="K48" s="30"/>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B46" s="30"/>
-      <x:c r="C46" s="30"/>
-      <x:c r="D46" s="30"/>
-      <x:c r="E46" s="30"/>
-      <x:c r="F46" s="30"/>
-      <x:c r="G46" s="30"/>
-      <x:c r="H46" s="30"/>
-      <x:c r="I46" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I41:I44),0),1)</x:f>
+      <x:c r="B49" s="30"/>
+      <x:c r="C49" s="30"/>
+      <x:c r="D49" s="30"/>
+      <x:c r="E49" s="30"/>
+      <x:c r="F49" s="30"/>
+      <x:c r="G49" s="30"/>
+      <x:c r="H49" s="30"/>
+      <x:c r="I49" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I44:I47),0),1)</x:f>
         <x:v>408.3</x:v>
       </x:c>
-      <x:c r="J46" s="30"/>
-      <x:c r="K46" s="30"/>
-    </x:row>
-    <x:row r="48">
-      <x:c r="A48" s="17" t="str">
+      <x:c r="J49" s="30"/>
+      <x:c r="K49" s="30"/>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="17" t="str">
         <x:v>IF主力</x:v>
       </x:c>
-      <x:c r="B48" s="17"/>
-      <x:c r="C48" s="17"/>
-      <x:c r="D48" s="17"/>
-      <x:c r="E48" s="17"/>
-      <x:c r="F48" s="17"/>
-      <x:c r="G48" s="17"/>
-      <x:c r="H48" s="17"/>
-      <x:c r="I48" s="17"/>
-      <x:c r="J48" s="17"/>
-      <x:c r="K48" s="17"/>
-    </x:row>
-    <x:row r="49">
-      <x:c r="A49" s="20" t="str">
+      <x:c r="B51" s="17"/>
+      <x:c r="C51" s="17"/>
+      <x:c r="D51" s="17"/>
+      <x:c r="E51" s="17"/>
+      <x:c r="F51" s="17"/>
+      <x:c r="G51" s="17"/>
+      <x:c r="H51" s="17"/>
+      <x:c r="I51" s="17"/>
+      <x:c r="J51" s="17"/>
+      <x:c r="K51" s="17"/>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B49" s="20" t="str">
+      <x:c r="B52" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C49" s="20" t="str">
+      <x:c r="C52" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D49" s="20" t="str">
+      <x:c r="D52" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E49" s="20" t="str">
+      <x:c r="E52" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F49" s="20" t="str">
+      <x:c r="F52" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G49" s="20" t="str">
+      <x:c r="G52" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H49" s="20" t="str">
+      <x:c r="H52" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I49" s="20" t="str">
+      <x:c r="I52" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J49" s="20" t="str">
+      <x:c r="J52" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K49" s="20" t="str">
+      <x:c r="K52" s="20" t="str">
         <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="50">
-      <x:c r="A50" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B50" s="22" t="str">
-        <x:v>8月3日-8月7日</x:v>
-      </x:c>
-      <x:c r="C50" s="23" t="n">
-        <x:v>4526.4</x:v>
-      </x:c>
-      <x:c r="D50" s="23" t="n">
-        <x:v>4656.2</x:v>
-      </x:c>
-      <x:c r="E50" s="23" t="n">
-        <x:v>4494.2</x:v>
-      </x:c>
-      <x:c r="F50" s="23" t="n">
-        <x:v>4645.6</x:v>
-      </x:c>
-      <x:c r="G50" s="23"/>
-      <x:c r="H50" s="24"/>
-      <x:c r="I50" s="26" t="n">
-        <x:f>ROUND(D50-E50,1)</x:f>
-        <x:v>162</x:v>
-      </x:c>
-      <x:c r="J50" s="22" t="str">
-        <x:v>IF2609</x:v>
-      </x:c>
-      <x:c r="K50" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="51">
-      <x:c r="A51" s="22" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B51" s="22" t="str">
-        <x:v>8月10日-8月14日</x:v>
-      </x:c>
-      <x:c r="C51" s="23" t="n">
-        <x:v>4656.8</x:v>
-      </x:c>
-      <x:c r="D51" s="23" t="n">
-        <x:v>4681</x:v>
-      </x:c>
-      <x:c r="E51" s="23" t="n">
-        <x:v>4598</x:v>
-      </x:c>
-      <x:c r="F51" s="23" t="n">
-        <x:v>4620.4</x:v>
-      </x:c>
-      <x:c r="G51" s="23" t="n">
-        <x:f>ROUND(F51-F50,1)</x:f>
-        <x:v>-25.2</x:v>
-      </x:c>
-      <x:c r="H51" s="24" t="n">
-        <x:f>IFERROR(F51/F50-1,"")</x:f>
-        <x:v>-0.005424487687274104</x:v>
-      </x:c>
-      <x:c r="I51" s="23" t="n">
-        <x:f>ROUND(D51-E51,1)</x:f>
-        <x:v>83</x:v>
-      </x:c>
-      <x:c r="J51" s="22" t="str">
-        <x:v>IF2609</x:v>
-      </x:c>
-      <x:c r="K51" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="52">
-      <x:c r="A52" s="22" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B52" s="22" t="str">
-        <x:v>8月17日-8月21日</x:v>
-      </x:c>
-      <x:c r="C52" s="23" t="n">
-        <x:v>4624</x:v>
-      </x:c>
-      <x:c r="D52" s="23" t="n">
-        <x:v>4700.6</x:v>
-      </x:c>
-      <x:c r="E52" s="23" t="n">
-        <x:v>4531.8</x:v>
-      </x:c>
-      <x:c r="F52" s="23" t="n">
-        <x:v>4576</x:v>
-      </x:c>
-      <x:c r="G52" s="23" t="n">
-        <x:f>ROUND(F52-F51,1)</x:f>
-        <x:v>-44.4</x:v>
-      </x:c>
-      <x:c r="H52" s="24" t="n">
-        <x:f>IFERROR(F52/F51-1,"")</x:f>
-        <x:v>-0.00960955761405935</x:v>
-      </x:c>
-      <x:c r="I52" s="26" t="n">
-        <x:f>ROUND(D52-E52,1)</x:f>
-        <x:v>168.8</x:v>
-      </x:c>
-      <x:c r="J52" s="22" t="str">
-        <x:v>IF2609</x:v>
-      </x:c>
-      <x:c r="K52" s="22" t="n">
-        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="B53" s="22" t="str">
-        <x:v>8月24日-8月28日</x:v>
+        <x:v>8月3日-8月7日</x:v>
       </x:c>
       <x:c r="C53" s="23" t="n">
-        <x:v>4607.4</x:v>
+        <x:v>4526.4</x:v>
       </x:c>
       <x:c r="D53" s="23" t="n">
-        <x:v>4620</x:v>
+        <x:v>4656.2</x:v>
       </x:c>
       <x:c r="E53" s="23" t="n">
-        <x:v>4486.4</x:v>
+        <x:v>4494.2</x:v>
       </x:c>
       <x:c r="F53" s="23" t="n">
-        <x:v>4593.6</x:v>
-      </x:c>
-      <x:c r="G53" s="23" t="n">
-        <x:f>ROUND(F53-F52,1)</x:f>
-        <x:v>17.6</x:v>
-      </x:c>
-      <x:c r="H53" s="24" t="n">
-        <x:f>IFERROR(F53/F52-1,"")</x:f>
-        <x:v>0.0038461538461538325</x:v>
-      </x:c>
+        <x:v>4645.6</x:v>
+      </x:c>
+      <x:c r="G53" s="23"/>
+      <x:c r="H53" s="24"/>
       <x:c r="I53" s="26" t="n">
         <x:f>ROUND(D53-E53,1)</x:f>
-        <x:v>133.6</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="J53" s="22" t="str">
         <x:v>IF2609</x:v>
@@ -3093,522 +3093,674 @@
       </x:c>
     </x:row>
     <x:row r="54">
-      <x:c r="A54" s="31" t="str">
+      <x:c r="A54" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B54" s="22" t="str">
+        <x:v>8月10日-8月14日</x:v>
+      </x:c>
+      <x:c r="C54" s="23" t="n">
+        <x:v>4656.8</x:v>
+      </x:c>
+      <x:c r="D54" s="23" t="n">
+        <x:v>4681</x:v>
+      </x:c>
+      <x:c r="E54" s="23" t="n">
+        <x:v>4598</x:v>
+      </x:c>
+      <x:c r="F54" s="23" t="n">
+        <x:v>4620.4</x:v>
+      </x:c>
+      <x:c r="G54" s="23" t="n">
+        <x:f>ROUND(F54-F53,1)</x:f>
+        <x:v>-25.2</x:v>
+      </x:c>
+      <x:c r="H54" s="24" t="n">
+        <x:f>IFERROR(F54/F53-1,"")</x:f>
+        <x:v>-0.005424487687274104</x:v>
+      </x:c>
+      <x:c r="I54" s="23" t="n">
+        <x:f>ROUND(D54-E54,1)</x:f>
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="J54" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+      <x:c r="K54" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B55" s="22" t="str">
+        <x:v>8月17日-8月21日</x:v>
+      </x:c>
+      <x:c r="C55" s="23" t="n">
+        <x:v>4624</x:v>
+      </x:c>
+      <x:c r="D55" s="23" t="n">
+        <x:v>4700.6</x:v>
+      </x:c>
+      <x:c r="E55" s="23" t="n">
+        <x:v>4531.8</x:v>
+      </x:c>
+      <x:c r="F55" s="23" t="n">
+        <x:v>4576</x:v>
+      </x:c>
+      <x:c r="G55" s="23" t="n">
+        <x:f>ROUND(F55-F54,1)</x:f>
+        <x:v>-44.4</x:v>
+      </x:c>
+      <x:c r="H55" s="24" t="n">
+        <x:f>IFERROR(F55/F54-1,"")</x:f>
+        <x:v>-0.00960955761405935</x:v>
+      </x:c>
+      <x:c r="I55" s="26" t="n">
+        <x:f>ROUND(D55-E55,1)</x:f>
+        <x:v>168.8</x:v>
+      </x:c>
+      <x:c r="J55" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+      <x:c r="K55" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B56" s="22" t="str">
+        <x:v>8月24日-8月28日</x:v>
+      </x:c>
+      <x:c r="C56" s="23" t="n">
+        <x:v>4607.4</x:v>
+      </x:c>
+      <x:c r="D56" s="23" t="n">
+        <x:v>4620</x:v>
+      </x:c>
+      <x:c r="E56" s="23" t="n">
+        <x:v>4486.4</x:v>
+      </x:c>
+      <x:c r="F56" s="23" t="n">
+        <x:v>4593.6</x:v>
+      </x:c>
+      <x:c r="G56" s="23" t="n">
+        <x:f>ROUND(F56-F55,1)</x:f>
+        <x:v>17.6</x:v>
+      </x:c>
+      <x:c r="H56" s="24" t="n">
+        <x:f>IFERROR(F56/F55-1,"")</x:f>
+        <x:v>0.0038461538461538325</x:v>
+      </x:c>
+      <x:c r="I56" s="26" t="n">
+        <x:f>ROUND(D56-E56,1)</x:f>
+        <x:v>133.6</x:v>
+      </x:c>
+      <x:c r="J56" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+      <x:c r="K56" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B57" s="22" t="str">
+        <x:v>8月31日</x:v>
+      </x:c>
+      <x:c r="C57" s="23" t="n">
+        <x:v>4553</x:v>
+      </x:c>
+      <x:c r="D57" s="23" t="n">
+        <x:v>4608.6</x:v>
+      </x:c>
+      <x:c r="E57" s="23" t="n">
+        <x:v>4530</x:v>
+      </x:c>
+      <x:c r="F57" s="23" t="n">
+        <x:v>4601.6</x:v>
+      </x:c>
+      <x:c r="G57" s="23" t="n">
+        <x:f>ROUND(F57-F56,1)</x:f>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H57" s="24" t="n">
+        <x:f>IFERROR(F57/F56-1,"")</x:f>
+        <x:v>0.0017415534656914922</x:v>
+      </x:c>
+      <x:c r="I57" s="23" t="n">
+        <x:f>ROUND(D57-E57,1)</x:f>
+        <x:v>78.6</x:v>
+      </x:c>
+      <x:c r="J57" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+      <x:c r="K57" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B54" s="30" t="n">
+      <x:c r="B58" s="30" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C58" s="30"/>
+      <x:c r="D58" s="30"/>
+      <x:c r="E58" s="30"/>
+      <x:c r="F58" s="30"/>
+      <x:c r="G58" s="30"/>
+      <x:c r="H58" s="30"/>
+      <x:c r="I58" s="32" t="n">
+        <x:f>ROUND(SUM(I53:I57),1)</x:f>
+        <x:v>626</x:v>
+      </x:c>
+      <x:c r="J58" s="30"/>
+      <x:c r="K58" s="30"/>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B59" s="30"/>
+      <x:c r="C59" s="30"/>
+      <x:c r="D59" s="30"/>
+      <x:c r="E59" s="30"/>
+      <x:c r="F59" s="30"/>
+      <x:c r="G59" s="30"/>
+      <x:c r="H59" s="30"/>
+      <x:c r="I59" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I53:I57),0),1)</x:f>
+        <x:v>125.2</x:v>
+      </x:c>
+      <x:c r="J59" s="30"/>
+      <x:c r="K59" s="30"/>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="17" t="str">
+        <x:v>IH主力</x:v>
+      </x:c>
+      <x:c r="B61" s="17"/>
+      <x:c r="C61" s="17"/>
+      <x:c r="D61" s="17"/>
+      <x:c r="E61" s="17"/>
+      <x:c r="F61" s="17"/>
+      <x:c r="G61" s="17"/>
+      <x:c r="H61" s="17"/>
+      <x:c r="I61" s="17"/>
+      <x:c r="J61" s="17"/>
+      <x:c r="K61" s="17"/>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="20" t="str">
+        <x:v>序号</x:v>
+      </x:c>
+      <x:c r="B62" s="20" t="str">
+        <x:v>周期</x:v>
+      </x:c>
+      <x:c r="C62" s="20" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="D62" s="20" t="str">
+        <x:v>高点</x:v>
+      </x:c>
+      <x:c r="E62" s="20" t="str">
+        <x:v>低点</x:v>
+      </x:c>
+      <x:c r="F62" s="20" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="G62" s="20" t="str">
+        <x:v>涨跌点数</x:v>
+      </x:c>
+      <x:c r="H62" s="20" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I62" s="20" t="str">
+        <x:v>振幅</x:v>
+      </x:c>
+      <x:c r="J62" s="20" t="str">
+        <x:v>标的</x:v>
+      </x:c>
+      <x:c r="K62" s="20" t="str">
+        <x:v>交易日</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B63" s="22" t="str">
+        <x:v>8月3日-8月7日</x:v>
+      </x:c>
+      <x:c r="C63" s="23" t="n">
+        <x:v>2882.4</x:v>
+      </x:c>
+      <x:c r="D63" s="23" t="n">
+        <x:v>2930.6</x:v>
+      </x:c>
+      <x:c r="E63" s="23" t="n">
+        <x:v>2845.8</x:v>
+      </x:c>
+      <x:c r="F63" s="23" t="n">
+        <x:v>2930</x:v>
+      </x:c>
+      <x:c r="G63" s="23"/>
+      <x:c r="H63" s="24"/>
+      <x:c r="I63" s="26" t="n">
+        <x:f>ROUND(D63-E63,1)</x:f>
+        <x:v>84.8</x:v>
+      </x:c>
+      <x:c r="J63" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+      <x:c r="K63" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B64" s="22" t="str">
+        <x:v>8月10日-8月14日</x:v>
+      </x:c>
+      <x:c r="C64" s="23" t="n">
+        <x:v>2930</x:v>
+      </x:c>
+      <x:c r="D64" s="23" t="n">
+        <x:v>2949.6</x:v>
+      </x:c>
+      <x:c r="E64" s="23" t="n">
+        <x:v>2877</x:v>
+      </x:c>
+      <x:c r="F64" s="23" t="n">
+        <x:v>2890</x:v>
+      </x:c>
+      <x:c r="G64" s="23" t="n">
+        <x:f>ROUND(F64-F63,1)</x:f>
+        <x:v>-40</x:v>
+      </x:c>
+      <x:c r="H64" s="24" t="n">
+        <x:f>IFERROR(F64/F63-1,"")</x:f>
+        <x:v>-0.013651877133105783</x:v>
+      </x:c>
+      <x:c r="I64" s="26" t="n">
+        <x:f>ROUND(D64-E64,1)</x:f>
+        <x:v>72.6</x:v>
+      </x:c>
+      <x:c r="J64" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+      <x:c r="K64" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B65" s="22" t="str">
+        <x:v>8月17日-8月21日</x:v>
+      </x:c>
+      <x:c r="C65" s="23" t="n">
+        <x:v>2886</x:v>
+      </x:c>
+      <x:c r="D65" s="23" t="n">
+        <x:v>2921.2</x:v>
+      </x:c>
+      <x:c r="E65" s="23" t="n">
+        <x:v>2843</x:v>
+      </x:c>
+      <x:c r="F65" s="23" t="n">
+        <x:v>2861</x:v>
+      </x:c>
+      <x:c r="G65" s="23" t="n">
+        <x:f>ROUND(F65-F64,1)</x:f>
+        <x:v>-29</x:v>
+      </x:c>
+      <x:c r="H65" s="24" t="n">
+        <x:f>IFERROR(F65/F64-1,"")</x:f>
+        <x:v>-0.01003460207612461</x:v>
+      </x:c>
+      <x:c r="I65" s="26" t="n">
+        <x:f>ROUND(D65-E65,1)</x:f>
+        <x:v>78.2</x:v>
+      </x:c>
+      <x:c r="J65" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+      <x:c r="K65" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" s="22" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C54" s="30"/>
-      <x:c r="D54" s="30"/>
-      <x:c r="E54" s="30"/>
-      <x:c r="F54" s="30"/>
-      <x:c r="G54" s="30"/>
-      <x:c r="H54" s="30"/>
-      <x:c r="I54" s="32" t="n">
-        <x:f>ROUND(SUM(I50:I53),1)</x:f>
-        <x:v>547.4</x:v>
-      </x:c>
-      <x:c r="J54" s="30"/>
-      <x:c r="K54" s="30"/>
-    </x:row>
-    <x:row r="55">
-      <x:c r="A55" s="31" t="str">
+      <x:c r="B66" s="22" t="str">
+        <x:v>8月24日-8月28日</x:v>
+      </x:c>
+      <x:c r="C66" s="23" t="n">
+        <x:v>2856.4</x:v>
+      </x:c>
+      <x:c r="D66" s="23" t="n">
+        <x:v>2918.2</x:v>
+      </x:c>
+      <x:c r="E66" s="23" t="n">
+        <x:v>2837.4</x:v>
+      </x:c>
+      <x:c r="F66" s="23" t="n">
+        <x:v>2911.4</x:v>
+      </x:c>
+      <x:c r="G66" s="23" t="n">
+        <x:f>ROUND(F66-F65,1)</x:f>
+        <x:v>50.4</x:v>
+      </x:c>
+      <x:c r="H66" s="24" t="n">
+        <x:f>IFERROR(F66/F65-1,"")</x:f>
+        <x:v>0.01761621810555747</x:v>
+      </x:c>
+      <x:c r="I66" s="26" t="n">
+        <x:f>ROUND(D66-E66,1)</x:f>
+        <x:v>80.8</x:v>
+      </x:c>
+      <x:c r="J66" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+      <x:c r="K66" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" s="31" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B67" s="30" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C67" s="30"/>
+      <x:c r="D67" s="30"/>
+      <x:c r="E67" s="30"/>
+      <x:c r="F67" s="30"/>
+      <x:c r="G67" s="30"/>
+      <x:c r="H67" s="30"/>
+      <x:c r="I67" s="32" t="n">
+        <x:f>ROUND(SUM(I63:I66),1)</x:f>
+        <x:v>316.4</x:v>
+      </x:c>
+      <x:c r="J67" s="30"/>
+      <x:c r="K67" s="30"/>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B55" s="30"/>
-      <x:c r="C55" s="30"/>
-      <x:c r="D55" s="30"/>
-      <x:c r="E55" s="30"/>
-      <x:c r="F55" s="30"/>
-      <x:c r="G55" s="30"/>
-      <x:c r="H55" s="30"/>
-      <x:c r="I55" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I50:I53),0),1)</x:f>
-        <x:v>136.9</x:v>
-      </x:c>
-      <x:c r="J55" s="30"/>
-      <x:c r="K55" s="30"/>
-    </x:row>
-    <x:row r="57">
-      <x:c r="A57" s="17" t="str">
-        <x:v>IH主力</x:v>
-      </x:c>
-      <x:c r="B57" s="17"/>
-      <x:c r="C57" s="17"/>
-      <x:c r="D57" s="17"/>
-      <x:c r="E57" s="17"/>
-      <x:c r="F57" s="17"/>
-      <x:c r="G57" s="17"/>
-      <x:c r="H57" s="17"/>
-      <x:c r="I57" s="17"/>
-      <x:c r="J57" s="17"/>
-      <x:c r="K57" s="17"/>
-    </x:row>
-    <x:row r="58">
-      <x:c r="A58" s="20" t="str">
+      <x:c r="B68" s="30"/>
+      <x:c r="C68" s="30"/>
+      <x:c r="D68" s="30"/>
+      <x:c r="E68" s="30"/>
+      <x:c r="F68" s="30"/>
+      <x:c r="G68" s="30"/>
+      <x:c r="H68" s="30"/>
+      <x:c r="I68" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I63:I66),0),1)</x:f>
+        <x:v>79.1</x:v>
+      </x:c>
+      <x:c r="J68" s="30"/>
+      <x:c r="K68" s="30"/>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" s="17" t="str">
+        <x:v>碳酸锂2609</x:v>
+      </x:c>
+      <x:c r="B70" s="17"/>
+      <x:c r="C70" s="17"/>
+      <x:c r="D70" s="17"/>
+      <x:c r="E70" s="17"/>
+      <x:c r="F70" s="17"/>
+      <x:c r="G70" s="17"/>
+      <x:c r="H70" s="17"/>
+      <x:c r="I70" s="17"/>
+      <x:c r="J70" s="17"/>
+      <x:c r="K70" s="17"/>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B58" s="20" t="str">
+      <x:c r="B71" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C58" s="20" t="str">
+      <x:c r="C71" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D58" s="20" t="str">
+      <x:c r="D71" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E58" s="20" t="str">
+      <x:c r="E71" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F58" s="20" t="str">
+      <x:c r="F71" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G58" s="20" t="str">
+      <x:c r="G71" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H58" s="20" t="str">
+      <x:c r="H71" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I58" s="20" t="str">
+      <x:c r="I71" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J58" s="20" t="str">
+      <x:c r="J71" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K58" s="20" t="str">
+      <x:c r="K71" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="59">
-      <x:c r="A59" s="22" t="n">
+    <x:row r="72">
+      <x:c r="A72" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B59" s="22" t="str">
+      <x:c r="B72" s="22" t="str">
         <x:v>8月3日-8月7日</x:v>
       </x:c>
-      <x:c r="C59" s="23" t="n">
-        <x:v>2882.4</x:v>
-      </x:c>
-      <x:c r="D59" s="23" t="n">
-        <x:v>2930.6</x:v>
-      </x:c>
-      <x:c r="E59" s="23" t="n">
-        <x:v>2845.8</x:v>
-      </x:c>
-      <x:c r="F59" s="23" t="n">
-        <x:v>2930</x:v>
-      </x:c>
-      <x:c r="G59" s="23"/>
-      <x:c r="H59" s="24"/>
-      <x:c r="I59" s="26" t="n">
-        <x:f>ROUND(D59-E59,1)</x:f>
-        <x:v>84.8</x:v>
-      </x:c>
-      <x:c r="J59" s="22" t="str">
-        <x:v>IH2609</x:v>
-      </x:c>
-      <x:c r="K59" s="22" t="n">
+      <x:c r="C72" s="23" t="n">
+        <x:v>137500</x:v>
+      </x:c>
+      <x:c r="D72" s="23" t="n">
+        <x:v>144800</x:v>
+      </x:c>
+      <x:c r="E72" s="23" t="n">
+        <x:v>135560</x:v>
+      </x:c>
+      <x:c r="F72" s="23" t="n">
+        <x:v>140000</x:v>
+      </x:c>
+      <x:c r="G72" s="23"/>
+      <x:c r="H72" s="24"/>
+      <x:c r="I72" s="26" t="n">
+        <x:f>ROUND(D72-E72,1)</x:f>
+        <x:v>9240</x:v>
+      </x:c>
+      <x:c r="J72" s="22" t="str">
+        <x:v>LC2609</x:v>
+      </x:c>
+      <x:c r="K72" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="60">
-      <x:c r="A60" s="22" t="n">
+    <x:row r="73">
+      <x:c r="A73" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B60" s="22" t="str">
+      <x:c r="B73" s="22" t="str">
         <x:v>8月10日-8月14日</x:v>
       </x:c>
-      <x:c r="C60" s="23" t="n">
-        <x:v>2930</x:v>
-      </x:c>
-      <x:c r="D60" s="23" t="n">
-        <x:v>2949.6</x:v>
-      </x:c>
-      <x:c r="E60" s="23" t="n">
-        <x:v>2877</x:v>
-      </x:c>
-      <x:c r="F60" s="23" t="n">
-        <x:v>2890</x:v>
-      </x:c>
-      <x:c r="G60" s="23" t="n">
-        <x:f>ROUND(F60-F59,1)</x:f>
-        <x:v>-40</x:v>
-      </x:c>
-      <x:c r="H60" s="24" t="n">
-        <x:f>IFERROR(F60/F59-1,"")</x:f>
-        <x:v>-0.013651877133105783</x:v>
-      </x:c>
-      <x:c r="I60" s="26" t="n">
-        <x:f>ROUND(D60-E60,1)</x:f>
-        <x:v>72.6</x:v>
-      </x:c>
-      <x:c r="J60" s="22" t="str">
-        <x:v>IH2609</x:v>
-      </x:c>
-      <x:c r="K60" s="22" t="n">
+      <x:c r="C73" s="23" t="n">
+        <x:v>140500</x:v>
+      </x:c>
+      <x:c r="D73" s="23" t="n">
+        <x:v>154500</x:v>
+      </x:c>
+      <x:c r="E73" s="23" t="n">
+        <x:v>139280</x:v>
+      </x:c>
+      <x:c r="F73" s="23" t="n">
+        <x:v>153940</x:v>
+      </x:c>
+      <x:c r="G73" s="28" t="n">
+        <x:f>ROUND(F73-F72,1)</x:f>
+        <x:v>13940</x:v>
+      </x:c>
+      <x:c r="H73" s="24" t="n">
+        <x:f>IFERROR(F73/F72-1,"")</x:f>
+        <x:v>0.09957142857142864</x:v>
+      </x:c>
+      <x:c r="I73" s="26" t="n">
+        <x:f>ROUND(D73-E73,1)</x:f>
+        <x:v>15220</x:v>
+      </x:c>
+      <x:c r="J73" s="22" t="str">
+        <x:v>LC2609</x:v>
+      </x:c>
+      <x:c r="K73" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="61">
-      <x:c r="A61" s="22" t="n">
+    <x:row r="74">
+      <x:c r="A74" s="22" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B61" s="22" t="str">
+      <x:c r="B74" s="22" t="str">
         <x:v>8月17日-8月21日</x:v>
       </x:c>
-      <x:c r="C61" s="23" t="n">
-        <x:v>2886</x:v>
-      </x:c>
-      <x:c r="D61" s="23" t="n">
-        <x:v>2921.2</x:v>
-      </x:c>
-      <x:c r="E61" s="23" t="n">
-        <x:v>2843</x:v>
-      </x:c>
-      <x:c r="F61" s="23" t="n">
-        <x:v>2861</x:v>
-      </x:c>
-      <x:c r="G61" s="23" t="n">
-        <x:f>ROUND(F61-F60,1)</x:f>
-        <x:v>-29</x:v>
-      </x:c>
-      <x:c r="H61" s="24" t="n">
-        <x:f>IFERROR(F61/F60-1,"")</x:f>
-        <x:v>-0.01003460207612461</x:v>
-      </x:c>
-      <x:c r="I61" s="26" t="n">
-        <x:f>ROUND(D61-E61,1)</x:f>
-        <x:v>78.2</x:v>
-      </x:c>
-      <x:c r="J61" s="22" t="str">
-        <x:v>IH2609</x:v>
-      </x:c>
-      <x:c r="K61" s="22" t="n">
+      <x:c r="C74" s="23" t="n">
+        <x:v>154300</x:v>
+      </x:c>
+      <x:c r="D74" s="23" t="n">
+        <x:v>157000</x:v>
+      </x:c>
+      <x:c r="E74" s="23" t="n">
+        <x:v>148400</x:v>
+      </x:c>
+      <x:c r="F74" s="23" t="n">
+        <x:v>156140</x:v>
+      </x:c>
+      <x:c r="G74" s="28" t="n">
+        <x:f>ROUND(F74-F73,1)</x:f>
+        <x:v>2200</x:v>
+      </x:c>
+      <x:c r="H74" s="24" t="n">
+        <x:f>IFERROR(F74/F73-1,"")</x:f>
+        <x:v>0.014291282317786091</x:v>
+      </x:c>
+      <x:c r="I74" s="26" t="n">
+        <x:f>ROUND(D74-E74,1)</x:f>
+        <x:v>8600</x:v>
+      </x:c>
+      <x:c r="J74" s="22" t="str">
+        <x:v>LC2609</x:v>
+      </x:c>
+      <x:c r="K74" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="62">
-      <x:c r="A62" s="22" t="n">
+    <x:row r="75">
+      <x:c r="A75" s="22" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B62" s="22" t="str">
+      <x:c r="B75" s="22" t="str">
         <x:v>8月24日-8月28日</x:v>
       </x:c>
-      <x:c r="C62" s="23" t="n">
-        <x:v>2856.4</x:v>
-      </x:c>
-      <x:c r="D62" s="23" t="n">
-        <x:v>2918.2</x:v>
-      </x:c>
-      <x:c r="E62" s="23" t="n">
-        <x:v>2837.4</x:v>
-      </x:c>
-      <x:c r="F62" s="23" t="n">
-        <x:v>2911.4</x:v>
-      </x:c>
-      <x:c r="G62" s="23" t="n">
-        <x:f>ROUND(F62-F61,1)</x:f>
-        <x:v>50.4</x:v>
-      </x:c>
-      <x:c r="H62" s="24" t="n">
-        <x:f>IFERROR(F62/F61-1,"")</x:f>
-        <x:v>0.01761621810555747</x:v>
-      </x:c>
-      <x:c r="I62" s="26" t="n">
-        <x:f>ROUND(D62-E62,1)</x:f>
-        <x:v>80.8</x:v>
-      </x:c>
-      <x:c r="J62" s="22" t="str">
-        <x:v>IH2609</x:v>
-      </x:c>
-      <x:c r="K62" s="22" t="n">
+      <x:c r="C75" s="23" t="n">
+        <x:v>158500</x:v>
+      </x:c>
+      <x:c r="D75" s="23" t="n">
+        <x:v>160000</x:v>
+      </x:c>
+      <x:c r="E75" s="23" t="n">
+        <x:v>147000</x:v>
+      </x:c>
+      <x:c r="F75" s="23" t="n">
+        <x:v>157080</x:v>
+      </x:c>
+      <x:c r="G75" s="28" t="n">
+        <x:f>ROUND(F75-F74,1)</x:f>
+        <x:v>940</x:v>
+      </x:c>
+      <x:c r="H75" s="24" t="n">
+        <x:f>IFERROR(F75/F74-1,"")</x:f>
+        <x:v>0.0060202382477263505</x:v>
+      </x:c>
+      <x:c r="I75" s="26" t="n">
+        <x:f>ROUND(D75-E75,1)</x:f>
+        <x:v>13000</x:v>
+      </x:c>
+      <x:c r="J75" s="22" t="str">
+        <x:v>LC2609</x:v>
+      </x:c>
+      <x:c r="K75" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="63">
-      <x:c r="A63" s="31" t="str">
+    <x:row r="76">
+      <x:c r="A76" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B63" s="30" t="n">
+      <x:c r="B76" s="30" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C63" s="30"/>
-      <x:c r="D63" s="30"/>
-      <x:c r="E63" s="30"/>
-      <x:c r="F63" s="30"/>
-      <x:c r="G63" s="30"/>
-      <x:c r="H63" s="30"/>
-      <x:c r="I63" s="32" t="n">
-        <x:f>ROUND(SUM(I59:I62),1)</x:f>
-        <x:v>316.4</x:v>
-      </x:c>
-      <x:c r="J63" s="30"/>
-      <x:c r="K63" s="30"/>
-    </x:row>
-    <x:row r="64">
-      <x:c r="A64" s="31" t="str">
+      <x:c r="C76" s="30"/>
+      <x:c r="D76" s="30"/>
+      <x:c r="E76" s="30"/>
+      <x:c r="F76" s="30"/>
+      <x:c r="G76" s="30"/>
+      <x:c r="H76" s="30"/>
+      <x:c r="I76" s="32" t="n">
+        <x:f>ROUND(SUM(I72:I75),1)</x:f>
+        <x:v>46060</x:v>
+      </x:c>
+      <x:c r="J76" s="30"/>
+      <x:c r="K76" s="30"/>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B64" s="30"/>
-      <x:c r="C64" s="30"/>
-      <x:c r="D64" s="30"/>
-      <x:c r="E64" s="30"/>
-      <x:c r="F64" s="30"/>
-      <x:c r="G64" s="30"/>
-      <x:c r="H64" s="30"/>
-      <x:c r="I64" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I59:I62),0),1)</x:f>
-        <x:v>79.1</x:v>
-      </x:c>
-      <x:c r="J64" s="30"/>
-      <x:c r="K64" s="30"/>
-    </x:row>
-    <x:row r="66">
-      <x:c r="A66" s="17" t="str">
-        <x:v>碳酸锂2609</x:v>
-      </x:c>
-      <x:c r="B66" s="17"/>
-      <x:c r="C66" s="17"/>
-      <x:c r="D66" s="17"/>
-      <x:c r="E66" s="17"/>
-      <x:c r="F66" s="17"/>
-      <x:c r="G66" s="17"/>
-      <x:c r="H66" s="17"/>
-      <x:c r="I66" s="17"/>
-      <x:c r="J66" s="17"/>
-      <x:c r="K66" s="17"/>
-    </x:row>
-    <x:row r="67">
-      <x:c r="A67" s="20" t="str">
-        <x:v>序号</x:v>
-      </x:c>
-      <x:c r="B67" s="20" t="str">
-        <x:v>周期</x:v>
-      </x:c>
-      <x:c r="C67" s="20" t="str">
-        <x:v>开盘</x:v>
-      </x:c>
-      <x:c r="D67" s="20" t="str">
-        <x:v>高点</x:v>
-      </x:c>
-      <x:c r="E67" s="20" t="str">
-        <x:v>低点</x:v>
-      </x:c>
-      <x:c r="F67" s="20" t="str">
-        <x:v>收盘</x:v>
-      </x:c>
-      <x:c r="G67" s="20" t="str">
-        <x:v>涨跌点数</x:v>
-      </x:c>
-      <x:c r="H67" s="20" t="str">
-        <x:v>涨幅</x:v>
-      </x:c>
-      <x:c r="I67" s="20" t="str">
-        <x:v>振幅</x:v>
-      </x:c>
-      <x:c r="J67" s="20" t="str">
-        <x:v>标的</x:v>
-      </x:c>
-      <x:c r="K67" s="20" t="str">
-        <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="68">
-      <x:c r="A68" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B68" s="22" t="str">
-        <x:v>8月3日-8月7日</x:v>
-      </x:c>
-      <x:c r="C68" s="23" t="n">
-        <x:v>137500</x:v>
-      </x:c>
-      <x:c r="D68" s="23" t="n">
-        <x:v>144800</x:v>
-      </x:c>
-      <x:c r="E68" s="23" t="n">
-        <x:v>135560</x:v>
-      </x:c>
-      <x:c r="F68" s="23" t="n">
-        <x:v>140000</x:v>
-      </x:c>
-      <x:c r="G68" s="23"/>
-      <x:c r="H68" s="24"/>
-      <x:c r="I68" s="26" t="n">
-        <x:f>ROUND(D68-E68,1)</x:f>
-        <x:v>9240</x:v>
-      </x:c>
-      <x:c r="J68" s="22" t="str">
-        <x:v>LC2609</x:v>
-      </x:c>
-      <x:c r="K68" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="69">
-      <x:c r="A69" s="22" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B69" s="22" t="str">
-        <x:v>8月10日-8月14日</x:v>
-      </x:c>
-      <x:c r="C69" s="23" t="n">
-        <x:v>140500</x:v>
-      </x:c>
-      <x:c r="D69" s="23" t="n">
-        <x:v>154500</x:v>
-      </x:c>
-      <x:c r="E69" s="23" t="n">
-        <x:v>139280</x:v>
-      </x:c>
-      <x:c r="F69" s="23" t="n">
-        <x:v>153940</x:v>
-      </x:c>
-      <x:c r="G69" s="28" t="n">
-        <x:f>ROUND(F69-F68,1)</x:f>
-        <x:v>13940</x:v>
-      </x:c>
-      <x:c r="H69" s="24" t="n">
-        <x:f>IFERROR(F69/F68-1,"")</x:f>
-        <x:v>0.09957142857142864</x:v>
-      </x:c>
-      <x:c r="I69" s="26" t="n">
-        <x:f>ROUND(D69-E69,1)</x:f>
-        <x:v>15220</x:v>
-      </x:c>
-      <x:c r="J69" s="22" t="str">
-        <x:v>LC2609</x:v>
-      </x:c>
-      <x:c r="K69" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="70">
-      <x:c r="A70" s="22" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B70" s="22" t="str">
-        <x:v>8月17日-8月21日</x:v>
-      </x:c>
-      <x:c r="C70" s="23" t="n">
-        <x:v>154300</x:v>
-      </x:c>
-      <x:c r="D70" s="23" t="n">
-        <x:v>157000</x:v>
-      </x:c>
-      <x:c r="E70" s="23" t="n">
-        <x:v>148400</x:v>
-      </x:c>
-      <x:c r="F70" s="23" t="n">
-        <x:v>156140</x:v>
-      </x:c>
-      <x:c r="G70" s="28" t="n">
-        <x:f>ROUND(F70-F69,1)</x:f>
-        <x:v>2200</x:v>
-      </x:c>
-      <x:c r="H70" s="24" t="n">
-        <x:f>IFERROR(F70/F69-1,"")</x:f>
-        <x:v>0.014291282317786091</x:v>
-      </x:c>
-      <x:c r="I70" s="26" t="n">
-        <x:f>ROUND(D70-E70,1)</x:f>
-        <x:v>8600</x:v>
-      </x:c>
-      <x:c r="J70" s="22" t="str">
-        <x:v>LC2609</x:v>
-      </x:c>
-      <x:c r="K70" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="71">
-      <x:c r="A71" s="22" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B71" s="22" t="str">
-        <x:v>8月24日-8月28日</x:v>
-      </x:c>
-      <x:c r="C71" s="23" t="n">
-        <x:v>158500</x:v>
-      </x:c>
-      <x:c r="D71" s="23" t="n">
-        <x:v>160000</x:v>
-      </x:c>
-      <x:c r="E71" s="23" t="n">
-        <x:v>147000</x:v>
-      </x:c>
-      <x:c r="F71" s="23" t="n">
-        <x:v>157080</x:v>
-      </x:c>
-      <x:c r="G71" s="28" t="n">
-        <x:f>ROUND(F71-F70,1)</x:f>
-        <x:v>940</x:v>
-      </x:c>
-      <x:c r="H71" s="24" t="n">
-        <x:f>IFERROR(F71/F70-1,"")</x:f>
-        <x:v>0.0060202382477263505</x:v>
-      </x:c>
-      <x:c r="I71" s="26" t="n">
-        <x:f>ROUND(D71-E71,1)</x:f>
-        <x:v>13000</x:v>
-      </x:c>
-      <x:c r="J71" s="22" t="str">
-        <x:v>LC2609</x:v>
-      </x:c>
-      <x:c r="K71" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="72">
-      <x:c r="A72" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B72" s="30" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C72" s="30"/>
-      <x:c r="D72" s="30"/>
-      <x:c r="E72" s="30"/>
-      <x:c r="F72" s="30"/>
-      <x:c r="G72" s="30"/>
-      <x:c r="H72" s="30"/>
-      <x:c r="I72" s="32" t="n">
-        <x:f>ROUND(SUM(I68:I71),1)</x:f>
-        <x:v>46060</x:v>
-      </x:c>
-      <x:c r="J72" s="30"/>
-      <x:c r="K72" s="30"/>
-    </x:row>
-    <x:row r="73">
-      <x:c r="A73" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B73" s="30"/>
-      <x:c r="C73" s="30"/>
-      <x:c r="D73" s="30"/>
-      <x:c r="E73" s="30"/>
-      <x:c r="F73" s="30"/>
-      <x:c r="G73" s="30"/>
-      <x:c r="H73" s="30"/>
-      <x:c r="I73" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I68:I71),0),1)</x:f>
+      <x:c r="B77" s="30"/>
+      <x:c r="C77" s="30"/>
+      <x:c r="D77" s="30"/>
+      <x:c r="E77" s="30"/>
+      <x:c r="F77" s="30"/>
+      <x:c r="G77" s="30"/>
+      <x:c r="H77" s="30"/>
+      <x:c r="I77" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I72:I75),0),1)</x:f>
         <x:v>11515</x:v>
       </x:c>
-      <x:c r="J73" s="30"/>
-      <x:c r="K73" s="30"/>
+      <x:c r="J77" s="30"/>
+      <x:c r="K77" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:K1"/>
     <x:mergeCell ref="A3:K3"/>
-    <x:mergeCell ref="A12:K12"/>
-    <x:mergeCell ref="A21:K21"/>
-    <x:mergeCell ref="A30:K30"/>
-    <x:mergeCell ref="A39:K39"/>
-    <x:mergeCell ref="A48:K48"/>
-    <x:mergeCell ref="A57:K57"/>
-    <x:mergeCell ref="A66:K66"/>
+    <x:mergeCell ref="A13:K13"/>
+    <x:mergeCell ref="A23:K23"/>
+    <x:mergeCell ref="A33:K33"/>
+    <x:mergeCell ref="A42:K42"/>
+    <x:mergeCell ref="A51:K51"/>
+    <x:mergeCell ref="A61:K61"/>
+    <x:mergeCell ref="A70:K70"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -4391,31 +4543,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B26" s="30" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="C26" s="30"/>
-      <x:c r="D26" s="30"/>
-      <x:c r="E26" s="30"/>
-      <x:c r="F26" s="30"/>
-      <x:c r="G26" s="30"/>
-      <x:c r="H26" s="30"/>
-      <x:c r="I26" s="30"/>
-      <x:c r="J26" s="32" t="n">
-        <x:f>SUM(J4:J23)</x:f>
-        <x:v>3448.3</x:v>
-      </x:c>
-      <x:c r="K26" s="30"/>
+    <x:row r="24">
+      <x:c r="A24" s="22" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B24" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C24" s="22" t="str">
+        <x:v>8月31日</x:v>
+      </x:c>
+      <x:c r="D24" s="23" t="n">
+        <x:v>7607.23</x:v>
+      </x:c>
+      <x:c r="E24" s="23" t="n">
+        <x:v>7771.55</x:v>
+      </x:c>
+      <x:c r="F24" s="23" t="n">
+        <x:v>7604.95</x:v>
+      </x:c>
+      <x:c r="G24" s="23" t="n">
+        <x:v>7770.42</x:v>
+      </x:c>
+      <x:c r="H24" s="23" t="n">
+        <x:v>65.4</x:v>
+      </x:c>
+      <x:c r="I24" s="24" t="n">
+        <x:v>0.00848666390656505</x:v>
+      </x:c>
+      <x:c r="J24" s="23" t="n">
+        <x:f>ROUND(E24-F24,1)</x:f>
+        <x:v>166.6</x:v>
+      </x:c>
+      <x:c r="K24" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B27" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B27" s="30" t="n">
+        <x:v>21</x:v>
+      </x:c>
       <x:c r="C27" s="30"/>
       <x:c r="D27" s="30"/>
       <x:c r="E27" s="30"/>
@@ -4423,11 +4593,29 @@
       <x:c r="G27" s="30"/>
       <x:c r="H27" s="30"/>
       <x:c r="I27" s="30"/>
-      <x:c r="J27" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J23),0),1)</x:f>
-        <x:v>172.4</x:v>
+      <x:c r="J27" s="32" t="n">
+        <x:f>SUM(J4:J24)</x:f>
+        <x:v>3614.9</x:v>
       </x:c>
       <x:c r="K27" s="30"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B28" s="30"/>
+      <x:c r="C28" s="30"/>
+      <x:c r="D28" s="30"/>
+      <x:c r="E28" s="30"/>
+      <x:c r="F28" s="30"/>
+      <x:c r="G28" s="30"/>
+      <x:c r="H28" s="30"/>
+      <x:c r="I28" s="30"/>
+      <x:c r="J28" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J24),0),1)</x:f>
+        <x:v>172.1</x:v>
+      </x:c>
+      <x:c r="K28" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5214,31 +5402,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B26" s="30" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="C26" s="30"/>
-      <x:c r="D26" s="30"/>
-      <x:c r="E26" s="30"/>
-      <x:c r="F26" s="30"/>
-      <x:c r="G26" s="30"/>
-      <x:c r="H26" s="30"/>
-      <x:c r="I26" s="30"/>
-      <x:c r="J26" s="32" t="n">
-        <x:f>SUM(J4:J23)</x:f>
-        <x:v>3298.7</x:v>
-      </x:c>
-      <x:c r="K26" s="30"/>
+    <x:row r="24">
+      <x:c r="A24" s="22" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B24" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C24" s="22" t="str">
+        <x:v>8月31日</x:v>
+      </x:c>
+      <x:c r="D24" s="23" t="n">
+        <x:v>7797.23</x:v>
+      </x:c>
+      <x:c r="E24" s="23" t="n">
+        <x:v>7953.93</x:v>
+      </x:c>
+      <x:c r="F24" s="23" t="n">
+        <x:v>7764.98</x:v>
+      </x:c>
+      <x:c r="G24" s="23" t="n">
+        <x:v>7952.1</x:v>
+      </x:c>
+      <x:c r="H24" s="23" t="n">
+        <x:v>56.7</x:v>
+      </x:c>
+      <x:c r="I24" s="24" t="n">
+        <x:v>0.007175018523326804</x:v>
+      </x:c>
+      <x:c r="J24" s="26" t="n">
+        <x:f>ROUND(E24-F24,1)</x:f>
+        <x:v>189</x:v>
+      </x:c>
+      <x:c r="K24" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B27" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B27" s="30" t="n">
+        <x:v>21</x:v>
+      </x:c>
       <x:c r="C27" s="30"/>
       <x:c r="D27" s="30"/>
       <x:c r="E27" s="30"/>
@@ -5246,11 +5452,29 @@
       <x:c r="G27" s="30"/>
       <x:c r="H27" s="30"/>
       <x:c r="I27" s="30"/>
-      <x:c r="J27" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J23),0),1)</x:f>
-        <x:v>164.9</x:v>
+      <x:c r="J27" s="32" t="n">
+        <x:f>SUM(J4:J24)</x:f>
+        <x:v>3487.7</x:v>
       </x:c>
       <x:c r="K27" s="30"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B28" s="30"/>
+      <x:c r="C28" s="30"/>
+      <x:c r="D28" s="30"/>
+      <x:c r="E28" s="30"/>
+      <x:c r="F28" s="30"/>
+      <x:c r="G28" s="30"/>
+      <x:c r="H28" s="30"/>
+      <x:c r="I28" s="30"/>
+      <x:c r="J28" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J24),0),1)</x:f>
+        <x:v>166.1</x:v>
+      </x:c>
+      <x:c r="K28" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -6037,31 +6261,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B26" s="30" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="C26" s="30"/>
-      <x:c r="D26" s="30"/>
-      <x:c r="E26" s="30"/>
-      <x:c r="F26" s="30"/>
-      <x:c r="G26" s="30"/>
-      <x:c r="H26" s="30"/>
-      <x:c r="I26" s="30"/>
-      <x:c r="J26" s="32" t="n">
-        <x:f>SUM(J4:J23)</x:f>
-        <x:v>846</x:v>
-      </x:c>
-      <x:c r="K26" s="30"/>
+    <x:row r="24">
+      <x:c r="A24" s="22" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B24" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C24" s="22" t="str">
+        <x:v>8月31日</x:v>
+      </x:c>
+      <x:c r="D24" s="23" t="n">
+        <x:v>3926.53</x:v>
+      </x:c>
+      <x:c r="E24" s="23" t="n">
+        <x:v>3986.3</x:v>
+      </x:c>
+      <x:c r="F24" s="23" t="n">
+        <x:v>3926.5</x:v>
+      </x:c>
+      <x:c r="G24" s="23" t="n">
+        <x:v>3986.3</x:v>
+      </x:c>
+      <x:c r="H24" s="23" t="n">
+        <x:v>34.1</x:v>
+      </x:c>
+      <x:c r="I24" s="24" t="n">
+        <x:v>0.008633210025859261</x:v>
+      </x:c>
+      <x:c r="J24" s="26" t="n">
+        <x:f>ROUND(E24-F24,1)</x:f>
+        <x:v>59.8</x:v>
+      </x:c>
+      <x:c r="K24" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B27" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B27" s="30" t="n">
+        <x:v>21</x:v>
+      </x:c>
       <x:c r="C27" s="30"/>
       <x:c r="D27" s="30"/>
       <x:c r="E27" s="30"/>
@@ -6069,11 +6311,29 @@
       <x:c r="G27" s="30"/>
       <x:c r="H27" s="30"/>
       <x:c r="I27" s="30"/>
-      <x:c r="J27" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J23),0),1)</x:f>
-        <x:v>42.3</x:v>
+      <x:c r="J27" s="32" t="n">
+        <x:f>SUM(J4:J24)</x:f>
+        <x:v>905.8</x:v>
       </x:c>
       <x:c r="K27" s="30"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B28" s="30"/>
+      <x:c r="C28" s="30"/>
+      <x:c r="D28" s="30"/>
+      <x:c r="E28" s="30"/>
+      <x:c r="F28" s="30"/>
+      <x:c r="G28" s="30"/>
+      <x:c r="H28" s="30"/>
+      <x:c r="I28" s="30"/>
+      <x:c r="J28" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J24),0),1)</x:f>
+        <x:v>43.1</x:v>
+      </x:c>
+      <x:c r="K28" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -8506,31 +8766,49 @@
         <x:v>IF2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B26" s="30" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="C26" s="30"/>
-      <x:c r="D26" s="30"/>
-      <x:c r="E26" s="30"/>
-      <x:c r="F26" s="30"/>
-      <x:c r="G26" s="30"/>
-      <x:c r="H26" s="30"/>
-      <x:c r="I26" s="30"/>
-      <x:c r="J26" s="32" t="n">
-        <x:f>SUM(J4:J23)</x:f>
-        <x:v>1248.4</x:v>
-      </x:c>
-      <x:c r="K26" s="30"/>
+    <x:row r="24">
+      <x:c r="A24" s="22" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B24" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C24" s="22" t="str">
+        <x:v>8月31日</x:v>
+      </x:c>
+      <x:c r="D24" s="23" t="n">
+        <x:v>4553</x:v>
+      </x:c>
+      <x:c r="E24" s="23" t="n">
+        <x:v>4608.6</x:v>
+      </x:c>
+      <x:c r="F24" s="23" t="n">
+        <x:v>4530</x:v>
+      </x:c>
+      <x:c r="G24" s="23" t="n">
+        <x:v>4601.6</x:v>
+      </x:c>
+      <x:c r="H24" s="23" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="I24" s="24" t="n">
+        <x:v>0.0017415534656914922</x:v>
+      </x:c>
+      <x:c r="J24" s="23" t="n">
+        <x:f>ROUND(E24-F24,1)</x:f>
+        <x:v>78.6</x:v>
+      </x:c>
+      <x:c r="K24" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B27" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B27" s="30" t="n">
+        <x:v>21</x:v>
+      </x:c>
       <x:c r="C27" s="30"/>
       <x:c r="D27" s="30"/>
       <x:c r="E27" s="30"/>
@@ -8538,11 +8816,29 @@
       <x:c r="G27" s="30"/>
       <x:c r="H27" s="30"/>
       <x:c r="I27" s="30"/>
-      <x:c r="J27" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J23),0),1)</x:f>
-        <x:v>62.4</x:v>
+      <x:c r="J27" s="32" t="n">
+        <x:f>SUM(J4:J24)</x:f>
+        <x:v>1327</x:v>
       </x:c>
       <x:c r="K27" s="30"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B28" s="30"/>
+      <x:c r="C28" s="30"/>
+      <x:c r="D28" s="30"/>
+      <x:c r="E28" s="30"/>
+      <x:c r="F28" s="30"/>
+      <x:c r="G28" s="30"/>
+      <x:c r="H28" s="30"/>
+      <x:c r="I28" s="30"/>
+      <x:c r="J28" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J24),0),1)</x:f>
+        <x:v>63.2</x:v>
+      </x:c>
+      <x:c r="K28" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-09-01
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R47edc68742394aee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Rf32c71ef07794850"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R79d6b50b705546ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R96a191c295004ad1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R2e6198bcc83b45e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rc502c0d84fd6458b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R1e9e0a14e3a3462f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rd46f81aedf264378"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rc2d7a8b35e434d3f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R28948b218c894d2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Ra60f897f76bf48d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R04ee92ae0eb141af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Re3f116e14b6940a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R17e16424038a41b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Re66d73e6db794bb8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R9c565b84cf944385"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Ra150f2e93ad44d8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rb40efbf6b1494709"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rb558ff3e29ec4833"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R705c2c2a237f44be"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -26,7 +26,7 @@
     <x:numFmt numFmtId="200" formatCode="General"/>
     <x:numFmt numFmtId="201" formatCode="0.0%"/>
   </x:numFmts>
-  <x:fonts count="8">
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -71,8 +71,14 @@
       <x:color rgb="FFE11D48"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF1D4ED8"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -97,6 +103,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFFF00"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFBFDBFE"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -134,7 +145,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="36">
+  <x:cellXfs count="37">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -200,9 +211,6 @@
     <x:xf numFmtId="200" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
@@ -213,6 +221,12 @@
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="8" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -580,17 +594,27 @@
       <x:c r="A8" s="9" t="str">
         <x:v>IC主力</x:v>
       </x:c>
-      <x:c r="B8" s="9" t="str"/>
-      <x:c r="C8" s="10" t="str"/>
-      <x:c r="D8" s="10" t="str"/>
-      <x:c r="E8" s="12" t="str"/>
+      <x:c r="B8" s="9" t="str">
+        <x:v>2026-09-01</x:v>
+      </x:c>
+      <x:c r="C8" s="10" t="n">
+        <x:v>7903</x:v>
+      </x:c>
+      <x:c r="D8" s="10" t="n">
+        <x:v>7765</x:v>
+      </x:c>
+      <x:c r="E8" s="12" t="n">
+        <x:v>138</x:v>
+      </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H8" s="10" t="str"/>
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="H8" s="10" t="n">
+        <x:v>138</x:v>
+      </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
       </x:c>
@@ -599,17 +623,27 @@
       <x:c r="A9" s="9" t="str">
         <x:v>IF主力</x:v>
       </x:c>
-      <x:c r="B9" s="9" t="str"/>
-      <x:c r="C9" s="10" t="str"/>
-      <x:c r="D9" s="10" t="str"/>
-      <x:c r="E9" s="12" t="str"/>
+      <x:c r="B9" s="9" t="str">
+        <x:v>2026-09-01</x:v>
+      </x:c>
+      <x:c r="C9" s="10" t="n">
+        <x:v>4617.8</x:v>
+      </x:c>
+      <x:c r="D9" s="10" t="n">
+        <x:v>4576</x:v>
+      </x:c>
+      <x:c r="E9" s="12" t="n">
+        <x:v>41.8</x:v>
+      </x:c>
       <x:c r="F9" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G9" s="10" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H9" s="10" t="str"/>
+        <x:v>41.8</x:v>
+      </x:c>
+      <x:c r="H9" s="10" t="n">
+        <x:v>41.8</x:v>
+      </x:c>
       <x:c r="I9" s="10" t="n">
         <x:v>90</x:v>
       </x:c>
@@ -647,17 +681,27 @@
       <x:c r="A11" s="9" t="str">
         <x:v>碳酸锂2609</x:v>
       </x:c>
-      <x:c r="B11" s="9" t="str"/>
-      <x:c r="C11" s="10" t="str"/>
-      <x:c r="D11" s="10" t="str"/>
-      <x:c r="E11" s="12" t="str"/>
+      <x:c r="B11" s="9" t="str">
+        <x:v>2026-09-01</x:v>
+      </x:c>
+      <x:c r="C11" s="10" t="n">
+        <x:v>160480</x:v>
+      </x:c>
+      <x:c r="D11" s="10" t="n">
+        <x:v>155800</x:v>
+      </x:c>
+      <x:c r="E11" s="12" t="n">
+        <x:v>4680</x:v>
+      </x:c>
       <x:c r="F11" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G11" s="10" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H11" s="10" t="str"/>
+        <x:v>4680</x:v>
+      </x:c>
+      <x:c r="H11" s="10" t="n">
+        <x:v>4680</x:v>
+      </x:c>
       <x:c r="I11" s="10" t="n">
         <x:v>6000</x:v>
       </x:c>
@@ -854,24 +898,47 @@
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="22"/>
-      <x:c r="B4" s="22"/>
-      <x:c r="C4" s="22"/>
-      <x:c r="D4" s="23"/>
-      <x:c r="E4" s="23"/>
-      <x:c r="F4" s="23"/>
-      <x:c r="G4" s="23"/>
-      <x:c r="H4" s="23"/>
-      <x:c r="I4" s="24"/>
-      <x:c r="J4" s="23"/>
-      <x:c r="K4" s="22"/>
+      <x:c r="A4" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B4" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C4" s="22" t="str">
+        <x:v>9月1日</x:v>
+      </x:c>
+      <x:c r="D4" s="23" t="n">
+        <x:v>159000</x:v>
+      </x:c>
+      <x:c r="E4" s="23" t="n">
+        <x:v>160480</x:v>
+      </x:c>
+      <x:c r="F4" s="23" t="n">
+        <x:v>155800</x:v>
+      </x:c>
+      <x:c r="G4" s="23" t="n">
+        <x:v>155820</x:v>
+      </x:c>
+      <x:c r="H4" s="36" t="n">
+        <x:v>-3180</x:v>
+      </x:c>
+      <x:c r="I4" s="24" t="n">
+        <x:v>-0.020000000000000018</x:v>
+      </x:c>
+      <x:c r="J4" s="23" t="n">
+        <x:f>ROUND(E4-F4,1)</x:f>
+        <x:v>4680</x:v>
+      </x:c>
+      <x:c r="K4" s="22" t="str">
+        <x:v>LC2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="27" t="str">
         <x:v>合计</x:v>
       </x:c>
       <x:c r="B7" s="26" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C7" s="26"/>
       <x:c r="D7" s="26"/>
@@ -882,7 +949,7 @@
       <x:c r="I7" s="26"/>
       <x:c r="J7" s="28" t="n">
         <x:f>SUM(J4:J4)</x:f>
-        <x:v>0</x:v>
+        <x:v>4680</x:v>
       </x:c>
       <x:c r="K7" s="26"/>
     </x:row>
@@ -900,7 +967,7 @@
       <x:c r="I8" s="26"/>
       <x:c r="J8" s="30" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J4),0),1)</x:f>
-        <x:v>0</x:v>
+        <x:v>4680</x:v>
       </x:c>
       <x:c r="K8" s="26"/>
     </x:row>
@@ -1465,269 +1532,434 @@
       </x:c>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="31" t="str">
-        <x:v>暂无数据</x:v>
-      </x:c>
-      <x:c r="B29" s="31"/>
-      <x:c r="C29" s="31"/>
-      <x:c r="D29" s="31"/>
-      <x:c r="E29" s="31"/>
-      <x:c r="F29" s="31"/>
-      <x:c r="G29" s="31"/>
-      <x:c r="H29" s="31"/>
-      <x:c r="I29" s="31"/>
-      <x:c r="J29" s="31"/>
-      <x:c r="K29" s="31"/>
+      <x:c r="A29" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B29" s="22" t="str">
+        <x:v>9月1日</x:v>
+      </x:c>
+      <x:c r="C29" s="23" t="n">
+        <x:v>7880.8</x:v>
+      </x:c>
+      <x:c r="D29" s="23" t="n">
+        <x:v>7903</x:v>
+      </x:c>
+      <x:c r="E29" s="23" t="n">
+        <x:v>7765</x:v>
+      </x:c>
+      <x:c r="F29" s="23" t="n">
+        <x:v>7801.6</x:v>
+      </x:c>
+      <x:c r="G29" s="23"/>
+      <x:c r="H29" s="24"/>
+      <x:c r="I29" s="23" t="n">
+        <x:f>ROUND(D29-E29,1)</x:f>
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="J29" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+      <x:c r="K29" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="27" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B30" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C30" s="26"/>
+      <x:c r="D30" s="26"/>
+      <x:c r="E30" s="26"/>
+      <x:c r="F30" s="26"/>
+      <x:c r="G30" s="26"/>
+      <x:c r="H30" s="26"/>
+      <x:c r="I30" s="28" t="n">
+        <x:f>ROUND(SUM(I29:I29),1)</x:f>
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="J30" s="26"/>
+      <x:c r="K30" s="26"/>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="17" t="str">
+      <x:c r="A31" s="27" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B31" s="26"/>
+      <x:c r="C31" s="26"/>
+      <x:c r="D31" s="26"/>
+      <x:c r="E31" s="26"/>
+      <x:c r="F31" s="26"/>
+      <x:c r="G31" s="26"/>
+      <x:c r="H31" s="26"/>
+      <x:c r="I31" s="30" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I29:I29),0),1)</x:f>
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="J31" s="26"/>
+      <x:c r="K31" s="26"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="17" t="str">
         <x:v>IF主力</x:v>
       </x:c>
-      <x:c r="B31" s="17"/>
-      <x:c r="C31" s="17"/>
-      <x:c r="D31" s="17"/>
-      <x:c r="E31" s="17"/>
-      <x:c r="F31" s="17"/>
-      <x:c r="G31" s="17"/>
-      <x:c r="H31" s="17"/>
-      <x:c r="I31" s="17"/>
-      <x:c r="J31" s="17"/>
-      <x:c r="K31" s="17"/>
-    </x:row>
-    <x:row r="32">
-      <x:c r="A32" s="20" t="str">
+      <x:c r="B33" s="17"/>
+      <x:c r="C33" s="17"/>
+      <x:c r="D33" s="17"/>
+      <x:c r="E33" s="17"/>
+      <x:c r="F33" s="17"/>
+      <x:c r="G33" s="17"/>
+      <x:c r="H33" s="17"/>
+      <x:c r="I33" s="17"/>
+      <x:c r="J33" s="17"/>
+      <x:c r="K33" s="17"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B32" s="20" t="str">
+      <x:c r="B34" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C32" s="20" t="str">
+      <x:c r="C34" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D32" s="20" t="str">
+      <x:c r="D34" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E32" s="20" t="str">
+      <x:c r="E34" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F32" s="20" t="str">
+      <x:c r="F34" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G32" s="20" t="str">
+      <x:c r="G34" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H32" s="20" t="str">
+      <x:c r="H34" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I32" s="20" t="str">
+      <x:c r="I34" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J32" s="20" t="str">
+      <x:c r="J34" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K32" s="20" t="str">
+      <x:c r="K34" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="33">
-      <x:c r="A33" s="31" t="str">
-        <x:v>暂无数据</x:v>
-      </x:c>
-      <x:c r="B33" s="31"/>
-      <x:c r="C33" s="31"/>
-      <x:c r="D33" s="31"/>
-      <x:c r="E33" s="31"/>
-      <x:c r="F33" s="31"/>
-      <x:c r="G33" s="31"/>
-      <x:c r="H33" s="31"/>
-      <x:c r="I33" s="31"/>
-      <x:c r="J33" s="31"/>
-      <x:c r="K33" s="31"/>
-    </x:row>
     <x:row r="35">
-      <x:c r="A35" s="17" t="str">
+      <x:c r="A35" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B35" s="22" t="str">
+        <x:v>9月1日</x:v>
+      </x:c>
+      <x:c r="C35" s="23" t="n">
+        <x:v>4602</x:v>
+      </x:c>
+      <x:c r="D35" s="23" t="n">
+        <x:v>4617.8</x:v>
+      </x:c>
+      <x:c r="E35" s="23" t="n">
+        <x:v>4576</x:v>
+      </x:c>
+      <x:c r="F35" s="23" t="n">
+        <x:v>4597.2</x:v>
+      </x:c>
+      <x:c r="G35" s="23"/>
+      <x:c r="H35" s="24"/>
+      <x:c r="I35" s="23" t="n">
+        <x:f>ROUND(D35-E35,1)</x:f>
+        <x:v>41.8</x:v>
+      </x:c>
+      <x:c r="J35" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+      <x:c r="K35" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="27" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B36" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C36" s="26"/>
+      <x:c r="D36" s="26"/>
+      <x:c r="E36" s="26"/>
+      <x:c r="F36" s="26"/>
+      <x:c r="G36" s="26"/>
+      <x:c r="H36" s="26"/>
+      <x:c r="I36" s="28" t="n">
+        <x:f>ROUND(SUM(I35:I35),1)</x:f>
+        <x:v>41.8</x:v>
+      </x:c>
+      <x:c r="J36" s="26"/>
+      <x:c r="K36" s="26"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="27" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B37" s="26"/>
+      <x:c r="C37" s="26"/>
+      <x:c r="D37" s="26"/>
+      <x:c r="E37" s="26"/>
+      <x:c r="F37" s="26"/>
+      <x:c r="G37" s="26"/>
+      <x:c r="H37" s="26"/>
+      <x:c r="I37" s="30" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I35:I35),0),1)</x:f>
+        <x:v>41.8</x:v>
+      </x:c>
+      <x:c r="J37" s="26"/>
+      <x:c r="K37" s="26"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="17" t="str">
         <x:v>IH主力</x:v>
       </x:c>
-      <x:c r="B35" s="17"/>
-      <x:c r="C35" s="17"/>
-      <x:c r="D35" s="17"/>
-      <x:c r="E35" s="17"/>
-      <x:c r="F35" s="17"/>
-      <x:c r="G35" s="17"/>
-      <x:c r="H35" s="17"/>
-      <x:c r="I35" s="17"/>
-      <x:c r="J35" s="17"/>
-      <x:c r="K35" s="17"/>
-    </x:row>
-    <x:row r="36">
-      <x:c r="A36" s="20" t="str">
+      <x:c r="B39" s="17"/>
+      <x:c r="C39" s="17"/>
+      <x:c r="D39" s="17"/>
+      <x:c r="E39" s="17"/>
+      <x:c r="F39" s="17"/>
+      <x:c r="G39" s="17"/>
+      <x:c r="H39" s="17"/>
+      <x:c r="I39" s="17"/>
+      <x:c r="J39" s="17"/>
+      <x:c r="K39" s="17"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B36" s="20" t="str">
+      <x:c r="B40" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C36" s="20" t="str">
+      <x:c r="C40" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D36" s="20" t="str">
+      <x:c r="D40" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E36" s="20" t="str">
+      <x:c r="E40" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F36" s="20" t="str">
+      <x:c r="F40" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G36" s="20" t="str">
+      <x:c r="G40" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H36" s="20" t="str">
+      <x:c r="H40" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I36" s="20" t="str">
+      <x:c r="I40" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J36" s="20" t="str">
+      <x:c r="J40" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K36" s="20" t="str">
+      <x:c r="K40" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="37">
-      <x:c r="A37" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B37" s="22" t="str">
+    <x:row r="41">
+      <x:c r="A41" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B41" s="22" t="str">
         <x:v>9月1日</x:v>
       </x:c>
-      <x:c r="C37" s="23" t="n">
+      <x:c r="C41" s="23" t="n">
         <x:v>2913</x:v>
       </x:c>
-      <x:c r="D37" s="23" t="n">
+      <x:c r="D41" s="23" t="n">
         <x:v>2934.8</x:v>
       </x:c>
-      <x:c r="E37" s="23" t="n">
+      <x:c r="E41" s="23" t="n">
         <x:v>2912</x:v>
       </x:c>
-      <x:c r="F37" s="23" t="n">
+      <x:c r="F41" s="23" t="n">
         <x:v>2928.6</x:v>
       </x:c>
-      <x:c r="G37" s="23"/>
-      <x:c r="H37" s="24"/>
-      <x:c r="I37" s="23" t="n">
-        <x:f>ROUND(D37-E37,1)</x:f>
+      <x:c r="G41" s="23"/>
+      <x:c r="H41" s="24"/>
+      <x:c r="I41" s="23" t="n">
+        <x:f>ROUND(D41-E41,1)</x:f>
         <x:v>22.8</x:v>
       </x:c>
-      <x:c r="J37" s="22" t="str">
+      <x:c r="J41" s="22" t="str">
         <x:v>IH2609</x:v>
       </x:c>
-      <x:c r="K37" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38">
-      <x:c r="A38" s="27" t="str">
+      <x:c r="K41" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="27" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B38" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C38" s="26"/>
-      <x:c r="D38" s="26"/>
-      <x:c r="E38" s="26"/>
-      <x:c r="F38" s="26"/>
-      <x:c r="G38" s="26"/>
-      <x:c r="H38" s="26"/>
-      <x:c r="I38" s="28" t="n">
-        <x:f>ROUND(SUM(I37:I37),1)</x:f>
+      <x:c r="B42" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C42" s="26"/>
+      <x:c r="D42" s="26"/>
+      <x:c r="E42" s="26"/>
+      <x:c r="F42" s="26"/>
+      <x:c r="G42" s="26"/>
+      <x:c r="H42" s="26"/>
+      <x:c r="I42" s="28" t="n">
+        <x:f>ROUND(SUM(I41:I41),1)</x:f>
         <x:v>22.8</x:v>
       </x:c>
-      <x:c r="J38" s="26"/>
-      <x:c r="K38" s="26"/>
-    </x:row>
-    <x:row r="39">
-      <x:c r="A39" s="27" t="str">
+      <x:c r="J42" s="26"/>
+      <x:c r="K42" s="26"/>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="27" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B39" s="26"/>
-      <x:c r="C39" s="26"/>
-      <x:c r="D39" s="26"/>
-      <x:c r="E39" s="26"/>
-      <x:c r="F39" s="26"/>
-      <x:c r="G39" s="26"/>
-      <x:c r="H39" s="26"/>
-      <x:c r="I39" s="30" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I37:I37),0),1)</x:f>
+      <x:c r="B43" s="26"/>
+      <x:c r="C43" s="26"/>
+      <x:c r="D43" s="26"/>
+      <x:c r="E43" s="26"/>
+      <x:c r="F43" s="26"/>
+      <x:c r="G43" s="26"/>
+      <x:c r="H43" s="26"/>
+      <x:c r="I43" s="30" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I41:I41),0),1)</x:f>
         <x:v>22.8</x:v>
       </x:c>
-      <x:c r="J39" s="26"/>
-      <x:c r="K39" s="26"/>
-    </x:row>
-    <x:row r="41">
-      <x:c r="A41" s="17" t="str">
+      <x:c r="J43" s="26"/>
+      <x:c r="K43" s="26"/>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="17" t="str">
         <x:v>碳酸锂2609</x:v>
       </x:c>
-      <x:c r="B41" s="17"/>
-      <x:c r="C41" s="17"/>
-      <x:c r="D41" s="17"/>
-      <x:c r="E41" s="17"/>
-      <x:c r="F41" s="17"/>
-      <x:c r="G41" s="17"/>
-      <x:c r="H41" s="17"/>
-      <x:c r="I41" s="17"/>
-      <x:c r="J41" s="17"/>
-      <x:c r="K41" s="17"/>
-    </x:row>
-    <x:row r="42">
-      <x:c r="A42" s="20" t="str">
+      <x:c r="B45" s="17"/>
+      <x:c r="C45" s="17"/>
+      <x:c r="D45" s="17"/>
+      <x:c r="E45" s="17"/>
+      <x:c r="F45" s="17"/>
+      <x:c r="G45" s="17"/>
+      <x:c r="H45" s="17"/>
+      <x:c r="I45" s="17"/>
+      <x:c r="J45" s="17"/>
+      <x:c r="K45" s="17"/>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B42" s="20" t="str">
+      <x:c r="B46" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C42" s="20" t="str">
+      <x:c r="C46" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D42" s="20" t="str">
+      <x:c r="D46" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E42" s="20" t="str">
+      <x:c r="E46" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F42" s="20" t="str">
+      <x:c r="F46" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G42" s="20" t="str">
+      <x:c r="G46" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H42" s="20" t="str">
+      <x:c r="H46" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I42" s="20" t="str">
+      <x:c r="I46" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J42" s="20" t="str">
+      <x:c r="J46" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K42" s="20" t="str">
+      <x:c r="K46" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="43">
-      <x:c r="A43" s="31" t="str">
-        <x:v>暂无数据</x:v>
-      </x:c>
-      <x:c r="B43" s="31"/>
-      <x:c r="C43" s="31"/>
-      <x:c r="D43" s="31"/>
-      <x:c r="E43" s="31"/>
-      <x:c r="F43" s="31"/>
-      <x:c r="G43" s="31"/>
-      <x:c r="H43" s="31"/>
-      <x:c r="I43" s="31"/>
-      <x:c r="J43" s="31"/>
-      <x:c r="K43" s="31"/>
+    <x:row r="47">
+      <x:c r="A47" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B47" s="22" t="str">
+        <x:v>9月1日</x:v>
+      </x:c>
+      <x:c r="C47" s="23" t="n">
+        <x:v>159000</x:v>
+      </x:c>
+      <x:c r="D47" s="23" t="n">
+        <x:v>160480</x:v>
+      </x:c>
+      <x:c r="E47" s="23" t="n">
+        <x:v>155800</x:v>
+      </x:c>
+      <x:c r="F47" s="23" t="n">
+        <x:v>155820</x:v>
+      </x:c>
+      <x:c r="G47" s="23"/>
+      <x:c r="H47" s="24"/>
+      <x:c r="I47" s="23" t="n">
+        <x:f>ROUND(D47-E47,1)</x:f>
+        <x:v>4680</x:v>
+      </x:c>
+      <x:c r="J47" s="22" t="str">
+        <x:v>LC2609</x:v>
+      </x:c>
+      <x:c r="K47" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="27" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B48" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C48" s="26"/>
+      <x:c r="D48" s="26"/>
+      <x:c r="E48" s="26"/>
+      <x:c r="F48" s="26"/>
+      <x:c r="G48" s="26"/>
+      <x:c r="H48" s="26"/>
+      <x:c r="I48" s="28" t="n">
+        <x:f>ROUND(SUM(I47:I47),1)</x:f>
+        <x:v>4680</x:v>
+      </x:c>
+      <x:c r="J48" s="26"/>
+      <x:c r="K48" s="26"/>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="27" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B49" s="26"/>
+      <x:c r="C49" s="26"/>
+      <x:c r="D49" s="26"/>
+      <x:c r="E49" s="26"/>
+      <x:c r="F49" s="26"/>
+      <x:c r="G49" s="26"/>
+      <x:c r="H49" s="26"/>
+      <x:c r="I49" s="30" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I47:I47),0),1)</x:f>
+        <x:v>4680</x:v>
+      </x:c>
+      <x:c r="J49" s="26"/>
+      <x:c r="K49" s="26"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1737,12 +1969,9 @@
     <x:mergeCell ref="A15:K15"/>
     <x:mergeCell ref="A21:K21"/>
     <x:mergeCell ref="A27:K27"/>
-    <x:mergeCell ref="A29:K29"/>
-    <x:mergeCell ref="A31:K31"/>
     <x:mergeCell ref="A33:K33"/>
-    <x:mergeCell ref="A35:K35"/>
-    <x:mergeCell ref="A41:K41"/>
-    <x:mergeCell ref="A43:K43"/>
+    <x:mergeCell ref="A39:K39"/>
+    <x:mergeCell ref="A45:K45"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2362,24 +2591,47 @@
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="22"/>
-      <x:c r="B4" s="22"/>
-      <x:c r="C4" s="22"/>
-      <x:c r="D4" s="23"/>
-      <x:c r="E4" s="23"/>
-      <x:c r="F4" s="23"/>
-      <x:c r="G4" s="23"/>
-      <x:c r="H4" s="23"/>
-      <x:c r="I4" s="24"/>
-      <x:c r="J4" s="23"/>
-      <x:c r="K4" s="22"/>
+      <x:c r="A4" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B4" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C4" s="22" t="str">
+        <x:v>9月1日</x:v>
+      </x:c>
+      <x:c r="D4" s="23" t="n">
+        <x:v>7880.8</x:v>
+      </x:c>
+      <x:c r="E4" s="23" t="n">
+        <x:v>7903</x:v>
+      </x:c>
+      <x:c r="F4" s="23" t="n">
+        <x:v>7765</x:v>
+      </x:c>
+      <x:c r="G4" s="23" t="n">
+        <x:v>7801.6</x:v>
+      </x:c>
+      <x:c r="H4" s="23" t="n">
+        <x:v>-94.2</x:v>
+      </x:c>
+      <x:c r="I4" s="24" t="n">
+        <x:v>-0.011930393373692283</x:v>
+      </x:c>
+      <x:c r="J4" s="23" t="n">
+        <x:f>ROUND(E4-F4,1)</x:f>
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="K4" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="27" t="str">
         <x:v>合计</x:v>
       </x:c>
       <x:c r="B7" s="26" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C7" s="26"/>
       <x:c r="D7" s="26"/>
@@ -2390,7 +2642,7 @@
       <x:c r="I7" s="26"/>
       <x:c r="J7" s="28" t="n">
         <x:f>SUM(J4:J4)</x:f>
-        <x:v>0</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="K7" s="26"/>
     </x:row>
@@ -2408,7 +2660,7 @@
       <x:c r="I8" s="26"/>
       <x:c r="J8" s="30" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J4),0),1)</x:f>
-        <x:v>0</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="K8" s="26"/>
     </x:row>
@@ -2478,24 +2730,47 @@
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="22"/>
-      <x:c r="B4" s="22"/>
-      <x:c r="C4" s="22"/>
-      <x:c r="D4" s="23"/>
-      <x:c r="E4" s="23"/>
-      <x:c r="F4" s="23"/>
-      <x:c r="G4" s="23"/>
-      <x:c r="H4" s="23"/>
-      <x:c r="I4" s="24"/>
-      <x:c r="J4" s="23"/>
-      <x:c r="K4" s="22"/>
+      <x:c r="A4" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B4" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C4" s="22" t="str">
+        <x:v>9月1日</x:v>
+      </x:c>
+      <x:c r="D4" s="23" t="n">
+        <x:v>4602</x:v>
+      </x:c>
+      <x:c r="E4" s="23" t="n">
+        <x:v>4617.8</x:v>
+      </x:c>
+      <x:c r="F4" s="23" t="n">
+        <x:v>4576</x:v>
+      </x:c>
+      <x:c r="G4" s="23" t="n">
+        <x:v>4597.2</x:v>
+      </x:c>
+      <x:c r="H4" s="23" t="n">
+        <x:v>-4.4</x:v>
+      </x:c>
+      <x:c r="I4" s="24" t="n">
+        <x:v>-0.0009561891515995624</x:v>
+      </x:c>
+      <x:c r="J4" s="23" t="n">
+        <x:f>ROUND(E4-F4,1)</x:f>
+        <x:v>41.8</x:v>
+      </x:c>
+      <x:c r="K4" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="27" t="str">
         <x:v>合计</x:v>
       </x:c>
       <x:c r="B7" s="26" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C7" s="26"/>
       <x:c r="D7" s="26"/>
@@ -2506,7 +2781,7 @@
       <x:c r="I7" s="26"/>
       <x:c r="J7" s="28" t="n">
         <x:f>SUM(J4:J4)</x:f>
-        <x:v>0</x:v>
+        <x:v>41.8</x:v>
       </x:c>
       <x:c r="K7" s="26"/>
     </x:row>
@@ -2524,7 +2799,7 @@
       <x:c r="I8" s="26"/>
       <x:c r="J8" s="30" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J4),0),1)</x:f>
-        <x:v>0</x:v>
+        <x:v>41.8</x:v>
       </x:c>
       <x:c r="K8" s="26"/>
     </x:row>

</xml_diff>

<commit_message>
Update amplitude website 2026-09-02
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Ra60f897f76bf48d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R04ee92ae0eb141af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Re3f116e14b6940a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R17e16424038a41b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Re66d73e6db794bb8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R9c565b84cf944385"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Ra150f2e93ad44d8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rb40efbf6b1494709"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rb558ff3e29ec4833"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R705c2c2a237f44be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rad250b89f27d4eb8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R1a20422860e54645"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R46adb995f30f4682"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R9432ef4517de4409"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R59361234a0204944"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R125b7c67df8e4cc9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Rd0368e3491df4dc7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Ra3d8fb5163e64889"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R2aaeed7845cf4644"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R2f57ff91d3fa4ce9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -145,7 +145,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="37">
+  <x:cellXfs count="39">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -193,6 +193,12 @@
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="201" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="7" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -479,25 +485,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-09-01</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7773.06</x:v>
+        <x:v>7624.71</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7667.33</x:v>
+        <x:v>7539.08</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>105.7</x:v>
+        <x:v>85.6</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>105.7</x:v>
+        <x:v>191.3</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>105.7</x:v>
+        <x:v>95.7</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -508,25 +514,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-09-01</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7955.57</x:v>
+        <x:v>7783.05</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7852.87</x:v>
+        <x:v>7692.15</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>102.7</x:v>
+        <x:v>90.9</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>102.7</x:v>
+        <x:v>193.6</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>102.7</x:v>
+        <x:v>96.8</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -537,25 +543,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-09-01</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3995.18</x:v>
+        <x:v>3965.81</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3976.47</x:v>
+        <x:v>3932.25</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>18.7</x:v>
+        <x:v>33.6</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>18.7</x:v>
+        <x:v>52.3</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>18.7</x:v>
+        <x:v>26.2</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -566,25 +572,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-09-01</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>7721</x:v>
+        <x:v>7575</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>7598.4</x:v>
+        <x:v>7466.2</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>122.6</x:v>
+        <x:v>108.8</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>122.6</x:v>
+        <x:v>231.4</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>122.6</x:v>
+        <x:v>115.7</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -682,25 +688,25 @@
         <x:v>碳酸锂2609</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>2026-09-01</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:v>160480</x:v>
+        <x:v>156200</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
-        <x:v>155800</x:v>
+        <x:v>152840</x:v>
       </x:c>
       <x:c r="E11" s="12" t="n">
-        <x:v>4680</x:v>
+        <x:v>3360</x:v>
       </x:c>
       <x:c r="F11" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G11" s="10" t="n">
-        <x:v>4680</x:v>
+        <x:v>8040</x:v>
       </x:c>
       <x:c r="H11" s="10" t="n">
-        <x:v>4680</x:v>
+        <x:v>4020</x:v>
       </x:c>
       <x:c r="I11" s="10" t="n">
         <x:v>6000</x:v>
@@ -714,7 +720,7 @@
         <x:v>2026-09-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-09-01</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -919,7 +925,7 @@
       <x:c r="G4" s="23" t="n">
         <x:v>155820</x:v>
       </x:c>
-      <x:c r="H4" s="36" t="n">
+      <x:c r="H4" s="38" t="n">
         <x:v>-3180</x:v>
       </x:c>
       <x:c r="I4" s="24" t="n">
@@ -933,43 +939,79 @@
         <x:v>LC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="27" t="str">
+    <x:row r="5">
+      <x:c r="A5" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B5" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C5" s="22" t="str">
+        <x:v>9月2日</x:v>
+      </x:c>
+      <x:c r="D5" s="23" t="n">
+        <x:v>156200</x:v>
+      </x:c>
+      <x:c r="E5" s="23" t="n">
+        <x:v>156200</x:v>
+      </x:c>
+      <x:c r="F5" s="23" t="n">
+        <x:v>152840</x:v>
+      </x:c>
+      <x:c r="G5" s="23" t="n">
+        <x:v>155000</x:v>
+      </x:c>
+      <x:c r="H5" s="38" t="n">
+        <x:v>-820</x:v>
+      </x:c>
+      <x:c r="I5" s="24" t="n">
+        <x:v>-0.005262482351431119</x:v>
+      </x:c>
+      <x:c r="J5" s="23" t="n">
+        <x:f>ROUND(E5-F5,1)</x:f>
+        <x:v>3360</x:v>
+      </x:c>
+      <x:c r="K5" s="22" t="str">
+        <x:v>LC2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B7" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C7" s="26"/>
-      <x:c r="D7" s="26"/>
-      <x:c r="E7" s="26"/>
-      <x:c r="F7" s="26"/>
-      <x:c r="G7" s="26"/>
-      <x:c r="H7" s="26"/>
-      <x:c r="I7" s="26"/>
-      <x:c r="J7" s="28" t="n">
-        <x:f>SUM(J4:J4)</x:f>
-        <x:v>4680</x:v>
-      </x:c>
-      <x:c r="K7" s="26"/>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="27" t="str">
+      <x:c r="B8" s="28" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C8" s="28"/>
+      <x:c r="D8" s="28"/>
+      <x:c r="E8" s="28"/>
+      <x:c r="F8" s="28"/>
+      <x:c r="G8" s="28"/>
+      <x:c r="H8" s="28"/>
+      <x:c r="I8" s="28"/>
+      <x:c r="J8" s="30" t="n">
+        <x:f>SUM(J4:J5)</x:f>
+        <x:v>8040</x:v>
+      </x:c>
+      <x:c r="K8" s="28"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B8" s="26"/>
-      <x:c r="C8" s="26"/>
-      <x:c r="D8" s="26"/>
-      <x:c r="E8" s="26"/>
-      <x:c r="F8" s="26"/>
-      <x:c r="G8" s="26"/>
-      <x:c r="H8" s="26"/>
-      <x:c r="I8" s="26"/>
-      <x:c r="J8" s="30" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J4),0),1)</x:f>
-        <x:v>4680</x:v>
-      </x:c>
-      <x:c r="K8" s="26"/>
+      <x:c r="B9" s="28"/>
+      <x:c r="C9" s="28"/>
+      <x:c r="D9" s="28"/>
+      <x:c r="E9" s="28"/>
+      <x:c r="F9" s="28"/>
+      <x:c r="G9" s="28"/>
+      <x:c r="H9" s="28"/>
+      <x:c r="I9" s="28"/>
+      <x:c r="J9" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J5),0),1)</x:f>
+        <x:v>4020</x:v>
+      </x:c>
+      <x:c r="K9" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1056,7 +1098,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B5" s="22" t="str">
-        <x:v>9月1日</x:v>
+        <x:v>9月1日-9月2日</x:v>
       </x:c>
       <x:c r="C5" s="23" t="n">
         <x:v>7773.06</x:v>
@@ -1065,61 +1107,61 @@
         <x:v>7773.06</x:v>
       </x:c>
       <x:c r="E5" s="23" t="n">
-        <x:v>7667.33</x:v>
+        <x:v>7539.08</x:v>
       </x:c>
       <x:c r="F5" s="23" t="n">
-        <x:v>7691.37</x:v>
+        <x:v>7583.76</x:v>
       </x:c>
       <x:c r="G5" s="23"/>
       <x:c r="H5" s="24"/>
-      <x:c r="I5" s="23" t="n">
+      <x:c r="I5" s="26" t="n">
         <x:f>ROUND(D5-E5,1)</x:f>
-        <x:v>105.7</x:v>
+        <x:v>234</x:v>
       </x:c>
       <x:c r="J5" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K5" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="27" t="str">
+      <x:c r="A6" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B6" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C6" s="26"/>
-      <x:c r="D6" s="26"/>
-      <x:c r="E6" s="26"/>
-      <x:c r="F6" s="26"/>
-      <x:c r="G6" s="26"/>
-      <x:c r="H6" s="26"/>
-      <x:c r="I6" s="28" t="n">
+      <x:c r="B6" s="28" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C6" s="28"/>
+      <x:c r="D6" s="28"/>
+      <x:c r="E6" s="28"/>
+      <x:c r="F6" s="28"/>
+      <x:c r="G6" s="28"/>
+      <x:c r="H6" s="28"/>
+      <x:c r="I6" s="30" t="n">
         <x:f>ROUND(SUM(I5:I5),1)</x:f>
-        <x:v>105.7</x:v>
-      </x:c>
-      <x:c r="J6" s="26"/>
-      <x:c r="K6" s="26"/>
+        <x:v>234</x:v>
+      </x:c>
+      <x:c r="J6" s="28"/>
+      <x:c r="K6" s="28"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="27" t="str">
+      <x:c r="A7" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B7" s="26"/>
-      <x:c r="C7" s="26"/>
-      <x:c r="D7" s="26"/>
-      <x:c r="E7" s="26"/>
-      <x:c r="F7" s="26"/>
-      <x:c r="G7" s="26"/>
-      <x:c r="H7" s="26"/>
-      <x:c r="I7" s="30" t="n">
+      <x:c r="B7" s="28"/>
+      <x:c r="C7" s="28"/>
+      <x:c r="D7" s="28"/>
+      <x:c r="E7" s="28"/>
+      <x:c r="F7" s="28"/>
+      <x:c r="G7" s="28"/>
+      <x:c r="H7" s="28"/>
+      <x:c r="I7" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I5),0),1)</x:f>
-        <x:v>105.7</x:v>
-      </x:c>
-      <x:c r="J7" s="26"/>
-      <x:c r="K7" s="26"/>
+        <x:v>234</x:v>
+      </x:c>
+      <x:c r="J7" s="28"/>
+      <x:c r="K7" s="28"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="17" t="str">
@@ -1176,7 +1218,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B11" s="22" t="str">
-        <x:v>9月1日</x:v>
+        <x:v>9月1日-9月2日</x:v>
       </x:c>
       <x:c r="C11" s="23" t="n">
         <x:v>7944.29</x:v>
@@ -1185,61 +1227,61 @@
         <x:v>7955.57</x:v>
       </x:c>
       <x:c r="E11" s="23" t="n">
-        <x:v>7852.87</x:v>
+        <x:v>7692.15</x:v>
       </x:c>
       <x:c r="F11" s="23" t="n">
-        <x:v>7858.52</x:v>
+        <x:v>7729.23</x:v>
       </x:c>
       <x:c r="G11" s="23"/>
       <x:c r="H11" s="24"/>
-      <x:c r="I11" s="23" t="n">
+      <x:c r="I11" s="26" t="n">
         <x:f>ROUND(D11-E11,1)</x:f>
-        <x:v>102.7</x:v>
+        <x:v>263.4</x:v>
       </x:c>
       <x:c r="J11" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K11" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="27" t="str">
+      <x:c r="A12" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B12" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C12" s="26"/>
-      <x:c r="D12" s="26"/>
-      <x:c r="E12" s="26"/>
-      <x:c r="F12" s="26"/>
-      <x:c r="G12" s="26"/>
-      <x:c r="H12" s="26"/>
-      <x:c r="I12" s="28" t="n">
+      <x:c r="B12" s="28" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C12" s="28"/>
+      <x:c r="D12" s="28"/>
+      <x:c r="E12" s="28"/>
+      <x:c r="F12" s="28"/>
+      <x:c r="G12" s="28"/>
+      <x:c r="H12" s="28"/>
+      <x:c r="I12" s="30" t="n">
         <x:f>ROUND(SUM(I11:I11),1)</x:f>
-        <x:v>102.7</x:v>
-      </x:c>
-      <x:c r="J12" s="26"/>
-      <x:c r="K12" s="26"/>
+        <x:v>263.4</x:v>
+      </x:c>
+      <x:c r="J12" s="28"/>
+      <x:c r="K12" s="28"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="27" t="str">
+      <x:c r="A13" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B13" s="26"/>
-      <x:c r="C13" s="26"/>
-      <x:c r="D13" s="26"/>
-      <x:c r="E13" s="26"/>
-      <x:c r="F13" s="26"/>
-      <x:c r="G13" s="26"/>
-      <x:c r="H13" s="26"/>
-      <x:c r="I13" s="30" t="n">
+      <x:c r="B13" s="28"/>
+      <x:c r="C13" s="28"/>
+      <x:c r="D13" s="28"/>
+      <x:c r="E13" s="28"/>
+      <x:c r="F13" s="28"/>
+      <x:c r="G13" s="28"/>
+      <x:c r="H13" s="28"/>
+      <x:c r="I13" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I11:I11),0),1)</x:f>
-        <x:v>102.7</x:v>
-      </x:c>
-      <x:c r="J13" s="26"/>
-      <x:c r="K13" s="26"/>
+        <x:v>263.4</x:v>
+      </x:c>
+      <x:c r="J13" s="28"/>
+      <x:c r="K13" s="28"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="17" t="str">
@@ -1296,7 +1338,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B17" s="22" t="str">
-        <x:v>9月1日</x:v>
+        <x:v>9月1日-9月2日</x:v>
       </x:c>
       <x:c r="C17" s="23" t="n">
         <x:v>3979.88</x:v>
@@ -1305,61 +1347,61 @@
         <x:v>3995.18</x:v>
       </x:c>
       <x:c r="E17" s="23" t="n">
-        <x:v>3976.47</x:v>
+        <x:v>3932.25</x:v>
       </x:c>
       <x:c r="F17" s="23" t="n">
-        <x:v>3979.89</x:v>
+        <x:v>3941.39</x:v>
       </x:c>
       <x:c r="G17" s="23"/>
       <x:c r="H17" s="24"/>
-      <x:c r="I17" s="23" t="n">
+      <x:c r="I17" s="26" t="n">
         <x:f>ROUND(D17-E17,1)</x:f>
-        <x:v>18.7</x:v>
+        <x:v>62.9</x:v>
       </x:c>
       <x:c r="J17" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K17" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="27" t="str">
+      <x:c r="A18" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B18" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C18" s="26"/>
-      <x:c r="D18" s="26"/>
-      <x:c r="E18" s="26"/>
-      <x:c r="F18" s="26"/>
-      <x:c r="G18" s="26"/>
-      <x:c r="H18" s="26"/>
-      <x:c r="I18" s="28" t="n">
+      <x:c r="B18" s="28" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C18" s="28"/>
+      <x:c r="D18" s="28"/>
+      <x:c r="E18" s="28"/>
+      <x:c r="F18" s="28"/>
+      <x:c r="G18" s="28"/>
+      <x:c r="H18" s="28"/>
+      <x:c r="I18" s="30" t="n">
         <x:f>ROUND(SUM(I17:I17),1)</x:f>
-        <x:v>18.7</x:v>
-      </x:c>
-      <x:c r="J18" s="26"/>
-      <x:c r="K18" s="26"/>
+        <x:v>62.9</x:v>
+      </x:c>
+      <x:c r="J18" s="28"/>
+      <x:c r="K18" s="28"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="27" t="str">
+      <x:c r="A19" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B19" s="26"/>
-      <x:c r="C19" s="26"/>
-      <x:c r="D19" s="26"/>
-      <x:c r="E19" s="26"/>
-      <x:c r="F19" s="26"/>
-      <x:c r="G19" s="26"/>
-      <x:c r="H19" s="26"/>
-      <x:c r="I19" s="30" t="n">
+      <x:c r="B19" s="28"/>
+      <x:c r="C19" s="28"/>
+      <x:c r="D19" s="28"/>
+      <x:c r="E19" s="28"/>
+      <x:c r="F19" s="28"/>
+      <x:c r="G19" s="28"/>
+      <x:c r="H19" s="28"/>
+      <x:c r="I19" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I17:I17),0),1)</x:f>
-        <x:v>18.7</x:v>
-      </x:c>
-      <x:c r="J19" s="26"/>
-      <x:c r="K19" s="26"/>
+        <x:v>62.9</x:v>
+      </x:c>
+      <x:c r="J19" s="28"/>
+      <x:c r="K19" s="28"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="17" t="str">
@@ -1416,7 +1458,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B23" s="22" t="str">
-        <x:v>9月1日</x:v>
+        <x:v>9月1日-9月2日</x:v>
       </x:c>
       <x:c r="C23" s="23" t="n">
         <x:v>7713.4</x:v>
@@ -1425,61 +1467,61 @@
         <x:v>7721</x:v>
       </x:c>
       <x:c r="E23" s="23" t="n">
-        <x:v>7598.4</x:v>
+        <x:v>7466.2</x:v>
       </x:c>
       <x:c r="F23" s="23" t="n">
-        <x:v>7645</x:v>
+        <x:v>7540.4</x:v>
       </x:c>
       <x:c r="G23" s="23"/>
       <x:c r="H23" s="24"/>
-      <x:c r="I23" s="23" t="n">
+      <x:c r="I23" s="26" t="n">
         <x:f>ROUND(D23-E23,1)</x:f>
-        <x:v>122.6</x:v>
+        <x:v>254.8</x:v>
       </x:c>
       <x:c r="J23" s="22" t="str">
         <x:v>IM2609</x:v>
       </x:c>
       <x:c r="K23" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="27" t="str">
+      <x:c r="A24" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B24" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C24" s="26"/>
-      <x:c r="D24" s="26"/>
-      <x:c r="E24" s="26"/>
-      <x:c r="F24" s="26"/>
-      <x:c r="G24" s="26"/>
-      <x:c r="H24" s="26"/>
-      <x:c r="I24" s="28" t="n">
+      <x:c r="B24" s="28" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C24" s="28"/>
+      <x:c r="D24" s="28"/>
+      <x:c r="E24" s="28"/>
+      <x:c r="F24" s="28"/>
+      <x:c r="G24" s="28"/>
+      <x:c r="H24" s="28"/>
+      <x:c r="I24" s="30" t="n">
         <x:f>ROUND(SUM(I23:I23),1)</x:f>
-        <x:v>122.6</x:v>
-      </x:c>
-      <x:c r="J24" s="26"/>
-      <x:c r="K24" s="26"/>
+        <x:v>254.8</x:v>
+      </x:c>
+      <x:c r="J24" s="28"/>
+      <x:c r="K24" s="28"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="27" t="str">
+      <x:c r="A25" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B25" s="26"/>
-      <x:c r="C25" s="26"/>
-      <x:c r="D25" s="26"/>
-      <x:c r="E25" s="26"/>
-      <x:c r="F25" s="26"/>
-      <x:c r="G25" s="26"/>
-      <x:c r="H25" s="26"/>
-      <x:c r="I25" s="30" t="n">
+      <x:c r="B25" s="28"/>
+      <x:c r="C25" s="28"/>
+      <x:c r="D25" s="28"/>
+      <x:c r="E25" s="28"/>
+      <x:c r="F25" s="28"/>
+      <x:c r="G25" s="28"/>
+      <x:c r="H25" s="28"/>
+      <x:c r="I25" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I23:I23),0),1)</x:f>
-        <x:v>122.6</x:v>
-      </x:c>
-      <x:c r="J25" s="26"/>
-      <x:c r="K25" s="26"/>
+        <x:v>254.8</x:v>
+      </x:c>
+      <x:c r="J25" s="28"/>
+      <x:c r="K25" s="28"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="17" t="str">
@@ -1564,42 +1606,42 @@
       </x:c>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="27" t="str">
+      <x:c r="A30" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B30" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C30" s="26"/>
-      <x:c r="D30" s="26"/>
-      <x:c r="E30" s="26"/>
-      <x:c r="F30" s="26"/>
-      <x:c r="G30" s="26"/>
-      <x:c r="H30" s="26"/>
-      <x:c r="I30" s="28" t="n">
+      <x:c r="B30" s="28" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C30" s="28"/>
+      <x:c r="D30" s="28"/>
+      <x:c r="E30" s="28"/>
+      <x:c r="F30" s="28"/>
+      <x:c r="G30" s="28"/>
+      <x:c r="H30" s="28"/>
+      <x:c r="I30" s="30" t="n">
         <x:f>ROUND(SUM(I29:I29),1)</x:f>
         <x:v>138</x:v>
       </x:c>
-      <x:c r="J30" s="26"/>
-      <x:c r="K30" s="26"/>
+      <x:c r="J30" s="28"/>
+      <x:c r="K30" s="28"/>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="27" t="str">
+      <x:c r="A31" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B31" s="26"/>
-      <x:c r="C31" s="26"/>
-      <x:c r="D31" s="26"/>
-      <x:c r="E31" s="26"/>
-      <x:c r="F31" s="26"/>
-      <x:c r="G31" s="26"/>
-      <x:c r="H31" s="26"/>
-      <x:c r="I31" s="30" t="n">
+      <x:c r="B31" s="28"/>
+      <x:c r="C31" s="28"/>
+      <x:c r="D31" s="28"/>
+      <x:c r="E31" s="28"/>
+      <x:c r="F31" s="28"/>
+      <x:c r="G31" s="28"/>
+      <x:c r="H31" s="28"/>
+      <x:c r="I31" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I29:I29),0),1)</x:f>
         <x:v>138</x:v>
       </x:c>
-      <x:c r="J31" s="26"/>
-      <x:c r="K31" s="26"/>
+      <x:c r="J31" s="28"/>
+      <x:c r="K31" s="28"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="17" t="str">
@@ -1684,42 +1726,42 @@
       </x:c>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="27" t="str">
+      <x:c r="A36" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B36" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C36" s="26"/>
-      <x:c r="D36" s="26"/>
-      <x:c r="E36" s="26"/>
-      <x:c r="F36" s="26"/>
-      <x:c r="G36" s="26"/>
-      <x:c r="H36" s="26"/>
-      <x:c r="I36" s="28" t="n">
+      <x:c r="B36" s="28" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C36" s="28"/>
+      <x:c r="D36" s="28"/>
+      <x:c r="E36" s="28"/>
+      <x:c r="F36" s="28"/>
+      <x:c r="G36" s="28"/>
+      <x:c r="H36" s="28"/>
+      <x:c r="I36" s="30" t="n">
         <x:f>ROUND(SUM(I35:I35),1)</x:f>
         <x:v>41.8</x:v>
       </x:c>
-      <x:c r="J36" s="26"/>
-      <x:c r="K36" s="26"/>
+      <x:c r="J36" s="28"/>
+      <x:c r="K36" s="28"/>
     </x:row>
     <x:row r="37">
-      <x:c r="A37" s="27" t="str">
+      <x:c r="A37" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B37" s="26"/>
-      <x:c r="C37" s="26"/>
-      <x:c r="D37" s="26"/>
-      <x:c r="E37" s="26"/>
-      <x:c r="F37" s="26"/>
-      <x:c r="G37" s="26"/>
-      <x:c r="H37" s="26"/>
-      <x:c r="I37" s="30" t="n">
+      <x:c r="B37" s="28"/>
+      <x:c r="C37" s="28"/>
+      <x:c r="D37" s="28"/>
+      <x:c r="E37" s="28"/>
+      <x:c r="F37" s="28"/>
+      <x:c r="G37" s="28"/>
+      <x:c r="H37" s="28"/>
+      <x:c r="I37" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I35:I35),0),1)</x:f>
         <x:v>41.8</x:v>
       </x:c>
-      <x:c r="J37" s="26"/>
-      <x:c r="K37" s="26"/>
+      <x:c r="J37" s="28"/>
+      <x:c r="K37" s="28"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="17" t="str">
@@ -1804,42 +1846,42 @@
       </x:c>
     </x:row>
     <x:row r="42">
-      <x:c r="A42" s="27" t="str">
+      <x:c r="A42" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B42" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C42" s="26"/>
-      <x:c r="D42" s="26"/>
-      <x:c r="E42" s="26"/>
-      <x:c r="F42" s="26"/>
-      <x:c r="G42" s="26"/>
-      <x:c r="H42" s="26"/>
-      <x:c r="I42" s="28" t="n">
+      <x:c r="B42" s="28" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C42" s="28"/>
+      <x:c r="D42" s="28"/>
+      <x:c r="E42" s="28"/>
+      <x:c r="F42" s="28"/>
+      <x:c r="G42" s="28"/>
+      <x:c r="H42" s="28"/>
+      <x:c r="I42" s="30" t="n">
         <x:f>ROUND(SUM(I41:I41),1)</x:f>
         <x:v>22.8</x:v>
       </x:c>
-      <x:c r="J42" s="26"/>
-      <x:c r="K42" s="26"/>
+      <x:c r="J42" s="28"/>
+      <x:c r="K42" s="28"/>
     </x:row>
     <x:row r="43">
-      <x:c r="A43" s="27" t="str">
+      <x:c r="A43" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B43" s="26"/>
-      <x:c r="C43" s="26"/>
-      <x:c r="D43" s="26"/>
-      <x:c r="E43" s="26"/>
-      <x:c r="F43" s="26"/>
-      <x:c r="G43" s="26"/>
-      <x:c r="H43" s="26"/>
-      <x:c r="I43" s="30" t="n">
+      <x:c r="B43" s="28"/>
+      <x:c r="C43" s="28"/>
+      <x:c r="D43" s="28"/>
+      <x:c r="E43" s="28"/>
+      <x:c r="F43" s="28"/>
+      <x:c r="G43" s="28"/>
+      <x:c r="H43" s="28"/>
+      <x:c r="I43" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I41:I41),0),1)</x:f>
         <x:v>22.8</x:v>
       </x:c>
-      <x:c r="J43" s="26"/>
-      <x:c r="K43" s="26"/>
+      <x:c r="J43" s="28"/>
+      <x:c r="K43" s="28"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="17" t="str">
@@ -1896,7 +1938,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B47" s="22" t="str">
-        <x:v>9月1日</x:v>
+        <x:v>9月1日-9月2日</x:v>
       </x:c>
       <x:c r="C47" s="23" t="n">
         <x:v>159000</x:v>
@@ -1905,61 +1947,61 @@
         <x:v>160480</x:v>
       </x:c>
       <x:c r="E47" s="23" t="n">
-        <x:v>155800</x:v>
+        <x:v>152840</x:v>
       </x:c>
       <x:c r="F47" s="23" t="n">
-        <x:v>155820</x:v>
+        <x:v>155000</x:v>
       </x:c>
       <x:c r="G47" s="23"/>
       <x:c r="H47" s="24"/>
-      <x:c r="I47" s="23" t="n">
+      <x:c r="I47" s="26" t="n">
         <x:f>ROUND(D47-E47,1)</x:f>
-        <x:v>4680</x:v>
+        <x:v>7640</x:v>
       </x:c>
       <x:c r="J47" s="22" t="str">
         <x:v>LC2609</x:v>
       </x:c>
       <x:c r="K47" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
-      <x:c r="A48" s="27" t="str">
+      <x:c r="A48" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B48" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C48" s="26"/>
-      <x:c r="D48" s="26"/>
-      <x:c r="E48" s="26"/>
-      <x:c r="F48" s="26"/>
-      <x:c r="G48" s="26"/>
-      <x:c r="H48" s="26"/>
-      <x:c r="I48" s="28" t="n">
+      <x:c r="B48" s="28" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C48" s="28"/>
+      <x:c r="D48" s="28"/>
+      <x:c r="E48" s="28"/>
+      <x:c r="F48" s="28"/>
+      <x:c r="G48" s="28"/>
+      <x:c r="H48" s="28"/>
+      <x:c r="I48" s="30" t="n">
         <x:f>ROUND(SUM(I47:I47),1)</x:f>
-        <x:v>4680</x:v>
-      </x:c>
-      <x:c r="J48" s="26"/>
-      <x:c r="K48" s="26"/>
+        <x:v>7640</x:v>
+      </x:c>
+      <x:c r="J48" s="28"/>
+      <x:c r="K48" s="28"/>
     </x:row>
     <x:row r="49">
-      <x:c r="A49" s="27" t="str">
+      <x:c r="A49" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B49" s="26"/>
-      <x:c r="C49" s="26"/>
-      <x:c r="D49" s="26"/>
-      <x:c r="E49" s="26"/>
-      <x:c r="F49" s="26"/>
-      <x:c r="G49" s="26"/>
-      <x:c r="H49" s="26"/>
-      <x:c r="I49" s="30" t="n">
+      <x:c r="B49" s="28"/>
+      <x:c r="C49" s="28"/>
+      <x:c r="D49" s="28"/>
+      <x:c r="E49" s="28"/>
+      <x:c r="F49" s="28"/>
+      <x:c r="G49" s="28"/>
+      <x:c r="H49" s="28"/>
+      <x:c r="I49" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I47:I47),0),1)</x:f>
-        <x:v>4680</x:v>
-      </x:c>
-      <x:c r="J49" s="26"/>
-      <x:c r="K49" s="26"/>
+        <x:v>7640</x:v>
+      </x:c>
+      <x:c r="J49" s="28"/>
+      <x:c r="K49" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2070,43 +2112,79 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="27" t="str">
+    <x:row r="5">
+      <x:c r="A5" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B5" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C5" s="22" t="str">
+        <x:v>9月2日</x:v>
+      </x:c>
+      <x:c r="D5" s="23" t="n">
+        <x:v>7616.23</x:v>
+      </x:c>
+      <x:c r="E5" s="23" t="n">
+        <x:v>7624.71</x:v>
+      </x:c>
+      <x:c r="F5" s="23" t="n">
+        <x:v>7539.08</x:v>
+      </x:c>
+      <x:c r="G5" s="23" t="n">
+        <x:v>7583.76</x:v>
+      </x:c>
+      <x:c r="H5" s="23" t="n">
+        <x:v>-107.6</x:v>
+      </x:c>
+      <x:c r="I5" s="24" t="n">
+        <x:v>-0.013991005503570797</x:v>
+      </x:c>
+      <x:c r="J5" s="23" t="n">
+        <x:f>ROUND(E5-F5,1)</x:f>
+        <x:v>85.6</x:v>
+      </x:c>
+      <x:c r="K5" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B7" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C7" s="26"/>
-      <x:c r="D7" s="26"/>
-      <x:c r="E7" s="26"/>
-      <x:c r="F7" s="26"/>
-      <x:c r="G7" s="26"/>
-      <x:c r="H7" s="26"/>
-      <x:c r="I7" s="26"/>
-      <x:c r="J7" s="28" t="n">
-        <x:f>SUM(J4:J4)</x:f>
-        <x:v>105.7</x:v>
-      </x:c>
-      <x:c r="K7" s="26"/>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="27" t="str">
+      <x:c r="B8" s="28" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C8" s="28"/>
+      <x:c r="D8" s="28"/>
+      <x:c r="E8" s="28"/>
+      <x:c r="F8" s="28"/>
+      <x:c r="G8" s="28"/>
+      <x:c r="H8" s="28"/>
+      <x:c r="I8" s="28"/>
+      <x:c r="J8" s="30" t="n">
+        <x:f>SUM(J4:J5)</x:f>
+        <x:v>191.3</x:v>
+      </x:c>
+      <x:c r="K8" s="28"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B8" s="26"/>
-      <x:c r="C8" s="26"/>
-      <x:c r="D8" s="26"/>
-      <x:c r="E8" s="26"/>
-      <x:c r="F8" s="26"/>
-      <x:c r="G8" s="26"/>
-      <x:c r="H8" s="26"/>
-      <x:c r="I8" s="26"/>
-      <x:c r="J8" s="30" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J4),0),1)</x:f>
-        <x:v>105.7</x:v>
-      </x:c>
-      <x:c r="K8" s="26"/>
+      <x:c r="B9" s="28"/>
+      <x:c r="C9" s="28"/>
+      <x:c r="D9" s="28"/>
+      <x:c r="E9" s="28"/>
+      <x:c r="F9" s="28"/>
+      <x:c r="G9" s="28"/>
+      <x:c r="H9" s="28"/>
+      <x:c r="I9" s="28"/>
+      <x:c r="J9" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J5),0),1)</x:f>
+        <x:v>95.7</x:v>
+      </x:c>
+      <x:c r="K9" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2209,43 +2287,79 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="27" t="str">
+    <x:row r="5">
+      <x:c r="A5" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B5" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C5" s="22" t="str">
+        <x:v>9月2日</x:v>
+      </x:c>
+      <x:c r="D5" s="23" t="n">
+        <x:v>7781.29</x:v>
+      </x:c>
+      <x:c r="E5" s="23" t="n">
+        <x:v>7783.05</x:v>
+      </x:c>
+      <x:c r="F5" s="23" t="n">
+        <x:v>7692.15</x:v>
+      </x:c>
+      <x:c r="G5" s="23" t="n">
+        <x:v>7729.23</x:v>
+      </x:c>
+      <x:c r="H5" s="23" t="n">
+        <x:v>-129.3</x:v>
+      </x:c>
+      <x:c r="I5" s="24" t="n">
+        <x:v>-0.016452207285850395</x:v>
+      </x:c>
+      <x:c r="J5" s="23" t="n">
+        <x:f>ROUND(E5-F5,1)</x:f>
+        <x:v>90.9</x:v>
+      </x:c>
+      <x:c r="K5" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B7" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C7" s="26"/>
-      <x:c r="D7" s="26"/>
-      <x:c r="E7" s="26"/>
-      <x:c r="F7" s="26"/>
-      <x:c r="G7" s="26"/>
-      <x:c r="H7" s="26"/>
-      <x:c r="I7" s="26"/>
-      <x:c r="J7" s="28" t="n">
-        <x:f>SUM(J4:J4)</x:f>
-        <x:v>102.7</x:v>
-      </x:c>
-      <x:c r="K7" s="26"/>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="27" t="str">
+      <x:c r="B8" s="28" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C8" s="28"/>
+      <x:c r="D8" s="28"/>
+      <x:c r="E8" s="28"/>
+      <x:c r="F8" s="28"/>
+      <x:c r="G8" s="28"/>
+      <x:c r="H8" s="28"/>
+      <x:c r="I8" s="28"/>
+      <x:c r="J8" s="30" t="n">
+        <x:f>SUM(J4:J5)</x:f>
+        <x:v>193.60000000000002</x:v>
+      </x:c>
+      <x:c r="K8" s="28"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B8" s="26"/>
-      <x:c r="C8" s="26"/>
-      <x:c r="D8" s="26"/>
-      <x:c r="E8" s="26"/>
-      <x:c r="F8" s="26"/>
-      <x:c r="G8" s="26"/>
-      <x:c r="H8" s="26"/>
-      <x:c r="I8" s="26"/>
-      <x:c r="J8" s="30" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J4),0),1)</x:f>
-        <x:v>102.7</x:v>
-      </x:c>
-      <x:c r="K8" s="26"/>
+      <x:c r="B9" s="28"/>
+      <x:c r="C9" s="28"/>
+      <x:c r="D9" s="28"/>
+      <x:c r="E9" s="28"/>
+      <x:c r="F9" s="28"/>
+      <x:c r="G9" s="28"/>
+      <x:c r="H9" s="28"/>
+      <x:c r="I9" s="28"/>
+      <x:c r="J9" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J5),0),1)</x:f>
+        <x:v>96.8</x:v>
+      </x:c>
+      <x:c r="K9" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2348,43 +2462,79 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="27" t="str">
+    <x:row r="5">
+      <x:c r="A5" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B5" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C5" s="22" t="str">
+        <x:v>9月2日</x:v>
+      </x:c>
+      <x:c r="D5" s="23" t="n">
+        <x:v>3963.07</x:v>
+      </x:c>
+      <x:c r="E5" s="23" t="n">
+        <x:v>3965.81</x:v>
+      </x:c>
+      <x:c r="F5" s="23" t="n">
+        <x:v>3932.25</x:v>
+      </x:c>
+      <x:c r="G5" s="23" t="n">
+        <x:v>3941.39</x:v>
+      </x:c>
+      <x:c r="H5" s="23" t="n">
+        <x:v>-38.5</x:v>
+      </x:c>
+      <x:c r="I5" s="24" t="n">
+        <x:v>-0.009673634195919933</x:v>
+      </x:c>
+      <x:c r="J5" s="23" t="n">
+        <x:f>ROUND(E5-F5,1)</x:f>
+        <x:v>33.6</x:v>
+      </x:c>
+      <x:c r="K5" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B7" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C7" s="26"/>
-      <x:c r="D7" s="26"/>
-      <x:c r="E7" s="26"/>
-      <x:c r="F7" s="26"/>
-      <x:c r="G7" s="26"/>
-      <x:c r="H7" s="26"/>
-      <x:c r="I7" s="26"/>
-      <x:c r="J7" s="28" t="n">
-        <x:f>SUM(J4:J4)</x:f>
-        <x:v>18.7</x:v>
-      </x:c>
-      <x:c r="K7" s="26"/>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="27" t="str">
+      <x:c r="B8" s="28" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C8" s="28"/>
+      <x:c r="D8" s="28"/>
+      <x:c r="E8" s="28"/>
+      <x:c r="F8" s="28"/>
+      <x:c r="G8" s="28"/>
+      <x:c r="H8" s="28"/>
+      <x:c r="I8" s="28"/>
+      <x:c r="J8" s="30" t="n">
+        <x:f>SUM(J4:J5)</x:f>
+        <x:v>52.3</x:v>
+      </x:c>
+      <x:c r="K8" s="28"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B8" s="26"/>
-      <x:c r="C8" s="26"/>
-      <x:c r="D8" s="26"/>
-      <x:c r="E8" s="26"/>
-      <x:c r="F8" s="26"/>
-      <x:c r="G8" s="26"/>
-      <x:c r="H8" s="26"/>
-      <x:c r="I8" s="26"/>
-      <x:c r="J8" s="30" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J4),0),1)</x:f>
-        <x:v>18.7</x:v>
-      </x:c>
-      <x:c r="K8" s="26"/>
+      <x:c r="B9" s="28"/>
+      <x:c r="C9" s="28"/>
+      <x:c r="D9" s="28"/>
+      <x:c r="E9" s="28"/>
+      <x:c r="F9" s="28"/>
+      <x:c r="G9" s="28"/>
+      <x:c r="H9" s="28"/>
+      <x:c r="I9" s="28"/>
+      <x:c r="J9" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J5),0),1)</x:f>
+        <x:v>26.2</x:v>
+      </x:c>
+      <x:c r="K9" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2487,43 +2637,79 @@
         <x:v>IM2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="27" t="str">
+    <x:row r="5">
+      <x:c r="A5" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B5" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C5" s="22" t="str">
+        <x:v>9月2日</x:v>
+      </x:c>
+      <x:c r="D5" s="23" t="n">
+        <x:v>7570</x:v>
+      </x:c>
+      <x:c r="E5" s="23" t="n">
+        <x:v>7575</x:v>
+      </x:c>
+      <x:c r="F5" s="23" t="n">
+        <x:v>7466.2</x:v>
+      </x:c>
+      <x:c r="G5" s="23" t="n">
+        <x:v>7540.4</x:v>
+      </x:c>
+      <x:c r="H5" s="23" t="n">
+        <x:v>-104.6</x:v>
+      </x:c>
+      <x:c r="I5" s="24" t="n">
+        <x:v>-0.013682145192936646</x:v>
+      </x:c>
+      <x:c r="J5" s="23" t="n">
+        <x:f>ROUND(E5-F5,1)</x:f>
+        <x:v>108.8</x:v>
+      </x:c>
+      <x:c r="K5" s="22" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B7" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C7" s="26"/>
-      <x:c r="D7" s="26"/>
-      <x:c r="E7" s="26"/>
-      <x:c r="F7" s="26"/>
-      <x:c r="G7" s="26"/>
-      <x:c r="H7" s="26"/>
-      <x:c r="I7" s="26"/>
-      <x:c r="J7" s="28" t="n">
-        <x:f>SUM(J4:J4)</x:f>
-        <x:v>122.6</x:v>
-      </x:c>
-      <x:c r="K7" s="26"/>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="27" t="str">
+      <x:c r="B8" s="28" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C8" s="28"/>
+      <x:c r="D8" s="28"/>
+      <x:c r="E8" s="28"/>
+      <x:c r="F8" s="28"/>
+      <x:c r="G8" s="28"/>
+      <x:c r="H8" s="28"/>
+      <x:c r="I8" s="28"/>
+      <x:c r="J8" s="30" t="n">
+        <x:f>SUM(J4:J5)</x:f>
+        <x:v>231.39999999999998</x:v>
+      </x:c>
+      <x:c r="K8" s="28"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B8" s="26"/>
-      <x:c r="C8" s="26"/>
-      <x:c r="D8" s="26"/>
-      <x:c r="E8" s="26"/>
-      <x:c r="F8" s="26"/>
-      <x:c r="G8" s="26"/>
-      <x:c r="H8" s="26"/>
-      <x:c r="I8" s="26"/>
-      <x:c r="J8" s="30" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J4),0),1)</x:f>
-        <x:v>122.6</x:v>
-      </x:c>
-      <x:c r="K8" s="26"/>
+      <x:c r="B9" s="28"/>
+      <x:c r="C9" s="28"/>
+      <x:c r="D9" s="28"/>
+      <x:c r="E9" s="28"/>
+      <x:c r="F9" s="28"/>
+      <x:c r="G9" s="28"/>
+      <x:c r="H9" s="28"/>
+      <x:c r="I9" s="28"/>
+      <x:c r="J9" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J5),0),1)</x:f>
+        <x:v>115.7</x:v>
+      </x:c>
+      <x:c r="K9" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2627,42 +2813,42 @@
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="27" t="str">
+      <x:c r="A7" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B7" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C7" s="26"/>
-      <x:c r="D7" s="26"/>
-      <x:c r="E7" s="26"/>
-      <x:c r="F7" s="26"/>
-      <x:c r="G7" s="26"/>
-      <x:c r="H7" s="26"/>
-      <x:c r="I7" s="26"/>
-      <x:c r="J7" s="28" t="n">
+      <x:c r="B7" s="28" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C7" s="28"/>
+      <x:c r="D7" s="28"/>
+      <x:c r="E7" s="28"/>
+      <x:c r="F7" s="28"/>
+      <x:c r="G7" s="28"/>
+      <x:c r="H7" s="28"/>
+      <x:c r="I7" s="28"/>
+      <x:c r="J7" s="30" t="n">
         <x:f>SUM(J4:J4)</x:f>
         <x:v>138</x:v>
       </x:c>
-      <x:c r="K7" s="26"/>
+      <x:c r="K7" s="28"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="27" t="str">
+      <x:c r="A8" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B8" s="26"/>
-      <x:c r="C8" s="26"/>
-      <x:c r="D8" s="26"/>
-      <x:c r="E8" s="26"/>
-      <x:c r="F8" s="26"/>
-      <x:c r="G8" s="26"/>
-      <x:c r="H8" s="26"/>
-      <x:c r="I8" s="26"/>
-      <x:c r="J8" s="30" t="n">
+      <x:c r="B8" s="28"/>
+      <x:c r="C8" s="28"/>
+      <x:c r="D8" s="28"/>
+      <x:c r="E8" s="28"/>
+      <x:c r="F8" s="28"/>
+      <x:c r="G8" s="28"/>
+      <x:c r="H8" s="28"/>
+      <x:c r="I8" s="28"/>
+      <x:c r="J8" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J4),0),1)</x:f>
         <x:v>138</x:v>
       </x:c>
-      <x:c r="K8" s="26"/>
+      <x:c r="K8" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2766,42 +2952,42 @@
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="27" t="str">
+      <x:c r="A7" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B7" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C7" s="26"/>
-      <x:c r="D7" s="26"/>
-      <x:c r="E7" s="26"/>
-      <x:c r="F7" s="26"/>
-      <x:c r="G7" s="26"/>
-      <x:c r="H7" s="26"/>
-      <x:c r="I7" s="26"/>
-      <x:c r="J7" s="28" t="n">
+      <x:c r="B7" s="28" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C7" s="28"/>
+      <x:c r="D7" s="28"/>
+      <x:c r="E7" s="28"/>
+      <x:c r="F7" s="28"/>
+      <x:c r="G7" s="28"/>
+      <x:c r="H7" s="28"/>
+      <x:c r="I7" s="28"/>
+      <x:c r="J7" s="30" t="n">
         <x:f>SUM(J4:J4)</x:f>
         <x:v>41.8</x:v>
       </x:c>
-      <x:c r="K7" s="26"/>
+      <x:c r="K7" s="28"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="27" t="str">
+      <x:c r="A8" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B8" s="26"/>
-      <x:c r="C8" s="26"/>
-      <x:c r="D8" s="26"/>
-      <x:c r="E8" s="26"/>
-      <x:c r="F8" s="26"/>
-      <x:c r="G8" s="26"/>
-      <x:c r="H8" s="26"/>
-      <x:c r="I8" s="26"/>
-      <x:c r="J8" s="30" t="n">
+      <x:c r="B8" s="28"/>
+      <x:c r="C8" s="28"/>
+      <x:c r="D8" s="28"/>
+      <x:c r="E8" s="28"/>
+      <x:c r="F8" s="28"/>
+      <x:c r="G8" s="28"/>
+      <x:c r="H8" s="28"/>
+      <x:c r="I8" s="28"/>
+      <x:c r="J8" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J4),0),1)</x:f>
         <x:v>41.8</x:v>
       </x:c>
-      <x:c r="K8" s="26"/>
+      <x:c r="K8" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2905,42 +3091,42 @@
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="27" t="str">
+      <x:c r="A7" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B7" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C7" s="26"/>
-      <x:c r="D7" s="26"/>
-      <x:c r="E7" s="26"/>
-      <x:c r="F7" s="26"/>
-      <x:c r="G7" s="26"/>
-      <x:c r="H7" s="26"/>
-      <x:c r="I7" s="26"/>
-      <x:c r="J7" s="28" t="n">
+      <x:c r="B7" s="28" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C7" s="28"/>
+      <x:c r="D7" s="28"/>
+      <x:c r="E7" s="28"/>
+      <x:c r="F7" s="28"/>
+      <x:c r="G7" s="28"/>
+      <x:c r="H7" s="28"/>
+      <x:c r="I7" s="28"/>
+      <x:c r="J7" s="30" t="n">
         <x:f>SUM(J4:J4)</x:f>
         <x:v>22.8</x:v>
       </x:c>
-      <x:c r="K7" s="26"/>
+      <x:c r="K7" s="28"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="27" t="str">
+      <x:c r="A8" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B8" s="26"/>
-      <x:c r="C8" s="26"/>
-      <x:c r="D8" s="26"/>
-      <x:c r="E8" s="26"/>
-      <x:c r="F8" s="26"/>
-      <x:c r="G8" s="26"/>
-      <x:c r="H8" s="26"/>
-      <x:c r="I8" s="26"/>
-      <x:c r="J8" s="30" t="n">
+      <x:c r="B8" s="28"/>
+      <x:c r="C8" s="28"/>
+      <x:c r="D8" s="28"/>
+      <x:c r="E8" s="28"/>
+      <x:c r="F8" s="28"/>
+      <x:c r="G8" s="28"/>
+      <x:c r="H8" s="28"/>
+      <x:c r="I8" s="28"/>
+      <x:c r="J8" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J4),0),1)</x:f>
         <x:v>22.8</x:v>
       </x:c>
-      <x:c r="K8" s="26"/>
+      <x:c r="K8" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-09-03
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R0c445ccaf62e4fe1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R14476857929141af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R3d9bd18d14d6490e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rbb2da6df0a804210"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Rf23402dfa7df4666"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rb8aa456522d541d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Radd853c24ae04c07"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R02f674aaa6ce4da1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R3e844be564614654"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R0f7b34de7ec84735"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R1ec50ce396804baa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R8aeecc7253be4999"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R3677b9ae0e52465c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rfe44e4cfda4944c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R6c385e9b81404899"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rb014f5f13ccc4cea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R5c5673786a8d4fae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rd1046d491a4a4e97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rdd727beeb9114f27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R8d03f0ace0134a29"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -485,25 +485,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-09-02</x:v>
+        <x:v>2026-09-03</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7624.71</x:v>
+        <x:v>7657.75</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7539.08</x:v>
+        <x:v>7531.67</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>85.6</x:v>
+        <x:v>126.1</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>191.3</x:v>
+        <x:v>317.4</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>95.7</x:v>
+        <x:v>105.8</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -514,25 +514,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-09-02</x:v>
+        <x:v>2026-09-03</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7783.05</x:v>
+        <x:v>7799.63</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7692.15</x:v>
+        <x:v>7686.44</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>90.9</x:v>
+        <x:v>113.2</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>193.6</x:v>
+        <x:v>306.8</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>96.8</x:v>
+        <x:v>102.3</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -543,25 +543,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-09-02</x:v>
+        <x:v>2026-09-03</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3965.81</x:v>
+        <x:v>3968.11</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3932.25</x:v>
+        <x:v>3930.45</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>33.6</x:v>
+        <x:v>37.7</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>52.3</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>26.2</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -601,25 +601,25 @@
         <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>2026-09-02</x:v>
+        <x:v>2026-09-03</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:v>7720</x:v>
+        <x:v>7752.8</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>7593</x:v>
+        <x:v>7601.6</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>127</x:v>
+        <x:v>151.2</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>265</x:v>
+        <x:v>416.2</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
-        <x:v>132.5</x:v>
+        <x:v>138.7</x:v>
       </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
@@ -630,25 +630,25 @@
         <x:v>IF主力</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>2026-09-02</x:v>
+        <x:v>2026-09-03</x:v>
       </x:c>
       <x:c r="C9" s="10" t="n">
-        <x:v>4567</x:v>
+        <x:v>4561.2</x:v>
       </x:c>
       <x:c r="D9" s="10" t="n">
-        <x:v>4497.6</x:v>
+        <x:v>4510.4</x:v>
       </x:c>
       <x:c r="E9" s="12" t="n">
-        <x:v>69.4</x:v>
+        <x:v>50.8</x:v>
       </x:c>
       <x:c r="F9" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G9" s="10" t="n">
-        <x:v>111.2</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="H9" s="10" t="n">
-        <x:v>55.6</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="I9" s="10" t="n">
         <x:v>90</x:v>
@@ -659,25 +659,25 @@
         <x:v>IH主力</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>2026-09-02</x:v>
+        <x:v>2026-09-03</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:v>2917.4</x:v>
+        <x:v>2922.8</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
-        <x:v>2881.4</x:v>
+        <x:v>2893.6</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
-        <x:v>36</x:v>
+        <x:v>29.2</x:v>
       </x:c>
       <x:c r="F10" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G10" s="10" t="n">
-        <x:v>58.8</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="H10" s="10" t="n">
-        <x:v>29.4</x:v>
+        <x:v>29.3</x:v>
       </x:c>
       <x:c r="I10" s="10" t="n">
         <x:v>60</x:v>
@@ -688,25 +688,25 @@
         <x:v>碳酸锂2609</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>2026-09-02</x:v>
+        <x:v>2026-09-03</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:v>156200</x:v>
+        <x:v>155600</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
-        <x:v>152840</x:v>
+        <x:v>148880</x:v>
       </x:c>
       <x:c r="E11" s="12" t="n">
-        <x:v>3360</x:v>
+        <x:v>6720</x:v>
       </x:c>
       <x:c r="F11" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G11" s="10" t="n">
-        <x:v>8040</x:v>
+        <x:v>14760</x:v>
       </x:c>
       <x:c r="H11" s="10" t="n">
-        <x:v>4020</x:v>
+        <x:v>4920</x:v>
       </x:c>
       <x:c r="I11" s="10" t="n">
         <x:v>6000</x:v>
@@ -720,7 +720,7 @@
         <x:v>2026-09-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-09-02</x:v>
+        <x:v>2026-09-03</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -975,31 +975,49 @@
         <x:v>LC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B8" s="28" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C8" s="28"/>
-      <x:c r="D8" s="28"/>
-      <x:c r="E8" s="28"/>
-      <x:c r="F8" s="28"/>
-      <x:c r="G8" s="28"/>
-      <x:c r="H8" s="28"/>
-      <x:c r="I8" s="28"/>
-      <x:c r="J8" s="30" t="n">
-        <x:f>SUM(J4:J5)</x:f>
-        <x:v>8040</x:v>
-      </x:c>
-      <x:c r="K8" s="28"/>
+    <x:row r="6">
+      <x:c r="A6" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B6" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C6" s="22" t="str">
+        <x:v>9月3日</x:v>
+      </x:c>
+      <x:c r="D6" s="23" t="n">
+        <x:v>154860</x:v>
+      </x:c>
+      <x:c r="E6" s="23" t="n">
+        <x:v>155600</x:v>
+      </x:c>
+      <x:c r="F6" s="23" t="n">
+        <x:v>148880</x:v>
+      </x:c>
+      <x:c r="G6" s="23" t="n">
+        <x:v>148900</x:v>
+      </x:c>
+      <x:c r="H6" s="38" t="n">
+        <x:v>-6100</x:v>
+      </x:c>
+      <x:c r="I6" s="24" t="n">
+        <x:v>-0.039354838709677376</x:v>
+      </x:c>
+      <x:c r="J6" s="26" t="n">
+        <x:f>ROUND(E6-F6,1)</x:f>
+        <x:v>6720</x:v>
+      </x:c>
+      <x:c r="K6" s="22" t="str">
+        <x:v>LC2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B9" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B9" s="28" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="C9" s="28"/>
       <x:c r="D9" s="28"/>
       <x:c r="E9" s="28"/>
@@ -1007,11 +1025,29 @@
       <x:c r="G9" s="28"/>
       <x:c r="H9" s="28"/>
       <x:c r="I9" s="28"/>
-      <x:c r="J9" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J5),0),1)</x:f>
-        <x:v>4020</x:v>
+      <x:c r="J9" s="30" t="n">
+        <x:f>SUM(J4:J6)</x:f>
+        <x:v>14760</x:v>
       </x:c>
       <x:c r="K9" s="28"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B10" s="28"/>
+      <x:c r="C10" s="28"/>
+      <x:c r="D10" s="28"/>
+      <x:c r="E10" s="28"/>
+      <x:c r="F10" s="28"/>
+      <x:c r="G10" s="28"/>
+      <x:c r="H10" s="28"/>
+      <x:c r="I10" s="28"/>
+      <x:c r="J10" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J6),0),1)</x:f>
+        <x:v>4920</x:v>
+      </x:c>
+      <x:c r="K10" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1098,7 +1134,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B5" s="22" t="str">
-        <x:v>9月1日-9月2日</x:v>
+        <x:v>9月1日-9月3日</x:v>
       </x:c>
       <x:c r="C5" s="23" t="n">
         <x:v>7773.06</x:v>
@@ -1107,22 +1143,22 @@
         <x:v>7773.06</x:v>
       </x:c>
       <x:c r="E5" s="23" t="n">
-        <x:v>7539.08</x:v>
+        <x:v>7531.67</x:v>
       </x:c>
       <x:c r="F5" s="23" t="n">
-        <x:v>7583.76</x:v>
+        <x:v>7600.1</x:v>
       </x:c>
       <x:c r="G5" s="23"/>
       <x:c r="H5" s="24"/>
       <x:c r="I5" s="26" t="n">
         <x:f>ROUND(D5-E5,1)</x:f>
-        <x:v>234</x:v>
+        <x:v>241.4</x:v>
       </x:c>
       <x:c r="J5" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K5" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -1140,7 +1176,7 @@
       <x:c r="H6" s="28"/>
       <x:c r="I6" s="30" t="n">
         <x:f>ROUND(SUM(I5:I5),1)</x:f>
-        <x:v>234</x:v>
+        <x:v>241.4</x:v>
       </x:c>
       <x:c r="J6" s="28"/>
       <x:c r="K6" s="28"/>
@@ -1158,7 +1194,7 @@
       <x:c r="H7" s="28"/>
       <x:c r="I7" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I5),0),1)</x:f>
-        <x:v>234</x:v>
+        <x:v>241.4</x:v>
       </x:c>
       <x:c r="J7" s="28"/>
       <x:c r="K7" s="28"/>
@@ -1218,7 +1254,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B11" s="22" t="str">
-        <x:v>9月1日-9月2日</x:v>
+        <x:v>9月1日-9月3日</x:v>
       </x:c>
       <x:c r="C11" s="23" t="n">
         <x:v>7944.29</x:v>
@@ -1227,22 +1263,22 @@
         <x:v>7955.57</x:v>
       </x:c>
       <x:c r="E11" s="23" t="n">
-        <x:v>7692.15</x:v>
+        <x:v>7686.44</x:v>
       </x:c>
       <x:c r="F11" s="23" t="n">
-        <x:v>7729.23</x:v>
+        <x:v>7755.36</x:v>
       </x:c>
       <x:c r="G11" s="23"/>
       <x:c r="H11" s="24"/>
       <x:c r="I11" s="26" t="n">
         <x:f>ROUND(D11-E11,1)</x:f>
-        <x:v>263.4</x:v>
+        <x:v>269.1</x:v>
       </x:c>
       <x:c r="J11" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K11" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -1260,7 +1296,7 @@
       <x:c r="H12" s="28"/>
       <x:c r="I12" s="30" t="n">
         <x:f>ROUND(SUM(I11:I11),1)</x:f>
-        <x:v>263.4</x:v>
+        <x:v>269.1</x:v>
       </x:c>
       <x:c r="J12" s="28"/>
       <x:c r="K12" s="28"/>
@@ -1278,7 +1314,7 @@
       <x:c r="H13" s="28"/>
       <x:c r="I13" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I11:I11),0),1)</x:f>
-        <x:v>263.4</x:v>
+        <x:v>269.1</x:v>
       </x:c>
       <x:c r="J13" s="28"/>
       <x:c r="K13" s="28"/>
@@ -1338,7 +1374,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B17" s="22" t="str">
-        <x:v>9月1日-9月2日</x:v>
+        <x:v>9月1日-9月3日</x:v>
       </x:c>
       <x:c r="C17" s="23" t="n">
         <x:v>3979.88</x:v>
@@ -1347,22 +1383,22 @@
         <x:v>3995.18</x:v>
       </x:c>
       <x:c r="E17" s="23" t="n">
-        <x:v>3932.25</x:v>
+        <x:v>3930.45</x:v>
       </x:c>
       <x:c r="F17" s="23" t="n">
-        <x:v>3941.39</x:v>
+        <x:v>3942.09</x:v>
       </x:c>
       <x:c r="G17" s="23"/>
       <x:c r="H17" s="24"/>
       <x:c r="I17" s="26" t="n">
         <x:f>ROUND(D17-E17,1)</x:f>
-        <x:v>62.9</x:v>
+        <x:v>64.7</x:v>
       </x:c>
       <x:c r="J17" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K17" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -1380,7 +1416,7 @@
       <x:c r="H18" s="28"/>
       <x:c r="I18" s="30" t="n">
         <x:f>ROUND(SUM(I17:I17),1)</x:f>
-        <x:v>62.9</x:v>
+        <x:v>64.7</x:v>
       </x:c>
       <x:c r="J18" s="28"/>
       <x:c r="K18" s="28"/>
@@ -1398,7 +1434,7 @@
       <x:c r="H19" s="28"/>
       <x:c r="I19" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I17:I17),0),1)</x:f>
-        <x:v>62.9</x:v>
+        <x:v>64.7</x:v>
       </x:c>
       <x:c r="J19" s="28"/>
       <x:c r="K19" s="28"/>
@@ -1578,7 +1614,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B29" s="22" t="str">
-        <x:v>9月1日-9月2日</x:v>
+        <x:v>9月1日-9月3日</x:v>
       </x:c>
       <x:c r="C29" s="23" t="n">
         <x:v>7880.8</x:v>
@@ -1590,7 +1626,7 @@
         <x:v>7593</x:v>
       </x:c>
       <x:c r="F29" s="23" t="n">
-        <x:v>7675.6</x:v>
+        <x:v>7706.2</x:v>
       </x:c>
       <x:c r="G29" s="23"/>
       <x:c r="H29" s="24"/>
@@ -1602,7 +1638,7 @@
         <x:v>IC2609</x:v>
       </x:c>
       <x:c r="K29" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -1698,7 +1734,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B35" s="22" t="str">
-        <x:v>9月1日-9月2日</x:v>
+        <x:v>9月1日-9月3日</x:v>
       </x:c>
       <x:c r="C35" s="23" t="n">
         <x:v>4602</x:v>
@@ -1710,7 +1746,7 @@
         <x:v>4497.6</x:v>
       </x:c>
       <x:c r="F35" s="23" t="n">
-        <x:v>4532.2</x:v>
+        <x:v>4536.8</x:v>
       </x:c>
       <x:c r="G35" s="23"/>
       <x:c r="H35" s="24"/>
@@ -1722,7 +1758,7 @@
         <x:v>IF2609</x:v>
       </x:c>
       <x:c r="K35" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -1818,7 +1854,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B41" s="22" t="str">
-        <x:v>9月1日-9月2日</x:v>
+        <x:v>9月1日-9月3日</x:v>
       </x:c>
       <x:c r="C41" s="23" t="n">
         <x:v>2913</x:v>
@@ -1830,7 +1866,7 @@
         <x:v>2881.4</x:v>
       </x:c>
       <x:c r="F41" s="23" t="n">
-        <x:v>2898.8</x:v>
+        <x:v>2907.6</x:v>
       </x:c>
       <x:c r="G41" s="23"/>
       <x:c r="H41" s="24"/>
@@ -1842,7 +1878,7 @@
         <x:v>IH2609</x:v>
       </x:c>
       <x:c r="K41" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -1938,7 +1974,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B47" s="22" t="str">
-        <x:v>9月1日-9月2日</x:v>
+        <x:v>9月1日-9月3日</x:v>
       </x:c>
       <x:c r="C47" s="23" t="n">
         <x:v>159000</x:v>
@@ -1947,22 +1983,22 @@
         <x:v>160480</x:v>
       </x:c>
       <x:c r="E47" s="23" t="n">
-        <x:v>152840</x:v>
+        <x:v>148880</x:v>
       </x:c>
       <x:c r="F47" s="23" t="n">
-        <x:v>155000</x:v>
+        <x:v>148900</x:v>
       </x:c>
       <x:c r="G47" s="23"/>
       <x:c r="H47" s="24"/>
       <x:c r="I47" s="26" t="n">
         <x:f>ROUND(D47-E47,1)</x:f>
-        <x:v>7640</x:v>
+        <x:v>11600</x:v>
       </x:c>
       <x:c r="J47" s="22" t="str">
         <x:v>LC2609</x:v>
       </x:c>
       <x:c r="K47" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -1980,7 +2016,7 @@
       <x:c r="H48" s="28"/>
       <x:c r="I48" s="30" t="n">
         <x:f>ROUND(SUM(I47:I47),1)</x:f>
-        <x:v>7640</x:v>
+        <x:v>11600</x:v>
       </x:c>
       <x:c r="J48" s="28"/>
       <x:c r="K48" s="28"/>
@@ -1998,7 +2034,7 @@
       <x:c r="H49" s="28"/>
       <x:c r="I49" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I47:I47),0),1)</x:f>
-        <x:v>7640</x:v>
+        <x:v>11600</x:v>
       </x:c>
       <x:c r="J49" s="28"/>
       <x:c r="K49" s="28"/>
@@ -2148,31 +2184,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B8" s="28" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C8" s="28"/>
-      <x:c r="D8" s="28"/>
-      <x:c r="E8" s="28"/>
-      <x:c r="F8" s="28"/>
-      <x:c r="G8" s="28"/>
-      <x:c r="H8" s="28"/>
-      <x:c r="I8" s="28"/>
-      <x:c r="J8" s="30" t="n">
-        <x:f>SUM(J4:J5)</x:f>
-        <x:v>191.3</x:v>
-      </x:c>
-      <x:c r="K8" s="28"/>
+    <x:row r="6">
+      <x:c r="A6" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B6" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C6" s="22" t="str">
+        <x:v>9月3日</x:v>
+      </x:c>
+      <x:c r="D6" s="23" t="n">
+        <x:v>7629.65</x:v>
+      </x:c>
+      <x:c r="E6" s="23" t="n">
+        <x:v>7657.75</x:v>
+      </x:c>
+      <x:c r="F6" s="23" t="n">
+        <x:v>7531.67</x:v>
+      </x:c>
+      <x:c r="G6" s="23" t="n">
+        <x:v>7600.1</x:v>
+      </x:c>
+      <x:c r="H6" s="23" t="n">
+        <x:v>16.3</x:v>
+      </x:c>
+      <x:c r="I6" s="24" t="n">
+        <x:v>0.0021546040486513096</x:v>
+      </x:c>
+      <x:c r="J6" s="23" t="n">
+        <x:f>ROUND(E6-F6,1)</x:f>
+        <x:v>126.1</x:v>
+      </x:c>
+      <x:c r="K6" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B9" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B9" s="28" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="C9" s="28"/>
       <x:c r="D9" s="28"/>
       <x:c r="E9" s="28"/>
@@ -2180,11 +2234,29 @@
       <x:c r="G9" s="28"/>
       <x:c r="H9" s="28"/>
       <x:c r="I9" s="28"/>
-      <x:c r="J9" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J5),0),1)</x:f>
-        <x:v>95.7</x:v>
+      <x:c r="J9" s="30" t="n">
+        <x:f>SUM(J4:J6)</x:f>
+        <x:v>317.4</x:v>
       </x:c>
       <x:c r="K9" s="28"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B10" s="28"/>
+      <x:c r="C10" s="28"/>
+      <x:c r="D10" s="28"/>
+      <x:c r="E10" s="28"/>
+      <x:c r="F10" s="28"/>
+      <x:c r="G10" s="28"/>
+      <x:c r="H10" s="28"/>
+      <x:c r="I10" s="28"/>
+      <x:c r="J10" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J6),0),1)</x:f>
+        <x:v>105.8</x:v>
+      </x:c>
+      <x:c r="K10" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2323,31 +2395,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B8" s="28" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C8" s="28"/>
-      <x:c r="D8" s="28"/>
-      <x:c r="E8" s="28"/>
-      <x:c r="F8" s="28"/>
-      <x:c r="G8" s="28"/>
-      <x:c r="H8" s="28"/>
-      <x:c r="I8" s="28"/>
-      <x:c r="J8" s="30" t="n">
-        <x:f>SUM(J4:J5)</x:f>
-        <x:v>193.60000000000002</x:v>
-      </x:c>
-      <x:c r="K8" s="28"/>
+    <x:row r="6">
+      <x:c r="A6" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B6" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C6" s="22" t="str">
+        <x:v>9月3日</x:v>
+      </x:c>
+      <x:c r="D6" s="23" t="n">
+        <x:v>7776.82</x:v>
+      </x:c>
+      <x:c r="E6" s="23" t="n">
+        <x:v>7799.63</x:v>
+      </x:c>
+      <x:c r="F6" s="23" t="n">
+        <x:v>7686.44</x:v>
+      </x:c>
+      <x:c r="G6" s="23" t="n">
+        <x:v>7755.36</x:v>
+      </x:c>
+      <x:c r="H6" s="23" t="n">
+        <x:v>26.1</x:v>
+      </x:c>
+      <x:c r="I6" s="24" t="n">
+        <x:v>0.003380673107153065</x:v>
+      </x:c>
+      <x:c r="J6" s="23" t="n">
+        <x:f>ROUND(E6-F6,1)</x:f>
+        <x:v>113.2</x:v>
+      </x:c>
+      <x:c r="K6" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B9" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B9" s="28" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="C9" s="28"/>
       <x:c r="D9" s="28"/>
       <x:c r="E9" s="28"/>
@@ -2355,11 +2445,29 @@
       <x:c r="G9" s="28"/>
       <x:c r="H9" s="28"/>
       <x:c r="I9" s="28"/>
-      <x:c r="J9" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J5),0),1)</x:f>
-        <x:v>96.8</x:v>
+      <x:c r="J9" s="30" t="n">
+        <x:f>SUM(J4:J6)</x:f>
+        <x:v>306.8</x:v>
       </x:c>
       <x:c r="K9" s="28"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B10" s="28"/>
+      <x:c r="C10" s="28"/>
+      <x:c r="D10" s="28"/>
+      <x:c r="E10" s="28"/>
+      <x:c r="F10" s="28"/>
+      <x:c r="G10" s="28"/>
+      <x:c r="H10" s="28"/>
+      <x:c r="I10" s="28"/>
+      <x:c r="J10" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J6),0),1)</x:f>
+        <x:v>102.3</x:v>
+      </x:c>
+      <x:c r="K10" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2498,31 +2606,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B8" s="28" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C8" s="28"/>
-      <x:c r="D8" s="28"/>
-      <x:c r="E8" s="28"/>
-      <x:c r="F8" s="28"/>
-      <x:c r="G8" s="28"/>
-      <x:c r="H8" s="28"/>
-      <x:c r="I8" s="28"/>
-      <x:c r="J8" s="30" t="n">
-        <x:f>SUM(J4:J5)</x:f>
-        <x:v>52.3</x:v>
-      </x:c>
-      <x:c r="K8" s="28"/>
+    <x:row r="6">
+      <x:c r="A6" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B6" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C6" s="22" t="str">
+        <x:v>9月3日</x:v>
+      </x:c>
+      <x:c r="D6" s="23" t="n">
+        <x:v>3952.79</x:v>
+      </x:c>
+      <x:c r="E6" s="23" t="n">
+        <x:v>3968.11</x:v>
+      </x:c>
+      <x:c r="F6" s="23" t="n">
+        <x:v>3930.45</x:v>
+      </x:c>
+      <x:c r="G6" s="23" t="n">
+        <x:v>3942.09</x:v>
+      </x:c>
+      <x:c r="H6" s="23" t="n">
+        <x:v>0.7</x:v>
+      </x:c>
+      <x:c r="I6" s="24" t="n">
+        <x:v>0.0001776023179640429</x:v>
+      </x:c>
+      <x:c r="J6" s="23" t="n">
+        <x:f>ROUND(E6-F6,1)</x:f>
+        <x:v>37.7</x:v>
+      </x:c>
+      <x:c r="K6" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B9" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B9" s="28" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="C9" s="28"/>
       <x:c r="D9" s="28"/>
       <x:c r="E9" s="28"/>
@@ -2530,11 +2656,29 @@
       <x:c r="G9" s="28"/>
       <x:c r="H9" s="28"/>
       <x:c r="I9" s="28"/>
-      <x:c r="J9" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J5),0),1)</x:f>
-        <x:v>26.2</x:v>
+      <x:c r="J9" s="30" t="n">
+        <x:f>SUM(J4:J6)</x:f>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="K9" s="28"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B10" s="28"/>
+      <x:c r="C10" s="28"/>
+      <x:c r="D10" s="28"/>
+      <x:c r="E10" s="28"/>
+      <x:c r="F10" s="28"/>
+      <x:c r="G10" s="28"/>
+      <x:c r="H10" s="28"/>
+      <x:c r="I10" s="28"/>
+      <x:c r="J10" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J6),0),1)</x:f>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="K10" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2848,31 +2992,49 @@
         <x:v>IC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B8" s="28" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C8" s="28"/>
-      <x:c r="D8" s="28"/>
-      <x:c r="E8" s="28"/>
-      <x:c r="F8" s="28"/>
-      <x:c r="G8" s="28"/>
-      <x:c r="H8" s="28"/>
-      <x:c r="I8" s="28"/>
-      <x:c r="J8" s="30" t="n">
-        <x:f>SUM(J4:J5)</x:f>
-        <x:v>265</x:v>
-      </x:c>
-      <x:c r="K8" s="28"/>
+    <x:row r="6">
+      <x:c r="A6" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B6" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C6" s="22" t="str">
+        <x:v>9月3日</x:v>
+      </x:c>
+      <x:c r="D6" s="23" t="n">
+        <x:v>7720</x:v>
+      </x:c>
+      <x:c r="E6" s="23" t="n">
+        <x:v>7752.8</x:v>
+      </x:c>
+      <x:c r="F6" s="23" t="n">
+        <x:v>7601.6</x:v>
+      </x:c>
+      <x:c r="G6" s="23" t="n">
+        <x:v>7706.2</x:v>
+      </x:c>
+      <x:c r="H6" s="23" t="n">
+        <x:v>30.6</x:v>
+      </x:c>
+      <x:c r="I6" s="24" t="n">
+        <x:v>0.003986659023398786</x:v>
+      </x:c>
+      <x:c r="J6" s="26" t="n">
+        <x:f>ROUND(E6-F6,1)</x:f>
+        <x:v>151.2</x:v>
+      </x:c>
+      <x:c r="K6" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B9" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B9" s="28" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="C9" s="28"/>
       <x:c r="D9" s="28"/>
       <x:c r="E9" s="28"/>
@@ -2880,11 +3042,29 @@
       <x:c r="G9" s="28"/>
       <x:c r="H9" s="28"/>
       <x:c r="I9" s="28"/>
-      <x:c r="J9" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J5),0),1)</x:f>
-        <x:v>132.5</x:v>
+      <x:c r="J9" s="30" t="n">
+        <x:f>SUM(J4:J6)</x:f>
+        <x:v>416.2</x:v>
       </x:c>
       <x:c r="K9" s="28"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B10" s="28"/>
+      <x:c r="C10" s="28"/>
+      <x:c r="D10" s="28"/>
+      <x:c r="E10" s="28"/>
+      <x:c r="F10" s="28"/>
+      <x:c r="G10" s="28"/>
+      <x:c r="H10" s="28"/>
+      <x:c r="I10" s="28"/>
+      <x:c r="J10" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J6),0),1)</x:f>
+        <x:v>138.7</x:v>
+      </x:c>
+      <x:c r="K10" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3023,31 +3203,49 @@
         <x:v>IF2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B8" s="28" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C8" s="28"/>
-      <x:c r="D8" s="28"/>
-      <x:c r="E8" s="28"/>
-      <x:c r="F8" s="28"/>
-      <x:c r="G8" s="28"/>
-      <x:c r="H8" s="28"/>
-      <x:c r="I8" s="28"/>
-      <x:c r="J8" s="30" t="n">
-        <x:f>SUM(J4:J5)</x:f>
-        <x:v>111.2</x:v>
-      </x:c>
-      <x:c r="K8" s="28"/>
+    <x:row r="6">
+      <x:c r="A6" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B6" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C6" s="22" t="str">
+        <x:v>9月3日</x:v>
+      </x:c>
+      <x:c r="D6" s="23" t="n">
+        <x:v>4541</x:v>
+      </x:c>
+      <x:c r="E6" s="23" t="n">
+        <x:v>4561.2</x:v>
+      </x:c>
+      <x:c r="F6" s="23" t="n">
+        <x:v>4510.4</x:v>
+      </x:c>
+      <x:c r="G6" s="23" t="n">
+        <x:v>4536.8</x:v>
+      </x:c>
+      <x:c r="H6" s="23" t="n">
+        <x:v>4.6</x:v>
+      </x:c>
+      <x:c r="I6" s="24" t="n">
+        <x:v>0.0010149596222586155</x:v>
+      </x:c>
+      <x:c r="J6" s="23" t="n">
+        <x:f>ROUND(E6-F6,1)</x:f>
+        <x:v>50.8</x:v>
+      </x:c>
+      <x:c r="K6" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B9" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B9" s="28" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="C9" s="28"/>
       <x:c r="D9" s="28"/>
       <x:c r="E9" s="28"/>
@@ -3055,11 +3253,29 @@
       <x:c r="G9" s="28"/>
       <x:c r="H9" s="28"/>
       <x:c r="I9" s="28"/>
-      <x:c r="J9" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J5),0),1)</x:f>
-        <x:v>55.6</x:v>
+      <x:c r="J9" s="30" t="n">
+        <x:f>SUM(J4:J6)</x:f>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="K9" s="28"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B10" s="28"/>
+      <x:c r="C10" s="28"/>
+      <x:c r="D10" s="28"/>
+      <x:c r="E10" s="28"/>
+      <x:c r="F10" s="28"/>
+      <x:c r="G10" s="28"/>
+      <x:c r="H10" s="28"/>
+      <x:c r="I10" s="28"/>
+      <x:c r="J10" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J6),0),1)</x:f>
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="K10" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3198,31 +3414,49 @@
         <x:v>IH2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B8" s="28" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C8" s="28"/>
-      <x:c r="D8" s="28"/>
-      <x:c r="E8" s="28"/>
-      <x:c r="F8" s="28"/>
-      <x:c r="G8" s="28"/>
-      <x:c r="H8" s="28"/>
-      <x:c r="I8" s="28"/>
-      <x:c r="J8" s="30" t="n">
-        <x:f>SUM(J4:J5)</x:f>
-        <x:v>58.8</x:v>
-      </x:c>
-      <x:c r="K8" s="28"/>
+    <x:row r="6">
+      <x:c r="A6" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B6" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C6" s="22" t="str">
+        <x:v>9月3日</x:v>
+      </x:c>
+      <x:c r="D6" s="23" t="n">
+        <x:v>2909.2</x:v>
+      </x:c>
+      <x:c r="E6" s="23" t="n">
+        <x:v>2922.8</x:v>
+      </x:c>
+      <x:c r="F6" s="23" t="n">
+        <x:v>2893.6</x:v>
+      </x:c>
+      <x:c r="G6" s="23" t="n">
+        <x:v>2907.6</x:v>
+      </x:c>
+      <x:c r="H6" s="23" t="n">
+        <x:v>8.8</x:v>
+      </x:c>
+      <x:c r="I6" s="24" t="n">
+        <x:v>0.0030357389264521473</x:v>
+      </x:c>
+      <x:c r="J6" s="23" t="n">
+        <x:f>ROUND(E6-F6,1)</x:f>
+        <x:v>29.2</x:v>
+      </x:c>
+      <x:c r="K6" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B9" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B9" s="28" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="C9" s="28"/>
       <x:c r="D9" s="28"/>
       <x:c r="E9" s="28"/>
@@ -3230,11 +3464,29 @@
       <x:c r="G9" s="28"/>
       <x:c r="H9" s="28"/>
       <x:c r="I9" s="28"/>
-      <x:c r="J9" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J5),0),1)</x:f>
-        <x:v>29.4</x:v>
+      <x:c r="J9" s="30" t="n">
+        <x:f>SUM(J4:J6)</x:f>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="K9" s="28"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B10" s="28"/>
+      <x:c r="C10" s="28"/>
+      <x:c r="D10" s="28"/>
+      <x:c r="E10" s="28"/>
+      <x:c r="F10" s="28"/>
+      <x:c r="G10" s="28"/>
+      <x:c r="H10" s="28"/>
+      <x:c r="I10" s="28"/>
+      <x:c r="J10" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J6),0),1)</x:f>
+        <x:v>29.3</x:v>
+      </x:c>
+      <x:c r="K10" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-09-04
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rfa6d45977f554ef7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R0443400a908f4069"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Rd91fb2ca62ff4c48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R8dd738705d0c40c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R7548f9043010497a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R8fa249a2770e4fce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Ra5b185bf11ec4f60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rb9b84f2fd55d4922"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Ra8f9c7c192844aeb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="Ref96d2818adc4354"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rbd9d10c53e5b472b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Rfd933b48cf6f4629"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R6c5aa6aeca2443ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R415475a021754e03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R11337a5994714f68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rb2f5e7c8d2af412b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R95338373ab0e47d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R48c0800b23fe446b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rf4a389c57eee41b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="Rbdb24296d77a4b09"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -485,25 +485,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-09-03</x:v>
+        <x:v>2026-09-04</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7657.75</x:v>
+        <x:v>7717.93</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7531.67</x:v>
+        <x:v>7464.98</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>126.1</x:v>
+        <x:v>253</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>317.4</x:v>
+        <x:v>570.4</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>105.8</x:v>
+        <x:v>142.6</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -514,25 +514,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-09-03</x:v>
+        <x:v>2026-09-04</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7799.63</x:v>
+        <x:v>7850.4</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7686.44</x:v>
+        <x:v>7610.58</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>113.2</x:v>
+        <x:v>239.8</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>306.8</x:v>
+        <x:v>546.6</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>102.3</x:v>
+        <x:v>136.7</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -543,25 +543,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-09-03</x:v>
+        <x:v>2026-09-04</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3968.11</x:v>
+        <x:v>3980.2</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3930.45</x:v>
+        <x:v>3915.22</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>37.7</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>90</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>30</x:v>
+        <x:v>38.8</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -659,25 +659,25 @@
         <x:v>IH主力</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>2026-09-03</x:v>
+        <x:v>2026-09-04</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:v>2922.8</x:v>
+        <x:v>2949.4</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
-        <x:v>2893.6</x:v>
+        <x:v>2904.8</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
-        <x:v>29.2</x:v>
+        <x:v>44.6</x:v>
       </x:c>
       <x:c r="F10" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G10" s="10" t="n">
-        <x:v>88</x:v>
+        <x:v>132.6</x:v>
       </x:c>
       <x:c r="H10" s="10" t="n">
-        <x:v>29.3</x:v>
+        <x:v>33.2</x:v>
       </x:c>
       <x:c r="I10" s="10" t="n">
         <x:v>60</x:v>
@@ -688,25 +688,25 @@
         <x:v>碳酸锂2609</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>2026-09-03</x:v>
+        <x:v>2026-09-04</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:v>155600</x:v>
+        <x:v>152400</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
-        <x:v>148880</x:v>
+        <x:v>140940</x:v>
       </x:c>
       <x:c r="E11" s="12" t="n">
-        <x:v>6720</x:v>
+        <x:v>11460</x:v>
       </x:c>
       <x:c r="F11" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G11" s="10" t="n">
-        <x:v>14760</x:v>
+        <x:v>26220</x:v>
       </x:c>
       <x:c r="H11" s="10" t="n">
-        <x:v>4920</x:v>
+        <x:v>6555</x:v>
       </x:c>
       <x:c r="I11" s="10" t="n">
         <x:v>6000</x:v>
@@ -720,7 +720,7 @@
         <x:v>2026-09-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-09-03</x:v>
+        <x:v>2026-09-04</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1011,31 +1011,49 @@
         <x:v>LC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B9" s="28" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C9" s="28"/>
-      <x:c r="D9" s="28"/>
-      <x:c r="E9" s="28"/>
-      <x:c r="F9" s="28"/>
-      <x:c r="G9" s="28"/>
-      <x:c r="H9" s="28"/>
-      <x:c r="I9" s="28"/>
-      <x:c r="J9" s="30" t="n">
-        <x:f>SUM(J4:J6)</x:f>
-        <x:v>14760</x:v>
-      </x:c>
-      <x:c r="K9" s="28"/>
+    <x:row r="7">
+      <x:c r="A7" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C7" s="22" t="str">
+        <x:v>9月4日</x:v>
+      </x:c>
+      <x:c r="D7" s="23" t="n">
+        <x:v>152400</x:v>
+      </x:c>
+      <x:c r="E7" s="23" t="n">
+        <x:v>152400</x:v>
+      </x:c>
+      <x:c r="F7" s="23" t="n">
+        <x:v>140940</x:v>
+      </x:c>
+      <x:c r="G7" s="23" t="n">
+        <x:v>140980</x:v>
+      </x:c>
+      <x:c r="H7" s="38" t="n">
+        <x:v>-7920</x:v>
+      </x:c>
+      <x:c r="I7" s="24" t="n">
+        <x:v>-0.053190060443250475</x:v>
+      </x:c>
+      <x:c r="J7" s="26" t="n">
+        <x:f>ROUND(E7-F7,1)</x:f>
+        <x:v>11460</x:v>
+      </x:c>
+      <x:c r="K7" s="22" t="str">
+        <x:v>LC2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B10" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B10" s="28" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="C10" s="28"/>
       <x:c r="D10" s="28"/>
       <x:c r="E10" s="28"/>
@@ -1043,11 +1061,29 @@
       <x:c r="G10" s="28"/>
       <x:c r="H10" s="28"/>
       <x:c r="I10" s="28"/>
-      <x:c r="J10" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J6),0),1)</x:f>
-        <x:v>4920</x:v>
+      <x:c r="J10" s="30" t="n">
+        <x:f>SUM(J4:J7)</x:f>
+        <x:v>26220</x:v>
       </x:c>
       <x:c r="K10" s="28"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B11" s="28"/>
+      <x:c r="C11" s="28"/>
+      <x:c r="D11" s="28"/>
+      <x:c r="E11" s="28"/>
+      <x:c r="F11" s="28"/>
+      <x:c r="G11" s="28"/>
+      <x:c r="H11" s="28"/>
+      <x:c r="I11" s="28"/>
+      <x:c r="J11" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
+        <x:v>6555</x:v>
+      </x:c>
+      <x:c r="K11" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1134,7 +1170,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B5" s="22" t="str">
-        <x:v>9月1日-9月3日</x:v>
+        <x:v>9月1日-9月4日</x:v>
       </x:c>
       <x:c r="C5" s="23" t="n">
         <x:v>7773.06</x:v>
@@ -1143,22 +1179,22 @@
         <x:v>7773.06</x:v>
       </x:c>
       <x:c r="E5" s="23" t="n">
-        <x:v>7531.67</x:v>
+        <x:v>7464.98</x:v>
       </x:c>
       <x:c r="F5" s="23" t="n">
-        <x:v>7600.1</x:v>
+        <x:v>7508.09</x:v>
       </x:c>
       <x:c r="G5" s="23"/>
       <x:c r="H5" s="24"/>
       <x:c r="I5" s="26" t="n">
         <x:f>ROUND(D5-E5,1)</x:f>
-        <x:v>241.4</x:v>
+        <x:v>308.1</x:v>
       </x:c>
       <x:c r="J5" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K5" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -1176,7 +1212,7 @@
       <x:c r="H6" s="28"/>
       <x:c r="I6" s="30" t="n">
         <x:f>ROUND(SUM(I5:I5),1)</x:f>
-        <x:v>241.4</x:v>
+        <x:v>308.1</x:v>
       </x:c>
       <x:c r="J6" s="28"/>
       <x:c r="K6" s="28"/>
@@ -1194,7 +1230,7 @@
       <x:c r="H7" s="28"/>
       <x:c r="I7" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I5),0),1)</x:f>
-        <x:v>241.4</x:v>
+        <x:v>308.1</x:v>
       </x:c>
       <x:c r="J7" s="28"/>
       <x:c r="K7" s="28"/>
@@ -1254,7 +1290,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B11" s="22" t="str">
-        <x:v>9月1日-9月3日</x:v>
+        <x:v>9月1日-9月4日</x:v>
       </x:c>
       <x:c r="C11" s="23" t="n">
         <x:v>7944.29</x:v>
@@ -1263,22 +1299,22 @@
         <x:v>7955.57</x:v>
       </x:c>
       <x:c r="E11" s="23" t="n">
-        <x:v>7686.44</x:v>
+        <x:v>7610.58</x:v>
       </x:c>
       <x:c r="F11" s="23" t="n">
-        <x:v>7755.36</x:v>
+        <x:v>7652.69</x:v>
       </x:c>
       <x:c r="G11" s="23"/>
       <x:c r="H11" s="24"/>
       <x:c r="I11" s="26" t="n">
         <x:f>ROUND(D11-E11,1)</x:f>
-        <x:v>269.1</x:v>
+        <x:v>345</x:v>
       </x:c>
       <x:c r="J11" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K11" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -1296,7 +1332,7 @@
       <x:c r="H12" s="28"/>
       <x:c r="I12" s="30" t="n">
         <x:f>ROUND(SUM(I11:I11),1)</x:f>
-        <x:v>269.1</x:v>
+        <x:v>345</x:v>
       </x:c>
       <x:c r="J12" s="28"/>
       <x:c r="K12" s="28"/>
@@ -1314,7 +1350,7 @@
       <x:c r="H13" s="28"/>
       <x:c r="I13" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I11:I11),0),1)</x:f>
-        <x:v>269.1</x:v>
+        <x:v>345</x:v>
       </x:c>
       <x:c r="J13" s="28"/>
       <x:c r="K13" s="28"/>
@@ -1374,7 +1410,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B17" s="22" t="str">
-        <x:v>9月1日-9月3日</x:v>
+        <x:v>9月1日-9月4日</x:v>
       </x:c>
       <x:c r="C17" s="23" t="n">
         <x:v>3979.88</x:v>
@@ -1383,22 +1419,22 @@
         <x:v>3995.18</x:v>
       </x:c>
       <x:c r="E17" s="23" t="n">
-        <x:v>3930.45</x:v>
+        <x:v>3915.22</x:v>
       </x:c>
       <x:c r="F17" s="23" t="n">
-        <x:v>3942.09</x:v>
+        <x:v>3930.12</x:v>
       </x:c>
       <x:c r="G17" s="23"/>
       <x:c r="H17" s="24"/>
       <x:c r="I17" s="26" t="n">
         <x:f>ROUND(D17-E17,1)</x:f>
-        <x:v>64.7</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="J17" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K17" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -1416,7 +1452,7 @@
       <x:c r="H18" s="28"/>
       <x:c r="I18" s="30" t="n">
         <x:f>ROUND(SUM(I17:I17),1)</x:f>
-        <x:v>64.7</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="J18" s="28"/>
       <x:c r="K18" s="28"/>
@@ -1434,7 +1470,7 @@
       <x:c r="H19" s="28"/>
       <x:c r="I19" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I17:I17),0),1)</x:f>
-        <x:v>64.7</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="J19" s="28"/>
       <x:c r="K19" s="28"/>
@@ -1854,31 +1890,31 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B41" s="22" t="str">
-        <x:v>9月1日-9月3日</x:v>
+        <x:v>9月1日-9月4日</x:v>
       </x:c>
       <x:c r="C41" s="23" t="n">
         <x:v>2913</x:v>
       </x:c>
       <x:c r="D41" s="23" t="n">
-        <x:v>2934.8</x:v>
+        <x:v>2949.4</x:v>
       </x:c>
       <x:c r="E41" s="23" t="n">
         <x:v>2881.4</x:v>
       </x:c>
       <x:c r="F41" s="23" t="n">
-        <x:v>2907.6</x:v>
+        <x:v>2915.8</x:v>
       </x:c>
       <x:c r="G41" s="23"/>
       <x:c r="H41" s="24"/>
-      <x:c r="I41" s="23" t="n">
+      <x:c r="I41" s="26" t="n">
         <x:f>ROUND(D41-E41,1)</x:f>
-        <x:v>53.4</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="J41" s="22" t="str">
         <x:v>IH2609</x:v>
       </x:c>
       <x:c r="K41" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -1896,7 +1932,7 @@
       <x:c r="H42" s="28"/>
       <x:c r="I42" s="30" t="n">
         <x:f>ROUND(SUM(I41:I41),1)</x:f>
-        <x:v>53.4</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="J42" s="28"/>
       <x:c r="K42" s="28"/>
@@ -1914,7 +1950,7 @@
       <x:c r="H43" s="28"/>
       <x:c r="I43" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I41:I41),0),1)</x:f>
-        <x:v>53.4</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="J43" s="28"/>
       <x:c r="K43" s="28"/>
@@ -1974,7 +2010,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B47" s="22" t="str">
-        <x:v>9月1日-9月3日</x:v>
+        <x:v>9月1日-9月4日</x:v>
       </x:c>
       <x:c r="C47" s="23" t="n">
         <x:v>159000</x:v>
@@ -1983,22 +2019,22 @@
         <x:v>160480</x:v>
       </x:c>
       <x:c r="E47" s="23" t="n">
-        <x:v>148880</x:v>
+        <x:v>140940</x:v>
       </x:c>
       <x:c r="F47" s="23" t="n">
-        <x:v>148900</x:v>
+        <x:v>140980</x:v>
       </x:c>
       <x:c r="G47" s="23"/>
       <x:c r="H47" s="24"/>
       <x:c r="I47" s="26" t="n">
         <x:f>ROUND(D47-E47,1)</x:f>
-        <x:v>11600</x:v>
+        <x:v>19540</x:v>
       </x:c>
       <x:c r="J47" s="22" t="str">
         <x:v>LC2609</x:v>
       </x:c>
       <x:c r="K47" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -2016,7 +2052,7 @@
       <x:c r="H48" s="28"/>
       <x:c r="I48" s="30" t="n">
         <x:f>ROUND(SUM(I47:I47),1)</x:f>
-        <x:v>11600</x:v>
+        <x:v>19540</x:v>
       </x:c>
       <x:c r="J48" s="28"/>
       <x:c r="K48" s="28"/>
@@ -2034,7 +2070,7 @@
       <x:c r="H49" s="28"/>
       <x:c r="I49" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I47:I47),0),1)</x:f>
-        <x:v>11600</x:v>
+        <x:v>19540</x:v>
       </x:c>
       <x:c r="J49" s="28"/>
       <x:c r="K49" s="28"/>
@@ -2220,31 +2256,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B9" s="28" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C9" s="28"/>
-      <x:c r="D9" s="28"/>
-      <x:c r="E9" s="28"/>
-      <x:c r="F9" s="28"/>
-      <x:c r="G9" s="28"/>
-      <x:c r="H9" s="28"/>
-      <x:c r="I9" s="28"/>
-      <x:c r="J9" s="30" t="n">
-        <x:f>SUM(J4:J6)</x:f>
-        <x:v>317.4</x:v>
-      </x:c>
-      <x:c r="K9" s="28"/>
+    <x:row r="7">
+      <x:c r="A7" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C7" s="22" t="str">
+        <x:v>9月4日</x:v>
+      </x:c>
+      <x:c r="D7" s="23" t="n">
+        <x:v>7655.97</x:v>
+      </x:c>
+      <x:c r="E7" s="23" t="n">
+        <x:v>7717.93</x:v>
+      </x:c>
+      <x:c r="F7" s="23" t="n">
+        <x:v>7464.98</x:v>
+      </x:c>
+      <x:c r="G7" s="23" t="n">
+        <x:v>7508.09</x:v>
+      </x:c>
+      <x:c r="H7" s="23" t="n">
+        <x:v>-92</x:v>
+      </x:c>
+      <x:c r="I7" s="24" t="n">
+        <x:v>-0.012106419652373024</x:v>
+      </x:c>
+      <x:c r="J7" s="26" t="n">
+        <x:f>ROUND(E7-F7,1)</x:f>
+        <x:v>253</x:v>
+      </x:c>
+      <x:c r="K7" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B10" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B10" s="28" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="C10" s="28"/>
       <x:c r="D10" s="28"/>
       <x:c r="E10" s="28"/>
@@ -2252,11 +2306,29 @@
       <x:c r="G10" s="28"/>
       <x:c r="H10" s="28"/>
       <x:c r="I10" s="28"/>
-      <x:c r="J10" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J6),0),1)</x:f>
-        <x:v>105.8</x:v>
+      <x:c r="J10" s="30" t="n">
+        <x:f>SUM(J4:J7)</x:f>
+        <x:v>570.4</x:v>
       </x:c>
       <x:c r="K10" s="28"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B11" s="28"/>
+      <x:c r="C11" s="28"/>
+      <x:c r="D11" s="28"/>
+      <x:c r="E11" s="28"/>
+      <x:c r="F11" s="28"/>
+      <x:c r="G11" s="28"/>
+      <x:c r="H11" s="28"/>
+      <x:c r="I11" s="28"/>
+      <x:c r="J11" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
+        <x:v>142.6</x:v>
+      </x:c>
+      <x:c r="K11" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2431,31 +2503,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B9" s="28" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C9" s="28"/>
-      <x:c r="D9" s="28"/>
-      <x:c r="E9" s="28"/>
-      <x:c r="F9" s="28"/>
-      <x:c r="G9" s="28"/>
-      <x:c r="H9" s="28"/>
-      <x:c r="I9" s="28"/>
-      <x:c r="J9" s="30" t="n">
-        <x:f>SUM(J4:J6)</x:f>
-        <x:v>306.8</x:v>
-      </x:c>
-      <x:c r="K9" s="28"/>
+    <x:row r="7">
+      <x:c r="A7" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C7" s="22" t="str">
+        <x:v>9月4日</x:v>
+      </x:c>
+      <x:c r="D7" s="23" t="n">
+        <x:v>7806.61</x:v>
+      </x:c>
+      <x:c r="E7" s="23" t="n">
+        <x:v>7850.4</x:v>
+      </x:c>
+      <x:c r="F7" s="23" t="n">
+        <x:v>7610.58</x:v>
+      </x:c>
+      <x:c r="G7" s="23" t="n">
+        <x:v>7652.69</x:v>
+      </x:c>
+      <x:c r="H7" s="23" t="n">
+        <x:v>-102.7</x:v>
+      </x:c>
+      <x:c r="I7" s="24" t="n">
+        <x:v>-0.01323858595861449</x:v>
+      </x:c>
+      <x:c r="J7" s="26" t="n">
+        <x:f>ROUND(E7-F7,1)</x:f>
+        <x:v>239.8</x:v>
+      </x:c>
+      <x:c r="K7" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B10" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B10" s="28" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="C10" s="28"/>
       <x:c r="D10" s="28"/>
       <x:c r="E10" s="28"/>
@@ -2463,11 +2553,29 @@
       <x:c r="G10" s="28"/>
       <x:c r="H10" s="28"/>
       <x:c r="I10" s="28"/>
-      <x:c r="J10" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J6),0),1)</x:f>
-        <x:v>102.3</x:v>
+      <x:c r="J10" s="30" t="n">
+        <x:f>SUM(J4:J7)</x:f>
+        <x:v>546.6</x:v>
       </x:c>
       <x:c r="K10" s="28"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B11" s="28"/>
+      <x:c r="C11" s="28"/>
+      <x:c r="D11" s="28"/>
+      <x:c r="E11" s="28"/>
+      <x:c r="F11" s="28"/>
+      <x:c r="G11" s="28"/>
+      <x:c r="H11" s="28"/>
+      <x:c r="I11" s="28"/>
+      <x:c r="J11" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
+        <x:v>136.7</x:v>
+      </x:c>
+      <x:c r="K11" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2642,31 +2750,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B9" s="28" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C9" s="28"/>
-      <x:c r="D9" s="28"/>
-      <x:c r="E9" s="28"/>
-      <x:c r="F9" s="28"/>
-      <x:c r="G9" s="28"/>
-      <x:c r="H9" s="28"/>
-      <x:c r="I9" s="28"/>
-      <x:c r="J9" s="30" t="n">
-        <x:f>SUM(J4:J6)</x:f>
-        <x:v>90</x:v>
-      </x:c>
-      <x:c r="K9" s="28"/>
+    <x:row r="7">
+      <x:c r="A7" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C7" s="22" t="str">
+        <x:v>9月4日</x:v>
+      </x:c>
+      <x:c r="D7" s="23" t="n">
+        <x:v>3955.55</x:v>
+      </x:c>
+      <x:c r="E7" s="23" t="n">
+        <x:v>3980.2</x:v>
+      </x:c>
+      <x:c r="F7" s="23" t="n">
+        <x:v>3915.22</x:v>
+      </x:c>
+      <x:c r="G7" s="23" t="n">
+        <x:v>3930.12</x:v>
+      </x:c>
+      <x:c r="H7" s="23" t="n">
+        <x:v>-12</x:v>
+      </x:c>
+      <x:c r="I7" s="24" t="n">
+        <x:v>-0.003036460354786441</x:v>
+      </x:c>
+      <x:c r="J7" s="26" t="n">
+        <x:f>ROUND(E7-F7,1)</x:f>
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="K7" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B10" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B10" s="28" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="C10" s="28"/>
       <x:c r="D10" s="28"/>
       <x:c r="E10" s="28"/>
@@ -2674,11 +2800,29 @@
       <x:c r="G10" s="28"/>
       <x:c r="H10" s="28"/>
       <x:c r="I10" s="28"/>
-      <x:c r="J10" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J6),0),1)</x:f>
-        <x:v>30</x:v>
+      <x:c r="J10" s="30" t="n">
+        <x:f>SUM(J4:J7)</x:f>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="K10" s="28"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B11" s="28"/>
+      <x:c r="C11" s="28"/>
+      <x:c r="D11" s="28"/>
+      <x:c r="E11" s="28"/>
+      <x:c r="F11" s="28"/>
+      <x:c r="G11" s="28"/>
+      <x:c r="H11" s="28"/>
+      <x:c r="I11" s="28"/>
+      <x:c r="J11" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
+        <x:v>38.8</x:v>
+      </x:c>
+      <x:c r="K11" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3486,31 +3630,49 @@
         <x:v>IH2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B9" s="28" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C9" s="28"/>
-      <x:c r="D9" s="28"/>
-      <x:c r="E9" s="28"/>
-      <x:c r="F9" s="28"/>
-      <x:c r="G9" s="28"/>
-      <x:c r="H9" s="28"/>
-      <x:c r="I9" s="28"/>
-      <x:c r="J9" s="30" t="n">
-        <x:f>SUM(J4:J6)</x:f>
-        <x:v>88</x:v>
-      </x:c>
-      <x:c r="K9" s="28"/>
+    <x:row r="7">
+      <x:c r="A7" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C7" s="22" t="str">
+        <x:v>9月4日</x:v>
+      </x:c>
+      <x:c r="D7" s="23" t="n">
+        <x:v>2922</x:v>
+      </x:c>
+      <x:c r="E7" s="23" t="n">
+        <x:v>2949.4</x:v>
+      </x:c>
+      <x:c r="F7" s="23" t="n">
+        <x:v>2904.8</x:v>
+      </x:c>
+      <x:c r="G7" s="23" t="n">
+        <x:v>2915.8</x:v>
+      </x:c>
+      <x:c r="H7" s="23" t="n">
+        <x:v>8.2</x:v>
+      </x:c>
+      <x:c r="I7" s="24" t="n">
+        <x:v>0.0028201953501170163</x:v>
+      </x:c>
+      <x:c r="J7" s="23" t="n">
+        <x:f>ROUND(E7-F7,1)</x:f>
+        <x:v>44.6</x:v>
+      </x:c>
+      <x:c r="K7" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B10" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B10" s="28" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="C10" s="28"/>
       <x:c r="D10" s="28"/>
       <x:c r="E10" s="28"/>
@@ -3518,11 +3680,29 @@
       <x:c r="G10" s="28"/>
       <x:c r="H10" s="28"/>
       <x:c r="I10" s="28"/>
-      <x:c r="J10" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J6),0),1)</x:f>
-        <x:v>29.3</x:v>
+      <x:c r="J10" s="30" t="n">
+        <x:f>SUM(J4:J7)</x:f>
+        <x:v>132.6</x:v>
       </x:c>
       <x:c r="K10" s="28"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B11" s="28"/>
+      <x:c r="C11" s="28"/>
+      <x:c r="D11" s="28"/>
+      <x:c r="E11" s="28"/>
+      <x:c r="F11" s="28"/>
+      <x:c r="G11" s="28"/>
+      <x:c r="H11" s="28"/>
+      <x:c r="I11" s="28"/>
+      <x:c r="J11" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
+        <x:v>33.2</x:v>
+      </x:c>
+      <x:c r="K11" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>